<commit_message>
Startup state reconciliation — mounts, jobs, and USB drives must be idempotent after reboot
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I208"/>
+  <dimension ref="A1:I218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6529,14 +6529,312 @@
       <c r="H206" s="4" t="n"/>
       <c r="I206" s="4" t="n"/>
     </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>§12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t>12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C207" s="3" t="n"/>
+      <c r="D207" s="3" t="n"/>
+      <c r="E207" s="3" t="n"/>
+      <c r="F207" s="3" t="n"/>
+      <c r="G207" s="3" t="n"/>
+      <c r="H207" s="3" t="n"/>
+      <c r="I207" s="3" t="n"/>
+    </row>
     <row r="208">
-      <c r="A208" s="5" t="inlineStr">
+      <c r="A208" s="4" t="inlineStr">
+        <is>
+          <t>TC-1101</t>
+        </is>
+      </c>
+      <c r="B208" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C208" s="4" t="inlineStr">
+        <is>
+          <t>Running job failed after restart</t>
+        </is>
+      </c>
+      <c r="D208" s="4" t="inlineStr">
+        <is>
+          <t>Create a job, start it, restart the service while RUNNING</t>
+        </is>
+      </c>
+      <c r="E208" s="4" t="inlineStr">
+        <is>
+          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
+        </is>
+      </c>
+      <c r="F208" s="4" t="n"/>
+      <c r="G208" s="4" t="n"/>
+      <c r="H208" s="4" t="n"/>
+      <c r="I208" s="4" t="n"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="4" t="inlineStr">
+        <is>
+          <t>TC-1102</t>
+        </is>
+      </c>
+      <c r="B209" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C209" s="4" t="inlineStr">
+        <is>
+          <t>Verifying job failed after restart</t>
+        </is>
+      </c>
+      <c r="D209" s="4" t="inlineStr">
+        <is>
+          <t>Start a job, let it reach VERIFYING, restart the service</t>
+        </is>
+      </c>
+      <c r="E209" s="4" t="inlineStr">
+        <is>
+          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
+        </is>
+      </c>
+      <c r="F209" s="4" t="n"/>
+      <c r="G209" s="4" t="n"/>
+      <c r="H209" s="4" t="n"/>
+      <c r="I209" s="4" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="4" t="inlineStr">
+        <is>
+          <t>TC-1103</t>
+        </is>
+      </c>
+      <c r="B210" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C210" s="4" t="inlineStr">
+        <is>
+          <t>Pending job not affected</t>
+        </is>
+      </c>
+      <c r="D210" s="4" t="inlineStr">
+        <is>
+          <t>Create a job (PENDING), restart the service</t>
+        </is>
+      </c>
+      <c r="E210" s="4" t="inlineStr">
+        <is>
+          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
+        </is>
+      </c>
+      <c r="F210" s="4" t="n"/>
+      <c r="G210" s="4" t="n"/>
+      <c r="H210" s="4" t="n"/>
+      <c r="I210" s="4" t="n"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="4" t="inlineStr">
+        <is>
+          <t>TC-1104</t>
+        </is>
+      </c>
+      <c r="B211" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C211" s="4" t="inlineStr">
+        <is>
+          <t>Completed job not affected</t>
+        </is>
+      </c>
+      <c r="D211" s="4" t="inlineStr">
+        <is>
+          <t>Complete a job, restart the service</t>
+        </is>
+      </c>
+      <c r="E211" s="4" t="inlineStr">
+        <is>
+          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
+        </is>
+      </c>
+      <c r="F211" s="4" t="n"/>
+      <c r="G211" s="4" t="n"/>
+      <c r="H211" s="4" t="n"/>
+      <c r="I211" s="4" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="4" t="inlineStr">
+        <is>
+          <t>TC-1105</t>
+        </is>
+      </c>
+      <c r="B212" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C212" s="4" t="inlineStr">
+        <is>
+          <t>Stale mount corrected</t>
+        </is>
+      </c>
+      <c r="D212" s="4" t="inlineStr">
+        <is>
+          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
+        </is>
+      </c>
+      <c r="E212" s="4" t="inlineStr">
+        <is>
+          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
+        </is>
+      </c>
+      <c r="F212" s="4" t="n"/>
+      <c r="G212" s="4" t="n"/>
+      <c r="H212" s="4" t="n"/>
+      <c r="I212" s="4" t="n"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="4" t="inlineStr">
+        <is>
+          <t>TC-1106</t>
+        </is>
+      </c>
+      <c r="B213" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C213" s="4" t="inlineStr">
+        <is>
+          <t>Active mount preserved</t>
+        </is>
+      </c>
+      <c r="D213" s="4" t="inlineStr">
+        <is>
+          <t>Add and mount a network share (leave it mounted), restart the service</t>
+        </is>
+      </c>
+      <c r="E213" s="4" t="inlineStr">
+        <is>
+          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
+        </is>
+      </c>
+      <c r="F213" s="4" t="n"/>
+      <c r="G213" s="4" t="n"/>
+      <c r="H213" s="4" t="n"/>
+      <c r="I213" s="4" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="4" t="inlineStr">
+        <is>
+          <t>TC-1107</t>
+        </is>
+      </c>
+      <c r="B214" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C214" s="4" t="inlineStr">
+        <is>
+          <t>USB drives re-discovered</t>
+        </is>
+      </c>
+      <c r="D214" s="4" t="inlineStr">
+        <is>
+          <t>Insert USB drives, restart the service</t>
+        </is>
+      </c>
+      <c r="E214" s="4" t="inlineStr">
+        <is>
+          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
+        </is>
+      </c>
+      <c r="F214" s="4" t="n"/>
+      <c r="G214" s="4" t="n"/>
+      <c r="H214" s="4" t="n"/>
+      <c r="I214" s="4" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="4" t="inlineStr">
+        <is>
+          <t>TC-1108</t>
+        </is>
+      </c>
+      <c r="B215" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C215" s="4" t="inlineStr">
+        <is>
+          <t>Idempotency</t>
+        </is>
+      </c>
+      <c r="D215" s="4" t="inlineStr">
+        <is>
+          <t>Restart the service twice without any state changes between restarts</t>
+        </is>
+      </c>
+      <c r="E215" s="4" t="inlineStr">
+        <is>
+          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
+        </is>
+      </c>
+      <c r="F215" s="4" t="n"/>
+      <c r="G215" s="4" t="n"/>
+      <c r="H215" s="4" t="n"/>
+      <c r="I215" s="4" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="4" t="inlineStr">
+        <is>
+          <t>TC-1109</t>
+        </is>
+      </c>
+      <c r="B216" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C216" s="4" t="inlineStr">
+        <is>
+          <t>Partial failure isolation</t>
+        </is>
+      </c>
+      <c r="D216" s="4" t="inlineStr">
+        <is>
+          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
+        </is>
+      </c>
+      <c r="E216" s="4" t="inlineStr">
+        <is>
+          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
+        </is>
+      </c>
+      <c r="F216" s="4" t="n"/>
+      <c r="G216" s="4" t="n"/>
+      <c r="H216" s="4" t="n"/>
+      <c r="I216" s="4" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B208" s="5" t="n">
-        <v>190</v>
+      <c r="B218" s="5" t="n">
+        <v>199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update QA test cases in ecube-qa-test-cases.xlsx
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I218"/>
+  <dimension ref="A1:I221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6827,14 +6827,107 @@
       <c r="H216" s="4" t="n"/>
       <c r="I216" s="4" t="n"/>
     </row>
+    <row r="217">
+      <c r="A217" s="4" t="inlineStr">
+        <is>
+          <t>TC-1110</t>
+        </is>
+      </c>
+      <c r="B217" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C217" s="4" t="inlineStr">
+        <is>
+          <t>Cross-process lock — only one worker reconciles</t>
+        </is>
+      </c>
+      <c r="D217" s="4" t="inlineStr">
+        <is>
+          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
+        </is>
+      </c>
+      <c r="E217" s="4" t="inlineStr">
+        <is>
+          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
+        </is>
+      </c>
+      <c r="F217" s="4" t="n"/>
+      <c r="G217" s="4" t="n"/>
+      <c r="H217" s="4" t="n"/>
+      <c r="I217" s="4" t="n"/>
+    </row>
     <row r="218">
-      <c r="A218" s="5" t="inlineStr">
+      <c r="A218" s="4" t="inlineStr">
+        <is>
+          <t>TC-1111</t>
+        </is>
+      </c>
+      <c r="B218" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C218" s="4" t="inlineStr">
+        <is>
+          <t>Stale lock reclaim</t>
+        </is>
+      </c>
+      <c r="D218" s="4" t="inlineStr">
+        <is>
+          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
+        </is>
+      </c>
+      <c r="E218" s="4" t="inlineStr">
+        <is>
+          <t>Service reclaims the stale lock, reconciliation runs normally</t>
+        </is>
+      </c>
+      <c r="F218" s="4" t="n"/>
+      <c r="G218" s="4" t="n"/>
+      <c r="H218" s="4" t="n"/>
+      <c r="I218" s="4" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="4" t="inlineStr">
+        <is>
+          <t>TC-1112</t>
+        </is>
+      </c>
+      <c r="B219" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C219" s="4" t="inlineStr">
+        <is>
+          <t>Lock released after failure</t>
+        </is>
+      </c>
+      <c r="D219" s="4" t="inlineStr">
+        <is>
+          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
+        </is>
+      </c>
+      <c r="E219" s="4" t="inlineStr">
+        <is>
+          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
+        </is>
+      </c>
+      <c r="F219" s="4" t="n"/>
+      <c r="G219" s="4" t="n"/>
+      <c r="H219" s="4" t="n"/>
+      <c r="I219" s="4" t="n"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B218" s="5" t="n">
-        <v>199</v>
+      <c r="B221" s="5" t="n">
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ecube-qa-test-cases.xlsx with new test cases and improvements
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -4463,7 +4463,7 @@
       </c>
       <c r="D139" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with username, password, groups, roles</t>
+          <t>POST /admin/os-users with username, password, roles</t>
         </is>
       </c>
       <c r="E139" s="4" t="inlineStr">
@@ -4675,17 +4675,17 @@
       </c>
       <c r="C146" s="4" t="inlineStr">
         <is>
-          <t>Create user — no ecube-* group</t>
+          <t>Create user — no roles</t>
         </is>
       </c>
       <c r="D146" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with no groups or only non-ecube-* groups</t>
+          <t>POST /admin/os-users with empty/omitted roles</t>
         </is>
       </c>
       <c r="E146" s="4" t="inlineStr">
         <is>
-          <t>422, at least one ecube-* group required</t>
+          <t>422, at least one role required</t>
         </is>
       </c>
       <c r="F146" s="4" t="n"/>

</xml_diff>

<commit_message>
Add system-info and provision-status endpoint tests for database setup
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I221"/>
+  <dimension ref="A1:I225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5581,17 +5581,17 @@
       </c>
       <c r="C176" s="4" t="inlineStr">
         <is>
-          <t>Test connection — success</t>
+          <t>System info — bare-metal defaults</t>
         </is>
       </c>
       <c r="D176" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with valid PostgreSQL credentials</t>
+          <t>GET /setup/database/system-info before setup</t>
         </is>
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
-          <t>200, {"status": "ok", "server_version": "..."}</t>
+          <t>200, {"in_docker": false, "suggested_db_host": "localhost"}</t>
         </is>
       </c>
       <c r="F176" s="4" t="n"/>
@@ -5612,17 +5612,17 @@
       </c>
       <c r="C177" s="4" t="inlineStr">
         <is>
-          <t>Test connection — bad host</t>
+          <t>Provision status — pre-init public</t>
         </is>
       </c>
       <c r="D177" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with unreachable host</t>
+          <t>GET /setup/database/provision-status before any admin exists</t>
         </is>
       </c>
       <c r="E177" s="4" t="inlineStr">
         <is>
-          <t>400, connection error</t>
+          <t>200, {"provisioned": false}</t>
         </is>
       </c>
       <c r="F177" s="4" t="n"/>
@@ -5643,17 +5643,17 @@
       </c>
       <c r="C178" s="4" t="inlineStr">
         <is>
-          <t>Test connection — SSRF host</t>
+          <t>Provision status — post-init requires admin</t>
         </is>
       </c>
       <c r="D178" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with "host": "http://evil.com"</t>
+          <t>GET /setup/database/provision-status without token after setup</t>
         </is>
       </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
-          <t>422, invalid host</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F178" s="4" t="n"/>
@@ -5674,17 +5674,17 @@
       </c>
       <c r="C179" s="4" t="inlineStr">
         <is>
-          <t>Test connection — port out of range</t>
+          <t>Provision status — state unknown</t>
         </is>
       </c>
       <c r="D179" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with "port": 99999</t>
+          <t>Stop PostgreSQL, GET /setup/database/provision-status during initial setup</t>
         </is>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>503, cannot determine provisioning state</t>
         </is>
       </c>
       <c r="F179" s="4" t="n"/>
@@ -5705,17 +5705,17 @@
       </c>
       <c r="C180" s="4" t="inlineStr">
         <is>
-          <t>Provision — success</t>
+          <t>Test connection — success</t>
         </is>
       </c>
       <c r="D180" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with valid credentials</t>
+          <t>POST /setup/database/test-connection with valid PostgreSQL credentials</t>
         </is>
       </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
-          <t>200, returns database, user, migrations_applied</t>
+          <t>200, {"status": "ok", "server_version": "..."}</t>
         </is>
       </c>
       <c r="F180" s="4" t="n"/>
@@ -5736,12 +5736,12 @@
       </c>
       <c r="C181" s="4" t="inlineStr">
         <is>
-          <t>Provision — bad admin credentials</t>
+          <t>Test connection — bad host</t>
         </is>
       </c>
       <c r="D181" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with wrong admin password</t>
+          <t>POST /setup/database/test-connection with unreachable host</t>
         </is>
       </c>
       <c r="E181" s="4" t="inlineStr">
@@ -5767,17 +5767,17 @@
       </c>
       <c r="C182" s="4" t="inlineStr">
         <is>
-          <t>Provision — invalid database name</t>
+          <t>Test connection — SSRF host</t>
         </is>
       </c>
       <c r="D182" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with "app_database": "drop;--"</t>
+          <t>POST /setup/database/test-connection with "host": "http://evil.com"</t>
         </is>
       </c>
       <c r="E182" s="4" t="inlineStr">
         <is>
-          <t>422, invalid identifier</t>
+          <t>422, invalid host</t>
         </is>
       </c>
       <c r="F182" s="4" t="n"/>
@@ -5798,17 +5798,17 @@
       </c>
       <c r="C183" s="4" t="inlineStr">
         <is>
-          <t>Status — connected</t>
+          <t>Test connection — port out of range</t>
         </is>
       </c>
       <c r="D183" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/status with admin token</t>
+          <t>POST /setup/database/test-connection with "port": 99999</t>
         </is>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>200, connected: true, migration info</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F183" s="4" t="n"/>
@@ -5829,17 +5829,17 @@
       </c>
       <c r="C184" s="4" t="inlineStr">
         <is>
-          <t>Status — requires auth</t>
+          <t>Provision — success</t>
         </is>
       </c>
       <c r="D184" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/status without token</t>
+          <t>POST /setup/database/provision with valid credentials</t>
         </is>
       </c>
       <c r="E184" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>200, returns database, user, migrations_applied</t>
         </is>
       </c>
       <c r="F184" s="4" t="n"/>
@@ -5860,17 +5860,17 @@
       </c>
       <c r="C185" s="4" t="inlineStr">
         <is>
-          <t>Status — requires admin</t>
+          <t>Provision — bad admin credentials</t>
         </is>
       </c>
       <c r="D185" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/status with processor token</t>
+          <t>POST /setup/database/provision with wrong admin password</t>
         </is>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>403</t>
+          <t>400, connection error</t>
         </is>
       </c>
       <c r="F185" s="4" t="n"/>
@@ -5891,17 +5891,17 @@
       </c>
       <c r="C186" s="4" t="inlineStr">
         <is>
-          <t>Settings update — success</t>
+          <t>Provision — invalid database name</t>
         </is>
       </c>
       <c r="D186" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with valid partial update</t>
+          <t>POST /setup/database/provision with "app_database": "drop;--"</t>
         </is>
       </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
-          <t>200, {"status": "updated", ...}</t>
+          <t>422, invalid identifier</t>
         </is>
       </c>
       <c r="F186" s="4" t="n"/>
@@ -5922,17 +5922,17 @@
       </c>
       <c r="C187" s="4" t="inlineStr">
         <is>
-          <t>Settings update — bad connection</t>
+          <t>Status — connected</t>
         </is>
       </c>
       <c r="D187" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with unreachable host</t>
+          <t>GET /setup/database/status with admin token</t>
         </is>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>400, connection test failed</t>
+          <t>200, connected: true, migration info</t>
         </is>
       </c>
       <c r="F187" s="4" t="n"/>
@@ -5953,17 +5953,17 @@
       </c>
       <c r="C188" s="4" t="inlineStr">
         <is>
-          <t>Settings update — empty body</t>
+          <t>Status — requires auth</t>
         </is>
       </c>
       <c r="D188" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with {}</t>
+          <t>GET /setup/database/status without token</t>
         </is>
       </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
-          <t>422, at least one field required</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F188" s="4" t="n"/>
@@ -5984,12 +5984,12 @@
       </c>
       <c r="C189" s="4" t="inlineStr">
         <is>
-          <t>Settings update — requires admin</t>
+          <t>Status — requires admin</t>
         </is>
       </c>
       <c r="D189" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with processor token</t>
+          <t>GET /setup/database/status with processor token</t>
         </is>
       </c>
       <c r="E189" s="4" t="inlineStr">
@@ -6015,17 +6015,17 @@
       </c>
       <c r="C190" s="4" t="inlineStr">
         <is>
-          <t>Auth after setup — test-connection</t>
+          <t>Settings update — success</t>
         </is>
       </c>
       <c r="D190" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection without token (after admin exists)</t>
+          <t>PUT /setup/database/settings with valid partial update</t>
         </is>
       </c>
       <c r="E190" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>200, {"status": "updated", ...}</t>
         </is>
       </c>
       <c r="F190" s="4" t="n"/>
@@ -6046,17 +6046,17 @@
       </c>
       <c r="C191" s="4" t="inlineStr">
         <is>
-          <t>Auth after setup — provision</t>
+          <t>Settings update — bad connection</t>
         </is>
       </c>
       <c r="D191" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision without token (after admin exists)</t>
+          <t>PUT /setup/database/settings with unreachable host</t>
         </is>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>400, connection test failed</t>
         </is>
       </c>
       <c r="F191" s="4" t="n"/>
@@ -6077,17 +6077,17 @@
       </c>
       <c r="C192" s="4" t="inlineStr">
         <is>
-          <t>Password redaction</t>
+          <t>Settings update — empty body</t>
         </is>
       </c>
       <c r="D192" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision and check response</t>
+          <t>PUT /setup/database/settings with {}</t>
         </is>
       </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
-          <t>No password in response body</t>
+          <t>422, at least one field required</t>
         </is>
       </c>
       <c r="F192" s="4" t="n"/>
@@ -6108,17 +6108,17 @@
       </c>
       <c r="C193" s="4" t="inlineStr">
         <is>
-          <t>Re-provision blocked</t>
+          <t>Settings update — requires admin</t>
         </is>
       </c>
       <c r="D193" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision after successful provisioning (no force)</t>
+          <t>PUT /setup/database/settings with processor token</t>
         </is>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>409, already provisioned</t>
+          <t>403</t>
         </is>
       </c>
       <c r="F193" s="4" t="n"/>
@@ -6139,17 +6139,17 @@
       </c>
       <c r="C194" s="4" t="inlineStr">
         <is>
-          <t>Force re-provision (admin)</t>
+          <t>Auth after setup — test-connection</t>
         </is>
       </c>
       <c r="D194" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with "force": true and admin token after successful provisioning</t>
+          <t>POST /setup/database/test-connection without token (after admin exists)</t>
         </is>
       </c>
       <c r="E194" s="4" t="inlineStr">
         <is>
-          <t>200, returns database, user, migrations_applied</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F194" s="4" t="n"/>
@@ -6170,17 +6170,17 @@
       </c>
       <c r="C195" s="4" t="inlineStr">
         <is>
-          <t>Force rejected unauthenticated</t>
+          <t>Auth after setup — provision</t>
         </is>
       </c>
       <c r="D195" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with "force": true during initial setup (no admin exists)</t>
+          <t>POST /setup/database/provision without token (after admin exists)</t>
         </is>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>403, force requires admin</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F195" s="4" t="n"/>
@@ -6201,17 +6201,17 @@
       </c>
       <c r="C196" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — DB unreachable, no JWT</t>
+          <t>Password redaction</t>
         </is>
       </c>
       <c r="D196" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/test-connection without token</t>
+          <t>POST /setup/database/provision and check response</t>
         </is>
       </c>
       <c r="E196" s="4" t="inlineStr">
         <is>
-          <t>503, database unavailable message</t>
+          <t>No password in response body</t>
         </is>
       </c>
       <c r="F196" s="4" t="n"/>
@@ -6232,17 +6232,17 @@
       </c>
       <c r="C197" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — DB unreachable, admin JWT</t>
+          <t>Re-provision blocked</t>
         </is>
       </c>
       <c r="D197" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/test-connection with valid admin token</t>
+          <t>POST /setup/database/provision after successful provisioning (no force)</t>
         </is>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>Request proceeds (not blocked by 503)</t>
+          <t>409, already provisioned</t>
         </is>
       </c>
       <c r="F197" s="4" t="n"/>
@@ -6263,17 +6263,17 @@
       </c>
       <c r="C198" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — provision state unknown</t>
+          <t>Force re-provision (admin)</t>
         </is>
       </c>
       <c r="D198" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/provision without "force": true</t>
+          <t>POST /setup/database/provision with "force": true and admin token after successful provisioning</t>
         </is>
       </c>
       <c r="E198" s="4" t="inlineStr">
         <is>
-          <t>503, cannot determine provisioning state</t>
+          <t>200, returns database, user, migrations_applied</t>
         </is>
       </c>
       <c r="F198" s="4" t="n"/>
@@ -6294,17 +6294,17 @@
       </c>
       <c r="C199" s="4" t="inlineStr">
         <is>
-          <t>Force bypasses state check</t>
+          <t>Force rejected unauthenticated</t>
         </is>
       </c>
       <c r="D199" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/provision with "force": true and admin token</t>
+          <t>POST /setup/database/provision with "force": true during initial setup (no admin exists)</t>
         </is>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>Proceeds to provisioning (no 503 from state check)</t>
+          <t>403, force requires admin</t>
         </is>
       </c>
       <c r="F199" s="4" t="n"/>
@@ -6325,17 +6325,17 @@
       </c>
       <c r="C200" s="4" t="inlineStr">
         <is>
-          <t>Unmigrated DB treated as initial setup</t>
+          <t>Fail-closed — DB unreachable, no JWT</t>
         </is>
       </c>
       <c r="D200" s="4" t="inlineStr">
         <is>
-          <t>Drop user_roles table (or use a fresh empty database), POST /setup/database/test-connection without token</t>
+          <t>Stop PostgreSQL, POST /setup/database/test-connection without token</t>
         </is>
       </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
-          <t>200, request allowed (not 503)</t>
+          <t>503, database unavailable message</t>
         </is>
       </c>
       <c r="F200" s="4" t="n"/>
@@ -6356,17 +6356,17 @@
       </c>
       <c r="C201" s="4" t="inlineStr">
         <is>
-          <t>Fresh install — DB/role missing</t>
+          <t>Fail-closed — DB unreachable, admin JWT</t>
         </is>
       </c>
       <c r="D201" s="4" t="inlineStr">
         <is>
-          <t>With PostgreSQL running but the application database or role not yet created, POST /setup/database/provision without force</t>
+          <t>Stop PostgreSQL, POST /setup/database/test-connection with valid admin token</t>
         </is>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>200, provisioning proceeds (not 503)</t>
+          <t>Request proceeds (not blocked by 503)</t>
         </is>
       </c>
       <c r="F201" s="4" t="n"/>
@@ -6387,17 +6387,17 @@
       </c>
       <c r="C202" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — OperationalError on reachable DB</t>
+          <t>Fail-closed — provision state unknown</t>
         </is>
       </c>
       <c r="D202" s="4" t="inlineStr">
         <is>
-          <t>Revoke SELECT on user_roles (or simulate permission denied), POST /setup/database/test-connection without token</t>
+          <t>Stop PostgreSQL, POST /setup/database/provision without "force": true</t>
         </is>
       </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
-          <t>503, does NOT grant unauthenticated access</t>
+          <t>503, cannot determine provisioning state</t>
         </is>
       </c>
       <c r="F202" s="4" t="n"/>
@@ -6418,17 +6418,17 @@
       </c>
       <c r="C203" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — unexpected error</t>
+          <t>Force bypasses state check</t>
         </is>
       </c>
       <c r="D203" s="4" t="inlineStr">
         <is>
-          <t>Trigger an unexpected exception from admin-check (e.g. coding bug), POST /setup/database/test-connection without token</t>
+          <t>Stop PostgreSQL, POST /setup/database/provision with "force": true and admin token</t>
         </is>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
-          <t>503, does NOT grant unauthenticated access</t>
+          <t>Proceeds to provisioning (no 503 from state check)</t>
         </is>
       </c>
       <c r="F203" s="4" t="n"/>
@@ -6449,17 +6449,17 @@
       </c>
       <c r="C204" s="4" t="inlineStr">
         <is>
-          <t>Provision — migration failure</t>
+          <t>Unmigrated DB treated as initial setup</t>
         </is>
       </c>
       <c r="D204" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with valid credentials but a broken Alembic migration (e.g. conflicting schema)</t>
+          <t>Drop user_roles table (or use a fresh empty database), POST /setup/database/test-connection without token</t>
         </is>
       </c>
       <c r="E204" s="4" t="inlineStr">
         <is>
-          <t>500, "migration failed" message; .env not updated, engine not swapped</t>
+          <t>200, request allowed (not 503)</t>
         </is>
       </c>
       <c r="F204" s="4" t="n"/>
@@ -6480,17 +6480,17 @@
       </c>
       <c r="C205" s="4" t="inlineStr">
         <is>
-          <t>Provision — .env write failure</t>
+          <t>Fresh install — DB/role missing</t>
         </is>
       </c>
       <c r="D205" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision after making .env read-only (or disk full)</t>
+          <t>With PostgreSQL running but the application database or role not yet created, POST /setup/database/provision without force</t>
         </is>
       </c>
       <c r="E205" s="4" t="inlineStr">
         <is>
-          <t>500, "failed to persist" message; engine not swapped</t>
+          <t>200, provisioning proceeds (not 503)</t>
         </is>
       </c>
       <c r="F205" s="4" t="n"/>
@@ -6511,17 +6511,17 @@
       </c>
       <c r="C206" s="4" t="inlineStr">
         <is>
-          <t>Provision — engine reinit failure</t>
+          <t>Fail-closed — OperationalError on reachable DB</t>
         </is>
       </c>
       <c r="D206" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision while another reinit is in progress (lock contention)</t>
+          <t>Revoke SELECT on user_roles (or simulate permission denied), POST /setup/database/test-connection without token</t>
         </is>
       </c>
       <c r="E206" s="4" t="inlineStr">
         <is>
-          <t>500, "engine could not be switched" message; .env already written</t>
+          <t>503, does NOT grant unauthenticated access</t>
         </is>
       </c>
       <c r="F206" s="4" t="n"/>
@@ -6530,48 +6530,60 @@
       <c r="I206" s="4" t="n"/>
     </row>
     <row r="207">
-      <c r="A207" s="2" t="inlineStr">
-        <is>
-          <t>§12.11 Startup State Reconciliation</t>
-        </is>
-      </c>
-      <c r="B207" s="2" t="inlineStr">
-        <is>
-          <t>12.11 Startup State Reconciliation</t>
-        </is>
-      </c>
-      <c r="C207" s="3" t="n"/>
-      <c r="D207" s="3" t="n"/>
-      <c r="E207" s="3" t="n"/>
-      <c r="F207" s="3" t="n"/>
-      <c r="G207" s="3" t="n"/>
-      <c r="H207" s="3" t="n"/>
-      <c r="I207" s="3" t="n"/>
+      <c r="A207" s="4" t="inlineStr">
+        <is>
+          <t>TC-1132</t>
+        </is>
+      </c>
+      <c r="B207" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C207" s="4" t="inlineStr">
+        <is>
+          <t>Fail-closed — unexpected error</t>
+        </is>
+      </c>
+      <c r="D207" s="4" t="inlineStr">
+        <is>
+          <t>Trigger an unexpected exception from admin-check (e.g. coding bug), POST /setup/database/test-connection without token</t>
+        </is>
+      </c>
+      <c r="E207" s="4" t="inlineStr">
+        <is>
+          <t>503, does NOT grant unauthenticated access</t>
+        </is>
+      </c>
+      <c r="F207" s="4" t="n"/>
+      <c r="G207" s="4" t="n"/>
+      <c r="H207" s="4" t="n"/>
+      <c r="I207" s="4" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
         <is>
-          <t>TC-1101</t>
+          <t>TC-1133</t>
         </is>
       </c>
       <c r="B208" s="4" t="inlineStr">
         <is>
-          <t>12.11 Startup State Reconciliation</t>
+          <t>12.11 Database Provisioning</t>
         </is>
       </c>
       <c r="C208" s="4" t="inlineStr">
         <is>
-          <t>Running job failed after restart</t>
+          <t>Provision — migration failure</t>
         </is>
       </c>
       <c r="D208" s="4" t="inlineStr">
         <is>
-          <t>Create a job, start it, restart the service while RUNNING</t>
+          <t>POST /setup/database/provision with valid credentials but a broken Alembic migration (e.g. conflicting schema)</t>
         </is>
       </c>
       <c r="E208" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
+          <t>500, "migration failed" message; .env not updated, engine not swapped</t>
         </is>
       </c>
       <c r="F208" s="4" t="n"/>
@@ -6582,27 +6594,27 @@
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
         <is>
-          <t>TC-1102</t>
+          <t>TC-1134</t>
         </is>
       </c>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>12.11 Startup State Reconciliation</t>
+          <t>12.11 Database Provisioning</t>
         </is>
       </c>
       <c r="C209" s="4" t="inlineStr">
         <is>
-          <t>Verifying job failed after restart</t>
+          <t>Provision — .env write failure</t>
         </is>
       </c>
       <c r="D209" s="4" t="inlineStr">
         <is>
-          <t>Start a job, let it reach VERIFYING, restart the service</t>
+          <t>POST /setup/database/provision after making .env read-only (or disk full)</t>
         </is>
       </c>
       <c r="E209" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
+          <t>500, "failed to persist" message; engine not swapped</t>
         </is>
       </c>
       <c r="F209" s="4" t="n"/>
@@ -6613,27 +6625,27 @@
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
         <is>
-          <t>TC-1103</t>
+          <t>TC-1135</t>
         </is>
       </c>
       <c r="B210" s="4" t="inlineStr">
         <is>
-          <t>12.11 Startup State Reconciliation</t>
+          <t>12.11 Database Provisioning</t>
         </is>
       </c>
       <c r="C210" s="4" t="inlineStr">
         <is>
-          <t>Pending job not affected</t>
+          <t>Provision — engine reinit failure</t>
         </is>
       </c>
       <c r="D210" s="4" t="inlineStr">
         <is>
-          <t>Create a job (PENDING), restart the service</t>
+          <t>POST /setup/database/provision while another reinit is in progress (lock contention)</t>
         </is>
       </c>
       <c r="E210" s="4" t="inlineStr">
         <is>
-          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
+          <t>500, "engine could not be switched" message; .env already written</t>
         </is>
       </c>
       <c r="F210" s="4" t="n"/>
@@ -6642,40 +6654,28 @@
       <c r="I210" s="4" t="n"/>
     </row>
     <row r="211">
-      <c r="A211" s="4" t="inlineStr">
-        <is>
-          <t>TC-1104</t>
-        </is>
-      </c>
-      <c r="B211" s="4" t="inlineStr">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>§12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
         <is>
           <t>12.11 Startup State Reconciliation</t>
         </is>
       </c>
-      <c r="C211" s="4" t="inlineStr">
-        <is>
-          <t>Completed job not affected</t>
-        </is>
-      </c>
-      <c r="D211" s="4" t="inlineStr">
-        <is>
-          <t>Complete a job, restart the service</t>
-        </is>
-      </c>
-      <c r="E211" s="4" t="inlineStr">
-        <is>
-          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
-        </is>
-      </c>
-      <c r="F211" s="4" t="n"/>
-      <c r="G211" s="4" t="n"/>
-      <c r="H211" s="4" t="n"/>
-      <c r="I211" s="4" t="n"/>
+      <c r="C211" s="3" t="n"/>
+      <c r="D211" s="3" t="n"/>
+      <c r="E211" s="3" t="n"/>
+      <c r="F211" s="3" t="n"/>
+      <c r="G211" s="3" t="n"/>
+      <c r="H211" s="3" t="n"/>
+      <c r="I211" s="3" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
         <is>
-          <t>TC-1105</t>
+          <t>TC-1101</t>
         </is>
       </c>
       <c r="B212" s="4" t="inlineStr">
@@ -6685,17 +6685,17 @@
       </c>
       <c r="C212" s="4" t="inlineStr">
         <is>
-          <t>Stale mount corrected</t>
+          <t>Running job failed after restart</t>
         </is>
       </c>
       <c r="D212" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
+          <t>Create a job, start it, restart the service while RUNNING</t>
         </is>
       </c>
       <c r="E212" s="4" t="inlineStr">
         <is>
-          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
+          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
         </is>
       </c>
       <c r="F212" s="4" t="n"/>
@@ -6706,7 +6706,7 @@
     <row r="213">
       <c r="A213" s="4" t="inlineStr">
         <is>
-          <t>TC-1106</t>
+          <t>TC-1102</t>
         </is>
       </c>
       <c r="B213" s="4" t="inlineStr">
@@ -6716,17 +6716,17 @@
       </c>
       <c r="C213" s="4" t="inlineStr">
         <is>
-          <t>Active mount preserved</t>
+          <t>Verifying job failed after restart</t>
         </is>
       </c>
       <c r="D213" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share (leave it mounted), restart the service</t>
+          <t>Start a job, let it reach VERIFYING, restart the service</t>
         </is>
       </c>
       <c r="E213" s="4" t="inlineStr">
         <is>
-          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
+          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
         </is>
       </c>
       <c r="F213" s="4" t="n"/>
@@ -6737,7 +6737,7 @@
     <row r="214">
       <c r="A214" s="4" t="inlineStr">
         <is>
-          <t>TC-1107</t>
+          <t>TC-1103</t>
         </is>
       </c>
       <c r="B214" s="4" t="inlineStr">
@@ -6747,17 +6747,17 @@
       </c>
       <c r="C214" s="4" t="inlineStr">
         <is>
-          <t>USB drives re-discovered</t>
+          <t>Pending job not affected</t>
         </is>
       </c>
       <c r="D214" s="4" t="inlineStr">
         <is>
-          <t>Insert USB drives, restart the service</t>
+          <t>Create a job (PENDING), restart the service</t>
         </is>
       </c>
       <c r="E214" s="4" t="inlineStr">
         <is>
-          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
+          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
         </is>
       </c>
       <c r="F214" s="4" t="n"/>
@@ -6768,7 +6768,7 @@
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
         <is>
-          <t>TC-1108</t>
+          <t>TC-1104</t>
         </is>
       </c>
       <c r="B215" s="4" t="inlineStr">
@@ -6778,17 +6778,17 @@
       </c>
       <c r="C215" s="4" t="inlineStr">
         <is>
-          <t>Idempotency</t>
+          <t>Completed job not affected</t>
         </is>
       </c>
       <c r="D215" s="4" t="inlineStr">
         <is>
-          <t>Restart the service twice without any state changes between restarts</t>
+          <t>Complete a job, restart the service</t>
         </is>
       </c>
       <c r="E215" s="4" t="inlineStr">
         <is>
-          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
+          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F215" s="4" t="n"/>
@@ -6799,7 +6799,7 @@
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
         <is>
-          <t>TC-1109</t>
+          <t>TC-1105</t>
         </is>
       </c>
       <c r="B216" s="4" t="inlineStr">
@@ -6809,17 +6809,17 @@
       </c>
       <c r="C216" s="4" t="inlineStr">
         <is>
-          <t>Partial failure isolation</t>
+          <t>Stale mount corrected</t>
         </is>
       </c>
       <c r="D216" s="4" t="inlineStr">
         <is>
-          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
+          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
         </is>
       </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
-          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
+          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
         </is>
       </c>
       <c r="F216" s="4" t="n"/>
@@ -6830,7 +6830,7 @@
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
         <is>
-          <t>TC-1110</t>
+          <t>TC-1106</t>
         </is>
       </c>
       <c r="B217" s="4" t="inlineStr">
@@ -6840,17 +6840,17 @@
       </c>
       <c r="C217" s="4" t="inlineStr">
         <is>
-          <t>Cross-process lock — only one worker reconciles</t>
+          <t>Active mount preserved</t>
         </is>
       </c>
       <c r="D217" s="4" t="inlineStr">
         <is>
-          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
+          <t>Add and mount a network share (leave it mounted), restart the service</t>
         </is>
       </c>
       <c r="E217" s="4" t="inlineStr">
         <is>
-          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
+          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F217" s="4" t="n"/>
@@ -6861,7 +6861,7 @@
     <row r="218">
       <c r="A218" s="4" t="inlineStr">
         <is>
-          <t>TC-1111</t>
+          <t>TC-1107</t>
         </is>
       </c>
       <c r="B218" s="4" t="inlineStr">
@@ -6871,17 +6871,17 @@
       </c>
       <c r="C218" s="4" t="inlineStr">
         <is>
-          <t>Stale lock reclaim</t>
+          <t>USB drives re-discovered</t>
         </is>
       </c>
       <c r="D218" s="4" t="inlineStr">
         <is>
-          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
+          <t>Insert USB drives, restart the service</t>
         </is>
       </c>
       <c r="E218" s="4" t="inlineStr">
         <is>
-          <t>Service reclaims the stale lock, reconciliation runs normally</t>
+          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
         </is>
       </c>
       <c r="F218" s="4" t="n"/>
@@ -6892,7 +6892,7 @@
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
         <is>
-          <t>TC-1112</t>
+          <t>TC-1108</t>
         </is>
       </c>
       <c r="B219" s="4" t="inlineStr">
@@ -6902,17 +6902,17 @@
       </c>
       <c r="C219" s="4" t="inlineStr">
         <is>
-          <t>Lock released after failure</t>
+          <t>Idempotency</t>
         </is>
       </c>
       <c r="D219" s="4" t="inlineStr">
         <is>
-          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
+          <t>Restart the service twice without any state changes between restarts</t>
         </is>
       </c>
       <c r="E219" s="4" t="inlineStr">
         <is>
-          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
+          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
         </is>
       </c>
       <c r="F219" s="4" t="n"/>
@@ -6920,14 +6920,138 @@
       <c r="H219" s="4" t="n"/>
       <c r="I219" s="4" t="n"/>
     </row>
+    <row r="220">
+      <c r="A220" s="4" t="inlineStr">
+        <is>
+          <t>TC-1109</t>
+        </is>
+      </c>
+      <c r="B220" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C220" s="4" t="inlineStr">
+        <is>
+          <t>Partial failure isolation</t>
+        </is>
+      </c>
+      <c r="D220" s="4" t="inlineStr">
+        <is>
+          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
+        </is>
+      </c>
+      <c r="E220" s="4" t="inlineStr">
+        <is>
+          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
+        </is>
+      </c>
+      <c r="F220" s="4" t="n"/>
+      <c r="G220" s="4" t="n"/>
+      <c r="H220" s="4" t="n"/>
+      <c r="I220" s="4" t="n"/>
+    </row>
     <row r="221">
-      <c r="A221" s="5" t="inlineStr">
+      <c r="A221" s="4" t="inlineStr">
+        <is>
+          <t>TC-1110</t>
+        </is>
+      </c>
+      <c r="B221" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C221" s="4" t="inlineStr">
+        <is>
+          <t>Cross-process lock — only one worker reconciles</t>
+        </is>
+      </c>
+      <c r="D221" s="4" t="inlineStr">
+        <is>
+          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
+        </is>
+      </c>
+      <c r="E221" s="4" t="inlineStr">
+        <is>
+          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
+        </is>
+      </c>
+      <c r="F221" s="4" t="n"/>
+      <c r="G221" s="4" t="n"/>
+      <c r="H221" s="4" t="n"/>
+      <c r="I221" s="4" t="n"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="4" t="inlineStr">
+        <is>
+          <t>TC-1111</t>
+        </is>
+      </c>
+      <c r="B222" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C222" s="4" t="inlineStr">
+        <is>
+          <t>Stale lock reclaim</t>
+        </is>
+      </c>
+      <c r="D222" s="4" t="inlineStr">
+        <is>
+          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
+        </is>
+      </c>
+      <c r="E222" s="4" t="inlineStr">
+        <is>
+          <t>Service reclaims the stale lock, reconciliation runs normally</t>
+        </is>
+      </c>
+      <c r="F222" s="4" t="n"/>
+      <c r="G222" s="4" t="n"/>
+      <c r="H222" s="4" t="n"/>
+      <c r="I222" s="4" t="n"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="4" t="inlineStr">
+        <is>
+          <t>TC-1112</t>
+        </is>
+      </c>
+      <c r="B223" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C223" s="4" t="inlineStr">
+        <is>
+          <t>Lock released after failure</t>
+        </is>
+      </c>
+      <c r="D223" s="4" t="inlineStr">
+        <is>
+          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
+        </is>
+      </c>
+      <c r="E223" s="4" t="inlineStr">
+        <is>
+          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
+        </is>
+      </c>
+      <c r="F223" s="4" t="n"/>
+      <c r="G223" s="4" t="n"/>
+      <c r="H223" s="4" t="n"/>
+      <c r="I223" s="4" t="n"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B221" s="5" t="n">
-        <v>202</v>
+      <c r="B225" s="5" t="n">
+        <v>206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add CPU, memory, and disk I/O metrics to system health endpoint and update related documentation
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I227"/>
+  <dimension ref="A1:I238"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6714,12 +6714,12 @@
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>§12.11 Startup State Reconciliation</t>
+          <t>§12.12 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
         <is>
-          <t>12.11 Startup State Reconciliation</t>
+          <t>12.12 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C213" s="3" t="n"/>
@@ -6733,12 +6733,12 @@
     <row r="214">
       <c r="A214" s="4" t="inlineStr">
         <is>
-          <t>TC-1101</t>
+          <t>TC-1201</t>
         </is>
       </c>
       <c r="B214" s="4" t="inlineStr">
         <is>
-          <t>12.11 Startup State Reconciliation</t>
+          <t>12.12 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C214" s="4" t="inlineStr">
@@ -6764,12 +6764,12 @@
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
         <is>
-          <t>TC-1102</t>
+          <t>TC-1202</t>
         </is>
       </c>
       <c r="B215" s="4" t="inlineStr">
         <is>
-          <t>12.11 Startup State Reconciliation</t>
+          <t>12.12 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C215" s="4" t="inlineStr">
@@ -6795,12 +6795,12 @@
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
         <is>
-          <t>TC-1103</t>
+          <t>TC-1203</t>
         </is>
       </c>
       <c r="B216" s="4" t="inlineStr">
         <is>
-          <t>12.11 Startup State Reconciliation</t>
+          <t>12.12 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C216" s="4" t="inlineStr">
@@ -6826,12 +6826,12 @@
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
         <is>
-          <t>TC-1104</t>
+          <t>TC-1204</t>
         </is>
       </c>
       <c r="B217" s="4" t="inlineStr">
         <is>
-          <t>12.11 Startup State Reconciliation</t>
+          <t>12.12 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C217" s="4" t="inlineStr">
@@ -6855,60 +6855,48 @@
       <c r="I217" s="4" t="n"/>
     </row>
     <row r="218">
-      <c r="A218" s="4" t="inlineStr">
-        <is>
-          <t>TC-1105</t>
-        </is>
-      </c>
-      <c r="B218" s="4" t="inlineStr">
-        <is>
-          <t>12.11 Startup State Reconciliation</t>
-        </is>
-      </c>
-      <c r="C218" s="4" t="inlineStr">
-        <is>
-          <t>Stale mount corrected</t>
-        </is>
-      </c>
-      <c r="D218" s="4" t="inlineStr">
-        <is>
-          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
-        </is>
-      </c>
-      <c r="E218" s="4" t="inlineStr">
-        <is>
-          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
-        </is>
-      </c>
-      <c r="F218" s="4" t="n"/>
-      <c r="G218" s="4" t="n"/>
-      <c r="H218" s="4" t="n"/>
-      <c r="I218" s="4" t="n"/>
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>§12.13 System Health</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>12.13 System Health</t>
+        </is>
+      </c>
+      <c r="C218" s="3" t="n"/>
+      <c r="D218" s="3" t="n"/>
+      <c r="E218" s="3" t="n"/>
+      <c r="F218" s="3" t="n"/>
+      <c r="G218" s="3" t="n"/>
+      <c r="H218" s="3" t="n"/>
+      <c r="I218" s="3" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
         <is>
-          <t>TC-1106</t>
+          <t>TC-1301</t>
         </is>
       </c>
       <c r="B219" s="4" t="inlineStr">
         <is>
-          <t>12.11 Startup State Reconciliation</t>
+          <t>12.13 System Health</t>
         </is>
       </c>
       <c r="C219" s="4" t="inlineStr">
         <is>
-          <t>Active mount preserved</t>
+          <t>Healthy response</t>
         </is>
       </c>
       <c r="D219" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share (leave it mounted), restart the service</t>
+          <t>GET /introspection/system-health with valid token</t>
         </is>
       </c>
       <c r="E219" s="4" t="inlineStr">
         <is>
-          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
+          <t>200, status: "ok", database: "connected"</t>
         </is>
       </c>
       <c r="F219" s="4" t="n"/>
@@ -6919,27 +6907,27 @@
     <row r="220">
       <c r="A220" s="4" t="inlineStr">
         <is>
-          <t>TC-1107</t>
+          <t>TC-1302</t>
         </is>
       </c>
       <c r="B220" s="4" t="inlineStr">
         <is>
-          <t>12.11 Startup State Reconciliation</t>
+          <t>12.13 System Health</t>
         </is>
       </c>
       <c r="C220" s="4" t="inlineStr">
         <is>
-          <t>USB drives re-discovered</t>
+          <t>CPU metric present</t>
         </is>
       </c>
       <c r="D220" s="4" t="inlineStr">
         <is>
-          <t>Insert USB drives, restart the service</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
-          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
+          <t>cpu_percent is a number between 0 and 100</t>
         </is>
       </c>
       <c r="F220" s="4" t="n"/>
@@ -6950,27 +6938,27 @@
     <row r="221">
       <c r="A221" s="4" t="inlineStr">
         <is>
-          <t>TC-1108</t>
+          <t>TC-1303</t>
         </is>
       </c>
       <c r="B221" s="4" t="inlineStr">
         <is>
-          <t>12.11 Startup State Reconciliation</t>
+          <t>12.13 System Health</t>
         </is>
       </c>
       <c r="C221" s="4" t="inlineStr">
         <is>
-          <t>Idempotency</t>
+          <t>Memory metrics present</t>
         </is>
       </c>
       <c r="D221" s="4" t="inlineStr">
         <is>
-          <t>Restart the service twice without any state changes between restarts</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E221" s="4" t="inlineStr">
         <is>
-          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
+          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
         </is>
       </c>
       <c r="F221" s="4" t="n"/>
@@ -6981,27 +6969,27 @@
     <row r="222">
       <c r="A222" s="4" t="inlineStr">
         <is>
-          <t>TC-1109</t>
+          <t>TC-1304</t>
         </is>
       </c>
       <c r="B222" s="4" t="inlineStr">
         <is>
-          <t>12.11 Startup State Reconciliation</t>
+          <t>12.13 System Health</t>
         </is>
       </c>
       <c r="C222" s="4" t="inlineStr">
         <is>
-          <t>Partial failure isolation</t>
+          <t>Disk I/O metrics present</t>
         </is>
       </c>
       <c r="D222" s="4" t="inlineStr">
         <is>
-          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E222" s="4" t="inlineStr">
         <is>
-          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
+          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
         </is>
       </c>
       <c r="F222" s="4" t="n"/>
@@ -7012,27 +7000,27 @@
     <row r="223">
       <c r="A223" s="4" t="inlineStr">
         <is>
-          <t>TC-1110</t>
+          <t>TC-1305</t>
         </is>
       </c>
       <c r="B223" s="4" t="inlineStr">
         <is>
-          <t>12.11 Startup State Reconciliation</t>
+          <t>12.13 System Health</t>
         </is>
       </c>
       <c r="C223" s="4" t="inlineStr">
         <is>
-          <t>Cross-process lock — only one worker reconciles</t>
+          <t>Active jobs count</t>
         </is>
       </c>
       <c r="D223" s="4" t="inlineStr">
         <is>
-          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
+          <t>Start an export job, call endpoint</t>
         </is>
       </c>
       <c r="E223" s="4" t="inlineStr">
         <is>
-          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
+          <t>active_jobs ≥ 1</t>
         </is>
       </c>
       <c r="F223" s="4" t="n"/>
@@ -7043,27 +7031,27 @@
     <row r="224">
       <c r="A224" s="4" t="inlineStr">
         <is>
-          <t>TC-1111</t>
+          <t>TC-1306</t>
         </is>
       </c>
       <c r="B224" s="4" t="inlineStr">
         <is>
-          <t>12.11 Startup State Reconciliation</t>
+          <t>12.13 System Health</t>
         </is>
       </c>
       <c r="C224" s="4" t="inlineStr">
         <is>
-          <t>Stale lock reclaim</t>
+          <t>Worker queue size</t>
         </is>
       </c>
       <c r="D224" s="4" t="inlineStr">
         <is>
-          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
+          <t>Create a PENDING job (created but not started), call endpoint</t>
         </is>
       </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
-          <t>Service reclaims the stale lock, reconciliation runs normally</t>
+          <t>worker_queue_size ≥ 1</t>
         </is>
       </c>
       <c r="F224" s="4" t="n"/>
@@ -7074,27 +7062,27 @@
     <row r="225">
       <c r="A225" s="4" t="inlineStr">
         <is>
-          <t>TC-1112</t>
+          <t>TC-1307</t>
         </is>
       </c>
       <c r="B225" s="4" t="inlineStr">
         <is>
-          <t>12.11 Startup State Reconciliation</t>
+          <t>12.13 System Health</t>
         </is>
       </c>
       <c r="C225" s="4" t="inlineStr">
         <is>
-          <t>Lock released after failure</t>
+          <t>Worker queue size decrements</t>
         </is>
       </c>
       <c r="D225" s="4" t="inlineStr">
         <is>
-          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
+          <t>Start the pending job, call endpoint again</t>
         </is>
       </c>
       <c r="E225" s="4" t="inlineStr">
         <is>
-          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
+          <t>worker_queue_size is 0 (job moved to RUNNING)</t>
         </is>
       </c>
       <c r="F225" s="4" t="n"/>
@@ -7102,14 +7090,355 @@
       <c r="H225" s="4" t="n"/>
       <c r="I225" s="4" t="n"/>
     </row>
+    <row r="226">
+      <c r="A226" s="4" t="inlineStr">
+        <is>
+          <t>TC-1308</t>
+        </is>
+      </c>
+      <c r="B226" s="4" t="inlineStr">
+        <is>
+          <t>12.13 System Health</t>
+        </is>
+      </c>
+      <c r="C226" s="4" t="inlineStr">
+        <is>
+          <t>Degraded when DB down</t>
+        </is>
+      </c>
+      <c r="D226" s="4" t="inlineStr">
+        <is>
+          <t>Stop PostgreSQL, call endpoint with valid token</t>
+        </is>
+      </c>
+      <c r="E226" s="4" t="inlineStr">
+        <is>
+          <t>200, status: "degraded", database: "error", database_error is non-null</t>
+        </is>
+      </c>
+      <c r="F226" s="4" t="n"/>
+      <c r="G226" s="4" t="n"/>
+      <c r="H226" s="4" t="n"/>
+      <c r="I226" s="4" t="n"/>
+    </row>
     <row r="227">
-      <c r="A227" s="5" t="inlineStr">
+      <c r="A227" s="4" t="inlineStr">
+        <is>
+          <t>TC-1309</t>
+        </is>
+      </c>
+      <c r="B227" s="4" t="inlineStr">
+        <is>
+          <t>12.13 System Health</t>
+        </is>
+      </c>
+      <c r="C227" s="4" t="inlineStr">
+        <is>
+          <t>Unauthenticated rejected</t>
+        </is>
+      </c>
+      <c r="D227" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/system-health without token</t>
+        </is>
+      </c>
+      <c r="E227" s="4" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="F227" s="4" t="n"/>
+      <c r="G227" s="4" t="n"/>
+      <c r="H227" s="4" t="n"/>
+      <c r="I227" s="4" t="n"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="4" t="inlineStr">
+        <is>
+          <t>TC-1310</t>
+        </is>
+      </c>
+      <c r="B228" s="4" t="inlineStr">
+        <is>
+          <t>12.13 System Health</t>
+        </is>
+      </c>
+      <c r="C228" s="4" t="inlineStr">
+        <is>
+          <t>Processor role allowed</t>
+        </is>
+      </c>
+      <c r="D228" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/system-health with processor token</t>
+        </is>
+      </c>
+      <c r="E228" s="4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F228" s="4" t="n"/>
+      <c r="G228" s="4" t="n"/>
+      <c r="H228" s="4" t="n"/>
+      <c r="I228" s="4" t="n"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="4" t="inlineStr">
+        <is>
+          <t>TC-1305</t>
+        </is>
+      </c>
+      <c r="B229" s="4" t="inlineStr">
+        <is>
+          <t>12.13 System Health</t>
+        </is>
+      </c>
+      <c r="C229" s="4" t="inlineStr">
+        <is>
+          <t>Stale mount corrected</t>
+        </is>
+      </c>
+      <c r="D229" s="4" t="inlineStr">
+        <is>
+          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
+        </is>
+      </c>
+      <c r="E229" s="4" t="inlineStr">
+        <is>
+          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
+        </is>
+      </c>
+      <c r="F229" s="4" t="n"/>
+      <c r="G229" s="4" t="n"/>
+      <c r="H229" s="4" t="n"/>
+      <c r="I229" s="4" t="n"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="4" t="inlineStr">
+        <is>
+          <t>TC-1306</t>
+        </is>
+      </c>
+      <c r="B230" s="4" t="inlineStr">
+        <is>
+          <t>12.13 System Health</t>
+        </is>
+      </c>
+      <c r="C230" s="4" t="inlineStr">
+        <is>
+          <t>Active mount preserved</t>
+        </is>
+      </c>
+      <c r="D230" s="4" t="inlineStr">
+        <is>
+          <t>Add and mount a network share (leave it mounted), restart the service</t>
+        </is>
+      </c>
+      <c r="E230" s="4" t="inlineStr">
+        <is>
+          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
+        </is>
+      </c>
+      <c r="F230" s="4" t="n"/>
+      <c r="G230" s="4" t="n"/>
+      <c r="H230" s="4" t="n"/>
+      <c r="I230" s="4" t="n"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="4" t="inlineStr">
+        <is>
+          <t>TC-1307</t>
+        </is>
+      </c>
+      <c r="B231" s="4" t="inlineStr">
+        <is>
+          <t>12.13 System Health</t>
+        </is>
+      </c>
+      <c r="C231" s="4" t="inlineStr">
+        <is>
+          <t>USB drives re-discovered</t>
+        </is>
+      </c>
+      <c r="D231" s="4" t="inlineStr">
+        <is>
+          <t>Insert USB drives, restart the service</t>
+        </is>
+      </c>
+      <c r="E231" s="4" t="inlineStr">
+        <is>
+          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
+        </is>
+      </c>
+      <c r="F231" s="4" t="n"/>
+      <c r="G231" s="4" t="n"/>
+      <c r="H231" s="4" t="n"/>
+      <c r="I231" s="4" t="n"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="4" t="inlineStr">
+        <is>
+          <t>TC-1308</t>
+        </is>
+      </c>
+      <c r="B232" s="4" t="inlineStr">
+        <is>
+          <t>12.13 System Health</t>
+        </is>
+      </c>
+      <c r="C232" s="4" t="inlineStr">
+        <is>
+          <t>Idempotency</t>
+        </is>
+      </c>
+      <c r="D232" s="4" t="inlineStr">
+        <is>
+          <t>Restart the service twice without any state changes between restarts</t>
+        </is>
+      </c>
+      <c r="E232" s="4" t="inlineStr">
+        <is>
+          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
+        </is>
+      </c>
+      <c r="F232" s="4" t="n"/>
+      <c r="G232" s="4" t="n"/>
+      <c r="H232" s="4" t="n"/>
+      <c r="I232" s="4" t="n"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="4" t="inlineStr">
+        <is>
+          <t>TC-1309</t>
+        </is>
+      </c>
+      <c r="B233" s="4" t="inlineStr">
+        <is>
+          <t>12.13 System Health</t>
+        </is>
+      </c>
+      <c r="C233" s="4" t="inlineStr">
+        <is>
+          <t>Partial failure isolation</t>
+        </is>
+      </c>
+      <c r="D233" s="4" t="inlineStr">
+        <is>
+          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
+        </is>
+      </c>
+      <c r="E233" s="4" t="inlineStr">
+        <is>
+          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
+        </is>
+      </c>
+      <c r="F233" s="4" t="n"/>
+      <c r="G233" s="4" t="n"/>
+      <c r="H233" s="4" t="n"/>
+      <c r="I233" s="4" t="n"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="4" t="inlineStr">
+        <is>
+          <t>TC-1310</t>
+        </is>
+      </c>
+      <c r="B234" s="4" t="inlineStr">
+        <is>
+          <t>12.13 System Health</t>
+        </is>
+      </c>
+      <c r="C234" s="4" t="inlineStr">
+        <is>
+          <t>Cross-process lock — only one worker reconciles</t>
+        </is>
+      </c>
+      <c r="D234" s="4" t="inlineStr">
+        <is>
+          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
+        </is>
+      </c>
+      <c r="E234" s="4" t="inlineStr">
+        <is>
+          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
+        </is>
+      </c>
+      <c r="F234" s="4" t="n"/>
+      <c r="G234" s="4" t="n"/>
+      <c r="H234" s="4" t="n"/>
+      <c r="I234" s="4" t="n"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="4" t="inlineStr">
+        <is>
+          <t>TC-1311</t>
+        </is>
+      </c>
+      <c r="B235" s="4" t="inlineStr">
+        <is>
+          <t>12.13 System Health</t>
+        </is>
+      </c>
+      <c r="C235" s="4" t="inlineStr">
+        <is>
+          <t>Stale lock reclaim</t>
+        </is>
+      </c>
+      <c r="D235" s="4" t="inlineStr">
+        <is>
+          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
+        </is>
+      </c>
+      <c r="E235" s="4" t="inlineStr">
+        <is>
+          <t>Service reclaims the stale lock, reconciliation runs normally</t>
+        </is>
+      </c>
+      <c r="F235" s="4" t="n"/>
+      <c r="G235" s="4" t="n"/>
+      <c r="H235" s="4" t="n"/>
+      <c r="I235" s="4" t="n"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="4" t="inlineStr">
+        <is>
+          <t>TC-1312</t>
+        </is>
+      </c>
+      <c r="B236" s="4" t="inlineStr">
+        <is>
+          <t>12.13 System Health</t>
+        </is>
+      </c>
+      <c r="C236" s="4" t="inlineStr">
+        <is>
+          <t>Lock released after failure</t>
+        </is>
+      </c>
+      <c r="D236" s="4" t="inlineStr">
+        <is>
+          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
+        </is>
+      </c>
+      <c r="E236" s="4" t="inlineStr">
+        <is>
+          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
+        </is>
+      </c>
+      <c r="F236" s="4" t="n"/>
+      <c r="G236" s="4" t="n"/>
+      <c r="H236" s="4" t="n"/>
+      <c r="I236" s="4" t="n"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B227" s="5" t="n">
-        <v>208</v>
+      <c r="B238" s="5" t="n">
+        <v>218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update QA test cases spreadsheet with new scenarios
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -6855,48 +6855,60 @@
       <c r="I217" s="4" t="n"/>
     </row>
     <row r="218">
-      <c r="A218" s="2" t="inlineStr">
-        <is>
-          <t>§12.13 System Health</t>
-        </is>
-      </c>
-      <c r="B218" s="2" t="inlineStr">
-        <is>
-          <t>12.13 System Health</t>
-        </is>
-      </c>
-      <c r="C218" s="3" t="n"/>
-      <c r="D218" s="3" t="n"/>
-      <c r="E218" s="3" t="n"/>
-      <c r="F218" s="3" t="n"/>
-      <c r="G218" s="3" t="n"/>
-      <c r="H218" s="3" t="n"/>
-      <c r="I218" s="3" t="n"/>
+      <c r="A218" s="4" t="inlineStr">
+        <is>
+          <t>TC-1205</t>
+        </is>
+      </c>
+      <c r="B218" s="4" t="inlineStr">
+        <is>
+          <t>12.12 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C218" s="4" t="inlineStr">
+        <is>
+          <t>Stale mount corrected</t>
+        </is>
+      </c>
+      <c r="D218" s="4" t="inlineStr">
+        <is>
+          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
+        </is>
+      </c>
+      <c r="E218" s="4" t="inlineStr">
+        <is>
+          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
+        </is>
+      </c>
+      <c r="F218" s="4" t="n"/>
+      <c r="G218" s="4" t="n"/>
+      <c r="H218" s="4" t="n"/>
+      <c r="I218" s="4" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
         <is>
-          <t>TC-1301</t>
+          <t>TC-1206</t>
         </is>
       </c>
       <c r="B219" s="4" t="inlineStr">
         <is>
-          <t>12.13 System Health</t>
+          <t>12.12 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C219" s="4" t="inlineStr">
         <is>
-          <t>Healthy response</t>
+          <t>Active mount preserved</t>
         </is>
       </c>
       <c r="D219" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with valid token</t>
+          <t>Add and mount a network share (leave it mounted), restart the service</t>
         </is>
       </c>
       <c r="E219" s="4" t="inlineStr">
         <is>
-          <t>200, status: "ok", database: "connected"</t>
+          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F219" s="4" t="n"/>
@@ -6907,27 +6919,27 @@
     <row r="220">
       <c r="A220" s="4" t="inlineStr">
         <is>
-          <t>TC-1302</t>
+          <t>TC-1207</t>
         </is>
       </c>
       <c r="B220" s="4" t="inlineStr">
         <is>
-          <t>12.13 System Health</t>
+          <t>12.12 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C220" s="4" t="inlineStr">
         <is>
-          <t>CPU metric present</t>
+          <t>USB drives re-discovered</t>
         </is>
       </c>
       <c r="D220" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Insert USB drives, restart the service</t>
         </is>
       </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
-          <t>cpu_percent is a number between 0 and 100</t>
+          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
         </is>
       </c>
       <c r="F220" s="4" t="n"/>
@@ -6938,27 +6950,27 @@
     <row r="221">
       <c r="A221" s="4" t="inlineStr">
         <is>
-          <t>TC-1303</t>
+          <t>TC-1208</t>
         </is>
       </c>
       <c r="B221" s="4" t="inlineStr">
         <is>
-          <t>12.13 System Health</t>
+          <t>12.12 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C221" s="4" t="inlineStr">
         <is>
-          <t>Memory metrics present</t>
+          <t>Idempotency</t>
         </is>
       </c>
       <c r="D221" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Restart the service twice without any state changes between restarts</t>
         </is>
       </c>
       <c r="E221" s="4" t="inlineStr">
         <is>
-          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
+          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
         </is>
       </c>
       <c r="F221" s="4" t="n"/>
@@ -6969,27 +6981,27 @@
     <row r="222">
       <c r="A222" s="4" t="inlineStr">
         <is>
-          <t>TC-1304</t>
+          <t>TC-1209</t>
         </is>
       </c>
       <c r="B222" s="4" t="inlineStr">
         <is>
-          <t>12.13 System Health</t>
+          <t>12.12 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C222" s="4" t="inlineStr">
         <is>
-          <t>Disk I/O metrics present</t>
+          <t>Partial failure isolation</t>
         </is>
       </c>
       <c r="D222" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
         </is>
       </c>
       <c r="E222" s="4" t="inlineStr">
         <is>
-          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
+          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
         </is>
       </c>
       <c r="F222" s="4" t="n"/>
@@ -7000,27 +7012,27 @@
     <row r="223">
       <c r="A223" s="4" t="inlineStr">
         <is>
-          <t>TC-1305</t>
+          <t>TC-1210</t>
         </is>
       </c>
       <c r="B223" s="4" t="inlineStr">
         <is>
-          <t>12.13 System Health</t>
+          <t>12.12 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C223" s="4" t="inlineStr">
         <is>
-          <t>Active jobs count</t>
+          <t>Cross-process lock — only one worker reconciles</t>
         </is>
       </c>
       <c r="D223" s="4" t="inlineStr">
         <is>
-          <t>Start an export job, call endpoint</t>
+          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
         </is>
       </c>
       <c r="E223" s="4" t="inlineStr">
         <is>
-          <t>active_jobs ≥ 1</t>
+          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
         </is>
       </c>
       <c r="F223" s="4" t="n"/>
@@ -7031,27 +7043,27 @@
     <row r="224">
       <c r="A224" s="4" t="inlineStr">
         <is>
-          <t>TC-1306</t>
+          <t>TC-1211</t>
         </is>
       </c>
       <c r="B224" s="4" t="inlineStr">
         <is>
-          <t>12.13 System Health</t>
+          <t>12.12 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C224" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size</t>
+          <t>Stale lock reclaim</t>
         </is>
       </c>
       <c r="D224" s="4" t="inlineStr">
         <is>
-          <t>Create a PENDING job (created but not started), call endpoint</t>
+          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
         </is>
       </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size ≥ 1</t>
+          <t>Service reclaims the stale lock, reconciliation runs normally</t>
         </is>
       </c>
       <c r="F224" s="4" t="n"/>
@@ -7062,27 +7074,27 @@
     <row r="225">
       <c r="A225" s="4" t="inlineStr">
         <is>
-          <t>TC-1307</t>
+          <t>TC-1212</t>
         </is>
       </c>
       <c r="B225" s="4" t="inlineStr">
         <is>
-          <t>12.13 System Health</t>
+          <t>12.12 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C225" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size decrements</t>
+          <t>Lock released after failure</t>
         </is>
       </c>
       <c r="D225" s="4" t="inlineStr">
         <is>
-          <t>Start the pending job, call endpoint again</t>
+          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
         </is>
       </c>
       <c r="E225" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size is 0 (job moved to RUNNING)</t>
+          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
         </is>
       </c>
       <c r="F225" s="4" t="n"/>
@@ -7091,40 +7103,28 @@
       <c r="I225" s="4" t="n"/>
     </row>
     <row r="226">
-      <c r="A226" s="4" t="inlineStr">
-        <is>
-          <t>TC-1308</t>
-        </is>
-      </c>
-      <c r="B226" s="4" t="inlineStr">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>§12.13 System Health</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
         <is>
           <t>12.13 System Health</t>
         </is>
       </c>
-      <c r="C226" s="4" t="inlineStr">
-        <is>
-          <t>Degraded when DB down</t>
-        </is>
-      </c>
-      <c r="D226" s="4" t="inlineStr">
-        <is>
-          <t>Stop PostgreSQL, call endpoint with valid token</t>
-        </is>
-      </c>
-      <c r="E226" s="4" t="inlineStr">
-        <is>
-          <t>200, status: "degraded", database: "error", database_error is non-null</t>
-        </is>
-      </c>
-      <c r="F226" s="4" t="n"/>
-      <c r="G226" s="4" t="n"/>
-      <c r="H226" s="4" t="n"/>
-      <c r="I226" s="4" t="n"/>
+      <c r="C226" s="3" t="n"/>
+      <c r="D226" s="3" t="n"/>
+      <c r="E226" s="3" t="n"/>
+      <c r="F226" s="3" t="n"/>
+      <c r="G226" s="3" t="n"/>
+      <c r="H226" s="3" t="n"/>
+      <c r="I226" s="3" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="4" t="inlineStr">
         <is>
-          <t>TC-1309</t>
+          <t>TC-1301</t>
         </is>
       </c>
       <c r="B227" s="4" t="inlineStr">
@@ -7134,17 +7134,17 @@
       </c>
       <c r="C227" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated rejected</t>
+          <t>Healthy response</t>
         </is>
       </c>
       <c r="D227" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health without token</t>
+          <t>GET /introspection/system-health with valid token</t>
         </is>
       </c>
       <c r="E227" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>200, status: "ok", database: "connected"</t>
         </is>
       </c>
       <c r="F227" s="4" t="n"/>
@@ -7155,7 +7155,7 @@
     <row r="228">
       <c r="A228" s="4" t="inlineStr">
         <is>
-          <t>TC-1310</t>
+          <t>TC-1302</t>
         </is>
       </c>
       <c r="B228" s="4" t="inlineStr">
@@ -7165,17 +7165,17 @@
       </c>
       <c r="C228" s="4" t="inlineStr">
         <is>
-          <t>Processor role allowed</t>
+          <t>CPU metric present</t>
         </is>
       </c>
       <c r="D228" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with processor token</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>cpu_percent is a number between 0 and 100</t>
         </is>
       </c>
       <c r="F228" s="4" t="n"/>
@@ -7186,7 +7186,7 @@
     <row r="229">
       <c r="A229" s="4" t="inlineStr">
         <is>
-          <t>TC-1305</t>
+          <t>TC-1303</t>
         </is>
       </c>
       <c r="B229" s="4" t="inlineStr">
@@ -7196,17 +7196,17 @@
       </c>
       <c r="C229" s="4" t="inlineStr">
         <is>
-          <t>Stale mount corrected</t>
+          <t>Memory metrics present</t>
         </is>
       </c>
       <c r="D229" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E229" s="4" t="inlineStr">
         <is>
-          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
+          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
         </is>
       </c>
       <c r="F229" s="4" t="n"/>
@@ -7217,7 +7217,7 @@
     <row r="230">
       <c r="A230" s="4" t="inlineStr">
         <is>
-          <t>TC-1306</t>
+          <t>TC-1304</t>
         </is>
       </c>
       <c r="B230" s="4" t="inlineStr">
@@ -7227,17 +7227,17 @@
       </c>
       <c r="C230" s="4" t="inlineStr">
         <is>
-          <t>Active mount preserved</t>
+          <t>Disk I/O metrics present</t>
         </is>
       </c>
       <c r="D230" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share (leave it mounted), restart the service</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E230" s="4" t="inlineStr">
         <is>
-          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
+          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
         </is>
       </c>
       <c r="F230" s="4" t="n"/>
@@ -7248,7 +7248,7 @@
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
         <is>
-          <t>TC-1307</t>
+          <t>TC-1305</t>
         </is>
       </c>
       <c r="B231" s="4" t="inlineStr">
@@ -7258,17 +7258,17 @@
       </c>
       <c r="C231" s="4" t="inlineStr">
         <is>
-          <t>USB drives re-discovered</t>
+          <t>Active jobs count</t>
         </is>
       </c>
       <c r="D231" s="4" t="inlineStr">
         <is>
-          <t>Insert USB drives, restart the service</t>
+          <t>Start an export job, call endpoint</t>
         </is>
       </c>
       <c r="E231" s="4" t="inlineStr">
         <is>
-          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
+          <t>active_jobs ≥ 1</t>
         </is>
       </c>
       <c r="F231" s="4" t="n"/>
@@ -7279,7 +7279,7 @@
     <row r="232">
       <c r="A232" s="4" t="inlineStr">
         <is>
-          <t>TC-1308</t>
+          <t>TC-1306</t>
         </is>
       </c>
       <c r="B232" s="4" t="inlineStr">
@@ -7289,17 +7289,17 @@
       </c>
       <c r="C232" s="4" t="inlineStr">
         <is>
-          <t>Idempotency</t>
+          <t>Worker queue size</t>
         </is>
       </c>
       <c r="D232" s="4" t="inlineStr">
         <is>
-          <t>Restart the service twice without any state changes between restarts</t>
+          <t>Create a PENDING job (created but not started), call endpoint</t>
         </is>
       </c>
       <c r="E232" s="4" t="inlineStr">
         <is>
-          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
+          <t>worker_queue_size ≥ 1</t>
         </is>
       </c>
       <c r="F232" s="4" t="n"/>
@@ -7310,7 +7310,7 @@
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
         <is>
-          <t>TC-1309</t>
+          <t>TC-1307</t>
         </is>
       </c>
       <c r="B233" s="4" t="inlineStr">
@@ -7320,17 +7320,17 @@
       </c>
       <c r="C233" s="4" t="inlineStr">
         <is>
-          <t>Partial failure isolation</t>
+          <t>Worker queue size decrements</t>
         </is>
       </c>
       <c r="D233" s="4" t="inlineStr">
         <is>
-          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
+          <t>Start the pending job, call endpoint again</t>
         </is>
       </c>
       <c r="E233" s="4" t="inlineStr">
         <is>
-          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
+          <t>worker_queue_size is 0 (job moved to RUNNING)</t>
         </is>
       </c>
       <c r="F233" s="4" t="n"/>
@@ -7341,7 +7341,7 @@
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
         <is>
-          <t>TC-1310</t>
+          <t>TC-1308</t>
         </is>
       </c>
       <c r="B234" s="4" t="inlineStr">
@@ -7351,17 +7351,17 @@
       </c>
       <c r="C234" s="4" t="inlineStr">
         <is>
-          <t>Cross-process lock — only one worker reconciles</t>
+          <t>Degraded when DB down</t>
         </is>
       </c>
       <c r="D234" s="4" t="inlineStr">
         <is>
-          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
+          <t>Stop PostgreSQL, call endpoint with valid token</t>
         </is>
       </c>
       <c r="E234" s="4" t="inlineStr">
         <is>
-          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
+          <t>200, status: "degraded", database: "error", database_error is non-null</t>
         </is>
       </c>
       <c r="F234" s="4" t="n"/>
@@ -7372,7 +7372,7 @@
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
         <is>
-          <t>TC-1311</t>
+          <t>TC-1309</t>
         </is>
       </c>
       <c r="B235" s="4" t="inlineStr">
@@ -7382,17 +7382,17 @@
       </c>
       <c r="C235" s="4" t="inlineStr">
         <is>
-          <t>Stale lock reclaim</t>
+          <t>Unauthenticated rejected</t>
         </is>
       </c>
       <c r="D235" s="4" t="inlineStr">
         <is>
-          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
+          <t>GET /introspection/system-health without token</t>
         </is>
       </c>
       <c r="E235" s="4" t="inlineStr">
         <is>
-          <t>Service reclaims the stale lock, reconciliation runs normally</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F235" s="4" t="n"/>
@@ -7403,7 +7403,7 @@
     <row r="236">
       <c r="A236" s="4" t="inlineStr">
         <is>
-          <t>TC-1312</t>
+          <t>TC-1310</t>
         </is>
       </c>
       <c r="B236" s="4" t="inlineStr">
@@ -7413,17 +7413,17 @@
       </c>
       <c r="C236" s="4" t="inlineStr">
         <is>
-          <t>Lock released after failure</t>
+          <t>Processor role allowed</t>
         </is>
       </c>
       <c r="D236" s="4" t="inlineStr">
         <is>
-          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
+          <t>GET /introspection/system-health with processor token</t>
         </is>
       </c>
       <c r="E236" s="4" t="inlineStr">
         <is>
-          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F236" s="4" t="n"/>

</xml_diff>

<commit_message>
Update API documentation to exclude reserved system accounts from OS user listings and add username search filter
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -1050,7 +1050,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>POST /drives/{id}/initialize with processor token</t>
+          <t>POST /drives/{drive_id}/initialize with processor token</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>POST /drives/{id}/format with processor token</t>
+          <t>POST /drives/{drive_id}/format with processor token</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{id}/files with admin/manager/processor/auditor tokens</t>
+          <t>GET /jobs/{job_id}/files with admin/manager/processor/auditor tokens</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>PATCH /admin/ports/{id} with {"enabled": true}</t>
+          <t>PATCH /admin/ports/{port_id} with {"enabled": true}</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
@@ -2300,7 +2300,7 @@
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>PATCH /admin/ports/{id} with {"enabled": false}</t>
+          <t>PATCH /admin/ports/{port_id} with {"enabled": false}</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
@@ -2331,7 +2331,7 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>PATCH /admin/ports/{id} with manager token</t>
+          <t>PATCH /admin/ports/{port_id} with manager token</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>PATCH /admin/ports/{id} with processor token</t>
+          <t>PATCH /admin/ports/{port_id} with processor token</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
@@ -2815,7 +2815,7 @@
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>PATCH /admin/hubs/{id} with {"location_hint": "back-left rack"}</t>
+          <t>PATCH /admin/hubs/{hub_id} with {"location_hint": "back-left rack"}</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
@@ -2846,7 +2846,7 @@
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>PATCH /admin/hubs/{id} with manager token</t>
+          <t>PATCH /admin/hubs/{hub_id} with manager token</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
@@ -2877,7 +2877,7 @@
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>PATCH /admin/hubs/{id} with processor token</t>
+          <t>PATCH /admin/hubs/{hub_id} with processor token</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>PATCH /admin/ports/{id}/label with {"friendly_label": "Bay 3"}</t>
+          <t>PATCH /admin/ports/{port_id}/label with {"friendly_label": "Bay 3"}</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>PATCH /admin/ports/{id}/label with manager token</t>
+          <t>PATCH /admin/ports/{port_id}/label with manager token</t>
         </is>
       </c>
       <c r="E89" s="4" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>PATCH /admin/ports/{id}/label with processor token</t>
+          <t>PATCH /admin/ports/{port_id}/label with processor token</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
@@ -3063,7 +3063,7 @@
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>PATCH /admin/ports/{id}/label for non-existent port</t>
+          <t>PATCH /admin/ports/{port_id}/label for non-existent port</t>
         </is>
       </c>
       <c r="E91" s="4" t="inlineStr">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>POST /drives/{id}/format with {"filesystem_type": "ntfs"}</t>
+          <t>POST /drives/{drive_id}/format with {"filesystem_type": "ntfs"}</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr"/>
@@ -3707,7 +3707,7 @@
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>POST /drives/{id}/format with empty body</t>
+          <t>POST /drives/{drive_id}/format with empty body</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Enhance API documentation for admin log endpoints and update QA testing guide with new log viewing tests
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I238"/>
+  <dimension ref="A1:I255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5312,12 +5312,12 @@
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>§12.10 First-Run Setup</t>
+          <t>§12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C167" s="3" t="n"/>
@@ -5336,22 +5336,22 @@
       </c>
       <c r="B168" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
-          <t>Status — not initialized</t>
+          <t>View logs — unauthenticated</t>
         </is>
       </c>
       <c r="D168" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/status on fresh database</t>
+          <t>GET /admin/logs/view without token</t>
         </is>
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>200, {"initialized": false}</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F168" s="4" t="n"/>
@@ -5367,22 +5367,22 @@
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>Initialize</t>
+          <t>View logs — non-admin denied</t>
         </is>
       </c>
       <c r="D169" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with valid username and password</t>
+          <t>GET /admin/logs/view with manager/processor/auditor token</t>
         </is>
       </c>
       <c r="E169" s="4" t="inlineStr">
         <is>
-          <t>200, returns message, username, groups_created</t>
+          <t>403, FORBIDDEN; denied audit event recorded</t>
         </is>
       </c>
       <c r="F169" s="4" t="n"/>
@@ -5398,22 +5398,22 @@
       </c>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C170" s="4" t="inlineStr">
         <is>
-          <t>Status — initialized</t>
+          <t>View logs — unknown source</t>
         </is>
       </c>
       <c r="D170" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/status after initialization</t>
+          <t>GET /admin/logs/view?source=unknown with admin token</t>
         </is>
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>200, {"initialized": true}</t>
+          <t>404, unknown log source</t>
         </is>
       </c>
       <c r="F170" s="4" t="n"/>
@@ -5429,22 +5429,22 @@
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C171" s="4" t="inlineStr">
         <is>
-          <t>Re-initialize rejected</t>
+          <t>View logs — baseline response shape</t>
         </is>
       </c>
       <c r="D171" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize again</t>
+          <t>GET /admin/logs/view?source=app&amp;limit=5&amp;offset=0</t>
         </is>
       </c>
       <c r="E171" s="4" t="inlineStr">
         <is>
-          <t>409, Conflict</t>
+          <t>200 with object fields: source, fetched_at, file_modified_at, offset, limit, returned, has_more, lines</t>
         </is>
       </c>
       <c r="F171" s="4" t="n"/>
@@ -5460,22 +5460,22 @@
       </c>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C172" s="4" t="inlineStr">
         <is>
-          <t>Invalid username</t>
+          <t>View logs — source path redaction</t>
         </is>
       </c>
       <c r="D172" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with uppercase or special chars</t>
+          <t>Inspect source.path in successful response</t>
         </is>
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>Basename only (for example app.log), no absolute filesystem path</t>
         </is>
       </c>
       <c r="F172" s="4" t="n"/>
@@ -5491,22 +5491,22 @@
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C173" s="4" t="inlineStr">
         <is>
-          <t>Empty password</t>
+          <t>View logs — offset pagination</t>
         </is>
       </c>
       <c r="D173" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with {"password": ""}</t>
+          <t>Create known numbered lines, call GET /admin/logs/view?limit=5&amp;offset=2</t>
         </is>
       </c>
       <c r="E173" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>Returns correct window from tail semantics, returned &lt;= limit</t>
         </is>
       </c>
       <c r="F173" s="4" t="n"/>
@@ -5522,22 +5522,22 @@
       </c>
       <c r="B174" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C174" s="4" t="inlineStr">
         <is>
-          <t>Unsafe password chars</t>
+          <t>View logs — reverse ordering</t>
         </is>
       </c>
       <c r="D174" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with password containing newline or colon</t>
+          <t>Compare reverse=false vs reverse=true on same query</t>
         </is>
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>Same selected window; line order is inverted when reverse=true</t>
         </is>
       </c>
       <c r="F174" s="4" t="n"/>
@@ -5553,22 +5553,22 @@
       </c>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C175" s="4" t="inlineStr">
         <is>
-          <t>Login as initialized admin</t>
+          <t>View logs — search filtering</t>
         </is>
       </c>
       <c r="D175" s="4" t="inlineStr">
         <is>
-          <t>POST /auth/token with the admin credentials from step 2</t>
+          <t>GET /admin/logs/view?search=error</t>
         </is>
       </c>
       <c r="E175" s="4" t="inlineStr">
         <is>
-          <t>200, JWT contains admin role</t>
+          <t>Only matching lines are returned (case-insensitive contains)</t>
         </is>
       </c>
       <c r="F175" s="4" t="n"/>
@@ -5584,22 +5584,22 @@
       </c>
       <c r="B176" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C176" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM_INITIALIZED audit log</t>
+          <t>View logs — sensitive value redaction</t>
         </is>
       </c>
       <c r="D176" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
+          <t>Include tokens/passwords in source log lines, call view endpoint</t>
         </is>
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor</t>
+          <t>Sensitive values replaced with redacted markers in lines[].content</t>
         </is>
       </c>
       <c r="F176" s="4" t="n"/>
@@ -5608,48 +5608,60 @@
       <c r="I176" s="4" t="n"/>
     </row>
     <row r="177">
-      <c r="A177" s="2" t="inlineStr">
-        <is>
-          <t>§12.11 Database Provisioning</t>
-        </is>
-      </c>
-      <c r="B177" s="2" t="inlineStr">
-        <is>
-          <t>12.11 Database Provisioning</t>
-        </is>
-      </c>
-      <c r="C177" s="3" t="n"/>
-      <c r="D177" s="3" t="n"/>
-      <c r="E177" s="3" t="n"/>
-      <c r="F177" s="3" t="n"/>
-      <c r="G177" s="3" t="n"/>
-      <c r="H177" s="3" t="n"/>
-      <c r="I177" s="3" t="n"/>
+      <c r="A177" s="4" t="inlineStr">
+        <is>
+          <t>TC-1010</t>
+        </is>
+      </c>
+      <c r="B177" s="4" t="inlineStr">
+        <is>
+          <t>12.10 Admin Log Viewing API</t>
+        </is>
+      </c>
+      <c r="C177" s="4" t="inlineStr">
+        <is>
+          <t>View logs — success audit</t>
+        </is>
+      </c>
+      <c r="D177" s="4" t="inlineStr">
+        <is>
+          <t>GET /audit?action=LOG_LINES_VIEWED after successful view</t>
+        </is>
+      </c>
+      <c r="E177" s="4" t="inlineStr">
+        <is>
+          <t>Audit entry includes source, limit, offset, returned, has_more, and basename log_file</t>
+        </is>
+      </c>
+      <c r="F177" s="4" t="n"/>
+      <c r="G177" s="4" t="n"/>
+      <c r="H177" s="4" t="n"/>
+      <c r="I177" s="4" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>TC-1101</t>
+          <t>TC-1011</t>
         </is>
       </c>
       <c r="B178" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C178" s="4" t="inlineStr">
         <is>
-          <t>System info — bare-metal defaults</t>
+          <t>List logs — unauthenticated</t>
         </is>
       </c>
       <c r="D178" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/system-info before setup</t>
+          <t>GET /admin/logs without token</t>
         </is>
       </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
-          <t>200, {"in_docker": false, "suggested_db_host": "localhost"}</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F178" s="4" t="n"/>
@@ -5660,27 +5672,27 @@
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>TC-1102</t>
+          <t>TC-1012</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C179" s="4" t="inlineStr">
         <is>
-          <t>Provision status — pre-init public</t>
+          <t>List logs — non-admin denied</t>
         </is>
       </c>
       <c r="D179" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/provision-status before any admin exists</t>
+          <t>GET /admin/logs with non-admin token</t>
         </is>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>200, {"provisioned": false}</t>
+          <t>403, FORBIDDEN; denied audit event recorded</t>
         </is>
       </c>
       <c r="F179" s="4" t="n"/>
@@ -5691,27 +5703,27 @@
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>TC-1103</t>
+          <t>TC-1013</t>
         </is>
       </c>
       <c r="B180" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C180" s="4" t="inlineStr">
         <is>
-          <t>Provision status — post-init requires admin</t>
+          <t>List logs — response envelope</t>
         </is>
       </c>
       <c r="D180" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/provision-status without token after setup</t>
+          <t>GET /admin/logs with admin token and file logging configured</t>
         </is>
       </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>200 object with log_files array, total_size, and log_directory</t>
         </is>
       </c>
       <c r="F180" s="4" t="n"/>
@@ -5722,27 +5734,27 @@
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>TC-1104</t>
+          <t>TC-1014</t>
         </is>
       </c>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C181" s="4" t="inlineStr">
         <is>
-          <t>Provision status — state unknown</t>
+          <t>Download log — non-admin denied</t>
         </is>
       </c>
       <c r="D181" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, GET /setup/database/provision-status during initial setup</t>
+          <t>GET /admin/logs/app.log with non-admin token</t>
         </is>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>503, cannot determine provisioning state</t>
+          <t>403, FORBIDDEN; denied audit event recorded</t>
         </is>
       </c>
       <c r="F181" s="4" t="n"/>
@@ -5753,27 +5765,27 @@
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>TC-1105</t>
+          <t>TC-1015</t>
         </is>
       </c>
       <c r="B182" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C182" s="4" t="inlineStr">
         <is>
-          <t>Test connection — success</t>
+          <t>Download log — path traversal blocked</t>
         </is>
       </c>
       <c r="D182" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with valid PostgreSQL credentials</t>
+          <t>GET /admin/logs/../../../etc/passwd</t>
         </is>
       </c>
       <c r="E182" s="4" t="inlineStr">
         <is>
-          <t>200, {"status": "ok", "server_version": "..."}</t>
+          <t>Rejected (400/404/422), no file disclosure</t>
         </is>
       </c>
       <c r="F182" s="4" t="n"/>
@@ -5784,27 +5796,27 @@
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>TC-1106</t>
+          <t>TC-1016</t>
         </is>
       </c>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C183" s="4" t="inlineStr">
         <is>
-          <t>Test connection — bad host</t>
+          <t>Download log — success audit</t>
         </is>
       </c>
       <c r="D183" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with unreachable host</t>
+          <t>Download valid file as admin, then query audit</t>
         </is>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>400, connection error</t>
+          <t>LOG_FILE_DOWNLOADED entry includes requested filename</t>
         </is>
       </c>
       <c r="F183" s="4" t="n"/>
@@ -5813,60 +5825,48 @@
       <c r="I183" s="4" t="n"/>
     </row>
     <row r="184">
-      <c r="A184" s="4" t="inlineStr">
-        <is>
-          <t>TC-1107</t>
-        </is>
-      </c>
-      <c r="B184" s="4" t="inlineStr">
-        <is>
-          <t>12.11 Database Provisioning</t>
-        </is>
-      </c>
-      <c r="C184" s="4" t="inlineStr">
-        <is>
-          <t>Test connection — SSRF host</t>
-        </is>
-      </c>
-      <c r="D184" s="4" t="inlineStr">
-        <is>
-          <t>POST /setup/database/test-connection with "host": "http://evil.com"</t>
-        </is>
-      </c>
-      <c r="E184" s="4" t="inlineStr">
-        <is>
-          <t>422, invalid host</t>
-        </is>
-      </c>
-      <c r="F184" s="4" t="n"/>
-      <c r="G184" s="4" t="n"/>
-      <c r="H184" s="4" t="n"/>
-      <c r="I184" s="4" t="n"/>
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>§12.11 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>12.11 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C184" s="3" t="n"/>
+      <c r="D184" s="3" t="n"/>
+      <c r="E184" s="3" t="n"/>
+      <c r="F184" s="3" t="n"/>
+      <c r="G184" s="3" t="n"/>
+      <c r="H184" s="3" t="n"/>
+      <c r="I184" s="3" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>TC-1108</t>
+          <t>TC-1101</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C185" s="4" t="inlineStr">
         <is>
-          <t>Test connection — port out of range</t>
+          <t>Status — not initialized</t>
         </is>
       </c>
       <c r="D185" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with "port": 99999</t>
+          <t>GET /setup/status on fresh database</t>
         </is>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>200, {"initialized": false}</t>
         </is>
       </c>
       <c r="F185" s="4" t="n"/>
@@ -5877,27 +5877,27 @@
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>TC-1109</t>
+          <t>TC-1102</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C186" s="4" t="inlineStr">
         <is>
-          <t>Provision — success</t>
+          <t>Initialize</t>
         </is>
       </c>
       <c r="D186" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with valid credentials</t>
+          <t>POST /setup/initialize with valid username and password</t>
         </is>
       </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
-          <t>200, returns database, user, migrations_applied</t>
+          <t>200, returns message, username, groups_created</t>
         </is>
       </c>
       <c r="F186" s="4" t="n"/>
@@ -5908,27 +5908,27 @@
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>TC-1110</t>
+          <t>TC-1103</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C187" s="4" t="inlineStr">
         <is>
-          <t>Provision — bad admin credentials</t>
+          <t>Status — initialized</t>
         </is>
       </c>
       <c r="D187" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with wrong admin password</t>
+          <t>GET /setup/status after initialization</t>
         </is>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>400, connection error</t>
+          <t>200, {"initialized": true}</t>
         </is>
       </c>
       <c r="F187" s="4" t="n"/>
@@ -5939,27 +5939,27 @@
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>TC-1111</t>
+          <t>TC-1104</t>
         </is>
       </c>
       <c r="B188" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C188" s="4" t="inlineStr">
         <is>
-          <t>Provision — invalid database name</t>
+          <t>Re-initialize rejected</t>
         </is>
       </c>
       <c r="D188" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with "app_database": "drop;--"</t>
+          <t>POST /setup/initialize again</t>
         </is>
       </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
-          <t>422, invalid identifier</t>
+          <t>409, Conflict</t>
         </is>
       </c>
       <c r="F188" s="4" t="n"/>
@@ -5970,27 +5970,27 @@
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>TC-1112</t>
+          <t>TC-1105</t>
         </is>
       </c>
       <c r="B189" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C189" s="4" t="inlineStr">
         <is>
-          <t>Status — connected</t>
+          <t>Invalid username</t>
         </is>
       </c>
       <c r="D189" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/status with admin token</t>
+          <t>POST /setup/initialize with uppercase or special chars</t>
         </is>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>200, connected: true, migration info</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F189" s="4" t="n"/>
@@ -6001,27 +6001,27 @@
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>TC-1113</t>
+          <t>TC-1106</t>
         </is>
       </c>
       <c r="B190" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C190" s="4" t="inlineStr">
         <is>
-          <t>Status — requires auth</t>
+          <t>Empty password</t>
         </is>
       </c>
       <c r="D190" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/status without token</t>
+          <t>POST /setup/initialize with {"password": ""}</t>
         </is>
       </c>
       <c r="E190" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F190" s="4" t="n"/>
@@ -6032,27 +6032,27 @@
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>TC-1114</t>
+          <t>TC-1107</t>
         </is>
       </c>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C191" s="4" t="inlineStr">
         <is>
-          <t>Status — requires admin</t>
+          <t>Unsafe password chars</t>
         </is>
       </c>
       <c r="D191" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/status with processor token</t>
+          <t>POST /setup/initialize with password containing newline or colon</t>
         </is>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>403</t>
+          <t>422, unsafe characters</t>
         </is>
       </c>
       <c r="F191" s="4" t="n"/>
@@ -6063,27 +6063,27 @@
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>TC-1115</t>
+          <t>TC-1108</t>
         </is>
       </c>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C192" s="4" t="inlineStr">
         <is>
-          <t>Settings update — success</t>
+          <t>Login as initialized admin</t>
         </is>
       </c>
       <c r="D192" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with valid partial update</t>
+          <t>POST /auth/token with the admin credentials from step 2</t>
         </is>
       </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
-          <t>200, {"status": "updated", ...}</t>
+          <t>200, JWT contains admin role</t>
         </is>
       </c>
       <c r="F192" s="4" t="n"/>
@@ -6094,27 +6094,27 @@
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>TC-1116</t>
+          <t>TC-1109</t>
         </is>
       </c>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C193" s="4" t="inlineStr">
         <is>
-          <t>Settings update — bad connection</t>
+          <t>SYSTEM_INITIALIZED audit log</t>
         </is>
       </c>
       <c r="D193" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with unreachable host</t>
+          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
         </is>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>400, connection test failed</t>
+          <t>Audit entry with actor</t>
         </is>
       </c>
       <c r="F193" s="4" t="n"/>
@@ -6123,60 +6123,48 @@
       <c r="I193" s="4" t="n"/>
     </row>
     <row r="194">
-      <c r="A194" s="4" t="inlineStr">
-        <is>
-          <t>TC-1117</t>
-        </is>
-      </c>
-      <c r="B194" s="4" t="inlineStr">
-        <is>
-          <t>12.11 Database Provisioning</t>
-        </is>
-      </c>
-      <c r="C194" s="4" t="inlineStr">
-        <is>
-          <t>Settings update — empty body</t>
-        </is>
-      </c>
-      <c r="D194" s="4" t="inlineStr">
-        <is>
-          <t>PUT /setup/database/settings with {}</t>
-        </is>
-      </c>
-      <c r="E194" s="4" t="inlineStr">
-        <is>
-          <t>422, at least one field required</t>
-        </is>
-      </c>
-      <c r="F194" s="4" t="n"/>
-      <c r="G194" s="4" t="n"/>
-      <c r="H194" s="4" t="n"/>
-      <c r="I194" s="4" t="n"/>
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>§12.12 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>12.12 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C194" s="3" t="n"/>
+      <c r="D194" s="3" t="n"/>
+      <c r="E194" s="3" t="n"/>
+      <c r="F194" s="3" t="n"/>
+      <c r="G194" s="3" t="n"/>
+      <c r="H194" s="3" t="n"/>
+      <c r="I194" s="3" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>TC-1118</t>
+          <t>TC-1201</t>
         </is>
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr">
         <is>
-          <t>Settings update — requires admin</t>
+          <t>System info — bare-metal defaults</t>
         </is>
       </c>
       <c r="D195" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with processor token</t>
+          <t>GET /setup/database/system-info before setup</t>
         </is>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>403</t>
+          <t>200, {"in_docker": false, "suggested_db_host": "localhost"}</t>
         </is>
       </c>
       <c r="F195" s="4" t="n"/>
@@ -6187,27 +6175,27 @@
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>TC-1119</t>
+          <t>TC-1202</t>
         </is>
       </c>
       <c r="B196" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C196" s="4" t="inlineStr">
         <is>
-          <t>Auth after setup — test-connection</t>
+          <t>Provision status — pre-init public</t>
         </is>
       </c>
       <c r="D196" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection without token (after admin exists)</t>
+          <t>GET /setup/database/provision-status before any admin exists</t>
         </is>
       </c>
       <c r="E196" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>200, {"provisioned": false}</t>
         </is>
       </c>
       <c r="F196" s="4" t="n"/>
@@ -6218,22 +6206,22 @@
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>TC-1120</t>
+          <t>TC-1203</t>
         </is>
       </c>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C197" s="4" t="inlineStr">
         <is>
-          <t>Auth after setup — provision</t>
+          <t>Provision status — post-init requires admin</t>
         </is>
       </c>
       <c r="D197" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision without token (after admin exists)</t>
+          <t>GET /setup/database/provision-status without token after setup</t>
         </is>
       </c>
       <c r="E197" s="4" t="inlineStr">
@@ -6249,27 +6237,27 @@
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>TC-1121</t>
+          <t>TC-1204</t>
         </is>
       </c>
       <c r="B198" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C198" s="4" t="inlineStr">
         <is>
-          <t>Password redaction</t>
+          <t>Provision status — state unknown</t>
         </is>
       </c>
       <c r="D198" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision and check response</t>
+          <t>Stop PostgreSQL, GET /setup/database/provision-status during initial setup</t>
         </is>
       </c>
       <c r="E198" s="4" t="inlineStr">
         <is>
-          <t>No password in response body</t>
+          <t>503, cannot determine provisioning state</t>
         </is>
       </c>
       <c r="F198" s="4" t="n"/>
@@ -6280,27 +6268,27 @@
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>TC-1122</t>
+          <t>TC-1205</t>
         </is>
       </c>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C199" s="4" t="inlineStr">
         <is>
-          <t>Re-provision blocked</t>
+          <t>Test connection — success</t>
         </is>
       </c>
       <c r="D199" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision after successful provisioning (no force)</t>
+          <t>POST /setup/database/test-connection with valid PostgreSQL credentials</t>
         </is>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>409, already provisioned</t>
+          <t>200, {"status": "ok", "server_version": "..."}</t>
         </is>
       </c>
       <c r="F199" s="4" t="n"/>
@@ -6311,27 +6299,27 @@
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t>TC-1123</t>
+          <t>TC-1206</t>
         </is>
       </c>
       <c r="B200" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C200" s="4" t="inlineStr">
         <is>
-          <t>Force re-provision (admin)</t>
+          <t>Test connection — bad host</t>
         </is>
       </c>
       <c r="D200" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with "force": true and admin token after successful provisioning</t>
+          <t>POST /setup/database/test-connection with unreachable host</t>
         </is>
       </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
-          <t>200, returns database, user, migrations_applied</t>
+          <t>400, connection error</t>
         </is>
       </c>
       <c r="F200" s="4" t="n"/>
@@ -6342,27 +6330,27 @@
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
         <is>
-          <t>TC-1124</t>
+          <t>TC-1207</t>
         </is>
       </c>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C201" s="4" t="inlineStr">
         <is>
-          <t>Force rejected unauthenticated</t>
+          <t>Test connection — SSRF host</t>
         </is>
       </c>
       <c r="D201" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with "force": true during initial setup (no admin exists)</t>
+          <t>POST /setup/database/test-connection with "host": "http://evil.com"</t>
         </is>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>403, force requires admin</t>
+          <t>422, invalid host</t>
         </is>
       </c>
       <c r="F201" s="4" t="n"/>
@@ -6373,27 +6361,27 @@
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>TC-1125</t>
+          <t>TC-1208</t>
         </is>
       </c>
       <c r="B202" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C202" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — DB unreachable, no JWT</t>
+          <t>Test connection — port out of range</t>
         </is>
       </c>
       <c r="D202" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/test-connection without token</t>
+          <t>POST /setup/database/test-connection with "port": 99999</t>
         </is>
       </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
-          <t>503, database unavailable message</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F202" s="4" t="n"/>
@@ -6404,27 +6392,27 @@
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>TC-1126</t>
+          <t>TC-1209</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C203" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — DB unreachable, admin JWT</t>
+          <t>Provision — success</t>
         </is>
       </c>
       <c r="D203" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/test-connection with valid admin token</t>
+          <t>POST /setup/database/provision with valid credentials</t>
         </is>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
-          <t>Request proceeds (not blocked by 503)</t>
+          <t>200, returns database, user, migrations_applied</t>
         </is>
       </c>
       <c r="F203" s="4" t="n"/>
@@ -6435,27 +6423,27 @@
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>TC-1127</t>
+          <t>TC-1210</t>
         </is>
       </c>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C204" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — provision state unknown</t>
+          <t>Provision — bad admin credentials</t>
         </is>
       </c>
       <c r="D204" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/provision without "force": true</t>
+          <t>POST /setup/database/provision with wrong admin password</t>
         </is>
       </c>
       <c r="E204" s="4" t="inlineStr">
         <is>
-          <t>503, cannot determine provisioning state</t>
+          <t>400, connection error</t>
         </is>
       </c>
       <c r="F204" s="4" t="n"/>
@@ -6466,27 +6454,27 @@
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>TC-1128</t>
+          <t>TC-1211</t>
         </is>
       </c>
       <c r="B205" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C205" s="4" t="inlineStr">
         <is>
-          <t>Force bypasses state check</t>
+          <t>Provision — invalid database name</t>
         </is>
       </c>
       <c r="D205" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/provision with "force": true and admin token</t>
+          <t>POST /setup/database/provision with "app_database": "drop;--"</t>
         </is>
       </c>
       <c r="E205" s="4" t="inlineStr">
         <is>
-          <t>Proceeds to provisioning (no 503 from state check)</t>
+          <t>422, invalid identifier</t>
         </is>
       </c>
       <c r="F205" s="4" t="n"/>
@@ -6497,27 +6485,27 @@
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
         <is>
-          <t>TC-1129</t>
+          <t>TC-1212</t>
         </is>
       </c>
       <c r="B206" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C206" s="4" t="inlineStr">
         <is>
-          <t>Unmigrated DB treated as initial setup</t>
+          <t>Status — connected</t>
         </is>
       </c>
       <c r="D206" s="4" t="inlineStr">
         <is>
-          <t>Drop user_roles table (or use a fresh empty database), POST /setup/database/test-connection without token</t>
+          <t>GET /setup/database/status with admin token</t>
         </is>
       </c>
       <c r="E206" s="4" t="inlineStr">
         <is>
-          <t>200, request allowed (not 503)</t>
+          <t>200, connected: true, migration info</t>
         </is>
       </c>
       <c r="F206" s="4" t="n"/>
@@ -6528,27 +6516,27 @@
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t>TC-1130</t>
+          <t>TC-1213</t>
         </is>
       </c>
       <c r="B207" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C207" s="4" t="inlineStr">
         <is>
-          <t>Fresh install — DB/role missing</t>
+          <t>Status — requires auth</t>
         </is>
       </c>
       <c r="D207" s="4" t="inlineStr">
         <is>
-          <t>With PostgreSQL running but the application database or role not yet created, POST /setup/database/provision without force</t>
+          <t>GET /setup/database/status without token</t>
         </is>
       </c>
       <c r="E207" s="4" t="inlineStr">
         <is>
-          <t>200, provisioning proceeds (not 503)</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F207" s="4" t="n"/>
@@ -6559,27 +6547,27 @@
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
         <is>
-          <t>TC-1131</t>
+          <t>TC-1214</t>
         </is>
       </c>
       <c r="B208" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C208" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — OperationalError on reachable DB</t>
+          <t>Status — requires admin</t>
         </is>
       </c>
       <c r="D208" s="4" t="inlineStr">
         <is>
-          <t>Revoke SELECT on user_roles (or simulate permission denied), POST /setup/database/test-connection without token</t>
+          <t>GET /setup/database/status with processor token</t>
         </is>
       </c>
       <c r="E208" s="4" t="inlineStr">
         <is>
-          <t>503, does NOT grant unauthenticated access</t>
+          <t>403</t>
         </is>
       </c>
       <c r="F208" s="4" t="n"/>
@@ -6590,27 +6578,27 @@
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
         <is>
-          <t>TC-1132</t>
+          <t>TC-1215</t>
         </is>
       </c>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C209" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — unexpected error</t>
+          <t>Settings update — success</t>
         </is>
       </c>
       <c r="D209" s="4" t="inlineStr">
         <is>
-          <t>Trigger an unexpected exception from admin-check (e.g. coding bug), POST /setup/database/test-connection without token</t>
+          <t>PUT /setup/database/settings with valid partial update</t>
         </is>
       </c>
       <c r="E209" s="4" t="inlineStr">
         <is>
-          <t>503, does NOT grant unauthenticated access</t>
+          <t>200, {"status": "updated", ...}</t>
         </is>
       </c>
       <c r="F209" s="4" t="n"/>
@@ -6621,27 +6609,27 @@
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
         <is>
-          <t>TC-1133</t>
+          <t>TC-1216</t>
         </is>
       </c>
       <c r="B210" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C210" s="4" t="inlineStr">
         <is>
-          <t>Provision — migration failure</t>
+          <t>Settings update — bad connection</t>
         </is>
       </c>
       <c r="D210" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with valid credentials but a broken Alembic migration (e.g. conflicting schema)</t>
+          <t>PUT /setup/database/settings with unreachable host</t>
         </is>
       </c>
       <c r="E210" s="4" t="inlineStr">
         <is>
-          <t>500, "migration failed" message; .env not updated, engine not swapped</t>
+          <t>400, connection test failed</t>
         </is>
       </c>
       <c r="F210" s="4" t="n"/>
@@ -6652,27 +6640,27 @@
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
         <is>
-          <t>TC-1134</t>
+          <t>TC-1217</t>
         </is>
       </c>
       <c r="B211" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C211" s="4" t="inlineStr">
         <is>
-          <t>Provision — .env write failure</t>
+          <t>Settings update — empty body</t>
         </is>
       </c>
       <c r="D211" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision after making .env read-only (or disk full)</t>
+          <t>PUT /setup/database/settings with {}</t>
         </is>
       </c>
       <c r="E211" s="4" t="inlineStr">
         <is>
-          <t>500, "failed to persist" message; engine not swapped</t>
+          <t>422, at least one field required</t>
         </is>
       </c>
       <c r="F211" s="4" t="n"/>
@@ -6683,27 +6671,27 @@
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
         <is>
-          <t>TC-1135</t>
+          <t>TC-1218</t>
         </is>
       </c>
       <c r="B212" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C212" s="4" t="inlineStr">
         <is>
-          <t>Provision — engine reinit failure</t>
+          <t>Settings update — requires admin</t>
         </is>
       </c>
       <c r="D212" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision while another reinit is in progress (lock contention)</t>
+          <t>PUT /setup/database/settings with processor token</t>
         </is>
       </c>
       <c r="E212" s="4" t="inlineStr">
         <is>
-          <t>500, "engine could not be switched" message; .env already written</t>
+          <t>403</t>
         </is>
       </c>
       <c r="F212" s="4" t="n"/>
@@ -6712,48 +6700,60 @@
       <c r="I212" s="4" t="n"/>
     </row>
     <row r="213">
-      <c r="A213" s="2" t="inlineStr">
-        <is>
-          <t>§12.12 Startup State Reconciliation</t>
-        </is>
-      </c>
-      <c r="B213" s="2" t="inlineStr">
-        <is>
-          <t>12.12 Startup State Reconciliation</t>
-        </is>
-      </c>
-      <c r="C213" s="3" t="n"/>
-      <c r="D213" s="3" t="n"/>
-      <c r="E213" s="3" t="n"/>
-      <c r="F213" s="3" t="n"/>
-      <c r="G213" s="3" t="n"/>
-      <c r="H213" s="3" t="n"/>
-      <c r="I213" s="3" t="n"/>
+      <c r="A213" s="4" t="inlineStr">
+        <is>
+          <t>TC-1219</t>
+        </is>
+      </c>
+      <c r="B213" s="4" t="inlineStr">
+        <is>
+          <t>12.12 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C213" s="4" t="inlineStr">
+        <is>
+          <t>Auth after setup — test-connection</t>
+        </is>
+      </c>
+      <c r="D213" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/test-connection without token (after admin exists)</t>
+        </is>
+      </c>
+      <c r="E213" s="4" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="F213" s="4" t="n"/>
+      <c r="G213" s="4" t="n"/>
+      <c r="H213" s="4" t="n"/>
+      <c r="I213" s="4" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="4" t="inlineStr">
         <is>
-          <t>TC-1201</t>
+          <t>TC-1220</t>
         </is>
       </c>
       <c r="B214" s="4" t="inlineStr">
         <is>
-          <t>12.12 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C214" s="4" t="inlineStr">
         <is>
-          <t>Running job failed after restart</t>
+          <t>Auth after setup — provision</t>
         </is>
       </c>
       <c r="D214" s="4" t="inlineStr">
         <is>
-          <t>Create a job, start it, restart the service while RUNNING</t>
+          <t>POST /setup/database/provision without token (after admin exists)</t>
         </is>
       </c>
       <c r="E214" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F214" s="4" t="n"/>
@@ -6764,27 +6764,27 @@
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
         <is>
-          <t>TC-1202</t>
+          <t>TC-1221</t>
         </is>
       </c>
       <c r="B215" s="4" t="inlineStr">
         <is>
-          <t>12.12 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C215" s="4" t="inlineStr">
         <is>
-          <t>Verifying job failed after restart</t>
+          <t>Password redaction</t>
         </is>
       </c>
       <c r="D215" s="4" t="inlineStr">
         <is>
-          <t>Start a job, let it reach VERIFYING, restart the service</t>
+          <t>POST /setup/database/provision and check response</t>
         </is>
       </c>
       <c r="E215" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
+          <t>No password in response body</t>
         </is>
       </c>
       <c r="F215" s="4" t="n"/>
@@ -6795,27 +6795,27 @@
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
         <is>
-          <t>TC-1203</t>
+          <t>TC-1222</t>
         </is>
       </c>
       <c r="B216" s="4" t="inlineStr">
         <is>
-          <t>12.12 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C216" s="4" t="inlineStr">
         <is>
-          <t>Pending job not affected</t>
+          <t>Re-provision blocked</t>
         </is>
       </c>
       <c r="D216" s="4" t="inlineStr">
         <is>
-          <t>Create a job (PENDING), restart the service</t>
+          <t>POST /setup/database/provision after successful provisioning (no force)</t>
         </is>
       </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
-          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
+          <t>409, already provisioned</t>
         </is>
       </c>
       <c r="F216" s="4" t="n"/>
@@ -6826,27 +6826,27 @@
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
         <is>
-          <t>TC-1204</t>
+          <t>TC-1223</t>
         </is>
       </c>
       <c r="B217" s="4" t="inlineStr">
         <is>
-          <t>12.12 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C217" s="4" t="inlineStr">
         <is>
-          <t>Completed job not affected</t>
+          <t>Force re-provision (admin)</t>
         </is>
       </c>
       <c r="D217" s="4" t="inlineStr">
         <is>
-          <t>Complete a job, restart the service</t>
+          <t>POST /setup/database/provision with "force": true and admin token after successful provisioning</t>
         </is>
       </c>
       <c r="E217" s="4" t="inlineStr">
         <is>
-          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
+          <t>200, returns database, user, migrations_applied</t>
         </is>
       </c>
       <c r="F217" s="4" t="n"/>
@@ -6857,27 +6857,27 @@
     <row r="218">
       <c r="A218" s="4" t="inlineStr">
         <is>
-          <t>TC-1205</t>
+          <t>TC-1224</t>
         </is>
       </c>
       <c r="B218" s="4" t="inlineStr">
         <is>
-          <t>12.12 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C218" s="4" t="inlineStr">
         <is>
-          <t>Stale mount corrected</t>
+          <t>Force rejected unauthenticated</t>
         </is>
       </c>
       <c r="D218" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
+          <t>POST /setup/database/provision with "force": true during initial setup (no admin exists)</t>
         </is>
       </c>
       <c r="E218" s="4" t="inlineStr">
         <is>
-          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
+          <t>403, force requires admin</t>
         </is>
       </c>
       <c r="F218" s="4" t="n"/>
@@ -6888,27 +6888,27 @@
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
         <is>
-          <t>TC-1206</t>
+          <t>TC-1225</t>
         </is>
       </c>
       <c r="B219" s="4" t="inlineStr">
         <is>
-          <t>12.12 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C219" s="4" t="inlineStr">
         <is>
-          <t>Active mount preserved</t>
+          <t>Fail-closed — DB unreachable, no JWT</t>
         </is>
       </c>
       <c r="D219" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share (leave it mounted), restart the service</t>
+          <t>Stop PostgreSQL, POST /setup/database/test-connection without token</t>
         </is>
       </c>
       <c r="E219" s="4" t="inlineStr">
         <is>
-          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
+          <t>503, database unavailable message</t>
         </is>
       </c>
       <c r="F219" s="4" t="n"/>
@@ -6919,27 +6919,27 @@
     <row r="220">
       <c r="A220" s="4" t="inlineStr">
         <is>
-          <t>TC-1207</t>
+          <t>TC-1226</t>
         </is>
       </c>
       <c r="B220" s="4" t="inlineStr">
         <is>
-          <t>12.12 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C220" s="4" t="inlineStr">
         <is>
-          <t>USB drives re-discovered</t>
+          <t>Fail-closed — DB unreachable, admin JWT</t>
         </is>
       </c>
       <c r="D220" s="4" t="inlineStr">
         <is>
-          <t>Insert USB drives, restart the service</t>
+          <t>Stop PostgreSQL, POST /setup/database/test-connection with valid admin token</t>
         </is>
       </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
-          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
+          <t>Request proceeds (not blocked by 503)</t>
         </is>
       </c>
       <c r="F220" s="4" t="n"/>
@@ -6950,27 +6950,27 @@
     <row r="221">
       <c r="A221" s="4" t="inlineStr">
         <is>
-          <t>TC-1208</t>
+          <t>TC-1227</t>
         </is>
       </c>
       <c r="B221" s="4" t="inlineStr">
         <is>
-          <t>12.12 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C221" s="4" t="inlineStr">
         <is>
-          <t>Idempotency</t>
+          <t>Fail-closed — provision state unknown</t>
         </is>
       </c>
       <c r="D221" s="4" t="inlineStr">
         <is>
-          <t>Restart the service twice without any state changes between restarts</t>
+          <t>Stop PostgreSQL, POST /setup/database/provision without "force": true</t>
         </is>
       </c>
       <c r="E221" s="4" t="inlineStr">
         <is>
-          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
+          <t>503, cannot determine provisioning state</t>
         </is>
       </c>
       <c r="F221" s="4" t="n"/>
@@ -6981,27 +6981,27 @@
     <row r="222">
       <c r="A222" s="4" t="inlineStr">
         <is>
-          <t>TC-1209</t>
+          <t>TC-1228</t>
         </is>
       </c>
       <c r="B222" s="4" t="inlineStr">
         <is>
-          <t>12.12 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C222" s="4" t="inlineStr">
         <is>
-          <t>Partial failure isolation</t>
+          <t>Force bypasses state check</t>
         </is>
       </c>
       <c r="D222" s="4" t="inlineStr">
         <is>
-          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
+          <t>Stop PostgreSQL, POST /setup/database/provision with "force": true and admin token</t>
         </is>
       </c>
       <c r="E222" s="4" t="inlineStr">
         <is>
-          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
+          <t>Proceeds to provisioning (no 503 from state check)</t>
         </is>
       </c>
       <c r="F222" s="4" t="n"/>
@@ -7012,27 +7012,27 @@
     <row r="223">
       <c r="A223" s="4" t="inlineStr">
         <is>
-          <t>TC-1210</t>
+          <t>TC-1229</t>
         </is>
       </c>
       <c r="B223" s="4" t="inlineStr">
         <is>
-          <t>12.12 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C223" s="4" t="inlineStr">
         <is>
-          <t>Cross-process lock — only one worker reconciles</t>
+          <t>Unmigrated DB treated as initial setup</t>
         </is>
       </c>
       <c r="D223" s="4" t="inlineStr">
         <is>
-          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
+          <t>Drop user_roles table (or use a fresh empty database), POST /setup/database/test-connection without token</t>
         </is>
       </c>
       <c r="E223" s="4" t="inlineStr">
         <is>
-          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
+          <t>200, request allowed (not 503)</t>
         </is>
       </c>
       <c r="F223" s="4" t="n"/>
@@ -7043,27 +7043,27 @@
     <row r="224">
       <c r="A224" s="4" t="inlineStr">
         <is>
-          <t>TC-1211</t>
+          <t>TC-1230</t>
         </is>
       </c>
       <c r="B224" s="4" t="inlineStr">
         <is>
-          <t>12.12 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C224" s="4" t="inlineStr">
         <is>
-          <t>Stale lock reclaim</t>
+          <t>Fresh install — DB/role missing</t>
         </is>
       </c>
       <c r="D224" s="4" t="inlineStr">
         <is>
-          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
+          <t>With PostgreSQL running but the application database or role not yet created, POST /setup/database/provision without force</t>
         </is>
       </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
-          <t>Service reclaims the stale lock, reconciliation runs normally</t>
+          <t>200, provisioning proceeds (not 503)</t>
         </is>
       </c>
       <c r="F224" s="4" t="n"/>
@@ -7074,27 +7074,27 @@
     <row r="225">
       <c r="A225" s="4" t="inlineStr">
         <is>
-          <t>TC-1212</t>
+          <t>TC-1231</t>
         </is>
       </c>
       <c r="B225" s="4" t="inlineStr">
         <is>
-          <t>12.12 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C225" s="4" t="inlineStr">
         <is>
-          <t>Lock released after failure</t>
+          <t>Fail-closed — OperationalError on reachable DB</t>
         </is>
       </c>
       <c r="D225" s="4" t="inlineStr">
         <is>
-          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
+          <t>Revoke SELECT on user_roles (or simulate permission denied), POST /setup/database/test-connection without token</t>
         </is>
       </c>
       <c r="E225" s="4" t="inlineStr">
         <is>
-          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
+          <t>503, does NOT grant unauthenticated access</t>
         </is>
       </c>
       <c r="F225" s="4" t="n"/>
@@ -7103,48 +7103,60 @@
       <c r="I225" s="4" t="n"/>
     </row>
     <row r="226">
-      <c r="A226" s="2" t="inlineStr">
-        <is>
-          <t>§12.13 System Health</t>
-        </is>
-      </c>
-      <c r="B226" s="2" t="inlineStr">
-        <is>
-          <t>12.13 System Health</t>
-        </is>
-      </c>
-      <c r="C226" s="3" t="n"/>
-      <c r="D226" s="3" t="n"/>
-      <c r="E226" s="3" t="n"/>
-      <c r="F226" s="3" t="n"/>
-      <c r="G226" s="3" t="n"/>
-      <c r="H226" s="3" t="n"/>
-      <c r="I226" s="3" t="n"/>
+      <c r="A226" s="4" t="inlineStr">
+        <is>
+          <t>TC-1232</t>
+        </is>
+      </c>
+      <c r="B226" s="4" t="inlineStr">
+        <is>
+          <t>12.12 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C226" s="4" t="inlineStr">
+        <is>
+          <t>Fail-closed — unexpected error</t>
+        </is>
+      </c>
+      <c r="D226" s="4" t="inlineStr">
+        <is>
+          <t>Trigger an unexpected exception from admin-check (e.g. coding bug), POST /setup/database/test-connection without token</t>
+        </is>
+      </c>
+      <c r="E226" s="4" t="inlineStr">
+        <is>
+          <t>503, does NOT grant unauthenticated access</t>
+        </is>
+      </c>
+      <c r="F226" s="4" t="n"/>
+      <c r="G226" s="4" t="n"/>
+      <c r="H226" s="4" t="n"/>
+      <c r="I226" s="4" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="4" t="inlineStr">
         <is>
-          <t>TC-1301</t>
+          <t>TC-1233</t>
         </is>
       </c>
       <c r="B227" s="4" t="inlineStr">
         <is>
-          <t>12.13 System Health</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C227" s="4" t="inlineStr">
         <is>
-          <t>Healthy response</t>
+          <t>Provision — migration failure</t>
         </is>
       </c>
       <c r="D227" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with valid token</t>
+          <t>POST /setup/database/provision with valid credentials but a broken Alembic migration (e.g. conflicting schema)</t>
         </is>
       </c>
       <c r="E227" s="4" t="inlineStr">
         <is>
-          <t>200, status: "ok", database: "connected"</t>
+          <t>500, "migration failed" message; .env not updated, engine not swapped</t>
         </is>
       </c>
       <c r="F227" s="4" t="n"/>
@@ -7155,27 +7167,27 @@
     <row r="228">
       <c r="A228" s="4" t="inlineStr">
         <is>
-          <t>TC-1302</t>
+          <t>TC-1234</t>
         </is>
       </c>
       <c r="B228" s="4" t="inlineStr">
         <is>
-          <t>12.13 System Health</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C228" s="4" t="inlineStr">
         <is>
-          <t>CPU metric present</t>
+          <t>Provision — .env write failure</t>
         </is>
       </c>
       <c r="D228" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>POST /setup/database/provision after making .env read-only (or disk full)</t>
         </is>
       </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
-          <t>cpu_percent is a number between 0 and 100</t>
+          <t>500, "failed to persist" message; engine not swapped</t>
         </is>
       </c>
       <c r="F228" s="4" t="n"/>
@@ -7186,27 +7198,27 @@
     <row r="229">
       <c r="A229" s="4" t="inlineStr">
         <is>
-          <t>TC-1303</t>
+          <t>TC-1235</t>
         </is>
       </c>
       <c r="B229" s="4" t="inlineStr">
         <is>
-          <t>12.13 System Health</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C229" s="4" t="inlineStr">
         <is>
-          <t>Memory metrics present</t>
+          <t>Provision — engine reinit failure</t>
         </is>
       </c>
       <c r="D229" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>POST /setup/database/provision while another reinit is in progress (lock contention)</t>
         </is>
       </c>
       <c r="E229" s="4" t="inlineStr">
         <is>
-          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
+          <t>500, "engine could not be switched" message; .env already written</t>
         </is>
       </c>
       <c r="F229" s="4" t="n"/>
@@ -7215,60 +7227,48 @@
       <c r="I229" s="4" t="n"/>
     </row>
     <row r="230">
-      <c r="A230" s="4" t="inlineStr">
-        <is>
-          <t>TC-1304</t>
-        </is>
-      </c>
-      <c r="B230" s="4" t="inlineStr">
-        <is>
-          <t>12.13 System Health</t>
-        </is>
-      </c>
-      <c r="C230" s="4" t="inlineStr">
-        <is>
-          <t>Disk I/O metrics present</t>
-        </is>
-      </c>
-      <c r="D230" s="4" t="inlineStr">
-        <is>
-          <t>Inspect response body</t>
-        </is>
-      </c>
-      <c r="E230" s="4" t="inlineStr">
-        <is>
-          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
-        </is>
-      </c>
-      <c r="F230" s="4" t="n"/>
-      <c r="G230" s="4" t="n"/>
-      <c r="H230" s="4" t="n"/>
-      <c r="I230" s="4" t="n"/>
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>§12.13 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>12.13 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C230" s="3" t="n"/>
+      <c r="D230" s="3" t="n"/>
+      <c r="E230" s="3" t="n"/>
+      <c r="F230" s="3" t="n"/>
+      <c r="G230" s="3" t="n"/>
+      <c r="H230" s="3" t="n"/>
+      <c r="I230" s="3" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
         <is>
-          <t>TC-1305</t>
+          <t>TC-1301</t>
         </is>
       </c>
       <c r="B231" s="4" t="inlineStr">
         <is>
-          <t>12.13 System Health</t>
+          <t>12.13 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C231" s="4" t="inlineStr">
         <is>
-          <t>Active jobs count</t>
+          <t>Running job failed after restart</t>
         </is>
       </c>
       <c r="D231" s="4" t="inlineStr">
         <is>
-          <t>Start an export job, call endpoint</t>
+          <t>Create a job, start it, restart the service while RUNNING</t>
         </is>
       </c>
       <c r="E231" s="4" t="inlineStr">
         <is>
-          <t>active_jobs ≥ 1</t>
+          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
         </is>
       </c>
       <c r="F231" s="4" t="n"/>
@@ -7279,27 +7279,27 @@
     <row r="232">
       <c r="A232" s="4" t="inlineStr">
         <is>
-          <t>TC-1306</t>
+          <t>TC-1302</t>
         </is>
       </c>
       <c r="B232" s="4" t="inlineStr">
         <is>
-          <t>12.13 System Health</t>
+          <t>12.13 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C232" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size</t>
+          <t>Verifying job failed after restart</t>
         </is>
       </c>
       <c r="D232" s="4" t="inlineStr">
         <is>
-          <t>Create a PENDING job (created but not started), call endpoint</t>
+          <t>Start a job, let it reach VERIFYING, restart the service</t>
         </is>
       </c>
       <c r="E232" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size ≥ 1</t>
+          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
         </is>
       </c>
       <c r="F232" s="4" t="n"/>
@@ -7310,27 +7310,27 @@
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
         <is>
-          <t>TC-1307</t>
+          <t>TC-1303</t>
         </is>
       </c>
       <c r="B233" s="4" t="inlineStr">
         <is>
-          <t>12.13 System Health</t>
+          <t>12.13 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C233" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size decrements</t>
+          <t>Pending job not affected</t>
         </is>
       </c>
       <c r="D233" s="4" t="inlineStr">
         <is>
-          <t>Start the pending job, call endpoint again</t>
+          <t>Create a job (PENDING), restart the service</t>
         </is>
       </c>
       <c r="E233" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
+          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
         </is>
       </c>
       <c r="F233" s="4" t="n"/>
@@ -7341,27 +7341,27 @@
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
         <is>
-          <t>TC-1308</t>
+          <t>TC-1304</t>
         </is>
       </c>
       <c r="B234" s="4" t="inlineStr">
         <is>
-          <t>12.13 System Health</t>
+          <t>12.13 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C234" s="4" t="inlineStr">
         <is>
-          <t>Degraded when DB down</t>
+          <t>Completed job not affected</t>
         </is>
       </c>
       <c r="D234" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, call endpoint with valid token</t>
+          <t>Complete a job, restart the service</t>
         </is>
       </c>
       <c r="E234" s="4" t="inlineStr">
         <is>
-          <t>200, status: "degraded", database: "error", database_error is non-null</t>
+          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F234" s="4" t="n"/>
@@ -7372,27 +7372,27 @@
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
         <is>
-          <t>TC-1309</t>
+          <t>TC-1305</t>
         </is>
       </c>
       <c r="B235" s="4" t="inlineStr">
         <is>
-          <t>12.13 System Health</t>
+          <t>12.13 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C235" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated rejected</t>
+          <t>Stale mount corrected</t>
         </is>
       </c>
       <c r="D235" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health without token</t>
+          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
         </is>
       </c>
       <c r="E235" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
         </is>
       </c>
       <c r="F235" s="4" t="n"/>
@@ -7403,27 +7403,27 @@
     <row r="236">
       <c r="A236" s="4" t="inlineStr">
         <is>
-          <t>TC-1310</t>
+          <t>TC-1306</t>
         </is>
       </c>
       <c r="B236" s="4" t="inlineStr">
         <is>
-          <t>12.13 System Health</t>
+          <t>12.13 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C236" s="4" t="inlineStr">
         <is>
-          <t>Processor role allowed</t>
+          <t>Active mount preserved</t>
         </is>
       </c>
       <c r="D236" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with processor token</t>
+          <t>Add and mount a network share (leave it mounted), restart the service</t>
         </is>
       </c>
       <c r="E236" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F236" s="4" t="n"/>
@@ -7431,14 +7431,529 @@
       <c r="H236" s="4" t="n"/>
       <c r="I236" s="4" t="n"/>
     </row>
+    <row r="237">
+      <c r="A237" s="4" t="inlineStr">
+        <is>
+          <t>TC-1307</t>
+        </is>
+      </c>
+      <c r="B237" s="4" t="inlineStr">
+        <is>
+          <t>12.13 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C237" s="4" t="inlineStr">
+        <is>
+          <t>USB drives re-discovered</t>
+        </is>
+      </c>
+      <c r="D237" s="4" t="inlineStr">
+        <is>
+          <t>Insert USB drives, restart the service</t>
+        </is>
+      </c>
+      <c r="E237" s="4" t="inlineStr">
+        <is>
+          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
+        </is>
+      </c>
+      <c r="F237" s="4" t="n"/>
+      <c r="G237" s="4" t="n"/>
+      <c r="H237" s="4" t="n"/>
+      <c r="I237" s="4" t="n"/>
+    </row>
     <row r="238">
-      <c r="A238" s="5" t="inlineStr">
+      <c r="A238" s="4" t="inlineStr">
+        <is>
+          <t>TC-1308</t>
+        </is>
+      </c>
+      <c r="B238" s="4" t="inlineStr">
+        <is>
+          <t>12.13 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C238" s="4" t="inlineStr">
+        <is>
+          <t>Idempotency</t>
+        </is>
+      </c>
+      <c r="D238" s="4" t="inlineStr">
+        <is>
+          <t>Restart the service twice without any state changes between restarts</t>
+        </is>
+      </c>
+      <c r="E238" s="4" t="inlineStr">
+        <is>
+          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
+        </is>
+      </c>
+      <c r="F238" s="4" t="n"/>
+      <c r="G238" s="4" t="n"/>
+      <c r="H238" s="4" t="n"/>
+      <c r="I238" s="4" t="n"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="4" t="inlineStr">
+        <is>
+          <t>TC-1309</t>
+        </is>
+      </c>
+      <c r="B239" s="4" t="inlineStr">
+        <is>
+          <t>12.13 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C239" s="4" t="inlineStr">
+        <is>
+          <t>Partial failure isolation</t>
+        </is>
+      </c>
+      <c r="D239" s="4" t="inlineStr">
+        <is>
+          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
+        </is>
+      </c>
+      <c r="E239" s="4" t="inlineStr">
+        <is>
+          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
+        </is>
+      </c>
+      <c r="F239" s="4" t="n"/>
+      <c r="G239" s="4" t="n"/>
+      <c r="H239" s="4" t="n"/>
+      <c r="I239" s="4" t="n"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="4" t="inlineStr">
+        <is>
+          <t>TC-1310</t>
+        </is>
+      </c>
+      <c r="B240" s="4" t="inlineStr">
+        <is>
+          <t>12.13 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C240" s="4" t="inlineStr">
+        <is>
+          <t>Cross-process lock — only one worker reconciles</t>
+        </is>
+      </c>
+      <c r="D240" s="4" t="inlineStr">
+        <is>
+          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
+        </is>
+      </c>
+      <c r="E240" s="4" t="inlineStr">
+        <is>
+          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
+        </is>
+      </c>
+      <c r="F240" s="4" t="n"/>
+      <c r="G240" s="4" t="n"/>
+      <c r="H240" s="4" t="n"/>
+      <c r="I240" s="4" t="n"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="4" t="inlineStr">
+        <is>
+          <t>TC-1311</t>
+        </is>
+      </c>
+      <c r="B241" s="4" t="inlineStr">
+        <is>
+          <t>12.13 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C241" s="4" t="inlineStr">
+        <is>
+          <t>Stale lock reclaim</t>
+        </is>
+      </c>
+      <c r="D241" s="4" t="inlineStr">
+        <is>
+          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
+        </is>
+      </c>
+      <c r="E241" s="4" t="inlineStr">
+        <is>
+          <t>Service reclaims the stale lock, reconciliation runs normally</t>
+        </is>
+      </c>
+      <c r="F241" s="4" t="n"/>
+      <c r="G241" s="4" t="n"/>
+      <c r="H241" s="4" t="n"/>
+      <c r="I241" s="4" t="n"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="4" t="inlineStr">
+        <is>
+          <t>TC-1312</t>
+        </is>
+      </c>
+      <c r="B242" s="4" t="inlineStr">
+        <is>
+          <t>12.13 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C242" s="4" t="inlineStr">
+        <is>
+          <t>Lock released after failure</t>
+        </is>
+      </c>
+      <c r="D242" s="4" t="inlineStr">
+        <is>
+          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
+        </is>
+      </c>
+      <c r="E242" s="4" t="inlineStr">
+        <is>
+          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
+        </is>
+      </c>
+      <c r="F242" s="4" t="n"/>
+      <c r="G242" s="4" t="n"/>
+      <c r="H242" s="4" t="n"/>
+      <c r="I242" s="4" t="n"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>§12.14 System Health</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C243" s="3" t="n"/>
+      <c r="D243" s="3" t="n"/>
+      <c r="E243" s="3" t="n"/>
+      <c r="F243" s="3" t="n"/>
+      <c r="G243" s="3" t="n"/>
+      <c r="H243" s="3" t="n"/>
+      <c r="I243" s="3" t="n"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="4" t="inlineStr">
+        <is>
+          <t>TC-1401</t>
+        </is>
+      </c>
+      <c r="B244" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C244" s="4" t="inlineStr">
+        <is>
+          <t>Healthy response</t>
+        </is>
+      </c>
+      <c r="D244" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/system-health with valid token</t>
+        </is>
+      </c>
+      <c r="E244" s="4" t="inlineStr">
+        <is>
+          <t>200, status: "ok", database: "connected"</t>
+        </is>
+      </c>
+      <c r="F244" s="4" t="n"/>
+      <c r="G244" s="4" t="n"/>
+      <c r="H244" s="4" t="n"/>
+      <c r="I244" s="4" t="n"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="4" t="inlineStr">
+        <is>
+          <t>TC-1402</t>
+        </is>
+      </c>
+      <c r="B245" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C245" s="4" t="inlineStr">
+        <is>
+          <t>CPU metric present</t>
+        </is>
+      </c>
+      <c r="D245" s="4" t="inlineStr">
+        <is>
+          <t>Inspect response body</t>
+        </is>
+      </c>
+      <c r="E245" s="4" t="inlineStr">
+        <is>
+          <t>cpu_percent is a number between 0 and 100</t>
+        </is>
+      </c>
+      <c r="F245" s="4" t="n"/>
+      <c r="G245" s="4" t="n"/>
+      <c r="H245" s="4" t="n"/>
+      <c r="I245" s="4" t="n"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="4" t="inlineStr">
+        <is>
+          <t>TC-1403</t>
+        </is>
+      </c>
+      <c r="B246" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C246" s="4" t="inlineStr">
+        <is>
+          <t>Memory metrics present</t>
+        </is>
+      </c>
+      <c r="D246" s="4" t="inlineStr">
+        <is>
+          <t>Inspect response body</t>
+        </is>
+      </c>
+      <c r="E246" s="4" t="inlineStr">
+        <is>
+          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
+        </is>
+      </c>
+      <c r="F246" s="4" t="n"/>
+      <c r="G246" s="4" t="n"/>
+      <c r="H246" s="4" t="n"/>
+      <c r="I246" s="4" t="n"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="4" t="inlineStr">
+        <is>
+          <t>TC-1404</t>
+        </is>
+      </c>
+      <c r="B247" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C247" s="4" t="inlineStr">
+        <is>
+          <t>Disk I/O metrics present</t>
+        </is>
+      </c>
+      <c r="D247" s="4" t="inlineStr">
+        <is>
+          <t>Inspect response body</t>
+        </is>
+      </c>
+      <c r="E247" s="4" t="inlineStr">
+        <is>
+          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
+        </is>
+      </c>
+      <c r="F247" s="4" t="n"/>
+      <c r="G247" s="4" t="n"/>
+      <c r="H247" s="4" t="n"/>
+      <c r="I247" s="4" t="n"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="4" t="inlineStr">
+        <is>
+          <t>TC-1405</t>
+        </is>
+      </c>
+      <c r="B248" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C248" s="4" t="inlineStr">
+        <is>
+          <t>Active jobs count</t>
+        </is>
+      </c>
+      <c r="D248" s="4" t="inlineStr">
+        <is>
+          <t>Start an export job, call endpoint</t>
+        </is>
+      </c>
+      <c r="E248" s="4" t="inlineStr">
+        <is>
+          <t>active_jobs ≥ 1</t>
+        </is>
+      </c>
+      <c r="F248" s="4" t="n"/>
+      <c r="G248" s="4" t="n"/>
+      <c r="H248" s="4" t="n"/>
+      <c r="I248" s="4" t="n"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="4" t="inlineStr">
+        <is>
+          <t>TC-1406</t>
+        </is>
+      </c>
+      <c r="B249" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C249" s="4" t="inlineStr">
+        <is>
+          <t>Worker queue size</t>
+        </is>
+      </c>
+      <c r="D249" s="4" t="inlineStr">
+        <is>
+          <t>Create a PENDING job (created but not started), call endpoint</t>
+        </is>
+      </c>
+      <c r="E249" s="4" t="inlineStr">
+        <is>
+          <t>worker_queue_size ≥ 1</t>
+        </is>
+      </c>
+      <c r="F249" s="4" t="n"/>
+      <c r="G249" s="4" t="n"/>
+      <c r="H249" s="4" t="n"/>
+      <c r="I249" s="4" t="n"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="4" t="inlineStr">
+        <is>
+          <t>TC-1407</t>
+        </is>
+      </c>
+      <c r="B250" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C250" s="4" t="inlineStr">
+        <is>
+          <t>Worker queue size decrements</t>
+        </is>
+      </c>
+      <c r="D250" s="4" t="inlineStr">
+        <is>
+          <t>Start the pending job, call endpoint again</t>
+        </is>
+      </c>
+      <c r="E250" s="4" t="inlineStr">
+        <is>
+          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
+        </is>
+      </c>
+      <c r="F250" s="4" t="n"/>
+      <c r="G250" s="4" t="n"/>
+      <c r="H250" s="4" t="n"/>
+      <c r="I250" s="4" t="n"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="4" t="inlineStr">
+        <is>
+          <t>TC-1408</t>
+        </is>
+      </c>
+      <c r="B251" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C251" s="4" t="inlineStr">
+        <is>
+          <t>Degraded when DB down</t>
+        </is>
+      </c>
+      <c r="D251" s="4" t="inlineStr">
+        <is>
+          <t>Stop PostgreSQL, call endpoint with valid token</t>
+        </is>
+      </c>
+      <c r="E251" s="4" t="inlineStr">
+        <is>
+          <t>200, status: "degraded", database: "error", database_error is non-null</t>
+        </is>
+      </c>
+      <c r="F251" s="4" t="n"/>
+      <c r="G251" s="4" t="n"/>
+      <c r="H251" s="4" t="n"/>
+      <c r="I251" s="4" t="n"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="4" t="inlineStr">
+        <is>
+          <t>TC-1409</t>
+        </is>
+      </c>
+      <c r="B252" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C252" s="4" t="inlineStr">
+        <is>
+          <t>Unauthenticated rejected</t>
+        </is>
+      </c>
+      <c r="D252" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/system-health without token</t>
+        </is>
+      </c>
+      <c r="E252" s="4" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="F252" s="4" t="n"/>
+      <c r="G252" s="4" t="n"/>
+      <c r="H252" s="4" t="n"/>
+      <c r="I252" s="4" t="n"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="4" t="inlineStr">
+        <is>
+          <t>TC-1410</t>
+        </is>
+      </c>
+      <c r="B253" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C253" s="4" t="inlineStr">
+        <is>
+          <t>Processor role allowed</t>
+        </is>
+      </c>
+      <c r="D253" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/system-health with processor token</t>
+        </is>
+      </c>
+      <c r="E253" s="4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F253" s="4" t="n"/>
+      <c r="G253" s="4" t="n"/>
+      <c r="H253" s="4" t="n"/>
+      <c r="I253" s="4" t="n"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B238" s="5" t="n">
-        <v>218</v>
+      <c r="B255" s="5" t="n">
+        <v>234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update QA test cases for ECUBE user integration
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I255"/>
+  <dimension ref="A1:I271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4516,7 +4516,7 @@
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>Create user</t>
+          <t>Create new user</t>
         </is>
       </c>
       <c r="D141" s="4" t="inlineStr">
@@ -4547,12 +4547,12 @@
       </c>
       <c r="C142" s="4" t="inlineStr">
         <is>
-          <t>Create user — duplicate</t>
+          <t>Create user — existing ECUBE mapping</t>
         </is>
       </c>
       <c r="D142" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with existing username</t>
+          <t>POST /admin/os-users with username that already has DB roles</t>
         </is>
       </c>
       <c r="E142" s="4" t="inlineStr">
@@ -4578,17 +4578,17 @@
       </c>
       <c r="C143" s="4" t="inlineStr">
         <is>
-          <t>Create user — reserved name</t>
+          <t>Create user — existing OS/directory account (step 1)</t>
         </is>
       </c>
       <c r="D143" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with {"username": "root", ...}</t>
+          <t>POST /admin/os-users with username+roles and no confirm_existing_os_user</t>
         </is>
       </c>
       <c r="E143" s="4" t="inlineStr">
         <is>
-          <t>422, reserved username</t>
+          <t>200, status: "confirmation_required"</t>
         </is>
       </c>
       <c r="F143" s="4" t="n"/>
@@ -4609,17 +4609,17 @@
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>Create user — empty password</t>
+          <t>Create user — existing OS/directory account (confirm)</t>
         </is>
       </c>
       <c r="D144" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with {"password": "", ...}</t>
+          <t>POST /admin/os-users with confirm_existing_os_user: true</t>
         </is>
       </c>
       <c r="E144" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>200, status: "synced_existing_user"</t>
         </is>
       </c>
       <c r="F144" s="4" t="n"/>
@@ -4640,17 +4640,17 @@
       </c>
       <c r="C145" s="4" t="inlineStr">
         <is>
-          <t>Create user — password with newline</t>
+          <t>Create user — existing OS/directory account (cancel)</t>
         </is>
       </c>
       <c r="D145" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with password containing \n</t>
+          <t>POST /admin/os-users with confirm_existing_os_user: false</t>
         </is>
       </c>
       <c r="E145" s="4" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>200, status: "canceled"</t>
         </is>
       </c>
       <c r="F145" s="4" t="n"/>
@@ -4671,17 +4671,17 @@
       </c>
       <c r="C146" s="4" t="inlineStr">
         <is>
-          <t>Create user — password with colon</t>
+          <t>Create user — reserved name</t>
         </is>
       </c>
       <c r="D146" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with password containing :</t>
+          <t>POST /admin/os-users with {"username": "root", ...}</t>
         </is>
       </c>
       <c r="E146" s="4" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>422, reserved username</t>
         </is>
       </c>
       <c r="F146" s="4" t="n"/>
@@ -4702,17 +4702,17 @@
       </c>
       <c r="C147" s="4" t="inlineStr">
         <is>
-          <t>Create user — invalid group</t>
+          <t>Create user — empty password (new user path)</t>
         </is>
       </c>
       <c r="D147" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with non-existent group in groups list</t>
+          <t>POST /admin/os-users with {"password": "", ...}</t>
         </is>
       </c>
       <c r="E147" s="4" t="inlineStr">
         <is>
-          <t>422, group does not exist</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F147" s="4" t="n"/>
@@ -4733,17 +4733,17 @@
       </c>
       <c r="C148" s="4" t="inlineStr">
         <is>
-          <t>Create user — no roles</t>
+          <t>Create user — password with newline</t>
         </is>
       </c>
       <c r="D148" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with empty/omitted roles</t>
+          <t>POST /admin/os-users with password containing \n</t>
         </is>
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
-          <t>422, at least one role required</t>
+          <t>422, unsafe characters</t>
         </is>
       </c>
       <c r="F148" s="4" t="n"/>
@@ -4764,17 +4764,17 @@
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>List users</t>
+          <t>Create user — password with colon</t>
         </is>
       </c>
       <c r="D149" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/os-users</t>
+          <t>POST /admin/os-users with password containing :</t>
         </is>
       </c>
       <c r="E149" s="4" t="inlineStr">
         <is>
-          <t>200, only users in ecube-* groups listed</t>
+          <t>422, unsafe characters</t>
         </is>
       </c>
       <c r="F149" s="4" t="n"/>
@@ -4795,17 +4795,17 @@
       </c>
       <c r="C150" s="4" t="inlineStr">
         <is>
-          <t>Reset password</t>
+          <t>Create user — invalid group</t>
         </is>
       </c>
       <c r="D150" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/{username}/password with {"password": "NewPass!"}</t>
+          <t>POST /admin/os-users with non-existent group in groups list</t>
         </is>
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>422, group does not exist</t>
         </is>
       </c>
       <c r="F150" s="4" t="n"/>
@@ -4826,17 +4826,17 @@
       </c>
       <c r="C151" s="4" t="inlineStr">
         <is>
-          <t>Reset password — non-ECUBE user</t>
+          <t>Create user — no roles</t>
         </is>
       </c>
       <c r="D151" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/postgres/password</t>
+          <t>POST /admin/os-users with empty/omitted roles</t>
         </is>
       </c>
       <c r="E151" s="4" t="inlineStr">
         <is>
-          <t>422, user is not ECUBE-managed</t>
+          <t>422, at least one role required</t>
         </is>
       </c>
       <c r="F151" s="4" t="n"/>
@@ -4857,17 +4857,17 @@
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
-          <t>Replace groups</t>
+          <t>List users</t>
         </is>
       </c>
       <c r="D152" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/{username}/groups with {"groups": ["ecube-admins"]}</t>
+          <t>GET /admin/os-users</t>
         </is>
       </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
-          <t>200, updated group list; non-ecube-* groups preserved</t>
+          <t>200, includes users in ecube-* groups and users with DB role assignments</t>
         </is>
       </c>
       <c r="F152" s="4" t="n"/>
@@ -4888,17 +4888,17 @@
       </c>
       <c r="C153" s="4" t="inlineStr">
         <is>
-          <t>Replace groups — empty list</t>
+          <t>List users — directory-backed role-only account</t>
         </is>
       </c>
       <c r="D153" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/{username}/groups with {"groups": []}</t>
+          <t>Assign DB roles for a directory user that is not in OS enumeration, then GET /admin/os-users</t>
         </is>
       </c>
       <c r="E153" s="4" t="inlineStr">
         <is>
-          <t>422, at least one ecube-* group required</t>
+          <t>200, user appears with placeholder host fields (uid=-1, gid=-1)</t>
         </is>
       </c>
       <c r="F153" s="4" t="n"/>
@@ -4919,17 +4919,17 @@
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>Replace groups — non-ecube name</t>
+          <t>Reset password</t>
         </is>
       </c>
       <c r="D154" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/{username}/groups with {"groups": ["docker"]}</t>
+          <t>PUT /admin/os-users/{username}/password with {"password": "NewPass!"}</t>
         </is>
       </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
-          <t>422, group does not start with ecube-</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F154" s="4" t="n"/>
@@ -4950,17 +4950,17 @@
       </c>
       <c r="C155" s="4" t="inlineStr">
         <is>
-          <t>Append groups</t>
+          <t>Reset password — non-ECUBE user</t>
         </is>
       </c>
       <c r="D155" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users/{username}/groups with {"groups": ["ecube-managers"]}</t>
+          <t>PUT /admin/os-users/postgres/password</t>
         </is>
       </c>
       <c r="E155" s="4" t="inlineStr">
         <is>
-          <t>200, updated group list</t>
+          <t>422, user is not ECUBE-managed</t>
         </is>
       </c>
       <c r="F155" s="4" t="n"/>
@@ -4981,17 +4981,17 @@
       </c>
       <c r="C156" s="4" t="inlineStr">
         <is>
-          <t>Modify groups — non-ECUBE user</t>
+          <t>Replace groups</t>
         </is>
       </c>
       <c r="D156" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/www-data/groups</t>
+          <t>PUT /admin/os-users/{username}/groups with {"groups": ["ecube-admins"]}</t>
         </is>
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
-          <t>422, user is not ECUBE-managed</t>
+          <t>200, updated group list; non-ecube-* groups preserved</t>
         </is>
       </c>
       <c r="F156" s="4" t="n"/>
@@ -5012,17 +5012,17 @@
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
-          <t>Delete user</t>
+          <t>Replace groups — empty list</t>
         </is>
       </c>
       <c r="D157" s="4" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-users/{username}</t>
+          <t>PUT /admin/os-users/{username}/groups with {"groups": []}</t>
         </is>
       </c>
       <c r="E157" s="4" t="inlineStr">
         <is>
-          <t>200, user and DB roles removed</t>
+          <t>422, at least one ecube-* group required</t>
         </is>
       </c>
       <c r="F157" s="4" t="n"/>
@@ -5043,17 +5043,17 @@
       </c>
       <c r="C158" s="4" t="inlineStr">
         <is>
-          <t>Delete user — non-ECUBE user</t>
+          <t>Replace groups — non-ecube name</t>
         </is>
       </c>
       <c r="D158" s="4" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-users/daemon</t>
+          <t>PUT /admin/os-users/{username}/groups with {"groups": ["docker"]}</t>
         </is>
       </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
-          <t>422, user is not ECUBE-managed</t>
+          <t>422, group does not start with ecube-</t>
         </is>
       </c>
       <c r="F158" s="4" t="n"/>
@@ -5074,17 +5074,17 @@
       </c>
       <c r="C159" s="4" t="inlineStr">
         <is>
-          <t>Delete user — not found</t>
+          <t>Append groups</t>
         </is>
       </c>
       <c r="D159" s="4" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-users/nonexistent</t>
+          <t>POST /admin/os-users/{username}/groups with {"groups": ["ecube-managers"]}</t>
         </is>
       </c>
       <c r="E159" s="4" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>200, updated group list</t>
         </is>
       </c>
       <c r="F159" s="4" t="n"/>
@@ -5105,17 +5105,17 @@
       </c>
       <c r="C160" s="4" t="inlineStr">
         <is>
-          <t>Processor cannot access OS endpoints</t>
+          <t>Modify groups — non-ECUBE user</t>
         </is>
       </c>
       <c r="D160" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/os-users with processor token</t>
+          <t>PUT /admin/os-users/www-data/groups</t>
         </is>
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>422, user is not ECUBE-managed</t>
         </is>
       </c>
       <c r="F160" s="4" t="n"/>
@@ -5136,17 +5136,17 @@
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>Non-local mode returns 404</t>
+          <t>Delete user</t>
         </is>
       </c>
       <c r="D161" s="4" t="inlineStr">
         <is>
-          <t>All /admin/os-* endpoints when role_resolver != "local"</t>
+          <t>DELETE /admin/os-users/{username}</t>
         </is>
       </c>
       <c r="E161" s="4" t="inlineStr">
         <is>
-          <t>404, Not Found</t>
+          <t>200, user and DB roles removed</t>
         </is>
       </c>
       <c r="F161" s="4" t="n"/>
@@ -5167,17 +5167,17 @@
       </c>
       <c r="C162" s="4" t="inlineStr">
         <is>
-          <t>OS_USER_CREATED audit log</t>
+          <t>Delete user — non-ECUBE user</t>
         </is>
       </c>
       <c r="D162" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_USER_CREATED after creating user</t>
+          <t>DELETE /admin/os-users/daemon</t>
         </is>
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor and username</t>
+          <t>422, user is not ECUBE-managed</t>
         </is>
       </c>
       <c r="F162" s="4" t="n"/>
@@ -5198,17 +5198,17 @@
       </c>
       <c r="C163" s="4" t="inlineStr">
         <is>
-          <t>OS_USER_DELETED audit log</t>
+          <t>Delete user — not found</t>
         </is>
       </c>
       <c r="D163" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_USER_DELETED after deleting user</t>
+          <t>DELETE /admin/os-users/nonexistent</t>
         </is>
       </c>
       <c r="E163" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor and username</t>
+          <t>404</t>
         </is>
       </c>
       <c r="F163" s="4" t="n"/>
@@ -5229,17 +5229,17 @@
       </c>
       <c r="C164" s="4" t="inlineStr">
         <is>
-          <t>OS_PASSWORD_RESET audit log</t>
+          <t>Processor cannot access OS endpoints</t>
         </is>
       </c>
       <c r="D164" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_PASSWORD_RESET after resetting password</t>
+          <t>GET /admin/os-users with processor token</t>
         </is>
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>Audit entry (no password in details)</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F164" s="4" t="n"/>
@@ -5260,17 +5260,17 @@
       </c>
       <c r="C165" s="4" t="inlineStr">
         <is>
-          <t>OS_GROUP_CREATED audit log</t>
+          <t>Non-local mode returns 404</t>
         </is>
       </c>
       <c r="D165" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_GROUP_CREATED after creating group</t>
+          <t>All /admin/os-* endpoints when role_resolver != "local"</t>
         </is>
       </c>
       <c r="E165" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with group name</t>
+          <t>404, Not Found</t>
         </is>
       </c>
       <c r="F165" s="4" t="n"/>
@@ -5291,17 +5291,17 @@
       </c>
       <c r="C166" s="4" t="inlineStr">
         <is>
-          <t>OS_GROUP_DELETED audit log</t>
+          <t>OS_USER_CREATED audit log</t>
         </is>
       </c>
       <c r="D166" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_GROUP_DELETED after deleting group</t>
+          <t>GET /audit?action=OS_USER_CREATED after creating user</t>
         </is>
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with group name</t>
+          <t>Audit entry with actor and username</t>
         </is>
       </c>
       <c r="F166" s="4" t="n"/>
@@ -5310,48 +5310,60 @@
       <c r="I166" s="4" t="n"/>
     </row>
     <row r="167">
-      <c r="A167" s="2" t="inlineStr">
-        <is>
-          <t>§12.10 Admin Log Viewing API</t>
-        </is>
-      </c>
-      <c r="B167" s="2" t="inlineStr">
-        <is>
-          <t>12.10 Admin Log Viewing API</t>
-        </is>
-      </c>
-      <c r="C167" s="3" t="n"/>
-      <c r="D167" s="3" t="n"/>
-      <c r="E167" s="3" t="n"/>
-      <c r="F167" s="3" t="n"/>
-      <c r="G167" s="3" t="n"/>
-      <c r="H167" s="3" t="n"/>
-      <c r="I167" s="3" t="n"/>
+      <c r="A167" s="4" t="inlineStr">
+        <is>
+          <t>TC-932</t>
+        </is>
+      </c>
+      <c r="B167" s="4" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C167" s="4" t="inlineStr">
+        <is>
+          <t>OS_USER_CREATE_CONFIRMATION_REQUIRED audit log</t>
+        </is>
+      </c>
+      <c r="D167" s="4" t="inlineStr">
+        <is>
+          <t>GET /audit?action=OS_USER_CREATE_CONFIRMATION_REQUIRED after existing-user step 1</t>
+        </is>
+      </c>
+      <c r="E167" s="4" t="inlineStr">
+        <is>
+          <t>Audit entry with actor and target username</t>
+        </is>
+      </c>
+      <c r="F167" s="4" t="n"/>
+      <c r="G167" s="4" t="n"/>
+      <c r="H167" s="4" t="n"/>
+      <c r="I167" s="4" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>TC-1001</t>
+          <t>TC-933</t>
         </is>
       </c>
       <c r="B168" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
-          <t>View logs — unauthenticated</t>
+          <t>OS_USER_CREATE_CANCELED audit log</t>
         </is>
       </c>
       <c r="D168" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/view without token</t>
+          <t>GET /audit?action=OS_USER_CREATE_CANCELED after cancel path</t>
         </is>
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>401, UNAUTHORIZED</t>
+          <t>Audit entry with actor and target username</t>
         </is>
       </c>
       <c r="F168" s="4" t="n"/>
@@ -5362,27 +5374,27 @@
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>TC-1002</t>
+          <t>TC-934</t>
         </is>
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>View logs — non-admin denied</t>
+          <t>OS_USER_SYNCED_EXISTING audit log</t>
         </is>
       </c>
       <c r="D169" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/view with manager/processor/auditor token</t>
+          <t>GET /audit?action=OS_USER_SYNCED_EXISTING after confirm path</t>
         </is>
       </c>
       <c r="E169" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN; denied audit event recorded</t>
+          <t>Audit entry with actor and target username</t>
         </is>
       </c>
       <c r="F169" s="4" t="n"/>
@@ -5393,27 +5405,27 @@
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>TC-1003</t>
+          <t>TC-935</t>
         </is>
       </c>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C170" s="4" t="inlineStr">
         <is>
-          <t>View logs — unknown source</t>
+          <t>OS_USER_DELETED audit log</t>
         </is>
       </c>
       <c r="D170" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/view?source=unknown with admin token</t>
+          <t>GET /audit?action=OS_USER_DELETED after deleting user</t>
         </is>
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>404, unknown log source</t>
+          <t>Audit entry with actor and username</t>
         </is>
       </c>
       <c r="F170" s="4" t="n"/>
@@ -5424,27 +5436,27 @@
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>TC-1004</t>
+          <t>TC-936</t>
         </is>
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C171" s="4" t="inlineStr">
         <is>
-          <t>View logs — baseline response shape</t>
+          <t>OS_PASSWORD_RESET audit log</t>
         </is>
       </c>
       <c r="D171" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/view?source=app&amp;limit=5&amp;offset=0</t>
+          <t>GET /audit?action=OS_PASSWORD_RESET after resetting password</t>
         </is>
       </c>
       <c r="E171" s="4" t="inlineStr">
         <is>
-          <t>200 with object fields: source, fetched_at, file_modified_at, offset, limit, returned, has_more, lines</t>
+          <t>Audit entry (no password in details)</t>
         </is>
       </c>
       <c r="F171" s="4" t="n"/>
@@ -5455,27 +5467,27 @@
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>TC-1005</t>
+          <t>TC-937</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C172" s="4" t="inlineStr">
         <is>
-          <t>View logs — source path redaction</t>
+          <t>OS_GROUP_CREATED audit log</t>
         </is>
       </c>
       <c r="D172" s="4" t="inlineStr">
         <is>
-          <t>Inspect source.path in successful response</t>
+          <t>GET /audit?action=OS_GROUP_CREATED after creating group</t>
         </is>
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t>Basename only (for example app.log), no absolute filesystem path</t>
+          <t>Audit entry with group name</t>
         </is>
       </c>
       <c r="F172" s="4" t="n"/>
@@ -5486,27 +5498,27 @@
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>TC-1006</t>
+          <t>TC-938</t>
         </is>
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C173" s="4" t="inlineStr">
         <is>
-          <t>View logs — offset pagination</t>
+          <t>OS_GROUP_DELETED audit log</t>
         </is>
       </c>
       <c r="D173" s="4" t="inlineStr">
         <is>
-          <t>Create known numbered lines, call GET /admin/logs/view?limit=5&amp;offset=2</t>
+          <t>GET /audit?action=OS_GROUP_DELETED after deleting group</t>
         </is>
       </c>
       <c r="E173" s="4" t="inlineStr">
         <is>
-          <t>Returns correct window from tail semantics, returned &lt;= limit</t>
+          <t>Audit entry with group name</t>
         </is>
       </c>
       <c r="F173" s="4" t="n"/>
@@ -5515,60 +5527,48 @@
       <c r="I173" s="4" t="n"/>
     </row>
     <row r="174">
-      <c r="A174" s="4" t="inlineStr">
-        <is>
-          <t>TC-1007</t>
-        </is>
-      </c>
-      <c r="B174" s="4" t="inlineStr">
-        <is>
-          <t>12.10 Admin Log Viewing API</t>
-        </is>
-      </c>
-      <c r="C174" s="4" t="inlineStr">
-        <is>
-          <t>View logs — reverse ordering</t>
-        </is>
-      </c>
-      <c r="D174" s="4" t="inlineStr">
-        <is>
-          <t>Compare reverse=false vs reverse=true on same query</t>
-        </is>
-      </c>
-      <c r="E174" s="4" t="inlineStr">
-        <is>
-          <t>Same selected window; line order is inverted when reverse=true</t>
-        </is>
-      </c>
-      <c r="F174" s="4" t="n"/>
-      <c r="G174" s="4" t="n"/>
-      <c r="H174" s="4" t="n"/>
-      <c r="I174" s="4" t="n"/>
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>§12.9.1 UI Validation Checklist — Create User Modal Flow</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>12.9.1 UI Validation Checklist — Create User Modal Flow</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="n"/>
+      <c r="D174" s="3" t="n"/>
+      <c r="E174" s="3" t="n"/>
+      <c r="F174" s="3" t="n"/>
+      <c r="G174" s="3" t="n"/>
+      <c r="H174" s="3" t="n"/>
+      <c r="I174" s="3" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>TC-1008</t>
+          <t>TC-911</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.9.1 UI Validation Checklist — Create User Modal Flow</t>
         </is>
       </c>
       <c r="C175" s="4" t="inlineStr">
         <is>
-          <t>View logs — search filtering</t>
+          <t>Existing user shows confirmation prompt</t>
         </is>
       </c>
       <c r="D175" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/view?search=error</t>
+          <t>In Users -&gt; Create User, enter username that exists in OS/directory, select roles, click Create</t>
         </is>
       </c>
       <c r="E175" s="4" t="inlineStr">
         <is>
-          <t>Only matching lines are returned (case-insensitive contains)</t>
+          <t>Create dialog closes and existing-user confirmation dialog appears</t>
         </is>
       </c>
       <c r="F175" s="4" t="n"/>
@@ -5579,27 +5579,27 @@
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>TC-1009</t>
+          <t>TC-912</t>
         </is>
       </c>
       <c r="B176" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.9.1 UI Validation Checklist — Create User Modal Flow</t>
         </is>
       </c>
       <c r="C176" s="4" t="inlineStr">
         <is>
-          <t>View logs — sensitive value redaction</t>
+          <t>Existing user confirm path</t>
         </is>
       </c>
       <c r="D176" s="4" t="inlineStr">
         <is>
-          <t>Include tokens/passwords in source log lines, call view endpoint</t>
+          <t>From confirmation dialog click confirm (Add to ECUBE)</t>
         </is>
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
-          <t>Sensitive values replaced with redacted markers in lines[].content</t>
+          <t>Confirmation dialog closes, user is linked to ECUBE roles, no password dialog appears</t>
         </is>
       </c>
       <c r="F176" s="4" t="n"/>
@@ -5610,27 +5610,27 @@
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>TC-1010</t>
+          <t>TC-913</t>
         </is>
       </c>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.9.1 UI Validation Checklist — Create User Modal Flow</t>
         </is>
       </c>
       <c r="C177" s="4" t="inlineStr">
         <is>
-          <t>View logs — success audit</t>
+          <t>Existing user cancel path</t>
         </is>
       </c>
       <c r="D177" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=LOG_LINES_VIEWED after successful view</t>
+          <t>From confirmation dialog click Cancel</t>
         </is>
       </c>
       <c r="E177" s="4" t="inlineStr">
         <is>
-          <t>Audit entry includes source, limit, offset, returned, has_more, and basename log_file</t>
+          <t>Dialog closes, returns to Users page (no create dialog reopened)</t>
         </is>
       </c>
       <c r="F177" s="4" t="n"/>
@@ -5641,27 +5641,27 @@
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>TC-1011</t>
+          <t>TC-914</t>
         </is>
       </c>
       <c r="B178" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.9.1 UI Validation Checklist — Create User Modal Flow</t>
         </is>
       </c>
       <c r="C178" s="4" t="inlineStr">
         <is>
-          <t>List logs — unauthenticated</t>
+          <t>New user opens password dialog</t>
         </is>
       </c>
       <c r="D178" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs without token</t>
+          <t>In Create User, enter brand-new username + roles and click Create</t>
         </is>
       </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
-          <t>401, UNAUTHORIZED</t>
+          <t>Password dialog appears (with password + confirm-password fields)</t>
         </is>
       </c>
       <c r="F178" s="4" t="n"/>
@@ -5672,27 +5672,27 @@
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>TC-1012</t>
+          <t>TC-915</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.9.1 UI Validation Checklist — Create User Modal Flow</t>
         </is>
       </c>
       <c r="C179" s="4" t="inlineStr">
         <is>
-          <t>List logs — non-admin denied</t>
+          <t>Password mismatch validation</t>
         </is>
       </c>
       <c r="D179" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs with non-admin token</t>
+          <t>In password dialog enter different values in password and confirm fields</t>
         </is>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN; denied audit event recorded</t>
+          <t>Inline mismatch message appears and submit remains disabled</t>
         </is>
       </c>
       <c r="F179" s="4" t="n"/>
@@ -5703,27 +5703,27 @@
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>TC-1013</t>
+          <t>TC-916</t>
         </is>
       </c>
       <c r="B180" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.9.1 UI Validation Checklist — Create User Modal Flow</t>
         </is>
       </c>
       <c r="C180" s="4" t="inlineStr">
         <is>
-          <t>List logs — response envelope</t>
+          <t>Show/hide password toggle</t>
         </is>
       </c>
       <c r="D180" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs with admin token and file logging configured</t>
+          <t>In password dialog click show/hide control</t>
         </is>
       </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
-          <t>200 object with log_files array and total_size; no log_directory field in response</t>
+          <t>Password field visibility toggles between masked and plain text</t>
         </is>
       </c>
       <c r="F180" s="4" t="n"/>
@@ -5734,27 +5734,27 @@
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>TC-1014</t>
+          <t>TC-917</t>
         </is>
       </c>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.9.1 UI Validation Checklist — Create User Modal Flow</t>
         </is>
       </c>
       <c r="C181" s="4" t="inlineStr">
         <is>
-          <t>Download log — non-admin denied</t>
+          <t>New user completion</t>
         </is>
       </c>
       <c r="D181" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/app.log with non-admin token</t>
+          <t>Enter matching password/confirm values and submit</t>
         </is>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN; denied audit event recorded</t>
+          <t>Dialog closes and newly created user appears in Users list with expected roles</t>
         </is>
       </c>
       <c r="F181" s="4" t="n"/>
@@ -5765,27 +5765,27 @@
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>TC-1015</t>
+          <t>TC-918</t>
         </is>
       </c>
       <c r="B182" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.9.1 UI Validation Checklist — Create User Modal Flow</t>
         </is>
       </c>
       <c r="C182" s="4" t="inlineStr">
         <is>
-          <t>Download log — path traversal blocked</t>
+          <t>Directory-backed visibility</t>
         </is>
       </c>
       <c r="D182" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/../../../etc/passwd</t>
+          <t>Link a directory-backed user with DB roles and refresh Users page</t>
         </is>
       </c>
       <c r="E182" s="4" t="inlineStr">
         <is>
-          <t>Rejected (400/404/422), no file disclosure</t>
+          <t>User is visible in list even if host-level fields are placeholders</t>
         </is>
       </c>
       <c r="F182" s="4" t="n"/>
@@ -5794,79 +5794,79 @@
       <c r="I182" s="4" t="n"/>
     </row>
     <row r="183">
-      <c r="A183" s="4" t="inlineStr">
-        <is>
-          <t>TC-1016</t>
-        </is>
-      </c>
-      <c r="B183" s="4" t="inlineStr">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>§12.10 Admin Log Viewing API</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
         <is>
           <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
-      <c r="C183" s="4" t="inlineStr">
-        <is>
-          <t>Download log — success audit</t>
-        </is>
-      </c>
-      <c r="D183" s="4" t="inlineStr">
-        <is>
-          <t>Download valid file as admin, then query audit</t>
-        </is>
-      </c>
-      <c r="E183" s="4" t="inlineStr">
-        <is>
-          <t>LOG_FILE_DOWNLOADED entry includes requested filename</t>
-        </is>
-      </c>
-      <c r="F183" s="4" t="n"/>
-      <c r="G183" s="4" t="n"/>
-      <c r="H183" s="4" t="n"/>
-      <c r="I183" s="4" t="n"/>
+      <c r="C183" s="3" t="n"/>
+      <c r="D183" s="3" t="n"/>
+      <c r="E183" s="3" t="n"/>
+      <c r="F183" s="3" t="n"/>
+      <c r="G183" s="3" t="n"/>
+      <c r="H183" s="3" t="n"/>
+      <c r="I183" s="3" t="n"/>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="inlineStr">
-        <is>
-          <t>§12.11 First-Run Setup</t>
-        </is>
-      </c>
-      <c r="B184" s="2" t="inlineStr">
-        <is>
-          <t>12.11 First-Run Setup</t>
-        </is>
-      </c>
-      <c r="C184" s="3" t="n"/>
-      <c r="D184" s="3" t="n"/>
-      <c r="E184" s="3" t="n"/>
-      <c r="F184" s="3" t="n"/>
-      <c r="G184" s="3" t="n"/>
-      <c r="H184" s="3" t="n"/>
-      <c r="I184" s="3" t="n"/>
+      <c r="A184" s="4" t="inlineStr">
+        <is>
+          <t>TC-1001</t>
+        </is>
+      </c>
+      <c r="B184" s="4" t="inlineStr">
+        <is>
+          <t>12.10 Admin Log Viewing API</t>
+        </is>
+      </c>
+      <c r="C184" s="4" t="inlineStr">
+        <is>
+          <t>View logs — unauthenticated</t>
+        </is>
+      </c>
+      <c r="D184" s="4" t="inlineStr">
+        <is>
+          <t>GET /admin/logs/view without token</t>
+        </is>
+      </c>
+      <c r="E184" s="4" t="inlineStr">
+        <is>
+          <t>401, UNAUTHORIZED</t>
+        </is>
+      </c>
+      <c r="F184" s="4" t="n"/>
+      <c r="G184" s="4" t="n"/>
+      <c r="H184" s="4" t="n"/>
+      <c r="I184" s="4" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>TC-1101</t>
+          <t>TC-1002</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C185" s="4" t="inlineStr">
         <is>
-          <t>Status — not initialized</t>
+          <t>View logs — non-admin denied</t>
         </is>
       </c>
       <c r="D185" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/status on fresh database</t>
+          <t>GET /admin/logs/view with manager/processor/auditor token</t>
         </is>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>200, {"initialized": false}</t>
+          <t>403, FORBIDDEN; denied audit event recorded</t>
         </is>
       </c>
       <c r="F185" s="4" t="n"/>
@@ -5877,27 +5877,27 @@
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>TC-1102</t>
+          <t>TC-1003</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C186" s="4" t="inlineStr">
         <is>
-          <t>Initialize</t>
+          <t>View logs — unknown source</t>
         </is>
       </c>
       <c r="D186" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with valid username and password</t>
+          <t>GET /admin/logs/view?source=unknown with admin token</t>
         </is>
       </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
-          <t>200, returns message, username, groups_created</t>
+          <t>404, unknown log source</t>
         </is>
       </c>
       <c r="F186" s="4" t="n"/>
@@ -5908,27 +5908,27 @@
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>TC-1103</t>
+          <t>TC-1004</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C187" s="4" t="inlineStr">
         <is>
-          <t>Status — initialized</t>
+          <t>View logs — baseline response shape</t>
         </is>
       </c>
       <c r="D187" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/status after initialization</t>
+          <t>GET /admin/logs/view?source=app&amp;limit=5&amp;offset=0</t>
         </is>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>200, {"initialized": true}</t>
+          <t>200 with object fields: source, fetched_at, file_modified_at, offset, limit, returned, has_more, lines</t>
         </is>
       </c>
       <c r="F187" s="4" t="n"/>
@@ -5939,27 +5939,27 @@
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>TC-1104</t>
+          <t>TC-1005</t>
         </is>
       </c>
       <c r="B188" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C188" s="4" t="inlineStr">
         <is>
-          <t>Re-initialize rejected</t>
+          <t>View logs — source path redaction</t>
         </is>
       </c>
       <c r="D188" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize again</t>
+          <t>Inspect source.path in successful response</t>
         </is>
       </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
-          <t>409, Conflict</t>
+          <t>Basename only (for example app.log), no absolute filesystem path</t>
         </is>
       </c>
       <c r="F188" s="4" t="n"/>
@@ -5970,27 +5970,27 @@
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>TC-1105</t>
+          <t>TC-1006</t>
         </is>
       </c>
       <c r="B189" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C189" s="4" t="inlineStr">
         <is>
-          <t>Invalid username</t>
+          <t>View logs — offset pagination</t>
         </is>
       </c>
       <c r="D189" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with uppercase or special chars</t>
+          <t>Create known numbered lines, call GET /admin/logs/view?limit=5&amp;offset=2</t>
         </is>
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>Returns correct window from tail semantics, returned &lt;= limit</t>
         </is>
       </c>
       <c r="F189" s="4" t="n"/>
@@ -6001,27 +6001,27 @@
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>TC-1106</t>
+          <t>TC-1007</t>
         </is>
       </c>
       <c r="B190" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C190" s="4" t="inlineStr">
         <is>
-          <t>Empty password</t>
+          <t>View logs — reverse ordering</t>
         </is>
       </c>
       <c r="D190" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with {"password": ""}</t>
+          <t>Compare reverse=false vs reverse=true on same query</t>
         </is>
       </c>
       <c r="E190" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>Same selected window; line order is inverted when reverse=true</t>
         </is>
       </c>
       <c r="F190" s="4" t="n"/>
@@ -6032,27 +6032,27 @@
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>TC-1107</t>
+          <t>TC-1008</t>
         </is>
       </c>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C191" s="4" t="inlineStr">
         <is>
-          <t>Unsafe password chars</t>
+          <t>View logs — search filtering</t>
         </is>
       </c>
       <c r="D191" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with password containing newline or colon</t>
+          <t>GET /admin/logs/view?search=error</t>
         </is>
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>Only matching lines are returned (case-insensitive contains)</t>
         </is>
       </c>
       <c r="F191" s="4" t="n"/>
@@ -6063,27 +6063,27 @@
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>TC-1108</t>
+          <t>TC-1009</t>
         </is>
       </c>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C192" s="4" t="inlineStr">
         <is>
-          <t>Login as initialized admin</t>
+          <t>View logs — sensitive value redaction</t>
         </is>
       </c>
       <c r="D192" s="4" t="inlineStr">
         <is>
-          <t>POST /auth/token with the admin credentials from step 2</t>
+          <t>Include tokens/passwords in source log lines, call view endpoint</t>
         </is>
       </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
-          <t>200, JWT contains admin role</t>
+          <t>Sensitive values replaced with redacted markers in lines[].content</t>
         </is>
       </c>
       <c r="F192" s="4" t="n"/>
@@ -6094,27 +6094,27 @@
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>TC-1109</t>
+          <t>TC-1010</t>
         </is>
       </c>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C193" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM_INITIALIZED audit log</t>
+          <t>View logs — success audit</t>
         </is>
       </c>
       <c r="D193" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
+          <t>GET /audit?action=LOG_LINES_VIEWED after successful view</t>
         </is>
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor</t>
+          <t>Audit entry includes source, limit, offset, returned, has_more, and basename log_file</t>
         </is>
       </c>
       <c r="F193" s="4" t="n"/>
@@ -6123,48 +6123,60 @@
       <c r="I193" s="4" t="n"/>
     </row>
     <row r="194">
-      <c r="A194" s="2" t="inlineStr">
-        <is>
-          <t>§12.12 Database Provisioning</t>
-        </is>
-      </c>
-      <c r="B194" s="2" t="inlineStr">
-        <is>
-          <t>12.12 Database Provisioning</t>
-        </is>
-      </c>
-      <c r="C194" s="3" t="n"/>
-      <c r="D194" s="3" t="n"/>
-      <c r="E194" s="3" t="n"/>
-      <c r="F194" s="3" t="n"/>
-      <c r="G194" s="3" t="n"/>
-      <c r="H194" s="3" t="n"/>
-      <c r="I194" s="3" t="n"/>
+      <c r="A194" s="4" t="inlineStr">
+        <is>
+          <t>TC-1011</t>
+        </is>
+      </c>
+      <c r="B194" s="4" t="inlineStr">
+        <is>
+          <t>12.10 Admin Log Viewing API</t>
+        </is>
+      </c>
+      <c r="C194" s="4" t="inlineStr">
+        <is>
+          <t>List logs — unauthenticated</t>
+        </is>
+      </c>
+      <c r="D194" s="4" t="inlineStr">
+        <is>
+          <t>GET /admin/logs without token</t>
+        </is>
+      </c>
+      <c r="E194" s="4" t="inlineStr">
+        <is>
+          <t>401, UNAUTHORIZED</t>
+        </is>
+      </c>
+      <c r="F194" s="4" t="n"/>
+      <c r="G194" s="4" t="n"/>
+      <c r="H194" s="4" t="n"/>
+      <c r="I194" s="4" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>TC-1201</t>
+          <t>TC-1012</t>
         </is>
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>12.12 Database Provisioning</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr">
         <is>
-          <t>System info — bare-metal defaults</t>
+          <t>List logs — non-admin denied</t>
         </is>
       </c>
       <c r="D195" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/system-info before setup</t>
+          <t>GET /admin/logs with non-admin token</t>
         </is>
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>200, {"in_docker": false, "suggested_db_host": "localhost"}</t>
+          <t>403, FORBIDDEN; denied audit event recorded</t>
         </is>
       </c>
       <c r="F195" s="4" t="n"/>
@@ -6175,27 +6187,27 @@
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>TC-1202</t>
+          <t>TC-1013</t>
         </is>
       </c>
       <c r="B196" s="4" t="inlineStr">
         <is>
-          <t>12.12 Database Provisioning</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C196" s="4" t="inlineStr">
         <is>
-          <t>Provision status — pre-init public</t>
+          <t>List logs — response envelope</t>
         </is>
       </c>
       <c r="D196" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/provision-status before any admin exists</t>
+          <t>GET /admin/logs with admin token and file logging configured</t>
         </is>
       </c>
       <c r="E196" s="4" t="inlineStr">
         <is>
-          <t>200, {"provisioned": false}</t>
+          <t>200 object with log_files array and total_size; no log_directory field in response</t>
         </is>
       </c>
       <c r="F196" s="4" t="n"/>
@@ -6206,27 +6218,27 @@
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>TC-1203</t>
+          <t>TC-1014</t>
         </is>
       </c>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>12.12 Database Provisioning</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C197" s="4" t="inlineStr">
         <is>
-          <t>Provision status — post-init requires admin</t>
+          <t>Download log — non-admin denied</t>
         </is>
       </c>
       <c r="D197" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/provision-status without token after setup</t>
+          <t>GET /admin/logs/app.log with non-admin token</t>
         </is>
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>403, FORBIDDEN; denied audit event recorded</t>
         </is>
       </c>
       <c r="F197" s="4" t="n"/>
@@ -6237,27 +6249,27 @@
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>TC-1204</t>
+          <t>TC-1015</t>
         </is>
       </c>
       <c r="B198" s="4" t="inlineStr">
         <is>
-          <t>12.12 Database Provisioning</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C198" s="4" t="inlineStr">
         <is>
-          <t>Provision status — state unknown</t>
+          <t>Download log — path traversal blocked</t>
         </is>
       </c>
       <c r="D198" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, GET /setup/database/provision-status during initial setup</t>
+          <t>GET /admin/logs/../../../etc/passwd</t>
         </is>
       </c>
       <c r="E198" s="4" t="inlineStr">
         <is>
-          <t>503, cannot determine provisioning state</t>
+          <t>Rejected (400/404/422), no file disclosure</t>
         </is>
       </c>
       <c r="F198" s="4" t="n"/>
@@ -6268,27 +6280,27 @@
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>TC-1205</t>
+          <t>TC-1016</t>
         </is>
       </c>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>12.12 Database Provisioning</t>
+          <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
       <c r="C199" s="4" t="inlineStr">
         <is>
-          <t>Test connection — success</t>
+          <t>Download log — success audit</t>
         </is>
       </c>
       <c r="D199" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with valid PostgreSQL credentials</t>
+          <t>Download valid file as admin, then query audit</t>
         </is>
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>200, {"status": "ok", "server_version": "..."}</t>
+          <t>LOG_FILE_DOWNLOADED entry includes requested filename</t>
         </is>
       </c>
       <c r="F199" s="4" t="n"/>
@@ -6297,60 +6309,48 @@
       <c r="I199" s="4" t="n"/>
     </row>
     <row r="200">
-      <c r="A200" s="4" t="inlineStr">
-        <is>
-          <t>TC-1206</t>
-        </is>
-      </c>
-      <c r="B200" s="4" t="inlineStr">
-        <is>
-          <t>12.12 Database Provisioning</t>
-        </is>
-      </c>
-      <c r="C200" s="4" t="inlineStr">
-        <is>
-          <t>Test connection — bad host</t>
-        </is>
-      </c>
-      <c r="D200" s="4" t="inlineStr">
-        <is>
-          <t>POST /setup/database/test-connection with unreachable host</t>
-        </is>
-      </c>
-      <c r="E200" s="4" t="inlineStr">
-        <is>
-          <t>400, connection error</t>
-        </is>
-      </c>
-      <c r="F200" s="4" t="n"/>
-      <c r="G200" s="4" t="n"/>
-      <c r="H200" s="4" t="n"/>
-      <c r="I200" s="4" t="n"/>
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>§12.11 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>12.11 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C200" s="3" t="n"/>
+      <c r="D200" s="3" t="n"/>
+      <c r="E200" s="3" t="n"/>
+      <c r="F200" s="3" t="n"/>
+      <c r="G200" s="3" t="n"/>
+      <c r="H200" s="3" t="n"/>
+      <c r="I200" s="3" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
         <is>
-          <t>TC-1207</t>
+          <t>TC-1101</t>
         </is>
       </c>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t>12.12 Database Provisioning</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C201" s="4" t="inlineStr">
         <is>
-          <t>Test connection — SSRF host</t>
+          <t>Status — not initialized</t>
         </is>
       </c>
       <c r="D201" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with "host": "http://evil.com"</t>
+          <t>GET /setup/status on fresh database</t>
         </is>
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>422, invalid host</t>
+          <t>200, {"initialized": false}</t>
         </is>
       </c>
       <c r="F201" s="4" t="n"/>
@@ -6361,27 +6361,27 @@
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>TC-1208</t>
+          <t>TC-1102</t>
         </is>
       </c>
       <c r="B202" s="4" t="inlineStr">
         <is>
-          <t>12.12 Database Provisioning</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C202" s="4" t="inlineStr">
         <is>
-          <t>Test connection — port out of range</t>
+          <t>Initialize</t>
         </is>
       </c>
       <c r="D202" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with "port": 99999</t>
+          <t>POST /setup/initialize with valid username and password</t>
         </is>
       </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>200, returns message, username, groups_created</t>
         </is>
       </c>
       <c r="F202" s="4" t="n"/>
@@ -6392,27 +6392,27 @@
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>TC-1209</t>
+          <t>TC-1103</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>12.12 Database Provisioning</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C203" s="4" t="inlineStr">
         <is>
-          <t>Provision — success</t>
+          <t>Status — initialized</t>
         </is>
       </c>
       <c r="D203" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with valid credentials</t>
+          <t>GET /setup/status after initialization</t>
         </is>
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
-          <t>200, returns database, user, migrations_applied</t>
+          <t>200, {"initialized": true}</t>
         </is>
       </c>
       <c r="F203" s="4" t="n"/>
@@ -6423,27 +6423,27 @@
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>TC-1210</t>
+          <t>TC-1104</t>
         </is>
       </c>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t>12.12 Database Provisioning</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C204" s="4" t="inlineStr">
         <is>
-          <t>Provision — bad admin credentials</t>
+          <t>Re-initialize rejected</t>
         </is>
       </c>
       <c r="D204" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with wrong admin password</t>
+          <t>POST /setup/initialize again</t>
         </is>
       </c>
       <c r="E204" s="4" t="inlineStr">
         <is>
-          <t>400, connection error</t>
+          <t>409, Conflict</t>
         </is>
       </c>
       <c r="F204" s="4" t="n"/>
@@ -6454,27 +6454,27 @@
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>TC-1211</t>
+          <t>TC-1105</t>
         </is>
       </c>
       <c r="B205" s="4" t="inlineStr">
         <is>
-          <t>12.12 Database Provisioning</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C205" s="4" t="inlineStr">
         <is>
-          <t>Provision — invalid database name</t>
+          <t>Invalid username</t>
         </is>
       </c>
       <c r="D205" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with "app_database": "drop;--"</t>
+          <t>POST /setup/initialize with uppercase or special chars</t>
         </is>
       </c>
       <c r="E205" s="4" t="inlineStr">
         <is>
-          <t>422, invalid identifier</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F205" s="4" t="n"/>
@@ -6485,27 +6485,27 @@
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
         <is>
-          <t>TC-1212</t>
+          <t>TC-1106</t>
         </is>
       </c>
       <c r="B206" s="4" t="inlineStr">
         <is>
-          <t>12.12 Database Provisioning</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C206" s="4" t="inlineStr">
         <is>
-          <t>Status — connected</t>
+          <t>Empty password</t>
         </is>
       </c>
       <c r="D206" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/status with admin token</t>
+          <t>POST /setup/initialize with {"password": ""}</t>
         </is>
       </c>
       <c r="E206" s="4" t="inlineStr">
         <is>
-          <t>200, connected: true, migration info</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F206" s="4" t="n"/>
@@ -6516,27 +6516,27 @@
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t>TC-1213</t>
+          <t>TC-1107</t>
         </is>
       </c>
       <c r="B207" s="4" t="inlineStr">
         <is>
-          <t>12.12 Database Provisioning</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C207" s="4" t="inlineStr">
         <is>
-          <t>Status — requires auth</t>
+          <t>Unsafe password chars</t>
         </is>
       </c>
       <c r="D207" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/status without token</t>
+          <t>POST /setup/initialize with password containing newline or colon</t>
         </is>
       </c>
       <c r="E207" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>422, unsafe characters</t>
         </is>
       </c>
       <c r="F207" s="4" t="n"/>
@@ -6547,27 +6547,27 @@
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
         <is>
-          <t>TC-1214</t>
+          <t>TC-1108</t>
         </is>
       </c>
       <c r="B208" s="4" t="inlineStr">
         <is>
-          <t>12.12 Database Provisioning</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C208" s="4" t="inlineStr">
         <is>
-          <t>Status — requires admin</t>
+          <t>Login as initialized admin</t>
         </is>
       </c>
       <c r="D208" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/status with processor token</t>
+          <t>POST /auth/token with the admin credentials from step 2</t>
         </is>
       </c>
       <c r="E208" s="4" t="inlineStr">
         <is>
-          <t>403</t>
+          <t>200, JWT contains admin role</t>
         </is>
       </c>
       <c r="F208" s="4" t="n"/>
@@ -6578,27 +6578,27 @@
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
         <is>
-          <t>TC-1215</t>
+          <t>TC-1109</t>
         </is>
       </c>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>12.12 Database Provisioning</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C209" s="4" t="inlineStr">
         <is>
-          <t>Settings update — success</t>
+          <t>SYSTEM_INITIALIZED audit log</t>
         </is>
       </c>
       <c r="D209" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with valid partial update</t>
+          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
         </is>
       </c>
       <c r="E209" s="4" t="inlineStr">
         <is>
-          <t>200, {"status": "updated", ...}</t>
+          <t>Audit entry with actor</t>
         </is>
       </c>
       <c r="F209" s="4" t="n"/>
@@ -6607,40 +6607,28 @@
       <c r="I209" s="4" t="n"/>
     </row>
     <row r="210">
-      <c r="A210" s="4" t="inlineStr">
-        <is>
-          <t>TC-1216</t>
-        </is>
-      </c>
-      <c r="B210" s="4" t="inlineStr">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>§12.12 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
         <is>
           <t>12.12 Database Provisioning</t>
         </is>
       </c>
-      <c r="C210" s="4" t="inlineStr">
-        <is>
-          <t>Settings update — bad connection</t>
-        </is>
-      </c>
-      <c r="D210" s="4" t="inlineStr">
-        <is>
-          <t>PUT /setup/database/settings with unreachable host</t>
-        </is>
-      </c>
-      <c r="E210" s="4" t="inlineStr">
-        <is>
-          <t>400, connection test failed</t>
-        </is>
-      </c>
-      <c r="F210" s="4" t="n"/>
-      <c r="G210" s="4" t="n"/>
-      <c r="H210" s="4" t="n"/>
-      <c r="I210" s="4" t="n"/>
+      <c r="C210" s="3" t="n"/>
+      <c r="D210" s="3" t="n"/>
+      <c r="E210" s="3" t="n"/>
+      <c r="F210" s="3" t="n"/>
+      <c r="G210" s="3" t="n"/>
+      <c r="H210" s="3" t="n"/>
+      <c r="I210" s="3" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
         <is>
-          <t>TC-1217</t>
+          <t>TC-1201</t>
         </is>
       </c>
       <c r="B211" s="4" t="inlineStr">
@@ -6650,17 +6638,17 @@
       </c>
       <c r="C211" s="4" t="inlineStr">
         <is>
-          <t>Settings update — empty body</t>
+          <t>System info — bare-metal defaults</t>
         </is>
       </c>
       <c r="D211" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with {}</t>
+          <t>GET /setup/database/system-info before setup</t>
         </is>
       </c>
       <c r="E211" s="4" t="inlineStr">
         <is>
-          <t>422, at least one field required</t>
+          <t>200, {"in_docker": false, "suggested_db_host": "localhost"}</t>
         </is>
       </c>
       <c r="F211" s="4" t="n"/>
@@ -6671,7 +6659,7 @@
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
         <is>
-          <t>TC-1218</t>
+          <t>TC-1202</t>
         </is>
       </c>
       <c r="B212" s="4" t="inlineStr">
@@ -6681,17 +6669,17 @@
       </c>
       <c r="C212" s="4" t="inlineStr">
         <is>
-          <t>Settings update — requires admin</t>
+          <t>Provision status — pre-init public</t>
         </is>
       </c>
       <c r="D212" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with processor token</t>
+          <t>GET /setup/database/provision-status before any admin exists</t>
         </is>
       </c>
       <c r="E212" s="4" t="inlineStr">
         <is>
-          <t>403</t>
+          <t>200, {"provisioned": false}</t>
         </is>
       </c>
       <c r="F212" s="4" t="n"/>
@@ -6702,7 +6690,7 @@
     <row r="213">
       <c r="A213" s="4" t="inlineStr">
         <is>
-          <t>TC-1219</t>
+          <t>TC-1203</t>
         </is>
       </c>
       <c r="B213" s="4" t="inlineStr">
@@ -6712,12 +6700,12 @@
       </c>
       <c r="C213" s="4" t="inlineStr">
         <is>
-          <t>Auth after setup — test-connection</t>
+          <t>Provision status — post-init requires admin</t>
         </is>
       </c>
       <c r="D213" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection without token (after admin exists)</t>
+          <t>GET /setup/database/provision-status without token after setup</t>
         </is>
       </c>
       <c r="E213" s="4" t="inlineStr">
@@ -6733,7 +6721,7 @@
     <row r="214">
       <c r="A214" s="4" t="inlineStr">
         <is>
-          <t>TC-1220</t>
+          <t>TC-1204</t>
         </is>
       </c>
       <c r="B214" s="4" t="inlineStr">
@@ -6743,17 +6731,17 @@
       </c>
       <c r="C214" s="4" t="inlineStr">
         <is>
-          <t>Auth after setup — provision</t>
+          <t>Provision status — state unknown</t>
         </is>
       </c>
       <c r="D214" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision without token (after admin exists)</t>
+          <t>Stop PostgreSQL, GET /setup/database/provision-status during initial setup</t>
         </is>
       </c>
       <c r="E214" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>503, cannot determine provisioning state</t>
         </is>
       </c>
       <c r="F214" s="4" t="n"/>
@@ -6764,7 +6752,7 @@
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
         <is>
-          <t>TC-1221</t>
+          <t>TC-1205</t>
         </is>
       </c>
       <c r="B215" s="4" t="inlineStr">
@@ -6774,17 +6762,17 @@
       </c>
       <c r="C215" s="4" t="inlineStr">
         <is>
-          <t>Password redaction</t>
+          <t>Test connection — success</t>
         </is>
       </c>
       <c r="D215" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision and check response</t>
+          <t>POST /setup/database/test-connection with valid PostgreSQL credentials</t>
         </is>
       </c>
       <c r="E215" s="4" t="inlineStr">
         <is>
-          <t>No password in response body</t>
+          <t>200, {"status": "ok", "server_version": "..."}</t>
         </is>
       </c>
       <c r="F215" s="4" t="n"/>
@@ -6795,7 +6783,7 @@
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
         <is>
-          <t>TC-1222</t>
+          <t>TC-1206</t>
         </is>
       </c>
       <c r="B216" s="4" t="inlineStr">
@@ -6805,17 +6793,17 @@
       </c>
       <c r="C216" s="4" t="inlineStr">
         <is>
-          <t>Re-provision blocked</t>
+          <t>Test connection — bad host</t>
         </is>
       </c>
       <c r="D216" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision after successful provisioning (no force)</t>
+          <t>POST /setup/database/test-connection with unreachable host</t>
         </is>
       </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
-          <t>409, already provisioned</t>
+          <t>400, connection error</t>
         </is>
       </c>
       <c r="F216" s="4" t="n"/>
@@ -6826,7 +6814,7 @@
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
         <is>
-          <t>TC-1223</t>
+          <t>TC-1207</t>
         </is>
       </c>
       <c r="B217" s="4" t="inlineStr">
@@ -6836,17 +6824,17 @@
       </c>
       <c r="C217" s="4" t="inlineStr">
         <is>
-          <t>Force re-provision (admin)</t>
+          <t>Test connection — SSRF host</t>
         </is>
       </c>
       <c r="D217" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with "force": true and admin token after successful provisioning</t>
+          <t>POST /setup/database/test-connection with "host": "http://evil.com"</t>
         </is>
       </c>
       <c r="E217" s="4" t="inlineStr">
         <is>
-          <t>200, returns database, user, migrations_applied</t>
+          <t>422, invalid host</t>
         </is>
       </c>
       <c r="F217" s="4" t="n"/>
@@ -6857,7 +6845,7 @@
     <row r="218">
       <c r="A218" s="4" t="inlineStr">
         <is>
-          <t>TC-1224</t>
+          <t>TC-1208</t>
         </is>
       </c>
       <c r="B218" s="4" t="inlineStr">
@@ -6867,17 +6855,17 @@
       </c>
       <c r="C218" s="4" t="inlineStr">
         <is>
-          <t>Force rejected unauthenticated</t>
+          <t>Test connection — port out of range</t>
         </is>
       </c>
       <c r="D218" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with "force": true during initial setup (no admin exists)</t>
+          <t>POST /setup/database/test-connection with "port": 99999</t>
         </is>
       </c>
       <c r="E218" s="4" t="inlineStr">
         <is>
-          <t>403, force requires admin</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F218" s="4" t="n"/>
@@ -6888,7 +6876,7 @@
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
         <is>
-          <t>TC-1225</t>
+          <t>TC-1209</t>
         </is>
       </c>
       <c r="B219" s="4" t="inlineStr">
@@ -6898,17 +6886,17 @@
       </c>
       <c r="C219" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — DB unreachable, no JWT</t>
+          <t>Provision — success</t>
         </is>
       </c>
       <c r="D219" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/test-connection without token</t>
+          <t>POST /setup/database/provision with valid credentials</t>
         </is>
       </c>
       <c r="E219" s="4" t="inlineStr">
         <is>
-          <t>503, database unavailable message</t>
+          <t>200, returns database, user, migrations_applied</t>
         </is>
       </c>
       <c r="F219" s="4" t="n"/>
@@ -6919,7 +6907,7 @@
     <row r="220">
       <c r="A220" s="4" t="inlineStr">
         <is>
-          <t>TC-1226</t>
+          <t>TC-1210</t>
         </is>
       </c>
       <c r="B220" s="4" t="inlineStr">
@@ -6929,17 +6917,17 @@
       </c>
       <c r="C220" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — DB unreachable, admin JWT</t>
+          <t>Provision — bad admin credentials</t>
         </is>
       </c>
       <c r="D220" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/test-connection with valid admin token</t>
+          <t>POST /setup/database/provision with wrong admin password</t>
         </is>
       </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
-          <t>Request proceeds (not blocked by 503)</t>
+          <t>400, connection error</t>
         </is>
       </c>
       <c r="F220" s="4" t="n"/>
@@ -6950,7 +6938,7 @@
     <row r="221">
       <c r="A221" s="4" t="inlineStr">
         <is>
-          <t>TC-1227</t>
+          <t>TC-1211</t>
         </is>
       </c>
       <c r="B221" s="4" t="inlineStr">
@@ -6960,17 +6948,17 @@
       </c>
       <c r="C221" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — provision state unknown</t>
+          <t>Provision — invalid database name</t>
         </is>
       </c>
       <c r="D221" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/provision without "force": true</t>
+          <t>POST /setup/database/provision with "app_database": "drop;--"</t>
         </is>
       </c>
       <c r="E221" s="4" t="inlineStr">
         <is>
-          <t>503, cannot determine provisioning state</t>
+          <t>422, invalid identifier</t>
         </is>
       </c>
       <c r="F221" s="4" t="n"/>
@@ -6981,7 +6969,7 @@
     <row r="222">
       <c r="A222" s="4" t="inlineStr">
         <is>
-          <t>TC-1228</t>
+          <t>TC-1212</t>
         </is>
       </c>
       <c r="B222" s="4" t="inlineStr">
@@ -6991,17 +6979,17 @@
       </c>
       <c r="C222" s="4" t="inlineStr">
         <is>
-          <t>Force bypasses state check</t>
+          <t>Status — connected</t>
         </is>
       </c>
       <c r="D222" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/provision with "force": true and admin token</t>
+          <t>GET /setup/database/status with admin token</t>
         </is>
       </c>
       <c r="E222" s="4" t="inlineStr">
         <is>
-          <t>Proceeds to provisioning (no 503 from state check)</t>
+          <t>200, connected: true, migration info</t>
         </is>
       </c>
       <c r="F222" s="4" t="n"/>
@@ -7012,7 +7000,7 @@
     <row r="223">
       <c r="A223" s="4" t="inlineStr">
         <is>
-          <t>TC-1229</t>
+          <t>TC-1213</t>
         </is>
       </c>
       <c r="B223" s="4" t="inlineStr">
@@ -7022,17 +7010,17 @@
       </c>
       <c r="C223" s="4" t="inlineStr">
         <is>
-          <t>Unmigrated DB treated as initial setup</t>
+          <t>Status — requires auth</t>
         </is>
       </c>
       <c r="D223" s="4" t="inlineStr">
         <is>
-          <t>Drop user_roles table (or use a fresh empty database), POST /setup/database/test-connection without token</t>
+          <t>GET /setup/database/status without token</t>
         </is>
       </c>
       <c r="E223" s="4" t="inlineStr">
         <is>
-          <t>200, request allowed (not 503)</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F223" s="4" t="n"/>
@@ -7043,7 +7031,7 @@
     <row r="224">
       <c r="A224" s="4" t="inlineStr">
         <is>
-          <t>TC-1230</t>
+          <t>TC-1214</t>
         </is>
       </c>
       <c r="B224" s="4" t="inlineStr">
@@ -7053,17 +7041,17 @@
       </c>
       <c r="C224" s="4" t="inlineStr">
         <is>
-          <t>Fresh install — DB/role missing</t>
+          <t>Status — requires admin</t>
         </is>
       </c>
       <c r="D224" s="4" t="inlineStr">
         <is>
-          <t>With PostgreSQL running but the application database or role not yet created, POST /setup/database/provision without force</t>
+          <t>GET /setup/database/status with processor token</t>
         </is>
       </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
-          <t>200, provisioning proceeds (not 503)</t>
+          <t>403</t>
         </is>
       </c>
       <c r="F224" s="4" t="n"/>
@@ -7074,7 +7062,7 @@
     <row r="225">
       <c r="A225" s="4" t="inlineStr">
         <is>
-          <t>TC-1231</t>
+          <t>TC-1215</t>
         </is>
       </c>
       <c r="B225" s="4" t="inlineStr">
@@ -7084,17 +7072,17 @@
       </c>
       <c r="C225" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — OperationalError on reachable DB</t>
+          <t>Settings update — success</t>
         </is>
       </c>
       <c r="D225" s="4" t="inlineStr">
         <is>
-          <t>Revoke SELECT on user_roles (or simulate permission denied), POST /setup/database/test-connection without token</t>
+          <t>PUT /setup/database/settings with valid partial update</t>
         </is>
       </c>
       <c r="E225" s="4" t="inlineStr">
         <is>
-          <t>503, does NOT grant unauthenticated access</t>
+          <t>200, {"status": "updated", ...}</t>
         </is>
       </c>
       <c r="F225" s="4" t="n"/>
@@ -7105,7 +7093,7 @@
     <row r="226">
       <c r="A226" s="4" t="inlineStr">
         <is>
-          <t>TC-1232</t>
+          <t>TC-1216</t>
         </is>
       </c>
       <c r="B226" s="4" t="inlineStr">
@@ -7115,17 +7103,17 @@
       </c>
       <c r="C226" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — unexpected error</t>
+          <t>Settings update — bad connection</t>
         </is>
       </c>
       <c r="D226" s="4" t="inlineStr">
         <is>
-          <t>Trigger an unexpected exception from admin-check (e.g. coding bug), POST /setup/database/test-connection without token</t>
+          <t>PUT /setup/database/settings with unreachable host</t>
         </is>
       </c>
       <c r="E226" s="4" t="inlineStr">
         <is>
-          <t>503, does NOT grant unauthenticated access</t>
+          <t>400, connection test failed</t>
         </is>
       </c>
       <c r="F226" s="4" t="n"/>
@@ -7136,7 +7124,7 @@
     <row r="227">
       <c r="A227" s="4" t="inlineStr">
         <is>
-          <t>TC-1233</t>
+          <t>TC-1217</t>
         </is>
       </c>
       <c r="B227" s="4" t="inlineStr">
@@ -7146,17 +7134,17 @@
       </c>
       <c r="C227" s="4" t="inlineStr">
         <is>
-          <t>Provision — migration failure</t>
+          <t>Settings update — empty body</t>
         </is>
       </c>
       <c r="D227" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with valid credentials but a broken Alembic migration (e.g. conflicting schema)</t>
+          <t>PUT /setup/database/settings with {}</t>
         </is>
       </c>
       <c r="E227" s="4" t="inlineStr">
         <is>
-          <t>500, "migration failed" message; .env not updated, engine not swapped</t>
+          <t>422, at least one field required</t>
         </is>
       </c>
       <c r="F227" s="4" t="n"/>
@@ -7167,7 +7155,7 @@
     <row r="228">
       <c r="A228" s="4" t="inlineStr">
         <is>
-          <t>TC-1234</t>
+          <t>TC-1218</t>
         </is>
       </c>
       <c r="B228" s="4" t="inlineStr">
@@ -7177,17 +7165,17 @@
       </c>
       <c r="C228" s="4" t="inlineStr">
         <is>
-          <t>Provision — .env write failure</t>
+          <t>Settings update — requires admin</t>
         </is>
       </c>
       <c r="D228" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision after making .env read-only (or disk full)</t>
+          <t>PUT /setup/database/settings with processor token</t>
         </is>
       </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
-          <t>500, "failed to persist" message; engine not swapped</t>
+          <t>403</t>
         </is>
       </c>
       <c r="F228" s="4" t="n"/>
@@ -7198,7 +7186,7 @@
     <row r="229">
       <c r="A229" s="4" t="inlineStr">
         <is>
-          <t>TC-1235</t>
+          <t>TC-1219</t>
         </is>
       </c>
       <c r="B229" s="4" t="inlineStr">
@@ -7208,17 +7196,17 @@
       </c>
       <c r="C229" s="4" t="inlineStr">
         <is>
-          <t>Provision — engine reinit failure</t>
+          <t>Auth after setup — test-connection</t>
         </is>
       </c>
       <c r="D229" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision while another reinit is in progress (lock contention)</t>
+          <t>POST /setup/database/test-connection without token (after admin exists)</t>
         </is>
       </c>
       <c r="E229" s="4" t="inlineStr">
         <is>
-          <t>500, "engine could not be switched" message; .env already written</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F229" s="4" t="n"/>
@@ -7227,48 +7215,60 @@
       <c r="I229" s="4" t="n"/>
     </row>
     <row r="230">
-      <c r="A230" s="2" t="inlineStr">
-        <is>
-          <t>§12.13 Startup State Reconciliation</t>
-        </is>
-      </c>
-      <c r="B230" s="2" t="inlineStr">
-        <is>
-          <t>12.13 Startup State Reconciliation</t>
-        </is>
-      </c>
-      <c r="C230" s="3" t="n"/>
-      <c r="D230" s="3" t="n"/>
-      <c r="E230" s="3" t="n"/>
-      <c r="F230" s="3" t="n"/>
-      <c r="G230" s="3" t="n"/>
-      <c r="H230" s="3" t="n"/>
-      <c r="I230" s="3" t="n"/>
+      <c r="A230" s="4" t="inlineStr">
+        <is>
+          <t>TC-1220</t>
+        </is>
+      </c>
+      <c r="B230" s="4" t="inlineStr">
+        <is>
+          <t>12.12 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C230" s="4" t="inlineStr">
+        <is>
+          <t>Auth after setup — provision</t>
+        </is>
+      </c>
+      <c r="D230" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision without token (after admin exists)</t>
+        </is>
+      </c>
+      <c r="E230" s="4" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="F230" s="4" t="n"/>
+      <c r="G230" s="4" t="n"/>
+      <c r="H230" s="4" t="n"/>
+      <c r="I230" s="4" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
         <is>
-          <t>TC-1301</t>
+          <t>TC-1221</t>
         </is>
       </c>
       <c r="B231" s="4" t="inlineStr">
         <is>
-          <t>12.13 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C231" s="4" t="inlineStr">
         <is>
-          <t>Running job failed after restart</t>
+          <t>Password redaction</t>
         </is>
       </c>
       <c r="D231" s="4" t="inlineStr">
         <is>
-          <t>Create a job, start it, restart the service while RUNNING</t>
+          <t>POST /setup/database/provision and check response</t>
         </is>
       </c>
       <c r="E231" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
+          <t>No password in response body</t>
         </is>
       </c>
       <c r="F231" s="4" t="n"/>
@@ -7279,27 +7279,27 @@
     <row r="232">
       <c r="A232" s="4" t="inlineStr">
         <is>
-          <t>TC-1302</t>
+          <t>TC-1222</t>
         </is>
       </c>
       <c r="B232" s="4" t="inlineStr">
         <is>
-          <t>12.13 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C232" s="4" t="inlineStr">
         <is>
-          <t>Verifying job failed after restart</t>
+          <t>Re-provision blocked</t>
         </is>
       </c>
       <c r="D232" s="4" t="inlineStr">
         <is>
-          <t>Start a job, let it reach VERIFYING, restart the service</t>
+          <t>POST /setup/database/provision after successful provisioning (no force)</t>
         </is>
       </c>
       <c r="E232" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
+          <t>409, already provisioned</t>
         </is>
       </c>
       <c r="F232" s="4" t="n"/>
@@ -7310,27 +7310,27 @@
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
         <is>
-          <t>TC-1303</t>
+          <t>TC-1223</t>
         </is>
       </c>
       <c r="B233" s="4" t="inlineStr">
         <is>
-          <t>12.13 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C233" s="4" t="inlineStr">
         <is>
-          <t>Pending job not affected</t>
+          <t>Force re-provision (admin)</t>
         </is>
       </c>
       <c r="D233" s="4" t="inlineStr">
         <is>
-          <t>Create a job (PENDING), restart the service</t>
+          <t>POST /setup/database/provision with "force": true and admin token after successful provisioning</t>
         </is>
       </c>
       <c r="E233" s="4" t="inlineStr">
         <is>
-          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
+          <t>200, returns database, user, migrations_applied</t>
         </is>
       </c>
       <c r="F233" s="4" t="n"/>
@@ -7341,27 +7341,27 @@
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
         <is>
-          <t>TC-1304</t>
+          <t>TC-1224</t>
         </is>
       </c>
       <c r="B234" s="4" t="inlineStr">
         <is>
-          <t>12.13 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C234" s="4" t="inlineStr">
         <is>
-          <t>Completed job not affected</t>
+          <t>Force rejected unauthenticated</t>
         </is>
       </c>
       <c r="D234" s="4" t="inlineStr">
         <is>
-          <t>Complete a job, restart the service</t>
+          <t>POST /setup/database/provision with "force": true during initial setup (no admin exists)</t>
         </is>
       </c>
       <c r="E234" s="4" t="inlineStr">
         <is>
-          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
+          <t>403, force requires admin</t>
         </is>
       </c>
       <c r="F234" s="4" t="n"/>
@@ -7372,27 +7372,27 @@
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
         <is>
-          <t>TC-1305</t>
+          <t>TC-1225</t>
         </is>
       </c>
       <c r="B235" s="4" t="inlineStr">
         <is>
-          <t>12.13 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C235" s="4" t="inlineStr">
         <is>
-          <t>Stale mount corrected</t>
+          <t>Fail-closed — DB unreachable, no JWT</t>
         </is>
       </c>
       <c r="D235" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
+          <t>Stop PostgreSQL, POST /setup/database/test-connection without token</t>
         </is>
       </c>
       <c r="E235" s="4" t="inlineStr">
         <is>
-          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
+          <t>503, database unavailable message</t>
         </is>
       </c>
       <c r="F235" s="4" t="n"/>
@@ -7403,27 +7403,27 @@
     <row r="236">
       <c r="A236" s="4" t="inlineStr">
         <is>
-          <t>TC-1306</t>
+          <t>TC-1226</t>
         </is>
       </c>
       <c r="B236" s="4" t="inlineStr">
         <is>
-          <t>12.13 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C236" s="4" t="inlineStr">
         <is>
-          <t>Active mount preserved</t>
+          <t>Fail-closed — DB unreachable, admin JWT</t>
         </is>
       </c>
       <c r="D236" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share (leave it mounted), restart the service</t>
+          <t>Stop PostgreSQL, POST /setup/database/test-connection with valid admin token</t>
         </is>
       </c>
       <c r="E236" s="4" t="inlineStr">
         <is>
-          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
+          <t>Request proceeds (not blocked by 503)</t>
         </is>
       </c>
       <c r="F236" s="4" t="n"/>
@@ -7434,27 +7434,27 @@
     <row r="237">
       <c r="A237" s="4" t="inlineStr">
         <is>
-          <t>TC-1307</t>
+          <t>TC-1227</t>
         </is>
       </c>
       <c r="B237" s="4" t="inlineStr">
         <is>
-          <t>12.13 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C237" s="4" t="inlineStr">
         <is>
-          <t>USB drives re-discovered</t>
+          <t>Fail-closed — provision state unknown</t>
         </is>
       </c>
       <c r="D237" s="4" t="inlineStr">
         <is>
-          <t>Insert USB drives, restart the service</t>
+          <t>Stop PostgreSQL, POST /setup/database/provision without "force": true</t>
         </is>
       </c>
       <c r="E237" s="4" t="inlineStr">
         <is>
-          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
+          <t>503, cannot determine provisioning state</t>
         </is>
       </c>
       <c r="F237" s="4" t="n"/>
@@ -7465,27 +7465,27 @@
     <row r="238">
       <c r="A238" s="4" t="inlineStr">
         <is>
-          <t>TC-1308</t>
+          <t>TC-1228</t>
         </is>
       </c>
       <c r="B238" s="4" t="inlineStr">
         <is>
-          <t>12.13 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C238" s="4" t="inlineStr">
         <is>
-          <t>Idempotency</t>
+          <t>Force bypasses state check</t>
         </is>
       </c>
       <c r="D238" s="4" t="inlineStr">
         <is>
-          <t>Restart the service twice without any state changes between restarts</t>
+          <t>Stop PostgreSQL, POST /setup/database/provision with "force": true and admin token</t>
         </is>
       </c>
       <c r="E238" s="4" t="inlineStr">
         <is>
-          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
+          <t>Proceeds to provisioning (no 503 from state check)</t>
         </is>
       </c>
       <c r="F238" s="4" t="n"/>
@@ -7496,27 +7496,27 @@
     <row r="239">
       <c r="A239" s="4" t="inlineStr">
         <is>
-          <t>TC-1309</t>
+          <t>TC-1229</t>
         </is>
       </c>
       <c r="B239" s="4" t="inlineStr">
         <is>
-          <t>12.13 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C239" s="4" t="inlineStr">
         <is>
-          <t>Partial failure isolation</t>
+          <t>Unmigrated DB treated as initial setup</t>
         </is>
       </c>
       <c r="D239" s="4" t="inlineStr">
         <is>
-          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
+          <t>Drop user_roles table (or use a fresh empty database), POST /setup/database/test-connection without token</t>
         </is>
       </c>
       <c r="E239" s="4" t="inlineStr">
         <is>
-          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
+          <t>200, request allowed (not 503)</t>
         </is>
       </c>
       <c r="F239" s="4" t="n"/>
@@ -7527,27 +7527,27 @@
     <row r="240">
       <c r="A240" s="4" t="inlineStr">
         <is>
-          <t>TC-1310</t>
+          <t>TC-1230</t>
         </is>
       </c>
       <c r="B240" s="4" t="inlineStr">
         <is>
-          <t>12.13 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C240" s="4" t="inlineStr">
         <is>
-          <t>Cross-process lock — only one worker reconciles</t>
+          <t>Fresh install — DB/role missing</t>
         </is>
       </c>
       <c r="D240" s="4" t="inlineStr">
         <is>
-          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
+          <t>With PostgreSQL running but the application database or role not yet created, POST /setup/database/provision without force</t>
         </is>
       </c>
       <c r="E240" s="4" t="inlineStr">
         <is>
-          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
+          <t>200, provisioning proceeds (not 503)</t>
         </is>
       </c>
       <c r="F240" s="4" t="n"/>
@@ -7558,27 +7558,27 @@
     <row r="241">
       <c r="A241" s="4" t="inlineStr">
         <is>
-          <t>TC-1311</t>
+          <t>TC-1231</t>
         </is>
       </c>
       <c r="B241" s="4" t="inlineStr">
         <is>
-          <t>12.13 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C241" s="4" t="inlineStr">
         <is>
-          <t>Stale lock reclaim</t>
+          <t>Fail-closed — OperationalError on reachable DB</t>
         </is>
       </c>
       <c r="D241" s="4" t="inlineStr">
         <is>
-          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
+          <t>Revoke SELECT on user_roles (or simulate permission denied), POST /setup/database/test-connection without token</t>
         </is>
       </c>
       <c r="E241" s="4" t="inlineStr">
         <is>
-          <t>Service reclaims the stale lock, reconciliation runs normally</t>
+          <t>503, does NOT grant unauthenticated access</t>
         </is>
       </c>
       <c r="F241" s="4" t="n"/>
@@ -7589,27 +7589,27 @@
     <row r="242">
       <c r="A242" s="4" t="inlineStr">
         <is>
-          <t>TC-1312</t>
+          <t>TC-1232</t>
         </is>
       </c>
       <c r="B242" s="4" t="inlineStr">
         <is>
-          <t>12.13 Startup State Reconciliation</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C242" s="4" t="inlineStr">
         <is>
-          <t>Lock released after failure</t>
+          <t>Fail-closed — unexpected error</t>
         </is>
       </c>
       <c r="D242" s="4" t="inlineStr">
         <is>
-          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
+          <t>Trigger an unexpected exception from admin-check (e.g. coding bug), POST /setup/database/test-connection without token</t>
         </is>
       </c>
       <c r="E242" s="4" t="inlineStr">
         <is>
-          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
+          <t>503, does NOT grant unauthenticated access</t>
         </is>
       </c>
       <c r="F242" s="4" t="n"/>
@@ -7618,48 +7618,60 @@
       <c r="I242" s="4" t="n"/>
     </row>
     <row r="243">
-      <c r="A243" s="2" t="inlineStr">
-        <is>
-          <t>§12.14 System Health</t>
-        </is>
-      </c>
-      <c r="B243" s="2" t="inlineStr">
-        <is>
-          <t>12.14 System Health</t>
-        </is>
-      </c>
-      <c r="C243" s="3" t="n"/>
-      <c r="D243" s="3" t="n"/>
-      <c r="E243" s="3" t="n"/>
-      <c r="F243" s="3" t="n"/>
-      <c r="G243" s="3" t="n"/>
-      <c r="H243" s="3" t="n"/>
-      <c r="I243" s="3" t="n"/>
+      <c r="A243" s="4" t="inlineStr">
+        <is>
+          <t>TC-1233</t>
+        </is>
+      </c>
+      <c r="B243" s="4" t="inlineStr">
+        <is>
+          <t>12.12 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C243" s="4" t="inlineStr">
+        <is>
+          <t>Provision — migration failure</t>
+        </is>
+      </c>
+      <c r="D243" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision with valid credentials but a broken Alembic migration (e.g. conflicting schema)</t>
+        </is>
+      </c>
+      <c r="E243" s="4" t="inlineStr">
+        <is>
+          <t>500, "migration failed" message; .env not updated, engine not swapped</t>
+        </is>
+      </c>
+      <c r="F243" s="4" t="n"/>
+      <c r="G243" s="4" t="n"/>
+      <c r="H243" s="4" t="n"/>
+      <c r="I243" s="4" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="4" t="inlineStr">
         <is>
-          <t>TC-1401</t>
+          <t>TC-1234</t>
         </is>
       </c>
       <c r="B244" s="4" t="inlineStr">
         <is>
-          <t>12.14 System Health</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C244" s="4" t="inlineStr">
         <is>
-          <t>Healthy response</t>
+          <t>Provision — .env write failure</t>
         </is>
       </c>
       <c r="D244" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with valid token</t>
+          <t>POST /setup/database/provision after making .env read-only (or disk full)</t>
         </is>
       </c>
       <c r="E244" s="4" t="inlineStr">
         <is>
-          <t>200, status: "ok", database: "connected"</t>
+          <t>500, "failed to persist" message; engine not swapped</t>
         </is>
       </c>
       <c r="F244" s="4" t="n"/>
@@ -7670,27 +7682,27 @@
     <row r="245">
       <c r="A245" s="4" t="inlineStr">
         <is>
-          <t>TC-1402</t>
+          <t>TC-1235</t>
         </is>
       </c>
       <c r="B245" s="4" t="inlineStr">
         <is>
-          <t>12.14 System Health</t>
+          <t>12.12 Database Provisioning</t>
         </is>
       </c>
       <c r="C245" s="4" t="inlineStr">
         <is>
-          <t>CPU metric present</t>
+          <t>Provision — engine reinit failure</t>
         </is>
       </c>
       <c r="D245" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>POST /setup/database/provision while another reinit is in progress (lock contention)</t>
         </is>
       </c>
       <c r="E245" s="4" t="inlineStr">
         <is>
-          <t>cpu_percent is a number between 0 and 100</t>
+          <t>500, "engine could not be switched" message; .env already written</t>
         </is>
       </c>
       <c r="F245" s="4" t="n"/>
@@ -7699,60 +7711,48 @@
       <c r="I245" s="4" t="n"/>
     </row>
     <row r="246">
-      <c r="A246" s="4" t="inlineStr">
-        <is>
-          <t>TC-1403</t>
-        </is>
-      </c>
-      <c r="B246" s="4" t="inlineStr">
-        <is>
-          <t>12.14 System Health</t>
-        </is>
-      </c>
-      <c r="C246" s="4" t="inlineStr">
-        <is>
-          <t>Memory metrics present</t>
-        </is>
-      </c>
-      <c r="D246" s="4" t="inlineStr">
-        <is>
-          <t>Inspect response body</t>
-        </is>
-      </c>
-      <c r="E246" s="4" t="inlineStr">
-        <is>
-          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
-        </is>
-      </c>
-      <c r="F246" s="4" t="n"/>
-      <c r="G246" s="4" t="n"/>
-      <c r="H246" s="4" t="n"/>
-      <c r="I246" s="4" t="n"/>
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>§12.13 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="B246" s="2" t="inlineStr">
+        <is>
+          <t>12.13 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C246" s="3" t="n"/>
+      <c r="D246" s="3" t="n"/>
+      <c r="E246" s="3" t="n"/>
+      <c r="F246" s="3" t="n"/>
+      <c r="G246" s="3" t="n"/>
+      <c r="H246" s="3" t="n"/>
+      <c r="I246" s="3" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="4" t="inlineStr">
         <is>
-          <t>TC-1404</t>
+          <t>TC-1301</t>
         </is>
       </c>
       <c r="B247" s="4" t="inlineStr">
         <is>
-          <t>12.14 System Health</t>
+          <t>12.13 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C247" s="4" t="inlineStr">
         <is>
-          <t>Disk I/O metrics present</t>
+          <t>Running job failed after restart</t>
         </is>
       </c>
       <c r="D247" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Create a job, start it, restart the service while RUNNING</t>
         </is>
       </c>
       <c r="E247" s="4" t="inlineStr">
         <is>
-          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
+          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
         </is>
       </c>
       <c r="F247" s="4" t="n"/>
@@ -7763,27 +7763,27 @@
     <row r="248">
       <c r="A248" s="4" t="inlineStr">
         <is>
-          <t>TC-1405</t>
+          <t>TC-1302</t>
         </is>
       </c>
       <c r="B248" s="4" t="inlineStr">
         <is>
-          <t>12.14 System Health</t>
+          <t>12.13 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C248" s="4" t="inlineStr">
         <is>
-          <t>Active jobs count</t>
+          <t>Verifying job failed after restart</t>
         </is>
       </c>
       <c r="D248" s="4" t="inlineStr">
         <is>
-          <t>Start an export job, call endpoint</t>
+          <t>Start a job, let it reach VERIFYING, restart the service</t>
         </is>
       </c>
       <c r="E248" s="4" t="inlineStr">
         <is>
-          <t>active_jobs ≥ 1</t>
+          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
         </is>
       </c>
       <c r="F248" s="4" t="n"/>
@@ -7794,27 +7794,27 @@
     <row r="249">
       <c r="A249" s="4" t="inlineStr">
         <is>
-          <t>TC-1406</t>
+          <t>TC-1303</t>
         </is>
       </c>
       <c r="B249" s="4" t="inlineStr">
         <is>
-          <t>12.14 System Health</t>
+          <t>12.13 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C249" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size</t>
+          <t>Pending job not affected</t>
         </is>
       </c>
       <c r="D249" s="4" t="inlineStr">
         <is>
-          <t>Create a PENDING job (created but not started), call endpoint</t>
+          <t>Create a job (PENDING), restart the service</t>
         </is>
       </c>
       <c r="E249" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size ≥ 1</t>
+          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
         </is>
       </c>
       <c r="F249" s="4" t="n"/>
@@ -7825,27 +7825,27 @@
     <row r="250">
       <c r="A250" s="4" t="inlineStr">
         <is>
-          <t>TC-1407</t>
+          <t>TC-1304</t>
         </is>
       </c>
       <c r="B250" s="4" t="inlineStr">
         <is>
-          <t>12.14 System Health</t>
+          <t>12.13 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C250" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size decrements</t>
+          <t>Completed job not affected</t>
         </is>
       </c>
       <c r="D250" s="4" t="inlineStr">
         <is>
-          <t>Start the pending job, call endpoint again</t>
+          <t>Complete a job, restart the service</t>
         </is>
       </c>
       <c r="E250" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
+          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F250" s="4" t="n"/>
@@ -7856,27 +7856,27 @@
     <row r="251">
       <c r="A251" s="4" t="inlineStr">
         <is>
-          <t>TC-1408</t>
+          <t>TC-1305</t>
         </is>
       </c>
       <c r="B251" s="4" t="inlineStr">
         <is>
-          <t>12.14 System Health</t>
+          <t>12.13 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C251" s="4" t="inlineStr">
         <is>
-          <t>Degraded when DB down</t>
+          <t>Stale mount corrected</t>
         </is>
       </c>
       <c r="D251" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, call endpoint with valid token</t>
+          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
         </is>
       </c>
       <c r="E251" s="4" t="inlineStr">
         <is>
-          <t>200, status: "degraded", database: "error", database_error is non-null</t>
+          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
         </is>
       </c>
       <c r="F251" s="4" t="n"/>
@@ -7887,27 +7887,27 @@
     <row r="252">
       <c r="A252" s="4" t="inlineStr">
         <is>
-          <t>TC-1409</t>
+          <t>TC-1306</t>
         </is>
       </c>
       <c r="B252" s="4" t="inlineStr">
         <is>
-          <t>12.14 System Health</t>
+          <t>12.13 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C252" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated rejected</t>
+          <t>Active mount preserved</t>
         </is>
       </c>
       <c r="D252" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health without token</t>
+          <t>Add and mount a network share (leave it mounted), restart the service</t>
         </is>
       </c>
       <c r="E252" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F252" s="4" t="n"/>
@@ -7918,27 +7918,27 @@
     <row r="253">
       <c r="A253" s="4" t="inlineStr">
         <is>
-          <t>TC-1410</t>
+          <t>TC-1307</t>
         </is>
       </c>
       <c r="B253" s="4" t="inlineStr">
         <is>
-          <t>12.14 System Health</t>
+          <t>12.13 Startup State Reconciliation</t>
         </is>
       </c>
       <c r="C253" s="4" t="inlineStr">
         <is>
-          <t>Processor role allowed</t>
+          <t>USB drives re-discovered</t>
         </is>
       </c>
       <c r="D253" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with processor token</t>
+          <t>Insert USB drives, restart the service</t>
         </is>
       </c>
       <c r="E253" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
         </is>
       </c>
       <c r="F253" s="4" t="n"/>
@@ -7946,14 +7946,498 @@
       <c r="H253" s="4" t="n"/>
       <c r="I253" s="4" t="n"/>
     </row>
+    <row r="254">
+      <c r="A254" s="4" t="inlineStr">
+        <is>
+          <t>TC-1308</t>
+        </is>
+      </c>
+      <c r="B254" s="4" t="inlineStr">
+        <is>
+          <t>12.13 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C254" s="4" t="inlineStr">
+        <is>
+          <t>Idempotency</t>
+        </is>
+      </c>
+      <c r="D254" s="4" t="inlineStr">
+        <is>
+          <t>Restart the service twice without any state changes between restarts</t>
+        </is>
+      </c>
+      <c r="E254" s="4" t="inlineStr">
+        <is>
+          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
+        </is>
+      </c>
+      <c r="F254" s="4" t="n"/>
+      <c r="G254" s="4" t="n"/>
+      <c r="H254" s="4" t="n"/>
+      <c r="I254" s="4" t="n"/>
+    </row>
     <row r="255">
-      <c r="A255" s="5" t="inlineStr">
+      <c r="A255" s="4" t="inlineStr">
+        <is>
+          <t>TC-1309</t>
+        </is>
+      </c>
+      <c r="B255" s="4" t="inlineStr">
+        <is>
+          <t>12.13 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C255" s="4" t="inlineStr">
+        <is>
+          <t>Partial failure isolation</t>
+        </is>
+      </c>
+      <c r="D255" s="4" t="inlineStr">
+        <is>
+          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
+        </is>
+      </c>
+      <c r="E255" s="4" t="inlineStr">
+        <is>
+          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
+        </is>
+      </c>
+      <c r="F255" s="4" t="n"/>
+      <c r="G255" s="4" t="n"/>
+      <c r="H255" s="4" t="n"/>
+      <c r="I255" s="4" t="n"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="4" t="inlineStr">
+        <is>
+          <t>TC-1310</t>
+        </is>
+      </c>
+      <c r="B256" s="4" t="inlineStr">
+        <is>
+          <t>12.13 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C256" s="4" t="inlineStr">
+        <is>
+          <t>Cross-process lock — only one worker reconciles</t>
+        </is>
+      </c>
+      <c r="D256" s="4" t="inlineStr">
+        <is>
+          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
+        </is>
+      </c>
+      <c r="E256" s="4" t="inlineStr">
+        <is>
+          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
+        </is>
+      </c>
+      <c r="F256" s="4" t="n"/>
+      <c r="G256" s="4" t="n"/>
+      <c r="H256" s="4" t="n"/>
+      <c r="I256" s="4" t="n"/>
+    </row>
+    <row r="257">
+      <c r="A257" s="4" t="inlineStr">
+        <is>
+          <t>TC-1311</t>
+        </is>
+      </c>
+      <c r="B257" s="4" t="inlineStr">
+        <is>
+          <t>12.13 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C257" s="4" t="inlineStr">
+        <is>
+          <t>Stale lock reclaim</t>
+        </is>
+      </c>
+      <c r="D257" s="4" t="inlineStr">
+        <is>
+          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
+        </is>
+      </c>
+      <c r="E257" s="4" t="inlineStr">
+        <is>
+          <t>Service reclaims the stale lock, reconciliation runs normally</t>
+        </is>
+      </c>
+      <c r="F257" s="4" t="n"/>
+      <c r="G257" s="4" t="n"/>
+      <c r="H257" s="4" t="n"/>
+      <c r="I257" s="4" t="n"/>
+    </row>
+    <row r="258">
+      <c r="A258" s="4" t="inlineStr">
+        <is>
+          <t>TC-1312</t>
+        </is>
+      </c>
+      <c r="B258" s="4" t="inlineStr">
+        <is>
+          <t>12.13 Startup State Reconciliation</t>
+        </is>
+      </c>
+      <c r="C258" s="4" t="inlineStr">
+        <is>
+          <t>Lock released after failure</t>
+        </is>
+      </c>
+      <c r="D258" s="4" t="inlineStr">
+        <is>
+          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
+        </is>
+      </c>
+      <c r="E258" s="4" t="inlineStr">
+        <is>
+          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
+        </is>
+      </c>
+      <c r="F258" s="4" t="n"/>
+      <c r="G258" s="4" t="n"/>
+      <c r="H258" s="4" t="n"/>
+      <c r="I258" s="4" t="n"/>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>§12.14 System Health</t>
+        </is>
+      </c>
+      <c r="B259" s="2" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C259" s="3" t="n"/>
+      <c r="D259" s="3" t="n"/>
+      <c r="E259" s="3" t="n"/>
+      <c r="F259" s="3" t="n"/>
+      <c r="G259" s="3" t="n"/>
+      <c r="H259" s="3" t="n"/>
+      <c r="I259" s="3" t="n"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="4" t="inlineStr">
+        <is>
+          <t>TC-1401</t>
+        </is>
+      </c>
+      <c r="B260" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C260" s="4" t="inlineStr">
+        <is>
+          <t>Healthy response</t>
+        </is>
+      </c>
+      <c r="D260" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/system-health with valid token</t>
+        </is>
+      </c>
+      <c r="E260" s="4" t="inlineStr">
+        <is>
+          <t>200, status: "ok", database: "connected"</t>
+        </is>
+      </c>
+      <c r="F260" s="4" t="n"/>
+      <c r="G260" s="4" t="n"/>
+      <c r="H260" s="4" t="n"/>
+      <c r="I260" s="4" t="n"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="4" t="inlineStr">
+        <is>
+          <t>TC-1402</t>
+        </is>
+      </c>
+      <c r="B261" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C261" s="4" t="inlineStr">
+        <is>
+          <t>CPU metric present</t>
+        </is>
+      </c>
+      <c r="D261" s="4" t="inlineStr">
+        <is>
+          <t>Inspect response body</t>
+        </is>
+      </c>
+      <c r="E261" s="4" t="inlineStr">
+        <is>
+          <t>cpu_percent is a number between 0 and 100</t>
+        </is>
+      </c>
+      <c r="F261" s="4" t="n"/>
+      <c r="G261" s="4" t="n"/>
+      <c r="H261" s="4" t="n"/>
+      <c r="I261" s="4" t="n"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="4" t="inlineStr">
+        <is>
+          <t>TC-1403</t>
+        </is>
+      </c>
+      <c r="B262" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C262" s="4" t="inlineStr">
+        <is>
+          <t>Memory metrics present</t>
+        </is>
+      </c>
+      <c r="D262" s="4" t="inlineStr">
+        <is>
+          <t>Inspect response body</t>
+        </is>
+      </c>
+      <c r="E262" s="4" t="inlineStr">
+        <is>
+          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
+        </is>
+      </c>
+      <c r="F262" s="4" t="n"/>
+      <c r="G262" s="4" t="n"/>
+      <c r="H262" s="4" t="n"/>
+      <c r="I262" s="4" t="n"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="4" t="inlineStr">
+        <is>
+          <t>TC-1404</t>
+        </is>
+      </c>
+      <c r="B263" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C263" s="4" t="inlineStr">
+        <is>
+          <t>Disk I/O metrics present</t>
+        </is>
+      </c>
+      <c r="D263" s="4" t="inlineStr">
+        <is>
+          <t>Inspect response body</t>
+        </is>
+      </c>
+      <c r="E263" s="4" t="inlineStr">
+        <is>
+          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
+        </is>
+      </c>
+      <c r="F263" s="4" t="n"/>
+      <c r="G263" s="4" t="n"/>
+      <c r="H263" s="4" t="n"/>
+      <c r="I263" s="4" t="n"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="4" t="inlineStr">
+        <is>
+          <t>TC-1405</t>
+        </is>
+      </c>
+      <c r="B264" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C264" s="4" t="inlineStr">
+        <is>
+          <t>Active jobs count</t>
+        </is>
+      </c>
+      <c r="D264" s="4" t="inlineStr">
+        <is>
+          <t>Start an export job, call endpoint</t>
+        </is>
+      </c>
+      <c r="E264" s="4" t="inlineStr">
+        <is>
+          <t>active_jobs ≥ 1</t>
+        </is>
+      </c>
+      <c r="F264" s="4" t="n"/>
+      <c r="G264" s="4" t="n"/>
+      <c r="H264" s="4" t="n"/>
+      <c r="I264" s="4" t="n"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="4" t="inlineStr">
+        <is>
+          <t>TC-1406</t>
+        </is>
+      </c>
+      <c r="B265" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C265" s="4" t="inlineStr">
+        <is>
+          <t>Worker queue size</t>
+        </is>
+      </c>
+      <c r="D265" s="4" t="inlineStr">
+        <is>
+          <t>Create a PENDING job (created but not started), call endpoint</t>
+        </is>
+      </c>
+      <c r="E265" s="4" t="inlineStr">
+        <is>
+          <t>worker_queue_size ≥ 1</t>
+        </is>
+      </c>
+      <c r="F265" s="4" t="n"/>
+      <c r="G265" s="4" t="n"/>
+      <c r="H265" s="4" t="n"/>
+      <c r="I265" s="4" t="n"/>
+    </row>
+    <row r="266">
+      <c r="A266" s="4" t="inlineStr">
+        <is>
+          <t>TC-1407</t>
+        </is>
+      </c>
+      <c r="B266" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C266" s="4" t="inlineStr">
+        <is>
+          <t>Worker queue size decrements</t>
+        </is>
+      </c>
+      <c r="D266" s="4" t="inlineStr">
+        <is>
+          <t>Start the pending job, call endpoint again</t>
+        </is>
+      </c>
+      <c r="E266" s="4" t="inlineStr">
+        <is>
+          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
+        </is>
+      </c>
+      <c r="F266" s="4" t="n"/>
+      <c r="G266" s="4" t="n"/>
+      <c r="H266" s="4" t="n"/>
+      <c r="I266" s="4" t="n"/>
+    </row>
+    <row r="267">
+      <c r="A267" s="4" t="inlineStr">
+        <is>
+          <t>TC-1408</t>
+        </is>
+      </c>
+      <c r="B267" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C267" s="4" t="inlineStr">
+        <is>
+          <t>Degraded when DB down</t>
+        </is>
+      </c>
+      <c r="D267" s="4" t="inlineStr">
+        <is>
+          <t>Stop PostgreSQL, call endpoint with valid token</t>
+        </is>
+      </c>
+      <c r="E267" s="4" t="inlineStr">
+        <is>
+          <t>200, status: "degraded", database: "error", database_error is non-null</t>
+        </is>
+      </c>
+      <c r="F267" s="4" t="n"/>
+      <c r="G267" s="4" t="n"/>
+      <c r="H267" s="4" t="n"/>
+      <c r="I267" s="4" t="n"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="4" t="inlineStr">
+        <is>
+          <t>TC-1409</t>
+        </is>
+      </c>
+      <c r="B268" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C268" s="4" t="inlineStr">
+        <is>
+          <t>Unauthenticated rejected</t>
+        </is>
+      </c>
+      <c r="D268" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/system-health without token</t>
+        </is>
+      </c>
+      <c r="E268" s="4" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="F268" s="4" t="n"/>
+      <c r="G268" s="4" t="n"/>
+      <c r="H268" s="4" t="n"/>
+      <c r="I268" s="4" t="n"/>
+    </row>
+    <row r="269">
+      <c r="A269" s="4" t="inlineStr">
+        <is>
+          <t>TC-1410</t>
+        </is>
+      </c>
+      <c r="B269" s="4" t="inlineStr">
+        <is>
+          <t>12.14 System Health</t>
+        </is>
+      </c>
+      <c r="C269" s="4" t="inlineStr">
+        <is>
+          <t>Processor role allowed</t>
+        </is>
+      </c>
+      <c r="D269" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/system-health with processor token</t>
+        </is>
+      </c>
+      <c r="E269" s="4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F269" s="4" t="n"/>
+      <c r="G269" s="4" t="n"/>
+      <c r="H269" s="4" t="n"/>
+      <c r="I269" s="4" t="n"/>
+    </row>
+    <row r="271">
+      <c r="A271" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B255" s="5" t="n">
-        <v>234</v>
+      <c r="B271" s="5" t="n">
+        <v>249</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add real-world copy performance and hashing addendum to QA testing guide
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="QA Test Cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="RW Copy Perf &amp; Hash" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8443,4 +8444,448 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TC ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Test Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Steps / How</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Tester</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>RW-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>12.15</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Dataset provenance recorded</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Document dataset source (CFReDS/Digital Corpora/EDRM), exact path/filter, and download date before test start.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Source and scope are fully documented and reproducible.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>RW-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>12.15</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Source manifest generated</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Run deterministic source hashing (`find|sort|sha256sum`) and archive `source.sha256`.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>`source.sha256` exists and covers all test files.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>RW-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>12.15</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Baseline run RW-1 complete</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Execute RW-1 profile (10-25 GB, 1 drive, thread_count=4).</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Job reaches `COMPLETED` and verify endpoint passes.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>RW-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>12.15</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Throughput run RW-2 (4 threads)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Execute RW-2 profile (50-100 GB, 1 drive, thread_count=4) and capture `total_bytes`, `started_at`, `completed_at`.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Measured throughput is recorded in Notes/attachments.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>RW-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>12.15</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Throughput run RW-2 (8 threads)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Repeat RW-2 with `thread_count=8` on same hardware and compare.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Measured throughput is recorded; thread scaling behavior is documented.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>RW-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>12.15</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Scale-out run RW-3</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Execute RW-3 with 4 drives in parallel using same source corpus.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>All jobs complete and aggregate throughput is recorded.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RW-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>12.15</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Hash verify via ECUBE API</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Run `POST /jobs/{job_id}/verify` for each completed job.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>All verify results pass with no file mismatches.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>RW-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>12.15</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Independent destination hash check</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Mount destination read-only and run `sha256sum -c source.sha256` against copied data.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Zero SHA-256 mismatches.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>RW-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>12.15</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Performance repeatability check</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Repeat RW-1 on same hardware and compare MB/s against prior RW-1 runs.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Variance remains within +/-15%.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RW-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>12.15</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Scale-out improvement confirmed</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Compare RW-3 aggregate MB/s to RW-1 single-drive MB/s baseline.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>RW-3 aggregate throughput is higher than RW-1 baseline.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>RW-011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>12.15</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Audit and manifest evidence bundle</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Collect job JSON snapshots, verify responses, manifest outputs, and key audit events.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Evidence package is complete for defensible QA review.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RW-012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>12.15</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Failure classification completeness</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>If any mismatch/failure occurs, attach logs plus root-cause classification (media, host, network, app).</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>All failures are triaged with traceable evidence and disposition.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor mount management and update documentation
- Updated sudoers configuration to include permissions for mkdir and chown.
- Changed local mount point paths in documentation and UI to reflect automatic generation under /nfs and /smb.
- Modified installation scripts to create and set permissions for managed mount roots.
- Adjusted API endpoints and client code to remove local_mount_point from requests, relying on backend-generated paths.
- Enhanced tests to validate new mount point behavior and ensure proper handling of generated directories.
- Updated user manual and QA testing guides to reflect changes in mount management and connectivity testing.
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="QA Test Cases" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="RW Copy Perf &amp; Hash" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -438,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I271"/>
+  <dimension ref="A1:I272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8431,459 +8430,34 @@
       <c r="H269" s="4" t="n"/>
       <c r="I269" s="4" t="n"/>
     </row>
-    <row r="271">
-      <c r="A271" s="5" t="inlineStr">
+    <row r="270">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>§12.15 Real-World Copy Performance &amp; Hashing Addendum</t>
+        </is>
+      </c>
+      <c r="B270" s="2" t="inlineStr">
+        <is>
+          <t>12.15 Real-World Copy Performance &amp; Hashing Addendum</t>
+        </is>
+      </c>
+      <c r="C270" s="3" t="n"/>
+      <c r="D270" s="3" t="n"/>
+      <c r="E270" s="3" t="n"/>
+      <c r="F270" s="3" t="n"/>
+      <c r="G270" s="3" t="n"/>
+      <c r="H270" s="3" t="n"/>
+      <c r="I270" s="3" t="n"/>
+    </row>
+    <row r="272">
+      <c r="A272" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B271" s="5" t="n">
+      <c r="B272" s="5" t="n">
         <v>249</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>TC ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Test Name</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Steps / How</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Tester</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>RW-001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>12.15</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Dataset provenance recorded</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Document dataset source (CFReDS/Digital Corpora/EDRM), exact path/filter, and download date before test start.</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Source and scope are fully documented and reproducible.</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>RW-002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>12.15</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Source manifest generated</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Run deterministic source hashing (`find|sort|sha256sum`) and archive `source.sha256`.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>`source.sha256` exists and covers all test files.</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>RW-003</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>12.15</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Baseline run RW-1 complete</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Execute RW-1 profile (10-25 GB, 1 drive, thread_count=4).</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Job reaches `COMPLETED` and verify endpoint passes.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>RW-004</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>12.15</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Throughput run RW-2 (4 threads)</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Execute RW-2 profile (50-100 GB, 1 drive, thread_count=4) and capture `total_bytes`, `started_at`, `completed_at`.</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Measured throughput is recorded in Notes/attachments.</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>RW-005</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>12.15</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Throughput run RW-2 (8 threads)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Repeat RW-2 with `thread_count=8` on same hardware and compare.</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Measured throughput is recorded; thread scaling behavior is documented.</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>RW-006</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>12.15</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Scale-out run RW-3</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Execute RW-3 with 4 drives in parallel using same source corpus.</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>All jobs complete and aggregate throughput is recorded.</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>RW-007</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>12.15</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Hash verify via ECUBE API</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Run `POST /jobs/{job_id}/verify` for each completed job.</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>All verify results pass with no file mismatches.</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>RW-008</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>12.15</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Independent destination hash check</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Mount destination read-only and run `sha256sum -c source.sha256` against copied data.</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Zero SHA-256 mismatches.</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>RW-009</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>12.15</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Performance repeatability check</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Repeat RW-1 on same hardware and compare MB/s against prior RW-1 runs.</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Variance remains within +/-15%.</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>RW-010</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>12.15</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Scale-out improvement confirmed</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Compare RW-3 aggregate MB/s to RW-1 single-drive MB/s baseline.</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>RW-3 aggregate throughput is higher than RW-1 baseline.</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>RW-011</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>12.15</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Audit and manifest evidence bundle</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Collect job JSON snapshots, verify responses, manifest outputs, and key audit events.</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Evidence package is complete for defensible QA review.</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>RW-012</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>12.15</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Failure classification completeness</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>If any mismatch/failure occurs, attach logs plus root-cause classification (media, host, network, app).</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>All failures are triaged with traceable evidence and disposition.</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update qa test cases spreadsheet
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -1779,13 +1779,13 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Initialize an EMPTY drive (not present / disabled port)</t>
+          <t>Initialize a DISCONNECTED drive (not present / disabled port)</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr"/>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>409, CONFLICT; audit INIT_REJECTED_NOT_AVAILABLE recorded</t>
+          <t>409, CONFLICT; audit INIT_REJECTED_NOT_AVAILABLE recorded; note: GET /drives excludes disconnected drives by default — use include_disconnected=true to see them</t>
         </is>
       </c>
       <c r="F46" s="4" t="n"/>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Drive on disabled port stays EMPTY</t>
+          <t>Drive on disabled port stays DISCONNECTED</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>GET /drives shows drive in EMPTY state</t>
+          <t>GET /drives?include_disconnected=true shows drive in DISCONNECTED state</t>
         </is>
       </c>
       <c r="F84" s="4" t="n"/>
@@ -2924,7 +2924,7 @@
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>Drive transitions to EMPTY</t>
+          <t>Drive transitions to DISCONNECTED; GET /drives (default) no longer returns it</t>
         </is>
       </c>
       <c r="F87" s="4" t="n"/>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Orphan drive stays EMPTY</t>
+          <t>Orphan drive stays DISCONNECTED</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>Drive remains in EMPTY state (unknown port treated as disabled)</t>
+          <t>Drive remains in DISCONNECTED state (unknown port treated as disabled); only visible with include_disconnected=true</t>
         </is>
       </c>
       <c r="F88" s="4" t="n"/>
@@ -3849,7 +3849,7 @@
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>GET /drives shows the new drive (in EMPTY state if port is disabled, or AVAILABLE if port is enabled)</t>
+          <t>GET /drives shows the new drive (in DISCONNECTED state if port is disabled, or AVAILABLE if port is enabled); disconnected drives require include_disconnected=true</t>
         </is>
       </c>
       <c r="F118" s="4" t="n"/>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>After the next discovery cycle, GET /drives still lists the drive with current_state=EMPTY; audit shows DRIVE_EJECT_PREPARED</t>
+          <t>After the next discovery cycle, GET /drives?include_disconnected=true lists the drive with current_state=DISCONNECTED; audit shows DRIVE_EJECT_PREPARED</t>
         </is>
       </c>
       <c r="F120" s="4" t="n"/>
@@ -4035,7 +4035,7 @@
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
-          <t>Drive appears in EMPTY state; enable port + refresh → drive transitions to AVAILABLE</t>
+          <t>Drive appears in DISCONNECTED state (visible with include_disconnected=true); enable port + refresh → drive transitions to AVAILABLE</t>
         </is>
       </c>
       <c r="F124" s="4" t="n"/>

</xml_diff>

<commit_message>
Update ECUBE QA test cases spreadsheet
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I340"/>
+  <dimension ref="A1:I343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9861,48 +9861,60 @@
       <c r="I319" s="4" t="n"/>
     </row>
     <row r="320">
-      <c r="A320" s="2" t="inlineStr">
-        <is>
-          <t>§12.15 System Health</t>
-        </is>
-      </c>
-      <c r="B320" s="2" t="inlineStr">
-        <is>
-          <t>12.15 System Health</t>
-        </is>
-      </c>
-      <c r="C320" s="3" t="n"/>
-      <c r="D320" s="3" t="n"/>
-      <c r="E320" s="3" t="n"/>
-      <c r="F320" s="3" t="n"/>
-      <c r="G320" s="3" t="n"/>
-      <c r="H320" s="3" t="n"/>
-      <c r="I320" s="3" t="n"/>
+      <c r="A320" s="4" t="inlineStr">
+        <is>
+          <t>TC-1413</t>
+        </is>
+      </c>
+      <c r="B320" s="4" t="inlineStr">
+        <is>
+          <t>12.14 Startup Reconciliation</t>
+        </is>
+      </c>
+      <c r="C320" s="4" t="inlineStr">
+        <is>
+          <t>Jobs pass emits immediate startup result log</t>
+        </is>
+      </c>
+      <c r="D320" s="4" t="inlineStr">
+        <is>
+          <t>Create at least one RUNNING job, restart service, then inspect application logs around startup reconciliation</t>
+        </is>
+      </c>
+      <c r="E320" s="4" t="inlineStr">
+        <is>
+          <t>Logs include Startup reconciliation: checking jobs followed by an immediate Startup reconciliation: jobs result line with safe counts (jobs_checked, jobs_corrected) or safe failure classification</t>
+        </is>
+      </c>
+      <c r="F320" s="4" t="n"/>
+      <c r="G320" s="4" t="n"/>
+      <c r="H320" s="4" t="n"/>
+      <c r="I320" s="4" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="4" t="inlineStr">
         <is>
-          <t>TC-1501</t>
+          <t>TC-1414</t>
         </is>
       </c>
       <c r="B321" s="4" t="inlineStr">
         <is>
-          <t>12.15 System Health</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C321" s="4" t="inlineStr">
         <is>
-          <t>Healthy response</t>
+          <t>Reconciled job persists restart-interruption failure reason</t>
         </is>
       </c>
       <c r="D321" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with valid token</t>
+          <t>Create a RUNNING or VERIFYING job, restart service, then open Job Detail for that job</t>
         </is>
       </c>
       <c r="E321" s="4" t="inlineStr">
         <is>
-          <t>200, status: "ok", database: "connected"</t>
+          <t>Job status is FAILED and Job Detail shows a stable restart interruption reason (not the generic This job failed... fallback)</t>
         </is>
       </c>
       <c r="F321" s="4" t="n"/>
@@ -9913,27 +9925,27 @@
     <row r="322">
       <c r="A322" s="4" t="inlineStr">
         <is>
-          <t>TC-1502</t>
+          <t>TC-1415</t>
         </is>
       </c>
       <c r="B322" s="4" t="inlineStr">
         <is>
-          <t>12.15 System Health</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C322" s="4" t="inlineStr">
         <is>
-          <t>CPU metric present</t>
+          <t>Reconciled failed job shows correlated failure entry from audit fallback</t>
         </is>
       </c>
       <c r="D322" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Restart with a RUNNING job, then inspect Job Detail when no matching file-log failure line is present</t>
         </is>
       </c>
       <c r="E322" s="4" t="inlineStr">
         <is>
-          <t>cpu_percent is a number between 0 and 100</t>
+          <t>Job Detail still shows a related failure entry sourced from reconciliation evidence (JOB_RECONCILED) and the entry remains sanitized</t>
         </is>
       </c>
       <c r="F322" s="4" t="n"/>
@@ -9942,40 +9954,28 @@
       <c r="I322" s="4" t="n"/>
     </row>
     <row r="323">
-      <c r="A323" s="4" t="inlineStr">
-        <is>
-          <t>TC-1503</t>
-        </is>
-      </c>
-      <c r="B323" s="4" t="inlineStr">
+      <c r="A323" s="2" t="inlineStr">
+        <is>
+          <t>§12.15 System Health</t>
+        </is>
+      </c>
+      <c r="B323" s="2" t="inlineStr">
         <is>
           <t>12.15 System Health</t>
         </is>
       </c>
-      <c r="C323" s="4" t="inlineStr">
-        <is>
-          <t>Memory metrics present</t>
-        </is>
-      </c>
-      <c r="D323" s="4" t="inlineStr">
-        <is>
-          <t>Inspect response body</t>
-        </is>
-      </c>
-      <c r="E323" s="4" t="inlineStr">
-        <is>
-          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
-        </is>
-      </c>
-      <c r="F323" s="4" t="n"/>
-      <c r="G323" s="4" t="n"/>
-      <c r="H323" s="4" t="n"/>
-      <c r="I323" s="4" t="n"/>
+      <c r="C323" s="3" t="n"/>
+      <c r="D323" s="3" t="n"/>
+      <c r="E323" s="3" t="n"/>
+      <c r="F323" s="3" t="n"/>
+      <c r="G323" s="3" t="n"/>
+      <c r="H323" s="3" t="n"/>
+      <c r="I323" s="3" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="4" t="inlineStr">
         <is>
-          <t>TC-1504</t>
+          <t>TC-1501</t>
         </is>
       </c>
       <c r="B324" s="4" t="inlineStr">
@@ -9985,17 +9985,17 @@
       </c>
       <c r="C324" s="4" t="inlineStr">
         <is>
-          <t>Disk I/O metrics present</t>
+          <t>Healthy response</t>
         </is>
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>GET /introspection/system-health with valid token</t>
         </is>
       </c>
       <c r="E324" s="4" t="inlineStr">
         <is>
-          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
+          <t>200, status: "ok", database: "connected"</t>
         </is>
       </c>
       <c r="F324" s="4" t="n"/>
@@ -10006,7 +10006,7 @@
     <row r="325">
       <c r="A325" s="4" t="inlineStr">
         <is>
-          <t>TC-1505</t>
+          <t>TC-1502</t>
         </is>
       </c>
       <c r="B325" s="4" t="inlineStr">
@@ -10016,17 +10016,17 @@
       </c>
       <c r="C325" s="4" t="inlineStr">
         <is>
-          <t>Active jobs count</t>
+          <t>CPU metric present</t>
         </is>
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>Start an export job, call endpoint</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E325" s="4" t="inlineStr">
         <is>
-          <t>active_jobs ≥ 1</t>
+          <t>cpu_percent is a number between 0 and 100</t>
         </is>
       </c>
       <c r="F325" s="4" t="n"/>
@@ -10037,7 +10037,7 @@
     <row r="326">
       <c r="A326" s="4" t="inlineStr">
         <is>
-          <t>TC-1506</t>
+          <t>TC-1503</t>
         </is>
       </c>
       <c r="B326" s="4" t="inlineStr">
@@ -10047,17 +10047,17 @@
       </c>
       <c r="C326" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size</t>
+          <t>Memory metrics present</t>
         </is>
       </c>
       <c r="D326" s="4" t="inlineStr">
         <is>
-          <t>Create a PENDING job (created but not started), call endpoint</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E326" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size ≥ 1</t>
+          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
         </is>
       </c>
       <c r="F326" s="4" t="n"/>
@@ -10068,7 +10068,7 @@
     <row r="327">
       <c r="A327" s="4" t="inlineStr">
         <is>
-          <t>TC-1507</t>
+          <t>TC-1504</t>
         </is>
       </c>
       <c r="B327" s="4" t="inlineStr">
@@ -10078,17 +10078,17 @@
       </c>
       <c r="C327" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size decrements</t>
+          <t>Disk I/O metrics present</t>
         </is>
       </c>
       <c r="D327" s="4" t="inlineStr">
         <is>
-          <t>Start the pending job, call endpoint again</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E327" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
+          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
         </is>
       </c>
       <c r="F327" s="4" t="n"/>
@@ -10099,7 +10099,7 @@
     <row r="328">
       <c r="A328" s="4" t="inlineStr">
         <is>
-          <t>TC-1508</t>
+          <t>TC-1505</t>
         </is>
       </c>
       <c r="B328" s="4" t="inlineStr">
@@ -10109,17 +10109,17 @@
       </c>
       <c r="C328" s="4" t="inlineStr">
         <is>
-          <t>Degraded when DB down</t>
+          <t>Active jobs count</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, call endpoint with valid token</t>
+          <t>Start an export job, call endpoint</t>
         </is>
       </c>
       <c r="E328" s="4" t="inlineStr">
         <is>
-          <t>200, status: "degraded", database: "error", database_error is non-null</t>
+          <t>active_jobs ≥ 1</t>
         </is>
       </c>
       <c r="F328" s="4" t="n"/>
@@ -10130,7 +10130,7 @@
     <row r="329">
       <c r="A329" s="4" t="inlineStr">
         <is>
-          <t>TC-1509</t>
+          <t>TC-1506</t>
         </is>
       </c>
       <c r="B329" s="4" t="inlineStr">
@@ -10140,17 +10140,17 @@
       </c>
       <c r="C329" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated rejected</t>
+          <t>Worker queue size</t>
         </is>
       </c>
       <c r="D329" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health without token</t>
+          <t>Create a PENDING job (created but not started), call endpoint</t>
         </is>
       </c>
       <c r="E329" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>worker_queue_size ≥ 1</t>
         </is>
       </c>
       <c r="F329" s="4" t="n"/>
@@ -10161,7 +10161,7 @@
     <row r="330">
       <c r="A330" s="4" t="inlineStr">
         <is>
-          <t>TC-1510</t>
+          <t>TC-1507</t>
         </is>
       </c>
       <c r="B330" s="4" t="inlineStr">
@@ -10171,17 +10171,17 @@
       </c>
       <c r="C330" s="4" t="inlineStr">
         <is>
-          <t>Processor role allowed</t>
+          <t>Worker queue size decrements</t>
         </is>
       </c>
       <c r="D330" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with processor token</t>
+          <t>Start the pending job, call endpoint again</t>
         </is>
       </c>
       <c r="E330" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
         </is>
       </c>
       <c r="F330" s="4" t="n"/>
@@ -10190,48 +10190,60 @@
       <c r="I330" s="4" t="n"/>
     </row>
     <row r="331">
-      <c r="A331" s="2" t="inlineStr">
-        <is>
-          <t>§12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="B331" s="2" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C331" s="3" t="n"/>
-      <c r="D331" s="3" t="n"/>
-      <c r="E331" s="3" t="n"/>
-      <c r="F331" s="3" t="n"/>
-      <c r="G331" s="3" t="n"/>
-      <c r="H331" s="3" t="n"/>
-      <c r="I331" s="3" t="n"/>
+      <c r="A331" s="4" t="inlineStr">
+        <is>
+          <t>TC-1508</t>
+        </is>
+      </c>
+      <c r="B331" s="4" t="inlineStr">
+        <is>
+          <t>12.15 System Health</t>
+        </is>
+      </c>
+      <c r="C331" s="4" t="inlineStr">
+        <is>
+          <t>Degraded when DB down</t>
+        </is>
+      </c>
+      <c r="D331" s="4" t="inlineStr">
+        <is>
+          <t>Stop PostgreSQL, call endpoint with valid token</t>
+        </is>
+      </c>
+      <c r="E331" s="4" t="inlineStr">
+        <is>
+          <t>200, status: "degraded", database: "error", database_error is non-null</t>
+        </is>
+      </c>
+      <c r="F331" s="4" t="n"/>
+      <c r="G331" s="4" t="n"/>
+      <c r="H331" s="4" t="n"/>
+      <c r="I331" s="4" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="4" t="inlineStr">
         <is>
-          <t>TC-1511</t>
+          <t>TC-1509</t>
         </is>
       </c>
       <c r="B332" s="4" t="inlineStr">
         <is>
-          <t>12.15.1 Readiness &amp; Version</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C332" s="4" t="inlineStr">
         <is>
-          <t>Liveness endpoint is public</t>
+          <t>Unauthenticated rejected</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr">
         <is>
-          <t>GET /health/live without token</t>
+          <t>GET /introspection/system-health without token</t>
         </is>
       </c>
       <c r="E332" s="4" t="inlineStr">
         <is>
-          <t>200, service reports live</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F332" s="4" t="n"/>
@@ -10242,27 +10254,27 @@
     <row r="333">
       <c r="A333" s="4" t="inlineStr">
         <is>
-          <t>TC-1512</t>
+          <t>TC-1510</t>
         </is>
       </c>
       <c r="B333" s="4" t="inlineStr">
         <is>
-          <t>12.15.1 Readiness &amp; Version</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C333" s="4" t="inlineStr">
         <is>
-          <t>Readiness endpoint is public</t>
+          <t>Processor role allowed</t>
         </is>
       </c>
       <c r="D333" s="4" t="inlineStr">
         <is>
-          <t>GET /health/ready without token on a healthy system</t>
+          <t>GET /introspection/system-health with processor token</t>
         </is>
       </c>
       <c r="E333" s="4" t="inlineStr">
         <is>
-          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F333" s="4" t="n"/>
@@ -10271,40 +10283,28 @@
       <c r="I333" s="4" t="n"/>
     </row>
     <row r="334">
-      <c r="A334" s="4" t="inlineStr">
-        <is>
-          <t>TC-1513</t>
-        </is>
-      </c>
-      <c r="B334" s="4" t="inlineStr">
+      <c r="A334" s="2" t="inlineStr">
+        <is>
+          <t>§12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="B334" s="2" t="inlineStr">
         <is>
           <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
-      <c r="C334" s="4" t="inlineStr">
-        <is>
-          <t>Readiness reports missing database configuration</t>
-        </is>
-      </c>
-      <c r="D334" s="4" t="inlineStr">
-        <is>
-          <t>Clear DB config or test before configuration, then GET /health/ready</t>
-        </is>
-      </c>
-      <c r="E334" s="4" t="inlineStr">
-        <is>
-          <t>503, status: "not_ready", reason indicates database is not configured</t>
-        </is>
-      </c>
-      <c r="F334" s="4" t="n"/>
-      <c r="G334" s="4" t="n"/>
-      <c r="H334" s="4" t="n"/>
-      <c r="I334" s="4" t="n"/>
+      <c r="C334" s="3" t="n"/>
+      <c r="D334" s="3" t="n"/>
+      <c r="E334" s="3" t="n"/>
+      <c r="F334" s="3" t="n"/>
+      <c r="G334" s="3" t="n"/>
+      <c r="H334" s="3" t="n"/>
+      <c r="I334" s="3" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="4" t="inlineStr">
         <is>
-          <t>TC-1514</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B335" s="4" t="inlineStr">
@@ -10314,17 +10314,17 @@
       </c>
       <c r="C335" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports mount or provider problems</t>
+          <t>Liveness endpoint is public</t>
         </is>
       </c>
       <c r="D335" s="4" t="inlineStr">
         <is>
-          <t>Break a configured mount or provider, then GET /health/ready</t>
+          <t>GET /health/live without token</t>
         </is>
       </c>
       <c r="E335" s="4" t="inlineStr">
         <is>
-          <t>503, response identifies the failing check without using the generic error schema</t>
+          <t>200, service reports live</t>
         </is>
       </c>
       <c r="F335" s="4" t="n"/>
@@ -10335,7 +10335,7 @@
     <row r="336">
       <c r="A336" s="4" t="inlineStr">
         <is>
-          <t>TC-1515</t>
+          <t>TC-1512</t>
         </is>
       </c>
       <c r="B336" s="4" t="inlineStr">
@@ -10345,17 +10345,17 @@
       </c>
       <c r="C336" s="4" t="inlineStr">
         <is>
-          <t>Version endpoint is public</t>
+          <t>Readiness endpoint is public</t>
         </is>
       </c>
       <c r="D336" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/version without token</t>
+          <t>GET /health/ready without token on a healthy system</t>
         </is>
       </c>
       <c r="E336" s="4" t="inlineStr">
         <is>
-          <t>200, returns version/application metadata</t>
+          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
         </is>
       </c>
       <c r="F336" s="4" t="n"/>
@@ -10366,7 +10366,7 @@
     <row r="337">
       <c r="A337" s="4" t="inlineStr">
         <is>
-          <t>TC-1516</t>
+          <t>TC-1513</t>
         </is>
       </c>
       <c r="B337" s="4" t="inlineStr">
@@ -10376,17 +10376,17 @@
       </c>
       <c r="C337" s="4" t="inlineStr">
         <is>
-          <t>Readiness remains separate from authenticated system health</t>
+          <t>Readiness reports missing database configuration</t>
         </is>
       </c>
       <c r="D337" s="4" t="inlineStr">
         <is>
-          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+          <t>Clear DB config or test before configuration, then GET /health/ready</t>
         </is>
       </c>
       <c r="E337" s="4" t="inlineStr">
         <is>
-          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+          <t>503, status: "not_ready", reason indicates database is not configured</t>
         </is>
       </c>
       <c r="F337" s="4" t="n"/>
@@ -10395,32 +10395,125 @@
       <c r="I337" s="4" t="n"/>
     </row>
     <row r="338">
-      <c r="A338" s="2" t="inlineStr">
+      <c r="A338" s="4" t="inlineStr">
+        <is>
+          <t>TC-1514</t>
+        </is>
+      </c>
+      <c r="B338" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C338" s="4" t="inlineStr">
+        <is>
+          <t>Readiness reports mount or provider problems</t>
+        </is>
+      </c>
+      <c r="D338" s="4" t="inlineStr">
+        <is>
+          <t>Break a configured mount or provider, then GET /health/ready</t>
+        </is>
+      </c>
+      <c r="E338" s="4" t="inlineStr">
+        <is>
+          <t>503, response identifies the failing check without using the generic error schema</t>
+        </is>
+      </c>
+      <c r="F338" s="4" t="n"/>
+      <c r="G338" s="4" t="n"/>
+      <c r="H338" s="4" t="n"/>
+      <c r="I338" s="4" t="n"/>
+    </row>
+    <row r="339">
+      <c r="A339" s="4" t="inlineStr">
+        <is>
+          <t>TC-1515</t>
+        </is>
+      </c>
+      <c r="B339" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C339" s="4" t="inlineStr">
+        <is>
+          <t>Version endpoint is public</t>
+        </is>
+      </c>
+      <c r="D339" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/version without token</t>
+        </is>
+      </c>
+      <c r="E339" s="4" t="inlineStr">
+        <is>
+          <t>200, returns version/application metadata</t>
+        </is>
+      </c>
+      <c r="F339" s="4" t="n"/>
+      <c r="G339" s="4" t="n"/>
+      <c r="H339" s="4" t="n"/>
+      <c r="I339" s="4" t="n"/>
+    </row>
+    <row r="340">
+      <c r="A340" s="4" t="inlineStr">
+        <is>
+          <t>TC-1516</t>
+        </is>
+      </c>
+      <c r="B340" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C340" s="4" t="inlineStr">
+        <is>
+          <t>Readiness remains separate from authenticated system health</t>
+        </is>
+      </c>
+      <c r="D340" s="4" t="inlineStr">
+        <is>
+          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+        </is>
+      </c>
+      <c r="E340" s="4" t="inlineStr">
+        <is>
+          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+        </is>
+      </c>
+      <c r="F340" s="4" t="n"/>
+      <c r="G340" s="4" t="n"/>
+      <c r="H340" s="4" t="n"/>
+      <c r="I340" s="4" t="n"/>
+    </row>
+    <row r="341">
+      <c r="A341" s="2" t="inlineStr">
         <is>
           <t>§12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="B338" s="2" t="inlineStr">
+      <c r="B341" s="2" t="inlineStr">
         <is>
           <t>12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="C338" s="3" t="n"/>
-      <c r="D338" s="3" t="n"/>
-      <c r="E338" s="3" t="n"/>
-      <c r="F338" s="3" t="n"/>
-      <c r="G338" s="3" t="n"/>
-      <c r="H338" s="3" t="n"/>
-      <c r="I338" s="3" t="n"/>
-    </row>
-    <row r="340">
-      <c r="A340" s="5" t="inlineStr">
+      <c r="C341" s="3" t="n"/>
+      <c r="D341" s="3" t="n"/>
+      <c r="E341" s="3" t="n"/>
+      <c r="F341" s="3" t="n"/>
+      <c r="G341" s="3" t="n"/>
+      <c r="H341" s="3" t="n"/>
+      <c r="I341" s="3" t="n"/>
+    </row>
+    <row r="343">
+      <c r="A343" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B340" s="5" t="n">
-        <v>310</v>
+      <c r="B343" s="5" t="n">
+        <v>313</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Document reconciliation failure diagnostics and QA sync guidance
Clarify operator and API documentation for restart-reconciled failed jobs, including:
- stable restart interruption failure messaging in Job Detail
- sanitized audit-based failure evidence fallback when file-log correlation is unavailable
- deterministic startup jobs-pass result logging with safe success/failure fields

Update UI wireframe and QA guidance with new manual scenarios for API fallback and failure-path startup logging, and sync the QA test-case workbook to match the expanded reconciliation test matrix.
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I343"/>
+  <dimension ref="A1:I345"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9954,48 +9954,60 @@
       <c r="I322" s="4" t="n"/>
     </row>
     <row r="323">
-      <c r="A323" s="2" t="inlineStr">
-        <is>
-          <t>§12.15 System Health</t>
-        </is>
-      </c>
-      <c r="B323" s="2" t="inlineStr">
-        <is>
-          <t>12.15 System Health</t>
-        </is>
-      </c>
-      <c r="C323" s="3" t="n"/>
-      <c r="D323" s="3" t="n"/>
-      <c r="E323" s="3" t="n"/>
-      <c r="F323" s="3" t="n"/>
-      <c r="G323" s="3" t="n"/>
-      <c r="H323" s="3" t="n"/>
-      <c r="I323" s="3" t="n"/>
+      <c r="A323" s="4" t="inlineStr">
+        <is>
+          <t>TC-1416</t>
+        </is>
+      </c>
+      <c r="B323" s="4" t="inlineStr">
+        <is>
+          <t>12.14 Startup Reconciliation</t>
+        </is>
+      </c>
+      <c r="C323" s="4" t="inlineStr">
+        <is>
+          <t>Failed job API uses reconciliation audit fallback when file-log correlation is unavailable</t>
+        </is>
+      </c>
+      <c r="D323" s="4" t="inlineStr">
+        <is>
+          <t>In a test environment, disable file-log correlation (log_file unset), then request GET /jobs/{job_id} for a restart-reconciled failed job</t>
+        </is>
+      </c>
+      <c r="E323" s="4" t="inlineStr">
+        <is>
+          <t>Response remains 200 and includes the stable restart failure reason plus a sanitized failure_log_entry derived from audit evidence (JOB_RECONCILED)</t>
+        </is>
+      </c>
+      <c r="F323" s="4" t="n"/>
+      <c r="G323" s="4" t="n"/>
+      <c r="H323" s="4" t="n"/>
+      <c r="I323" s="4" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="4" t="inlineStr">
         <is>
-          <t>TC-1501</t>
+          <t>TC-1417</t>
         </is>
       </c>
       <c r="B324" s="4" t="inlineStr">
         <is>
-          <t>12.15 System Health</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C324" s="4" t="inlineStr">
         <is>
-          <t>Healthy response</t>
+          <t>Jobs pass failure path emits safe startup result classification</t>
         </is>
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with valid token</t>
+          <t>In a controlled test environment, force a jobs-pass reconciliation exception, then restart service and inspect startup logs</t>
         </is>
       </c>
       <c r="E324" s="4" t="inlineStr">
         <is>
-          <t>200, status: "ok", database: "connected"</t>
+          <t>Logs still include Startup reconciliation: jobs result with status=failed and reason=job_reconciliation_failed, without raw provider errors or host paths</t>
         </is>
       </c>
       <c r="F324" s="4" t="n"/>
@@ -10004,40 +10016,28 @@
       <c r="I324" s="4" t="n"/>
     </row>
     <row r="325">
-      <c r="A325" s="4" t="inlineStr">
-        <is>
-          <t>TC-1502</t>
-        </is>
-      </c>
-      <c r="B325" s="4" t="inlineStr">
+      <c r="A325" s="2" t="inlineStr">
+        <is>
+          <t>§12.15 System Health</t>
+        </is>
+      </c>
+      <c r="B325" s="2" t="inlineStr">
         <is>
           <t>12.15 System Health</t>
         </is>
       </c>
-      <c r="C325" s="4" t="inlineStr">
-        <is>
-          <t>CPU metric present</t>
-        </is>
-      </c>
-      <c r="D325" s="4" t="inlineStr">
-        <is>
-          <t>Inspect response body</t>
-        </is>
-      </c>
-      <c r="E325" s="4" t="inlineStr">
-        <is>
-          <t>cpu_percent is a number between 0 and 100</t>
-        </is>
-      </c>
-      <c r="F325" s="4" t="n"/>
-      <c r="G325" s="4" t="n"/>
-      <c r="H325" s="4" t="n"/>
-      <c r="I325" s="4" t="n"/>
+      <c r="C325" s="3" t="n"/>
+      <c r="D325" s="3" t="n"/>
+      <c r="E325" s="3" t="n"/>
+      <c r="F325" s="3" t="n"/>
+      <c r="G325" s="3" t="n"/>
+      <c r="H325" s="3" t="n"/>
+      <c r="I325" s="3" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="4" t="inlineStr">
         <is>
-          <t>TC-1503</t>
+          <t>TC-1501</t>
         </is>
       </c>
       <c r="B326" s="4" t="inlineStr">
@@ -10047,17 +10047,17 @@
       </c>
       <c r="C326" s="4" t="inlineStr">
         <is>
-          <t>Memory metrics present</t>
+          <t>Healthy response</t>
         </is>
       </c>
       <c r="D326" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>GET /introspection/system-health with valid token</t>
         </is>
       </c>
       <c r="E326" s="4" t="inlineStr">
         <is>
-          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
+          <t>200, status: "ok", database: "connected"</t>
         </is>
       </c>
       <c r="F326" s="4" t="n"/>
@@ -10068,7 +10068,7 @@
     <row r="327">
       <c r="A327" s="4" t="inlineStr">
         <is>
-          <t>TC-1504</t>
+          <t>TC-1502</t>
         </is>
       </c>
       <c r="B327" s="4" t="inlineStr">
@@ -10078,7 +10078,7 @@
       </c>
       <c r="C327" s="4" t="inlineStr">
         <is>
-          <t>Disk I/O metrics present</t>
+          <t>CPU metric present</t>
         </is>
       </c>
       <c r="D327" s="4" t="inlineStr">
@@ -10088,7 +10088,7 @@
       </c>
       <c r="E327" s="4" t="inlineStr">
         <is>
-          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
+          <t>cpu_percent is a number between 0 and 100</t>
         </is>
       </c>
       <c r="F327" s="4" t="n"/>
@@ -10099,7 +10099,7 @@
     <row r="328">
       <c r="A328" s="4" t="inlineStr">
         <is>
-          <t>TC-1505</t>
+          <t>TC-1503</t>
         </is>
       </c>
       <c r="B328" s="4" t="inlineStr">
@@ -10109,17 +10109,17 @@
       </c>
       <c r="C328" s="4" t="inlineStr">
         <is>
-          <t>Active jobs count</t>
+          <t>Memory metrics present</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr">
         <is>
-          <t>Start an export job, call endpoint</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E328" s="4" t="inlineStr">
         <is>
-          <t>active_jobs ≥ 1</t>
+          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
         </is>
       </c>
       <c r="F328" s="4" t="n"/>
@@ -10130,7 +10130,7 @@
     <row r="329">
       <c r="A329" s="4" t="inlineStr">
         <is>
-          <t>TC-1506</t>
+          <t>TC-1504</t>
         </is>
       </c>
       <c r="B329" s="4" t="inlineStr">
@@ -10140,17 +10140,17 @@
       </c>
       <c r="C329" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size</t>
+          <t>Disk I/O metrics present</t>
         </is>
       </c>
       <c r="D329" s="4" t="inlineStr">
         <is>
-          <t>Create a PENDING job (created but not started), call endpoint</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E329" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size ≥ 1</t>
+          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
         </is>
       </c>
       <c r="F329" s="4" t="n"/>
@@ -10161,7 +10161,7 @@
     <row r="330">
       <c r="A330" s="4" t="inlineStr">
         <is>
-          <t>TC-1507</t>
+          <t>TC-1505</t>
         </is>
       </c>
       <c r="B330" s="4" t="inlineStr">
@@ -10171,17 +10171,17 @@
       </c>
       <c r="C330" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size decrements</t>
+          <t>Active jobs count</t>
         </is>
       </c>
       <c r="D330" s="4" t="inlineStr">
         <is>
-          <t>Start the pending job, call endpoint again</t>
+          <t>Start an export job, call endpoint</t>
         </is>
       </c>
       <c r="E330" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
+          <t>active_jobs ≥ 1</t>
         </is>
       </c>
       <c r="F330" s="4" t="n"/>
@@ -10192,7 +10192,7 @@
     <row r="331">
       <c r="A331" s="4" t="inlineStr">
         <is>
-          <t>TC-1508</t>
+          <t>TC-1506</t>
         </is>
       </c>
       <c r="B331" s="4" t="inlineStr">
@@ -10202,17 +10202,17 @@
       </c>
       <c r="C331" s="4" t="inlineStr">
         <is>
-          <t>Degraded when DB down</t>
+          <t>Worker queue size</t>
         </is>
       </c>
       <c r="D331" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, call endpoint with valid token</t>
+          <t>Create a PENDING job (created but not started), call endpoint</t>
         </is>
       </c>
       <c r="E331" s="4" t="inlineStr">
         <is>
-          <t>200, status: "degraded", database: "error", database_error is non-null</t>
+          <t>worker_queue_size ≥ 1</t>
         </is>
       </c>
       <c r="F331" s="4" t="n"/>
@@ -10223,7 +10223,7 @@
     <row r="332">
       <c r="A332" s="4" t="inlineStr">
         <is>
-          <t>TC-1509</t>
+          <t>TC-1507</t>
         </is>
       </c>
       <c r="B332" s="4" t="inlineStr">
@@ -10233,17 +10233,17 @@
       </c>
       <c r="C332" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated rejected</t>
+          <t>Worker queue size decrements</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health without token</t>
+          <t>Start the pending job, call endpoint again</t>
         </is>
       </c>
       <c r="E332" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
         </is>
       </c>
       <c r="F332" s="4" t="n"/>
@@ -10254,7 +10254,7 @@
     <row r="333">
       <c r="A333" s="4" t="inlineStr">
         <is>
-          <t>TC-1510</t>
+          <t>TC-1508</t>
         </is>
       </c>
       <c r="B333" s="4" t="inlineStr">
@@ -10264,17 +10264,17 @@
       </c>
       <c r="C333" s="4" t="inlineStr">
         <is>
-          <t>Processor role allowed</t>
+          <t>Degraded when DB down</t>
         </is>
       </c>
       <c r="D333" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with processor token</t>
+          <t>Stop PostgreSQL, call endpoint with valid token</t>
         </is>
       </c>
       <c r="E333" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, status: "degraded", database: "error", database_error is non-null</t>
         </is>
       </c>
       <c r="F333" s="4" t="n"/>
@@ -10283,48 +10283,60 @@
       <c r="I333" s="4" t="n"/>
     </row>
     <row r="334">
-      <c r="A334" s="2" t="inlineStr">
-        <is>
-          <t>§12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="B334" s="2" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C334" s="3" t="n"/>
-      <c r="D334" s="3" t="n"/>
-      <c r="E334" s="3" t="n"/>
-      <c r="F334" s="3" t="n"/>
-      <c r="G334" s="3" t="n"/>
-      <c r="H334" s="3" t="n"/>
-      <c r="I334" s="3" t="n"/>
+      <c r="A334" s="4" t="inlineStr">
+        <is>
+          <t>TC-1509</t>
+        </is>
+      </c>
+      <c r="B334" s="4" t="inlineStr">
+        <is>
+          <t>12.15 System Health</t>
+        </is>
+      </c>
+      <c r="C334" s="4" t="inlineStr">
+        <is>
+          <t>Unauthenticated rejected</t>
+        </is>
+      </c>
+      <c r="D334" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/system-health without token</t>
+        </is>
+      </c>
+      <c r="E334" s="4" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="F334" s="4" t="n"/>
+      <c r="G334" s="4" t="n"/>
+      <c r="H334" s="4" t="n"/>
+      <c r="I334" s="4" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="4" t="inlineStr">
         <is>
-          <t>TC-1511</t>
+          <t>TC-1510</t>
         </is>
       </c>
       <c r="B335" s="4" t="inlineStr">
         <is>
-          <t>12.15.1 Readiness &amp; Version</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C335" s="4" t="inlineStr">
         <is>
-          <t>Liveness endpoint is public</t>
+          <t>Processor role allowed</t>
         </is>
       </c>
       <c r="D335" s="4" t="inlineStr">
         <is>
-          <t>GET /health/live without token</t>
+          <t>GET /introspection/system-health with processor token</t>
         </is>
       </c>
       <c r="E335" s="4" t="inlineStr">
         <is>
-          <t>200, service reports live</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F335" s="4" t="n"/>
@@ -10333,40 +10345,28 @@
       <c r="I335" s="4" t="n"/>
     </row>
     <row r="336">
-      <c r="A336" s="4" t="inlineStr">
-        <is>
-          <t>TC-1512</t>
-        </is>
-      </c>
-      <c r="B336" s="4" t="inlineStr">
+      <c r="A336" s="2" t="inlineStr">
+        <is>
+          <t>§12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="B336" s="2" t="inlineStr">
         <is>
           <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
-      <c r="C336" s="4" t="inlineStr">
-        <is>
-          <t>Readiness endpoint is public</t>
-        </is>
-      </c>
-      <c r="D336" s="4" t="inlineStr">
-        <is>
-          <t>GET /health/ready without token on a healthy system</t>
-        </is>
-      </c>
-      <c r="E336" s="4" t="inlineStr">
-        <is>
-          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
-        </is>
-      </c>
-      <c r="F336" s="4" t="n"/>
-      <c r="G336" s="4" t="n"/>
-      <c r="H336" s="4" t="n"/>
-      <c r="I336" s="4" t="n"/>
+      <c r="C336" s="3" t="n"/>
+      <c r="D336" s="3" t="n"/>
+      <c r="E336" s="3" t="n"/>
+      <c r="F336" s="3" t="n"/>
+      <c r="G336" s="3" t="n"/>
+      <c r="H336" s="3" t="n"/>
+      <c r="I336" s="3" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="4" t="inlineStr">
         <is>
-          <t>TC-1513</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B337" s="4" t="inlineStr">
@@ -10376,17 +10376,17 @@
       </c>
       <c r="C337" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports missing database configuration</t>
+          <t>Liveness endpoint is public</t>
         </is>
       </c>
       <c r="D337" s="4" t="inlineStr">
         <is>
-          <t>Clear DB config or test before configuration, then GET /health/ready</t>
+          <t>GET /health/live without token</t>
         </is>
       </c>
       <c r="E337" s="4" t="inlineStr">
         <is>
-          <t>503, status: "not_ready", reason indicates database is not configured</t>
+          <t>200, service reports live</t>
         </is>
       </c>
       <c r="F337" s="4" t="n"/>
@@ -10397,7 +10397,7 @@
     <row r="338">
       <c r="A338" s="4" t="inlineStr">
         <is>
-          <t>TC-1514</t>
+          <t>TC-1512</t>
         </is>
       </c>
       <c r="B338" s="4" t="inlineStr">
@@ -10407,17 +10407,17 @@
       </c>
       <c r="C338" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports mount or provider problems</t>
+          <t>Readiness endpoint is public</t>
         </is>
       </c>
       <c r="D338" s="4" t="inlineStr">
         <is>
-          <t>Break a configured mount or provider, then GET /health/ready</t>
+          <t>GET /health/ready without token on a healthy system</t>
         </is>
       </c>
       <c r="E338" s="4" t="inlineStr">
         <is>
-          <t>503, response identifies the failing check without using the generic error schema</t>
+          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
         </is>
       </c>
       <c r="F338" s="4" t="n"/>
@@ -10428,7 +10428,7 @@
     <row r="339">
       <c r="A339" s="4" t="inlineStr">
         <is>
-          <t>TC-1515</t>
+          <t>TC-1513</t>
         </is>
       </c>
       <c r="B339" s="4" t="inlineStr">
@@ -10438,17 +10438,17 @@
       </c>
       <c r="C339" s="4" t="inlineStr">
         <is>
-          <t>Version endpoint is public</t>
+          <t>Readiness reports missing database configuration</t>
         </is>
       </c>
       <c r="D339" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/version without token</t>
+          <t>Clear DB config or test before configuration, then GET /health/ready</t>
         </is>
       </c>
       <c r="E339" s="4" t="inlineStr">
         <is>
-          <t>200, returns version/application metadata</t>
+          <t>503, status: "not_ready", reason indicates database is not configured</t>
         </is>
       </c>
       <c r="F339" s="4" t="n"/>
@@ -10459,7 +10459,7 @@
     <row r="340">
       <c r="A340" s="4" t="inlineStr">
         <is>
-          <t>TC-1516</t>
+          <t>TC-1514</t>
         </is>
       </c>
       <c r="B340" s="4" t="inlineStr">
@@ -10469,17 +10469,17 @@
       </c>
       <c r="C340" s="4" t="inlineStr">
         <is>
-          <t>Readiness remains separate from authenticated system health</t>
+          <t>Readiness reports mount or provider problems</t>
         </is>
       </c>
       <c r="D340" s="4" t="inlineStr">
         <is>
-          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+          <t>Break a configured mount or provider, then GET /health/ready</t>
         </is>
       </c>
       <c r="E340" s="4" t="inlineStr">
         <is>
-          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+          <t>503, response identifies the failing check without using the generic error schema</t>
         </is>
       </c>
       <c r="F340" s="4" t="n"/>
@@ -10488,32 +10488,94 @@
       <c r="I340" s="4" t="n"/>
     </row>
     <row r="341">
-      <c r="A341" s="2" t="inlineStr">
+      <c r="A341" s="4" t="inlineStr">
+        <is>
+          <t>TC-1515</t>
+        </is>
+      </c>
+      <c r="B341" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C341" s="4" t="inlineStr">
+        <is>
+          <t>Version endpoint is public</t>
+        </is>
+      </c>
+      <c r="D341" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/version without token</t>
+        </is>
+      </c>
+      <c r="E341" s="4" t="inlineStr">
+        <is>
+          <t>200, returns version/application metadata</t>
+        </is>
+      </c>
+      <c r="F341" s="4" t="n"/>
+      <c r="G341" s="4" t="n"/>
+      <c r="H341" s="4" t="n"/>
+      <c r="I341" s="4" t="n"/>
+    </row>
+    <row r="342">
+      <c r="A342" s="4" t="inlineStr">
+        <is>
+          <t>TC-1516</t>
+        </is>
+      </c>
+      <c r="B342" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C342" s="4" t="inlineStr">
+        <is>
+          <t>Readiness remains separate from authenticated system health</t>
+        </is>
+      </c>
+      <c r="D342" s="4" t="inlineStr">
+        <is>
+          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+        </is>
+      </c>
+      <c r="E342" s="4" t="inlineStr">
+        <is>
+          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+        </is>
+      </c>
+      <c r="F342" s="4" t="n"/>
+      <c r="G342" s="4" t="n"/>
+      <c r="H342" s="4" t="n"/>
+      <c r="I342" s="4" t="n"/>
+    </row>
+    <row r="343">
+      <c r="A343" s="2" t="inlineStr">
         <is>
           <t>§12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="B341" s="2" t="inlineStr">
+      <c r="B343" s="2" t="inlineStr">
         <is>
           <t>12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="C341" s="3" t="n"/>
-      <c r="D341" s="3" t="n"/>
-      <c r="E341" s="3" t="n"/>
-      <c r="F341" s="3" t="n"/>
-      <c r="G341" s="3" t="n"/>
-      <c r="H341" s="3" t="n"/>
-      <c r="I341" s="3" t="n"/>
-    </row>
-    <row r="343">
-      <c r="A343" s="5" t="inlineStr">
+      <c r="C343" s="3" t="n"/>
+      <c r="D343" s="3" t="n"/>
+      <c r="E343" s="3" t="n"/>
+      <c r="F343" s="3" t="n"/>
+      <c r="G343" s="3" t="n"/>
+      <c r="H343" s="3" t="n"/>
+      <c r="I343" s="3" t="n"/>
+    </row>
+    <row r="345">
+      <c r="A345" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B343" s="5" t="n">
-        <v>313</v>
+      <c r="B345" s="5" t="n">
+        <v>315</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Persist setup proxy-header settings and harden install/uninstall runtime safety
Add a dedicated setup-wizard reverse-proxy step and persist `trust_proxy_headers` end-to-end, including idempotent `POST /setup/initialize` behavior (`already_initialized` with runtime-flag persistence).
Stabilize runtime `.env` targeting via `ECUBE_ENV_FILE` and systemd export so setup writes always hit the active install env file.
Preserve operator-selected `TRUST_PROXY_HEADERS` during install/upgrade, and make `--uninstall --drop-database` fail closed when the drop target is unsafe or cannot be dropped.
Update tests (unit, backend, and Playwright) plus operator/API/QA documentation to match the new setup and installer behavior.
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I348"/>
+  <dimension ref="A1:I353"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8986,7 +8986,7 @@
       </c>
       <c r="C291" s="4" t="inlineStr">
         <is>
-          <t>Re-initialize rejected</t>
+          <t>Re-initialize informational</t>
         </is>
       </c>
       <c r="D291" s="4" t="inlineStr">
@@ -8996,7 +8996,7 @@
       </c>
       <c r="E291" s="4" t="inlineStr">
         <is>
-          <t>409, Conflict</t>
+          <t>200, status=already_initialized</t>
         </is>
       </c>
       <c r="F291" s="4" t="n"/>
@@ -9160,48 +9160,60 @@
       <c r="I296" s="4" t="n"/>
     </row>
     <row r="297">
-      <c r="A297" s="2" t="inlineStr">
-        <is>
-          <t>§12.12 Chain-of-Custody Handoff</t>
-        </is>
-      </c>
-      <c r="B297" s="2" t="inlineStr">
-        <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
-        </is>
-      </c>
-      <c r="C297" s="3" t="n"/>
-      <c r="D297" s="3" t="n"/>
-      <c r="E297" s="3" t="n"/>
-      <c r="F297" s="3" t="n"/>
-      <c r="G297" s="3" t="n"/>
-      <c r="H297" s="3" t="n"/>
-      <c r="I297" s="3" t="n"/>
+      <c r="A297" s="4" t="inlineStr">
+        <is>
+          <t>TC-1110</t>
+        </is>
+      </c>
+      <c r="B297" s="4" t="inlineStr">
+        <is>
+          <t>12.11 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C297" s="4" t="inlineStr">
+        <is>
+          <t>Initialize default proxy trust</t>
+        </is>
+      </c>
+      <c r="D297" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/initialize without trust_proxy_headers</t>
+        </is>
+      </c>
+      <c r="E297" s="4" t="inlineStr">
+        <is>
+          <t>200, runtime TRUST_PROXY_HEADERS=false persisted</t>
+        </is>
+      </c>
+      <c r="F297" s="4" t="n"/>
+      <c r="G297" s="4" t="n"/>
+      <c r="H297" s="4" t="n"/>
+      <c r="I297" s="4" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="4" t="inlineStr">
         <is>
-          <t>TC-1201</t>
+          <t>TC-1111</t>
         </is>
       </c>
       <c r="B298" s="4" t="inlineStr">
         <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C298" s="4" t="inlineStr">
         <is>
-          <t>Retrieve CoC — by drive_id</t>
+          <t>Initialize explicit proxy trust</t>
         </is>
       </c>
       <c r="D298" s="4" t="inlineStr">
         <is>
-          <t>GET /audit/chain-of-custody?drive_id=42 with auditor/manager/admin token</t>
+          <t>POST /setup/initialize with "trust_proxy_headers": true</t>
         </is>
       </c>
       <c r="E298" s="4" t="inlineStr">
         <is>
-          <t>200, selector_mode: "DRIVE_ID", report contains events for that drive</t>
+          <t>200, runtime TRUST_PROXY_HEADERS=true persisted</t>
         </is>
       </c>
       <c r="F298" s="4" t="n"/>
@@ -9212,27 +9224,27 @@
     <row r="299">
       <c r="A299" s="4" t="inlineStr">
         <is>
-          <t>TC-1202</t>
+          <t>TC-1112</t>
         </is>
       </c>
       <c r="B299" s="4" t="inlineStr">
         <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C299" s="4" t="inlineStr">
         <is>
-          <t>Retrieve CoC — by drive_sn</t>
+          <t>Re-initialize persists runtime flags</t>
         </is>
       </c>
       <c r="D299" s="4" t="inlineStr">
         <is>
-          <t>GET /audit/chain-of-custody?drive_sn=ABC123DEF with manager token</t>
+          <t>Call POST /setup/initialize after setup with a different trust_proxy_headers value</t>
         </is>
       </c>
       <c r="E299" s="4" t="inlineStr">
         <is>
-          <t>200, selector_mode: "DRIVE_SN", report contains events for that drive</t>
+          <t>200, status=already_initialized, runtime flag updated</t>
         </is>
       </c>
       <c r="F299" s="4" t="n"/>
@@ -9243,27 +9255,27 @@
     <row r="300">
       <c r="A300" s="4" t="inlineStr">
         <is>
-          <t>TC-1203</t>
+          <t>TC-1113</t>
         </is>
       </c>
       <c r="B300" s="4" t="inlineStr">
         <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C300" s="4" t="inlineStr">
         <is>
-          <t>Retrieve CoC — by project_id</t>
+          <t>Runtime env target consistency</t>
         </is>
       </c>
       <c r="D300" s="4" t="inlineStr">
         <is>
-          <t>GET /audit/chain-of-custody?project_id=CASE-2026-007 with auditor token</t>
+          <t>Validate running service env file target and setup persistence target are the same (ECUBE_ENV_FILE)</t>
         </is>
       </c>
       <c r="E300" s="4" t="inlineStr">
         <is>
-          <t>200, selector_mode: "PROJECT", reports array contains all non-archived drives for project</t>
+          <t>Runtime env file is updated, not a workspace-relative .env</t>
         </is>
       </c>
       <c r="F300" s="4" t="n"/>
@@ -9274,27 +9286,27 @@
     <row r="301">
       <c r="A301" s="4" t="inlineStr">
         <is>
-          <t>TC-1204</t>
+          <t>TC-1114</t>
         </is>
       </c>
       <c r="B301" s="4" t="inlineStr">
         <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C301" s="4" t="inlineStr">
         <is>
-          <t>CoC — processor denied</t>
+          <t>Uninstall drop fails closed on invalid target</t>
         </is>
       </c>
       <c r="D301" s="4" t="inlineStr">
         <is>
-          <t>GET /audit/chain-of-custody?drive_id=42 with processor token</t>
+          <t>Run install.sh --uninstall --drop-database with missing/invalid/maintenance DATABASE_URL</t>
         </is>
       </c>
       <c r="E301" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>Installer exits non-zero with explicit drop-target error; uninstall does not silently continue</t>
         </is>
       </c>
       <c r="F301" s="4" t="n"/>
@@ -9303,40 +9315,28 @@
       <c r="I301" s="4" t="n"/>
     </row>
     <row r="302">
-      <c r="A302" s="4" t="inlineStr">
-        <is>
-          <t>TC-1205</t>
-        </is>
-      </c>
-      <c r="B302" s="4" t="inlineStr">
+      <c r="A302" s="2" t="inlineStr">
+        <is>
+          <t>§12.12 Chain-of-Custody Handoff</t>
+        </is>
+      </c>
+      <c r="B302" s="2" t="inlineStr">
         <is>
           <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
-      <c r="C302" s="4" t="inlineStr">
-        <is>
-          <t>CoC — unauthenticated denied</t>
-        </is>
-      </c>
-      <c r="D302" s="4" t="inlineStr">
-        <is>
-          <t>GET /audit/chain-of-custody?drive_id=42 without token</t>
-        </is>
-      </c>
-      <c r="E302" s="4" t="inlineStr">
-        <is>
-          <t>401, UNAUTHORIZED</t>
-        </is>
-      </c>
-      <c r="F302" s="4" t="n"/>
-      <c r="G302" s="4" t="n"/>
-      <c r="H302" s="4" t="n"/>
-      <c r="I302" s="4" t="n"/>
+      <c r="C302" s="3" t="n"/>
+      <c r="D302" s="3" t="n"/>
+      <c r="E302" s="3" t="n"/>
+      <c r="F302" s="3" t="n"/>
+      <c r="G302" s="3" t="n"/>
+      <c r="H302" s="3" t="n"/>
+      <c r="I302" s="3" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="4" t="inlineStr">
         <is>
-          <t>TC-1206</t>
+          <t>TC-1201</t>
         </is>
       </c>
       <c r="B303" s="4" t="inlineStr">
@@ -9346,17 +9346,17 @@
       </c>
       <c r="C303" s="4" t="inlineStr">
         <is>
-          <t>CoC — no selector</t>
+          <t>Retrieve CoC — by drive_id</t>
         </is>
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>GET /audit/chain-of-custody with no query parameters</t>
+          <t>GET /audit/chain-of-custody?drive_id=42 with auditor/manager/admin token</t>
         </is>
       </c>
       <c r="E303" s="4" t="inlineStr">
         <is>
-          <t>422, at least one selector required</t>
+          <t>200, selector_mode: "DRIVE_ID", report contains events for that drive</t>
         </is>
       </c>
       <c r="F303" s="4" t="n"/>
@@ -9367,7 +9367,7 @@
     <row r="304">
       <c r="A304" s="4" t="inlineStr">
         <is>
-          <t>TC-1207</t>
+          <t>TC-1202</t>
         </is>
       </c>
       <c r="B304" s="4" t="inlineStr">
@@ -9377,17 +9377,17 @@
       </c>
       <c r="C304" s="4" t="inlineStr">
         <is>
-          <t>CoC — drive_id takes precedence</t>
+          <t>Retrieve CoC — by drive_sn</t>
         </is>
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>GET /audit/chain-of-custody?drive_id=42&amp;drive_sn=ABC&amp;project_id=CASE-X</t>
+          <t>GET /audit/chain-of-custody?drive_sn=ABC123DEF with manager token</t>
         </is>
       </c>
       <c r="E304" s="4" t="inlineStr">
         <is>
-          <t>200, selector_mode: "DRIVE_ID" (ignores other selectors)</t>
+          <t>200, selector_mode: "DRIVE_SN", report contains events for that drive</t>
         </is>
       </c>
       <c r="F304" s="4" t="n"/>
@@ -9398,7 +9398,7 @@
     <row r="305">
       <c r="A305" s="4" t="inlineStr">
         <is>
-          <t>TC-1208</t>
+          <t>TC-1203</t>
         </is>
       </c>
       <c r="B305" s="4" t="inlineStr">
@@ -9408,17 +9408,17 @@
       </c>
       <c r="C305" s="4" t="inlineStr">
         <is>
-          <t>CoC — project_id mismatch</t>
+          <t>Retrieve CoC — by project_id</t>
         </is>
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>GET /audit/chain-of-custody?drive_id=42&amp;project_id=WRONG-PROJECT where drive is bound to different project</t>
+          <t>GET /audit/chain-of-custody?project_id=CASE-2026-007 with auditor token</t>
         </is>
       </c>
       <c r="E305" s="4" t="inlineStr">
         <is>
-          <t>409, CONFLICT, mismatch detail</t>
+          <t>200, selector_mode: "PROJECT", reports array contains all non-archived drives for project</t>
         </is>
       </c>
       <c r="F305" s="4" t="n"/>
@@ -9429,7 +9429,7 @@
     <row r="306">
       <c r="A306" s="4" t="inlineStr">
         <is>
-          <t>TC-1209</t>
+          <t>TC-1204</t>
         </is>
       </c>
       <c r="B306" s="4" t="inlineStr">
@@ -9439,17 +9439,17 @@
       </c>
       <c r="C306" s="4" t="inlineStr">
         <is>
-          <t>CoC report fields</t>
+          <t>CoC — processor denied</t>
         </is>
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>Inspect any GET /audit/chain-of-custody response</t>
+          <t>GET /audit/chain-of-custody?drive_id=42 with processor token</t>
         </is>
       </c>
       <c r="E306" s="4" t="inlineStr">
         <is>
-          <t>reports[].drive_id, reports[].drive_sn, reports[].project_id, reports[].custody_complete, reports[].chain_of_custody_events present</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F306" s="4" t="n"/>
@@ -9460,7 +9460,7 @@
     <row r="307">
       <c r="A307" s="4" t="inlineStr">
         <is>
-          <t>TC-1210</t>
+          <t>TC-1205</t>
         </is>
       </c>
       <c r="B307" s="4" t="inlineStr">
@@ -9470,17 +9470,17 @@
       </c>
       <c r="C307" s="4" t="inlineStr">
         <is>
-          <t>CoC events include lifecycle</t>
+          <t>CoC — unauthenticated denied</t>
         </is>
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>Inspect chain_of_custody_events in a report with completed job</t>
+          <t>GET /audit/chain-of-custody?drive_id=42 without token</t>
         </is>
       </c>
       <c r="E307" s="4" t="inlineStr">
         <is>
-          <t>Events include DRIVE_INITIALIZED, JOB_CREATED, JOB_STARTED, JOB_COMPLETED, DRIVE_EJECT_PREPARED, COC_HANDOFF_CONFIRMED (if handed off)</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F307" s="4" t="n"/>
@@ -9491,7 +9491,7 @@
     <row r="308">
       <c r="A308" s="4" t="inlineStr">
         <is>
-          <t>TC-1211</t>
+          <t>TC-1206</t>
         </is>
       </c>
       <c r="B308" s="4" t="inlineStr">
@@ -9501,17 +9501,17 @@
       </c>
       <c r="C308" s="4" t="inlineStr">
         <is>
-          <t>CoC manifest summary</t>
+          <t>CoC — no selector</t>
         </is>
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>Inspect manifest_summary in CoC report</t>
+          <t>GET /audit/chain-of-custody with no query parameters</t>
         </is>
       </c>
       <c r="E308" s="4" t="inlineStr">
         <is>
-          <t>Array of objects with job_id, total_files, total_bytes, manifest_count</t>
+          <t>422, at least one selector required</t>
         </is>
       </c>
       <c r="F308" s="4" t="n"/>
@@ -9522,7 +9522,7 @@
     <row r="309">
       <c r="A309" s="4" t="inlineStr">
         <is>
-          <t>TC-1212</t>
+          <t>TC-1207</t>
         </is>
       </c>
       <c r="B309" s="4" t="inlineStr">
@@ -9532,17 +9532,17 @@
       </c>
       <c r="C309" s="4" t="inlineStr">
         <is>
-          <t>CoC — delivery_time absence (no handoff)</t>
+          <t>CoC — drive_id takes precedence</t>
         </is>
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>Complete a job and eject without handoff, query GET /audit/chain-of-custody?drive_id=...</t>
+          <t>GET /audit/chain-of-custody?drive_id=42&amp;drive_sn=ABC&amp;project_id=CASE-X</t>
         </is>
       </c>
       <c r="E309" s="4" t="inlineStr">
         <is>
-          <t>chain_of_custody_events do not contain COC_HANDOFF_CONFIRMED; custody_complete is false</t>
+          <t>200, selector_mode: "DRIVE_ID" (ignores other selectors)</t>
         </is>
       </c>
       <c r="F309" s="4" t="n"/>
@@ -9551,48 +9551,60 @@
       <c r="I309" s="4" t="n"/>
     </row>
     <row r="310">
-      <c r="A310" s="2" t="inlineStr">
-        <is>
-          <t>§12.14 Startup Reconciliation</t>
-        </is>
-      </c>
-      <c r="B310" s="2" t="inlineStr">
-        <is>
-          <t>12.14 Startup Reconciliation</t>
-        </is>
-      </c>
-      <c r="C310" s="3" t="n"/>
-      <c r="D310" s="3" t="n"/>
-      <c r="E310" s="3" t="n"/>
-      <c r="F310" s="3" t="n"/>
-      <c r="G310" s="3" t="n"/>
-      <c r="H310" s="3" t="n"/>
-      <c r="I310" s="3" t="n"/>
+      <c r="A310" s="4" t="inlineStr">
+        <is>
+          <t>TC-1208</t>
+        </is>
+      </c>
+      <c r="B310" s="4" t="inlineStr">
+        <is>
+          <t>12.12 Chain-of-Custody Handoff</t>
+        </is>
+      </c>
+      <c r="C310" s="4" t="inlineStr">
+        <is>
+          <t>CoC — project_id mismatch</t>
+        </is>
+      </c>
+      <c r="D310" s="4" t="inlineStr">
+        <is>
+          <t>GET /audit/chain-of-custody?drive_id=42&amp;project_id=WRONG-PROJECT where drive is bound to different project</t>
+        </is>
+      </c>
+      <c r="E310" s="4" t="inlineStr">
+        <is>
+          <t>409, CONFLICT, mismatch detail</t>
+        </is>
+      </c>
+      <c r="F310" s="4" t="n"/>
+      <c r="G310" s="4" t="n"/>
+      <c r="H310" s="4" t="n"/>
+      <c r="I310" s="4" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="4" t="inlineStr">
         <is>
-          <t>TC-1401</t>
+          <t>TC-1209</t>
         </is>
       </c>
       <c r="B311" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
       <c r="C311" s="4" t="inlineStr">
         <is>
-          <t>Running job failed after restart</t>
+          <t>CoC report fields</t>
         </is>
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>Create a job, start it, restart the service while RUNNING</t>
+          <t>Inspect any GET /audit/chain-of-custody response</t>
         </is>
       </c>
       <c r="E311" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
+          <t>reports[].drive_id, reports[].drive_sn, reports[].project_id, reports[].custody_complete, reports[].chain_of_custody_events present</t>
         </is>
       </c>
       <c r="F311" s="4" t="n"/>
@@ -9603,27 +9615,27 @@
     <row r="312">
       <c r="A312" s="4" t="inlineStr">
         <is>
-          <t>TC-1402</t>
+          <t>TC-1210</t>
         </is>
       </c>
       <c r="B312" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
       <c r="C312" s="4" t="inlineStr">
         <is>
-          <t>Verifying job failed after restart</t>
+          <t>CoC events include lifecycle</t>
         </is>
       </c>
       <c r="D312" s="4" t="inlineStr">
         <is>
-          <t>Start a job, let it reach VERIFYING, restart the service</t>
+          <t>Inspect chain_of_custody_events in a report with completed job</t>
         </is>
       </c>
       <c r="E312" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
+          <t>Events include DRIVE_INITIALIZED, JOB_CREATED, JOB_STARTED, JOB_COMPLETED, DRIVE_EJECT_PREPARED, COC_HANDOFF_CONFIRMED (if handed off)</t>
         </is>
       </c>
       <c r="F312" s="4" t="n"/>
@@ -9634,27 +9646,27 @@
     <row r="313">
       <c r="A313" s="4" t="inlineStr">
         <is>
-          <t>TC-1403</t>
+          <t>TC-1211</t>
         </is>
       </c>
       <c r="B313" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
       <c r="C313" s="4" t="inlineStr">
         <is>
-          <t>Pending job not affected</t>
+          <t>CoC manifest summary</t>
         </is>
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>Create a job (PENDING), restart the service</t>
+          <t>Inspect manifest_summary in CoC report</t>
         </is>
       </c>
       <c r="E313" s="4" t="inlineStr">
         <is>
-          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
+          <t>Array of objects with job_id, total_files, total_bytes, manifest_count</t>
         </is>
       </c>
       <c r="F313" s="4" t="n"/>
@@ -9665,27 +9677,27 @@
     <row r="314">
       <c r="A314" s="4" t="inlineStr">
         <is>
-          <t>TC-1404</t>
+          <t>TC-1212</t>
         </is>
       </c>
       <c r="B314" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
       <c r="C314" s="4" t="inlineStr">
         <is>
-          <t>Completed job not affected</t>
+          <t>CoC — delivery_time absence (no handoff)</t>
         </is>
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>Complete a job, restart the service</t>
+          <t>Complete a job and eject without handoff, query GET /audit/chain-of-custody?drive_id=...</t>
         </is>
       </c>
       <c r="E314" s="4" t="inlineStr">
         <is>
-          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
+          <t>chain_of_custody_events do not contain COC_HANDOFF_CONFIRMED; custody_complete is false</t>
         </is>
       </c>
       <c r="F314" s="4" t="n"/>
@@ -9694,40 +9706,28 @@
       <c r="I314" s="4" t="n"/>
     </row>
     <row r="315">
-      <c r="A315" s="4" t="inlineStr">
-        <is>
-          <t>TC-1405</t>
-        </is>
-      </c>
-      <c r="B315" s="4" t="inlineStr">
+      <c r="A315" s="2" t="inlineStr">
+        <is>
+          <t>§12.14 Startup Reconciliation</t>
+        </is>
+      </c>
+      <c r="B315" s="2" t="inlineStr">
         <is>
           <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
-      <c r="C315" s="4" t="inlineStr">
-        <is>
-          <t>Stale mount corrected</t>
-        </is>
-      </c>
-      <c r="D315" s="4" t="inlineStr">
-        <is>
-          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
-        </is>
-      </c>
-      <c r="E315" s="4" t="inlineStr">
-        <is>
-          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
-        </is>
-      </c>
-      <c r="F315" s="4" t="n"/>
-      <c r="G315" s="4" t="n"/>
-      <c r="H315" s="4" t="n"/>
-      <c r="I315" s="4" t="n"/>
+      <c r="C315" s="3" t="n"/>
+      <c r="D315" s="3" t="n"/>
+      <c r="E315" s="3" t="n"/>
+      <c r="F315" s="3" t="n"/>
+      <c r="G315" s="3" t="n"/>
+      <c r="H315" s="3" t="n"/>
+      <c r="I315" s="3" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="4" t="inlineStr">
         <is>
-          <t>TC-1406</t>
+          <t>TC-1401</t>
         </is>
       </c>
       <c r="B316" s="4" t="inlineStr">
@@ -9737,17 +9737,17 @@
       </c>
       <c r="C316" s="4" t="inlineStr">
         <is>
-          <t>Active mount preserved</t>
+          <t>Running job failed after restart</t>
         </is>
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share (leave it mounted), restart the service</t>
+          <t>Create a job, start it, restart the service while RUNNING</t>
         </is>
       </c>
       <c r="E316" s="4" t="inlineStr">
         <is>
-          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
+          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
         </is>
       </c>
       <c r="F316" s="4" t="n"/>
@@ -9758,7 +9758,7 @@
     <row r="317">
       <c r="A317" s="4" t="inlineStr">
         <is>
-          <t>TC-1407</t>
+          <t>TC-1402</t>
         </is>
       </c>
       <c r="B317" s="4" t="inlineStr">
@@ -9768,17 +9768,17 @@
       </c>
       <c r="C317" s="4" t="inlineStr">
         <is>
-          <t>USB drives re-discovered</t>
+          <t>Verifying job failed after restart</t>
         </is>
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t>Insert USB drives, restart the service</t>
+          <t>Start a job, let it reach VERIFYING, restart the service</t>
         </is>
       </c>
       <c r="E317" s="4" t="inlineStr">
         <is>
-          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
+          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
         </is>
       </c>
       <c r="F317" s="4" t="n"/>
@@ -9789,7 +9789,7 @@
     <row r="318">
       <c r="A318" s="4" t="inlineStr">
         <is>
-          <t>TC-1408</t>
+          <t>TC-1403</t>
         </is>
       </c>
       <c r="B318" s="4" t="inlineStr">
@@ -9799,17 +9799,17 @@
       </c>
       <c r="C318" s="4" t="inlineStr">
         <is>
-          <t>Idempotency</t>
+          <t>Pending job not affected</t>
         </is>
       </c>
       <c r="D318" s="4" t="inlineStr">
         <is>
-          <t>Restart the service twice without any state changes between restarts</t>
+          <t>Create a job (PENDING), restart the service</t>
         </is>
       </c>
       <c r="E318" s="4" t="inlineStr">
         <is>
-          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
+          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
         </is>
       </c>
       <c r="F318" s="4" t="n"/>
@@ -9820,7 +9820,7 @@
     <row r="319">
       <c r="A319" s="4" t="inlineStr">
         <is>
-          <t>TC-1409</t>
+          <t>TC-1404</t>
         </is>
       </c>
       <c r="B319" s="4" t="inlineStr">
@@ -9830,17 +9830,17 @@
       </c>
       <c r="C319" s="4" t="inlineStr">
         <is>
-          <t>Partial failure isolation</t>
+          <t>Completed job not affected</t>
         </is>
       </c>
       <c r="D319" s="4" t="inlineStr">
         <is>
-          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
+          <t>Complete a job, restart the service</t>
         </is>
       </c>
       <c r="E319" s="4" t="inlineStr">
         <is>
-          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
+          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F319" s="4" t="n"/>
@@ -9851,7 +9851,7 @@
     <row r="320">
       <c r="A320" s="4" t="inlineStr">
         <is>
-          <t>TC-1410</t>
+          <t>TC-1405</t>
         </is>
       </c>
       <c r="B320" s="4" t="inlineStr">
@@ -9861,17 +9861,17 @@
       </c>
       <c r="C320" s="4" t="inlineStr">
         <is>
-          <t>Cross-process lock — only one worker reconciles</t>
+          <t>Stale mount corrected</t>
         </is>
       </c>
       <c r="D320" s="4" t="inlineStr">
         <is>
-          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
+          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
         </is>
       </c>
       <c r="E320" s="4" t="inlineStr">
         <is>
-          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
+          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
         </is>
       </c>
       <c r="F320" s="4" t="n"/>
@@ -9882,7 +9882,7 @@
     <row r="321">
       <c r="A321" s="4" t="inlineStr">
         <is>
-          <t>TC-1411</t>
+          <t>TC-1406</t>
         </is>
       </c>
       <c r="B321" s="4" t="inlineStr">
@@ -9892,17 +9892,17 @@
       </c>
       <c r="C321" s="4" t="inlineStr">
         <is>
-          <t>Stale lock reclaim</t>
+          <t>Active mount preserved</t>
         </is>
       </c>
       <c r="D321" s="4" t="inlineStr">
         <is>
-          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
+          <t>Add and mount a network share (leave it mounted), restart the service</t>
         </is>
       </c>
       <c r="E321" s="4" t="inlineStr">
         <is>
-          <t>Service reclaims the stale lock, reconciliation runs normally</t>
+          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F321" s="4" t="n"/>
@@ -9913,7 +9913,7 @@
     <row r="322">
       <c r="A322" s="4" t="inlineStr">
         <is>
-          <t>TC-1412</t>
+          <t>TC-1407</t>
         </is>
       </c>
       <c r="B322" s="4" t="inlineStr">
@@ -9923,17 +9923,17 @@
       </c>
       <c r="C322" s="4" t="inlineStr">
         <is>
-          <t>Lock released after failure</t>
+          <t>USB drives re-discovered</t>
         </is>
       </c>
       <c r="D322" s="4" t="inlineStr">
         <is>
-          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
+          <t>Insert USB drives, restart the service</t>
         </is>
       </c>
       <c r="E322" s="4" t="inlineStr">
         <is>
-          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
+          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
         </is>
       </c>
       <c r="F322" s="4" t="n"/>
@@ -9944,7 +9944,7 @@
     <row r="323">
       <c r="A323" s="4" t="inlineStr">
         <is>
-          <t>TC-1413</t>
+          <t>TC-1408</t>
         </is>
       </c>
       <c r="B323" s="4" t="inlineStr">
@@ -9954,17 +9954,17 @@
       </c>
       <c r="C323" s="4" t="inlineStr">
         <is>
-          <t>Jobs pass emits immediate startup result log</t>
+          <t>Idempotency</t>
         </is>
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>Create at least one RUNNING job, restart service, then inspect application logs around startup reconciliation</t>
+          <t>Restart the service twice without any state changes between restarts</t>
         </is>
       </c>
       <c r="E323" s="4" t="inlineStr">
         <is>
-          <t>Logs include Startup reconciliation: checking jobs followed by an immediate Startup reconciliation: jobs result line with safe counts (jobs_checked, jobs_corrected) or safe failure classification</t>
+          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
         </is>
       </c>
       <c r="F323" s="4" t="n"/>
@@ -9975,7 +9975,7 @@
     <row r="324">
       <c r="A324" s="4" t="inlineStr">
         <is>
-          <t>TC-1414</t>
+          <t>TC-1409</t>
         </is>
       </c>
       <c r="B324" s="4" t="inlineStr">
@@ -9985,17 +9985,17 @@
       </c>
       <c r="C324" s="4" t="inlineStr">
         <is>
-          <t>Reconciled job persists restart-interruption failure reason</t>
+          <t>Partial failure isolation</t>
         </is>
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>Create a RUNNING or VERIFYING job, restart service, then open Job Detail for that job</t>
+          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
         </is>
       </c>
       <c r="E324" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED and Job Detail shows a stable restart interruption reason (not the generic This job failed... fallback)</t>
+          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
         </is>
       </c>
       <c r="F324" s="4" t="n"/>
@@ -10006,7 +10006,7 @@
     <row r="325">
       <c r="A325" s="4" t="inlineStr">
         <is>
-          <t>TC-1415</t>
+          <t>TC-1410</t>
         </is>
       </c>
       <c r="B325" s="4" t="inlineStr">
@@ -10016,17 +10016,17 @@
       </c>
       <c r="C325" s="4" t="inlineStr">
         <is>
-          <t>Reconciled failed job shows correlated failure entry from audit fallback</t>
+          <t>Cross-process lock — only one worker reconciles</t>
         </is>
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>Restart with a RUNNING job, then inspect Job Detail when no matching file-log failure line is present</t>
+          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
         </is>
       </c>
       <c r="E325" s="4" t="inlineStr">
         <is>
-          <t>Job Detail still shows a related failure entry sourced from reconciliation evidence (JOB_RECONCILED) and the entry remains sanitized</t>
+          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
         </is>
       </c>
       <c r="F325" s="4" t="n"/>
@@ -10037,7 +10037,7 @@
     <row r="326">
       <c r="A326" s="4" t="inlineStr">
         <is>
-          <t>TC-1416</t>
+          <t>TC-1411</t>
         </is>
       </c>
       <c r="B326" s="4" t="inlineStr">
@@ -10047,17 +10047,17 @@
       </c>
       <c r="C326" s="4" t="inlineStr">
         <is>
-          <t>Failed job API uses reconciliation audit fallback when file-log correlation is unavailable</t>
+          <t>Stale lock reclaim</t>
         </is>
       </c>
       <c r="D326" s="4" t="inlineStr">
         <is>
-          <t>In a test environment, disable file-log correlation (log_file unset), then request GET /jobs/{job_id} for a restart-reconciled failed job</t>
+          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
         </is>
       </c>
       <c r="E326" s="4" t="inlineStr">
         <is>
-          <t>Response remains 200 and includes the stable restart failure reason plus a sanitized failure_log_entry derived from audit evidence (JOB_RECONCILED)</t>
+          <t>Service reclaims the stale lock, reconciliation runs normally</t>
         </is>
       </c>
       <c r="F326" s="4" t="n"/>
@@ -10068,7 +10068,7 @@
     <row r="327">
       <c r="A327" s="4" t="inlineStr">
         <is>
-          <t>TC-1417</t>
+          <t>TC-1412</t>
         </is>
       </c>
       <c r="B327" s="4" t="inlineStr">
@@ -10078,17 +10078,17 @@
       </c>
       <c r="C327" s="4" t="inlineStr">
         <is>
-          <t>Jobs pass failure path emits safe startup result classification</t>
+          <t>Lock released after failure</t>
         </is>
       </c>
       <c r="D327" s="4" t="inlineStr">
         <is>
-          <t>In a controlled test environment, force a jobs-pass reconciliation exception, then restart service and inspect startup logs</t>
+          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
         </is>
       </c>
       <c r="E327" s="4" t="inlineStr">
         <is>
-          <t>Logs still include Startup reconciliation: jobs result with status=failed and reason=job_reconciliation_failed, without raw provider errors or host paths</t>
+          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
         </is>
       </c>
       <c r="F327" s="4" t="n"/>
@@ -10097,48 +10097,60 @@
       <c r="I327" s="4" t="n"/>
     </row>
     <row r="328">
-      <c r="A328" s="2" t="inlineStr">
-        <is>
-          <t>§12.15 System Health</t>
-        </is>
-      </c>
-      <c r="B328" s="2" t="inlineStr">
-        <is>
-          <t>12.15 System Health</t>
-        </is>
-      </c>
-      <c r="C328" s="3" t="n"/>
-      <c r="D328" s="3" t="n"/>
-      <c r="E328" s="3" t="n"/>
-      <c r="F328" s="3" t="n"/>
-      <c r="G328" s="3" t="n"/>
-      <c r="H328" s="3" t="n"/>
-      <c r="I328" s="3" t="n"/>
+      <c r="A328" s="4" t="inlineStr">
+        <is>
+          <t>TC-1413</t>
+        </is>
+      </c>
+      <c r="B328" s="4" t="inlineStr">
+        <is>
+          <t>12.14 Startup Reconciliation</t>
+        </is>
+      </c>
+      <c r="C328" s="4" t="inlineStr">
+        <is>
+          <t>Jobs pass emits immediate startup result log</t>
+        </is>
+      </c>
+      <c r="D328" s="4" t="inlineStr">
+        <is>
+          <t>Create at least one RUNNING job, restart service, then inspect application logs around startup reconciliation</t>
+        </is>
+      </c>
+      <c r="E328" s="4" t="inlineStr">
+        <is>
+          <t>Logs include Startup reconciliation: checking jobs followed by an immediate Startup reconciliation: jobs result line with safe counts (jobs_checked, jobs_corrected) or safe failure classification</t>
+        </is>
+      </c>
+      <c r="F328" s="4" t="n"/>
+      <c r="G328" s="4" t="n"/>
+      <c r="H328" s="4" t="n"/>
+      <c r="I328" s="4" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="4" t="inlineStr">
         <is>
-          <t>TC-1501</t>
+          <t>TC-1414</t>
         </is>
       </c>
       <c r="B329" s="4" t="inlineStr">
         <is>
-          <t>12.15 System Health</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C329" s="4" t="inlineStr">
         <is>
-          <t>Healthy response</t>
+          <t>Reconciled job persists restart-interruption failure reason</t>
         </is>
       </c>
       <c r="D329" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with valid token</t>
+          <t>Create a RUNNING or VERIFYING job, restart service, then open Job Detail for that job</t>
         </is>
       </c>
       <c r="E329" s="4" t="inlineStr">
         <is>
-          <t>200, status: "ok", database: "connected"</t>
+          <t>Job status is FAILED and Job Detail shows a stable restart interruption reason (not the generic This job failed... fallback)</t>
         </is>
       </c>
       <c r="F329" s="4" t="n"/>
@@ -10149,27 +10161,27 @@
     <row r="330">
       <c r="A330" s="4" t="inlineStr">
         <is>
-          <t>TC-1502</t>
+          <t>TC-1415</t>
         </is>
       </c>
       <c r="B330" s="4" t="inlineStr">
         <is>
-          <t>12.15 System Health</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C330" s="4" t="inlineStr">
         <is>
-          <t>CPU metric present</t>
+          <t>Reconciled failed job shows correlated failure entry from audit fallback</t>
         </is>
       </c>
       <c r="D330" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Restart with a RUNNING job, then inspect Job Detail when no matching file-log failure line is present</t>
         </is>
       </c>
       <c r="E330" s="4" t="inlineStr">
         <is>
-          <t>cpu_percent is a number between 0 and 100</t>
+          <t>Job Detail still shows a related failure entry sourced from reconciliation evidence (JOB_RECONCILED) and the entry remains sanitized</t>
         </is>
       </c>
       <c r="F330" s="4" t="n"/>
@@ -10180,27 +10192,27 @@
     <row r="331">
       <c r="A331" s="4" t="inlineStr">
         <is>
-          <t>TC-1503</t>
+          <t>TC-1416</t>
         </is>
       </c>
       <c r="B331" s="4" t="inlineStr">
         <is>
-          <t>12.15 System Health</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C331" s="4" t="inlineStr">
         <is>
-          <t>Memory metrics present</t>
+          <t>Failed job API uses reconciliation audit fallback when file-log correlation is unavailable</t>
         </is>
       </c>
       <c r="D331" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>In a test environment, disable file-log correlation (log_file unset), then request GET /jobs/{job_id} for a restart-reconciled failed job</t>
         </is>
       </c>
       <c r="E331" s="4" t="inlineStr">
         <is>
-          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
+          <t>Response remains 200 and includes the stable restart failure reason plus a sanitized failure_log_entry derived from audit evidence (JOB_RECONCILED)</t>
         </is>
       </c>
       <c r="F331" s="4" t="n"/>
@@ -10211,27 +10223,27 @@
     <row r="332">
       <c r="A332" s="4" t="inlineStr">
         <is>
-          <t>TC-1504</t>
+          <t>TC-1417</t>
         </is>
       </c>
       <c r="B332" s="4" t="inlineStr">
         <is>
-          <t>12.15 System Health</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C332" s="4" t="inlineStr">
         <is>
-          <t>Disk I/O metrics present</t>
+          <t>Jobs pass failure path emits safe startup result classification</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>In a controlled test environment, force a jobs-pass reconciliation exception, then restart service and inspect startup logs</t>
         </is>
       </c>
       <c r="E332" s="4" t="inlineStr">
         <is>
-          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
+          <t>Logs still include Startup reconciliation: jobs result with status=failed and reason=job_reconciliation_failed, without raw provider errors or host paths</t>
         </is>
       </c>
       <c r="F332" s="4" t="n"/>
@@ -10240,40 +10252,28 @@
       <c r="I332" s="4" t="n"/>
     </row>
     <row r="333">
-      <c r="A333" s="4" t="inlineStr">
-        <is>
-          <t>TC-1505</t>
-        </is>
-      </c>
-      <c r="B333" s="4" t="inlineStr">
+      <c r="A333" s="2" t="inlineStr">
+        <is>
+          <t>§12.15 System Health</t>
+        </is>
+      </c>
+      <c r="B333" s="2" t="inlineStr">
         <is>
           <t>12.15 System Health</t>
         </is>
       </c>
-      <c r="C333" s="4" t="inlineStr">
-        <is>
-          <t>Active jobs count</t>
-        </is>
-      </c>
-      <c r="D333" s="4" t="inlineStr">
-        <is>
-          <t>Start an export job, call endpoint</t>
-        </is>
-      </c>
-      <c r="E333" s="4" t="inlineStr">
-        <is>
-          <t>active_jobs ≥ 1</t>
-        </is>
-      </c>
-      <c r="F333" s="4" t="n"/>
-      <c r="G333" s="4" t="n"/>
-      <c r="H333" s="4" t="n"/>
-      <c r="I333" s="4" t="n"/>
+      <c r="C333" s="3" t="n"/>
+      <c r="D333" s="3" t="n"/>
+      <c r="E333" s="3" t="n"/>
+      <c r="F333" s="3" t="n"/>
+      <c r="G333" s="3" t="n"/>
+      <c r="H333" s="3" t="n"/>
+      <c r="I333" s="3" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="4" t="inlineStr">
         <is>
-          <t>TC-1506</t>
+          <t>TC-1501</t>
         </is>
       </c>
       <c r="B334" s="4" t="inlineStr">
@@ -10283,17 +10283,17 @@
       </c>
       <c r="C334" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size</t>
+          <t>Healthy response</t>
         </is>
       </c>
       <c r="D334" s="4" t="inlineStr">
         <is>
-          <t>Create a PENDING job (created but not started), call endpoint</t>
+          <t>GET /introspection/system-health with valid token</t>
         </is>
       </c>
       <c r="E334" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size ≥ 1</t>
+          <t>200, status: "ok", database: "connected"</t>
         </is>
       </c>
       <c r="F334" s="4" t="n"/>
@@ -10304,7 +10304,7 @@
     <row r="335">
       <c r="A335" s="4" t="inlineStr">
         <is>
-          <t>TC-1507</t>
+          <t>TC-1502</t>
         </is>
       </c>
       <c r="B335" s="4" t="inlineStr">
@@ -10314,17 +10314,17 @@
       </c>
       <c r="C335" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size decrements</t>
+          <t>CPU metric present</t>
         </is>
       </c>
       <c r="D335" s="4" t="inlineStr">
         <is>
-          <t>Start the pending job, call endpoint again</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E335" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
+          <t>cpu_percent is a number between 0 and 100</t>
         </is>
       </c>
       <c r="F335" s="4" t="n"/>
@@ -10335,7 +10335,7 @@
     <row r="336">
       <c r="A336" s="4" t="inlineStr">
         <is>
-          <t>TC-1508</t>
+          <t>TC-1503</t>
         </is>
       </c>
       <c r="B336" s="4" t="inlineStr">
@@ -10345,17 +10345,17 @@
       </c>
       <c r="C336" s="4" t="inlineStr">
         <is>
-          <t>Degraded when DB down</t>
+          <t>Memory metrics present</t>
         </is>
       </c>
       <c r="D336" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, call endpoint with valid token</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E336" s="4" t="inlineStr">
         <is>
-          <t>200, status: "degraded", database: "error", database_error is non-null</t>
+          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
         </is>
       </c>
       <c r="F336" s="4" t="n"/>
@@ -10366,7 +10366,7 @@
     <row r="337">
       <c r="A337" s="4" t="inlineStr">
         <is>
-          <t>TC-1509</t>
+          <t>TC-1504</t>
         </is>
       </c>
       <c r="B337" s="4" t="inlineStr">
@@ -10376,17 +10376,17 @@
       </c>
       <c r="C337" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated rejected</t>
+          <t>Disk I/O metrics present</t>
         </is>
       </c>
       <c r="D337" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health without token</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E337" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
         </is>
       </c>
       <c r="F337" s="4" t="n"/>
@@ -10397,7 +10397,7 @@
     <row r="338">
       <c r="A338" s="4" t="inlineStr">
         <is>
-          <t>TC-1510</t>
+          <t>TC-1505</t>
         </is>
       </c>
       <c r="B338" s="4" t="inlineStr">
@@ -10407,17 +10407,17 @@
       </c>
       <c r="C338" s="4" t="inlineStr">
         <is>
-          <t>Processor role allowed</t>
+          <t>Active jobs count</t>
         </is>
       </c>
       <c r="D338" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with processor token</t>
+          <t>Start an export job, call endpoint</t>
         </is>
       </c>
       <c r="E338" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>active_jobs ≥ 1</t>
         </is>
       </c>
       <c r="F338" s="4" t="n"/>
@@ -10426,48 +10426,60 @@
       <c r="I338" s="4" t="n"/>
     </row>
     <row r="339">
-      <c r="A339" s="2" t="inlineStr">
-        <is>
-          <t>§12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="B339" s="2" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C339" s="3" t="n"/>
-      <c r="D339" s="3" t="n"/>
-      <c r="E339" s="3" t="n"/>
-      <c r="F339" s="3" t="n"/>
-      <c r="G339" s="3" t="n"/>
-      <c r="H339" s="3" t="n"/>
-      <c r="I339" s="3" t="n"/>
+      <c r="A339" s="4" t="inlineStr">
+        <is>
+          <t>TC-1506</t>
+        </is>
+      </c>
+      <c r="B339" s="4" t="inlineStr">
+        <is>
+          <t>12.15 System Health</t>
+        </is>
+      </c>
+      <c r="C339" s="4" t="inlineStr">
+        <is>
+          <t>Worker queue size</t>
+        </is>
+      </c>
+      <c r="D339" s="4" t="inlineStr">
+        <is>
+          <t>Create a PENDING job (created but not started), call endpoint</t>
+        </is>
+      </c>
+      <c r="E339" s="4" t="inlineStr">
+        <is>
+          <t>worker_queue_size ≥ 1</t>
+        </is>
+      </c>
+      <c r="F339" s="4" t="n"/>
+      <c r="G339" s="4" t="n"/>
+      <c r="H339" s="4" t="n"/>
+      <c r="I339" s="4" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="4" t="inlineStr">
         <is>
-          <t>TC-1511</t>
+          <t>TC-1507</t>
         </is>
       </c>
       <c r="B340" s="4" t="inlineStr">
         <is>
-          <t>12.15.1 Readiness &amp; Version</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C340" s="4" t="inlineStr">
         <is>
-          <t>Liveness endpoint is public</t>
+          <t>Worker queue size decrements</t>
         </is>
       </c>
       <c r="D340" s="4" t="inlineStr">
         <is>
-          <t>GET /health/live without token</t>
+          <t>Start the pending job, call endpoint again</t>
         </is>
       </c>
       <c r="E340" s="4" t="inlineStr">
         <is>
-          <t>200, service reports live</t>
+          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
         </is>
       </c>
       <c r="F340" s="4" t="n"/>
@@ -10478,27 +10490,27 @@
     <row r="341">
       <c r="A341" s="4" t="inlineStr">
         <is>
-          <t>TC-1512</t>
+          <t>TC-1508</t>
         </is>
       </c>
       <c r="B341" s="4" t="inlineStr">
         <is>
-          <t>12.15.1 Readiness &amp; Version</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C341" s="4" t="inlineStr">
         <is>
-          <t>Readiness endpoint is public</t>
+          <t>Degraded when DB down</t>
         </is>
       </c>
       <c r="D341" s="4" t="inlineStr">
         <is>
-          <t>GET /health/ready without token on a healthy system</t>
+          <t>Stop PostgreSQL, call endpoint with valid token</t>
         </is>
       </c>
       <c r="E341" s="4" t="inlineStr">
         <is>
-          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
+          <t>200, status: "degraded", database: "error", database_error is non-null</t>
         </is>
       </c>
       <c r="F341" s="4" t="n"/>
@@ -10509,27 +10521,27 @@
     <row r="342">
       <c r="A342" s="4" t="inlineStr">
         <is>
-          <t>TC-1513</t>
+          <t>TC-1509</t>
         </is>
       </c>
       <c r="B342" s="4" t="inlineStr">
         <is>
-          <t>12.15.1 Readiness &amp; Version</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C342" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports missing database configuration</t>
+          <t>Unauthenticated rejected</t>
         </is>
       </c>
       <c r="D342" s="4" t="inlineStr">
         <is>
-          <t>Clear DB config or test before configuration, then GET /health/ready</t>
+          <t>GET /introspection/system-health without token</t>
         </is>
       </c>
       <c r="E342" s="4" t="inlineStr">
         <is>
-          <t>503, status: "not_ready", reason indicates database is not configured</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F342" s="4" t="n"/>
@@ -10540,27 +10552,27 @@
     <row r="343">
       <c r="A343" s="4" t="inlineStr">
         <is>
-          <t>TC-1514</t>
+          <t>TC-1510</t>
         </is>
       </c>
       <c r="B343" s="4" t="inlineStr">
         <is>
-          <t>12.15.1 Readiness &amp; Version</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C343" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports mount or provider problems</t>
+          <t>Processor role allowed</t>
         </is>
       </c>
       <c r="D343" s="4" t="inlineStr">
         <is>
-          <t>Break a configured mount or provider, then GET /health/ready</t>
+          <t>GET /introspection/system-health with processor token</t>
         </is>
       </c>
       <c r="E343" s="4" t="inlineStr">
         <is>
-          <t>503, response identifies the failing check without using the generic error schema</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F343" s="4" t="n"/>
@@ -10569,40 +10581,28 @@
       <c r="I343" s="4" t="n"/>
     </row>
     <row r="344">
-      <c r="A344" s="4" t="inlineStr">
-        <is>
-          <t>TC-1515</t>
-        </is>
-      </c>
-      <c r="B344" s="4" t="inlineStr">
+      <c r="A344" s="2" t="inlineStr">
+        <is>
+          <t>§12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="B344" s="2" t="inlineStr">
         <is>
           <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
-      <c r="C344" s="4" t="inlineStr">
-        <is>
-          <t>Version endpoint is public</t>
-        </is>
-      </c>
-      <c r="D344" s="4" t="inlineStr">
-        <is>
-          <t>GET /introspection/version without token</t>
-        </is>
-      </c>
-      <c r="E344" s="4" t="inlineStr">
-        <is>
-          <t>200, returns version/application metadata</t>
-        </is>
-      </c>
-      <c r="F344" s="4" t="n"/>
-      <c r="G344" s="4" t="n"/>
-      <c r="H344" s="4" t="n"/>
-      <c r="I344" s="4" t="n"/>
+      <c r="C344" s="3" t="n"/>
+      <c r="D344" s="3" t="n"/>
+      <c r="E344" s="3" t="n"/>
+      <c r="F344" s="3" t="n"/>
+      <c r="G344" s="3" t="n"/>
+      <c r="H344" s="3" t="n"/>
+      <c r="I344" s="3" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="4" t="inlineStr">
         <is>
-          <t>TC-1516</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B345" s="4" t="inlineStr">
@@ -10612,17 +10612,17 @@
       </c>
       <c r="C345" s="4" t="inlineStr">
         <is>
-          <t>Readiness remains separate from authenticated system health</t>
+          <t>Liveness endpoint is public</t>
         </is>
       </c>
       <c r="D345" s="4" t="inlineStr">
         <is>
-          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+          <t>GET /health/live without token</t>
         </is>
       </c>
       <c r="E345" s="4" t="inlineStr">
         <is>
-          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+          <t>200, service reports live</t>
         </is>
       </c>
       <c r="F345" s="4" t="n"/>
@@ -10631,32 +10631,187 @@
       <c r="I345" s="4" t="n"/>
     </row>
     <row r="346">
-      <c r="A346" s="2" t="inlineStr">
+      <c r="A346" s="4" t="inlineStr">
+        <is>
+          <t>TC-1512</t>
+        </is>
+      </c>
+      <c r="B346" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C346" s="4" t="inlineStr">
+        <is>
+          <t>Readiness endpoint is public</t>
+        </is>
+      </c>
+      <c r="D346" s="4" t="inlineStr">
+        <is>
+          <t>GET /health/ready without token on a healthy system</t>
+        </is>
+      </c>
+      <c r="E346" s="4" t="inlineStr">
+        <is>
+          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
+        </is>
+      </c>
+      <c r="F346" s="4" t="n"/>
+      <c r="G346" s="4" t="n"/>
+      <c r="H346" s="4" t="n"/>
+      <c r="I346" s="4" t="n"/>
+    </row>
+    <row r="347">
+      <c r="A347" s="4" t="inlineStr">
+        <is>
+          <t>TC-1513</t>
+        </is>
+      </c>
+      <c r="B347" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C347" s="4" t="inlineStr">
+        <is>
+          <t>Readiness reports missing database configuration</t>
+        </is>
+      </c>
+      <c r="D347" s="4" t="inlineStr">
+        <is>
+          <t>Clear DB config or test before configuration, then GET /health/ready</t>
+        </is>
+      </c>
+      <c r="E347" s="4" t="inlineStr">
+        <is>
+          <t>503, status: "not_ready", reason indicates database is not configured</t>
+        </is>
+      </c>
+      <c r="F347" s="4" t="n"/>
+      <c r="G347" s="4" t="n"/>
+      <c r="H347" s="4" t="n"/>
+      <c r="I347" s="4" t="n"/>
+    </row>
+    <row r="348">
+      <c r="A348" s="4" t="inlineStr">
+        <is>
+          <t>TC-1514</t>
+        </is>
+      </c>
+      <c r="B348" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C348" s="4" t="inlineStr">
+        <is>
+          <t>Readiness reports mount or provider problems</t>
+        </is>
+      </c>
+      <c r="D348" s="4" t="inlineStr">
+        <is>
+          <t>Break a configured mount or provider, then GET /health/ready</t>
+        </is>
+      </c>
+      <c r="E348" s="4" t="inlineStr">
+        <is>
+          <t>503, response identifies the failing check without using the generic error schema</t>
+        </is>
+      </c>
+      <c r="F348" s="4" t="n"/>
+      <c r="G348" s="4" t="n"/>
+      <c r="H348" s="4" t="n"/>
+      <c r="I348" s="4" t="n"/>
+    </row>
+    <row r="349">
+      <c r="A349" s="4" t="inlineStr">
+        <is>
+          <t>TC-1515</t>
+        </is>
+      </c>
+      <c r="B349" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C349" s="4" t="inlineStr">
+        <is>
+          <t>Version endpoint is public</t>
+        </is>
+      </c>
+      <c r="D349" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/version without token</t>
+        </is>
+      </c>
+      <c r="E349" s="4" t="inlineStr">
+        <is>
+          <t>200, returns version/application metadata</t>
+        </is>
+      </c>
+      <c r="F349" s="4" t="n"/>
+      <c r="G349" s="4" t="n"/>
+      <c r="H349" s="4" t="n"/>
+      <c r="I349" s="4" t="n"/>
+    </row>
+    <row r="350">
+      <c r="A350" s="4" t="inlineStr">
+        <is>
+          <t>TC-1516</t>
+        </is>
+      </c>
+      <c r="B350" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C350" s="4" t="inlineStr">
+        <is>
+          <t>Readiness remains separate from authenticated system health</t>
+        </is>
+      </c>
+      <c r="D350" s="4" t="inlineStr">
+        <is>
+          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+        </is>
+      </c>
+      <c r="E350" s="4" t="inlineStr">
+        <is>
+          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+        </is>
+      </c>
+      <c r="F350" s="4" t="n"/>
+      <c r="G350" s="4" t="n"/>
+      <c r="H350" s="4" t="n"/>
+      <c r="I350" s="4" t="n"/>
+    </row>
+    <row r="351">
+      <c r="A351" s="2" t="inlineStr">
         <is>
           <t>§12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="B346" s="2" t="inlineStr">
+      <c r="B351" s="2" t="inlineStr">
         <is>
           <t>12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="C346" s="3" t="n"/>
-      <c r="D346" s="3" t="n"/>
-      <c r="E346" s="3" t="n"/>
-      <c r="F346" s="3" t="n"/>
-      <c r="G346" s="3" t="n"/>
-      <c r="H346" s="3" t="n"/>
-      <c r="I346" s="3" t="n"/>
-    </row>
-    <row r="348">
-      <c r="A348" s="5" t="inlineStr">
+      <c r="C351" s="3" t="n"/>
+      <c r="D351" s="3" t="n"/>
+      <c r="E351" s="3" t="n"/>
+      <c r="F351" s="3" t="n"/>
+      <c r="G351" s="3" t="n"/>
+      <c r="H351" s="3" t="n"/>
+      <c r="I351" s="3" t="n"/>
+    </row>
+    <row r="353">
+      <c r="A353" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B348" s="5" t="n">
-        <v>318</v>
+      <c r="B353" s="5" t="n">
+        <v>323</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Treat custody handoff delivery time as local input converted to UTC
Relabel the handoff delivery-time field to reflect browser-local entry,
convert the submitted value to UTC ISO 8601 before sending it to the API, and refresh QA documentation and visual baselines to match the updated UI behavior.
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -9234,7 +9234,7 @@
       </c>
       <c r="C299" s="4" t="inlineStr">
         <is>
-          <t>Re-initialize persists runtime flags</t>
+          <t>Re-initialize does not mutate runtime flags</t>
         </is>
       </c>
       <c r="D299" s="4" t="inlineStr">
@@ -9244,7 +9244,7 @@
       </c>
       <c r="E299" s="4" t="inlineStr">
         <is>
-          <t>200, status=already_initialized, runtime flag updated</t>
+          <t>200, status=already_initialized, runtime TRUST_PROXY_HEADERS remains unchanged</t>
         </is>
       </c>
       <c r="F299" s="4" t="n"/>

</xml_diff>

<commit_message>
Add partial-success retry flow for completed jobs
Expose a retry-failed job action that re-queues only ERROR and TIMEOUT file rows,
preserves successful copies, and audits the restart on completed jobs.

Update Job Detail to surface Retry Failed Files and flag partial-success
completions with red summary styling, with tests and operator/QA docs aligned.
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -4744,17 +4744,17 @@
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>Completion summary is visible</t>
+          <t>Completion summary reflects clean vs partial-success state</t>
         </is>
       </c>
       <c r="D149" s="4" t="inlineStr">
         <is>
-          <t>Let a job finish and open its detail page</t>
+          <t>Let one job finish cleanly and let a second job finish COMPLETED with at least one failed or timed-out file, then open each detail page</t>
         </is>
       </c>
       <c r="E149" s="4" t="inlineStr">
         <is>
-          <t>The detail screen shows start time, copy threads, files copied, files failed, files timed out, total copied, elapsed time, and copy rate</t>
+          <t>Both detail screens show start time, copy threads, files copied, files failed, files timed out, total copied, elapsed time, and copy rate; the clean completion keeps normal success styling while the partial-success completion uses the red failure styling</t>
         </is>
       </c>
       <c r="F149" s="4" t="n"/>

</xml_diff>

<commit_message>
Document stored job-scoped CoC snapshot workflow
Align operator, API, architecture, and QA docs with the job-detail CoC flow. Describe stored-snapshot reads, explicit refresh-and-persist behavior, archived-job recall, and updated handoff endpoints.
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -9489,17 +9489,17 @@
       </c>
       <c r="C308" s="4" t="inlineStr">
         <is>
-          <t>Retrieve CoC — by drive_id</t>
+          <t>Retrieve stored CoC snapshot — archived job</t>
         </is>
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>GET /audit/chain-of-custody?drive_id=42 with auditor/manager/admin token</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for an archived job that already has a stored snapshot</t>
         </is>
       </c>
       <c r="E308" s="4" t="inlineStr">
         <is>
-          <t>200, selector_mode: "DRIVE_ID", report contains events for that drive</t>
+          <t>200, response contains the stored snapshot and snapshot metadata</t>
         </is>
       </c>
       <c r="F308" s="4" t="n"/>
@@ -9520,17 +9520,17 @@
       </c>
       <c r="C309" s="4" t="inlineStr">
         <is>
-          <t>Retrieve CoC — by drive_sn</t>
+          <t>Retrieve stored CoC snapshot — active job</t>
         </is>
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>GET /audit/chain-of-custody?drive_sn=ABC123DEF with manager token</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job that already has a stored snapshot</t>
         </is>
       </c>
       <c r="E309" s="4" t="inlineStr">
         <is>
-          <t>200, selector_mode: "DRIVE_SN", report contains events for that drive</t>
+          <t>200, response contains the stored snapshot and does not regenerate it</t>
         </is>
       </c>
       <c r="F309" s="4" t="n"/>
@@ -9551,17 +9551,17 @@
       </c>
       <c r="C310" s="4" t="inlineStr">
         <is>
-          <t>Retrieve CoC — by project_id</t>
+          <t>CoC read — missing stored snapshot</t>
         </is>
       </c>
       <c r="D310" s="4" t="inlineStr">
         <is>
-          <t>GET /audit/chain-of-custody?project_id=CASE-2026-007 with auditor token</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job with no stored snapshot yet</t>
         </is>
       </c>
       <c r="E310" s="4" t="inlineStr">
         <is>
-          <t>200, selector_mode: "PROJECT", reports array contains all non-archived drives for project</t>
+          <t>404, message explains that the report must be refreshed first</t>
         </is>
       </c>
       <c r="F310" s="4" t="n"/>
@@ -9582,12 +9582,12 @@
       </c>
       <c r="C311" s="4" t="inlineStr">
         <is>
-          <t>CoC — processor denied</t>
+          <t>CoC read — processor denied</t>
         </is>
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>GET /audit/chain-of-custody?drive_id=42 with processor token</t>
+          <t>GET /jobs/{job_id}/chain-of-custody with processor token</t>
         </is>
       </c>
       <c r="E311" s="4" t="inlineStr">
@@ -9613,12 +9613,12 @@
       </c>
       <c r="C312" s="4" t="inlineStr">
         <is>
-          <t>CoC — unauthenticated denied</t>
+          <t>CoC read — unauthenticated denied</t>
         </is>
       </c>
       <c r="D312" s="4" t="inlineStr">
         <is>
-          <t>GET /audit/chain-of-custody?drive_id=42 without token</t>
+          <t>GET /jobs/{job_id}/chain-of-custody without token</t>
         </is>
       </c>
       <c r="E312" s="4" t="inlineStr">
@@ -9644,17 +9644,17 @@
       </c>
       <c r="C313" s="4" t="inlineStr">
         <is>
-          <t>CoC — no selector</t>
+          <t>CoC snapshot fields</t>
         </is>
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>GET /audit/chain-of-custody with no query parameters</t>
+          <t>Inspect any stored-snapshot response</t>
         </is>
       </c>
       <c r="E313" s="4" t="inlineStr">
         <is>
-          <t>422, at least one selector required</t>
+          <t>snapshot_stored_at, snapshot_updated_at, snapshot_stored_by, reports[], and manifest/custody fields are present</t>
         </is>
       </c>
       <c r="F313" s="4" t="n"/>
@@ -9675,17 +9675,17 @@
       </c>
       <c r="C314" s="4" t="inlineStr">
         <is>
-          <t>CoC — drive_id takes precedence</t>
+          <t>CoC events include lifecycle</t>
         </is>
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>GET /audit/chain-of-custody?drive_id=42&amp;drive_sn=ABC&amp;project_id=CASE-X</t>
+          <t>Inspect chain_of_custody_events in a stored report for a completed job</t>
         </is>
       </c>
       <c r="E314" s="4" t="inlineStr">
         <is>
-          <t>200, selector_mode: "DRIVE_ID" (ignores other selectors)</t>
+          <t>Events include DRIVE_INITIALIZED, JOB_CREATED, JOB_STARTED, JOB_COMPLETED, DRIVE_EJECT_PREPARED, and COC_HANDOFF_CONFIRMED when applicable</t>
         </is>
       </c>
       <c r="F314" s="4" t="n"/>
@@ -9706,17 +9706,17 @@
       </c>
       <c r="C315" s="4" t="inlineStr">
         <is>
-          <t>CoC — project_id mismatch</t>
+          <t>CoC manifest summary</t>
         </is>
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>GET /audit/chain-of-custody?drive_id=42&amp;project_id=WRONG-PROJECT where drive is bound to different project</t>
+          <t>Inspect manifest_summary in the stored report</t>
         </is>
       </c>
       <c r="E315" s="4" t="inlineStr">
         <is>
-          <t>409, CONFLICT, mismatch detail</t>
+          <t>Array of objects with job_id, evidence_number, processor_notes, total_files, total_bytes, and manifest_count</t>
         </is>
       </c>
       <c r="F315" s="4" t="n"/>
@@ -9737,17 +9737,17 @@
       </c>
       <c r="C316" s="4" t="inlineStr">
         <is>
-          <t>CoC report fields</t>
+          <t>CoC — delivery_time absence (no handoff)</t>
         </is>
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>Inspect any GET /audit/chain-of-custody response</t>
+          <t>Complete a job and store a snapshot before handoff</t>
         </is>
       </c>
       <c r="E316" s="4" t="inlineStr">
         <is>
-          <t>reports[].drive_id, reports[].drive_sn, reports[].project_id, reports[].custody_complete, reports[].chain_of_custody_events present</t>
+          <t>chain_of_custody_events do not contain COC_HANDOFF_CONFIRMED; custody_complete is false</t>
         </is>
       </c>
       <c r="F316" s="4" t="n"/>
@@ -9768,17 +9768,17 @@
       </c>
       <c r="C317" s="4" t="inlineStr">
         <is>
-          <t>CoC events include lifecycle</t>
+          <t>CoC refresh — valid</t>
         </is>
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t>Inspect chain_of_custody_events in a report with completed job</t>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh with admin or manager token for a non-archived job with assignments</t>
         </is>
       </c>
       <c r="E317" s="4" t="inlineStr">
         <is>
-          <t>Events include DRIVE_INITIALIZED, JOB_CREATED, JOB_STARTED, JOB_COMPLETED, DRIVE_EJECT_PREPARED, COC_HANDOFF_CONFIRMED (if handed off)</t>
+          <t>200, response contains the refreshed stored snapshot and updated snapshot metadata</t>
         </is>
       </c>
       <c r="F317" s="4" t="n"/>
@@ -9799,17 +9799,17 @@
       </c>
       <c r="C318" s="4" t="inlineStr">
         <is>
-          <t>CoC manifest summary</t>
+          <t>CoC refresh — auditor denied</t>
         </is>
       </c>
       <c r="D318" s="4" t="inlineStr">
         <is>
-          <t>Inspect manifest_summary in CoC report</t>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh with auditor token</t>
         </is>
       </c>
       <c r="E318" s="4" t="inlineStr">
         <is>
-          <t>Array of objects with job_id, total_files, total_bytes, manifest_count</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F318" s="4" t="n"/>
@@ -9830,17 +9830,17 @@
       </c>
       <c r="C319" s="4" t="inlineStr">
         <is>
-          <t>CoC — delivery_time absence (no handoff)</t>
+          <t>CoC refresh — archived job denied</t>
         </is>
       </c>
       <c r="D319" s="4" t="inlineStr">
         <is>
-          <t>Complete a job and eject without handoff, query GET /audit/chain-of-custody?drive_id=...</t>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh for an archived job</t>
         </is>
       </c>
       <c r="E319" s="4" t="inlineStr">
         <is>
-          <t>chain_of_custody_events do not contain COC_HANDOFF_CONFIRMED; custody_complete is false</t>
+          <t>409, archived jobs can only return the last stored snapshot</t>
         </is>
       </c>
       <c r="F319" s="4" t="n"/>

</xml_diff>

<commit_message>
Add configurable webhook callback payload mapping
Allow administrators to constrain and remap outbound callback payloads
with an explicit allowlist and deterministic field templates.

Expand the callback payload and docs to cover operator, timing, and
destination drive metadata, and add backend/frontend tests for
configuration validation, persistence, signing, and raw-body receiver
verification.
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I360"/>
+  <dimension ref="A1:I362"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8769,23 +8769,35 @@
       <c r="I283" s="4" t="n"/>
     </row>
     <row r="284">
-      <c r="A284" s="2" t="inlineStr">
-        <is>
-          <t>§12.10.2 Help System</t>
-        </is>
-      </c>
-      <c r="B284" s="2" t="inlineStr">
-        <is>
-          <t>12.10.2 Help System</t>
-        </is>
-      </c>
-      <c r="C284" s="3" t="n"/>
-      <c r="D284" s="3" t="n"/>
-      <c r="E284" s="3" t="n"/>
-      <c r="F284" s="3" t="n"/>
-      <c r="G284" s="3" t="n"/>
-      <c r="H284" s="3" t="n"/>
-      <c r="I284" s="3" t="n"/>
+      <c r="A284" s="4" t="inlineStr">
+        <is>
+          <t>TC-1020</t>
+        </is>
+      </c>
+      <c r="B284" s="4" t="inlineStr">
+        <is>
+          <t>12.10.1 Runtime Configuration</t>
+        </is>
+      </c>
+      <c r="C284" s="4" t="inlineStr">
+        <is>
+          <t>Accept callback payload allowlist and mapping</t>
+        </is>
+      </c>
+      <c r="D284" s="4" t="inlineStr">
+        <is>
+          <t>PUT /admin/configuration with {"callback_payload_fields": ["event", "project_id"], "callback_payload_field_map": {"type": "event", "project": "project_id"}}</t>
+        </is>
+      </c>
+      <c r="E284" s="4" t="inlineStr">
+        <is>
+          <t>200, changed settings include both callback payload fields</t>
+        </is>
+      </c>
+      <c r="F284" s="4" t="n"/>
+      <c r="G284" s="4" t="n"/>
+      <c r="H284" s="4" t="n"/>
+      <c r="I284" s="4" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="4" t="inlineStr">
@@ -8795,22 +8807,22 @@
       </c>
       <c r="B285" s="4" t="inlineStr">
         <is>
-          <t>12.10.2 Help System</t>
+          <t>12.10.1 Runtime Configuration</t>
         </is>
       </c>
       <c r="C285" s="4" t="inlineStr">
         <is>
-          <t>Help trigger is visible in authenticated shell</t>
+          <t>Reject invalid callback payload mapping</t>
         </is>
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t>Sign in to the application and inspect the shell/header</t>
+          <t>PUT /admin/configuration with {"callback_payload_field_map": {"summary": "${unknown_field}"}}</t>
         </is>
       </c>
       <c r="E285" s="4" t="inlineStr">
         <is>
-          <t>A Help trigger is visible without navigating away from the current page</t>
+          <t>422, validation error identifies the invalid mapping source field</t>
         </is>
       </c>
       <c r="F285" s="4" t="n"/>
@@ -8819,40 +8831,28 @@
       <c r="I285" s="4" t="n"/>
     </row>
     <row r="286">
-      <c r="A286" s="4" t="inlineStr">
-        <is>
-          <t>TC-1022</t>
-        </is>
-      </c>
-      <c r="B286" s="4" t="inlineStr">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>§12.10.2 Help System</t>
+        </is>
+      </c>
+      <c r="B286" s="2" t="inlineStr">
         <is>
           <t>12.10.2 Help System</t>
         </is>
       </c>
-      <c r="C286" s="4" t="inlineStr">
-        <is>
-          <t>Help opens in-app</t>
-        </is>
-      </c>
-      <c r="D286" s="4" t="inlineStr">
-        <is>
-          <t>Activate the Help trigger from any primary page</t>
-        </is>
-      </c>
-      <c r="E286" s="4" t="inlineStr">
-        <is>
-          <t>Help opens in a modal or equivalent in-app panel</t>
-        </is>
-      </c>
-      <c r="F286" s="4" t="n"/>
-      <c r="G286" s="4" t="n"/>
-      <c r="H286" s="4" t="n"/>
-      <c r="I286" s="4" t="n"/>
+      <c r="C286" s="3" t="n"/>
+      <c r="D286" s="3" t="n"/>
+      <c r="E286" s="3" t="n"/>
+      <c r="F286" s="3" t="n"/>
+      <c r="G286" s="3" t="n"/>
+      <c r="H286" s="3" t="n"/>
+      <c r="I286" s="3" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="4" t="inlineStr">
         <is>
-          <t>TC-1023</t>
+          <t>TC-1021</t>
         </is>
       </c>
       <c r="B287" s="4" t="inlineStr">
@@ -8862,17 +8862,17 @@
       </c>
       <c r="C287" s="4" t="inlineStr">
         <is>
-          <t>Help does not break current workflow context</t>
+          <t>Help trigger is visible in authenticated shell</t>
         </is>
       </c>
       <c r="D287" s="4" t="inlineStr">
         <is>
-          <t>Open Help while on Drives, Mounts, Jobs, or Audit, then close it</t>
+          <t>Sign in to the application and inspect the shell/header</t>
         </is>
       </c>
       <c r="E287" s="4" t="inlineStr">
         <is>
-          <t>Closing Help returns to the same page and preserved workflow context</t>
+          <t>A Help trigger is visible without navigating away from the current page</t>
         </is>
       </c>
       <c r="F287" s="4" t="n"/>
@@ -8883,7 +8883,7 @@
     <row r="288">
       <c r="A288" s="4" t="inlineStr">
         <is>
-          <t>TC-1024</t>
+          <t>TC-1022</t>
         </is>
       </c>
       <c r="B288" s="4" t="inlineStr">
@@ -8893,17 +8893,17 @@
       </c>
       <c r="C288" s="4" t="inlineStr">
         <is>
-          <t>Help content is curated and user-facing</t>
+          <t>Help opens in-app</t>
         </is>
       </c>
       <c r="D288" s="4" t="inlineStr">
         <is>
-          <t>Review Help content in the modal</t>
+          <t>Activate the Help trigger from any primary page</t>
         </is>
       </c>
       <c r="E288" s="4" t="inlineStr">
         <is>
-          <t>Content is derived from the user manual and excludes installer-only or operator-only internals</t>
+          <t>Help opens in a modal or equivalent in-app panel</t>
         </is>
       </c>
       <c r="F288" s="4" t="n"/>
@@ -8914,7 +8914,7 @@
     <row r="289">
       <c r="A289" s="4" t="inlineStr">
         <is>
-          <t>TC-1025</t>
+          <t>TC-1023</t>
         </is>
       </c>
       <c r="B289" s="4" t="inlineStr">
@@ -8924,17 +8924,17 @@
       </c>
       <c r="C289" s="4" t="inlineStr">
         <is>
-          <t>Open full help document works</t>
+          <t>Help does not break current workflow context</t>
         </is>
       </c>
       <c r="D289" s="4" t="inlineStr">
         <is>
-          <t>Use the Help modal action to open the full document if present</t>
+          <t>Open Help while on Drives, Mounts, Jobs, or Audit, then close it</t>
         </is>
       </c>
       <c r="E289" s="4" t="inlineStr">
         <is>
-          <t>Full help content opens successfully and remains consistent with the in-app content</t>
+          <t>Closing Help returns to the same page and preserved workflow context</t>
         </is>
       </c>
       <c r="F289" s="4" t="n"/>
@@ -8945,7 +8945,7 @@
     <row r="290">
       <c r="A290" s="4" t="inlineStr">
         <is>
-          <t>TC-1026</t>
+          <t>TC-1024</t>
         </is>
       </c>
       <c r="B290" s="4" t="inlineStr">
@@ -8955,17 +8955,17 @@
       </c>
       <c r="C290" s="4" t="inlineStr">
         <is>
-          <t>Missing help asset fails gracefully</t>
+          <t>Help content is curated and user-facing</t>
         </is>
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>Test a build with the Help asset intentionally missing or inaccessible</t>
+          <t>Review Help content in the modal</t>
         </is>
       </c>
       <c r="E290" s="4" t="inlineStr">
         <is>
-          <t>UI shows a non-fatal fallback state with retry or operator guidance instead of breaking the app shell</t>
+          <t>Content is derived from the user manual and excludes installer-only or operator-only internals</t>
         </is>
       </c>
       <c r="F290" s="4" t="n"/>
@@ -8974,48 +8974,60 @@
       <c r="I290" s="4" t="n"/>
     </row>
     <row r="291">
-      <c r="A291" s="2" t="inlineStr">
-        <is>
-          <t>§12.11 First-Run Setup</t>
-        </is>
-      </c>
-      <c r="B291" s="2" t="inlineStr">
-        <is>
-          <t>12.11 First-Run Setup</t>
-        </is>
-      </c>
-      <c r="C291" s="3" t="n"/>
-      <c r="D291" s="3" t="n"/>
-      <c r="E291" s="3" t="n"/>
-      <c r="F291" s="3" t="n"/>
-      <c r="G291" s="3" t="n"/>
-      <c r="H291" s="3" t="n"/>
-      <c r="I291" s="3" t="n"/>
+      <c r="A291" s="4" t="inlineStr">
+        <is>
+          <t>TC-1025</t>
+        </is>
+      </c>
+      <c r="B291" s="4" t="inlineStr">
+        <is>
+          <t>12.10.2 Help System</t>
+        </is>
+      </c>
+      <c r="C291" s="4" t="inlineStr">
+        <is>
+          <t>Open full help document works</t>
+        </is>
+      </c>
+      <c r="D291" s="4" t="inlineStr">
+        <is>
+          <t>Use the Help modal action to open the full document if present</t>
+        </is>
+      </c>
+      <c r="E291" s="4" t="inlineStr">
+        <is>
+          <t>Full help content opens successfully and remains consistent with the in-app content</t>
+        </is>
+      </c>
+      <c r="F291" s="4" t="n"/>
+      <c r="G291" s="4" t="n"/>
+      <c r="H291" s="4" t="n"/>
+      <c r="I291" s="4" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="4" t="inlineStr">
         <is>
-          <t>TC-1101</t>
+          <t>TC-1026</t>
         </is>
       </c>
       <c r="B292" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.10.2 Help System</t>
         </is>
       </c>
       <c r="C292" s="4" t="inlineStr">
         <is>
-          <t>Status — not initialized</t>
+          <t>Missing help asset fails gracefully</t>
         </is>
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/status on fresh database</t>
+          <t>Test a build with the Help asset intentionally missing or inaccessible</t>
         </is>
       </c>
       <c r="E292" s="4" t="inlineStr">
         <is>
-          <t>200, {"initialized": false}</t>
+          <t>UI shows a non-fatal fallback state with retry or operator guidance instead of breaking the app shell</t>
         </is>
       </c>
       <c r="F292" s="4" t="n"/>
@@ -9024,40 +9036,28 @@
       <c r="I292" s="4" t="n"/>
     </row>
     <row r="293">
-      <c r="A293" s="4" t="inlineStr">
-        <is>
-          <t>TC-1102</t>
-        </is>
-      </c>
-      <c r="B293" s="4" t="inlineStr">
+      <c r="A293" s="2" t="inlineStr">
+        <is>
+          <t>§12.11 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="B293" s="2" t="inlineStr">
         <is>
           <t>12.11 First-Run Setup</t>
         </is>
       </c>
-      <c r="C293" s="4" t="inlineStr">
-        <is>
-          <t>Initialize</t>
-        </is>
-      </c>
-      <c r="D293" s="4" t="inlineStr">
-        <is>
-          <t>POST /setup/initialize with valid username and password</t>
-        </is>
-      </c>
-      <c r="E293" s="4" t="inlineStr">
-        <is>
-          <t>200, returns message, username, groups_created</t>
-        </is>
-      </c>
-      <c r="F293" s="4" t="n"/>
-      <c r="G293" s="4" t="n"/>
-      <c r="H293" s="4" t="n"/>
-      <c r="I293" s="4" t="n"/>
+      <c r="C293" s="3" t="n"/>
+      <c r="D293" s="3" t="n"/>
+      <c r="E293" s="3" t="n"/>
+      <c r="F293" s="3" t="n"/>
+      <c r="G293" s="3" t="n"/>
+      <c r="H293" s="3" t="n"/>
+      <c r="I293" s="3" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="4" t="inlineStr">
         <is>
-          <t>TC-1103</t>
+          <t>TC-1101</t>
         </is>
       </c>
       <c r="B294" s="4" t="inlineStr">
@@ -9067,17 +9067,17 @@
       </c>
       <c r="C294" s="4" t="inlineStr">
         <is>
-          <t>Status — initialized</t>
+          <t>Status — not initialized</t>
         </is>
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/status after initialization</t>
+          <t>GET /setup/status on fresh database</t>
         </is>
       </c>
       <c r="E294" s="4" t="inlineStr">
         <is>
-          <t>200, {"initialized": true}</t>
+          <t>200, {"initialized": false}</t>
         </is>
       </c>
       <c r="F294" s="4" t="n"/>
@@ -9088,7 +9088,7 @@
     <row r="295">
       <c r="A295" s="4" t="inlineStr">
         <is>
-          <t>TC-1104</t>
+          <t>TC-1102</t>
         </is>
       </c>
       <c r="B295" s="4" t="inlineStr">
@@ -9098,17 +9098,17 @@
       </c>
       <c r="C295" s="4" t="inlineStr">
         <is>
-          <t>Re-initialize informational</t>
+          <t>Initialize</t>
         </is>
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize again</t>
+          <t>POST /setup/initialize with valid username and password</t>
         </is>
       </c>
       <c r="E295" s="4" t="inlineStr">
         <is>
-          <t>200, status=already_initialized</t>
+          <t>200, returns message, username, groups_created</t>
         </is>
       </c>
       <c r="F295" s="4" t="n"/>
@@ -9119,7 +9119,7 @@
     <row r="296">
       <c r="A296" s="4" t="inlineStr">
         <is>
-          <t>TC-1105</t>
+          <t>TC-1103</t>
         </is>
       </c>
       <c r="B296" s="4" t="inlineStr">
@@ -9129,17 +9129,17 @@
       </c>
       <c r="C296" s="4" t="inlineStr">
         <is>
-          <t>Invalid username</t>
+          <t>Status — initialized</t>
         </is>
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with uppercase or special chars</t>
+          <t>GET /setup/status after initialization</t>
         </is>
       </c>
       <c r="E296" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>200, {"initialized": true}</t>
         </is>
       </c>
       <c r="F296" s="4" t="n"/>
@@ -9150,7 +9150,7 @@
     <row r="297">
       <c r="A297" s="4" t="inlineStr">
         <is>
-          <t>TC-1106</t>
+          <t>TC-1104</t>
         </is>
       </c>
       <c r="B297" s="4" t="inlineStr">
@@ -9160,17 +9160,17 @@
       </c>
       <c r="C297" s="4" t="inlineStr">
         <is>
-          <t>Empty password</t>
+          <t>Re-initialize informational</t>
         </is>
       </c>
       <c r="D297" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with {"password": ""}</t>
+          <t>POST /setup/initialize again</t>
         </is>
       </c>
       <c r="E297" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>200, status=already_initialized</t>
         </is>
       </c>
       <c r="F297" s="4" t="n"/>
@@ -9181,7 +9181,7 @@
     <row r="298">
       <c r="A298" s="4" t="inlineStr">
         <is>
-          <t>TC-1107</t>
+          <t>TC-1105</t>
         </is>
       </c>
       <c r="B298" s="4" t="inlineStr">
@@ -9191,17 +9191,17 @@
       </c>
       <c r="C298" s="4" t="inlineStr">
         <is>
-          <t>Unsafe password chars</t>
+          <t>Invalid username</t>
         </is>
       </c>
       <c r="D298" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with password containing newline or colon</t>
+          <t>POST /setup/initialize with uppercase or special chars</t>
         </is>
       </c>
       <c r="E298" s="4" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F298" s="4" t="n"/>
@@ -9212,7 +9212,7 @@
     <row r="299">
       <c r="A299" s="4" t="inlineStr">
         <is>
-          <t>TC-1108</t>
+          <t>TC-1106</t>
         </is>
       </c>
       <c r="B299" s="4" t="inlineStr">
@@ -9222,17 +9222,17 @@
       </c>
       <c r="C299" s="4" t="inlineStr">
         <is>
-          <t>Login as initialized admin</t>
+          <t>Empty password</t>
         </is>
       </c>
       <c r="D299" s="4" t="inlineStr">
         <is>
-          <t>POST /auth/token with the admin credentials from step 2</t>
+          <t>POST /setup/initialize with {"password": ""}</t>
         </is>
       </c>
       <c r="E299" s="4" t="inlineStr">
         <is>
-          <t>200, JWT contains admin role</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F299" s="4" t="n"/>
@@ -9243,7 +9243,7 @@
     <row r="300">
       <c r="A300" s="4" t="inlineStr">
         <is>
-          <t>TC-1109</t>
+          <t>TC-1107</t>
         </is>
       </c>
       <c r="B300" s="4" t="inlineStr">
@@ -9253,17 +9253,17 @@
       </c>
       <c r="C300" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM_INITIALIZED audit log</t>
+          <t>Unsafe password chars</t>
         </is>
       </c>
       <c r="D300" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
+          <t>POST /setup/initialize with password containing newline or colon</t>
         </is>
       </c>
       <c r="E300" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor</t>
+          <t>422, unsafe characters</t>
         </is>
       </c>
       <c r="F300" s="4" t="n"/>
@@ -9274,7 +9274,7 @@
     <row r="301">
       <c r="A301" s="4" t="inlineStr">
         <is>
-          <t>TC-1110</t>
+          <t>TC-1108</t>
         </is>
       </c>
       <c r="B301" s="4" t="inlineStr">
@@ -9284,17 +9284,17 @@
       </c>
       <c r="C301" s="4" t="inlineStr">
         <is>
-          <t>Initialize default proxy trust</t>
+          <t>Login as initialized admin</t>
         </is>
       </c>
       <c r="D301" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize without trust_proxy_headers</t>
+          <t>POST /auth/token with the admin credentials from step 2</t>
         </is>
       </c>
       <c r="E301" s="4" t="inlineStr">
         <is>
-          <t>200, runtime TRUST_PROXY_HEADERS=false persisted</t>
+          <t>200, JWT contains admin role</t>
         </is>
       </c>
       <c r="F301" s="4" t="n"/>
@@ -9305,7 +9305,7 @@
     <row r="302">
       <c r="A302" s="4" t="inlineStr">
         <is>
-          <t>TC-1111</t>
+          <t>TC-1109</t>
         </is>
       </c>
       <c r="B302" s="4" t="inlineStr">
@@ -9315,17 +9315,17 @@
       </c>
       <c r="C302" s="4" t="inlineStr">
         <is>
-          <t>Initialize explicit proxy trust</t>
+          <t>SYSTEM_INITIALIZED audit log</t>
         </is>
       </c>
       <c r="D302" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with "trust_proxy_headers": true</t>
+          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
         </is>
       </c>
       <c r="E302" s="4" t="inlineStr">
         <is>
-          <t>200, runtime TRUST_PROXY_HEADERS=true persisted</t>
+          <t>Audit entry with actor</t>
         </is>
       </c>
       <c r="F302" s="4" t="n"/>
@@ -9336,7 +9336,7 @@
     <row r="303">
       <c r="A303" s="4" t="inlineStr">
         <is>
-          <t>TC-1112</t>
+          <t>TC-1110</t>
         </is>
       </c>
       <c r="B303" s="4" t="inlineStr">
@@ -9346,17 +9346,17 @@
       </c>
       <c r="C303" s="4" t="inlineStr">
         <is>
-          <t>Re-initialize does not mutate runtime flags</t>
+          <t>Initialize default proxy trust</t>
         </is>
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>Call POST /setup/initialize after setup with a different trust_proxy_headers value</t>
+          <t>POST /setup/initialize without trust_proxy_headers</t>
         </is>
       </c>
       <c r="E303" s="4" t="inlineStr">
         <is>
-          <t>200, status=already_initialized, runtime TRUST_PROXY_HEADERS remains unchanged</t>
+          <t>200, runtime TRUST_PROXY_HEADERS=false persisted</t>
         </is>
       </c>
       <c r="F303" s="4" t="n"/>
@@ -9367,7 +9367,7 @@
     <row r="304">
       <c r="A304" s="4" t="inlineStr">
         <is>
-          <t>TC-1113</t>
+          <t>TC-1111</t>
         </is>
       </c>
       <c r="B304" s="4" t="inlineStr">
@@ -9377,17 +9377,17 @@
       </c>
       <c r="C304" s="4" t="inlineStr">
         <is>
-          <t>Runtime env target consistency</t>
+          <t>Initialize explicit proxy trust</t>
         </is>
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>Validate running service env file target and setup persistence target are the same (ECUBE_ENV_FILE)</t>
+          <t>POST /setup/initialize with "trust_proxy_headers": true</t>
         </is>
       </c>
       <c r="E304" s="4" t="inlineStr">
         <is>
-          <t>Runtime env file is updated, not a workspace-relative .env</t>
+          <t>200, runtime TRUST_PROXY_HEADERS=true persisted</t>
         </is>
       </c>
       <c r="F304" s="4" t="n"/>
@@ -9398,7 +9398,7 @@
     <row r="305">
       <c r="A305" s="4" t="inlineStr">
         <is>
-          <t>TC-1114</t>
+          <t>TC-1112</t>
         </is>
       </c>
       <c r="B305" s="4" t="inlineStr">
@@ -9408,17 +9408,17 @@
       </c>
       <c r="C305" s="4" t="inlineStr">
         <is>
-          <t>Uninstall drop fails closed on invalid target</t>
+          <t>Re-initialize does not mutate runtime flags</t>
         </is>
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>Run install.sh --uninstall --drop-database with missing/invalid/maintenance DATABASE_URL</t>
+          <t>Call POST /setup/initialize after setup with a different trust_proxy_headers value</t>
         </is>
       </c>
       <c r="E305" s="4" t="inlineStr">
         <is>
-          <t>Installer exits non-zero with explicit drop-target error; uninstall does not silently continue</t>
+          <t>200, status=already_initialized, runtime TRUST_PROXY_HEADERS remains unchanged</t>
         </is>
       </c>
       <c r="F305" s="4" t="n"/>
@@ -9427,48 +9427,60 @@
       <c r="I305" s="4" t="n"/>
     </row>
     <row r="306">
-      <c r="A306" s="2" t="inlineStr">
-        <is>
-          <t>§12.12 Chain-of-Custody Handoff</t>
-        </is>
-      </c>
-      <c r="B306" s="2" t="inlineStr">
-        <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
-        </is>
-      </c>
-      <c r="C306" s="3" t="n"/>
-      <c r="D306" s="3" t="n"/>
-      <c r="E306" s="3" t="n"/>
-      <c r="F306" s="3" t="n"/>
-      <c r="G306" s="3" t="n"/>
-      <c r="H306" s="3" t="n"/>
-      <c r="I306" s="3" t="n"/>
+      <c r="A306" s="4" t="inlineStr">
+        <is>
+          <t>TC-1113</t>
+        </is>
+      </c>
+      <c r="B306" s="4" t="inlineStr">
+        <is>
+          <t>12.11 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C306" s="4" t="inlineStr">
+        <is>
+          <t>Runtime env target consistency</t>
+        </is>
+      </c>
+      <c r="D306" s="4" t="inlineStr">
+        <is>
+          <t>Validate running service env file target and setup persistence target are the same (ECUBE_ENV_FILE)</t>
+        </is>
+      </c>
+      <c r="E306" s="4" t="inlineStr">
+        <is>
+          <t>Runtime env file is updated, not a workspace-relative .env</t>
+        </is>
+      </c>
+      <c r="F306" s="4" t="n"/>
+      <c r="G306" s="4" t="n"/>
+      <c r="H306" s="4" t="n"/>
+      <c r="I306" s="4" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="4" t="inlineStr">
         <is>
-          <t>TC-1201</t>
+          <t>TC-1114</t>
         </is>
       </c>
       <c r="B307" s="4" t="inlineStr">
         <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C307" s="4" t="inlineStr">
         <is>
-          <t>Retrieve stored CoC snapshot — archived job</t>
+          <t>Uninstall drop fails closed on invalid target</t>
         </is>
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for an archived job that already has a stored snapshot</t>
+          <t>Run install.sh --uninstall --drop-database with missing/invalid/maintenance DATABASE_URL</t>
         </is>
       </c>
       <c r="E307" s="4" t="inlineStr">
         <is>
-          <t>200, response contains the stored snapshot and snapshot metadata</t>
+          <t>Installer exits non-zero with explicit drop-target error; uninstall does not silently continue</t>
         </is>
       </c>
       <c r="F307" s="4" t="n"/>
@@ -9477,40 +9489,28 @@
       <c r="I307" s="4" t="n"/>
     </row>
     <row r="308">
-      <c r="A308" s="4" t="inlineStr">
-        <is>
-          <t>TC-1202</t>
-        </is>
-      </c>
-      <c r="B308" s="4" t="inlineStr">
+      <c r="A308" s="2" t="inlineStr">
+        <is>
+          <t>§12.12 Chain-of-Custody Handoff</t>
+        </is>
+      </c>
+      <c r="B308" s="2" t="inlineStr">
         <is>
           <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
-      <c r="C308" s="4" t="inlineStr">
-        <is>
-          <t>Retrieve stored CoC snapshot — active job</t>
-        </is>
-      </c>
-      <c r="D308" s="4" t="inlineStr">
-        <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job that already has a stored snapshot</t>
-        </is>
-      </c>
-      <c r="E308" s="4" t="inlineStr">
-        <is>
-          <t>200, response contains the stored snapshot and does not regenerate it</t>
-        </is>
-      </c>
-      <c r="F308" s="4" t="n"/>
-      <c r="G308" s="4" t="n"/>
-      <c r="H308" s="4" t="n"/>
-      <c r="I308" s="4" t="n"/>
+      <c r="C308" s="3" t="n"/>
+      <c r="D308" s="3" t="n"/>
+      <c r="E308" s="3" t="n"/>
+      <c r="F308" s="3" t="n"/>
+      <c r="G308" s="3" t="n"/>
+      <c r="H308" s="3" t="n"/>
+      <c r="I308" s="3" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="4" t="inlineStr">
         <is>
-          <t>TC-1203</t>
+          <t>TC-1201</t>
         </is>
       </c>
       <c r="B309" s="4" t="inlineStr">
@@ -9520,17 +9520,17 @@
       </c>
       <c r="C309" s="4" t="inlineStr">
         <is>
-          <t>CoC read — missing stored snapshot</t>
+          <t>Retrieve stored CoC snapshot — archived job</t>
         </is>
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job with no stored snapshot yet</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for an archived job that already has a stored snapshot</t>
         </is>
       </c>
       <c r="E309" s="4" t="inlineStr">
         <is>
-          <t>404, message explains that the report must be refreshed first</t>
+          <t>200, response contains the stored snapshot and snapshot metadata</t>
         </is>
       </c>
       <c r="F309" s="4" t="n"/>
@@ -9541,7 +9541,7 @@
     <row r="310">
       <c r="A310" s="4" t="inlineStr">
         <is>
-          <t>TC-1204</t>
+          <t>TC-1202</t>
         </is>
       </c>
       <c r="B310" s="4" t="inlineStr">
@@ -9551,17 +9551,17 @@
       </c>
       <c r="C310" s="4" t="inlineStr">
         <is>
-          <t>CoC read — processor denied</t>
+          <t>Retrieve stored CoC snapshot — active job</t>
         </is>
       </c>
       <c r="D310" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody with processor token</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job that already has a stored snapshot</t>
         </is>
       </c>
       <c r="E310" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>200, response contains the stored snapshot and does not regenerate it</t>
         </is>
       </c>
       <c r="F310" s="4" t="n"/>
@@ -9572,7 +9572,7 @@
     <row r="311">
       <c r="A311" s="4" t="inlineStr">
         <is>
-          <t>TC-1205</t>
+          <t>TC-1203</t>
         </is>
       </c>
       <c r="B311" s="4" t="inlineStr">
@@ -9582,17 +9582,17 @@
       </c>
       <c r="C311" s="4" t="inlineStr">
         <is>
-          <t>CoC read — unauthenticated denied</t>
+          <t>CoC read — missing stored snapshot</t>
         </is>
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody without token</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job with no stored snapshot yet</t>
         </is>
       </c>
       <c r="E311" s="4" t="inlineStr">
         <is>
-          <t>401, UNAUTHORIZED</t>
+          <t>404, message explains that the report must be refreshed first</t>
         </is>
       </c>
       <c r="F311" s="4" t="n"/>
@@ -9603,7 +9603,7 @@
     <row r="312">
       <c r="A312" s="4" t="inlineStr">
         <is>
-          <t>TC-1206</t>
+          <t>TC-1204</t>
         </is>
       </c>
       <c r="B312" s="4" t="inlineStr">
@@ -9613,17 +9613,17 @@
       </c>
       <c r="C312" s="4" t="inlineStr">
         <is>
-          <t>CoC snapshot fields</t>
+          <t>CoC read — processor denied</t>
         </is>
       </c>
       <c r="D312" s="4" t="inlineStr">
         <is>
-          <t>Inspect any stored-snapshot response</t>
+          <t>GET /jobs/{job_id}/chain-of-custody with processor token</t>
         </is>
       </c>
       <c r="E312" s="4" t="inlineStr">
         <is>
-          <t>snapshot_stored_at, snapshot_updated_at, snapshot_stored_by, reports[], and manifest/custody fields are present</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F312" s="4" t="n"/>
@@ -9634,7 +9634,7 @@
     <row r="313">
       <c r="A313" s="4" t="inlineStr">
         <is>
-          <t>TC-1207</t>
+          <t>TC-1205</t>
         </is>
       </c>
       <c r="B313" s="4" t="inlineStr">
@@ -9644,17 +9644,17 @@
       </c>
       <c r="C313" s="4" t="inlineStr">
         <is>
-          <t>CoC events include lifecycle</t>
+          <t>CoC read — unauthenticated denied</t>
         </is>
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>Inspect chain_of_custody_events in a stored report for a completed job</t>
+          <t>GET /jobs/{job_id}/chain-of-custody without token</t>
         </is>
       </c>
       <c r="E313" s="4" t="inlineStr">
         <is>
-          <t>Events include DRIVE_INITIALIZED, JOB_CREATED, JOB_STARTED, JOB_COMPLETED, DRIVE_EJECT_PREPARED, and COC_HANDOFF_CONFIRMED when applicable</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F313" s="4" t="n"/>
@@ -9665,7 +9665,7 @@
     <row r="314">
       <c r="A314" s="4" t="inlineStr">
         <is>
-          <t>TC-1208</t>
+          <t>TC-1206</t>
         </is>
       </c>
       <c r="B314" s="4" t="inlineStr">
@@ -9675,17 +9675,17 @@
       </c>
       <c r="C314" s="4" t="inlineStr">
         <is>
-          <t>CoC manifest summary</t>
+          <t>CoC snapshot fields</t>
         </is>
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>Inspect manifest_summary in the stored report</t>
+          <t>Inspect any stored-snapshot response</t>
         </is>
       </c>
       <c r="E314" s="4" t="inlineStr">
         <is>
-          <t>Array of objects with job_id, evidence_number, processor_notes, total_files, total_bytes, and manifest_count</t>
+          <t>snapshot_stored_at, snapshot_updated_at, snapshot_stored_by, reports[], and manifest/custody fields are present</t>
         </is>
       </c>
       <c r="F314" s="4" t="n"/>
@@ -9696,7 +9696,7 @@
     <row r="315">
       <c r="A315" s="4" t="inlineStr">
         <is>
-          <t>TC-1209</t>
+          <t>TC-1207</t>
         </is>
       </c>
       <c r="B315" s="4" t="inlineStr">
@@ -9706,17 +9706,17 @@
       </c>
       <c r="C315" s="4" t="inlineStr">
         <is>
-          <t>CoC — delivery_time absence (no handoff)</t>
+          <t>CoC events include lifecycle</t>
         </is>
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>Complete a job and store a snapshot before handoff</t>
+          <t>Inspect chain_of_custody_events in a stored report for a completed job</t>
         </is>
       </c>
       <c r="E315" s="4" t="inlineStr">
         <is>
-          <t>chain_of_custody_events do not contain COC_HANDOFF_CONFIRMED; custody_complete is false</t>
+          <t>Events include DRIVE_INITIALIZED, JOB_CREATED, JOB_STARTED, JOB_COMPLETED, DRIVE_EJECT_PREPARED, and COC_HANDOFF_CONFIRMED when applicable</t>
         </is>
       </c>
       <c r="F315" s="4" t="n"/>
@@ -9727,7 +9727,7 @@
     <row r="316">
       <c r="A316" s="4" t="inlineStr">
         <is>
-          <t>TC-1210</t>
+          <t>TC-1208</t>
         </is>
       </c>
       <c r="B316" s="4" t="inlineStr">
@@ -9737,17 +9737,17 @@
       </c>
       <c r="C316" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — valid</t>
+          <t>CoC manifest summary</t>
         </is>
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh with admin or manager token for a non-archived job with assignments</t>
+          <t>Inspect manifest_summary in the stored report</t>
         </is>
       </c>
       <c r="E316" s="4" t="inlineStr">
         <is>
-          <t>200, response contains the refreshed stored snapshot and updated snapshot metadata</t>
+          <t>Array of objects with job_id, evidence_number, processor_notes, total_files, total_bytes, and manifest_count</t>
         </is>
       </c>
       <c r="F316" s="4" t="n"/>
@@ -9758,7 +9758,7 @@
     <row r="317">
       <c r="A317" s="4" t="inlineStr">
         <is>
-          <t>TC-1211</t>
+          <t>TC-1209</t>
         </is>
       </c>
       <c r="B317" s="4" t="inlineStr">
@@ -9768,17 +9768,17 @@
       </c>
       <c r="C317" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — auditor denied</t>
+          <t>CoC — delivery_time absence (no handoff)</t>
         </is>
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh with auditor token</t>
+          <t>Complete a job and store a snapshot before handoff</t>
         </is>
       </c>
       <c r="E317" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>chain_of_custody_events do not contain COC_HANDOFF_CONFIRMED; custody_complete is false</t>
         </is>
       </c>
       <c r="F317" s="4" t="n"/>
@@ -9789,7 +9789,7 @@
     <row r="318">
       <c r="A318" s="4" t="inlineStr">
         <is>
-          <t>TC-1212</t>
+          <t>TC-1210</t>
         </is>
       </c>
       <c r="B318" s="4" t="inlineStr">
@@ -9799,17 +9799,17 @@
       </c>
       <c r="C318" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — archived job denied</t>
+          <t>CoC refresh — valid</t>
         </is>
       </c>
       <c r="D318" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh for an archived job</t>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh with admin or manager token for a non-archived job with assignments</t>
         </is>
       </c>
       <c r="E318" s="4" t="inlineStr">
         <is>
-          <t>409, archived jobs can only return the last stored snapshot</t>
+          <t>200, response contains the refreshed stored snapshot and updated snapshot metadata</t>
         </is>
       </c>
       <c r="F318" s="4" t="n"/>
@@ -9818,48 +9818,60 @@
       <c r="I318" s="4" t="n"/>
     </row>
     <row r="319">
-      <c r="A319" s="2" t="inlineStr">
-        <is>
-          <t>§12.14 Startup Reconciliation</t>
-        </is>
-      </c>
-      <c r="B319" s="2" t="inlineStr">
-        <is>
-          <t>12.14 Startup Reconciliation</t>
-        </is>
-      </c>
-      <c r="C319" s="3" t="n"/>
-      <c r="D319" s="3" t="n"/>
-      <c r="E319" s="3" t="n"/>
-      <c r="F319" s="3" t="n"/>
-      <c r="G319" s="3" t="n"/>
-      <c r="H319" s="3" t="n"/>
-      <c r="I319" s="3" t="n"/>
+      <c r="A319" s="4" t="inlineStr">
+        <is>
+          <t>TC-1211</t>
+        </is>
+      </c>
+      <c r="B319" s="4" t="inlineStr">
+        <is>
+          <t>12.12 Chain-of-Custody Handoff</t>
+        </is>
+      </c>
+      <c r="C319" s="4" t="inlineStr">
+        <is>
+          <t>CoC refresh — auditor denied</t>
+        </is>
+      </c>
+      <c r="D319" s="4" t="inlineStr">
+        <is>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh with auditor token</t>
+        </is>
+      </c>
+      <c r="E319" s="4" t="inlineStr">
+        <is>
+          <t>403, FORBIDDEN</t>
+        </is>
+      </c>
+      <c r="F319" s="4" t="n"/>
+      <c r="G319" s="4" t="n"/>
+      <c r="H319" s="4" t="n"/>
+      <c r="I319" s="4" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="4" t="inlineStr">
         <is>
-          <t>TC-1401</t>
+          <t>TC-1212</t>
         </is>
       </c>
       <c r="B320" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
       <c r="C320" s="4" t="inlineStr">
         <is>
-          <t>Running job failed after restart</t>
+          <t>CoC refresh — archived job denied</t>
         </is>
       </c>
       <c r="D320" s="4" t="inlineStr">
         <is>
-          <t>Create a job, start it, restart the service while RUNNING</t>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh for an archived job</t>
         </is>
       </c>
       <c r="E320" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
+          <t>409, archived jobs can only return the last stored snapshot</t>
         </is>
       </c>
       <c r="F320" s="4" t="n"/>
@@ -9868,40 +9880,28 @@
       <c r="I320" s="4" t="n"/>
     </row>
     <row r="321">
-      <c r="A321" s="4" t="inlineStr">
-        <is>
-          <t>TC-1402</t>
-        </is>
-      </c>
-      <c r="B321" s="4" t="inlineStr">
+      <c r="A321" s="2" t="inlineStr">
+        <is>
+          <t>§12.14 Startup Reconciliation</t>
+        </is>
+      </c>
+      <c r="B321" s="2" t="inlineStr">
         <is>
           <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
-      <c r="C321" s="4" t="inlineStr">
-        <is>
-          <t>Verifying job failed after restart</t>
-        </is>
-      </c>
-      <c r="D321" s="4" t="inlineStr">
-        <is>
-          <t>Start a job, let it reach VERIFYING, restart the service</t>
-        </is>
-      </c>
-      <c r="E321" s="4" t="inlineStr">
-        <is>
-          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
-        </is>
-      </c>
-      <c r="F321" s="4" t="n"/>
-      <c r="G321" s="4" t="n"/>
-      <c r="H321" s="4" t="n"/>
-      <c r="I321" s="4" t="n"/>
+      <c r="C321" s="3" t="n"/>
+      <c r="D321" s="3" t="n"/>
+      <c r="E321" s="3" t="n"/>
+      <c r="F321" s="3" t="n"/>
+      <c r="G321" s="3" t="n"/>
+      <c r="H321" s="3" t="n"/>
+      <c r="I321" s="3" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="4" t="inlineStr">
         <is>
-          <t>TC-1403</t>
+          <t>TC-1401</t>
         </is>
       </c>
       <c r="B322" s="4" t="inlineStr">
@@ -9911,17 +9911,17 @@
       </c>
       <c r="C322" s="4" t="inlineStr">
         <is>
-          <t>Pending job not affected</t>
+          <t>Running job failed after restart</t>
         </is>
       </c>
       <c r="D322" s="4" t="inlineStr">
         <is>
-          <t>Create a job (PENDING), restart the service</t>
+          <t>Create a job, start it, restart the service while RUNNING</t>
         </is>
       </c>
       <c r="E322" s="4" t="inlineStr">
         <is>
-          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
+          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
         </is>
       </c>
       <c r="F322" s="4" t="n"/>
@@ -9932,7 +9932,7 @@
     <row r="323">
       <c r="A323" s="4" t="inlineStr">
         <is>
-          <t>TC-1404</t>
+          <t>TC-1402</t>
         </is>
       </c>
       <c r="B323" s="4" t="inlineStr">
@@ -9942,17 +9942,17 @@
       </c>
       <c r="C323" s="4" t="inlineStr">
         <is>
-          <t>Completed job not affected</t>
+          <t>Verifying job failed after restart</t>
         </is>
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>Complete a job, restart the service</t>
+          <t>Start a job, let it reach VERIFYING, restart the service</t>
         </is>
       </c>
       <c r="E323" s="4" t="inlineStr">
         <is>
-          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
+          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
         </is>
       </c>
       <c r="F323" s="4" t="n"/>
@@ -9963,7 +9963,7 @@
     <row r="324">
       <c r="A324" s="4" t="inlineStr">
         <is>
-          <t>TC-1405</t>
+          <t>TC-1403</t>
         </is>
       </c>
       <c r="B324" s="4" t="inlineStr">
@@ -9973,17 +9973,17 @@
       </c>
       <c r="C324" s="4" t="inlineStr">
         <is>
-          <t>Stale mount corrected</t>
+          <t>Pending job not affected</t>
         </is>
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
+          <t>Create a job (PENDING), restart the service</t>
         </is>
       </c>
       <c r="E324" s="4" t="inlineStr">
         <is>
-          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
+          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
         </is>
       </c>
       <c r="F324" s="4" t="n"/>
@@ -9994,7 +9994,7 @@
     <row r="325">
       <c r="A325" s="4" t="inlineStr">
         <is>
-          <t>TC-1406</t>
+          <t>TC-1404</t>
         </is>
       </c>
       <c r="B325" s="4" t="inlineStr">
@@ -10004,17 +10004,17 @@
       </c>
       <c r="C325" s="4" t="inlineStr">
         <is>
-          <t>Active mount preserved</t>
+          <t>Completed job not affected</t>
         </is>
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share (leave it mounted), restart the service</t>
+          <t>Complete a job, restart the service</t>
         </is>
       </c>
       <c r="E325" s="4" t="inlineStr">
         <is>
-          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
+          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F325" s="4" t="n"/>
@@ -10025,7 +10025,7 @@
     <row r="326">
       <c r="A326" s="4" t="inlineStr">
         <is>
-          <t>TC-1407</t>
+          <t>TC-1405</t>
         </is>
       </c>
       <c r="B326" s="4" t="inlineStr">
@@ -10035,17 +10035,17 @@
       </c>
       <c r="C326" s="4" t="inlineStr">
         <is>
-          <t>USB drives re-discovered</t>
+          <t>Stale mount corrected</t>
         </is>
       </c>
       <c r="D326" s="4" t="inlineStr">
         <is>
-          <t>Insert USB drives, restart the service</t>
+          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
         </is>
       </c>
       <c r="E326" s="4" t="inlineStr">
         <is>
-          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
+          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
         </is>
       </c>
       <c r="F326" s="4" t="n"/>
@@ -10056,7 +10056,7 @@
     <row r="327">
       <c r="A327" s="4" t="inlineStr">
         <is>
-          <t>TC-1408</t>
+          <t>TC-1406</t>
         </is>
       </c>
       <c r="B327" s="4" t="inlineStr">
@@ -10066,17 +10066,17 @@
       </c>
       <c r="C327" s="4" t="inlineStr">
         <is>
-          <t>Idempotency</t>
+          <t>Active mount preserved</t>
         </is>
       </c>
       <c r="D327" s="4" t="inlineStr">
         <is>
-          <t>Restart the service twice without any state changes between restarts</t>
+          <t>Add and mount a network share (leave it mounted), restart the service</t>
         </is>
       </c>
       <c r="E327" s="4" t="inlineStr">
         <is>
-          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
+          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F327" s="4" t="n"/>
@@ -10087,7 +10087,7 @@
     <row r="328">
       <c r="A328" s="4" t="inlineStr">
         <is>
-          <t>TC-1409</t>
+          <t>TC-1407</t>
         </is>
       </c>
       <c r="B328" s="4" t="inlineStr">
@@ -10097,17 +10097,17 @@
       </c>
       <c r="C328" s="4" t="inlineStr">
         <is>
-          <t>Partial failure isolation</t>
+          <t>USB drives re-discovered</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr">
         <is>
-          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
+          <t>Insert USB drives, restart the service</t>
         </is>
       </c>
       <c r="E328" s="4" t="inlineStr">
         <is>
-          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
+          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
         </is>
       </c>
       <c r="F328" s="4" t="n"/>
@@ -10118,7 +10118,7 @@
     <row r="329">
       <c r="A329" s="4" t="inlineStr">
         <is>
-          <t>TC-1410</t>
+          <t>TC-1408</t>
         </is>
       </c>
       <c r="B329" s="4" t="inlineStr">
@@ -10128,17 +10128,17 @@
       </c>
       <c r="C329" s="4" t="inlineStr">
         <is>
-          <t>Cross-process lock — only one worker reconciles</t>
+          <t>Idempotency</t>
         </is>
       </c>
       <c r="D329" s="4" t="inlineStr">
         <is>
-          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
+          <t>Restart the service twice without any state changes between restarts</t>
         </is>
       </c>
       <c r="E329" s="4" t="inlineStr">
         <is>
-          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
+          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
         </is>
       </c>
       <c r="F329" s="4" t="n"/>
@@ -10149,7 +10149,7 @@
     <row r="330">
       <c r="A330" s="4" t="inlineStr">
         <is>
-          <t>TC-1411</t>
+          <t>TC-1409</t>
         </is>
       </c>
       <c r="B330" s="4" t="inlineStr">
@@ -10159,17 +10159,17 @@
       </c>
       <c r="C330" s="4" t="inlineStr">
         <is>
-          <t>Stale lock reclaim</t>
+          <t>Partial failure isolation</t>
         </is>
       </c>
       <c r="D330" s="4" t="inlineStr">
         <is>
-          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
+          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
         </is>
       </c>
       <c r="E330" s="4" t="inlineStr">
         <is>
-          <t>Service reclaims the stale lock, reconciliation runs normally</t>
+          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
         </is>
       </c>
       <c r="F330" s="4" t="n"/>
@@ -10180,7 +10180,7 @@
     <row r="331">
       <c r="A331" s="4" t="inlineStr">
         <is>
-          <t>TC-1412</t>
+          <t>TC-1410</t>
         </is>
       </c>
       <c r="B331" s="4" t="inlineStr">
@@ -10190,17 +10190,17 @@
       </c>
       <c r="C331" s="4" t="inlineStr">
         <is>
-          <t>Lock released after failure</t>
+          <t>Cross-process lock — only one worker reconciles</t>
         </is>
       </c>
       <c r="D331" s="4" t="inlineStr">
         <is>
-          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
+          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
         </is>
       </c>
       <c r="E331" s="4" t="inlineStr">
         <is>
-          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
+          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
         </is>
       </c>
       <c r="F331" s="4" t="n"/>
@@ -10211,7 +10211,7 @@
     <row r="332">
       <c r="A332" s="4" t="inlineStr">
         <is>
-          <t>TC-1413</t>
+          <t>TC-1411</t>
         </is>
       </c>
       <c r="B332" s="4" t="inlineStr">
@@ -10221,17 +10221,17 @@
       </c>
       <c r="C332" s="4" t="inlineStr">
         <is>
-          <t>Jobs pass emits immediate startup result log</t>
+          <t>Stale lock reclaim</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr">
         <is>
-          <t>Create at least one RUNNING job, restart service, then inspect application logs around startup reconciliation</t>
+          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
         </is>
       </c>
       <c r="E332" s="4" t="inlineStr">
         <is>
-          <t>Logs include Startup reconciliation: checking jobs followed by an immediate Startup reconciliation: jobs result line with safe counts (jobs_checked, jobs_corrected) or safe failure classification</t>
+          <t>Service reclaims the stale lock, reconciliation runs normally</t>
         </is>
       </c>
       <c r="F332" s="4" t="n"/>
@@ -10242,7 +10242,7 @@
     <row r="333">
       <c r="A333" s="4" t="inlineStr">
         <is>
-          <t>TC-1414</t>
+          <t>TC-1412</t>
         </is>
       </c>
       <c r="B333" s="4" t="inlineStr">
@@ -10252,17 +10252,17 @@
       </c>
       <c r="C333" s="4" t="inlineStr">
         <is>
-          <t>Reconciled job persists restart-interruption failure reason</t>
+          <t>Lock released after failure</t>
         </is>
       </c>
       <c r="D333" s="4" t="inlineStr">
         <is>
-          <t>Create a RUNNING or VERIFYING job, restart service, then open Job Detail for that job</t>
+          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
         </is>
       </c>
       <c r="E333" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED and Job Detail shows a stable restart interruption reason (not the generic This job failed... fallback)</t>
+          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
         </is>
       </c>
       <c r="F333" s="4" t="n"/>
@@ -10273,7 +10273,7 @@
     <row r="334">
       <c r="A334" s="4" t="inlineStr">
         <is>
-          <t>TC-1415</t>
+          <t>TC-1413</t>
         </is>
       </c>
       <c r="B334" s="4" t="inlineStr">
@@ -10283,17 +10283,17 @@
       </c>
       <c r="C334" s="4" t="inlineStr">
         <is>
-          <t>Reconciled failed job shows correlated failure entry from audit fallback</t>
+          <t>Jobs pass emits immediate startup result log</t>
         </is>
       </c>
       <c r="D334" s="4" t="inlineStr">
         <is>
-          <t>Restart with a RUNNING job, then inspect Job Detail when no matching file-log failure line is present</t>
+          <t>Create at least one RUNNING job, restart service, then inspect application logs around startup reconciliation</t>
         </is>
       </c>
       <c r="E334" s="4" t="inlineStr">
         <is>
-          <t>Job Detail still shows a related failure entry sourced from reconciliation evidence (JOB_RECONCILED) and the entry remains sanitized</t>
+          <t>Logs include Startup reconciliation: checking jobs followed by an immediate Startup reconciliation: jobs result line with safe counts (jobs_checked, jobs_corrected) or safe failure classification</t>
         </is>
       </c>
       <c r="F334" s="4" t="n"/>
@@ -10304,7 +10304,7 @@
     <row r="335">
       <c r="A335" s="4" t="inlineStr">
         <is>
-          <t>TC-1416</t>
+          <t>TC-1414</t>
         </is>
       </c>
       <c r="B335" s="4" t="inlineStr">
@@ -10314,17 +10314,17 @@
       </c>
       <c r="C335" s="4" t="inlineStr">
         <is>
-          <t>Failed job API uses reconciliation audit fallback when file-log correlation is unavailable</t>
+          <t>Reconciled job persists restart-interruption failure reason</t>
         </is>
       </c>
       <c r="D335" s="4" t="inlineStr">
         <is>
-          <t>In a test environment, disable file-log correlation (log_file unset), then request GET /jobs/{job_id} for a restart-reconciled failed job</t>
+          <t>Create a RUNNING or VERIFYING job, restart service, then open Job Detail for that job</t>
         </is>
       </c>
       <c r="E335" s="4" t="inlineStr">
         <is>
-          <t>Response remains 200 and includes the stable restart failure reason plus a sanitized failure_log_entry derived from audit evidence (JOB_RECONCILED)</t>
+          <t>Job status is FAILED and Job Detail shows a stable restart interruption reason (not the generic This job failed... fallback)</t>
         </is>
       </c>
       <c r="F335" s="4" t="n"/>
@@ -10335,7 +10335,7 @@
     <row r="336">
       <c r="A336" s="4" t="inlineStr">
         <is>
-          <t>TC-1417</t>
+          <t>TC-1415</t>
         </is>
       </c>
       <c r="B336" s="4" t="inlineStr">
@@ -10345,17 +10345,17 @@
       </c>
       <c r="C336" s="4" t="inlineStr">
         <is>
-          <t>Jobs pass failure path emits safe startup result classification</t>
+          <t>Reconciled failed job shows correlated failure entry from audit fallback</t>
         </is>
       </c>
       <c r="D336" s="4" t="inlineStr">
         <is>
-          <t>In a controlled test environment, force a jobs-pass reconciliation exception, then restart service and inspect startup logs</t>
+          <t>Restart with a RUNNING job, then inspect Job Detail when no matching file-log failure line is present</t>
         </is>
       </c>
       <c r="E336" s="4" t="inlineStr">
         <is>
-          <t>Logs still include Startup reconciliation: jobs result with status=failed and reason=job_reconciliation_failed, without raw provider errors or host paths</t>
+          <t>Job Detail still shows a related failure entry sourced from reconciliation evidence (JOB_RECONCILED) and the entry remains sanitized</t>
         </is>
       </c>
       <c r="F336" s="4" t="n"/>
@@ -10364,48 +10364,60 @@
       <c r="I336" s="4" t="n"/>
     </row>
     <row r="337">
-      <c r="A337" s="2" t="inlineStr">
-        <is>
-          <t>§12.15 System Health</t>
-        </is>
-      </c>
-      <c r="B337" s="2" t="inlineStr">
-        <is>
-          <t>12.15 System Health</t>
-        </is>
-      </c>
-      <c r="C337" s="3" t="n"/>
-      <c r="D337" s="3" t="n"/>
-      <c r="E337" s="3" t="n"/>
-      <c r="F337" s="3" t="n"/>
-      <c r="G337" s="3" t="n"/>
-      <c r="H337" s="3" t="n"/>
-      <c r="I337" s="3" t="n"/>
+      <c r="A337" s="4" t="inlineStr">
+        <is>
+          <t>TC-1416</t>
+        </is>
+      </c>
+      <c r="B337" s="4" t="inlineStr">
+        <is>
+          <t>12.14 Startup Reconciliation</t>
+        </is>
+      </c>
+      <c r="C337" s="4" t="inlineStr">
+        <is>
+          <t>Failed job API uses reconciliation audit fallback when file-log correlation is unavailable</t>
+        </is>
+      </c>
+      <c r="D337" s="4" t="inlineStr">
+        <is>
+          <t>In a test environment, disable file-log correlation (log_file unset), then request GET /jobs/{job_id} for a restart-reconciled failed job</t>
+        </is>
+      </c>
+      <c r="E337" s="4" t="inlineStr">
+        <is>
+          <t>Response remains 200 and includes the stable restart failure reason plus a sanitized failure_log_entry derived from audit evidence (JOB_RECONCILED)</t>
+        </is>
+      </c>
+      <c r="F337" s="4" t="n"/>
+      <c r="G337" s="4" t="n"/>
+      <c r="H337" s="4" t="n"/>
+      <c r="I337" s="4" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="4" t="inlineStr">
         <is>
-          <t>TC-1501</t>
+          <t>TC-1417</t>
         </is>
       </c>
       <c r="B338" s="4" t="inlineStr">
         <is>
-          <t>12.15 System Health</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C338" s="4" t="inlineStr">
         <is>
-          <t>Healthy response</t>
+          <t>Jobs pass failure path emits safe startup result classification</t>
         </is>
       </c>
       <c r="D338" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with valid token</t>
+          <t>In a controlled test environment, force a jobs-pass reconciliation exception, then restart service and inspect startup logs</t>
         </is>
       </c>
       <c r="E338" s="4" t="inlineStr">
         <is>
-          <t>200, status: "ok", database: "connected"</t>
+          <t>Logs still include Startup reconciliation: jobs result with status=failed and reason=job_reconciliation_failed, without raw provider errors or host paths</t>
         </is>
       </c>
       <c r="F338" s="4" t="n"/>
@@ -10414,40 +10426,28 @@
       <c r="I338" s="4" t="n"/>
     </row>
     <row r="339">
-      <c r="A339" s="4" t="inlineStr">
-        <is>
-          <t>TC-1502</t>
-        </is>
-      </c>
-      <c r="B339" s="4" t="inlineStr">
+      <c r="A339" s="2" t="inlineStr">
+        <is>
+          <t>§12.15 System Health</t>
+        </is>
+      </c>
+      <c r="B339" s="2" t="inlineStr">
         <is>
           <t>12.15 System Health</t>
         </is>
       </c>
-      <c r="C339" s="4" t="inlineStr">
-        <is>
-          <t>CPU metric present</t>
-        </is>
-      </c>
-      <c r="D339" s="4" t="inlineStr">
-        <is>
-          <t>Inspect response body</t>
-        </is>
-      </c>
-      <c r="E339" s="4" t="inlineStr">
-        <is>
-          <t>cpu_percent is a number between 0 and 100</t>
-        </is>
-      </c>
-      <c r="F339" s="4" t="n"/>
-      <c r="G339" s="4" t="n"/>
-      <c r="H339" s="4" t="n"/>
-      <c r="I339" s="4" t="n"/>
+      <c r="C339" s="3" t="n"/>
+      <c r="D339" s="3" t="n"/>
+      <c r="E339" s="3" t="n"/>
+      <c r="F339" s="3" t="n"/>
+      <c r="G339" s="3" t="n"/>
+      <c r="H339" s="3" t="n"/>
+      <c r="I339" s="3" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="4" t="inlineStr">
         <is>
-          <t>TC-1503</t>
+          <t>TC-1501</t>
         </is>
       </c>
       <c r="B340" s="4" t="inlineStr">
@@ -10457,17 +10457,17 @@
       </c>
       <c r="C340" s="4" t="inlineStr">
         <is>
-          <t>Memory metrics present</t>
+          <t>Healthy response</t>
         </is>
       </c>
       <c r="D340" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>GET /introspection/system-health with valid token</t>
         </is>
       </c>
       <c r="E340" s="4" t="inlineStr">
         <is>
-          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
+          <t>200, status: "ok", database: "connected"</t>
         </is>
       </c>
       <c r="F340" s="4" t="n"/>
@@ -10478,7 +10478,7 @@
     <row r="341">
       <c r="A341" s="4" t="inlineStr">
         <is>
-          <t>TC-1504</t>
+          <t>TC-1502</t>
         </is>
       </c>
       <c r="B341" s="4" t="inlineStr">
@@ -10488,7 +10488,7 @@
       </c>
       <c r="C341" s="4" t="inlineStr">
         <is>
-          <t>Disk I/O metrics present</t>
+          <t>CPU metric present</t>
         </is>
       </c>
       <c r="D341" s="4" t="inlineStr">
@@ -10498,7 +10498,7 @@
       </c>
       <c r="E341" s="4" t="inlineStr">
         <is>
-          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
+          <t>cpu_percent is a number between 0 and 100</t>
         </is>
       </c>
       <c r="F341" s="4" t="n"/>
@@ -10509,7 +10509,7 @@
     <row r="342">
       <c r="A342" s="4" t="inlineStr">
         <is>
-          <t>TC-1505</t>
+          <t>TC-1503</t>
         </is>
       </c>
       <c r="B342" s="4" t="inlineStr">
@@ -10519,17 +10519,17 @@
       </c>
       <c r="C342" s="4" t="inlineStr">
         <is>
-          <t>Active jobs count</t>
+          <t>Memory metrics present</t>
         </is>
       </c>
       <c r="D342" s="4" t="inlineStr">
         <is>
-          <t>Start an export job, call endpoint</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E342" s="4" t="inlineStr">
         <is>
-          <t>active_jobs ≥ 1</t>
+          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
         </is>
       </c>
       <c r="F342" s="4" t="n"/>
@@ -10540,7 +10540,7 @@
     <row r="343">
       <c r="A343" s="4" t="inlineStr">
         <is>
-          <t>TC-1506</t>
+          <t>TC-1504</t>
         </is>
       </c>
       <c r="B343" s="4" t="inlineStr">
@@ -10550,17 +10550,17 @@
       </c>
       <c r="C343" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size</t>
+          <t>Disk I/O metrics present</t>
         </is>
       </c>
       <c r="D343" s="4" t="inlineStr">
         <is>
-          <t>Create a PENDING job (created but not started), call endpoint</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E343" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size ≥ 1</t>
+          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
         </is>
       </c>
       <c r="F343" s="4" t="n"/>
@@ -10571,7 +10571,7 @@
     <row r="344">
       <c r="A344" s="4" t="inlineStr">
         <is>
-          <t>TC-1507</t>
+          <t>TC-1505</t>
         </is>
       </c>
       <c r="B344" s="4" t="inlineStr">
@@ -10581,17 +10581,17 @@
       </c>
       <c r="C344" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size decrements</t>
+          <t>Active jobs count</t>
         </is>
       </c>
       <c r="D344" s="4" t="inlineStr">
         <is>
-          <t>Start the pending job, call endpoint again</t>
+          <t>Start an export job, call endpoint</t>
         </is>
       </c>
       <c r="E344" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
+          <t>active_jobs ≥ 1</t>
         </is>
       </c>
       <c r="F344" s="4" t="n"/>
@@ -10602,7 +10602,7 @@
     <row r="345">
       <c r="A345" s="4" t="inlineStr">
         <is>
-          <t>TC-1508</t>
+          <t>TC-1506</t>
         </is>
       </c>
       <c r="B345" s="4" t="inlineStr">
@@ -10612,17 +10612,17 @@
       </c>
       <c r="C345" s="4" t="inlineStr">
         <is>
-          <t>ECUBE process metrics present</t>
+          <t>Worker queue size</t>
         </is>
       </c>
       <c r="D345" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Create a PENDING job (created but not started), call endpoint</t>
         </is>
       </c>
       <c r="E345" s="4" t="inlineStr">
         <is>
-          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
+          <t>worker_queue_size ≥ 1</t>
         </is>
       </c>
       <c r="F345" s="4" t="n"/>
@@ -10633,7 +10633,7 @@
     <row r="346">
       <c r="A346" s="4" t="inlineStr">
         <is>
-          <t>TC-1509</t>
+          <t>TC-1507</t>
         </is>
       </c>
       <c r="B346" s="4" t="inlineStr">
@@ -10643,17 +10643,17 @@
       </c>
       <c r="C346" s="4" t="inlineStr">
         <is>
-          <t>Active copy-thread correlation</t>
+          <t>Worker queue size decrements</t>
         </is>
       </c>
       <c r="D346" s="4" t="inlineStr">
         <is>
-          <t>Run an export job with active copy workers, call endpoint during the run</t>
+          <t>Start the pending job, call endpoint again</t>
         </is>
       </c>
       <c r="E346" s="4" t="inlineStr">
         <is>
-          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
+          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
         </is>
       </c>
       <c r="F346" s="4" t="n"/>
@@ -10664,7 +10664,7 @@
     <row r="347">
       <c r="A347" s="4" t="inlineStr">
         <is>
-          <t>TC-1510</t>
+          <t>TC-1508</t>
         </is>
       </c>
       <c r="B347" s="4" t="inlineStr">
@@ -10674,17 +10674,17 @@
       </c>
       <c r="C347" s="4" t="inlineStr">
         <is>
-          <t>ECUBE process metrics degrade safely</t>
+          <t>ECUBE process metrics present</t>
         </is>
       </c>
       <c r="D347" s="4" t="inlineStr">
         <is>
-          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E347" s="4" t="inlineStr">
         <is>
-          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
+          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
         </is>
       </c>
       <c r="F347" s="4" t="n"/>
@@ -10695,7 +10695,7 @@
     <row r="348">
       <c r="A348" s="4" t="inlineStr">
         <is>
-          <t>TC-1511</t>
+          <t>TC-1509</t>
         </is>
       </c>
       <c r="B348" s="4" t="inlineStr">
@@ -10705,17 +10705,17 @@
       </c>
       <c r="C348" s="4" t="inlineStr">
         <is>
-          <t>Degraded when DB down</t>
+          <t>Active copy-thread correlation</t>
         </is>
       </c>
       <c r="D348" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, call endpoint with valid token</t>
+          <t>Run an export job with active copy workers, call endpoint during the run</t>
         </is>
       </c>
       <c r="E348" s="4" t="inlineStr">
         <is>
-          <t>200, status: "degraded", database: "error", database_error is non-null</t>
+          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
         </is>
       </c>
       <c r="F348" s="4" t="n"/>
@@ -10726,7 +10726,7 @@
     <row r="349">
       <c r="A349" s="4" t="inlineStr">
         <is>
-          <t>TC-1512</t>
+          <t>TC-1510</t>
         </is>
       </c>
       <c r="B349" s="4" t="inlineStr">
@@ -10736,17 +10736,17 @@
       </c>
       <c r="C349" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated rejected</t>
+          <t>ECUBE process metrics degrade safely</t>
         </is>
       </c>
       <c r="D349" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health without token</t>
+          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
         </is>
       </c>
       <c r="E349" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
         </is>
       </c>
       <c r="F349" s="4" t="n"/>
@@ -10757,7 +10757,7 @@
     <row r="350">
       <c r="A350" s="4" t="inlineStr">
         <is>
-          <t>TC-1513</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B350" s="4" t="inlineStr">
@@ -10767,17 +10767,17 @@
       </c>
       <c r="C350" s="4" t="inlineStr">
         <is>
-          <t>Processor role allowed</t>
+          <t>Degraded when DB down</t>
         </is>
       </c>
       <c r="D350" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with processor token</t>
+          <t>Stop PostgreSQL, call endpoint with valid token</t>
         </is>
       </c>
       <c r="E350" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, status: "degraded", database: "error", database_error is non-null</t>
         </is>
       </c>
       <c r="F350" s="4" t="n"/>
@@ -10786,48 +10786,60 @@
       <c r="I350" s="4" t="n"/>
     </row>
     <row r="351">
-      <c r="A351" s="2" t="inlineStr">
-        <is>
-          <t>§12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="B351" s="2" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C351" s="3" t="n"/>
-      <c r="D351" s="3" t="n"/>
-      <c r="E351" s="3" t="n"/>
-      <c r="F351" s="3" t="n"/>
-      <c r="G351" s="3" t="n"/>
-      <c r="H351" s="3" t="n"/>
-      <c r="I351" s="3" t="n"/>
+      <c r="A351" s="4" t="inlineStr">
+        <is>
+          <t>TC-1512</t>
+        </is>
+      </c>
+      <c r="B351" s="4" t="inlineStr">
+        <is>
+          <t>12.15 System Health</t>
+        </is>
+      </c>
+      <c r="C351" s="4" t="inlineStr">
+        <is>
+          <t>Unauthenticated rejected</t>
+        </is>
+      </c>
+      <c r="D351" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/system-health without token</t>
+        </is>
+      </c>
+      <c r="E351" s="4" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="F351" s="4" t="n"/>
+      <c r="G351" s="4" t="n"/>
+      <c r="H351" s="4" t="n"/>
+      <c r="I351" s="4" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="4" t="inlineStr">
         <is>
-          <t>TC-1511</t>
+          <t>TC-1513</t>
         </is>
       </c>
       <c r="B352" s="4" t="inlineStr">
         <is>
-          <t>12.15.1 Readiness &amp; Version</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C352" s="4" t="inlineStr">
         <is>
-          <t>Liveness endpoint is public</t>
+          <t>Processor role allowed</t>
         </is>
       </c>
       <c r="D352" s="4" t="inlineStr">
         <is>
-          <t>GET /health/live without token</t>
+          <t>GET /introspection/system-health with processor token</t>
         </is>
       </c>
       <c r="E352" s="4" t="inlineStr">
         <is>
-          <t>200, service reports live</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F352" s="4" t="n"/>
@@ -10836,40 +10848,28 @@
       <c r="I352" s="4" t="n"/>
     </row>
     <row r="353">
-      <c r="A353" s="4" t="inlineStr">
-        <is>
-          <t>TC-1512</t>
-        </is>
-      </c>
-      <c r="B353" s="4" t="inlineStr">
+      <c r="A353" s="2" t="inlineStr">
+        <is>
+          <t>§12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="B353" s="2" t="inlineStr">
         <is>
           <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
-      <c r="C353" s="4" t="inlineStr">
-        <is>
-          <t>Readiness endpoint is public</t>
-        </is>
-      </c>
-      <c r="D353" s="4" t="inlineStr">
-        <is>
-          <t>GET /health/ready without token on a healthy system</t>
-        </is>
-      </c>
-      <c r="E353" s="4" t="inlineStr">
-        <is>
-          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
-        </is>
-      </c>
-      <c r="F353" s="4" t="n"/>
-      <c r="G353" s="4" t="n"/>
-      <c r="H353" s="4" t="n"/>
-      <c r="I353" s="4" t="n"/>
+      <c r="C353" s="3" t="n"/>
+      <c r="D353" s="3" t="n"/>
+      <c r="E353" s="3" t="n"/>
+      <c r="F353" s="3" t="n"/>
+      <c r="G353" s="3" t="n"/>
+      <c r="H353" s="3" t="n"/>
+      <c r="I353" s="3" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="4" t="inlineStr">
         <is>
-          <t>TC-1513</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B354" s="4" t="inlineStr">
@@ -10879,17 +10879,17 @@
       </c>
       <c r="C354" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports missing database configuration</t>
+          <t>Liveness endpoint is public</t>
         </is>
       </c>
       <c r="D354" s="4" t="inlineStr">
         <is>
-          <t>Clear DB config or test before configuration, then GET /health/ready</t>
+          <t>GET /health/live without token</t>
         </is>
       </c>
       <c r="E354" s="4" t="inlineStr">
         <is>
-          <t>503, status: "not_ready", reason indicates database is not configured</t>
+          <t>200, service reports live</t>
         </is>
       </c>
       <c r="F354" s="4" t="n"/>
@@ -10900,7 +10900,7 @@
     <row r="355">
       <c r="A355" s="4" t="inlineStr">
         <is>
-          <t>TC-1514</t>
+          <t>TC-1512</t>
         </is>
       </c>
       <c r="B355" s="4" t="inlineStr">
@@ -10910,17 +10910,17 @@
       </c>
       <c r="C355" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports mount or provider problems</t>
+          <t>Readiness endpoint is public</t>
         </is>
       </c>
       <c r="D355" s="4" t="inlineStr">
         <is>
-          <t>Break a configured mount or provider, then GET /health/ready</t>
+          <t>GET /health/ready without token on a healthy system</t>
         </is>
       </c>
       <c r="E355" s="4" t="inlineStr">
         <is>
-          <t>503, response identifies the failing check without using the generic error schema</t>
+          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
         </is>
       </c>
       <c r="F355" s="4" t="n"/>
@@ -10931,7 +10931,7 @@
     <row r="356">
       <c r="A356" s="4" t="inlineStr">
         <is>
-          <t>TC-1515</t>
+          <t>TC-1513</t>
         </is>
       </c>
       <c r="B356" s="4" t="inlineStr">
@@ -10941,17 +10941,17 @@
       </c>
       <c r="C356" s="4" t="inlineStr">
         <is>
-          <t>Version endpoint is public</t>
+          <t>Readiness reports missing database configuration</t>
         </is>
       </c>
       <c r="D356" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/version without token</t>
+          <t>Clear DB config or test before configuration, then GET /health/ready</t>
         </is>
       </c>
       <c r="E356" s="4" t="inlineStr">
         <is>
-          <t>200, returns version/application metadata</t>
+          <t>503, status: "not_ready", reason indicates database is not configured</t>
         </is>
       </c>
       <c r="F356" s="4" t="n"/>
@@ -10962,7 +10962,7 @@
     <row r="357">
       <c r="A357" s="4" t="inlineStr">
         <is>
-          <t>TC-1516</t>
+          <t>TC-1514</t>
         </is>
       </c>
       <c r="B357" s="4" t="inlineStr">
@@ -10972,17 +10972,17 @@
       </c>
       <c r="C357" s="4" t="inlineStr">
         <is>
-          <t>Readiness remains separate from authenticated system health</t>
+          <t>Readiness reports mount or provider problems</t>
         </is>
       </c>
       <c r="D357" s="4" t="inlineStr">
         <is>
-          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+          <t>Break a configured mount or provider, then GET /health/ready</t>
         </is>
       </c>
       <c r="E357" s="4" t="inlineStr">
         <is>
-          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+          <t>503, response identifies the failing check without using the generic error schema</t>
         </is>
       </c>
       <c r="F357" s="4" t="n"/>
@@ -10991,32 +10991,94 @@
       <c r="I357" s="4" t="n"/>
     </row>
     <row r="358">
-      <c r="A358" s="2" t="inlineStr">
+      <c r="A358" s="4" t="inlineStr">
+        <is>
+          <t>TC-1515</t>
+        </is>
+      </c>
+      <c r="B358" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C358" s="4" t="inlineStr">
+        <is>
+          <t>Version endpoint is public</t>
+        </is>
+      </c>
+      <c r="D358" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/version without token</t>
+        </is>
+      </c>
+      <c r="E358" s="4" t="inlineStr">
+        <is>
+          <t>200, returns version/application metadata</t>
+        </is>
+      </c>
+      <c r="F358" s="4" t="n"/>
+      <c r="G358" s="4" t="n"/>
+      <c r="H358" s="4" t="n"/>
+      <c r="I358" s="4" t="n"/>
+    </row>
+    <row r="359">
+      <c r="A359" s="4" t="inlineStr">
+        <is>
+          <t>TC-1516</t>
+        </is>
+      </c>
+      <c r="B359" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C359" s="4" t="inlineStr">
+        <is>
+          <t>Readiness remains separate from authenticated system health</t>
+        </is>
+      </c>
+      <c r="D359" s="4" t="inlineStr">
+        <is>
+          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+        </is>
+      </c>
+      <c r="E359" s="4" t="inlineStr">
+        <is>
+          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+        </is>
+      </c>
+      <c r="F359" s="4" t="n"/>
+      <c r="G359" s="4" t="n"/>
+      <c r="H359" s="4" t="n"/>
+      <c r="I359" s="4" t="n"/>
+    </row>
+    <row r="360">
+      <c r="A360" s="2" t="inlineStr">
         <is>
           <t>§12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="B358" s="2" t="inlineStr">
+      <c r="B360" s="2" t="inlineStr">
         <is>
           <t>12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="C358" s="3" t="n"/>
-      <c r="D358" s="3" t="n"/>
-      <c r="E358" s="3" t="n"/>
-      <c r="F358" s="3" t="n"/>
-      <c r="G358" s="3" t="n"/>
-      <c r="H358" s="3" t="n"/>
-      <c r="I358" s="3" t="n"/>
-    </row>
-    <row r="360">
-      <c r="A360" s="5" t="inlineStr">
+      <c r="C360" s="3" t="n"/>
+      <c r="D360" s="3" t="n"/>
+      <c r="E360" s="3" t="n"/>
+      <c r="F360" s="3" t="n"/>
+      <c r="G360" s="3" t="n"/>
+      <c r="H360" s="3" t="n"/>
+      <c r="I360" s="3" t="n"/>
+    </row>
+    <row r="362">
+      <c r="A362" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B360" s="5" t="n">
-        <v>330</v>
+      <c r="B362" s="5" t="n">
+        <v>332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Link Drive Detail job context to Job Detail
Surface the related Job ID on Drive Detail with direct navigation,
cover the new drive-job metadata behavior in frontend tests, and
sync the operator and QA documentation with the updated Drives UI.

Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -4740,7 +4740,7 @@
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>Project and Evidence link to the assigned job</t>
+          <t>Job ID links to the assigned job</t>
         </is>
       </c>
       <c r="D149" s="4" t="inlineStr">
@@ -4750,7 +4750,7 @@
       </c>
       <c r="E149" s="4" t="inlineStr">
         <is>
-          <t>Each row shows Project and Evidence, the Filesystem column is absent, and selecting either value opens the matching Job Detail for that drive's assignment rather than another drive on the same project</t>
+          <t>Each row shows Job ID, the Filesystem, Project, and Evidence columns are absent, and selecting the job ID opens the matching Job Detail for that drive's assignment rather than another drive on the same project</t>
         </is>
       </c>
       <c r="F149" s="4" t="n"/>
@@ -4771,7 +4771,7 @@
       </c>
       <c r="C150" s="4" t="inlineStr">
         <is>
-          <t>Drive Detail evidence follows the selected drive assignment</t>
+          <t>Drive Detail job metadata follows the selected drive assignment</t>
         </is>
       </c>
       <c r="D150" s="4" t="inlineStr">
@@ -4781,7 +4781,7 @@
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
-          <t>The Evidence value matches the selected drive's assigned job, even when another drive on the same project has a different evidence number</t>
+          <t>The Evidence and Job ID values match the selected drive's assigned job, even when another drive on the same project has a different evidence number</t>
         </is>
       </c>
       <c r="F150" s="4" t="n"/>
@@ -4802,7 +4802,7 @@
       </c>
       <c r="C151" s="4" t="inlineStr">
         <is>
-          <t>Formatted drives clear stale evidence UI state</t>
+          <t>Formatted drives clear stale drive-job UI state</t>
         </is>
       </c>
       <c r="D151" s="4" t="inlineStr">
@@ -4812,7 +4812,7 @@
       </c>
       <c r="E151" s="4" t="inlineStr">
         <is>
-          <t>Once formatting clears the project binding, Drive Detail shows Evidence as -, the Drives row no longer shows the old evidence value, and stale project or evidence links are not shown for that drive</t>
+          <t>Once formatting clears the project binding, Drive Detail shows Evidence and Job ID as -, the Drives row no longer shows the old job ID value, and stale job links are not shown for that drive</t>
         </is>
       </c>
       <c r="F151" s="4" t="n"/>
@@ -4895,7 +4895,7 @@
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>Device and serial columns stay aligned across UI</t>
+          <t>Device labels stay aligned across UI</t>
         </is>
       </c>
       <c r="D154" s="4" t="inlineStr">
@@ -4905,7 +4905,7 @@
       </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
-          <t>Drives shows Device plus Serial Number; Jobs list shows the same Device value; destination selector is labeled Select device and uses the same port-based label</t>
+          <t>Drives shows the same Device value used by the Jobs list and the destination selector, and Create/Edit Job keeps the destination control labeled Select device</t>
         </is>
       </c>
       <c r="F154" s="4" t="n"/>

</xml_diff>

<commit_message>
Add back Project column in Drives page
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -4740,7 +4740,7 @@
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>Job ID links to the assigned job</t>
+          <t>Project and Job ID reflect the assigned job</t>
         </is>
       </c>
       <c r="D149" s="4" t="inlineStr">
@@ -4750,7 +4750,7 @@
       </c>
       <c r="E149" s="4" t="inlineStr">
         <is>
-          <t>Each row shows Job ID, the Filesystem, Project, and Evidence columns are absent, and selecting the job ID opens the matching Job Detail for that drive's assignment rather than another drive on the same project</t>
+          <t>Each row shows Project and Job ID, the Filesystem and Evidence columns are absent, the project value matches the selected drive's assigned job, and selecting the job ID opens the matching Job Detail for that drive's assignment rather than another drive on the same project</t>
         </is>
       </c>
       <c r="F149" s="4" t="n"/>

</xml_diff>

<commit_message>
Align drive list docs with current UI
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -4931,12 +4931,12 @@
       </c>
       <c r="D155" s="4" t="inlineStr">
         <is>
-          <t>Open Drive Detail for a mounted managed USB drive, then return to Drives</t>
+          <t>Open Drive Detail for a mounted managed USB drive</t>
         </is>
       </c>
       <c r="E155" s="4" t="inlineStr">
         <is>
-          <t>Drive Detail shows total capacity plus the last known available space value or - when no reading is available yet, the mounted drive exposes a Browse button instead of a mount-path link, and the Drives page shows the matching available-space column value when present</t>
+          <t>Drive Detail shows total capacity plus the last known available space value or - when no reading is available yet, and the mounted drive exposes a Browse button instead of a mount-path link</t>
         </is>
       </c>
       <c r="F155" s="4" t="n"/>

</xml_diff>

<commit_message>
Remove size column from Drives view and update related tests
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -4750,7 +4750,7 @@
       </c>
       <c r="E149" s="4" t="inlineStr">
         <is>
-          <t>Each row shows Project and Job ID, the Filesystem and Evidence columns are absent, the project value matches the selected drive's assigned job, and selecting the job ID opens the matching Job Detail for that drive's assignment rather than another drive on the same project</t>
+          <t>Each row shows Project and Job ID, the Filesystem, Evidence, and Size columns are absent, the project value matches the selected drive's assigned job, and selecting the job ID opens the matching Job Detail for that drive's assignment rather than another drive on the same project</t>
         </is>
       </c>
       <c r="F149" s="4" t="n"/>
@@ -4926,7 +4926,7 @@
       </c>
       <c r="C155" s="4" t="inlineStr">
         <is>
-          <t>Mounted drive surfaces available space and Browse entry</t>
+          <t>Mounted drive surfaces capacity, available space, and Browse entry</t>
         </is>
       </c>
       <c r="D155" s="4" t="inlineStr">
@@ -4936,7 +4936,7 @@
       </c>
       <c r="E155" s="4" t="inlineStr">
         <is>
-          <t>Drive Detail shows total capacity plus the last known available space value or - when no reading is available yet, and the mounted drive exposes a Browse button instead of a mount-path link</t>
+          <t>The Drives list does not show a Size column, Drive Detail shows total capacity plus the last known available space value or - when no reading is available yet, and the mounted drive exposes a Browse button instead of a mount-path link</t>
         </is>
       </c>
       <c r="F155" s="4" t="n"/>

</xml_diff>

<commit_message>
Recover stale startup analysis after restart
Restore jobs left in startup_analysis_status=ANALYZING during startup reconciliation.
Recover READY when the cached analysis is still current, otherwise reset the job
to NOT_ANALYZED, record the reconciliation in audit logs, and document the
restart behavior for operators and QA.
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I337"/>
+  <dimension ref="A1:I339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9723,48 +9723,60 @@
       <c r="I313" s="4" t="n"/>
     </row>
     <row r="314">
-      <c r="A314" s="2" t="inlineStr">
-        <is>
-          <t>§12.15 System Health</t>
-        </is>
-      </c>
-      <c r="B314" s="2" t="inlineStr">
-        <is>
-          <t>12.15 System Health</t>
-        </is>
-      </c>
-      <c r="C314" s="3" t="n"/>
-      <c r="D314" s="3" t="n"/>
-      <c r="E314" s="3" t="n"/>
-      <c r="F314" s="3" t="n"/>
-      <c r="G314" s="3" t="n"/>
-      <c r="H314" s="3" t="n"/>
-      <c r="I314" s="3" t="n"/>
+      <c r="A314" s="4" t="inlineStr">
+        <is>
+          <t>TC-1418</t>
+        </is>
+      </c>
+      <c r="B314" s="4" t="inlineStr">
+        <is>
+          <t>12.14 Startup Reconciliation</t>
+        </is>
+      </c>
+      <c r="C314" s="4" t="inlineStr">
+        <is>
+          <t>Restart clears stale in-progress startup analysis when no valid cache remains</t>
+        </is>
+      </c>
+      <c r="D314" s="4" t="inlineStr">
+        <is>
+          <t>Trigger manual Analyze for a PENDING job, restart ECUBE before the scan completes, then reopen Job Detail</t>
+        </is>
+      </c>
+      <c r="E314" s="4" t="inlineStr">
+        <is>
+          <t>Job is no longer stuck in ANALYZING, startup-analysis state returns to NOT_ANALYZED, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "analysis_interrupted_by_restart", and Analyze or Start is available again</t>
+        </is>
+      </c>
+      <c r="F314" s="4" t="n"/>
+      <c r="G314" s="4" t="n"/>
+      <c r="H314" s="4" t="n"/>
+      <c r="I314" s="4" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="4" t="inlineStr">
         <is>
-          <t>TC-1501</t>
+          <t>TC-1419</t>
         </is>
       </c>
       <c r="B315" s="4" t="inlineStr">
         <is>
-          <t>12.15 System Health</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C315" s="4" t="inlineStr">
         <is>
-          <t>Healthy response</t>
+          <t>Restart restores READY when the interrupted startup-analysis cache is still current</t>
         </is>
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with valid token</t>
+          <t>Trigger manual Analyze for a job with a stable source tree, restart ECUBE after the reusable snapshot has been persisted but before the manual analyze workflow fully completes, then reopen Job Detail</t>
         </is>
       </c>
       <c r="E315" s="4" t="inlineStr">
         <is>
-          <t>200, status: "ok", database: "connected"</t>
+          <t>Job shows startup_analysis_status: READY, the previous file and byte totals are still available, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "valid_cache_restored_after_restart", and Start can proceed without forcing a fresh scan</t>
         </is>
       </c>
       <c r="F315" s="4" t="n"/>
@@ -9773,40 +9785,28 @@
       <c r="I315" s="4" t="n"/>
     </row>
     <row r="316">
-      <c r="A316" s="4" t="inlineStr">
-        <is>
-          <t>TC-1502</t>
-        </is>
-      </c>
-      <c r="B316" s="4" t="inlineStr">
+      <c r="A316" s="2" t="inlineStr">
+        <is>
+          <t>§12.15 System Health</t>
+        </is>
+      </c>
+      <c r="B316" s="2" t="inlineStr">
         <is>
           <t>12.15 System Health</t>
         </is>
       </c>
-      <c r="C316" s="4" t="inlineStr">
-        <is>
-          <t>CPU metric present</t>
-        </is>
-      </c>
-      <c r="D316" s="4" t="inlineStr">
-        <is>
-          <t>Inspect response body</t>
-        </is>
-      </c>
-      <c r="E316" s="4" t="inlineStr">
-        <is>
-          <t>cpu_percent is a number between 0 and 100</t>
-        </is>
-      </c>
-      <c r="F316" s="4" t="n"/>
-      <c r="G316" s="4" t="n"/>
-      <c r="H316" s="4" t="n"/>
-      <c r="I316" s="4" t="n"/>
+      <c r="C316" s="3" t="n"/>
+      <c r="D316" s="3" t="n"/>
+      <c r="E316" s="3" t="n"/>
+      <c r="F316" s="3" t="n"/>
+      <c r="G316" s="3" t="n"/>
+      <c r="H316" s="3" t="n"/>
+      <c r="I316" s="3" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="4" t="inlineStr">
         <is>
-          <t>TC-1503</t>
+          <t>TC-1501</t>
         </is>
       </c>
       <c r="B317" s="4" t="inlineStr">
@@ -9816,17 +9816,17 @@
       </c>
       <c r="C317" s="4" t="inlineStr">
         <is>
-          <t>Memory metrics present</t>
+          <t>Healthy response</t>
         </is>
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>GET /introspection/system-health with valid token</t>
         </is>
       </c>
       <c r="E317" s="4" t="inlineStr">
         <is>
-          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
+          <t>200, status: "ok", database: "connected"</t>
         </is>
       </c>
       <c r="F317" s="4" t="n"/>
@@ -9837,7 +9837,7 @@
     <row r="318">
       <c r="A318" s="4" t="inlineStr">
         <is>
-          <t>TC-1504</t>
+          <t>TC-1502</t>
         </is>
       </c>
       <c r="B318" s="4" t="inlineStr">
@@ -9847,7 +9847,7 @@
       </c>
       <c r="C318" s="4" t="inlineStr">
         <is>
-          <t>Disk I/O metrics present</t>
+          <t>CPU metric present</t>
         </is>
       </c>
       <c r="D318" s="4" t="inlineStr">
@@ -9857,7 +9857,7 @@
       </c>
       <c r="E318" s="4" t="inlineStr">
         <is>
-          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
+          <t>cpu_percent is a number between 0 and 100</t>
         </is>
       </c>
       <c r="F318" s="4" t="n"/>
@@ -9868,7 +9868,7 @@
     <row r="319">
       <c r="A319" s="4" t="inlineStr">
         <is>
-          <t>TC-1505</t>
+          <t>TC-1503</t>
         </is>
       </c>
       <c r="B319" s="4" t="inlineStr">
@@ -9878,17 +9878,17 @@
       </c>
       <c r="C319" s="4" t="inlineStr">
         <is>
-          <t>Active jobs count</t>
+          <t>Memory metrics present</t>
         </is>
       </c>
       <c r="D319" s="4" t="inlineStr">
         <is>
-          <t>Start an export job, call endpoint</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E319" s="4" t="inlineStr">
         <is>
-          <t>active_jobs ≥ 1</t>
+          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
         </is>
       </c>
       <c r="F319" s="4" t="n"/>
@@ -9899,7 +9899,7 @@
     <row r="320">
       <c r="A320" s="4" t="inlineStr">
         <is>
-          <t>TC-1506</t>
+          <t>TC-1504</t>
         </is>
       </c>
       <c r="B320" s="4" t="inlineStr">
@@ -9909,17 +9909,17 @@
       </c>
       <c r="C320" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size</t>
+          <t>Disk I/O metrics present</t>
         </is>
       </c>
       <c r="D320" s="4" t="inlineStr">
         <is>
-          <t>Create a PENDING job (created but not started), call endpoint</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E320" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size ≥ 1</t>
+          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
         </is>
       </c>
       <c r="F320" s="4" t="n"/>
@@ -9930,7 +9930,7 @@
     <row r="321">
       <c r="A321" s="4" t="inlineStr">
         <is>
-          <t>TC-1507</t>
+          <t>TC-1505</t>
         </is>
       </c>
       <c r="B321" s="4" t="inlineStr">
@@ -9940,17 +9940,17 @@
       </c>
       <c r="C321" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size decrements</t>
+          <t>Active jobs count</t>
         </is>
       </c>
       <c r="D321" s="4" t="inlineStr">
         <is>
-          <t>Start the pending job, call endpoint again</t>
+          <t>Start an export job, call endpoint</t>
         </is>
       </c>
       <c r="E321" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
+          <t>active_jobs ≥ 1</t>
         </is>
       </c>
       <c r="F321" s="4" t="n"/>
@@ -9961,7 +9961,7 @@
     <row r="322">
       <c r="A322" s="4" t="inlineStr">
         <is>
-          <t>TC-1508</t>
+          <t>TC-1506</t>
         </is>
       </c>
       <c r="B322" s="4" t="inlineStr">
@@ -9971,17 +9971,17 @@
       </c>
       <c r="C322" s="4" t="inlineStr">
         <is>
-          <t>ECUBE process metrics present</t>
+          <t>Worker queue size</t>
         </is>
       </c>
       <c r="D322" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Create a PENDING job (created but not started), call endpoint</t>
         </is>
       </c>
       <c r="E322" s="4" t="inlineStr">
         <is>
-          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
+          <t>worker_queue_size ≥ 1</t>
         </is>
       </c>
       <c r="F322" s="4" t="n"/>
@@ -9992,7 +9992,7 @@
     <row r="323">
       <c r="A323" s="4" t="inlineStr">
         <is>
-          <t>TC-1509</t>
+          <t>TC-1507</t>
         </is>
       </c>
       <c r="B323" s="4" t="inlineStr">
@@ -10002,17 +10002,17 @@
       </c>
       <c r="C323" s="4" t="inlineStr">
         <is>
-          <t>Active copy-thread correlation</t>
+          <t>Worker queue size decrements</t>
         </is>
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>Run an export job with active copy workers, call endpoint during the run</t>
+          <t>Start the pending job, call endpoint again</t>
         </is>
       </c>
       <c r="E323" s="4" t="inlineStr">
         <is>
-          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
+          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
         </is>
       </c>
       <c r="F323" s="4" t="n"/>
@@ -10023,7 +10023,7 @@
     <row r="324">
       <c r="A324" s="4" t="inlineStr">
         <is>
-          <t>TC-1510</t>
+          <t>TC-1508</t>
         </is>
       </c>
       <c r="B324" s="4" t="inlineStr">
@@ -10033,17 +10033,17 @@
       </c>
       <c r="C324" s="4" t="inlineStr">
         <is>
-          <t>ECUBE process metrics degrade safely</t>
+          <t>ECUBE process metrics present</t>
         </is>
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E324" s="4" t="inlineStr">
         <is>
-          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
+          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
         </is>
       </c>
       <c r="F324" s="4" t="n"/>
@@ -10054,7 +10054,7 @@
     <row r="325">
       <c r="A325" s="4" t="inlineStr">
         <is>
-          <t>TC-1511</t>
+          <t>TC-1509</t>
         </is>
       </c>
       <c r="B325" s="4" t="inlineStr">
@@ -10064,17 +10064,17 @@
       </c>
       <c r="C325" s="4" t="inlineStr">
         <is>
-          <t>Degraded when DB down</t>
+          <t>Active copy-thread correlation</t>
         </is>
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, call endpoint with valid token</t>
+          <t>Run an export job with active copy workers, call endpoint during the run</t>
         </is>
       </c>
       <c r="E325" s="4" t="inlineStr">
         <is>
-          <t>200, status: "degraded", database: "error", database_error is non-null</t>
+          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
         </is>
       </c>
       <c r="F325" s="4" t="n"/>
@@ -10085,7 +10085,7 @@
     <row r="326">
       <c r="A326" s="4" t="inlineStr">
         <is>
-          <t>TC-1512</t>
+          <t>TC-1510</t>
         </is>
       </c>
       <c r="B326" s="4" t="inlineStr">
@@ -10095,17 +10095,17 @@
       </c>
       <c r="C326" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated rejected</t>
+          <t>ECUBE process metrics degrade safely</t>
         </is>
       </c>
       <c r="D326" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health without token</t>
+          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
         </is>
       </c>
       <c r="E326" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
         </is>
       </c>
       <c r="F326" s="4" t="n"/>
@@ -10116,7 +10116,7 @@
     <row r="327">
       <c r="A327" s="4" t="inlineStr">
         <is>
-          <t>TC-1513</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B327" s="4" t="inlineStr">
@@ -10126,17 +10126,17 @@
       </c>
       <c r="C327" s="4" t="inlineStr">
         <is>
-          <t>Processor role allowed</t>
+          <t>Degraded when DB down</t>
         </is>
       </c>
       <c r="D327" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with processor token</t>
+          <t>Stop PostgreSQL, call endpoint with valid token</t>
         </is>
       </c>
       <c r="E327" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, status: "degraded", database: "error", database_error is non-null</t>
         </is>
       </c>
       <c r="F327" s="4" t="n"/>
@@ -10145,48 +10145,60 @@
       <c r="I327" s="4" t="n"/>
     </row>
     <row r="328">
-      <c r="A328" s="2" t="inlineStr">
-        <is>
-          <t>§12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="B328" s="2" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C328" s="3" t="n"/>
-      <c r="D328" s="3" t="n"/>
-      <c r="E328" s="3" t="n"/>
-      <c r="F328" s="3" t="n"/>
-      <c r="G328" s="3" t="n"/>
-      <c r="H328" s="3" t="n"/>
-      <c r="I328" s="3" t="n"/>
+      <c r="A328" s="4" t="inlineStr">
+        <is>
+          <t>TC-1512</t>
+        </is>
+      </c>
+      <c r="B328" s="4" t="inlineStr">
+        <is>
+          <t>12.15 System Health</t>
+        </is>
+      </c>
+      <c r="C328" s="4" t="inlineStr">
+        <is>
+          <t>Unauthenticated rejected</t>
+        </is>
+      </c>
+      <c r="D328" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/system-health without token</t>
+        </is>
+      </c>
+      <c r="E328" s="4" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="F328" s="4" t="n"/>
+      <c r="G328" s="4" t="n"/>
+      <c r="H328" s="4" t="n"/>
+      <c r="I328" s="4" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="4" t="inlineStr">
         <is>
-          <t>TC-1511</t>
+          <t>TC-1513</t>
         </is>
       </c>
       <c r="B329" s="4" t="inlineStr">
         <is>
-          <t>12.15.1 Readiness &amp; Version</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C329" s="4" t="inlineStr">
         <is>
-          <t>Liveness endpoint is public</t>
+          <t>Processor role allowed</t>
         </is>
       </c>
       <c r="D329" s="4" t="inlineStr">
         <is>
-          <t>GET /health/live without token</t>
+          <t>GET /introspection/system-health with processor token</t>
         </is>
       </c>
       <c r="E329" s="4" t="inlineStr">
         <is>
-          <t>200, service reports live</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F329" s="4" t="n"/>
@@ -10195,40 +10207,28 @@
       <c r="I329" s="4" t="n"/>
     </row>
     <row r="330">
-      <c r="A330" s="4" t="inlineStr">
-        <is>
-          <t>TC-1512</t>
-        </is>
-      </c>
-      <c r="B330" s="4" t="inlineStr">
+      <c r="A330" s="2" t="inlineStr">
+        <is>
+          <t>§12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="B330" s="2" t="inlineStr">
         <is>
           <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
-      <c r="C330" s="4" t="inlineStr">
-        <is>
-          <t>Readiness endpoint is public</t>
-        </is>
-      </c>
-      <c r="D330" s="4" t="inlineStr">
-        <is>
-          <t>GET /health/ready without token on a healthy system</t>
-        </is>
-      </c>
-      <c r="E330" s="4" t="inlineStr">
-        <is>
-          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
-        </is>
-      </c>
-      <c r="F330" s="4" t="n"/>
-      <c r="G330" s="4" t="n"/>
-      <c r="H330" s="4" t="n"/>
-      <c r="I330" s="4" t="n"/>
+      <c r="C330" s="3" t="n"/>
+      <c r="D330" s="3" t="n"/>
+      <c r="E330" s="3" t="n"/>
+      <c r="F330" s="3" t="n"/>
+      <c r="G330" s="3" t="n"/>
+      <c r="H330" s="3" t="n"/>
+      <c r="I330" s="3" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="4" t="inlineStr">
         <is>
-          <t>TC-1513</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B331" s="4" t="inlineStr">
@@ -10238,17 +10238,17 @@
       </c>
       <c r="C331" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports missing database configuration</t>
+          <t>Liveness endpoint is public</t>
         </is>
       </c>
       <c r="D331" s="4" t="inlineStr">
         <is>
-          <t>Clear DB config or test before configuration, then GET /health/ready</t>
+          <t>GET /health/live without token</t>
         </is>
       </c>
       <c r="E331" s="4" t="inlineStr">
         <is>
-          <t>503, status: "not_ready", reason indicates database is not configured</t>
+          <t>200, service reports live</t>
         </is>
       </c>
       <c r="F331" s="4" t="n"/>
@@ -10259,7 +10259,7 @@
     <row r="332">
       <c r="A332" s="4" t="inlineStr">
         <is>
-          <t>TC-1514</t>
+          <t>TC-1512</t>
         </is>
       </c>
       <c r="B332" s="4" t="inlineStr">
@@ -10269,17 +10269,17 @@
       </c>
       <c r="C332" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports mount or provider problems</t>
+          <t>Readiness endpoint is public</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr">
         <is>
-          <t>Break a configured mount or provider, then GET /health/ready</t>
+          <t>GET /health/ready without token on a healthy system</t>
         </is>
       </c>
       <c r="E332" s="4" t="inlineStr">
         <is>
-          <t>503, response identifies the failing check without using the generic error schema</t>
+          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
         </is>
       </c>
       <c r="F332" s="4" t="n"/>
@@ -10290,7 +10290,7 @@
     <row r="333">
       <c r="A333" s="4" t="inlineStr">
         <is>
-          <t>TC-1515</t>
+          <t>TC-1513</t>
         </is>
       </c>
       <c r="B333" s="4" t="inlineStr">
@@ -10300,17 +10300,17 @@
       </c>
       <c r="C333" s="4" t="inlineStr">
         <is>
-          <t>Version endpoint is public</t>
+          <t>Readiness reports missing database configuration</t>
         </is>
       </c>
       <c r="D333" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/version without token</t>
+          <t>Clear DB config or test before configuration, then GET /health/ready</t>
         </is>
       </c>
       <c r="E333" s="4" t="inlineStr">
         <is>
-          <t>200, returns version/application metadata</t>
+          <t>503, status: "not_ready", reason indicates database is not configured</t>
         </is>
       </c>
       <c r="F333" s="4" t="n"/>
@@ -10321,7 +10321,7 @@
     <row r="334">
       <c r="A334" s="4" t="inlineStr">
         <is>
-          <t>TC-1516</t>
+          <t>TC-1514</t>
         </is>
       </c>
       <c r="B334" s="4" t="inlineStr">
@@ -10331,17 +10331,17 @@
       </c>
       <c r="C334" s="4" t="inlineStr">
         <is>
-          <t>Readiness remains separate from authenticated system health</t>
+          <t>Readiness reports mount or provider problems</t>
         </is>
       </c>
       <c r="D334" s="4" t="inlineStr">
         <is>
-          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+          <t>Break a configured mount or provider, then GET /health/ready</t>
         </is>
       </c>
       <c r="E334" s="4" t="inlineStr">
         <is>
-          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+          <t>503, response identifies the failing check without using the generic error schema</t>
         </is>
       </c>
       <c r="F334" s="4" t="n"/>
@@ -10350,32 +10350,94 @@
       <c r="I334" s="4" t="n"/>
     </row>
     <row r="335">
-      <c r="A335" s="2" t="inlineStr">
+      <c r="A335" s="4" t="inlineStr">
+        <is>
+          <t>TC-1515</t>
+        </is>
+      </c>
+      <c r="B335" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C335" s="4" t="inlineStr">
+        <is>
+          <t>Version endpoint is public</t>
+        </is>
+      </c>
+      <c r="D335" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/version without token</t>
+        </is>
+      </c>
+      <c r="E335" s="4" t="inlineStr">
+        <is>
+          <t>200, returns version/application metadata</t>
+        </is>
+      </c>
+      <c r="F335" s="4" t="n"/>
+      <c r="G335" s="4" t="n"/>
+      <c r="H335" s="4" t="n"/>
+      <c r="I335" s="4" t="n"/>
+    </row>
+    <row r="336">
+      <c r="A336" s="4" t="inlineStr">
+        <is>
+          <t>TC-1516</t>
+        </is>
+      </c>
+      <c r="B336" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C336" s="4" t="inlineStr">
+        <is>
+          <t>Readiness remains separate from authenticated system health</t>
+        </is>
+      </c>
+      <c r="D336" s="4" t="inlineStr">
+        <is>
+          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+        </is>
+      </c>
+      <c r="E336" s="4" t="inlineStr">
+        <is>
+          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+        </is>
+      </c>
+      <c r="F336" s="4" t="n"/>
+      <c r="G336" s="4" t="n"/>
+      <c r="H336" s="4" t="n"/>
+      <c r="I336" s="4" t="n"/>
+    </row>
+    <row r="337">
+      <c r="A337" s="2" t="inlineStr">
         <is>
           <t>§12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="B335" s="2" t="inlineStr">
+      <c r="B337" s="2" t="inlineStr">
         <is>
           <t>12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="C335" s="3" t="n"/>
-      <c r="D335" s="3" t="n"/>
-      <c r="E335" s="3" t="n"/>
-      <c r="F335" s="3" t="n"/>
-      <c r="G335" s="3" t="n"/>
-      <c r="H335" s="3" t="n"/>
-      <c r="I335" s="3" t="n"/>
-    </row>
-    <row r="337">
-      <c r="A337" s="5" t="inlineStr">
+      <c r="C337" s="3" t="n"/>
+      <c r="D337" s="3" t="n"/>
+      <c r="E337" s="3" t="n"/>
+      <c r="F337" s="3" t="n"/>
+      <c r="G337" s="3" t="n"/>
+      <c r="H337" s="3" t="n"/>
+      <c r="I337" s="3" t="n"/>
+    </row>
+    <row r="339">
+      <c r="A339" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B337" s="5" t="n">
-        <v>307</v>
+      <c r="B339" s="5" t="n">
+        <v>309</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Redirect setup-required API failures back to the setup wizard
Handle the backend's database-not-configured 503 error contract in the shared frontend API client so normal UI requests return the browser to /setup instead of showing only a generic server-error toast.

Cover the redirect and fallback behavior in client tests, and sync operator, architecture, QA, UI-use-case, and generated help documentation with the new recovery flow.
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I339"/>
+  <dimension ref="A1:I340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8786,59 +8786,59 @@
       <c r="I282" s="4" t="n"/>
     </row>
     <row r="283">
-      <c r="A283" s="2" t="inlineStr">
+      <c r="A283" s="4" t="inlineStr">
+        <is>
+          <t>TC-1115</t>
+        </is>
+      </c>
+      <c r="B283" s="4" t="inlineStr">
+        <is>
+          <t>12.11 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C283" s="4" t="inlineStr">
+        <is>
+          <t>Setup-required API redirect</t>
+        </is>
+      </c>
+      <c r="D283" s="4" t="inlineStr">
+        <is>
+          <t>While using a normal UI screen, trigger a backend response with status 503, code HTTP_503, and message Database is not configured yet. Complete setup first.</t>
+        </is>
+      </c>
+      <c r="E283" s="4" t="inlineStr">
+        <is>
+          <t>The browser redirects to /setup and the operator is not left only with the generic server-error toast</t>
+        </is>
+      </c>
+      <c r="F283" s="4" t="n"/>
+      <c r="G283" s="4" t="n"/>
+      <c r="H283" s="4" t="n"/>
+      <c r="I283" s="4" t="n"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="inlineStr">
         <is>
           <t>§12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
-      <c r="B283" s="2" t="inlineStr">
+      <c r="B284" s="2" t="inlineStr">
         <is>
           <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
-      <c r="C283" s="3" t="n"/>
-      <c r="D283" s="3" t="n"/>
-      <c r="E283" s="3" t="n"/>
-      <c r="F283" s="3" t="n"/>
-      <c r="G283" s="3" t="n"/>
-      <c r="H283" s="3" t="n"/>
-      <c r="I283" s="3" t="n"/>
-    </row>
-    <row r="284">
-      <c r="A284" s="4" t="inlineStr">
-        <is>
-          <t>TC-1201</t>
-        </is>
-      </c>
-      <c r="B284" s="4" t="inlineStr">
-        <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
-        </is>
-      </c>
-      <c r="C284" s="4" t="inlineStr">
-        <is>
-          <t>Retrieve stored CoC snapshot — archived job</t>
-        </is>
-      </c>
-      <c r="D284" s="4" t="inlineStr">
-        <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for an archived job that already has a stored snapshot</t>
-        </is>
-      </c>
-      <c r="E284" s="4" t="inlineStr">
-        <is>
-          <t>200, response contains the stored snapshot and snapshot metadata</t>
-        </is>
-      </c>
-      <c r="F284" s="4" t="n"/>
-      <c r="G284" s="4" t="n"/>
-      <c r="H284" s="4" t="n"/>
-      <c r="I284" s="4" t="n"/>
+      <c r="C284" s="3" t="n"/>
+      <c r="D284" s="3" t="n"/>
+      <c r="E284" s="3" t="n"/>
+      <c r="F284" s="3" t="n"/>
+      <c r="G284" s="3" t="n"/>
+      <c r="H284" s="3" t="n"/>
+      <c r="I284" s="3" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="4" t="inlineStr">
         <is>
-          <t>TC-1202</t>
+          <t>TC-1201</t>
         </is>
       </c>
       <c r="B285" s="4" t="inlineStr">
@@ -8848,17 +8848,17 @@
       </c>
       <c r="C285" s="4" t="inlineStr">
         <is>
-          <t>Retrieve stored CoC snapshot — active job</t>
+          <t>Retrieve stored CoC snapshot — archived job</t>
         </is>
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job that already has a stored snapshot</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for an archived job that already has a stored snapshot</t>
         </is>
       </c>
       <c r="E285" s="4" t="inlineStr">
         <is>
-          <t>200, response contains the stored snapshot and does not regenerate it</t>
+          <t>200, response contains the stored snapshot and snapshot metadata</t>
         </is>
       </c>
       <c r="F285" s="4" t="n"/>
@@ -8869,7 +8869,7 @@
     <row r="286">
       <c r="A286" s="4" t="inlineStr">
         <is>
-          <t>TC-1203</t>
+          <t>TC-1202</t>
         </is>
       </c>
       <c r="B286" s="4" t="inlineStr">
@@ -8879,17 +8879,17 @@
       </c>
       <c r="C286" s="4" t="inlineStr">
         <is>
-          <t>CoC read — missing stored snapshot</t>
+          <t>Retrieve stored CoC snapshot — active job</t>
         </is>
       </c>
       <c r="D286" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job with no stored snapshot yet</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job that already has a stored snapshot</t>
         </is>
       </c>
       <c r="E286" s="4" t="inlineStr">
         <is>
-          <t>404, message explains that the report must be refreshed first</t>
+          <t>200, response contains the stored snapshot and does not regenerate it</t>
         </is>
       </c>
       <c r="F286" s="4" t="n"/>
@@ -8900,7 +8900,7 @@
     <row r="287">
       <c r="A287" s="4" t="inlineStr">
         <is>
-          <t>TC-1204</t>
+          <t>TC-1203</t>
         </is>
       </c>
       <c r="B287" s="4" t="inlineStr">
@@ -8910,17 +8910,17 @@
       </c>
       <c r="C287" s="4" t="inlineStr">
         <is>
-          <t>CoC read — processor denied</t>
+          <t>CoC read — missing stored snapshot</t>
         </is>
       </c>
       <c r="D287" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody with processor token</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job with no stored snapshot yet</t>
         </is>
       </c>
       <c r="E287" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>404, message explains that the report must be refreshed first</t>
         </is>
       </c>
       <c r="F287" s="4" t="n"/>
@@ -8931,7 +8931,7 @@
     <row r="288">
       <c r="A288" s="4" t="inlineStr">
         <is>
-          <t>TC-1205</t>
+          <t>TC-1204</t>
         </is>
       </c>
       <c r="B288" s="4" t="inlineStr">
@@ -8941,17 +8941,17 @@
       </c>
       <c r="C288" s="4" t="inlineStr">
         <is>
-          <t>CoC read — unauthenticated denied</t>
+          <t>CoC read — processor denied</t>
         </is>
       </c>
       <c r="D288" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody without token</t>
+          <t>GET /jobs/{job_id}/chain-of-custody with processor token</t>
         </is>
       </c>
       <c r="E288" s="4" t="inlineStr">
         <is>
-          <t>401, UNAUTHORIZED</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F288" s="4" t="n"/>
@@ -8962,7 +8962,7 @@
     <row r="289">
       <c r="A289" s="4" t="inlineStr">
         <is>
-          <t>TC-1206</t>
+          <t>TC-1205</t>
         </is>
       </c>
       <c r="B289" s="4" t="inlineStr">
@@ -8972,17 +8972,17 @@
       </c>
       <c r="C289" s="4" t="inlineStr">
         <is>
-          <t>CoC snapshot fields</t>
+          <t>CoC read — unauthenticated denied</t>
         </is>
       </c>
       <c r="D289" s="4" t="inlineStr">
         <is>
-          <t>Inspect any stored-snapshot response</t>
+          <t>GET /jobs/{job_id}/chain-of-custody without token</t>
         </is>
       </c>
       <c r="E289" s="4" t="inlineStr">
         <is>
-          <t>snapshot_stored_at, snapshot_updated_at, snapshot_stored_by, reports[], and manifest/custody fields are present</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F289" s="4" t="n"/>
@@ -8993,7 +8993,7 @@
     <row r="290">
       <c r="A290" s="4" t="inlineStr">
         <is>
-          <t>TC-1207</t>
+          <t>TC-1206</t>
         </is>
       </c>
       <c r="B290" s="4" t="inlineStr">
@@ -9003,17 +9003,17 @@
       </c>
       <c r="C290" s="4" t="inlineStr">
         <is>
-          <t>CoC events include lifecycle</t>
+          <t>CoC snapshot fields</t>
         </is>
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>Inspect chain_of_custody_events in a stored report for a completed job</t>
+          <t>Inspect any stored-snapshot response</t>
         </is>
       </c>
       <c r="E290" s="4" t="inlineStr">
         <is>
-          <t>Events include DRIVE_INITIALIZED, JOB_CREATED, JOB_STARTED, JOB_COMPLETED, DRIVE_EJECT_PREPARED, and COC_HANDOFF_CONFIRMED when applicable</t>
+          <t>snapshot_stored_at, snapshot_updated_at, snapshot_stored_by, reports[], and manifest/custody fields are present</t>
         </is>
       </c>
       <c r="F290" s="4" t="n"/>
@@ -9024,7 +9024,7 @@
     <row r="291">
       <c r="A291" s="4" t="inlineStr">
         <is>
-          <t>TC-1208</t>
+          <t>TC-1207</t>
         </is>
       </c>
       <c r="B291" s="4" t="inlineStr">
@@ -9034,17 +9034,17 @@
       </c>
       <c r="C291" s="4" t="inlineStr">
         <is>
-          <t>CoC manifest summary</t>
+          <t>CoC events include lifecycle</t>
         </is>
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>Inspect manifest_summary in the stored report</t>
+          <t>Inspect chain_of_custody_events in a stored report for a completed job</t>
         </is>
       </c>
       <c r="E291" s="4" t="inlineStr">
         <is>
-          <t>Array of objects with job_id, evidence_number, processor_notes, total_files, total_bytes, and manifest_count</t>
+          <t>Events include DRIVE_INITIALIZED, JOB_CREATED, JOB_STARTED, JOB_COMPLETED, DRIVE_EJECT_PREPARED, and COC_HANDOFF_CONFIRMED when applicable</t>
         </is>
       </c>
       <c r="F291" s="4" t="n"/>
@@ -9055,7 +9055,7 @@
     <row r="292">
       <c r="A292" s="4" t="inlineStr">
         <is>
-          <t>TC-1209</t>
+          <t>TC-1208</t>
         </is>
       </c>
       <c r="B292" s="4" t="inlineStr">
@@ -9065,17 +9065,17 @@
       </c>
       <c r="C292" s="4" t="inlineStr">
         <is>
-          <t>CoC — delivery_time absence (no handoff)</t>
+          <t>CoC manifest summary</t>
         </is>
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>Complete a job and store a snapshot before handoff</t>
+          <t>Inspect manifest_summary in the stored report</t>
         </is>
       </c>
       <c r="E292" s="4" t="inlineStr">
         <is>
-          <t>chain_of_custody_events do not contain COC_HANDOFF_CONFIRMED; custody_complete is false</t>
+          <t>Array of objects with job_id, evidence_number, processor_notes, total_files, total_bytes, and manifest_count</t>
         </is>
       </c>
       <c r="F292" s="4" t="n"/>
@@ -9086,7 +9086,7 @@
     <row r="293">
       <c r="A293" s="4" t="inlineStr">
         <is>
-          <t>TC-1210</t>
+          <t>TC-1209</t>
         </is>
       </c>
       <c r="B293" s="4" t="inlineStr">
@@ -9096,17 +9096,17 @@
       </c>
       <c r="C293" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — valid</t>
+          <t>CoC — delivery_time absence (no handoff)</t>
         </is>
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh with admin or manager token for a non-archived job with assignments</t>
+          <t>Complete a job and store a snapshot before handoff</t>
         </is>
       </c>
       <c r="E293" s="4" t="inlineStr">
         <is>
-          <t>200, response contains the refreshed stored snapshot and updated snapshot metadata</t>
+          <t>chain_of_custody_events do not contain COC_HANDOFF_CONFIRMED; custody_complete is false</t>
         </is>
       </c>
       <c r="F293" s="4" t="n"/>
@@ -9117,7 +9117,7 @@
     <row r="294">
       <c r="A294" s="4" t="inlineStr">
         <is>
-          <t>TC-1211</t>
+          <t>TC-1210</t>
         </is>
       </c>
       <c r="B294" s="4" t="inlineStr">
@@ -9127,17 +9127,17 @@
       </c>
       <c r="C294" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — auditor denied</t>
+          <t>CoC refresh — valid</t>
         </is>
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh with auditor token</t>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh with admin or manager token for a non-archived job with assignments</t>
         </is>
       </c>
       <c r="E294" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>200, response contains the refreshed stored snapshot and updated snapshot metadata</t>
         </is>
       </c>
       <c r="F294" s="4" t="n"/>
@@ -9148,7 +9148,7 @@
     <row r="295">
       <c r="A295" s="4" t="inlineStr">
         <is>
-          <t>TC-1212</t>
+          <t>TC-1211</t>
         </is>
       </c>
       <c r="B295" s="4" t="inlineStr">
@@ -9158,17 +9158,17 @@
       </c>
       <c r="C295" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — archived job denied</t>
+          <t>CoC refresh — auditor denied</t>
         </is>
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh for an archived job</t>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh with auditor token</t>
         </is>
       </c>
       <c r="E295" s="4" t="inlineStr">
         <is>
-          <t>409, archived jobs can only return the last stored snapshot</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F295" s="4" t="n"/>
@@ -9177,59 +9177,59 @@
       <c r="I295" s="4" t="n"/>
     </row>
     <row r="296">
-      <c r="A296" s="2" t="inlineStr">
+      <c r="A296" s="4" t="inlineStr">
+        <is>
+          <t>TC-1212</t>
+        </is>
+      </c>
+      <c r="B296" s="4" t="inlineStr">
+        <is>
+          <t>12.12 Chain-of-Custody Handoff</t>
+        </is>
+      </c>
+      <c r="C296" s="4" t="inlineStr">
+        <is>
+          <t>CoC refresh — archived job denied</t>
+        </is>
+      </c>
+      <c r="D296" s="4" t="inlineStr">
+        <is>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh for an archived job</t>
+        </is>
+      </c>
+      <c r="E296" s="4" t="inlineStr">
+        <is>
+          <t>409, archived jobs can only return the last stored snapshot</t>
+        </is>
+      </c>
+      <c r="F296" s="4" t="n"/>
+      <c r="G296" s="4" t="n"/>
+      <c r="H296" s="4" t="n"/>
+      <c r="I296" s="4" t="n"/>
+    </row>
+    <row r="297">
+      <c r="A297" s="2" t="inlineStr">
         <is>
           <t>§12.14 Startup Reconciliation</t>
         </is>
       </c>
-      <c r="B296" s="2" t="inlineStr">
+      <c r="B297" s="2" t="inlineStr">
         <is>
           <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
-      <c r="C296" s="3" t="n"/>
-      <c r="D296" s="3" t="n"/>
-      <c r="E296" s="3" t="n"/>
-      <c r="F296" s="3" t="n"/>
-      <c r="G296" s="3" t="n"/>
-      <c r="H296" s="3" t="n"/>
-      <c r="I296" s="3" t="n"/>
-    </row>
-    <row r="297">
-      <c r="A297" s="4" t="inlineStr">
-        <is>
-          <t>TC-1401</t>
-        </is>
-      </c>
-      <c r="B297" s="4" t="inlineStr">
-        <is>
-          <t>12.14 Startup Reconciliation</t>
-        </is>
-      </c>
-      <c r="C297" s="4" t="inlineStr">
-        <is>
-          <t>Running job failed after restart</t>
-        </is>
-      </c>
-      <c r="D297" s="4" t="inlineStr">
-        <is>
-          <t>Create a job, start it, restart the service while RUNNING</t>
-        </is>
-      </c>
-      <c r="E297" s="4" t="inlineStr">
-        <is>
-          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
-        </is>
-      </c>
-      <c r="F297" s="4" t="n"/>
-      <c r="G297" s="4" t="n"/>
-      <c r="H297" s="4" t="n"/>
-      <c r="I297" s="4" t="n"/>
+      <c r="C297" s="3" t="n"/>
+      <c r="D297" s="3" t="n"/>
+      <c r="E297" s="3" t="n"/>
+      <c r="F297" s="3" t="n"/>
+      <c r="G297" s="3" t="n"/>
+      <c r="H297" s="3" t="n"/>
+      <c r="I297" s="3" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="4" t="inlineStr">
         <is>
-          <t>TC-1402</t>
+          <t>TC-1401</t>
         </is>
       </c>
       <c r="B298" s="4" t="inlineStr">
@@ -9239,17 +9239,17 @@
       </c>
       <c r="C298" s="4" t="inlineStr">
         <is>
-          <t>Verifying job failed after restart</t>
+          <t>Running job failed after restart</t>
         </is>
       </c>
       <c r="D298" s="4" t="inlineStr">
         <is>
-          <t>Start a job, let it reach VERIFYING, restart the service</t>
+          <t>Create a job, start it, restart the service while RUNNING</t>
         </is>
       </c>
       <c r="E298" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
+          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
         </is>
       </c>
       <c r="F298" s="4" t="n"/>
@@ -9260,7 +9260,7 @@
     <row r="299">
       <c r="A299" s="4" t="inlineStr">
         <is>
-          <t>TC-1403</t>
+          <t>TC-1402</t>
         </is>
       </c>
       <c r="B299" s="4" t="inlineStr">
@@ -9270,17 +9270,17 @@
       </c>
       <c r="C299" s="4" t="inlineStr">
         <is>
-          <t>Pending job not affected</t>
+          <t>Verifying job failed after restart</t>
         </is>
       </c>
       <c r="D299" s="4" t="inlineStr">
         <is>
-          <t>Create a job (PENDING), restart the service</t>
+          <t>Start a job, let it reach VERIFYING, restart the service</t>
         </is>
       </c>
       <c r="E299" s="4" t="inlineStr">
         <is>
-          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
+          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
         </is>
       </c>
       <c r="F299" s="4" t="n"/>
@@ -9291,7 +9291,7 @@
     <row r="300">
       <c r="A300" s="4" t="inlineStr">
         <is>
-          <t>TC-1404</t>
+          <t>TC-1403</t>
         </is>
       </c>
       <c r="B300" s="4" t="inlineStr">
@@ -9301,17 +9301,17 @@
       </c>
       <c r="C300" s="4" t="inlineStr">
         <is>
-          <t>Completed job not affected</t>
+          <t>Pending job not affected</t>
         </is>
       </c>
       <c r="D300" s="4" t="inlineStr">
         <is>
-          <t>Complete a job, restart the service</t>
+          <t>Create a job (PENDING), restart the service</t>
         </is>
       </c>
       <c r="E300" s="4" t="inlineStr">
         <is>
-          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
+          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
         </is>
       </c>
       <c r="F300" s="4" t="n"/>
@@ -9322,7 +9322,7 @@
     <row r="301">
       <c r="A301" s="4" t="inlineStr">
         <is>
-          <t>TC-1405</t>
+          <t>TC-1404</t>
         </is>
       </c>
       <c r="B301" s="4" t="inlineStr">
@@ -9332,17 +9332,17 @@
       </c>
       <c r="C301" s="4" t="inlineStr">
         <is>
-          <t>Stale mount corrected</t>
+          <t>Completed job not affected</t>
         </is>
       </c>
       <c r="D301" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
+          <t>Complete a job, restart the service</t>
         </is>
       </c>
       <c r="E301" s="4" t="inlineStr">
         <is>
-          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
+          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F301" s="4" t="n"/>
@@ -9353,7 +9353,7 @@
     <row r="302">
       <c r="A302" s="4" t="inlineStr">
         <is>
-          <t>TC-1406</t>
+          <t>TC-1405</t>
         </is>
       </c>
       <c r="B302" s="4" t="inlineStr">
@@ -9363,17 +9363,17 @@
       </c>
       <c r="C302" s="4" t="inlineStr">
         <is>
-          <t>Active mount preserved</t>
+          <t>Stale mount corrected</t>
         </is>
       </c>
       <c r="D302" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share (leave it mounted), restart the service</t>
+          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
         </is>
       </c>
       <c r="E302" s="4" t="inlineStr">
         <is>
-          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
+          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
         </is>
       </c>
       <c r="F302" s="4" t="n"/>
@@ -9384,7 +9384,7 @@
     <row r="303">
       <c r="A303" s="4" t="inlineStr">
         <is>
-          <t>TC-1407</t>
+          <t>TC-1406</t>
         </is>
       </c>
       <c r="B303" s="4" t="inlineStr">
@@ -9394,17 +9394,17 @@
       </c>
       <c r="C303" s="4" t="inlineStr">
         <is>
-          <t>USB drives re-discovered</t>
+          <t>Active mount preserved</t>
         </is>
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>Insert USB drives, restart the service</t>
+          <t>Add and mount a network share (leave it mounted), restart the service</t>
         </is>
       </c>
       <c r="E303" s="4" t="inlineStr">
         <is>
-          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
+          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F303" s="4" t="n"/>
@@ -9415,7 +9415,7 @@
     <row r="304">
       <c r="A304" s="4" t="inlineStr">
         <is>
-          <t>TC-1408</t>
+          <t>TC-1407</t>
         </is>
       </c>
       <c r="B304" s="4" t="inlineStr">
@@ -9425,17 +9425,17 @@
       </c>
       <c r="C304" s="4" t="inlineStr">
         <is>
-          <t>Idempotency</t>
+          <t>USB drives re-discovered</t>
         </is>
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>Restart the service twice without any state changes between restarts</t>
+          <t>Insert USB drives, restart the service</t>
         </is>
       </c>
       <c r="E304" s="4" t="inlineStr">
         <is>
-          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
+          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
         </is>
       </c>
       <c r="F304" s="4" t="n"/>
@@ -9446,7 +9446,7 @@
     <row r="305">
       <c r="A305" s="4" t="inlineStr">
         <is>
-          <t>TC-1409</t>
+          <t>TC-1408</t>
         </is>
       </c>
       <c r="B305" s="4" t="inlineStr">
@@ -9456,17 +9456,17 @@
       </c>
       <c r="C305" s="4" t="inlineStr">
         <is>
-          <t>Partial failure isolation</t>
+          <t>Idempotency</t>
         </is>
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
+          <t>Restart the service twice without any state changes between restarts</t>
         </is>
       </c>
       <c r="E305" s="4" t="inlineStr">
         <is>
-          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
+          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
         </is>
       </c>
       <c r="F305" s="4" t="n"/>
@@ -9477,7 +9477,7 @@
     <row r="306">
       <c r="A306" s="4" t="inlineStr">
         <is>
-          <t>TC-1410</t>
+          <t>TC-1409</t>
         </is>
       </c>
       <c r="B306" s="4" t="inlineStr">
@@ -9487,17 +9487,17 @@
       </c>
       <c r="C306" s="4" t="inlineStr">
         <is>
-          <t>Cross-process lock — only one worker reconciles</t>
+          <t>Partial failure isolation</t>
         </is>
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
+          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
         </is>
       </c>
       <c r="E306" s="4" t="inlineStr">
         <is>
-          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
+          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
         </is>
       </c>
       <c r="F306" s="4" t="n"/>
@@ -9508,7 +9508,7 @@
     <row r="307">
       <c r="A307" s="4" t="inlineStr">
         <is>
-          <t>TC-1411</t>
+          <t>TC-1410</t>
         </is>
       </c>
       <c r="B307" s="4" t="inlineStr">
@@ -9518,17 +9518,17 @@
       </c>
       <c r="C307" s="4" t="inlineStr">
         <is>
-          <t>Stale lock reclaim</t>
+          <t>Cross-process lock — only one worker reconciles</t>
         </is>
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
+          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
         </is>
       </c>
       <c r="E307" s="4" t="inlineStr">
         <is>
-          <t>Service reclaims the stale lock, reconciliation runs normally</t>
+          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
         </is>
       </c>
       <c r="F307" s="4" t="n"/>
@@ -9539,7 +9539,7 @@
     <row r="308">
       <c r="A308" s="4" t="inlineStr">
         <is>
-          <t>TC-1412</t>
+          <t>TC-1411</t>
         </is>
       </c>
       <c r="B308" s="4" t="inlineStr">
@@ -9549,17 +9549,17 @@
       </c>
       <c r="C308" s="4" t="inlineStr">
         <is>
-          <t>Lock released after failure</t>
+          <t>Stale lock reclaim</t>
         </is>
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
+          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
         </is>
       </c>
       <c r="E308" s="4" t="inlineStr">
         <is>
-          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
+          <t>Service reclaims the stale lock, reconciliation runs normally</t>
         </is>
       </c>
       <c r="F308" s="4" t="n"/>
@@ -9570,7 +9570,7 @@
     <row r="309">
       <c r="A309" s="4" t="inlineStr">
         <is>
-          <t>TC-1413</t>
+          <t>TC-1412</t>
         </is>
       </c>
       <c r="B309" s="4" t="inlineStr">
@@ -9580,17 +9580,17 @@
       </c>
       <c r="C309" s="4" t="inlineStr">
         <is>
-          <t>Jobs pass emits immediate startup result log</t>
+          <t>Lock released after failure</t>
         </is>
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>Create at least one RUNNING job, restart service, then inspect application logs around startup reconciliation</t>
+          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
         </is>
       </c>
       <c r="E309" s="4" t="inlineStr">
         <is>
-          <t>Logs include Startup reconciliation: checking jobs followed by an immediate Startup reconciliation: jobs result line with safe counts (jobs_checked, jobs_corrected) or safe failure classification</t>
+          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
         </is>
       </c>
       <c r="F309" s="4" t="n"/>
@@ -9601,7 +9601,7 @@
     <row r="310">
       <c r="A310" s="4" t="inlineStr">
         <is>
-          <t>TC-1414</t>
+          <t>TC-1413</t>
         </is>
       </c>
       <c r="B310" s="4" t="inlineStr">
@@ -9611,17 +9611,17 @@
       </c>
       <c r="C310" s="4" t="inlineStr">
         <is>
-          <t>Reconciled job persists restart-interruption failure reason</t>
+          <t>Jobs pass emits immediate startup result log</t>
         </is>
       </c>
       <c r="D310" s="4" t="inlineStr">
         <is>
-          <t>Create a RUNNING or VERIFYING job, restart service, then open Job Detail for that job</t>
+          <t>Create at least one RUNNING job, restart service, then inspect application logs around startup reconciliation</t>
         </is>
       </c>
       <c r="E310" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED and Job Detail shows a stable restart interruption reason (not the generic This job failed... fallback)</t>
+          <t>Logs include Startup reconciliation: checking jobs followed by an immediate Startup reconciliation: jobs result line with safe counts (jobs_checked, jobs_corrected) or safe failure classification</t>
         </is>
       </c>
       <c r="F310" s="4" t="n"/>
@@ -9632,7 +9632,7 @@
     <row r="311">
       <c r="A311" s="4" t="inlineStr">
         <is>
-          <t>TC-1415</t>
+          <t>TC-1414</t>
         </is>
       </c>
       <c r="B311" s="4" t="inlineStr">
@@ -9642,17 +9642,17 @@
       </c>
       <c r="C311" s="4" t="inlineStr">
         <is>
-          <t>Reconciled failed job shows correlated failure entry from audit fallback</t>
+          <t>Reconciled job persists restart-interruption failure reason</t>
         </is>
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>Restart with a RUNNING job, then inspect Job Detail when no matching file-log failure line is present</t>
+          <t>Create a RUNNING or VERIFYING job, restart service, then open Job Detail for that job</t>
         </is>
       </c>
       <c r="E311" s="4" t="inlineStr">
         <is>
-          <t>Job Detail still shows a related failure entry sourced from reconciliation evidence (JOB_RECONCILED) and the entry remains sanitized</t>
+          <t>Job status is FAILED and Job Detail shows a stable restart interruption reason (not the generic This job failed... fallback)</t>
         </is>
       </c>
       <c r="F311" s="4" t="n"/>
@@ -9663,7 +9663,7 @@
     <row r="312">
       <c r="A312" s="4" t="inlineStr">
         <is>
-          <t>TC-1416</t>
+          <t>TC-1415</t>
         </is>
       </c>
       <c r="B312" s="4" t="inlineStr">
@@ -9673,17 +9673,17 @@
       </c>
       <c r="C312" s="4" t="inlineStr">
         <is>
-          <t>Failed job API uses reconciliation audit fallback when file-log correlation is unavailable</t>
+          <t>Reconciled failed job shows correlated failure entry from audit fallback</t>
         </is>
       </c>
       <c r="D312" s="4" t="inlineStr">
         <is>
-          <t>In a test environment, disable file-log correlation (log_file unset), then request GET /jobs/{job_id} for a restart-reconciled failed job</t>
+          <t>Restart with a RUNNING job, then inspect Job Detail when no matching file-log failure line is present</t>
         </is>
       </c>
       <c r="E312" s="4" t="inlineStr">
         <is>
-          <t>Response remains 200 and includes the stable restart failure reason plus a sanitized failure_log_entry derived from audit evidence (JOB_RECONCILED)</t>
+          <t>Job Detail still shows a related failure entry sourced from reconciliation evidence (JOB_RECONCILED) and the entry remains sanitized</t>
         </is>
       </c>
       <c r="F312" s="4" t="n"/>
@@ -9694,7 +9694,7 @@
     <row r="313">
       <c r="A313" s="4" t="inlineStr">
         <is>
-          <t>TC-1417</t>
+          <t>TC-1416</t>
         </is>
       </c>
       <c r="B313" s="4" t="inlineStr">
@@ -9704,17 +9704,17 @@
       </c>
       <c r="C313" s="4" t="inlineStr">
         <is>
-          <t>Jobs pass failure path emits safe startup result classification</t>
+          <t>Failed job API uses reconciliation audit fallback when file-log correlation is unavailable</t>
         </is>
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>In a controlled test environment, force a jobs-pass reconciliation exception, then restart service and inspect startup logs</t>
+          <t>In a test environment, disable file-log correlation (log_file unset), then request GET /jobs/{job_id} for a restart-reconciled failed job</t>
         </is>
       </c>
       <c r="E313" s="4" t="inlineStr">
         <is>
-          <t>Logs still include Startup reconciliation: jobs result with status=failed and reason=job_reconciliation_failed, without raw provider errors or host paths</t>
+          <t>Response remains 200 and includes the stable restart failure reason plus a sanitized failure_log_entry derived from audit evidence (JOB_RECONCILED)</t>
         </is>
       </c>
       <c r="F313" s="4" t="n"/>
@@ -9725,7 +9725,7 @@
     <row r="314">
       <c r="A314" s="4" t="inlineStr">
         <is>
-          <t>TC-1418</t>
+          <t>TC-1417</t>
         </is>
       </c>
       <c r="B314" s="4" t="inlineStr">
@@ -9735,17 +9735,17 @@
       </c>
       <c r="C314" s="4" t="inlineStr">
         <is>
-          <t>Restart clears stale in-progress startup analysis when no valid cache remains</t>
+          <t>Jobs pass failure path emits safe startup result classification</t>
         </is>
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>Trigger manual Analyze for a PENDING job, restart ECUBE before the scan completes, then reopen Job Detail</t>
+          <t>In a controlled test environment, force a jobs-pass reconciliation exception, then restart service and inspect startup logs</t>
         </is>
       </c>
       <c r="E314" s="4" t="inlineStr">
         <is>
-          <t>Job is no longer stuck in ANALYZING, startup-analysis state returns to NOT_ANALYZED, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "analysis_interrupted_by_restart", and Analyze or Start is available again</t>
+          <t>Logs still include Startup reconciliation: jobs result with status=failed and reason=job_reconciliation_failed, without raw provider errors or host paths</t>
         </is>
       </c>
       <c r="F314" s="4" t="n"/>
@@ -9756,7 +9756,7 @@
     <row r="315">
       <c r="A315" s="4" t="inlineStr">
         <is>
-          <t>TC-1419</t>
+          <t>TC-1418</t>
         </is>
       </c>
       <c r="B315" s="4" t="inlineStr">
@@ -9766,17 +9766,17 @@
       </c>
       <c r="C315" s="4" t="inlineStr">
         <is>
-          <t>Restart restores READY when the interrupted startup-analysis cache is still current</t>
+          <t>Restart clears stale in-progress startup analysis when no valid cache remains</t>
         </is>
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>Trigger manual Analyze for a job with a stable source tree, restart ECUBE after the reusable snapshot has been persisted but before the manual analyze workflow fully completes, then reopen Job Detail</t>
+          <t>Trigger manual Analyze for a PENDING job, restart ECUBE before the scan completes, then reopen Job Detail</t>
         </is>
       </c>
       <c r="E315" s="4" t="inlineStr">
         <is>
-          <t>Job shows startup_analysis_status: READY, the previous file and byte totals are still available, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "valid_cache_restored_after_restart", and Start can proceed without forcing a fresh scan</t>
+          <t>Job is no longer stuck in ANALYZING, startup-analysis state returns to NOT_ANALYZED, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "analysis_interrupted_by_restart", and Analyze or Start is available again</t>
         </is>
       </c>
       <c r="F315" s="4" t="n"/>
@@ -9785,59 +9785,59 @@
       <c r="I315" s="4" t="n"/>
     </row>
     <row r="316">
-      <c r="A316" s="2" t="inlineStr">
+      <c r="A316" s="4" t="inlineStr">
+        <is>
+          <t>TC-1419</t>
+        </is>
+      </c>
+      <c r="B316" s="4" t="inlineStr">
+        <is>
+          <t>12.14 Startup Reconciliation</t>
+        </is>
+      </c>
+      <c r="C316" s="4" t="inlineStr">
+        <is>
+          <t>Restart restores READY when the interrupted startup-analysis cache is still current</t>
+        </is>
+      </c>
+      <c r="D316" s="4" t="inlineStr">
+        <is>
+          <t>Trigger manual Analyze for a job with a stable source tree, restart ECUBE after the reusable snapshot has been persisted but before the manual analyze workflow fully completes, then reopen Job Detail</t>
+        </is>
+      </c>
+      <c r="E316" s="4" t="inlineStr">
+        <is>
+          <t>Job shows startup_analysis_status: READY, the previous file and byte totals are still available, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "valid_cache_restored_after_restart", and Start can proceed without forcing a fresh scan</t>
+        </is>
+      </c>
+      <c r="F316" s="4" t="n"/>
+      <c r="G316" s="4" t="n"/>
+      <c r="H316" s="4" t="n"/>
+      <c r="I316" s="4" t="n"/>
+    </row>
+    <row r="317">
+      <c r="A317" s="2" t="inlineStr">
         <is>
           <t>§12.15 System Health</t>
         </is>
       </c>
-      <c r="B316" s="2" t="inlineStr">
+      <c r="B317" s="2" t="inlineStr">
         <is>
           <t>12.15 System Health</t>
         </is>
       </c>
-      <c r="C316" s="3" t="n"/>
-      <c r="D316" s="3" t="n"/>
-      <c r="E316" s="3" t="n"/>
-      <c r="F316" s="3" t="n"/>
-      <c r="G316" s="3" t="n"/>
-      <c r="H316" s="3" t="n"/>
-      <c r="I316" s="3" t="n"/>
-    </row>
-    <row r="317">
-      <c r="A317" s="4" t="inlineStr">
-        <is>
-          <t>TC-1501</t>
-        </is>
-      </c>
-      <c r="B317" s="4" t="inlineStr">
-        <is>
-          <t>12.15 System Health</t>
-        </is>
-      </c>
-      <c r="C317" s="4" t="inlineStr">
-        <is>
-          <t>Healthy response</t>
-        </is>
-      </c>
-      <c r="D317" s="4" t="inlineStr">
-        <is>
-          <t>GET /introspection/system-health with valid token</t>
-        </is>
-      </c>
-      <c r="E317" s="4" t="inlineStr">
-        <is>
-          <t>200, status: "ok", database: "connected"</t>
-        </is>
-      </c>
-      <c r="F317" s="4" t="n"/>
-      <c r="G317" s="4" t="n"/>
-      <c r="H317" s="4" t="n"/>
-      <c r="I317" s="4" t="n"/>
+      <c r="C317" s="3" t="n"/>
+      <c r="D317" s="3" t="n"/>
+      <c r="E317" s="3" t="n"/>
+      <c r="F317" s="3" t="n"/>
+      <c r="G317" s="3" t="n"/>
+      <c r="H317" s="3" t="n"/>
+      <c r="I317" s="3" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="4" t="inlineStr">
         <is>
-          <t>TC-1502</t>
+          <t>TC-1501</t>
         </is>
       </c>
       <c r="B318" s="4" t="inlineStr">
@@ -9847,17 +9847,17 @@
       </c>
       <c r="C318" s="4" t="inlineStr">
         <is>
-          <t>CPU metric present</t>
+          <t>Healthy response</t>
         </is>
       </c>
       <c r="D318" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>GET /introspection/system-health with valid token</t>
         </is>
       </c>
       <c r="E318" s="4" t="inlineStr">
         <is>
-          <t>cpu_percent is a number between 0 and 100</t>
+          <t>200, status: "ok", database: "connected"</t>
         </is>
       </c>
       <c r="F318" s="4" t="n"/>
@@ -9868,7 +9868,7 @@
     <row r="319">
       <c r="A319" s="4" t="inlineStr">
         <is>
-          <t>TC-1503</t>
+          <t>TC-1502</t>
         </is>
       </c>
       <c r="B319" s="4" t="inlineStr">
@@ -9878,7 +9878,7 @@
       </c>
       <c r="C319" s="4" t="inlineStr">
         <is>
-          <t>Memory metrics present</t>
+          <t>CPU metric present</t>
         </is>
       </c>
       <c r="D319" s="4" t="inlineStr">
@@ -9888,7 +9888,7 @@
       </c>
       <c r="E319" s="4" t="inlineStr">
         <is>
-          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
+          <t>cpu_percent is a number between 0 and 100</t>
         </is>
       </c>
       <c r="F319" s="4" t="n"/>
@@ -9899,7 +9899,7 @@
     <row r="320">
       <c r="A320" s="4" t="inlineStr">
         <is>
-          <t>TC-1504</t>
+          <t>TC-1503</t>
         </is>
       </c>
       <c r="B320" s="4" t="inlineStr">
@@ -9909,7 +9909,7 @@
       </c>
       <c r="C320" s="4" t="inlineStr">
         <is>
-          <t>Disk I/O metrics present</t>
+          <t>Memory metrics present</t>
         </is>
       </c>
       <c r="D320" s="4" t="inlineStr">
@@ -9919,7 +9919,7 @@
       </c>
       <c r="E320" s="4" t="inlineStr">
         <is>
-          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
+          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
         </is>
       </c>
       <c r="F320" s="4" t="n"/>
@@ -9930,7 +9930,7 @@
     <row r="321">
       <c r="A321" s="4" t="inlineStr">
         <is>
-          <t>TC-1505</t>
+          <t>TC-1504</t>
         </is>
       </c>
       <c r="B321" s="4" t="inlineStr">
@@ -9940,17 +9940,17 @@
       </c>
       <c r="C321" s="4" t="inlineStr">
         <is>
-          <t>Active jobs count</t>
+          <t>Disk I/O metrics present</t>
         </is>
       </c>
       <c r="D321" s="4" t="inlineStr">
         <is>
-          <t>Start an export job, call endpoint</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E321" s="4" t="inlineStr">
         <is>
-          <t>active_jobs ≥ 1</t>
+          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
         </is>
       </c>
       <c r="F321" s="4" t="n"/>
@@ -9961,7 +9961,7 @@
     <row r="322">
       <c r="A322" s="4" t="inlineStr">
         <is>
-          <t>TC-1506</t>
+          <t>TC-1505</t>
         </is>
       </c>
       <c r="B322" s="4" t="inlineStr">
@@ -9971,17 +9971,17 @@
       </c>
       <c r="C322" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size</t>
+          <t>Active jobs count</t>
         </is>
       </c>
       <c r="D322" s="4" t="inlineStr">
         <is>
-          <t>Create a PENDING job (created but not started), call endpoint</t>
+          <t>Start an export job, call endpoint</t>
         </is>
       </c>
       <c r="E322" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size ≥ 1</t>
+          <t>active_jobs ≥ 1</t>
         </is>
       </c>
       <c r="F322" s="4" t="n"/>
@@ -9992,7 +9992,7 @@
     <row r="323">
       <c r="A323" s="4" t="inlineStr">
         <is>
-          <t>TC-1507</t>
+          <t>TC-1506</t>
         </is>
       </c>
       <c r="B323" s="4" t="inlineStr">
@@ -10002,17 +10002,17 @@
       </c>
       <c r="C323" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size decrements</t>
+          <t>Worker queue size</t>
         </is>
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>Start the pending job, call endpoint again</t>
+          <t>Create a PENDING job (created but not started), call endpoint</t>
         </is>
       </c>
       <c r="E323" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
+          <t>worker_queue_size ≥ 1</t>
         </is>
       </c>
       <c r="F323" s="4" t="n"/>
@@ -10023,7 +10023,7 @@
     <row r="324">
       <c r="A324" s="4" t="inlineStr">
         <is>
-          <t>TC-1508</t>
+          <t>TC-1507</t>
         </is>
       </c>
       <c r="B324" s="4" t="inlineStr">
@@ -10033,17 +10033,17 @@
       </c>
       <c r="C324" s="4" t="inlineStr">
         <is>
-          <t>ECUBE process metrics present</t>
+          <t>Worker queue size decrements</t>
         </is>
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Start the pending job, call endpoint again</t>
         </is>
       </c>
       <c r="E324" s="4" t="inlineStr">
         <is>
-          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
+          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
         </is>
       </c>
       <c r="F324" s="4" t="n"/>
@@ -10054,7 +10054,7 @@
     <row r="325">
       <c r="A325" s="4" t="inlineStr">
         <is>
-          <t>TC-1509</t>
+          <t>TC-1508</t>
         </is>
       </c>
       <c r="B325" s="4" t="inlineStr">
@@ -10064,17 +10064,17 @@
       </c>
       <c r="C325" s="4" t="inlineStr">
         <is>
-          <t>Active copy-thread correlation</t>
+          <t>ECUBE process metrics present</t>
         </is>
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>Run an export job with active copy workers, call endpoint during the run</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E325" s="4" t="inlineStr">
         <is>
-          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
+          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
         </is>
       </c>
       <c r="F325" s="4" t="n"/>
@@ -10085,7 +10085,7 @@
     <row r="326">
       <c r="A326" s="4" t="inlineStr">
         <is>
-          <t>TC-1510</t>
+          <t>TC-1509</t>
         </is>
       </c>
       <c r="B326" s="4" t="inlineStr">
@@ -10095,17 +10095,17 @@
       </c>
       <c r="C326" s="4" t="inlineStr">
         <is>
-          <t>ECUBE process metrics degrade safely</t>
+          <t>Active copy-thread correlation</t>
         </is>
       </c>
       <c r="D326" s="4" t="inlineStr">
         <is>
-          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
+          <t>Run an export job with active copy workers, call endpoint during the run</t>
         </is>
       </c>
       <c r="E326" s="4" t="inlineStr">
         <is>
-          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
+          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
         </is>
       </c>
       <c r="F326" s="4" t="n"/>
@@ -10116,7 +10116,7 @@
     <row r="327">
       <c r="A327" s="4" t="inlineStr">
         <is>
-          <t>TC-1511</t>
+          <t>TC-1510</t>
         </is>
       </c>
       <c r="B327" s="4" t="inlineStr">
@@ -10126,17 +10126,17 @@
       </c>
       <c r="C327" s="4" t="inlineStr">
         <is>
-          <t>Degraded when DB down</t>
+          <t>ECUBE process metrics degrade safely</t>
         </is>
       </c>
       <c r="D327" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, call endpoint with valid token</t>
+          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
         </is>
       </c>
       <c r="E327" s="4" t="inlineStr">
         <is>
-          <t>200, status: "degraded", database: "error", database_error is non-null</t>
+          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
         </is>
       </c>
       <c r="F327" s="4" t="n"/>
@@ -10147,7 +10147,7 @@
     <row r="328">
       <c r="A328" s="4" t="inlineStr">
         <is>
-          <t>TC-1512</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B328" s="4" t="inlineStr">
@@ -10157,17 +10157,17 @@
       </c>
       <c r="C328" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated rejected</t>
+          <t>Degraded when DB down</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health without token</t>
+          <t>Stop PostgreSQL, call endpoint with valid token</t>
         </is>
       </c>
       <c r="E328" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>200, status: "degraded", database: "error", database_error is non-null</t>
         </is>
       </c>
       <c r="F328" s="4" t="n"/>
@@ -10178,7 +10178,7 @@
     <row r="329">
       <c r="A329" s="4" t="inlineStr">
         <is>
-          <t>TC-1513</t>
+          <t>TC-1512</t>
         </is>
       </c>
       <c r="B329" s="4" t="inlineStr">
@@ -10188,17 +10188,17 @@
       </c>
       <c r="C329" s="4" t="inlineStr">
         <is>
-          <t>Processor role allowed</t>
+          <t>Unauthenticated rejected</t>
         </is>
       </c>
       <c r="D329" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with processor token</t>
+          <t>GET /introspection/system-health without token</t>
         </is>
       </c>
       <c r="E329" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F329" s="4" t="n"/>
@@ -10207,59 +10207,59 @@
       <c r="I329" s="4" t="n"/>
     </row>
     <row r="330">
-      <c r="A330" s="2" t="inlineStr">
+      <c r="A330" s="4" t="inlineStr">
+        <is>
+          <t>TC-1513</t>
+        </is>
+      </c>
+      <c r="B330" s="4" t="inlineStr">
+        <is>
+          <t>12.15 System Health</t>
+        </is>
+      </c>
+      <c r="C330" s="4" t="inlineStr">
+        <is>
+          <t>Processor role allowed</t>
+        </is>
+      </c>
+      <c r="D330" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/system-health with processor token</t>
+        </is>
+      </c>
+      <c r="E330" s="4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F330" s="4" t="n"/>
+      <c r="G330" s="4" t="n"/>
+      <c r="H330" s="4" t="n"/>
+      <c r="I330" s="4" t="n"/>
+    </row>
+    <row r="331">
+      <c r="A331" s="2" t="inlineStr">
         <is>
           <t>§12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
-      <c r="B330" s="2" t="inlineStr">
+      <c r="B331" s="2" t="inlineStr">
         <is>
           <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
-      <c r="C330" s="3" t="n"/>
-      <c r="D330" s="3" t="n"/>
-      <c r="E330" s="3" t="n"/>
-      <c r="F330" s="3" t="n"/>
-      <c r="G330" s="3" t="n"/>
-      <c r="H330" s="3" t="n"/>
-      <c r="I330" s="3" t="n"/>
-    </row>
-    <row r="331">
-      <c r="A331" s="4" t="inlineStr">
-        <is>
-          <t>TC-1511</t>
-        </is>
-      </c>
-      <c r="B331" s="4" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C331" s="4" t="inlineStr">
-        <is>
-          <t>Liveness endpoint is public</t>
-        </is>
-      </c>
-      <c r="D331" s="4" t="inlineStr">
-        <is>
-          <t>GET /health/live without token</t>
-        </is>
-      </c>
-      <c r="E331" s="4" t="inlineStr">
-        <is>
-          <t>200, service reports live</t>
-        </is>
-      </c>
-      <c r="F331" s="4" t="n"/>
-      <c r="G331" s="4" t="n"/>
-      <c r="H331" s="4" t="n"/>
-      <c r="I331" s="4" t="n"/>
+      <c r="C331" s="3" t="n"/>
+      <c r="D331" s="3" t="n"/>
+      <c r="E331" s="3" t="n"/>
+      <c r="F331" s="3" t="n"/>
+      <c r="G331" s="3" t="n"/>
+      <c r="H331" s="3" t="n"/>
+      <c r="I331" s="3" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="4" t="inlineStr">
         <is>
-          <t>TC-1512</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B332" s="4" t="inlineStr">
@@ -10269,17 +10269,17 @@
       </c>
       <c r="C332" s="4" t="inlineStr">
         <is>
-          <t>Readiness endpoint is public</t>
+          <t>Liveness endpoint is public</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr">
         <is>
-          <t>GET /health/ready without token on a healthy system</t>
+          <t>GET /health/live without token</t>
         </is>
       </c>
       <c r="E332" s="4" t="inlineStr">
         <is>
-          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
+          <t>200, service reports live</t>
         </is>
       </c>
       <c r="F332" s="4" t="n"/>
@@ -10290,7 +10290,7 @@
     <row r="333">
       <c r="A333" s="4" t="inlineStr">
         <is>
-          <t>TC-1513</t>
+          <t>TC-1512</t>
         </is>
       </c>
       <c r="B333" s="4" t="inlineStr">
@@ -10300,17 +10300,17 @@
       </c>
       <c r="C333" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports missing database configuration</t>
+          <t>Readiness endpoint is public</t>
         </is>
       </c>
       <c r="D333" s="4" t="inlineStr">
         <is>
-          <t>Clear DB config or test before configuration, then GET /health/ready</t>
+          <t>GET /health/ready without token on a healthy system</t>
         </is>
       </c>
       <c r="E333" s="4" t="inlineStr">
         <is>
-          <t>503, status: "not_ready", reason indicates database is not configured</t>
+          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
         </is>
       </c>
       <c r="F333" s="4" t="n"/>
@@ -10321,7 +10321,7 @@
     <row r="334">
       <c r="A334" s="4" t="inlineStr">
         <is>
-          <t>TC-1514</t>
+          <t>TC-1513</t>
         </is>
       </c>
       <c r="B334" s="4" t="inlineStr">
@@ -10331,17 +10331,17 @@
       </c>
       <c r="C334" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports mount or provider problems</t>
+          <t>Readiness reports missing database configuration</t>
         </is>
       </c>
       <c r="D334" s="4" t="inlineStr">
         <is>
-          <t>Break a configured mount or provider, then GET /health/ready</t>
+          <t>Clear DB config or test before configuration, then GET /health/ready</t>
         </is>
       </c>
       <c r="E334" s="4" t="inlineStr">
         <is>
-          <t>503, response identifies the failing check without using the generic error schema</t>
+          <t>503, status: "not_ready", reason indicates database is not configured</t>
         </is>
       </c>
       <c r="F334" s="4" t="n"/>
@@ -10352,7 +10352,7 @@
     <row r="335">
       <c r="A335" s="4" t="inlineStr">
         <is>
-          <t>TC-1515</t>
+          <t>TC-1514</t>
         </is>
       </c>
       <c r="B335" s="4" t="inlineStr">
@@ -10362,17 +10362,17 @@
       </c>
       <c r="C335" s="4" t="inlineStr">
         <is>
-          <t>Version endpoint is public</t>
+          <t>Readiness reports mount or provider problems</t>
         </is>
       </c>
       <c r="D335" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/version without token</t>
+          <t>Break a configured mount or provider, then GET /health/ready</t>
         </is>
       </c>
       <c r="E335" s="4" t="inlineStr">
         <is>
-          <t>200, returns version/application metadata</t>
+          <t>503, response identifies the failing check without using the generic error schema</t>
         </is>
       </c>
       <c r="F335" s="4" t="n"/>
@@ -10383,7 +10383,7 @@
     <row r="336">
       <c r="A336" s="4" t="inlineStr">
         <is>
-          <t>TC-1516</t>
+          <t>TC-1515</t>
         </is>
       </c>
       <c r="B336" s="4" t="inlineStr">
@@ -10393,17 +10393,17 @@
       </c>
       <c r="C336" s="4" t="inlineStr">
         <is>
-          <t>Readiness remains separate from authenticated system health</t>
+          <t>Version endpoint is public</t>
         </is>
       </c>
       <c r="D336" s="4" t="inlineStr">
         <is>
-          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+          <t>GET /introspection/version without token</t>
         </is>
       </c>
       <c r="E336" s="4" t="inlineStr">
         <is>
-          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+          <t>200, returns version/application metadata</t>
         </is>
       </c>
       <c r="F336" s="4" t="n"/>
@@ -10412,32 +10412,63 @@
       <c r="I336" s="4" t="n"/>
     </row>
     <row r="337">
-      <c r="A337" s="2" t="inlineStr">
+      <c r="A337" s="4" t="inlineStr">
+        <is>
+          <t>TC-1516</t>
+        </is>
+      </c>
+      <c r="B337" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C337" s="4" t="inlineStr">
+        <is>
+          <t>Readiness remains separate from authenticated system health</t>
+        </is>
+      </c>
+      <c r="D337" s="4" t="inlineStr">
+        <is>
+          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+        </is>
+      </c>
+      <c r="E337" s="4" t="inlineStr">
+        <is>
+          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+        </is>
+      </c>
+      <c r="F337" s="4" t="n"/>
+      <c r="G337" s="4" t="n"/>
+      <c r="H337" s="4" t="n"/>
+      <c r="I337" s="4" t="n"/>
+    </row>
+    <row r="338">
+      <c r="A338" s="2" t="inlineStr">
         <is>
           <t>§12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="B337" s="2" t="inlineStr">
+      <c r="B338" s="2" t="inlineStr">
         <is>
           <t>12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="C337" s="3" t="n"/>
-      <c r="D337" s="3" t="n"/>
-      <c r="E337" s="3" t="n"/>
-      <c r="F337" s="3" t="n"/>
-      <c r="G337" s="3" t="n"/>
-      <c r="H337" s="3" t="n"/>
-      <c r="I337" s="3" t="n"/>
-    </row>
-    <row r="339">
-      <c r="A339" s="5" t="inlineStr">
+      <c r="C338" s="3" t="n"/>
+      <c r="D338" s="3" t="n"/>
+      <c r="E338" s="3" t="n"/>
+      <c r="F338" s="3" t="n"/>
+      <c r="G338" s="3" t="n"/>
+      <c r="H338" s="3" t="n"/>
+      <c r="I338" s="3" t="n"/>
+    </row>
+    <row r="340">
+      <c r="A340" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B339" s="5" t="n">
-        <v>309</v>
+      <c r="B340" s="5" t="n">
+        <v>310</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Require password confirmation before setup admin creation
Add a confirmation field to the setup wizard’s final admin step so first-run setup only completes when the operator enters matching passwords, preventing accidental lockout from mistyped credentials.

Cover the mismatch and success paths in setup wizard tests, and sync operator, QA, UI-use-case, architecture, and generated help documentation with the new validation flow.

Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I340"/>
+  <dimension ref="A1:I341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8400,7 +8400,7 @@
       </c>
       <c r="D270" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with valid username and password</t>
+          <t>Complete the setup wizard with matching admin password and confirmation values</t>
         </is>
       </c>
       <c r="E270" s="4" t="inlineStr">
@@ -8817,59 +8817,59 @@
       <c r="I283" s="4" t="n"/>
     </row>
     <row r="284">
-      <c r="A284" s="2" t="inlineStr">
+      <c r="A284" s="4" t="inlineStr">
+        <is>
+          <t>TC-1116</t>
+        </is>
+      </c>
+      <c r="B284" s="4" t="inlineStr">
+        <is>
+          <t>12.11 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C284" s="4" t="inlineStr">
+        <is>
+          <t>Setup password confirmation mismatch</t>
+        </is>
+      </c>
+      <c r="D284" s="4" t="inlineStr">
+        <is>
+          <t>In the final setup wizard step, enter different values in the admin password and confirmation fields</t>
+        </is>
+      </c>
+      <c r="E284" s="4" t="inlineStr">
+        <is>
+          <t>The wizard shows a password-mismatch validation message and does not submit setup until the two values match</t>
+        </is>
+      </c>
+      <c r="F284" s="4" t="n"/>
+      <c r="G284" s="4" t="n"/>
+      <c r="H284" s="4" t="n"/>
+      <c r="I284" s="4" t="n"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="inlineStr">
         <is>
           <t>§12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
-      <c r="B284" s="2" t="inlineStr">
+      <c r="B285" s="2" t="inlineStr">
         <is>
           <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
-      <c r="C284" s="3" t="n"/>
-      <c r="D284" s="3" t="n"/>
-      <c r="E284" s="3" t="n"/>
-      <c r="F284" s="3" t="n"/>
-      <c r="G284" s="3" t="n"/>
-      <c r="H284" s="3" t="n"/>
-      <c r="I284" s="3" t="n"/>
-    </row>
-    <row r="285">
-      <c r="A285" s="4" t="inlineStr">
-        <is>
-          <t>TC-1201</t>
-        </is>
-      </c>
-      <c r="B285" s="4" t="inlineStr">
-        <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
-        </is>
-      </c>
-      <c r="C285" s="4" t="inlineStr">
-        <is>
-          <t>Retrieve stored CoC snapshot — archived job</t>
-        </is>
-      </c>
-      <c r="D285" s="4" t="inlineStr">
-        <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for an archived job that already has a stored snapshot</t>
-        </is>
-      </c>
-      <c r="E285" s="4" t="inlineStr">
-        <is>
-          <t>200, response contains the stored snapshot and snapshot metadata</t>
-        </is>
-      </c>
-      <c r="F285" s="4" t="n"/>
-      <c r="G285" s="4" t="n"/>
-      <c r="H285" s="4" t="n"/>
-      <c r="I285" s="4" t="n"/>
+      <c r="C285" s="3" t="n"/>
+      <c r="D285" s="3" t="n"/>
+      <c r="E285" s="3" t="n"/>
+      <c r="F285" s="3" t="n"/>
+      <c r="G285" s="3" t="n"/>
+      <c r="H285" s="3" t="n"/>
+      <c r="I285" s="3" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="4" t="inlineStr">
         <is>
-          <t>TC-1202</t>
+          <t>TC-1201</t>
         </is>
       </c>
       <c r="B286" s="4" t="inlineStr">
@@ -8879,17 +8879,17 @@
       </c>
       <c r="C286" s="4" t="inlineStr">
         <is>
-          <t>Retrieve stored CoC snapshot — active job</t>
+          <t>Retrieve stored CoC snapshot — archived job</t>
         </is>
       </c>
       <c r="D286" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job that already has a stored snapshot</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for an archived job that already has a stored snapshot</t>
         </is>
       </c>
       <c r="E286" s="4" t="inlineStr">
         <is>
-          <t>200, response contains the stored snapshot and does not regenerate it</t>
+          <t>200, response contains the stored snapshot and snapshot metadata</t>
         </is>
       </c>
       <c r="F286" s="4" t="n"/>
@@ -8900,7 +8900,7 @@
     <row r="287">
       <c r="A287" s="4" t="inlineStr">
         <is>
-          <t>TC-1203</t>
+          <t>TC-1202</t>
         </is>
       </c>
       <c r="B287" s="4" t="inlineStr">
@@ -8910,17 +8910,17 @@
       </c>
       <c r="C287" s="4" t="inlineStr">
         <is>
-          <t>CoC read — missing stored snapshot</t>
+          <t>Retrieve stored CoC snapshot — active job</t>
         </is>
       </c>
       <c r="D287" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job with no stored snapshot yet</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job that already has a stored snapshot</t>
         </is>
       </c>
       <c r="E287" s="4" t="inlineStr">
         <is>
-          <t>404, message explains that the report must be refreshed first</t>
+          <t>200, response contains the stored snapshot and does not regenerate it</t>
         </is>
       </c>
       <c r="F287" s="4" t="n"/>
@@ -8931,7 +8931,7 @@
     <row r="288">
       <c r="A288" s="4" t="inlineStr">
         <is>
-          <t>TC-1204</t>
+          <t>TC-1203</t>
         </is>
       </c>
       <c r="B288" s="4" t="inlineStr">
@@ -8941,17 +8941,17 @@
       </c>
       <c r="C288" s="4" t="inlineStr">
         <is>
-          <t>CoC read — processor denied</t>
+          <t>CoC read — missing stored snapshot</t>
         </is>
       </c>
       <c r="D288" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody with processor token</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job with no stored snapshot yet</t>
         </is>
       </c>
       <c r="E288" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>404, message explains that the report must be refreshed first</t>
         </is>
       </c>
       <c r="F288" s="4" t="n"/>
@@ -8962,7 +8962,7 @@
     <row r="289">
       <c r="A289" s="4" t="inlineStr">
         <is>
-          <t>TC-1205</t>
+          <t>TC-1204</t>
         </is>
       </c>
       <c r="B289" s="4" t="inlineStr">
@@ -8972,17 +8972,17 @@
       </c>
       <c r="C289" s="4" t="inlineStr">
         <is>
-          <t>CoC read — unauthenticated denied</t>
+          <t>CoC read — processor denied</t>
         </is>
       </c>
       <c r="D289" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody without token</t>
+          <t>GET /jobs/{job_id}/chain-of-custody with processor token</t>
         </is>
       </c>
       <c r="E289" s="4" t="inlineStr">
         <is>
-          <t>401, UNAUTHORIZED</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F289" s="4" t="n"/>
@@ -8993,7 +8993,7 @@
     <row r="290">
       <c r="A290" s="4" t="inlineStr">
         <is>
-          <t>TC-1206</t>
+          <t>TC-1205</t>
         </is>
       </c>
       <c r="B290" s="4" t="inlineStr">
@@ -9003,17 +9003,17 @@
       </c>
       <c r="C290" s="4" t="inlineStr">
         <is>
-          <t>CoC snapshot fields</t>
+          <t>CoC read — unauthenticated denied</t>
         </is>
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>Inspect any stored-snapshot response</t>
+          <t>GET /jobs/{job_id}/chain-of-custody without token</t>
         </is>
       </c>
       <c r="E290" s="4" t="inlineStr">
         <is>
-          <t>snapshot_stored_at, snapshot_updated_at, snapshot_stored_by, reports[], and manifest/custody fields are present</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F290" s="4" t="n"/>
@@ -9024,7 +9024,7 @@
     <row r="291">
       <c r="A291" s="4" t="inlineStr">
         <is>
-          <t>TC-1207</t>
+          <t>TC-1206</t>
         </is>
       </c>
       <c r="B291" s="4" t="inlineStr">
@@ -9034,17 +9034,17 @@
       </c>
       <c r="C291" s="4" t="inlineStr">
         <is>
-          <t>CoC events include lifecycle</t>
+          <t>CoC snapshot fields</t>
         </is>
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>Inspect chain_of_custody_events in a stored report for a completed job</t>
+          <t>Inspect any stored-snapshot response</t>
         </is>
       </c>
       <c r="E291" s="4" t="inlineStr">
         <is>
-          <t>Events include DRIVE_INITIALIZED, JOB_CREATED, JOB_STARTED, JOB_COMPLETED, DRIVE_EJECT_PREPARED, and COC_HANDOFF_CONFIRMED when applicable</t>
+          <t>snapshot_stored_at, snapshot_updated_at, snapshot_stored_by, reports[], and manifest/custody fields are present</t>
         </is>
       </c>
       <c r="F291" s="4" t="n"/>
@@ -9055,7 +9055,7 @@
     <row r="292">
       <c r="A292" s="4" t="inlineStr">
         <is>
-          <t>TC-1208</t>
+          <t>TC-1207</t>
         </is>
       </c>
       <c r="B292" s="4" t="inlineStr">
@@ -9065,17 +9065,17 @@
       </c>
       <c r="C292" s="4" t="inlineStr">
         <is>
-          <t>CoC manifest summary</t>
+          <t>CoC events include lifecycle</t>
         </is>
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>Inspect manifest_summary in the stored report</t>
+          <t>Inspect chain_of_custody_events in a stored report for a completed job</t>
         </is>
       </c>
       <c r="E292" s="4" t="inlineStr">
         <is>
-          <t>Array of objects with job_id, evidence_number, processor_notes, total_files, total_bytes, and manifest_count</t>
+          <t>Events include DRIVE_INITIALIZED, JOB_CREATED, JOB_STARTED, JOB_COMPLETED, DRIVE_EJECT_PREPARED, and COC_HANDOFF_CONFIRMED when applicable</t>
         </is>
       </c>
       <c r="F292" s="4" t="n"/>
@@ -9086,7 +9086,7 @@
     <row r="293">
       <c r="A293" s="4" t="inlineStr">
         <is>
-          <t>TC-1209</t>
+          <t>TC-1208</t>
         </is>
       </c>
       <c r="B293" s="4" t="inlineStr">
@@ -9096,17 +9096,17 @@
       </c>
       <c r="C293" s="4" t="inlineStr">
         <is>
-          <t>CoC — delivery_time absence (no handoff)</t>
+          <t>CoC manifest summary</t>
         </is>
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>Complete a job and store a snapshot before handoff</t>
+          <t>Inspect manifest_summary in the stored report</t>
         </is>
       </c>
       <c r="E293" s="4" t="inlineStr">
         <is>
-          <t>chain_of_custody_events do not contain COC_HANDOFF_CONFIRMED; custody_complete is false</t>
+          <t>Array of objects with job_id, evidence_number, processor_notes, total_files, total_bytes, and manifest_count</t>
         </is>
       </c>
       <c r="F293" s="4" t="n"/>
@@ -9117,7 +9117,7 @@
     <row r="294">
       <c r="A294" s="4" t="inlineStr">
         <is>
-          <t>TC-1210</t>
+          <t>TC-1209</t>
         </is>
       </c>
       <c r="B294" s="4" t="inlineStr">
@@ -9127,17 +9127,17 @@
       </c>
       <c r="C294" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — valid</t>
+          <t>CoC — delivery_time absence (no handoff)</t>
         </is>
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh with admin or manager token for a non-archived job with assignments</t>
+          <t>Complete a job and store a snapshot before handoff</t>
         </is>
       </c>
       <c r="E294" s="4" t="inlineStr">
         <is>
-          <t>200, response contains the refreshed stored snapshot and updated snapshot metadata</t>
+          <t>chain_of_custody_events do not contain COC_HANDOFF_CONFIRMED; custody_complete is false</t>
         </is>
       </c>
       <c r="F294" s="4" t="n"/>
@@ -9148,7 +9148,7 @@
     <row r="295">
       <c r="A295" s="4" t="inlineStr">
         <is>
-          <t>TC-1211</t>
+          <t>TC-1210</t>
         </is>
       </c>
       <c r="B295" s="4" t="inlineStr">
@@ -9158,17 +9158,17 @@
       </c>
       <c r="C295" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — auditor denied</t>
+          <t>CoC refresh — valid</t>
         </is>
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh with auditor token</t>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh with admin or manager token for a non-archived job with assignments</t>
         </is>
       </c>
       <c r="E295" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>200, response contains the refreshed stored snapshot and updated snapshot metadata</t>
         </is>
       </c>
       <c r="F295" s="4" t="n"/>
@@ -9179,7 +9179,7 @@
     <row r="296">
       <c r="A296" s="4" t="inlineStr">
         <is>
-          <t>TC-1212</t>
+          <t>TC-1211</t>
         </is>
       </c>
       <c r="B296" s="4" t="inlineStr">
@@ -9189,17 +9189,17 @@
       </c>
       <c r="C296" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — archived job denied</t>
+          <t>CoC refresh — auditor denied</t>
         </is>
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh for an archived job</t>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh with auditor token</t>
         </is>
       </c>
       <c r="E296" s="4" t="inlineStr">
         <is>
-          <t>409, archived jobs can only return the last stored snapshot</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F296" s="4" t="n"/>
@@ -9208,59 +9208,59 @@
       <c r="I296" s="4" t="n"/>
     </row>
     <row r="297">
-      <c r="A297" s="2" t="inlineStr">
+      <c r="A297" s="4" t="inlineStr">
+        <is>
+          <t>TC-1212</t>
+        </is>
+      </c>
+      <c r="B297" s="4" t="inlineStr">
+        <is>
+          <t>12.12 Chain-of-Custody Handoff</t>
+        </is>
+      </c>
+      <c r="C297" s="4" t="inlineStr">
+        <is>
+          <t>CoC refresh — archived job denied</t>
+        </is>
+      </c>
+      <c r="D297" s="4" t="inlineStr">
+        <is>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh for an archived job</t>
+        </is>
+      </c>
+      <c r="E297" s="4" t="inlineStr">
+        <is>
+          <t>409, archived jobs can only return the last stored snapshot</t>
+        </is>
+      </c>
+      <c r="F297" s="4" t="n"/>
+      <c r="G297" s="4" t="n"/>
+      <c r="H297" s="4" t="n"/>
+      <c r="I297" s="4" t="n"/>
+    </row>
+    <row r="298">
+      <c r="A298" s="2" t="inlineStr">
         <is>
           <t>§12.14 Startup Reconciliation</t>
         </is>
       </c>
-      <c r="B297" s="2" t="inlineStr">
+      <c r="B298" s="2" t="inlineStr">
         <is>
           <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
-      <c r="C297" s="3" t="n"/>
-      <c r="D297" s="3" t="n"/>
-      <c r="E297" s="3" t="n"/>
-      <c r="F297" s="3" t="n"/>
-      <c r="G297" s="3" t="n"/>
-      <c r="H297" s="3" t="n"/>
-      <c r="I297" s="3" t="n"/>
-    </row>
-    <row r="298">
-      <c r="A298" s="4" t="inlineStr">
-        <is>
-          <t>TC-1401</t>
-        </is>
-      </c>
-      <c r="B298" s="4" t="inlineStr">
-        <is>
-          <t>12.14 Startup Reconciliation</t>
-        </is>
-      </c>
-      <c r="C298" s="4" t="inlineStr">
-        <is>
-          <t>Running job failed after restart</t>
-        </is>
-      </c>
-      <c r="D298" s="4" t="inlineStr">
-        <is>
-          <t>Create a job, start it, restart the service while RUNNING</t>
-        </is>
-      </c>
-      <c r="E298" s="4" t="inlineStr">
-        <is>
-          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
-        </is>
-      </c>
-      <c r="F298" s="4" t="n"/>
-      <c r="G298" s="4" t="n"/>
-      <c r="H298" s="4" t="n"/>
-      <c r="I298" s="4" t="n"/>
+      <c r="C298" s="3" t="n"/>
+      <c r="D298" s="3" t="n"/>
+      <c r="E298" s="3" t="n"/>
+      <c r="F298" s="3" t="n"/>
+      <c r="G298" s="3" t="n"/>
+      <c r="H298" s="3" t="n"/>
+      <c r="I298" s="3" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="4" t="inlineStr">
         <is>
-          <t>TC-1402</t>
+          <t>TC-1401</t>
         </is>
       </c>
       <c r="B299" s="4" t="inlineStr">
@@ -9270,17 +9270,17 @@
       </c>
       <c r="C299" s="4" t="inlineStr">
         <is>
-          <t>Verifying job failed after restart</t>
+          <t>Running job failed after restart</t>
         </is>
       </c>
       <c r="D299" s="4" t="inlineStr">
         <is>
-          <t>Start a job, let it reach VERIFYING, restart the service</t>
+          <t>Create a job, start it, restart the service while RUNNING</t>
         </is>
       </c>
       <c r="E299" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
+          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
         </is>
       </c>
       <c r="F299" s="4" t="n"/>
@@ -9291,7 +9291,7 @@
     <row r="300">
       <c r="A300" s="4" t="inlineStr">
         <is>
-          <t>TC-1403</t>
+          <t>TC-1402</t>
         </is>
       </c>
       <c r="B300" s="4" t="inlineStr">
@@ -9301,17 +9301,17 @@
       </c>
       <c r="C300" s="4" t="inlineStr">
         <is>
-          <t>Pending job not affected</t>
+          <t>Verifying job failed after restart</t>
         </is>
       </c>
       <c r="D300" s="4" t="inlineStr">
         <is>
-          <t>Create a job (PENDING), restart the service</t>
+          <t>Start a job, let it reach VERIFYING, restart the service</t>
         </is>
       </c>
       <c r="E300" s="4" t="inlineStr">
         <is>
-          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
+          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
         </is>
       </c>
       <c r="F300" s="4" t="n"/>
@@ -9322,7 +9322,7 @@
     <row r="301">
       <c r="A301" s="4" t="inlineStr">
         <is>
-          <t>TC-1404</t>
+          <t>TC-1403</t>
         </is>
       </c>
       <c r="B301" s="4" t="inlineStr">
@@ -9332,17 +9332,17 @@
       </c>
       <c r="C301" s="4" t="inlineStr">
         <is>
-          <t>Completed job not affected</t>
+          <t>Pending job not affected</t>
         </is>
       </c>
       <c r="D301" s="4" t="inlineStr">
         <is>
-          <t>Complete a job, restart the service</t>
+          <t>Create a job (PENDING), restart the service</t>
         </is>
       </c>
       <c r="E301" s="4" t="inlineStr">
         <is>
-          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
+          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
         </is>
       </c>
       <c r="F301" s="4" t="n"/>
@@ -9353,7 +9353,7 @@
     <row r="302">
       <c r="A302" s="4" t="inlineStr">
         <is>
-          <t>TC-1405</t>
+          <t>TC-1404</t>
         </is>
       </c>
       <c r="B302" s="4" t="inlineStr">
@@ -9363,17 +9363,17 @@
       </c>
       <c r="C302" s="4" t="inlineStr">
         <is>
-          <t>Stale mount corrected</t>
+          <t>Completed job not affected</t>
         </is>
       </c>
       <c r="D302" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
+          <t>Complete a job, restart the service</t>
         </is>
       </c>
       <c r="E302" s="4" t="inlineStr">
         <is>
-          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
+          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F302" s="4" t="n"/>
@@ -9384,7 +9384,7 @@
     <row r="303">
       <c r="A303" s="4" t="inlineStr">
         <is>
-          <t>TC-1406</t>
+          <t>TC-1405</t>
         </is>
       </c>
       <c r="B303" s="4" t="inlineStr">
@@ -9394,17 +9394,17 @@
       </c>
       <c r="C303" s="4" t="inlineStr">
         <is>
-          <t>Active mount preserved</t>
+          <t>Stale mount corrected</t>
         </is>
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share (leave it mounted), restart the service</t>
+          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
         </is>
       </c>
       <c r="E303" s="4" t="inlineStr">
         <is>
-          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
+          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
         </is>
       </c>
       <c r="F303" s="4" t="n"/>
@@ -9415,7 +9415,7 @@
     <row r="304">
       <c r="A304" s="4" t="inlineStr">
         <is>
-          <t>TC-1407</t>
+          <t>TC-1406</t>
         </is>
       </c>
       <c r="B304" s="4" t="inlineStr">
@@ -9425,17 +9425,17 @@
       </c>
       <c r="C304" s="4" t="inlineStr">
         <is>
-          <t>USB drives re-discovered</t>
+          <t>Active mount preserved</t>
         </is>
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>Insert USB drives, restart the service</t>
+          <t>Add and mount a network share (leave it mounted), restart the service</t>
         </is>
       </c>
       <c r="E304" s="4" t="inlineStr">
         <is>
-          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
+          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F304" s="4" t="n"/>
@@ -9446,7 +9446,7 @@
     <row r="305">
       <c r="A305" s="4" t="inlineStr">
         <is>
-          <t>TC-1408</t>
+          <t>TC-1407</t>
         </is>
       </c>
       <c r="B305" s="4" t="inlineStr">
@@ -9456,17 +9456,17 @@
       </c>
       <c r="C305" s="4" t="inlineStr">
         <is>
-          <t>Idempotency</t>
+          <t>USB drives re-discovered</t>
         </is>
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>Restart the service twice without any state changes between restarts</t>
+          <t>Insert USB drives, restart the service</t>
         </is>
       </c>
       <c r="E305" s="4" t="inlineStr">
         <is>
-          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
+          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
         </is>
       </c>
       <c r="F305" s="4" t="n"/>
@@ -9477,7 +9477,7 @@
     <row r="306">
       <c r="A306" s="4" t="inlineStr">
         <is>
-          <t>TC-1409</t>
+          <t>TC-1408</t>
         </is>
       </c>
       <c r="B306" s="4" t="inlineStr">
@@ -9487,17 +9487,17 @@
       </c>
       <c r="C306" s="4" t="inlineStr">
         <is>
-          <t>Partial failure isolation</t>
+          <t>Idempotency</t>
         </is>
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
+          <t>Restart the service twice without any state changes between restarts</t>
         </is>
       </c>
       <c r="E306" s="4" t="inlineStr">
         <is>
-          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
+          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
         </is>
       </c>
       <c r="F306" s="4" t="n"/>
@@ -9508,7 +9508,7 @@
     <row r="307">
       <c r="A307" s="4" t="inlineStr">
         <is>
-          <t>TC-1410</t>
+          <t>TC-1409</t>
         </is>
       </c>
       <c r="B307" s="4" t="inlineStr">
@@ -9518,17 +9518,17 @@
       </c>
       <c r="C307" s="4" t="inlineStr">
         <is>
-          <t>Cross-process lock — only one worker reconciles</t>
+          <t>Partial failure isolation</t>
         </is>
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
+          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
         </is>
       </c>
       <c r="E307" s="4" t="inlineStr">
         <is>
-          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
+          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
         </is>
       </c>
       <c r="F307" s="4" t="n"/>
@@ -9539,7 +9539,7 @@
     <row r="308">
       <c r="A308" s="4" t="inlineStr">
         <is>
-          <t>TC-1411</t>
+          <t>TC-1410</t>
         </is>
       </c>
       <c r="B308" s="4" t="inlineStr">
@@ -9549,17 +9549,17 @@
       </c>
       <c r="C308" s="4" t="inlineStr">
         <is>
-          <t>Stale lock reclaim</t>
+          <t>Cross-process lock — only one worker reconciles</t>
         </is>
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
+          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
         </is>
       </c>
       <c r="E308" s="4" t="inlineStr">
         <is>
-          <t>Service reclaims the stale lock, reconciliation runs normally</t>
+          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
         </is>
       </c>
       <c r="F308" s="4" t="n"/>
@@ -9570,7 +9570,7 @@
     <row r="309">
       <c r="A309" s="4" t="inlineStr">
         <is>
-          <t>TC-1412</t>
+          <t>TC-1411</t>
         </is>
       </c>
       <c r="B309" s="4" t="inlineStr">
@@ -9580,17 +9580,17 @@
       </c>
       <c r="C309" s="4" t="inlineStr">
         <is>
-          <t>Lock released after failure</t>
+          <t>Stale lock reclaim</t>
         </is>
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
+          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
         </is>
       </c>
       <c r="E309" s="4" t="inlineStr">
         <is>
-          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
+          <t>Service reclaims the stale lock, reconciliation runs normally</t>
         </is>
       </c>
       <c r="F309" s="4" t="n"/>
@@ -9601,7 +9601,7 @@
     <row r="310">
       <c r="A310" s="4" t="inlineStr">
         <is>
-          <t>TC-1413</t>
+          <t>TC-1412</t>
         </is>
       </c>
       <c r="B310" s="4" t="inlineStr">
@@ -9611,17 +9611,17 @@
       </c>
       <c r="C310" s="4" t="inlineStr">
         <is>
-          <t>Jobs pass emits immediate startup result log</t>
+          <t>Lock released after failure</t>
         </is>
       </c>
       <c r="D310" s="4" t="inlineStr">
         <is>
-          <t>Create at least one RUNNING job, restart service, then inspect application logs around startup reconciliation</t>
+          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
         </is>
       </c>
       <c r="E310" s="4" t="inlineStr">
         <is>
-          <t>Logs include Startup reconciliation: checking jobs followed by an immediate Startup reconciliation: jobs result line with safe counts (jobs_checked, jobs_corrected) or safe failure classification</t>
+          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
         </is>
       </c>
       <c r="F310" s="4" t="n"/>
@@ -9632,7 +9632,7 @@
     <row r="311">
       <c r="A311" s="4" t="inlineStr">
         <is>
-          <t>TC-1414</t>
+          <t>TC-1413</t>
         </is>
       </c>
       <c r="B311" s="4" t="inlineStr">
@@ -9642,17 +9642,17 @@
       </c>
       <c r="C311" s="4" t="inlineStr">
         <is>
-          <t>Reconciled job persists restart-interruption failure reason</t>
+          <t>Jobs pass emits immediate startup result log</t>
         </is>
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>Create a RUNNING or VERIFYING job, restart service, then open Job Detail for that job</t>
+          <t>Create at least one RUNNING job, restart service, then inspect application logs around startup reconciliation</t>
         </is>
       </c>
       <c r="E311" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED and Job Detail shows a stable restart interruption reason (not the generic This job failed... fallback)</t>
+          <t>Logs include Startup reconciliation: checking jobs followed by an immediate Startup reconciliation: jobs result line with safe counts (jobs_checked, jobs_corrected) or safe failure classification</t>
         </is>
       </c>
       <c r="F311" s="4" t="n"/>
@@ -9663,7 +9663,7 @@
     <row r="312">
       <c r="A312" s="4" t="inlineStr">
         <is>
-          <t>TC-1415</t>
+          <t>TC-1414</t>
         </is>
       </c>
       <c r="B312" s="4" t="inlineStr">
@@ -9673,17 +9673,17 @@
       </c>
       <c r="C312" s="4" t="inlineStr">
         <is>
-          <t>Reconciled failed job shows correlated failure entry from audit fallback</t>
+          <t>Reconciled job persists restart-interruption failure reason</t>
         </is>
       </c>
       <c r="D312" s="4" t="inlineStr">
         <is>
-          <t>Restart with a RUNNING job, then inspect Job Detail when no matching file-log failure line is present</t>
+          <t>Create a RUNNING or VERIFYING job, restart service, then open Job Detail for that job</t>
         </is>
       </c>
       <c r="E312" s="4" t="inlineStr">
         <is>
-          <t>Job Detail still shows a related failure entry sourced from reconciliation evidence (JOB_RECONCILED) and the entry remains sanitized</t>
+          <t>Job status is FAILED and Job Detail shows a stable restart interruption reason (not the generic This job failed... fallback)</t>
         </is>
       </c>
       <c r="F312" s="4" t="n"/>
@@ -9694,7 +9694,7 @@
     <row r="313">
       <c r="A313" s="4" t="inlineStr">
         <is>
-          <t>TC-1416</t>
+          <t>TC-1415</t>
         </is>
       </c>
       <c r="B313" s="4" t="inlineStr">
@@ -9704,17 +9704,17 @@
       </c>
       <c r="C313" s="4" t="inlineStr">
         <is>
-          <t>Failed job API uses reconciliation audit fallback when file-log correlation is unavailable</t>
+          <t>Reconciled failed job shows correlated failure entry from audit fallback</t>
         </is>
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>In a test environment, disable file-log correlation (log_file unset), then request GET /jobs/{job_id} for a restart-reconciled failed job</t>
+          <t>Restart with a RUNNING job, then inspect Job Detail when no matching file-log failure line is present</t>
         </is>
       </c>
       <c r="E313" s="4" t="inlineStr">
         <is>
-          <t>Response remains 200 and includes the stable restart failure reason plus a sanitized failure_log_entry derived from audit evidence (JOB_RECONCILED)</t>
+          <t>Job Detail still shows a related failure entry sourced from reconciliation evidence (JOB_RECONCILED) and the entry remains sanitized</t>
         </is>
       </c>
       <c r="F313" s="4" t="n"/>
@@ -9725,7 +9725,7 @@
     <row r="314">
       <c r="A314" s="4" t="inlineStr">
         <is>
-          <t>TC-1417</t>
+          <t>TC-1416</t>
         </is>
       </c>
       <c r="B314" s="4" t="inlineStr">
@@ -9735,17 +9735,17 @@
       </c>
       <c r="C314" s="4" t="inlineStr">
         <is>
-          <t>Jobs pass failure path emits safe startup result classification</t>
+          <t>Failed job API uses reconciliation audit fallback when file-log correlation is unavailable</t>
         </is>
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>In a controlled test environment, force a jobs-pass reconciliation exception, then restart service and inspect startup logs</t>
+          <t>In a test environment, disable file-log correlation (log_file unset), then request GET /jobs/{job_id} for a restart-reconciled failed job</t>
         </is>
       </c>
       <c r="E314" s="4" t="inlineStr">
         <is>
-          <t>Logs still include Startup reconciliation: jobs result with status=failed and reason=job_reconciliation_failed, without raw provider errors or host paths</t>
+          <t>Response remains 200 and includes the stable restart failure reason plus a sanitized failure_log_entry derived from audit evidence (JOB_RECONCILED)</t>
         </is>
       </c>
       <c r="F314" s="4" t="n"/>
@@ -9756,7 +9756,7 @@
     <row r="315">
       <c r="A315" s="4" t="inlineStr">
         <is>
-          <t>TC-1418</t>
+          <t>TC-1417</t>
         </is>
       </c>
       <c r="B315" s="4" t="inlineStr">
@@ -9766,17 +9766,17 @@
       </c>
       <c r="C315" s="4" t="inlineStr">
         <is>
-          <t>Restart clears stale in-progress startup analysis when no valid cache remains</t>
+          <t>Jobs pass failure path emits safe startup result classification</t>
         </is>
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>Trigger manual Analyze for a PENDING job, restart ECUBE before the scan completes, then reopen Job Detail</t>
+          <t>In a controlled test environment, force a jobs-pass reconciliation exception, then restart service and inspect startup logs</t>
         </is>
       </c>
       <c r="E315" s="4" t="inlineStr">
         <is>
-          <t>Job is no longer stuck in ANALYZING, startup-analysis state returns to NOT_ANALYZED, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "analysis_interrupted_by_restart", and Analyze or Start is available again</t>
+          <t>Logs still include Startup reconciliation: jobs result with status=failed and reason=job_reconciliation_failed, without raw provider errors or host paths</t>
         </is>
       </c>
       <c r="F315" s="4" t="n"/>
@@ -9787,7 +9787,7 @@
     <row r="316">
       <c r="A316" s="4" t="inlineStr">
         <is>
-          <t>TC-1419</t>
+          <t>TC-1418</t>
         </is>
       </c>
       <c r="B316" s="4" t="inlineStr">
@@ -9797,17 +9797,17 @@
       </c>
       <c r="C316" s="4" t="inlineStr">
         <is>
-          <t>Restart restores READY when the interrupted startup-analysis cache is still current</t>
+          <t>Restart clears stale in-progress startup analysis when no valid cache remains</t>
         </is>
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>Trigger manual Analyze for a job with a stable source tree, restart ECUBE after the reusable snapshot has been persisted but before the manual analyze workflow fully completes, then reopen Job Detail</t>
+          <t>Trigger manual Analyze for a PENDING job, restart ECUBE before the scan completes, then reopen Job Detail</t>
         </is>
       </c>
       <c r="E316" s="4" t="inlineStr">
         <is>
-          <t>Job shows startup_analysis_status: READY, the previous file and byte totals are still available, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "valid_cache_restored_after_restart", and Start can proceed without forcing a fresh scan</t>
+          <t>Job is no longer stuck in ANALYZING, startup-analysis state returns to NOT_ANALYZED, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "analysis_interrupted_by_restart", and Analyze or Start is available again</t>
         </is>
       </c>
       <c r="F316" s="4" t="n"/>
@@ -9816,59 +9816,59 @@
       <c r="I316" s="4" t="n"/>
     </row>
     <row r="317">
-      <c r="A317" s="2" t="inlineStr">
+      <c r="A317" s="4" t="inlineStr">
+        <is>
+          <t>TC-1419</t>
+        </is>
+      </c>
+      <c r="B317" s="4" t="inlineStr">
+        <is>
+          <t>12.14 Startup Reconciliation</t>
+        </is>
+      </c>
+      <c r="C317" s="4" t="inlineStr">
+        <is>
+          <t>Restart restores READY when the interrupted startup-analysis cache is still current</t>
+        </is>
+      </c>
+      <c r="D317" s="4" t="inlineStr">
+        <is>
+          <t>Trigger manual Analyze for a job with a stable source tree, restart ECUBE after the reusable snapshot has been persisted but before the manual analyze workflow fully completes, then reopen Job Detail</t>
+        </is>
+      </c>
+      <c r="E317" s="4" t="inlineStr">
+        <is>
+          <t>Job shows startup_analysis_status: READY, the previous file and byte totals are still available, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "valid_cache_restored_after_restart", and Start can proceed without forcing a fresh scan</t>
+        </is>
+      </c>
+      <c r="F317" s="4" t="n"/>
+      <c r="G317" s="4" t="n"/>
+      <c r="H317" s="4" t="n"/>
+      <c r="I317" s="4" t="n"/>
+    </row>
+    <row r="318">
+      <c r="A318" s="2" t="inlineStr">
         <is>
           <t>§12.15 System Health</t>
         </is>
       </c>
-      <c r="B317" s="2" t="inlineStr">
+      <c r="B318" s="2" t="inlineStr">
         <is>
           <t>12.15 System Health</t>
         </is>
       </c>
-      <c r="C317" s="3" t="n"/>
-      <c r="D317" s="3" t="n"/>
-      <c r="E317" s="3" t="n"/>
-      <c r="F317" s="3" t="n"/>
-      <c r="G317" s="3" t="n"/>
-      <c r="H317" s="3" t="n"/>
-      <c r="I317" s="3" t="n"/>
-    </row>
-    <row r="318">
-      <c r="A318" s="4" t="inlineStr">
-        <is>
-          <t>TC-1501</t>
-        </is>
-      </c>
-      <c r="B318" s="4" t="inlineStr">
-        <is>
-          <t>12.15 System Health</t>
-        </is>
-      </c>
-      <c r="C318" s="4" t="inlineStr">
-        <is>
-          <t>Healthy response</t>
-        </is>
-      </c>
-      <c r="D318" s="4" t="inlineStr">
-        <is>
-          <t>GET /introspection/system-health with valid token</t>
-        </is>
-      </c>
-      <c r="E318" s="4" t="inlineStr">
-        <is>
-          <t>200, status: "ok", database: "connected"</t>
-        </is>
-      </c>
-      <c r="F318" s="4" t="n"/>
-      <c r="G318" s="4" t="n"/>
-      <c r="H318" s="4" t="n"/>
-      <c r="I318" s="4" t="n"/>
+      <c r="C318" s="3" t="n"/>
+      <c r="D318" s="3" t="n"/>
+      <c r="E318" s="3" t="n"/>
+      <c r="F318" s="3" t="n"/>
+      <c r="G318" s="3" t="n"/>
+      <c r="H318" s="3" t="n"/>
+      <c r="I318" s="3" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="4" t="inlineStr">
         <is>
-          <t>TC-1502</t>
+          <t>TC-1501</t>
         </is>
       </c>
       <c r="B319" s="4" t="inlineStr">
@@ -9878,17 +9878,17 @@
       </c>
       <c r="C319" s="4" t="inlineStr">
         <is>
-          <t>CPU metric present</t>
+          <t>Healthy response</t>
         </is>
       </c>
       <c r="D319" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>GET /introspection/system-health with valid token</t>
         </is>
       </c>
       <c r="E319" s="4" t="inlineStr">
         <is>
-          <t>cpu_percent is a number between 0 and 100</t>
+          <t>200, status: "ok", database: "connected"</t>
         </is>
       </c>
       <c r="F319" s="4" t="n"/>
@@ -9899,7 +9899,7 @@
     <row r="320">
       <c r="A320" s="4" t="inlineStr">
         <is>
-          <t>TC-1503</t>
+          <t>TC-1502</t>
         </is>
       </c>
       <c r="B320" s="4" t="inlineStr">
@@ -9909,7 +9909,7 @@
       </c>
       <c r="C320" s="4" t="inlineStr">
         <is>
-          <t>Memory metrics present</t>
+          <t>CPU metric present</t>
         </is>
       </c>
       <c r="D320" s="4" t="inlineStr">
@@ -9919,7 +9919,7 @@
       </c>
       <c r="E320" s="4" t="inlineStr">
         <is>
-          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
+          <t>cpu_percent is a number between 0 and 100</t>
         </is>
       </c>
       <c r="F320" s="4" t="n"/>
@@ -9930,7 +9930,7 @@
     <row r="321">
       <c r="A321" s="4" t="inlineStr">
         <is>
-          <t>TC-1504</t>
+          <t>TC-1503</t>
         </is>
       </c>
       <c r="B321" s="4" t="inlineStr">
@@ -9940,7 +9940,7 @@
       </c>
       <c r="C321" s="4" t="inlineStr">
         <is>
-          <t>Disk I/O metrics present</t>
+          <t>Memory metrics present</t>
         </is>
       </c>
       <c r="D321" s="4" t="inlineStr">
@@ -9950,7 +9950,7 @@
       </c>
       <c r="E321" s="4" t="inlineStr">
         <is>
-          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
+          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
         </is>
       </c>
       <c r="F321" s="4" t="n"/>
@@ -9961,7 +9961,7 @@
     <row r="322">
       <c r="A322" s="4" t="inlineStr">
         <is>
-          <t>TC-1505</t>
+          <t>TC-1504</t>
         </is>
       </c>
       <c r="B322" s="4" t="inlineStr">
@@ -9971,17 +9971,17 @@
       </c>
       <c r="C322" s="4" t="inlineStr">
         <is>
-          <t>Active jobs count</t>
+          <t>Disk I/O metrics present</t>
         </is>
       </c>
       <c r="D322" s="4" t="inlineStr">
         <is>
-          <t>Start an export job, call endpoint</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E322" s="4" t="inlineStr">
         <is>
-          <t>active_jobs ≥ 1</t>
+          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
         </is>
       </c>
       <c r="F322" s="4" t="n"/>
@@ -9992,7 +9992,7 @@
     <row r="323">
       <c r="A323" s="4" t="inlineStr">
         <is>
-          <t>TC-1506</t>
+          <t>TC-1505</t>
         </is>
       </c>
       <c r="B323" s="4" t="inlineStr">
@@ -10002,17 +10002,17 @@
       </c>
       <c r="C323" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size</t>
+          <t>Active jobs count</t>
         </is>
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>Create a PENDING job (created but not started), call endpoint</t>
+          <t>Start an export job, call endpoint</t>
         </is>
       </c>
       <c r="E323" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size ≥ 1</t>
+          <t>active_jobs ≥ 1</t>
         </is>
       </c>
       <c r="F323" s="4" t="n"/>
@@ -10023,7 +10023,7 @@
     <row r="324">
       <c r="A324" s="4" t="inlineStr">
         <is>
-          <t>TC-1507</t>
+          <t>TC-1506</t>
         </is>
       </c>
       <c r="B324" s="4" t="inlineStr">
@@ -10033,17 +10033,17 @@
       </c>
       <c r="C324" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size decrements</t>
+          <t>Worker queue size</t>
         </is>
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>Start the pending job, call endpoint again</t>
+          <t>Create a PENDING job (created but not started), call endpoint</t>
         </is>
       </c>
       <c r="E324" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
+          <t>worker_queue_size ≥ 1</t>
         </is>
       </c>
       <c r="F324" s="4" t="n"/>
@@ -10054,7 +10054,7 @@
     <row r="325">
       <c r="A325" s="4" t="inlineStr">
         <is>
-          <t>TC-1508</t>
+          <t>TC-1507</t>
         </is>
       </c>
       <c r="B325" s="4" t="inlineStr">
@@ -10064,17 +10064,17 @@
       </c>
       <c r="C325" s="4" t="inlineStr">
         <is>
-          <t>ECUBE process metrics present</t>
+          <t>Worker queue size decrements</t>
         </is>
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Start the pending job, call endpoint again</t>
         </is>
       </c>
       <c r="E325" s="4" t="inlineStr">
         <is>
-          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
+          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
         </is>
       </c>
       <c r="F325" s="4" t="n"/>
@@ -10085,7 +10085,7 @@
     <row r="326">
       <c r="A326" s="4" t="inlineStr">
         <is>
-          <t>TC-1509</t>
+          <t>TC-1508</t>
         </is>
       </c>
       <c r="B326" s="4" t="inlineStr">
@@ -10095,17 +10095,17 @@
       </c>
       <c r="C326" s="4" t="inlineStr">
         <is>
-          <t>Active copy-thread correlation</t>
+          <t>ECUBE process metrics present</t>
         </is>
       </c>
       <c r="D326" s="4" t="inlineStr">
         <is>
-          <t>Run an export job with active copy workers, call endpoint during the run</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E326" s="4" t="inlineStr">
         <is>
-          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
+          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
         </is>
       </c>
       <c r="F326" s="4" t="n"/>
@@ -10116,7 +10116,7 @@
     <row r="327">
       <c r="A327" s="4" t="inlineStr">
         <is>
-          <t>TC-1510</t>
+          <t>TC-1509</t>
         </is>
       </c>
       <c r="B327" s="4" t="inlineStr">
@@ -10126,17 +10126,17 @@
       </c>
       <c r="C327" s="4" t="inlineStr">
         <is>
-          <t>ECUBE process metrics degrade safely</t>
+          <t>Active copy-thread correlation</t>
         </is>
       </c>
       <c r="D327" s="4" t="inlineStr">
         <is>
-          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
+          <t>Run an export job with active copy workers, call endpoint during the run</t>
         </is>
       </c>
       <c r="E327" s="4" t="inlineStr">
         <is>
-          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
+          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
         </is>
       </c>
       <c r="F327" s="4" t="n"/>
@@ -10147,7 +10147,7 @@
     <row r="328">
       <c r="A328" s="4" t="inlineStr">
         <is>
-          <t>TC-1511</t>
+          <t>TC-1510</t>
         </is>
       </c>
       <c r="B328" s="4" t="inlineStr">
@@ -10157,17 +10157,17 @@
       </c>
       <c r="C328" s="4" t="inlineStr">
         <is>
-          <t>Degraded when DB down</t>
+          <t>ECUBE process metrics degrade safely</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, call endpoint with valid token</t>
+          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
         </is>
       </c>
       <c r="E328" s="4" t="inlineStr">
         <is>
-          <t>200, status: "degraded", database: "error", database_error is non-null</t>
+          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
         </is>
       </c>
       <c r="F328" s="4" t="n"/>
@@ -10178,7 +10178,7 @@
     <row r="329">
       <c r="A329" s="4" t="inlineStr">
         <is>
-          <t>TC-1512</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B329" s="4" t="inlineStr">
@@ -10188,17 +10188,17 @@
       </c>
       <c r="C329" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated rejected</t>
+          <t>Degraded when DB down</t>
         </is>
       </c>
       <c r="D329" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health without token</t>
+          <t>Stop PostgreSQL, call endpoint with valid token</t>
         </is>
       </c>
       <c r="E329" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>200, status: "degraded", database: "error", database_error is non-null</t>
         </is>
       </c>
       <c r="F329" s="4" t="n"/>
@@ -10209,7 +10209,7 @@
     <row r="330">
       <c r="A330" s="4" t="inlineStr">
         <is>
-          <t>TC-1513</t>
+          <t>TC-1512</t>
         </is>
       </c>
       <c r="B330" s="4" t="inlineStr">
@@ -10219,17 +10219,17 @@
       </c>
       <c r="C330" s="4" t="inlineStr">
         <is>
-          <t>Processor role allowed</t>
+          <t>Unauthenticated rejected</t>
         </is>
       </c>
       <c r="D330" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with processor token</t>
+          <t>GET /introspection/system-health without token</t>
         </is>
       </c>
       <c r="E330" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F330" s="4" t="n"/>
@@ -10238,59 +10238,59 @@
       <c r="I330" s="4" t="n"/>
     </row>
     <row r="331">
-      <c r="A331" s="2" t="inlineStr">
+      <c r="A331" s="4" t="inlineStr">
+        <is>
+          <t>TC-1513</t>
+        </is>
+      </c>
+      <c r="B331" s="4" t="inlineStr">
+        <is>
+          <t>12.15 System Health</t>
+        </is>
+      </c>
+      <c r="C331" s="4" t="inlineStr">
+        <is>
+          <t>Processor role allowed</t>
+        </is>
+      </c>
+      <c r="D331" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/system-health with processor token</t>
+        </is>
+      </c>
+      <c r="E331" s="4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F331" s="4" t="n"/>
+      <c r="G331" s="4" t="n"/>
+      <c r="H331" s="4" t="n"/>
+      <c r="I331" s="4" t="n"/>
+    </row>
+    <row r="332">
+      <c r="A332" s="2" t="inlineStr">
         <is>
           <t>§12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
-      <c r="B331" s="2" t="inlineStr">
+      <c r="B332" s="2" t="inlineStr">
         <is>
           <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
-      <c r="C331" s="3" t="n"/>
-      <c r="D331" s="3" t="n"/>
-      <c r="E331" s="3" t="n"/>
-      <c r="F331" s="3" t="n"/>
-      <c r="G331" s="3" t="n"/>
-      <c r="H331" s="3" t="n"/>
-      <c r="I331" s="3" t="n"/>
-    </row>
-    <row r="332">
-      <c r="A332" s="4" t="inlineStr">
-        <is>
-          <t>TC-1511</t>
-        </is>
-      </c>
-      <c r="B332" s="4" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C332" s="4" t="inlineStr">
-        <is>
-          <t>Liveness endpoint is public</t>
-        </is>
-      </c>
-      <c r="D332" s="4" t="inlineStr">
-        <is>
-          <t>GET /health/live without token</t>
-        </is>
-      </c>
-      <c r="E332" s="4" t="inlineStr">
-        <is>
-          <t>200, service reports live</t>
-        </is>
-      </c>
-      <c r="F332" s="4" t="n"/>
-      <c r="G332" s="4" t="n"/>
-      <c r="H332" s="4" t="n"/>
-      <c r="I332" s="4" t="n"/>
+      <c r="C332" s="3" t="n"/>
+      <c r="D332" s="3" t="n"/>
+      <c r="E332" s="3" t="n"/>
+      <c r="F332" s="3" t="n"/>
+      <c r="G332" s="3" t="n"/>
+      <c r="H332" s="3" t="n"/>
+      <c r="I332" s="3" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="4" t="inlineStr">
         <is>
-          <t>TC-1512</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B333" s="4" t="inlineStr">
@@ -10300,17 +10300,17 @@
       </c>
       <c r="C333" s="4" t="inlineStr">
         <is>
-          <t>Readiness endpoint is public</t>
+          <t>Liveness endpoint is public</t>
         </is>
       </c>
       <c r="D333" s="4" t="inlineStr">
         <is>
-          <t>GET /health/ready without token on a healthy system</t>
+          <t>GET /health/live without token</t>
         </is>
       </c>
       <c r="E333" s="4" t="inlineStr">
         <is>
-          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
+          <t>200, service reports live</t>
         </is>
       </c>
       <c r="F333" s="4" t="n"/>
@@ -10321,7 +10321,7 @@
     <row r="334">
       <c r="A334" s="4" t="inlineStr">
         <is>
-          <t>TC-1513</t>
+          <t>TC-1512</t>
         </is>
       </c>
       <c r="B334" s="4" t="inlineStr">
@@ -10331,17 +10331,17 @@
       </c>
       <c r="C334" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports missing database configuration</t>
+          <t>Readiness endpoint is public</t>
         </is>
       </c>
       <c r="D334" s="4" t="inlineStr">
         <is>
-          <t>Clear DB config or test before configuration, then GET /health/ready</t>
+          <t>GET /health/ready without token on a healthy system</t>
         </is>
       </c>
       <c r="E334" s="4" t="inlineStr">
         <is>
-          <t>503, status: "not_ready", reason indicates database is not configured</t>
+          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
         </is>
       </c>
       <c r="F334" s="4" t="n"/>
@@ -10352,7 +10352,7 @@
     <row r="335">
       <c r="A335" s="4" t="inlineStr">
         <is>
-          <t>TC-1514</t>
+          <t>TC-1513</t>
         </is>
       </c>
       <c r="B335" s="4" t="inlineStr">
@@ -10362,17 +10362,17 @@
       </c>
       <c r="C335" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports mount or provider problems</t>
+          <t>Readiness reports missing database configuration</t>
         </is>
       </c>
       <c r="D335" s="4" t="inlineStr">
         <is>
-          <t>Break a configured mount or provider, then GET /health/ready</t>
+          <t>Clear DB config or test before configuration, then GET /health/ready</t>
         </is>
       </c>
       <c r="E335" s="4" t="inlineStr">
         <is>
-          <t>503, response identifies the failing check without using the generic error schema</t>
+          <t>503, status: "not_ready", reason indicates database is not configured</t>
         </is>
       </c>
       <c r="F335" s="4" t="n"/>
@@ -10383,7 +10383,7 @@
     <row r="336">
       <c r="A336" s="4" t="inlineStr">
         <is>
-          <t>TC-1515</t>
+          <t>TC-1514</t>
         </is>
       </c>
       <c r="B336" s="4" t="inlineStr">
@@ -10393,17 +10393,17 @@
       </c>
       <c r="C336" s="4" t="inlineStr">
         <is>
-          <t>Version endpoint is public</t>
+          <t>Readiness reports mount or provider problems</t>
         </is>
       </c>
       <c r="D336" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/version without token</t>
+          <t>Break a configured mount or provider, then GET /health/ready</t>
         </is>
       </c>
       <c r="E336" s="4" t="inlineStr">
         <is>
-          <t>200, returns version/application metadata</t>
+          <t>503, response identifies the failing check without using the generic error schema</t>
         </is>
       </c>
       <c r="F336" s="4" t="n"/>
@@ -10414,7 +10414,7 @@
     <row r="337">
       <c r="A337" s="4" t="inlineStr">
         <is>
-          <t>TC-1516</t>
+          <t>TC-1515</t>
         </is>
       </c>
       <c r="B337" s="4" t="inlineStr">
@@ -10424,17 +10424,17 @@
       </c>
       <c r="C337" s="4" t="inlineStr">
         <is>
-          <t>Readiness remains separate from authenticated system health</t>
+          <t>Version endpoint is public</t>
         </is>
       </c>
       <c r="D337" s="4" t="inlineStr">
         <is>
-          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+          <t>GET /introspection/version without token</t>
         </is>
       </c>
       <c r="E337" s="4" t="inlineStr">
         <is>
-          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+          <t>200, returns version/application metadata</t>
         </is>
       </c>
       <c r="F337" s="4" t="n"/>
@@ -10443,32 +10443,63 @@
       <c r="I337" s="4" t="n"/>
     </row>
     <row r="338">
-      <c r="A338" s="2" t="inlineStr">
+      <c r="A338" s="4" t="inlineStr">
+        <is>
+          <t>TC-1516</t>
+        </is>
+      </c>
+      <c r="B338" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C338" s="4" t="inlineStr">
+        <is>
+          <t>Readiness remains separate from authenticated system health</t>
+        </is>
+      </c>
+      <c r="D338" s="4" t="inlineStr">
+        <is>
+          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+        </is>
+      </c>
+      <c r="E338" s="4" t="inlineStr">
+        <is>
+          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+        </is>
+      </c>
+      <c r="F338" s="4" t="n"/>
+      <c r="G338" s="4" t="n"/>
+      <c r="H338" s="4" t="n"/>
+      <c r="I338" s="4" t="n"/>
+    </row>
+    <row r="339">
+      <c r="A339" s="2" t="inlineStr">
         <is>
           <t>§12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="B338" s="2" t="inlineStr">
+      <c r="B339" s="2" t="inlineStr">
         <is>
           <t>12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="C338" s="3" t="n"/>
-      <c r="D338" s="3" t="n"/>
-      <c r="E338" s="3" t="n"/>
-      <c r="F338" s="3" t="n"/>
-      <c r="G338" s="3" t="n"/>
-      <c r="H338" s="3" t="n"/>
-      <c r="I338" s="3" t="n"/>
-    </row>
-    <row r="340">
-      <c r="A340" s="5" t="inlineStr">
+      <c r="C339" s="3" t="n"/>
+      <c r="D339" s="3" t="n"/>
+      <c r="E339" s="3" t="n"/>
+      <c r="F339" s="3" t="n"/>
+      <c r="G339" s="3" t="n"/>
+      <c r="H339" s="3" t="n"/>
+      <c r="I339" s="3" t="n"/>
+    </row>
+    <row r="341">
+      <c r="A341" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B340" s="5" t="n">
-        <v>310</v>
+      <c r="B341" s="5" t="n">
+        <v>311</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Simplify demo bootstrap and stop exposing demo passwords
Move demo mode to an install-root demo-metadata.json workflow and remove legacy
demo-data, generated sample content, USB, mount, and job seeding paths.

Generate a shared demo password during install/setup when metadata leaves it
blank, and keep that password out of the public auth payload and login UI.
Update docs and tests to match the new demo account seeding and recovery flow.
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -6986,17 +6986,17 @@
       </c>
       <c r="C223" s="4" t="inlineStr">
         <is>
-          <t>Public login guidance is shown</t>
+          <t>Public login guidance is shown without password disclosure</t>
         </is>
       </c>
       <c r="D223" s="4" t="inlineStr">
         <is>
-          <t>Enable demo mode, configure demo accounts, and open the login page</t>
+          <t>Run install.sh --demo, then open the login page</t>
         </is>
       </c>
       <c r="E223" s="4" t="inlineStr">
         <is>
-          <t>The login screen displays only the public-safe message plus username, label, and description fields</t>
+          <t>The login screen displays only the public-safe message plus username, label, and description fields, and it does not auto-fill or expose the shared demo password</t>
         </is>
       </c>
       <c r="F223" s="4" t="n"/>
@@ -7017,7 +7017,7 @@
       </c>
       <c r="C224" s="4" t="inlineStr">
         <is>
-          <t>No sensitive demo credentials are exposed</t>
+          <t>Shared demo password stays out of the public auth payload</t>
         </is>
       </c>
       <c r="D224" s="4" t="inlineStr">
@@ -7027,7 +7027,7 @@
       </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
-          <t>Passwords, internal paths, and private bootstrap-only fields are not present</t>
+          <t>The public payload does not expose shared passwords, per-account passwords, internal paths, or private bootstrap-only fields</t>
         </is>
       </c>
       <c r="F224" s="4" t="n"/>
@@ -7115,12 +7115,12 @@
       </c>
       <c r="D227" s="4" t="inlineStr">
         <is>
-          <t>Run the seed command twice against the same demo data root</t>
+          <t>Run the seed command twice against the same metadata file</t>
         </is>
       </c>
       <c r="E227" s="4" t="inlineStr">
         <is>
-          <t>Sample jobs, files, and role mappings return to a known good state without duplication</t>
+          <t>Demo users and role mappings return to the same known-good state without duplicate role assignments or seeded jobs</t>
         </is>
       </c>
       <c r="F227" s="4" t="n"/>
@@ -7141,17 +7141,17 @@
       </c>
       <c r="C228" s="4" t="inlineStr">
         <is>
-          <t>Demo reset is safe</t>
+          <t>Demo reset removes only seeded state</t>
         </is>
       </c>
       <c r="D228" s="4" t="inlineStr">
         <is>
-          <t>Run the reset command for the seeded demo root, then try an unmanaged directory path</t>
+          <t>Run the reset command against the seeded metadata file</t>
         </is>
       </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
-          <t>Managed demo content is removed; unmanaged directories are refused</t>
+          <t>Demo-seeded role assignments and seeded jobs are removed, but the metadata file itself is left in place</t>
         </is>
       </c>
       <c r="F228" s="4" t="n"/>
@@ -7172,17 +7172,17 @@
       </c>
       <c r="C229" s="4" t="inlineStr">
         <is>
-          <t>Numeric project references round-trip correctly</t>
+          <t>Installer uses colocated metadata and generates a password when blank</t>
         </is>
       </c>
       <c r="D229" s="4" t="inlineStr">
         <is>
-          <t>Seed a demo root whose projects[] use numeric project_id values and whose job_seed.jobs[].id is set to a stable integer such as 42</t>
+          <t>Place demo-metadata.json beside install.sh with demo_config.shared_password blank, run install.sh --demo, then inspect the install root and installer summary</t>
         </is>
       </c>
       <c r="E229" s="4" t="inlineStr">
         <is>
-          <t>The resulting metadata keeps the numeric project references, the seeded job is created for the expected project name, and the Jobs view or API shows the same numeric job ID</t>
+          <t>The install writes DEMO_MODE=true, generates and prints a strong demo password, stores it in the installed metadata, seeds from that metadata file, and does not create a separate demo-data directory or generated sample content</t>
         </is>
       </c>
       <c r="F229" s="4" t="n"/>
@@ -7234,17 +7234,17 @@
       </c>
       <c r="C231" s="4" t="inlineStr">
         <is>
-          <t>Sanitized sample data only</t>
+          <t>No sample content is staged automatically</t>
         </is>
       </c>
       <c r="D231" s="4" t="inlineStr">
         <is>
-          <t>Review the staged demo share contents</t>
+          <t>Review the install root and demo metadata after install.sh --demo</t>
         </is>
       </c>
       <c r="E231" s="4" t="inlineStr">
         <is>
-          <t>Files are clearly marked synthetic and contain no production or customer evidence</t>
+          <t>Demo bootstrap affects demo accounts, login guidance, and role state only; it does not stage sample projects, files, USB state, or network mounts</t>
         </is>
       </c>
       <c r="F231" s="4" t="n"/>

</xml_diff>

<commit_message>
Expose shared demo password for self-serve login
Restore the demo shared password in the public auth config so unattended demo
users can see it on the login page and sign in without operator handoff.

Prefill the login password field from the shared demo password and update the
demo install, bootstrap, user, and QA docs to reflect the public self-serve
workflow while still keeping per-account secrets private.
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -7017,7 +7017,7 @@
       </c>
       <c r="C224" s="4" t="inlineStr">
         <is>
-          <t>Shared demo password stays out of the public auth payload</t>
+          <t>Shared demo password is displayed for self-serve demo access</t>
         </is>
       </c>
       <c r="D224" s="4" t="inlineStr">
@@ -7027,7 +7027,7 @@
       </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
-          <t>The public payload does not expose shared passwords, per-account passwords, internal paths, or private bootstrap-only fields</t>
+          <t>The public payload exposes the shared demo password and the login page displays and prefills it, but still does not expose per-account passwords, internal paths, or private bootstrap-only fields</t>
         </is>
       </c>
       <c r="F224" s="4" t="n"/>

</xml_diff>

<commit_message>
Refactor demo mode to use runtime DEMO settings and reconcile demo accounts
Stop reading demo-metadata.json at runtime and treat it as install/bootstrap input only.
Populate DEMO_* values during demo install/post-install setup, derive the default shared password from the active password policy, and reconcile demo OS users, roles, and passwords from runtime settings at startup.
Document the new demo flow and cover the behavior with install, auth, configuration, and reconciliation tests.
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I341"/>
+  <dimension ref="A1:I342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7203,17 +7203,17 @@
       </c>
       <c r="C230" s="4" t="inlineStr">
         <is>
-          <t>Audit trail exists</t>
+          <t>Runtime default demo password follows Password Policy when unset</t>
         </is>
       </c>
       <c r="D230" s="4" t="inlineStr">
         <is>
-          <t>Query audit logs for demo bootstrap and denied password actions</t>
+          <t>Enable demo mode with DEMO_SHARED_PASSWORD unset, verify the login screen password, change Password Policy settings, restart ECUBE, then retry demo sign-in with the newly displayed password</t>
         </is>
       </c>
       <c r="E230" s="4" t="inlineStr">
         <is>
-          <t>Audit entries exist for seed, reset, and authorization denial events</t>
+          <t>The shared password shown on the login page changes to match the updated policy, and the restarted service accepts that password for the demo accounts</t>
         </is>
       </c>
       <c r="F230" s="4" t="n"/>
@@ -7224,7 +7224,7 @@
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
         <is>
-          <t>TC-929</t>
+          <t>TC-928</t>
         </is>
       </c>
       <c r="B231" s="4" t="inlineStr">
@@ -7234,17 +7234,17 @@
       </c>
       <c r="C231" s="4" t="inlineStr">
         <is>
-          <t>No sample content is staged automatically</t>
+          <t>Audit trail exists</t>
         </is>
       </c>
       <c r="D231" s="4" t="inlineStr">
         <is>
-          <t>Review the install root and demo metadata after install.sh --demo</t>
+          <t>Query audit logs for demo bootstrap and denied password actions</t>
         </is>
       </c>
       <c r="E231" s="4" t="inlineStr">
         <is>
-          <t>Demo bootstrap affects demo accounts, login guidance, and role state only; it does not stage sample projects, files, USB state, or network mounts</t>
+          <t>Audit entries exist for seed, reset, and authorization denial events</t>
         </is>
       </c>
       <c r="F231" s="4" t="n"/>
@@ -7253,59 +7253,59 @@
       <c r="I231" s="4" t="n"/>
     </row>
     <row r="232">
-      <c r="A232" s="2" t="inlineStr">
+      <c r="A232" s="4" t="inlineStr">
+        <is>
+          <t>TC-929</t>
+        </is>
+      </c>
+      <c r="B232" s="4" t="inlineStr">
+        <is>
+          <t>12.9.2 Demo Mode Rollout Validation Checklist</t>
+        </is>
+      </c>
+      <c r="C232" s="4" t="inlineStr">
+        <is>
+          <t>No sample content is staged automatically</t>
+        </is>
+      </c>
+      <c r="D232" s="4" t="inlineStr">
+        <is>
+          <t>Review the install root and demo metadata after install.sh --demo</t>
+        </is>
+      </c>
+      <c r="E232" s="4" t="inlineStr">
+        <is>
+          <t>Demo bootstrap affects demo accounts, login guidance, and role state only; it does not stage sample projects, files, USB state, or network mounts</t>
+        </is>
+      </c>
+      <c r="F232" s="4" t="n"/>
+      <c r="G232" s="4" t="n"/>
+      <c r="H232" s="4" t="n"/>
+      <c r="I232" s="4" t="n"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="inlineStr">
         <is>
           <t>§12.10 Admin Log Viewing API</t>
         </is>
       </c>
-      <c r="B232" s="2" t="inlineStr">
+      <c r="B233" s="2" t="inlineStr">
         <is>
           <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
-      <c r="C232" s="3" t="n"/>
-      <c r="D232" s="3" t="n"/>
-      <c r="E232" s="3" t="n"/>
-      <c r="F232" s="3" t="n"/>
-      <c r="G232" s="3" t="n"/>
-      <c r="H232" s="3" t="n"/>
-      <c r="I232" s="3" t="n"/>
-    </row>
-    <row r="233">
-      <c r="A233" s="4" t="inlineStr">
-        <is>
-          <t>TC-1001</t>
-        </is>
-      </c>
-      <c r="B233" s="4" t="inlineStr">
-        <is>
-          <t>12.10 Admin Log Viewing API</t>
-        </is>
-      </c>
-      <c r="C233" s="4" t="inlineStr">
-        <is>
-          <t>View logs — unauthenticated</t>
-        </is>
-      </c>
-      <c r="D233" s="4" t="inlineStr">
-        <is>
-          <t>GET /admin/logs/view without token</t>
-        </is>
-      </c>
-      <c r="E233" s="4" t="inlineStr">
-        <is>
-          <t>401, UNAUTHORIZED</t>
-        </is>
-      </c>
-      <c r="F233" s="4" t="n"/>
-      <c r="G233" s="4" t="n"/>
-      <c r="H233" s="4" t="n"/>
-      <c r="I233" s="4" t="n"/>
+      <c r="C233" s="3" t="n"/>
+      <c r="D233" s="3" t="n"/>
+      <c r="E233" s="3" t="n"/>
+      <c r="F233" s="3" t="n"/>
+      <c r="G233" s="3" t="n"/>
+      <c r="H233" s="3" t="n"/>
+      <c r="I233" s="3" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
         <is>
-          <t>TC-1002</t>
+          <t>TC-1001</t>
         </is>
       </c>
       <c r="B234" s="4" t="inlineStr">
@@ -7315,17 +7315,17 @@
       </c>
       <c r="C234" s="4" t="inlineStr">
         <is>
-          <t>View logs — non-admin denied</t>
+          <t>View logs — unauthenticated</t>
         </is>
       </c>
       <c r="D234" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/view with manager/processor/auditor token</t>
+          <t>GET /admin/logs/view without token</t>
         </is>
       </c>
       <c r="E234" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN; denied audit event recorded</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F234" s="4" t="n"/>
@@ -7336,7 +7336,7 @@
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
         <is>
-          <t>TC-1003</t>
+          <t>TC-1002</t>
         </is>
       </c>
       <c r="B235" s="4" t="inlineStr">
@@ -7346,17 +7346,17 @@
       </c>
       <c r="C235" s="4" t="inlineStr">
         <is>
-          <t>View logs — unknown source</t>
+          <t>View logs — non-admin denied</t>
         </is>
       </c>
       <c r="D235" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/view?source=unknown with admin token</t>
+          <t>GET /admin/logs/view with manager/processor/auditor token</t>
         </is>
       </c>
       <c r="E235" s="4" t="inlineStr">
         <is>
-          <t>404, unknown log source</t>
+          <t>403, FORBIDDEN; denied audit event recorded</t>
         </is>
       </c>
       <c r="F235" s="4" t="n"/>
@@ -7367,7 +7367,7 @@
     <row r="236">
       <c r="A236" s="4" t="inlineStr">
         <is>
-          <t>TC-1004</t>
+          <t>TC-1003</t>
         </is>
       </c>
       <c r="B236" s="4" t="inlineStr">
@@ -7377,17 +7377,17 @@
       </c>
       <c r="C236" s="4" t="inlineStr">
         <is>
-          <t>View logs — baseline response shape</t>
+          <t>View logs — unknown source</t>
         </is>
       </c>
       <c r="D236" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/view?source=app&amp;limit=5&amp;offset=0</t>
+          <t>GET /admin/logs/view?source=unknown with admin token</t>
         </is>
       </c>
       <c r="E236" s="4" t="inlineStr">
         <is>
-          <t>200 with object fields: source, fetched_at, file_modified_at, offset, limit, returned, has_more, lines</t>
+          <t>404, unknown log source</t>
         </is>
       </c>
       <c r="F236" s="4" t="n"/>
@@ -7398,7 +7398,7 @@
     <row r="237">
       <c r="A237" s="4" t="inlineStr">
         <is>
-          <t>TC-1005</t>
+          <t>TC-1004</t>
         </is>
       </c>
       <c r="B237" s="4" t="inlineStr">
@@ -7408,17 +7408,17 @@
       </c>
       <c r="C237" s="4" t="inlineStr">
         <is>
-          <t>View logs — source path redaction</t>
+          <t>View logs — baseline response shape</t>
         </is>
       </c>
       <c r="D237" s="4" t="inlineStr">
         <is>
-          <t>Inspect source.path in successful response</t>
+          <t>GET /admin/logs/view?source=app&amp;limit=5&amp;offset=0</t>
         </is>
       </c>
       <c r="E237" s="4" t="inlineStr">
         <is>
-          <t>Basename only (for example app.log), no absolute filesystem path</t>
+          <t>200 with object fields: source, fetched_at, file_modified_at, offset, limit, returned, has_more, lines</t>
         </is>
       </c>
       <c r="F237" s="4" t="n"/>
@@ -7429,7 +7429,7 @@
     <row r="238">
       <c r="A238" s="4" t="inlineStr">
         <is>
-          <t>TC-1006</t>
+          <t>TC-1005</t>
         </is>
       </c>
       <c r="B238" s="4" t="inlineStr">
@@ -7439,17 +7439,17 @@
       </c>
       <c r="C238" s="4" t="inlineStr">
         <is>
-          <t>View logs — offset pagination</t>
+          <t>View logs — source path redaction</t>
         </is>
       </c>
       <c r="D238" s="4" t="inlineStr">
         <is>
-          <t>Create known numbered lines, call GET /admin/logs/view?limit=5&amp;offset=2</t>
+          <t>Inspect source.path in successful response</t>
         </is>
       </c>
       <c r="E238" s="4" t="inlineStr">
         <is>
-          <t>Returns correct window from tail semantics, returned &lt;= limit</t>
+          <t>Basename only (for example app.log), no absolute filesystem path</t>
         </is>
       </c>
       <c r="F238" s="4" t="n"/>
@@ -7460,7 +7460,7 @@
     <row r="239">
       <c r="A239" s="4" t="inlineStr">
         <is>
-          <t>TC-1007</t>
+          <t>TC-1006</t>
         </is>
       </c>
       <c r="B239" s="4" t="inlineStr">
@@ -7470,17 +7470,17 @@
       </c>
       <c r="C239" s="4" t="inlineStr">
         <is>
-          <t>View logs — reverse ordering</t>
+          <t>View logs — offset pagination</t>
         </is>
       </c>
       <c r="D239" s="4" t="inlineStr">
         <is>
-          <t>Compare reverse=false vs reverse=true on same query</t>
+          <t>Create known numbered lines, call GET /admin/logs/view?limit=5&amp;offset=2</t>
         </is>
       </c>
       <c r="E239" s="4" t="inlineStr">
         <is>
-          <t>Same selected window; line order is inverted when reverse=true</t>
+          <t>Returns correct window from tail semantics, returned &lt;= limit</t>
         </is>
       </c>
       <c r="F239" s="4" t="n"/>
@@ -7491,7 +7491,7 @@
     <row r="240">
       <c r="A240" s="4" t="inlineStr">
         <is>
-          <t>TC-1008</t>
+          <t>TC-1007</t>
         </is>
       </c>
       <c r="B240" s="4" t="inlineStr">
@@ -7501,17 +7501,17 @@
       </c>
       <c r="C240" s="4" t="inlineStr">
         <is>
-          <t>View logs — search filtering</t>
+          <t>View logs — reverse ordering</t>
         </is>
       </c>
       <c r="D240" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/view?search=error</t>
+          <t>Compare reverse=false vs reverse=true on same query</t>
         </is>
       </c>
       <c r="E240" s="4" t="inlineStr">
         <is>
-          <t>Only matching lines are returned (case-insensitive contains)</t>
+          <t>Same selected window; line order is inverted when reverse=true</t>
         </is>
       </c>
       <c r="F240" s="4" t="n"/>
@@ -7522,7 +7522,7 @@
     <row r="241">
       <c r="A241" s="4" t="inlineStr">
         <is>
-          <t>TC-1009</t>
+          <t>TC-1008</t>
         </is>
       </c>
       <c r="B241" s="4" t="inlineStr">
@@ -7532,17 +7532,17 @@
       </c>
       <c r="C241" s="4" t="inlineStr">
         <is>
-          <t>View logs — sensitive value redaction</t>
+          <t>View logs — search filtering</t>
         </is>
       </c>
       <c r="D241" s="4" t="inlineStr">
         <is>
-          <t>Include tokens/passwords in source log lines, call view endpoint</t>
+          <t>GET /admin/logs/view?search=error</t>
         </is>
       </c>
       <c r="E241" s="4" t="inlineStr">
         <is>
-          <t>Sensitive values replaced with redacted markers in lines[].content</t>
+          <t>Only matching lines are returned (case-insensitive contains)</t>
         </is>
       </c>
       <c r="F241" s="4" t="n"/>
@@ -7553,7 +7553,7 @@
     <row r="242">
       <c r="A242" s="4" t="inlineStr">
         <is>
-          <t>TC-1010</t>
+          <t>TC-1009</t>
         </is>
       </c>
       <c r="B242" s="4" t="inlineStr">
@@ -7563,17 +7563,17 @@
       </c>
       <c r="C242" s="4" t="inlineStr">
         <is>
-          <t>View logs — success audit</t>
+          <t>View logs — sensitive value redaction</t>
         </is>
       </c>
       <c r="D242" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=LOG_LINES_VIEWED after successful view</t>
+          <t>Include tokens/passwords in source log lines, call view endpoint</t>
         </is>
       </c>
       <c r="E242" s="4" t="inlineStr">
         <is>
-          <t>Audit entry includes source, limit, offset, returned, has_more, and basename log_file</t>
+          <t>Sensitive values replaced with redacted markers in lines[].content</t>
         </is>
       </c>
       <c r="F242" s="4" t="n"/>
@@ -7584,7 +7584,7 @@
     <row r="243">
       <c r="A243" s="4" t="inlineStr">
         <is>
-          <t>TC-1011</t>
+          <t>TC-1010</t>
         </is>
       </c>
       <c r="B243" s="4" t="inlineStr">
@@ -7594,17 +7594,17 @@
       </c>
       <c r="C243" s="4" t="inlineStr">
         <is>
-          <t>List logs — unauthenticated</t>
+          <t>View logs — success audit</t>
         </is>
       </c>
       <c r="D243" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs without token</t>
+          <t>GET /audit?action=LOG_LINES_VIEWED after successful view</t>
         </is>
       </c>
       <c r="E243" s="4" t="inlineStr">
         <is>
-          <t>401, UNAUTHORIZED</t>
+          <t>Audit entry includes source, limit, offset, returned, has_more, and basename log_file</t>
         </is>
       </c>
       <c r="F243" s="4" t="n"/>
@@ -7615,7 +7615,7 @@
     <row r="244">
       <c r="A244" s="4" t="inlineStr">
         <is>
-          <t>TC-1012</t>
+          <t>TC-1011</t>
         </is>
       </c>
       <c r="B244" s="4" t="inlineStr">
@@ -7625,17 +7625,17 @@
       </c>
       <c r="C244" s="4" t="inlineStr">
         <is>
-          <t>List logs — non-admin denied</t>
+          <t>List logs — unauthenticated</t>
         </is>
       </c>
       <c r="D244" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs with non-admin token</t>
+          <t>GET /admin/logs without token</t>
         </is>
       </c>
       <c r="E244" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN; denied audit event recorded</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F244" s="4" t="n"/>
@@ -7646,7 +7646,7 @@
     <row r="245">
       <c r="A245" s="4" t="inlineStr">
         <is>
-          <t>TC-1013</t>
+          <t>TC-1012</t>
         </is>
       </c>
       <c r="B245" s="4" t="inlineStr">
@@ -7656,17 +7656,17 @@
       </c>
       <c r="C245" s="4" t="inlineStr">
         <is>
-          <t>List logs — response envelope</t>
+          <t>List logs — non-admin denied</t>
         </is>
       </c>
       <c r="D245" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs with admin token and file logging configured</t>
+          <t>GET /admin/logs with non-admin token</t>
         </is>
       </c>
       <c r="E245" s="4" t="inlineStr">
         <is>
-          <t>200 object with log_files array and total_size; no log_directory field in response</t>
+          <t>403, FORBIDDEN; denied audit event recorded</t>
         </is>
       </c>
       <c r="F245" s="4" t="n"/>
@@ -7677,7 +7677,7 @@
     <row r="246">
       <c r="A246" s="4" t="inlineStr">
         <is>
-          <t>TC-1014</t>
+          <t>TC-1013</t>
         </is>
       </c>
       <c r="B246" s="4" t="inlineStr">
@@ -7687,17 +7687,17 @@
       </c>
       <c r="C246" s="4" t="inlineStr">
         <is>
-          <t>Download log — non-admin denied</t>
+          <t>List logs — response envelope</t>
         </is>
       </c>
       <c r="D246" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/app.log with non-admin token</t>
+          <t>GET /admin/logs with admin token and file logging configured</t>
         </is>
       </c>
       <c r="E246" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN; denied audit event recorded</t>
+          <t>200 object with log_files array and total_size; no log_directory field in response</t>
         </is>
       </c>
       <c r="F246" s="4" t="n"/>
@@ -7708,7 +7708,7 @@
     <row r="247">
       <c r="A247" s="4" t="inlineStr">
         <is>
-          <t>TC-1015</t>
+          <t>TC-1014</t>
         </is>
       </c>
       <c r="B247" s="4" t="inlineStr">
@@ -7718,17 +7718,17 @@
       </c>
       <c r="C247" s="4" t="inlineStr">
         <is>
-          <t>Download log — path traversal blocked</t>
+          <t>Download log — non-admin denied</t>
         </is>
       </c>
       <c r="D247" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/../../../etc/passwd</t>
+          <t>GET /admin/logs/app.log with non-admin token</t>
         </is>
       </c>
       <c r="E247" s="4" t="inlineStr">
         <is>
-          <t>Rejected (400/404/422), no file disclosure</t>
+          <t>403, FORBIDDEN; denied audit event recorded</t>
         </is>
       </c>
       <c r="F247" s="4" t="n"/>
@@ -7739,7 +7739,7 @@
     <row r="248">
       <c r="A248" s="4" t="inlineStr">
         <is>
-          <t>TC-1016</t>
+          <t>TC-1015</t>
         </is>
       </c>
       <c r="B248" s="4" t="inlineStr">
@@ -7749,17 +7749,17 @@
       </c>
       <c r="C248" s="4" t="inlineStr">
         <is>
-          <t>Download log — success audit</t>
+          <t>Download log — path traversal blocked</t>
         </is>
       </c>
       <c r="D248" s="4" t="inlineStr">
         <is>
-          <t>Download valid file as admin, then query audit</t>
+          <t>GET /admin/logs/../../../etc/passwd</t>
         </is>
       </c>
       <c r="E248" s="4" t="inlineStr">
         <is>
-          <t>LOG_FILE_DOWNLOADED entry includes requested filename</t>
+          <t>Rejected (400/404/422), no file disclosure</t>
         </is>
       </c>
       <c r="F248" s="4" t="n"/>
@@ -7768,59 +7768,59 @@
       <c r="I248" s="4" t="n"/>
     </row>
     <row r="249">
-      <c r="A249" s="2" t="inlineStr">
+      <c r="A249" s="4" t="inlineStr">
+        <is>
+          <t>TC-1016</t>
+        </is>
+      </c>
+      <c r="B249" s="4" t="inlineStr">
+        <is>
+          <t>12.10 Admin Log Viewing API</t>
+        </is>
+      </c>
+      <c r="C249" s="4" t="inlineStr">
+        <is>
+          <t>Download log — success audit</t>
+        </is>
+      </c>
+      <c r="D249" s="4" t="inlineStr">
+        <is>
+          <t>Download valid file as admin, then query audit</t>
+        </is>
+      </c>
+      <c r="E249" s="4" t="inlineStr">
+        <is>
+          <t>LOG_FILE_DOWNLOADED entry includes requested filename</t>
+        </is>
+      </c>
+      <c r="F249" s="4" t="n"/>
+      <c r="G249" s="4" t="n"/>
+      <c r="H249" s="4" t="n"/>
+      <c r="I249" s="4" t="n"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
         <is>
           <t>§12.10.1 Runtime Configuration</t>
         </is>
       </c>
-      <c r="B249" s="2" t="inlineStr">
+      <c r="B250" s="2" t="inlineStr">
         <is>
           <t>12.10.1 Runtime Configuration</t>
         </is>
       </c>
-      <c r="C249" s="3" t="n"/>
-      <c r="D249" s="3" t="n"/>
-      <c r="E249" s="3" t="n"/>
-      <c r="F249" s="3" t="n"/>
-      <c r="G249" s="3" t="n"/>
-      <c r="H249" s="3" t="n"/>
-      <c r="I249" s="3" t="n"/>
-    </row>
-    <row r="250">
-      <c r="A250" s="4" t="inlineStr">
-        <is>
-          <t>TC-1011</t>
-        </is>
-      </c>
-      <c r="B250" s="4" t="inlineStr">
-        <is>
-          <t>12.10.1 Runtime Configuration</t>
-        </is>
-      </c>
-      <c r="C250" s="4" t="inlineStr">
-        <is>
-          <t>Get configuration — admin</t>
-        </is>
-      </c>
-      <c r="D250" s="4" t="inlineStr">
-        <is>
-          <t>GET /admin/configuration with admin token</t>
-        </is>
-      </c>
-      <c r="E250" s="4" t="inlineStr">
-        <is>
-          <t>200, response includes editable settings such as log_level and DB pool fields</t>
-        </is>
-      </c>
-      <c r="F250" s="4" t="n"/>
-      <c r="G250" s="4" t="n"/>
-      <c r="H250" s="4" t="n"/>
-      <c r="I250" s="4" t="n"/>
+      <c r="C250" s="3" t="n"/>
+      <c r="D250" s="3" t="n"/>
+      <c r="E250" s="3" t="n"/>
+      <c r="F250" s="3" t="n"/>
+      <c r="G250" s="3" t="n"/>
+      <c r="H250" s="3" t="n"/>
+      <c r="I250" s="3" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="4" t="inlineStr">
         <is>
-          <t>TC-1012</t>
+          <t>TC-1011</t>
         </is>
       </c>
       <c r="B251" s="4" t="inlineStr">
@@ -7830,17 +7830,17 @@
       </c>
       <c r="C251" s="4" t="inlineStr">
         <is>
-          <t>Get configuration — non-admin denied</t>
+          <t>Get configuration — admin</t>
         </is>
       </c>
       <c r="D251" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/configuration with manager/processor/auditor token</t>
+          <t>GET /admin/configuration with admin token</t>
         </is>
       </c>
       <c r="E251" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>200, response includes editable settings such as log_level and DB pool fields</t>
         </is>
       </c>
       <c r="F251" s="4" t="n"/>
@@ -7851,7 +7851,7 @@
     <row r="252">
       <c r="A252" s="4" t="inlineStr">
         <is>
-          <t>TC-1013</t>
+          <t>TC-1012</t>
         </is>
       </c>
       <c r="B252" s="4" t="inlineStr">
@@ -7861,17 +7861,17 @@
       </c>
       <c r="C252" s="4" t="inlineStr">
         <is>
-          <t>Update runtime-only setting</t>
+          <t>Get configuration — non-admin denied</t>
         </is>
       </c>
       <c r="D252" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/configuration with {"log_level": "DEBUG"}</t>
+          <t>GET /admin/configuration with manager/processor/auditor token</t>
         </is>
       </c>
       <c r="E252" s="4" t="inlineStr">
         <is>
-          <t>200, status: "updated", changed_settings includes log_level, restart_required is false</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F252" s="4" t="n"/>
@@ -7882,7 +7882,7 @@
     <row r="253">
       <c r="A253" s="4" t="inlineStr">
         <is>
-          <t>TC-1014</t>
+          <t>TC-1013</t>
         </is>
       </c>
       <c r="B253" s="4" t="inlineStr">
@@ -7892,17 +7892,17 @@
       </c>
       <c r="C253" s="4" t="inlineStr">
         <is>
-          <t>Update restart-required setting</t>
+          <t>Update runtime-only setting</t>
         </is>
       </c>
       <c r="D253" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/configuration with {"db_pool_recycle_seconds": 120}</t>
+          <t>PUT /admin/configuration with {"log_level": "DEBUG"}</t>
         </is>
       </c>
       <c r="E253" s="4" t="inlineStr">
         <is>
-          <t>200, restart_required is true and the response lists the restart-required setting</t>
+          <t>200, status: "updated", changed_settings includes log_level, restart_required is false</t>
         </is>
       </c>
       <c r="F253" s="4" t="n"/>
@@ -7913,7 +7913,7 @@
     <row r="254">
       <c r="A254" s="4" t="inlineStr">
         <is>
-          <t>TC-1015</t>
+          <t>TC-1014</t>
         </is>
       </c>
       <c r="B254" s="4" t="inlineStr">
@@ -7923,17 +7923,17 @@
       </c>
       <c r="C254" s="4" t="inlineStr">
         <is>
-          <t>Reject empty update payload</t>
+          <t>Update restart-required setting</t>
         </is>
       </c>
       <c r="D254" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/configuration with {}</t>
+          <t>PUT /admin/configuration with {"db_pool_recycle_seconds": 120}</t>
         </is>
       </c>
       <c r="E254" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>200, restart_required is true and the response lists the restart-required setting</t>
         </is>
       </c>
       <c r="F254" s="4" t="n"/>
@@ -7944,7 +7944,7 @@
     <row r="255">
       <c r="A255" s="4" t="inlineStr">
         <is>
-          <t>TC-1016</t>
+          <t>TC-1015</t>
         </is>
       </c>
       <c r="B255" s="4" t="inlineStr">
@@ -7954,17 +7954,17 @@
       </c>
       <c r="C255" s="4" t="inlineStr">
         <is>
-          <t>Reject unwritable log file path</t>
+          <t>Reject empty update payload</t>
         </is>
       </c>
       <c r="D255" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/configuration with {"log_file": "/var/log/ecube/denied.log"} when path is not writable</t>
+          <t>PUT /admin/configuration with {}</t>
         </is>
       </c>
       <c r="E255" s="4" t="inlineStr">
         <is>
-          <t>422, message indicates the log file cannot be written</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F255" s="4" t="n"/>
@@ -7975,7 +7975,7 @@
     <row r="256">
       <c r="A256" s="4" t="inlineStr">
         <is>
-          <t>TC-1017</t>
+          <t>TC-1016</t>
         </is>
       </c>
       <c r="B256" s="4" t="inlineStr">
@@ -7985,17 +7985,17 @@
       </c>
       <c r="C256" s="4" t="inlineStr">
         <is>
-          <t>Configuration update audit trail</t>
+          <t>Reject unwritable log file path</t>
         </is>
       </c>
       <c r="D256" s="4" t="inlineStr">
         <is>
-          <t>Update configuration, then query GET /audit?action=CONFIGURATION_UPDATED</t>
+          <t>PUT /admin/configuration with {"log_file": "/var/log/ecube/denied.log"} when path is not writable</t>
         </is>
       </c>
       <c r="E256" s="4" t="inlineStr">
         <is>
-          <t>Audit entry lists changed settings without leaking sensitive paths or secrets</t>
+          <t>422, message indicates the log file cannot be written</t>
         </is>
       </c>
       <c r="F256" s="4" t="n"/>
@@ -8006,7 +8006,7 @@
     <row r="257">
       <c r="A257" s="4" t="inlineStr">
         <is>
-          <t>TC-1018</t>
+          <t>TC-1017</t>
         </is>
       </c>
       <c r="B257" s="4" t="inlineStr">
@@ -8016,17 +8016,17 @@
       </c>
       <c r="C257" s="4" t="inlineStr">
         <is>
-          <t>Restart requires confirmation</t>
+          <t>Configuration update audit trail</t>
         </is>
       </c>
       <c r="D257" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/configuration/restart with {"confirm": false}</t>
+          <t>Update configuration, then query GET /audit?action=CONFIGURATION_UPDATED</t>
         </is>
       </c>
       <c r="E257" s="4" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>Audit entry lists changed settings without leaking sensitive paths or secrets</t>
         </is>
       </c>
       <c r="F257" s="4" t="n"/>
@@ -8037,7 +8037,7 @@
     <row r="258">
       <c r="A258" s="4" t="inlineStr">
         <is>
-          <t>TC-1019</t>
+          <t>TC-1018</t>
         </is>
       </c>
       <c r="B258" s="4" t="inlineStr">
@@ -8047,17 +8047,17 @@
       </c>
       <c r="C258" s="4" t="inlineStr">
         <is>
-          <t>Restart request accepted when confirmed</t>
+          <t>Restart requires confirmation</t>
         </is>
       </c>
       <c r="D258" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/configuration/restart with {"confirm": true}</t>
+          <t>POST /admin/configuration/restart with {"confirm": false}</t>
         </is>
       </c>
       <c r="E258" s="4" t="inlineStr">
         <is>
-          <t>200, status: "restart_requested", service: "ecube"</t>
+          <t>400</t>
         </is>
       </c>
       <c r="F258" s="4" t="n"/>
@@ -8068,7 +8068,7 @@
     <row r="259">
       <c r="A259" s="4" t="inlineStr">
         <is>
-          <t>TC-1020</t>
+          <t>TC-1019</t>
         </is>
       </c>
       <c r="B259" s="4" t="inlineStr">
@@ -8078,17 +8078,17 @@
       </c>
       <c r="C259" s="4" t="inlineStr">
         <is>
-          <t>Accept callback payload allowlist and mapping</t>
+          <t>Restart request accepted when confirmed</t>
         </is>
       </c>
       <c r="D259" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/configuration with {"callback_payload_fields": ["event", "project_id"], "callback_payload_field_map": {"type": "event", "project": "project_id"}}</t>
+          <t>POST /admin/configuration/restart with {"confirm": true}</t>
         </is>
       </c>
       <c r="E259" s="4" t="inlineStr">
         <is>
-          <t>200, changed settings include both callback payload fields</t>
+          <t>200, status: "restart_requested", service: "ecube"</t>
         </is>
       </c>
       <c r="F259" s="4" t="n"/>
@@ -8099,7 +8099,7 @@
     <row r="260">
       <c r="A260" s="4" t="inlineStr">
         <is>
-          <t>TC-1021</t>
+          <t>TC-1020</t>
         </is>
       </c>
       <c r="B260" s="4" t="inlineStr">
@@ -8109,17 +8109,17 @@
       </c>
       <c r="C260" s="4" t="inlineStr">
         <is>
-          <t>Reject invalid callback payload mapping</t>
+          <t>Accept callback payload allowlist and mapping</t>
         </is>
       </c>
       <c r="D260" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/configuration with {"callback_payload_field_map": {"summary": "${unknown_field}"}}</t>
+          <t>PUT /admin/configuration with {"callback_payload_fields": ["event", "project_id"], "callback_payload_field_map": {"type": "event", "project": "project_id"}}</t>
         </is>
       </c>
       <c r="E260" s="4" t="inlineStr">
         <is>
-          <t>422, validation error identifies the invalid mapping source field</t>
+          <t>200, changed settings include both callback payload fields</t>
         </is>
       </c>
       <c r="F260" s="4" t="n"/>
@@ -8128,59 +8128,59 @@
       <c r="I260" s="4" t="n"/>
     </row>
     <row r="261">
-      <c r="A261" s="2" t="inlineStr">
+      <c r="A261" s="4" t="inlineStr">
+        <is>
+          <t>TC-1021</t>
+        </is>
+      </c>
+      <c r="B261" s="4" t="inlineStr">
+        <is>
+          <t>12.10.1 Runtime Configuration</t>
+        </is>
+      </c>
+      <c r="C261" s="4" t="inlineStr">
+        <is>
+          <t>Reject invalid callback payload mapping</t>
+        </is>
+      </c>
+      <c r="D261" s="4" t="inlineStr">
+        <is>
+          <t>PUT /admin/configuration with {"callback_payload_field_map": {"summary": "${unknown_field}"}}</t>
+        </is>
+      </c>
+      <c r="E261" s="4" t="inlineStr">
+        <is>
+          <t>422, validation error identifies the invalid mapping source field</t>
+        </is>
+      </c>
+      <c r="F261" s="4" t="n"/>
+      <c r="G261" s="4" t="n"/>
+      <c r="H261" s="4" t="n"/>
+      <c r="I261" s="4" t="n"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="inlineStr">
         <is>
           <t>§12.10.2 Help System</t>
         </is>
       </c>
-      <c r="B261" s="2" t="inlineStr">
+      <c r="B262" s="2" t="inlineStr">
         <is>
           <t>12.10.2 Help System</t>
         </is>
       </c>
-      <c r="C261" s="3" t="n"/>
-      <c r="D261" s="3" t="n"/>
-      <c r="E261" s="3" t="n"/>
-      <c r="F261" s="3" t="n"/>
-      <c r="G261" s="3" t="n"/>
-      <c r="H261" s="3" t="n"/>
-      <c r="I261" s="3" t="n"/>
-    </row>
-    <row r="262">
-      <c r="A262" s="4" t="inlineStr">
-        <is>
-          <t>TC-1021</t>
-        </is>
-      </c>
-      <c r="B262" s="4" t="inlineStr">
-        <is>
-          <t>12.10.2 Help System</t>
-        </is>
-      </c>
-      <c r="C262" s="4" t="inlineStr">
-        <is>
-          <t>Help trigger is visible in authenticated shell</t>
-        </is>
-      </c>
-      <c r="D262" s="4" t="inlineStr">
-        <is>
-          <t>Sign in to the application and inspect the shell/header</t>
-        </is>
-      </c>
-      <c r="E262" s="4" t="inlineStr">
-        <is>
-          <t>A Help trigger is visible without navigating away from the current page</t>
-        </is>
-      </c>
-      <c r="F262" s="4" t="n"/>
-      <c r="G262" s="4" t="n"/>
-      <c r="H262" s="4" t="n"/>
-      <c r="I262" s="4" t="n"/>
+      <c r="C262" s="3" t="n"/>
+      <c r="D262" s="3" t="n"/>
+      <c r="E262" s="3" t="n"/>
+      <c r="F262" s="3" t="n"/>
+      <c r="G262" s="3" t="n"/>
+      <c r="H262" s="3" t="n"/>
+      <c r="I262" s="3" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="4" t="inlineStr">
         <is>
-          <t>TC-1022</t>
+          <t>TC-1021</t>
         </is>
       </c>
       <c r="B263" s="4" t="inlineStr">
@@ -8190,17 +8190,17 @@
       </c>
       <c r="C263" s="4" t="inlineStr">
         <is>
-          <t>Help opens in-app</t>
+          <t>Help trigger is visible in authenticated shell</t>
         </is>
       </c>
       <c r="D263" s="4" t="inlineStr">
         <is>
-          <t>Activate the Help trigger from any primary page</t>
+          <t>Sign in to the application and inspect the shell/header</t>
         </is>
       </c>
       <c r="E263" s="4" t="inlineStr">
         <is>
-          <t>Help opens in a modal or equivalent in-app panel</t>
+          <t>A Help trigger is visible without navigating away from the current page</t>
         </is>
       </c>
       <c r="F263" s="4" t="n"/>
@@ -8211,7 +8211,7 @@
     <row r="264">
       <c r="A264" s="4" t="inlineStr">
         <is>
-          <t>TC-1023</t>
+          <t>TC-1022</t>
         </is>
       </c>
       <c r="B264" s="4" t="inlineStr">
@@ -8221,17 +8221,17 @@
       </c>
       <c r="C264" s="4" t="inlineStr">
         <is>
-          <t>Help does not break current workflow context</t>
+          <t>Help opens in-app</t>
         </is>
       </c>
       <c r="D264" s="4" t="inlineStr">
         <is>
-          <t>Open Help while on Drives, Mounts, Jobs, or Audit, then close it</t>
+          <t>Activate the Help trigger from any primary page</t>
         </is>
       </c>
       <c r="E264" s="4" t="inlineStr">
         <is>
-          <t>Closing Help returns to the same page and preserved workflow context</t>
+          <t>Help opens in a modal or equivalent in-app panel</t>
         </is>
       </c>
       <c r="F264" s="4" t="n"/>
@@ -8242,7 +8242,7 @@
     <row r="265">
       <c r="A265" s="4" t="inlineStr">
         <is>
-          <t>TC-1024</t>
+          <t>TC-1023</t>
         </is>
       </c>
       <c r="B265" s="4" t="inlineStr">
@@ -8252,17 +8252,17 @@
       </c>
       <c r="C265" s="4" t="inlineStr">
         <is>
-          <t>Help content is curated and user-facing</t>
+          <t>Help does not break current workflow context</t>
         </is>
       </c>
       <c r="D265" s="4" t="inlineStr">
         <is>
-          <t>Review Help content in the modal</t>
+          <t>Open Help while on Drives, Mounts, Jobs, or Audit, then close it</t>
         </is>
       </c>
       <c r="E265" s="4" t="inlineStr">
         <is>
-          <t>Content is derived from the user manual and excludes installer-only or operator-only internals</t>
+          <t>Closing Help returns to the same page and preserved workflow context</t>
         </is>
       </c>
       <c r="F265" s="4" t="n"/>
@@ -8273,7 +8273,7 @@
     <row r="266">
       <c r="A266" s="4" t="inlineStr">
         <is>
-          <t>TC-1025</t>
+          <t>TC-1024</t>
         </is>
       </c>
       <c r="B266" s="4" t="inlineStr">
@@ -8283,17 +8283,17 @@
       </c>
       <c r="C266" s="4" t="inlineStr">
         <is>
-          <t>Open full help document works</t>
+          <t>Help content is curated and user-facing</t>
         </is>
       </c>
       <c r="D266" s="4" t="inlineStr">
         <is>
-          <t>Use the Help modal action to open the full document if present</t>
+          <t>Review Help content in the modal</t>
         </is>
       </c>
       <c r="E266" s="4" t="inlineStr">
         <is>
-          <t>Full help content opens successfully and remains consistent with the in-app content</t>
+          <t>Content is derived from the user manual and excludes installer-only or operator-only internals</t>
         </is>
       </c>
       <c r="F266" s="4" t="n"/>
@@ -8304,7 +8304,7 @@
     <row r="267">
       <c r="A267" s="4" t="inlineStr">
         <is>
-          <t>TC-1026</t>
+          <t>TC-1025</t>
         </is>
       </c>
       <c r="B267" s="4" t="inlineStr">
@@ -8314,17 +8314,17 @@
       </c>
       <c r="C267" s="4" t="inlineStr">
         <is>
-          <t>Missing help asset fails gracefully</t>
+          <t>Open full help document works</t>
         </is>
       </c>
       <c r="D267" s="4" t="inlineStr">
         <is>
-          <t>Test a build with the Help asset intentionally missing or inaccessible</t>
+          <t>Use the Help modal action to open the full document if present</t>
         </is>
       </c>
       <c r="E267" s="4" t="inlineStr">
         <is>
-          <t>UI shows a non-fatal fallback state with retry or operator guidance instead of breaking the app shell</t>
+          <t>Full help content opens successfully and remains consistent with the in-app content</t>
         </is>
       </c>
       <c r="F267" s="4" t="n"/>
@@ -8333,59 +8333,59 @@
       <c r="I267" s="4" t="n"/>
     </row>
     <row r="268">
-      <c r="A268" s="2" t="inlineStr">
+      <c r="A268" s="4" t="inlineStr">
+        <is>
+          <t>TC-1026</t>
+        </is>
+      </c>
+      <c r="B268" s="4" t="inlineStr">
+        <is>
+          <t>12.10.2 Help System</t>
+        </is>
+      </c>
+      <c r="C268" s="4" t="inlineStr">
+        <is>
+          <t>Missing help asset fails gracefully</t>
+        </is>
+      </c>
+      <c r="D268" s="4" t="inlineStr">
+        <is>
+          <t>Test a build with the Help asset intentionally missing or inaccessible</t>
+        </is>
+      </c>
+      <c r="E268" s="4" t="inlineStr">
+        <is>
+          <t>UI shows a non-fatal fallback state with retry or operator guidance instead of breaking the app shell</t>
+        </is>
+      </c>
+      <c r="F268" s="4" t="n"/>
+      <c r="G268" s="4" t="n"/>
+      <c r="H268" s="4" t="n"/>
+      <c r="I268" s="4" t="n"/>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="inlineStr">
         <is>
           <t>§12.11 First-Run Setup</t>
         </is>
       </c>
-      <c r="B268" s="2" t="inlineStr">
+      <c r="B269" s="2" t="inlineStr">
         <is>
           <t>12.11 First-Run Setup</t>
         </is>
       </c>
-      <c r="C268" s="3" t="n"/>
-      <c r="D268" s="3" t="n"/>
-      <c r="E268" s="3" t="n"/>
-      <c r="F268" s="3" t="n"/>
-      <c r="G268" s="3" t="n"/>
-      <c r="H268" s="3" t="n"/>
-      <c r="I268" s="3" t="n"/>
-    </row>
-    <row r="269">
-      <c r="A269" s="4" t="inlineStr">
-        <is>
-          <t>TC-1101</t>
-        </is>
-      </c>
-      <c r="B269" s="4" t="inlineStr">
-        <is>
-          <t>12.11 First-Run Setup</t>
-        </is>
-      </c>
-      <c r="C269" s="4" t="inlineStr">
-        <is>
-          <t>Status — not initialized</t>
-        </is>
-      </c>
-      <c r="D269" s="4" t="inlineStr">
-        <is>
-          <t>GET /setup/status on fresh database</t>
-        </is>
-      </c>
-      <c r="E269" s="4" t="inlineStr">
-        <is>
-          <t>200, {"initialized": false}</t>
-        </is>
-      </c>
-      <c r="F269" s="4" t="n"/>
-      <c r="G269" s="4" t="n"/>
-      <c r="H269" s="4" t="n"/>
-      <c r="I269" s="4" t="n"/>
+      <c r="C269" s="3" t="n"/>
+      <c r="D269" s="3" t="n"/>
+      <c r="E269" s="3" t="n"/>
+      <c r="F269" s="3" t="n"/>
+      <c r="G269" s="3" t="n"/>
+      <c r="H269" s="3" t="n"/>
+      <c r="I269" s="3" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="4" t="inlineStr">
         <is>
-          <t>TC-1102</t>
+          <t>TC-1101</t>
         </is>
       </c>
       <c r="B270" s="4" t="inlineStr">
@@ -8395,17 +8395,17 @@
       </c>
       <c r="C270" s="4" t="inlineStr">
         <is>
-          <t>Initialize</t>
+          <t>Status — not initialized</t>
         </is>
       </c>
       <c r="D270" s="4" t="inlineStr">
         <is>
-          <t>Complete the setup wizard with matching admin password and confirmation values</t>
+          <t>GET /setup/status on fresh database</t>
         </is>
       </c>
       <c r="E270" s="4" t="inlineStr">
         <is>
-          <t>200, returns message, username, groups_created</t>
+          <t>200, {"initialized": false}</t>
         </is>
       </c>
       <c r="F270" s="4" t="n"/>
@@ -8416,7 +8416,7 @@
     <row r="271">
       <c r="A271" s="4" t="inlineStr">
         <is>
-          <t>TC-1103</t>
+          <t>TC-1102</t>
         </is>
       </c>
       <c r="B271" s="4" t="inlineStr">
@@ -8426,17 +8426,17 @@
       </c>
       <c r="C271" s="4" t="inlineStr">
         <is>
-          <t>Status — initialized</t>
+          <t>Initialize</t>
         </is>
       </c>
       <c r="D271" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/status after initialization</t>
+          <t>Complete the setup wizard with matching admin password and confirmation values</t>
         </is>
       </c>
       <c r="E271" s="4" t="inlineStr">
         <is>
-          <t>200, {"initialized": true}</t>
+          <t>200, returns message, username, groups_created</t>
         </is>
       </c>
       <c r="F271" s="4" t="n"/>
@@ -8447,7 +8447,7 @@
     <row r="272">
       <c r="A272" s="4" t="inlineStr">
         <is>
-          <t>TC-1104</t>
+          <t>TC-1103</t>
         </is>
       </c>
       <c r="B272" s="4" t="inlineStr">
@@ -8457,17 +8457,17 @@
       </c>
       <c r="C272" s="4" t="inlineStr">
         <is>
-          <t>Re-initialize informational</t>
+          <t>Status — initialized</t>
         </is>
       </c>
       <c r="D272" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize again</t>
+          <t>GET /setup/status after initialization</t>
         </is>
       </c>
       <c r="E272" s="4" t="inlineStr">
         <is>
-          <t>200, status=already_initialized</t>
+          <t>200, {"initialized": true}</t>
         </is>
       </c>
       <c r="F272" s="4" t="n"/>
@@ -8478,7 +8478,7 @@
     <row r="273">
       <c r="A273" s="4" t="inlineStr">
         <is>
-          <t>TC-1105</t>
+          <t>TC-1104</t>
         </is>
       </c>
       <c r="B273" s="4" t="inlineStr">
@@ -8488,17 +8488,17 @@
       </c>
       <c r="C273" s="4" t="inlineStr">
         <is>
-          <t>Invalid username</t>
+          <t>Re-initialize informational</t>
         </is>
       </c>
       <c r="D273" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with uppercase or special chars</t>
+          <t>POST /setup/initialize again</t>
         </is>
       </c>
       <c r="E273" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>200, status=already_initialized</t>
         </is>
       </c>
       <c r="F273" s="4" t="n"/>
@@ -8509,7 +8509,7 @@
     <row r="274">
       <c r="A274" s="4" t="inlineStr">
         <is>
-          <t>TC-1106</t>
+          <t>TC-1105</t>
         </is>
       </c>
       <c r="B274" s="4" t="inlineStr">
@@ -8519,12 +8519,12 @@
       </c>
       <c r="C274" s="4" t="inlineStr">
         <is>
-          <t>Empty password</t>
+          <t>Invalid username</t>
         </is>
       </c>
       <c r="D274" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with {"password": ""}</t>
+          <t>POST /setup/initialize with uppercase or special chars</t>
         </is>
       </c>
       <c r="E274" s="4" t="inlineStr">
@@ -8540,7 +8540,7 @@
     <row r="275">
       <c r="A275" s="4" t="inlineStr">
         <is>
-          <t>TC-1107</t>
+          <t>TC-1106</t>
         </is>
       </c>
       <c r="B275" s="4" t="inlineStr">
@@ -8550,17 +8550,17 @@
       </c>
       <c r="C275" s="4" t="inlineStr">
         <is>
-          <t>Unsafe password chars</t>
+          <t>Empty password</t>
         </is>
       </c>
       <c r="D275" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with password containing newline or colon</t>
+          <t>POST /setup/initialize with {"password": ""}</t>
         </is>
       </c>
       <c r="E275" s="4" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F275" s="4" t="n"/>
@@ -8571,7 +8571,7 @@
     <row r="276">
       <c r="A276" s="4" t="inlineStr">
         <is>
-          <t>TC-1108</t>
+          <t>TC-1107</t>
         </is>
       </c>
       <c r="B276" s="4" t="inlineStr">
@@ -8581,17 +8581,17 @@
       </c>
       <c r="C276" s="4" t="inlineStr">
         <is>
-          <t>Login as initialized admin</t>
+          <t>Unsafe password chars</t>
         </is>
       </c>
       <c r="D276" s="4" t="inlineStr">
         <is>
-          <t>POST /auth/token with the admin credentials from step 2</t>
+          <t>POST /setup/initialize with password containing newline or colon</t>
         </is>
       </c>
       <c r="E276" s="4" t="inlineStr">
         <is>
-          <t>200, JWT contains admin role</t>
+          <t>422, unsafe characters</t>
         </is>
       </c>
       <c r="F276" s="4" t="n"/>
@@ -8602,7 +8602,7 @@
     <row r="277">
       <c r="A277" s="4" t="inlineStr">
         <is>
-          <t>TC-1109</t>
+          <t>TC-1108</t>
         </is>
       </c>
       <c r="B277" s="4" t="inlineStr">
@@ -8612,17 +8612,17 @@
       </c>
       <c r="C277" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM_INITIALIZED audit log</t>
+          <t>Login as initialized admin</t>
         </is>
       </c>
       <c r="D277" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
+          <t>POST /auth/token with the admin credentials from step 2</t>
         </is>
       </c>
       <c r="E277" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor</t>
+          <t>200, JWT contains admin role</t>
         </is>
       </c>
       <c r="F277" s="4" t="n"/>
@@ -8633,7 +8633,7 @@
     <row r="278">
       <c r="A278" s="4" t="inlineStr">
         <is>
-          <t>TC-1110</t>
+          <t>TC-1109</t>
         </is>
       </c>
       <c r="B278" s="4" t="inlineStr">
@@ -8643,17 +8643,17 @@
       </c>
       <c r="C278" s="4" t="inlineStr">
         <is>
-          <t>Initialize default proxy trust</t>
+          <t>SYSTEM_INITIALIZED audit log</t>
         </is>
       </c>
       <c r="D278" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize without trust_proxy_headers</t>
+          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
         </is>
       </c>
       <c r="E278" s="4" t="inlineStr">
         <is>
-          <t>200, runtime TRUST_PROXY_HEADERS=false persisted</t>
+          <t>Audit entry with actor</t>
         </is>
       </c>
       <c r="F278" s="4" t="n"/>
@@ -8664,7 +8664,7 @@
     <row r="279">
       <c r="A279" s="4" t="inlineStr">
         <is>
-          <t>TC-1111</t>
+          <t>TC-1110</t>
         </is>
       </c>
       <c r="B279" s="4" t="inlineStr">
@@ -8674,17 +8674,17 @@
       </c>
       <c r="C279" s="4" t="inlineStr">
         <is>
-          <t>Initialize explicit proxy trust</t>
+          <t>Initialize default proxy trust</t>
         </is>
       </c>
       <c r="D279" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with "trust_proxy_headers": true</t>
+          <t>POST /setup/initialize without trust_proxy_headers</t>
         </is>
       </c>
       <c r="E279" s="4" t="inlineStr">
         <is>
-          <t>200, runtime TRUST_PROXY_HEADERS=true persisted</t>
+          <t>200, runtime TRUST_PROXY_HEADERS=false persisted</t>
         </is>
       </c>
       <c r="F279" s="4" t="n"/>
@@ -8695,7 +8695,7 @@
     <row r="280">
       <c r="A280" s="4" t="inlineStr">
         <is>
-          <t>TC-1112</t>
+          <t>TC-1111</t>
         </is>
       </c>
       <c r="B280" s="4" t="inlineStr">
@@ -8705,17 +8705,17 @@
       </c>
       <c r="C280" s="4" t="inlineStr">
         <is>
-          <t>Re-initialize does not mutate runtime flags</t>
+          <t>Initialize explicit proxy trust</t>
         </is>
       </c>
       <c r="D280" s="4" t="inlineStr">
         <is>
-          <t>Call POST /setup/initialize after setup with a different trust_proxy_headers value</t>
+          <t>POST /setup/initialize with "trust_proxy_headers": true</t>
         </is>
       </c>
       <c r="E280" s="4" t="inlineStr">
         <is>
-          <t>200, status=already_initialized, runtime TRUST_PROXY_HEADERS remains unchanged</t>
+          <t>200, runtime TRUST_PROXY_HEADERS=true persisted</t>
         </is>
       </c>
       <c r="F280" s="4" t="n"/>
@@ -8726,7 +8726,7 @@
     <row r="281">
       <c r="A281" s="4" t="inlineStr">
         <is>
-          <t>TC-1113</t>
+          <t>TC-1112</t>
         </is>
       </c>
       <c r="B281" s="4" t="inlineStr">
@@ -8736,17 +8736,17 @@
       </c>
       <c r="C281" s="4" t="inlineStr">
         <is>
-          <t>Runtime env target consistency</t>
+          <t>Re-initialize does not mutate runtime flags</t>
         </is>
       </c>
       <c r="D281" s="4" t="inlineStr">
         <is>
-          <t>Validate running service env file target and setup persistence target are the same (ECUBE_ENV_FILE)</t>
+          <t>Call POST /setup/initialize after setup with a different trust_proxy_headers value</t>
         </is>
       </c>
       <c r="E281" s="4" t="inlineStr">
         <is>
-          <t>Runtime env file is updated, not a workspace-relative .env</t>
+          <t>200, status=already_initialized, runtime TRUST_PROXY_HEADERS remains unchanged</t>
         </is>
       </c>
       <c r="F281" s="4" t="n"/>
@@ -8757,7 +8757,7 @@
     <row r="282">
       <c r="A282" s="4" t="inlineStr">
         <is>
-          <t>TC-1114</t>
+          <t>TC-1113</t>
         </is>
       </c>
       <c r="B282" s="4" t="inlineStr">
@@ -8767,17 +8767,17 @@
       </c>
       <c r="C282" s="4" t="inlineStr">
         <is>
-          <t>Uninstall drop fails closed on invalid target</t>
+          <t>Runtime env target consistency</t>
         </is>
       </c>
       <c r="D282" s="4" t="inlineStr">
         <is>
-          <t>Run install.sh --uninstall --drop-database with missing/invalid/maintenance DATABASE_URL</t>
+          <t>Validate running service env file target and setup persistence target are the same (ECUBE_ENV_FILE)</t>
         </is>
       </c>
       <c r="E282" s="4" t="inlineStr">
         <is>
-          <t>Installer exits non-zero with explicit drop-target error; uninstall does not silently continue</t>
+          <t>Runtime env file is updated, not a workspace-relative .env</t>
         </is>
       </c>
       <c r="F282" s="4" t="n"/>
@@ -8788,7 +8788,7 @@
     <row r="283">
       <c r="A283" s="4" t="inlineStr">
         <is>
-          <t>TC-1115</t>
+          <t>TC-1114</t>
         </is>
       </c>
       <c r="B283" s="4" t="inlineStr">
@@ -8798,17 +8798,17 @@
       </c>
       <c r="C283" s="4" t="inlineStr">
         <is>
-          <t>Setup-required API redirect</t>
+          <t>Uninstall drop fails closed on invalid target</t>
         </is>
       </c>
       <c r="D283" s="4" t="inlineStr">
         <is>
-          <t>While using a normal UI screen, trigger a backend response with status 503, code HTTP_503, and message Database is not configured yet. Complete setup first.</t>
+          <t>Run install.sh --uninstall --drop-database with missing/invalid/maintenance DATABASE_URL</t>
         </is>
       </c>
       <c r="E283" s="4" t="inlineStr">
         <is>
-          <t>The browser redirects to /setup and the operator is not left only with the generic server-error toast</t>
+          <t>Installer exits non-zero with explicit drop-target error; uninstall does not silently continue</t>
         </is>
       </c>
       <c r="F283" s="4" t="n"/>
@@ -8819,7 +8819,7 @@
     <row r="284">
       <c r="A284" s="4" t="inlineStr">
         <is>
-          <t>TC-1116</t>
+          <t>TC-1115</t>
         </is>
       </c>
       <c r="B284" s="4" t="inlineStr">
@@ -8829,17 +8829,17 @@
       </c>
       <c r="C284" s="4" t="inlineStr">
         <is>
-          <t>Setup password confirmation mismatch</t>
+          <t>Setup-required API redirect</t>
         </is>
       </c>
       <c r="D284" s="4" t="inlineStr">
         <is>
-          <t>In the final setup wizard step, enter different values in the admin password and confirmation fields</t>
+          <t>While using a normal UI screen, trigger a backend response with status 503, code HTTP_503, and message Database is not configured yet. Complete setup first.</t>
         </is>
       </c>
       <c r="E284" s="4" t="inlineStr">
         <is>
-          <t>The wizard shows a password-mismatch validation message and does not submit setup until the two values match</t>
+          <t>The browser redirects to /setup and the operator is not left only with the generic server-error toast</t>
         </is>
       </c>
       <c r="F284" s="4" t="n"/>
@@ -8848,59 +8848,59 @@
       <c r="I284" s="4" t="n"/>
     </row>
     <row r="285">
-      <c r="A285" s="2" t="inlineStr">
+      <c r="A285" s="4" t="inlineStr">
+        <is>
+          <t>TC-1116</t>
+        </is>
+      </c>
+      <c r="B285" s="4" t="inlineStr">
+        <is>
+          <t>12.11 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C285" s="4" t="inlineStr">
+        <is>
+          <t>Setup password confirmation mismatch</t>
+        </is>
+      </c>
+      <c r="D285" s="4" t="inlineStr">
+        <is>
+          <t>In the final setup wizard step, enter different values in the admin password and confirmation fields</t>
+        </is>
+      </c>
+      <c r="E285" s="4" t="inlineStr">
+        <is>
+          <t>The wizard shows a password-mismatch validation message and does not submit setup until the two values match</t>
+        </is>
+      </c>
+      <c r="F285" s="4" t="n"/>
+      <c r="G285" s="4" t="n"/>
+      <c r="H285" s="4" t="n"/>
+      <c r="I285" s="4" t="n"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr">
         <is>
           <t>§12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
-      <c r="B285" s="2" t="inlineStr">
+      <c r="B286" s="2" t="inlineStr">
         <is>
           <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
-      <c r="C285" s="3" t="n"/>
-      <c r="D285" s="3" t="n"/>
-      <c r="E285" s="3" t="n"/>
-      <c r="F285" s="3" t="n"/>
-      <c r="G285" s="3" t="n"/>
-      <c r="H285" s="3" t="n"/>
-      <c r="I285" s="3" t="n"/>
-    </row>
-    <row r="286">
-      <c r="A286" s="4" t="inlineStr">
-        <is>
-          <t>TC-1201</t>
-        </is>
-      </c>
-      <c r="B286" s="4" t="inlineStr">
-        <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
-        </is>
-      </c>
-      <c r="C286" s="4" t="inlineStr">
-        <is>
-          <t>Retrieve stored CoC snapshot — archived job</t>
-        </is>
-      </c>
-      <c r="D286" s="4" t="inlineStr">
-        <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for an archived job that already has a stored snapshot</t>
-        </is>
-      </c>
-      <c r="E286" s="4" t="inlineStr">
-        <is>
-          <t>200, response contains the stored snapshot and snapshot metadata</t>
-        </is>
-      </c>
-      <c r="F286" s="4" t="n"/>
-      <c r="G286" s="4" t="n"/>
-      <c r="H286" s="4" t="n"/>
-      <c r="I286" s="4" t="n"/>
+      <c r="C286" s="3" t="n"/>
+      <c r="D286" s="3" t="n"/>
+      <c r="E286" s="3" t="n"/>
+      <c r="F286" s="3" t="n"/>
+      <c r="G286" s="3" t="n"/>
+      <c r="H286" s="3" t="n"/>
+      <c r="I286" s="3" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="4" t="inlineStr">
         <is>
-          <t>TC-1202</t>
+          <t>TC-1201</t>
         </is>
       </c>
       <c r="B287" s="4" t="inlineStr">
@@ -8910,17 +8910,17 @@
       </c>
       <c r="C287" s="4" t="inlineStr">
         <is>
-          <t>Retrieve stored CoC snapshot — active job</t>
+          <t>Retrieve stored CoC snapshot — archived job</t>
         </is>
       </c>
       <c r="D287" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job that already has a stored snapshot</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for an archived job that already has a stored snapshot</t>
         </is>
       </c>
       <c r="E287" s="4" t="inlineStr">
         <is>
-          <t>200, response contains the stored snapshot and does not regenerate it</t>
+          <t>200, response contains the stored snapshot and snapshot metadata</t>
         </is>
       </c>
       <c r="F287" s="4" t="n"/>
@@ -8931,7 +8931,7 @@
     <row r="288">
       <c r="A288" s="4" t="inlineStr">
         <is>
-          <t>TC-1203</t>
+          <t>TC-1202</t>
         </is>
       </c>
       <c r="B288" s="4" t="inlineStr">
@@ -8941,17 +8941,17 @@
       </c>
       <c r="C288" s="4" t="inlineStr">
         <is>
-          <t>CoC read — missing stored snapshot</t>
+          <t>Retrieve stored CoC snapshot — active job</t>
         </is>
       </c>
       <c r="D288" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job with no stored snapshot yet</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job that already has a stored snapshot</t>
         </is>
       </c>
       <c r="E288" s="4" t="inlineStr">
         <is>
-          <t>404, message explains that the report must be refreshed first</t>
+          <t>200, response contains the stored snapshot and does not regenerate it</t>
         </is>
       </c>
       <c r="F288" s="4" t="n"/>
@@ -8962,7 +8962,7 @@
     <row r="289">
       <c r="A289" s="4" t="inlineStr">
         <is>
-          <t>TC-1204</t>
+          <t>TC-1203</t>
         </is>
       </c>
       <c r="B289" s="4" t="inlineStr">
@@ -8972,17 +8972,17 @@
       </c>
       <c r="C289" s="4" t="inlineStr">
         <is>
-          <t>CoC read — processor denied</t>
+          <t>CoC read — missing stored snapshot</t>
         </is>
       </c>
       <c r="D289" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody with processor token</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job with no stored snapshot yet</t>
         </is>
       </c>
       <c r="E289" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>404, message explains that the report must be refreshed first</t>
         </is>
       </c>
       <c r="F289" s="4" t="n"/>
@@ -8993,7 +8993,7 @@
     <row r="290">
       <c r="A290" s="4" t="inlineStr">
         <is>
-          <t>TC-1205</t>
+          <t>TC-1204</t>
         </is>
       </c>
       <c r="B290" s="4" t="inlineStr">
@@ -9003,17 +9003,17 @@
       </c>
       <c r="C290" s="4" t="inlineStr">
         <is>
-          <t>CoC read — unauthenticated denied</t>
+          <t>CoC read — processor denied</t>
         </is>
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody without token</t>
+          <t>GET /jobs/{job_id}/chain-of-custody with processor token</t>
         </is>
       </c>
       <c r="E290" s="4" t="inlineStr">
         <is>
-          <t>401, UNAUTHORIZED</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F290" s="4" t="n"/>
@@ -9024,7 +9024,7 @@
     <row r="291">
       <c r="A291" s="4" t="inlineStr">
         <is>
-          <t>TC-1206</t>
+          <t>TC-1205</t>
         </is>
       </c>
       <c r="B291" s="4" t="inlineStr">
@@ -9034,17 +9034,17 @@
       </c>
       <c r="C291" s="4" t="inlineStr">
         <is>
-          <t>CoC snapshot fields</t>
+          <t>CoC read — unauthenticated denied</t>
         </is>
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>Inspect any stored-snapshot response</t>
+          <t>GET /jobs/{job_id}/chain-of-custody without token</t>
         </is>
       </c>
       <c r="E291" s="4" t="inlineStr">
         <is>
-          <t>snapshot_stored_at, snapshot_updated_at, snapshot_stored_by, reports[], and manifest/custody fields are present</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F291" s="4" t="n"/>
@@ -9055,7 +9055,7 @@
     <row r="292">
       <c r="A292" s="4" t="inlineStr">
         <is>
-          <t>TC-1207</t>
+          <t>TC-1206</t>
         </is>
       </c>
       <c r="B292" s="4" t="inlineStr">
@@ -9065,17 +9065,17 @@
       </c>
       <c r="C292" s="4" t="inlineStr">
         <is>
-          <t>CoC events include lifecycle</t>
+          <t>CoC snapshot fields</t>
         </is>
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>Inspect chain_of_custody_events in a stored report for a completed job</t>
+          <t>Inspect any stored-snapshot response</t>
         </is>
       </c>
       <c r="E292" s="4" t="inlineStr">
         <is>
-          <t>Events include DRIVE_INITIALIZED, JOB_CREATED, JOB_STARTED, JOB_COMPLETED, DRIVE_EJECT_PREPARED, and COC_HANDOFF_CONFIRMED when applicable</t>
+          <t>snapshot_stored_at, snapshot_updated_at, snapshot_stored_by, reports[], and manifest/custody fields are present</t>
         </is>
       </c>
       <c r="F292" s="4" t="n"/>
@@ -9086,7 +9086,7 @@
     <row r="293">
       <c r="A293" s="4" t="inlineStr">
         <is>
-          <t>TC-1208</t>
+          <t>TC-1207</t>
         </is>
       </c>
       <c r="B293" s="4" t="inlineStr">
@@ -9096,17 +9096,17 @@
       </c>
       <c r="C293" s="4" t="inlineStr">
         <is>
-          <t>CoC manifest summary</t>
+          <t>CoC events include lifecycle</t>
         </is>
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>Inspect manifest_summary in the stored report</t>
+          <t>Inspect chain_of_custody_events in a stored report for a completed job</t>
         </is>
       </c>
       <c r="E293" s="4" t="inlineStr">
         <is>
-          <t>Array of objects with job_id, evidence_number, processor_notes, total_files, total_bytes, and manifest_count</t>
+          <t>Events include DRIVE_INITIALIZED, JOB_CREATED, JOB_STARTED, JOB_COMPLETED, DRIVE_EJECT_PREPARED, and COC_HANDOFF_CONFIRMED when applicable</t>
         </is>
       </c>
       <c r="F293" s="4" t="n"/>
@@ -9117,7 +9117,7 @@
     <row r="294">
       <c r="A294" s="4" t="inlineStr">
         <is>
-          <t>TC-1209</t>
+          <t>TC-1208</t>
         </is>
       </c>
       <c r="B294" s="4" t="inlineStr">
@@ -9127,17 +9127,17 @@
       </c>
       <c r="C294" s="4" t="inlineStr">
         <is>
-          <t>CoC — delivery_time absence (no handoff)</t>
+          <t>CoC manifest summary</t>
         </is>
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>Complete a job and store a snapshot before handoff</t>
+          <t>Inspect manifest_summary in the stored report</t>
         </is>
       </c>
       <c r="E294" s="4" t="inlineStr">
         <is>
-          <t>chain_of_custody_events do not contain COC_HANDOFF_CONFIRMED; custody_complete is false</t>
+          <t>Array of objects with job_id, evidence_number, processor_notes, total_files, total_bytes, and manifest_count</t>
         </is>
       </c>
       <c r="F294" s="4" t="n"/>
@@ -9148,7 +9148,7 @@
     <row r="295">
       <c r="A295" s="4" t="inlineStr">
         <is>
-          <t>TC-1210</t>
+          <t>TC-1209</t>
         </is>
       </c>
       <c r="B295" s="4" t="inlineStr">
@@ -9158,17 +9158,17 @@
       </c>
       <c r="C295" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — valid</t>
+          <t>CoC — delivery_time absence (no handoff)</t>
         </is>
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh with admin or manager token for a non-archived job with assignments</t>
+          <t>Complete a job and store a snapshot before handoff</t>
         </is>
       </c>
       <c r="E295" s="4" t="inlineStr">
         <is>
-          <t>200, response contains the refreshed stored snapshot and updated snapshot metadata</t>
+          <t>chain_of_custody_events do not contain COC_HANDOFF_CONFIRMED; custody_complete is false</t>
         </is>
       </c>
       <c r="F295" s="4" t="n"/>
@@ -9179,7 +9179,7 @@
     <row r="296">
       <c r="A296" s="4" t="inlineStr">
         <is>
-          <t>TC-1211</t>
+          <t>TC-1210</t>
         </is>
       </c>
       <c r="B296" s="4" t="inlineStr">
@@ -9189,17 +9189,17 @@
       </c>
       <c r="C296" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — auditor denied</t>
+          <t>CoC refresh — valid</t>
         </is>
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh with auditor token</t>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh with admin or manager token for a non-archived job with assignments</t>
         </is>
       </c>
       <c r="E296" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>200, response contains the refreshed stored snapshot and updated snapshot metadata</t>
         </is>
       </c>
       <c r="F296" s="4" t="n"/>
@@ -9210,7 +9210,7 @@
     <row r="297">
       <c r="A297" s="4" t="inlineStr">
         <is>
-          <t>TC-1212</t>
+          <t>TC-1211</t>
         </is>
       </c>
       <c r="B297" s="4" t="inlineStr">
@@ -9220,17 +9220,17 @@
       </c>
       <c r="C297" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — archived job denied</t>
+          <t>CoC refresh — auditor denied</t>
         </is>
       </c>
       <c r="D297" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh for an archived job</t>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh with auditor token</t>
         </is>
       </c>
       <c r="E297" s="4" t="inlineStr">
         <is>
-          <t>409, archived jobs can only return the last stored snapshot</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F297" s="4" t="n"/>
@@ -9239,59 +9239,59 @@
       <c r="I297" s="4" t="n"/>
     </row>
     <row r="298">
-      <c r="A298" s="2" t="inlineStr">
+      <c r="A298" s="4" t="inlineStr">
+        <is>
+          <t>TC-1212</t>
+        </is>
+      </c>
+      <c r="B298" s="4" t="inlineStr">
+        <is>
+          <t>12.12 Chain-of-Custody Handoff</t>
+        </is>
+      </c>
+      <c r="C298" s="4" t="inlineStr">
+        <is>
+          <t>CoC refresh — archived job denied</t>
+        </is>
+      </c>
+      <c r="D298" s="4" t="inlineStr">
+        <is>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh for an archived job</t>
+        </is>
+      </c>
+      <c r="E298" s="4" t="inlineStr">
+        <is>
+          <t>409, archived jobs can only return the last stored snapshot</t>
+        </is>
+      </c>
+      <c r="F298" s="4" t="n"/>
+      <c r="G298" s="4" t="n"/>
+      <c r="H298" s="4" t="n"/>
+      <c r="I298" s="4" t="n"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="2" t="inlineStr">
         <is>
           <t>§12.14 Startup Reconciliation</t>
         </is>
       </c>
-      <c r="B298" s="2" t="inlineStr">
+      <c r="B299" s="2" t="inlineStr">
         <is>
           <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
-      <c r="C298" s="3" t="n"/>
-      <c r="D298" s="3" t="n"/>
-      <c r="E298" s="3" t="n"/>
-      <c r="F298" s="3" t="n"/>
-      <c r="G298" s="3" t="n"/>
-      <c r="H298" s="3" t="n"/>
-      <c r="I298" s="3" t="n"/>
-    </row>
-    <row r="299">
-      <c r="A299" s="4" t="inlineStr">
-        <is>
-          <t>TC-1401</t>
-        </is>
-      </c>
-      <c r="B299" s="4" t="inlineStr">
-        <is>
-          <t>12.14 Startup Reconciliation</t>
-        </is>
-      </c>
-      <c r="C299" s="4" t="inlineStr">
-        <is>
-          <t>Running job failed after restart</t>
-        </is>
-      </c>
-      <c r="D299" s="4" t="inlineStr">
-        <is>
-          <t>Create a job, start it, restart the service while RUNNING</t>
-        </is>
-      </c>
-      <c r="E299" s="4" t="inlineStr">
-        <is>
-          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
-        </is>
-      </c>
-      <c r="F299" s="4" t="n"/>
-      <c r="G299" s="4" t="n"/>
-      <c r="H299" s="4" t="n"/>
-      <c r="I299" s="4" t="n"/>
+      <c r="C299" s="3" t="n"/>
+      <c r="D299" s="3" t="n"/>
+      <c r="E299" s="3" t="n"/>
+      <c r="F299" s="3" t="n"/>
+      <c r="G299" s="3" t="n"/>
+      <c r="H299" s="3" t="n"/>
+      <c r="I299" s="3" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="4" t="inlineStr">
         <is>
-          <t>TC-1402</t>
+          <t>TC-1401</t>
         </is>
       </c>
       <c r="B300" s="4" t="inlineStr">
@@ -9301,17 +9301,17 @@
       </c>
       <c r="C300" s="4" t="inlineStr">
         <is>
-          <t>Verifying job failed after restart</t>
+          <t>Running job failed after restart</t>
         </is>
       </c>
       <c r="D300" s="4" t="inlineStr">
         <is>
-          <t>Start a job, let it reach VERIFYING, restart the service</t>
+          <t>Create a job, start it, restart the service while RUNNING</t>
         </is>
       </c>
       <c r="E300" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
+          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
         </is>
       </c>
       <c r="F300" s="4" t="n"/>
@@ -9322,7 +9322,7 @@
     <row r="301">
       <c r="A301" s="4" t="inlineStr">
         <is>
-          <t>TC-1403</t>
+          <t>TC-1402</t>
         </is>
       </c>
       <c r="B301" s="4" t="inlineStr">
@@ -9332,17 +9332,17 @@
       </c>
       <c r="C301" s="4" t="inlineStr">
         <is>
-          <t>Pending job not affected</t>
+          <t>Verifying job failed after restart</t>
         </is>
       </c>
       <c r="D301" s="4" t="inlineStr">
         <is>
-          <t>Create a job (PENDING), restart the service</t>
+          <t>Start a job, let it reach VERIFYING, restart the service</t>
         </is>
       </c>
       <c r="E301" s="4" t="inlineStr">
         <is>
-          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
+          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
         </is>
       </c>
       <c r="F301" s="4" t="n"/>
@@ -9353,7 +9353,7 @@
     <row r="302">
       <c r="A302" s="4" t="inlineStr">
         <is>
-          <t>TC-1404</t>
+          <t>TC-1403</t>
         </is>
       </c>
       <c r="B302" s="4" t="inlineStr">
@@ -9363,17 +9363,17 @@
       </c>
       <c r="C302" s="4" t="inlineStr">
         <is>
-          <t>Completed job not affected</t>
+          <t>Pending job not affected</t>
         </is>
       </c>
       <c r="D302" s="4" t="inlineStr">
         <is>
-          <t>Complete a job, restart the service</t>
+          <t>Create a job (PENDING), restart the service</t>
         </is>
       </c>
       <c r="E302" s="4" t="inlineStr">
         <is>
-          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
+          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
         </is>
       </c>
       <c r="F302" s="4" t="n"/>
@@ -9384,7 +9384,7 @@
     <row r="303">
       <c r="A303" s="4" t="inlineStr">
         <is>
-          <t>TC-1405</t>
+          <t>TC-1404</t>
         </is>
       </c>
       <c r="B303" s="4" t="inlineStr">
@@ -9394,17 +9394,17 @@
       </c>
       <c r="C303" s="4" t="inlineStr">
         <is>
-          <t>Stale mount corrected</t>
+          <t>Completed job not affected</t>
         </is>
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
+          <t>Complete a job, restart the service</t>
         </is>
       </c>
       <c r="E303" s="4" t="inlineStr">
         <is>
-          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
+          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F303" s="4" t="n"/>
@@ -9415,7 +9415,7 @@
     <row r="304">
       <c r="A304" s="4" t="inlineStr">
         <is>
-          <t>TC-1406</t>
+          <t>TC-1405</t>
         </is>
       </c>
       <c r="B304" s="4" t="inlineStr">
@@ -9425,17 +9425,17 @@
       </c>
       <c r="C304" s="4" t="inlineStr">
         <is>
-          <t>Active mount preserved</t>
+          <t>Stale mount corrected</t>
         </is>
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share (leave it mounted), restart the service</t>
+          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
         </is>
       </c>
       <c r="E304" s="4" t="inlineStr">
         <is>
-          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
+          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
         </is>
       </c>
       <c r="F304" s="4" t="n"/>
@@ -9446,7 +9446,7 @@
     <row r="305">
       <c r="A305" s="4" t="inlineStr">
         <is>
-          <t>TC-1407</t>
+          <t>TC-1406</t>
         </is>
       </c>
       <c r="B305" s="4" t="inlineStr">
@@ -9456,17 +9456,17 @@
       </c>
       <c r="C305" s="4" t="inlineStr">
         <is>
-          <t>USB drives re-discovered</t>
+          <t>Active mount preserved</t>
         </is>
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>Insert USB drives, restart the service</t>
+          <t>Add and mount a network share (leave it mounted), restart the service</t>
         </is>
       </c>
       <c r="E305" s="4" t="inlineStr">
         <is>
-          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
+          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F305" s="4" t="n"/>
@@ -9477,7 +9477,7 @@
     <row r="306">
       <c r="A306" s="4" t="inlineStr">
         <is>
-          <t>TC-1408</t>
+          <t>TC-1407</t>
         </is>
       </c>
       <c r="B306" s="4" t="inlineStr">
@@ -9487,17 +9487,17 @@
       </c>
       <c r="C306" s="4" t="inlineStr">
         <is>
-          <t>Idempotency</t>
+          <t>USB drives re-discovered</t>
         </is>
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>Restart the service twice without any state changes between restarts</t>
+          <t>Insert USB drives, restart the service</t>
         </is>
       </c>
       <c r="E306" s="4" t="inlineStr">
         <is>
-          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
+          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
         </is>
       </c>
       <c r="F306" s="4" t="n"/>
@@ -9508,7 +9508,7 @@
     <row r="307">
       <c r="A307" s="4" t="inlineStr">
         <is>
-          <t>TC-1409</t>
+          <t>TC-1408</t>
         </is>
       </c>
       <c r="B307" s="4" t="inlineStr">
@@ -9518,17 +9518,17 @@
       </c>
       <c r="C307" s="4" t="inlineStr">
         <is>
-          <t>Partial failure isolation</t>
+          <t>Idempotency</t>
         </is>
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
+          <t>Restart the service twice without any state changes between restarts</t>
         </is>
       </c>
       <c r="E307" s="4" t="inlineStr">
         <is>
-          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
+          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
         </is>
       </c>
       <c r="F307" s="4" t="n"/>
@@ -9539,7 +9539,7 @@
     <row r="308">
       <c r="A308" s="4" t="inlineStr">
         <is>
-          <t>TC-1410</t>
+          <t>TC-1409</t>
         </is>
       </c>
       <c r="B308" s="4" t="inlineStr">
@@ -9549,17 +9549,17 @@
       </c>
       <c r="C308" s="4" t="inlineStr">
         <is>
-          <t>Cross-process lock — only one worker reconciles</t>
+          <t>Partial failure isolation</t>
         </is>
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
+          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
         </is>
       </c>
       <c r="E308" s="4" t="inlineStr">
         <is>
-          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
+          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
         </is>
       </c>
       <c r="F308" s="4" t="n"/>
@@ -9570,7 +9570,7 @@
     <row r="309">
       <c r="A309" s="4" t="inlineStr">
         <is>
-          <t>TC-1411</t>
+          <t>TC-1410</t>
         </is>
       </c>
       <c r="B309" s="4" t="inlineStr">
@@ -9580,17 +9580,17 @@
       </c>
       <c r="C309" s="4" t="inlineStr">
         <is>
-          <t>Stale lock reclaim</t>
+          <t>Cross-process lock — only one worker reconciles</t>
         </is>
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
+          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
         </is>
       </c>
       <c r="E309" s="4" t="inlineStr">
         <is>
-          <t>Service reclaims the stale lock, reconciliation runs normally</t>
+          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
         </is>
       </c>
       <c r="F309" s="4" t="n"/>
@@ -9601,7 +9601,7 @@
     <row r="310">
       <c r="A310" s="4" t="inlineStr">
         <is>
-          <t>TC-1412</t>
+          <t>TC-1411</t>
         </is>
       </c>
       <c r="B310" s="4" t="inlineStr">
@@ -9611,17 +9611,17 @@
       </c>
       <c r="C310" s="4" t="inlineStr">
         <is>
-          <t>Lock released after failure</t>
+          <t>Stale lock reclaim</t>
         </is>
       </c>
       <c r="D310" s="4" t="inlineStr">
         <is>
-          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
+          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
         </is>
       </c>
       <c r="E310" s="4" t="inlineStr">
         <is>
-          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
+          <t>Service reclaims the stale lock, reconciliation runs normally</t>
         </is>
       </c>
       <c r="F310" s="4" t="n"/>
@@ -9632,7 +9632,7 @@
     <row r="311">
       <c r="A311" s="4" t="inlineStr">
         <is>
-          <t>TC-1413</t>
+          <t>TC-1412</t>
         </is>
       </c>
       <c r="B311" s="4" t="inlineStr">
@@ -9642,17 +9642,17 @@
       </c>
       <c r="C311" s="4" t="inlineStr">
         <is>
-          <t>Jobs pass emits immediate startup result log</t>
+          <t>Lock released after failure</t>
         </is>
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>Create at least one RUNNING job, restart service, then inspect application logs around startup reconciliation</t>
+          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
         </is>
       </c>
       <c r="E311" s="4" t="inlineStr">
         <is>
-          <t>Logs include Startup reconciliation: checking jobs followed by an immediate Startup reconciliation: jobs result line with safe counts (jobs_checked, jobs_corrected) or safe failure classification</t>
+          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
         </is>
       </c>
       <c r="F311" s="4" t="n"/>
@@ -9663,7 +9663,7 @@
     <row r="312">
       <c r="A312" s="4" t="inlineStr">
         <is>
-          <t>TC-1414</t>
+          <t>TC-1413</t>
         </is>
       </c>
       <c r="B312" s="4" t="inlineStr">
@@ -9673,17 +9673,17 @@
       </c>
       <c r="C312" s="4" t="inlineStr">
         <is>
-          <t>Reconciled job persists restart-interruption failure reason</t>
+          <t>Jobs pass emits immediate startup result log</t>
         </is>
       </c>
       <c r="D312" s="4" t="inlineStr">
         <is>
-          <t>Create a RUNNING or VERIFYING job, restart service, then open Job Detail for that job</t>
+          <t>Create at least one RUNNING job, restart service, then inspect application logs around startup reconciliation</t>
         </is>
       </c>
       <c r="E312" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED and Job Detail shows a stable restart interruption reason (not the generic This job failed... fallback)</t>
+          <t>Logs include Startup reconciliation: checking jobs followed by an immediate Startup reconciliation: jobs result line with safe counts (jobs_checked, jobs_corrected) or safe failure classification</t>
         </is>
       </c>
       <c r="F312" s="4" t="n"/>
@@ -9694,7 +9694,7 @@
     <row r="313">
       <c r="A313" s="4" t="inlineStr">
         <is>
-          <t>TC-1415</t>
+          <t>TC-1414</t>
         </is>
       </c>
       <c r="B313" s="4" t="inlineStr">
@@ -9704,17 +9704,17 @@
       </c>
       <c r="C313" s="4" t="inlineStr">
         <is>
-          <t>Reconciled failed job shows correlated failure entry from audit fallback</t>
+          <t>Reconciled job persists restart-interruption failure reason</t>
         </is>
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>Restart with a RUNNING job, then inspect Job Detail when no matching file-log failure line is present</t>
+          <t>Create a RUNNING or VERIFYING job, restart service, then open Job Detail for that job</t>
         </is>
       </c>
       <c r="E313" s="4" t="inlineStr">
         <is>
-          <t>Job Detail still shows a related failure entry sourced from reconciliation evidence (JOB_RECONCILED) and the entry remains sanitized</t>
+          <t>Job status is FAILED and Job Detail shows a stable restart interruption reason (not the generic This job failed... fallback)</t>
         </is>
       </c>
       <c r="F313" s="4" t="n"/>
@@ -9725,7 +9725,7 @@
     <row r="314">
       <c r="A314" s="4" t="inlineStr">
         <is>
-          <t>TC-1416</t>
+          <t>TC-1415</t>
         </is>
       </c>
       <c r="B314" s="4" t="inlineStr">
@@ -9735,17 +9735,17 @@
       </c>
       <c r="C314" s="4" t="inlineStr">
         <is>
-          <t>Failed job API uses reconciliation audit fallback when file-log correlation is unavailable</t>
+          <t>Reconciled failed job shows correlated failure entry from audit fallback</t>
         </is>
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>In a test environment, disable file-log correlation (log_file unset), then request GET /jobs/{job_id} for a restart-reconciled failed job</t>
+          <t>Restart with a RUNNING job, then inspect Job Detail when no matching file-log failure line is present</t>
         </is>
       </c>
       <c r="E314" s="4" t="inlineStr">
         <is>
-          <t>Response remains 200 and includes the stable restart failure reason plus a sanitized failure_log_entry derived from audit evidence (JOB_RECONCILED)</t>
+          <t>Job Detail still shows a related failure entry sourced from reconciliation evidence (JOB_RECONCILED) and the entry remains sanitized</t>
         </is>
       </c>
       <c r="F314" s="4" t="n"/>
@@ -9756,7 +9756,7 @@
     <row r="315">
       <c r="A315" s="4" t="inlineStr">
         <is>
-          <t>TC-1417</t>
+          <t>TC-1416</t>
         </is>
       </c>
       <c r="B315" s="4" t="inlineStr">
@@ -9766,17 +9766,17 @@
       </c>
       <c r="C315" s="4" t="inlineStr">
         <is>
-          <t>Jobs pass failure path emits safe startup result classification</t>
+          <t>Failed job API uses reconciliation audit fallback when file-log correlation is unavailable</t>
         </is>
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>In a controlled test environment, force a jobs-pass reconciliation exception, then restart service and inspect startup logs</t>
+          <t>In a test environment, disable file-log correlation (log_file unset), then request GET /jobs/{job_id} for a restart-reconciled failed job</t>
         </is>
       </c>
       <c r="E315" s="4" t="inlineStr">
         <is>
-          <t>Logs still include Startup reconciliation: jobs result with status=failed and reason=job_reconciliation_failed, without raw provider errors or host paths</t>
+          <t>Response remains 200 and includes the stable restart failure reason plus a sanitized failure_log_entry derived from audit evidence (JOB_RECONCILED)</t>
         </is>
       </c>
       <c r="F315" s="4" t="n"/>
@@ -9787,7 +9787,7 @@
     <row r="316">
       <c r="A316" s="4" t="inlineStr">
         <is>
-          <t>TC-1418</t>
+          <t>TC-1417</t>
         </is>
       </c>
       <c r="B316" s="4" t="inlineStr">
@@ -9797,17 +9797,17 @@
       </c>
       <c r="C316" s="4" t="inlineStr">
         <is>
-          <t>Restart clears stale in-progress startup analysis when no valid cache remains</t>
+          <t>Jobs pass failure path emits safe startup result classification</t>
         </is>
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>Trigger manual Analyze for a PENDING job, restart ECUBE before the scan completes, then reopen Job Detail</t>
+          <t>In a controlled test environment, force a jobs-pass reconciliation exception, then restart service and inspect startup logs</t>
         </is>
       </c>
       <c r="E316" s="4" t="inlineStr">
         <is>
-          <t>Job is no longer stuck in ANALYZING, startup-analysis state returns to NOT_ANALYZED, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "analysis_interrupted_by_restart", and Analyze or Start is available again</t>
+          <t>Logs still include Startup reconciliation: jobs result with status=failed and reason=job_reconciliation_failed, without raw provider errors or host paths</t>
         </is>
       </c>
       <c r="F316" s="4" t="n"/>
@@ -9818,7 +9818,7 @@
     <row r="317">
       <c r="A317" s="4" t="inlineStr">
         <is>
-          <t>TC-1419</t>
+          <t>TC-1418</t>
         </is>
       </c>
       <c r="B317" s="4" t="inlineStr">
@@ -9828,17 +9828,17 @@
       </c>
       <c r="C317" s="4" t="inlineStr">
         <is>
-          <t>Restart restores READY when the interrupted startup-analysis cache is still current</t>
+          <t>Restart clears stale in-progress startup analysis when no valid cache remains</t>
         </is>
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t>Trigger manual Analyze for a job with a stable source tree, restart ECUBE after the reusable snapshot has been persisted but before the manual analyze workflow fully completes, then reopen Job Detail</t>
+          <t>Trigger manual Analyze for a PENDING job, restart ECUBE before the scan completes, then reopen Job Detail</t>
         </is>
       </c>
       <c r="E317" s="4" t="inlineStr">
         <is>
-          <t>Job shows startup_analysis_status: READY, the previous file and byte totals are still available, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "valid_cache_restored_after_restart", and Start can proceed without forcing a fresh scan</t>
+          <t>Job is no longer stuck in ANALYZING, startup-analysis state returns to NOT_ANALYZED, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "analysis_interrupted_by_restart", and Analyze or Start is available again</t>
         </is>
       </c>
       <c r="F317" s="4" t="n"/>
@@ -9847,59 +9847,59 @@
       <c r="I317" s="4" t="n"/>
     </row>
     <row r="318">
-      <c r="A318" s="2" t="inlineStr">
+      <c r="A318" s="4" t="inlineStr">
+        <is>
+          <t>TC-1419</t>
+        </is>
+      </c>
+      <c r="B318" s="4" t="inlineStr">
+        <is>
+          <t>12.14 Startup Reconciliation</t>
+        </is>
+      </c>
+      <c r="C318" s="4" t="inlineStr">
+        <is>
+          <t>Restart restores READY when the interrupted startup-analysis cache is still current</t>
+        </is>
+      </c>
+      <c r="D318" s="4" t="inlineStr">
+        <is>
+          <t>Trigger manual Analyze for a job with a stable source tree, restart ECUBE after the reusable snapshot has been persisted but before the manual analyze workflow fully completes, then reopen Job Detail</t>
+        </is>
+      </c>
+      <c r="E318" s="4" t="inlineStr">
+        <is>
+          <t>Job shows startup_analysis_status: READY, the previous file and byte totals are still available, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "valid_cache_restored_after_restart", and Start can proceed without forcing a fresh scan</t>
+        </is>
+      </c>
+      <c r="F318" s="4" t="n"/>
+      <c r="G318" s="4" t="n"/>
+      <c r="H318" s="4" t="n"/>
+      <c r="I318" s="4" t="n"/>
+    </row>
+    <row r="319">
+      <c r="A319" s="2" t="inlineStr">
         <is>
           <t>§12.15 System Health</t>
         </is>
       </c>
-      <c r="B318" s="2" t="inlineStr">
+      <c r="B319" s="2" t="inlineStr">
         <is>
           <t>12.15 System Health</t>
         </is>
       </c>
-      <c r="C318" s="3" t="n"/>
-      <c r="D318" s="3" t="n"/>
-      <c r="E318" s="3" t="n"/>
-      <c r="F318" s="3" t="n"/>
-      <c r="G318" s="3" t="n"/>
-      <c r="H318" s="3" t="n"/>
-      <c r="I318" s="3" t="n"/>
-    </row>
-    <row r="319">
-      <c r="A319" s="4" t="inlineStr">
-        <is>
-          <t>TC-1501</t>
-        </is>
-      </c>
-      <c r="B319" s="4" t="inlineStr">
-        <is>
-          <t>12.15 System Health</t>
-        </is>
-      </c>
-      <c r="C319" s="4" t="inlineStr">
-        <is>
-          <t>Healthy response</t>
-        </is>
-      </c>
-      <c r="D319" s="4" t="inlineStr">
-        <is>
-          <t>GET /introspection/system-health with valid token</t>
-        </is>
-      </c>
-      <c r="E319" s="4" t="inlineStr">
-        <is>
-          <t>200, status: "ok", database: "connected"</t>
-        </is>
-      </c>
-      <c r="F319" s="4" t="n"/>
-      <c r="G319" s="4" t="n"/>
-      <c r="H319" s="4" t="n"/>
-      <c r="I319" s="4" t="n"/>
+      <c r="C319" s="3" t="n"/>
+      <c r="D319" s="3" t="n"/>
+      <c r="E319" s="3" t="n"/>
+      <c r="F319" s="3" t="n"/>
+      <c r="G319" s="3" t="n"/>
+      <c r="H319" s="3" t="n"/>
+      <c r="I319" s="3" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="4" t="inlineStr">
         <is>
-          <t>TC-1502</t>
+          <t>TC-1501</t>
         </is>
       </c>
       <c r="B320" s="4" t="inlineStr">
@@ -9909,17 +9909,17 @@
       </c>
       <c r="C320" s="4" t="inlineStr">
         <is>
-          <t>CPU metric present</t>
+          <t>Healthy response</t>
         </is>
       </c>
       <c r="D320" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>GET /introspection/system-health with valid token</t>
         </is>
       </c>
       <c r="E320" s="4" t="inlineStr">
         <is>
-          <t>cpu_percent is a number between 0 and 100</t>
+          <t>200, status: "ok", database: "connected"</t>
         </is>
       </c>
       <c r="F320" s="4" t="n"/>
@@ -9930,7 +9930,7 @@
     <row r="321">
       <c r="A321" s="4" t="inlineStr">
         <is>
-          <t>TC-1503</t>
+          <t>TC-1502</t>
         </is>
       </c>
       <c r="B321" s="4" t="inlineStr">
@@ -9940,7 +9940,7 @@
       </c>
       <c r="C321" s="4" t="inlineStr">
         <is>
-          <t>Memory metrics present</t>
+          <t>CPU metric present</t>
         </is>
       </c>
       <c r="D321" s="4" t="inlineStr">
@@ -9950,7 +9950,7 @@
       </c>
       <c r="E321" s="4" t="inlineStr">
         <is>
-          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
+          <t>cpu_percent is a number between 0 and 100</t>
         </is>
       </c>
       <c r="F321" s="4" t="n"/>
@@ -9961,7 +9961,7 @@
     <row r="322">
       <c r="A322" s="4" t="inlineStr">
         <is>
-          <t>TC-1504</t>
+          <t>TC-1503</t>
         </is>
       </c>
       <c r="B322" s="4" t="inlineStr">
@@ -9971,7 +9971,7 @@
       </c>
       <c r="C322" s="4" t="inlineStr">
         <is>
-          <t>Disk I/O metrics present</t>
+          <t>Memory metrics present</t>
         </is>
       </c>
       <c r="D322" s="4" t="inlineStr">
@@ -9981,7 +9981,7 @@
       </c>
       <c r="E322" s="4" t="inlineStr">
         <is>
-          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
+          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
         </is>
       </c>
       <c r="F322" s="4" t="n"/>
@@ -9992,7 +9992,7 @@
     <row r="323">
       <c r="A323" s="4" t="inlineStr">
         <is>
-          <t>TC-1505</t>
+          <t>TC-1504</t>
         </is>
       </c>
       <c r="B323" s="4" t="inlineStr">
@@ -10002,17 +10002,17 @@
       </c>
       <c r="C323" s="4" t="inlineStr">
         <is>
-          <t>Active jobs count</t>
+          <t>Disk I/O metrics present</t>
         </is>
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>Start an export job, call endpoint</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E323" s="4" t="inlineStr">
         <is>
-          <t>active_jobs ≥ 1</t>
+          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
         </is>
       </c>
       <c r="F323" s="4" t="n"/>
@@ -10023,7 +10023,7 @@
     <row r="324">
       <c r="A324" s="4" t="inlineStr">
         <is>
-          <t>TC-1506</t>
+          <t>TC-1505</t>
         </is>
       </c>
       <c r="B324" s="4" t="inlineStr">
@@ -10033,17 +10033,17 @@
       </c>
       <c r="C324" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size</t>
+          <t>Active jobs count</t>
         </is>
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>Create a PENDING job (created but not started), call endpoint</t>
+          <t>Start an export job, call endpoint</t>
         </is>
       </c>
       <c r="E324" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size ≥ 1</t>
+          <t>active_jobs ≥ 1</t>
         </is>
       </c>
       <c r="F324" s="4" t="n"/>
@@ -10054,7 +10054,7 @@
     <row r="325">
       <c r="A325" s="4" t="inlineStr">
         <is>
-          <t>TC-1507</t>
+          <t>TC-1506</t>
         </is>
       </c>
       <c r="B325" s="4" t="inlineStr">
@@ -10064,17 +10064,17 @@
       </c>
       <c r="C325" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size decrements</t>
+          <t>Worker queue size</t>
         </is>
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>Start the pending job, call endpoint again</t>
+          <t>Create a PENDING job (created but not started), call endpoint</t>
         </is>
       </c>
       <c r="E325" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
+          <t>worker_queue_size ≥ 1</t>
         </is>
       </c>
       <c r="F325" s="4" t="n"/>
@@ -10085,7 +10085,7 @@
     <row r="326">
       <c r="A326" s="4" t="inlineStr">
         <is>
-          <t>TC-1508</t>
+          <t>TC-1507</t>
         </is>
       </c>
       <c r="B326" s="4" t="inlineStr">
@@ -10095,17 +10095,17 @@
       </c>
       <c r="C326" s="4" t="inlineStr">
         <is>
-          <t>ECUBE process metrics present</t>
+          <t>Worker queue size decrements</t>
         </is>
       </c>
       <c r="D326" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Start the pending job, call endpoint again</t>
         </is>
       </c>
       <c r="E326" s="4" t="inlineStr">
         <is>
-          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
+          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
         </is>
       </c>
       <c r="F326" s="4" t="n"/>
@@ -10116,7 +10116,7 @@
     <row r="327">
       <c r="A327" s="4" t="inlineStr">
         <is>
-          <t>TC-1509</t>
+          <t>TC-1508</t>
         </is>
       </c>
       <c r="B327" s="4" t="inlineStr">
@@ -10126,17 +10126,17 @@
       </c>
       <c r="C327" s="4" t="inlineStr">
         <is>
-          <t>Active copy-thread correlation</t>
+          <t>ECUBE process metrics present</t>
         </is>
       </c>
       <c r="D327" s="4" t="inlineStr">
         <is>
-          <t>Run an export job with active copy workers, call endpoint during the run</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E327" s="4" t="inlineStr">
         <is>
-          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
+          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
         </is>
       </c>
       <c r="F327" s="4" t="n"/>
@@ -10147,7 +10147,7 @@
     <row r="328">
       <c r="A328" s="4" t="inlineStr">
         <is>
-          <t>TC-1510</t>
+          <t>TC-1509</t>
         </is>
       </c>
       <c r="B328" s="4" t="inlineStr">
@@ -10157,17 +10157,17 @@
       </c>
       <c r="C328" s="4" t="inlineStr">
         <is>
-          <t>ECUBE process metrics degrade safely</t>
+          <t>Active copy-thread correlation</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr">
         <is>
-          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
+          <t>Run an export job with active copy workers, call endpoint during the run</t>
         </is>
       </c>
       <c r="E328" s="4" t="inlineStr">
         <is>
-          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
+          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
         </is>
       </c>
       <c r="F328" s="4" t="n"/>
@@ -10178,7 +10178,7 @@
     <row r="329">
       <c r="A329" s="4" t="inlineStr">
         <is>
-          <t>TC-1511</t>
+          <t>TC-1510</t>
         </is>
       </c>
       <c r="B329" s="4" t="inlineStr">
@@ -10188,17 +10188,17 @@
       </c>
       <c r="C329" s="4" t="inlineStr">
         <is>
-          <t>Degraded when DB down</t>
+          <t>ECUBE process metrics degrade safely</t>
         </is>
       </c>
       <c r="D329" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, call endpoint with valid token</t>
+          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
         </is>
       </c>
       <c r="E329" s="4" t="inlineStr">
         <is>
-          <t>200, status: "degraded", database: "error", database_error is non-null</t>
+          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
         </is>
       </c>
       <c r="F329" s="4" t="n"/>
@@ -10209,7 +10209,7 @@
     <row r="330">
       <c r="A330" s="4" t="inlineStr">
         <is>
-          <t>TC-1512</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B330" s="4" t="inlineStr">
@@ -10219,17 +10219,17 @@
       </c>
       <c r="C330" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated rejected</t>
+          <t>Degraded when DB down</t>
         </is>
       </c>
       <c r="D330" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health without token</t>
+          <t>Stop PostgreSQL, call endpoint with valid token</t>
         </is>
       </c>
       <c r="E330" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>200, status: "degraded", database: "error", database_error is non-null</t>
         </is>
       </c>
       <c r="F330" s="4" t="n"/>
@@ -10240,7 +10240,7 @@
     <row r="331">
       <c r="A331" s="4" t="inlineStr">
         <is>
-          <t>TC-1513</t>
+          <t>TC-1512</t>
         </is>
       </c>
       <c r="B331" s="4" t="inlineStr">
@@ -10250,17 +10250,17 @@
       </c>
       <c r="C331" s="4" t="inlineStr">
         <is>
-          <t>Processor role allowed</t>
+          <t>Unauthenticated rejected</t>
         </is>
       </c>
       <c r="D331" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with processor token</t>
+          <t>GET /introspection/system-health without token</t>
         </is>
       </c>
       <c r="E331" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F331" s="4" t="n"/>
@@ -10269,59 +10269,59 @@
       <c r="I331" s="4" t="n"/>
     </row>
     <row r="332">
-      <c r="A332" s="2" t="inlineStr">
+      <c r="A332" s="4" t="inlineStr">
+        <is>
+          <t>TC-1513</t>
+        </is>
+      </c>
+      <c r="B332" s="4" t="inlineStr">
+        <is>
+          <t>12.15 System Health</t>
+        </is>
+      </c>
+      <c r="C332" s="4" t="inlineStr">
+        <is>
+          <t>Processor role allowed</t>
+        </is>
+      </c>
+      <c r="D332" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/system-health with processor token</t>
+        </is>
+      </c>
+      <c r="E332" s="4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F332" s="4" t="n"/>
+      <c r="G332" s="4" t="n"/>
+      <c r="H332" s="4" t="n"/>
+      <c r="I332" s="4" t="n"/>
+    </row>
+    <row r="333">
+      <c r="A333" s="2" t="inlineStr">
         <is>
           <t>§12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
-      <c r="B332" s="2" t="inlineStr">
+      <c r="B333" s="2" t="inlineStr">
         <is>
           <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
-      <c r="C332" s="3" t="n"/>
-      <c r="D332" s="3" t="n"/>
-      <c r="E332" s="3" t="n"/>
-      <c r="F332" s="3" t="n"/>
-      <c r="G332" s="3" t="n"/>
-      <c r="H332" s="3" t="n"/>
-      <c r="I332" s="3" t="n"/>
-    </row>
-    <row r="333">
-      <c r="A333" s="4" t="inlineStr">
-        <is>
-          <t>TC-1511</t>
-        </is>
-      </c>
-      <c r="B333" s="4" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C333" s="4" t="inlineStr">
-        <is>
-          <t>Liveness endpoint is public</t>
-        </is>
-      </c>
-      <c r="D333" s="4" t="inlineStr">
-        <is>
-          <t>GET /health/live without token</t>
-        </is>
-      </c>
-      <c r="E333" s="4" t="inlineStr">
-        <is>
-          <t>200, service reports live</t>
-        </is>
-      </c>
-      <c r="F333" s="4" t="n"/>
-      <c r="G333" s="4" t="n"/>
-      <c r="H333" s="4" t="n"/>
-      <c r="I333" s="4" t="n"/>
+      <c r="C333" s="3" t="n"/>
+      <c r="D333" s="3" t="n"/>
+      <c r="E333" s="3" t="n"/>
+      <c r="F333" s="3" t="n"/>
+      <c r="G333" s="3" t="n"/>
+      <c r="H333" s="3" t="n"/>
+      <c r="I333" s="3" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="4" t="inlineStr">
         <is>
-          <t>TC-1512</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B334" s="4" t="inlineStr">
@@ -10331,17 +10331,17 @@
       </c>
       <c r="C334" s="4" t="inlineStr">
         <is>
-          <t>Readiness endpoint is public</t>
+          <t>Liveness endpoint is public</t>
         </is>
       </c>
       <c r="D334" s="4" t="inlineStr">
         <is>
-          <t>GET /health/ready without token on a healthy system</t>
+          <t>GET /health/live without token</t>
         </is>
       </c>
       <c r="E334" s="4" t="inlineStr">
         <is>
-          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
+          <t>200, service reports live</t>
         </is>
       </c>
       <c r="F334" s="4" t="n"/>
@@ -10352,7 +10352,7 @@
     <row r="335">
       <c r="A335" s="4" t="inlineStr">
         <is>
-          <t>TC-1513</t>
+          <t>TC-1512</t>
         </is>
       </c>
       <c r="B335" s="4" t="inlineStr">
@@ -10362,17 +10362,17 @@
       </c>
       <c r="C335" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports missing database configuration</t>
+          <t>Readiness endpoint is public</t>
         </is>
       </c>
       <c r="D335" s="4" t="inlineStr">
         <is>
-          <t>Clear DB config or test before configuration, then GET /health/ready</t>
+          <t>GET /health/ready without token on a healthy system</t>
         </is>
       </c>
       <c r="E335" s="4" t="inlineStr">
         <is>
-          <t>503, status: "not_ready", reason indicates database is not configured</t>
+          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
         </is>
       </c>
       <c r="F335" s="4" t="n"/>
@@ -10383,7 +10383,7 @@
     <row r="336">
       <c r="A336" s="4" t="inlineStr">
         <is>
-          <t>TC-1514</t>
+          <t>TC-1513</t>
         </is>
       </c>
       <c r="B336" s="4" t="inlineStr">
@@ -10393,17 +10393,17 @@
       </c>
       <c r="C336" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports mount or provider problems</t>
+          <t>Readiness reports missing database configuration</t>
         </is>
       </c>
       <c r="D336" s="4" t="inlineStr">
         <is>
-          <t>Break a configured mount or provider, then GET /health/ready</t>
+          <t>Clear DB config or test before configuration, then GET /health/ready</t>
         </is>
       </c>
       <c r="E336" s="4" t="inlineStr">
         <is>
-          <t>503, response identifies the failing check without using the generic error schema</t>
+          <t>503, status: "not_ready", reason indicates database is not configured</t>
         </is>
       </c>
       <c r="F336" s="4" t="n"/>
@@ -10414,7 +10414,7 @@
     <row r="337">
       <c r="A337" s="4" t="inlineStr">
         <is>
-          <t>TC-1515</t>
+          <t>TC-1514</t>
         </is>
       </c>
       <c r="B337" s="4" t="inlineStr">
@@ -10424,17 +10424,17 @@
       </c>
       <c r="C337" s="4" t="inlineStr">
         <is>
-          <t>Version endpoint is public</t>
+          <t>Readiness reports mount or provider problems</t>
         </is>
       </c>
       <c r="D337" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/version without token</t>
+          <t>Break a configured mount or provider, then GET /health/ready</t>
         </is>
       </c>
       <c r="E337" s="4" t="inlineStr">
         <is>
-          <t>200, returns version/application metadata</t>
+          <t>503, response identifies the failing check without using the generic error schema</t>
         </is>
       </c>
       <c r="F337" s="4" t="n"/>
@@ -10445,7 +10445,7 @@
     <row r="338">
       <c r="A338" s="4" t="inlineStr">
         <is>
-          <t>TC-1516</t>
+          <t>TC-1515</t>
         </is>
       </c>
       <c r="B338" s="4" t="inlineStr">
@@ -10455,17 +10455,17 @@
       </c>
       <c r="C338" s="4" t="inlineStr">
         <is>
-          <t>Readiness remains separate from authenticated system health</t>
+          <t>Version endpoint is public</t>
         </is>
       </c>
       <c r="D338" s="4" t="inlineStr">
         <is>
-          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+          <t>GET /introspection/version without token</t>
         </is>
       </c>
       <c r="E338" s="4" t="inlineStr">
         <is>
-          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+          <t>200, returns version/application metadata</t>
         </is>
       </c>
       <c r="F338" s="4" t="n"/>
@@ -10474,32 +10474,63 @@
       <c r="I338" s="4" t="n"/>
     </row>
     <row r="339">
-      <c r="A339" s="2" t="inlineStr">
+      <c r="A339" s="4" t="inlineStr">
+        <is>
+          <t>TC-1516</t>
+        </is>
+      </c>
+      <c r="B339" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C339" s="4" t="inlineStr">
+        <is>
+          <t>Readiness remains separate from authenticated system health</t>
+        </is>
+      </c>
+      <c r="D339" s="4" t="inlineStr">
+        <is>
+          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+        </is>
+      </c>
+      <c r="E339" s="4" t="inlineStr">
+        <is>
+          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+        </is>
+      </c>
+      <c r="F339" s="4" t="n"/>
+      <c r="G339" s="4" t="n"/>
+      <c r="H339" s="4" t="n"/>
+      <c r="I339" s="4" t="n"/>
+    </row>
+    <row r="340">
+      <c r="A340" s="2" t="inlineStr">
         <is>
           <t>§12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="B339" s="2" t="inlineStr">
+      <c r="B340" s="2" t="inlineStr">
         <is>
           <t>12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="C339" s="3" t="n"/>
-      <c r="D339" s="3" t="n"/>
-      <c r="E339" s="3" t="n"/>
-      <c r="F339" s="3" t="n"/>
-      <c r="G339" s="3" t="n"/>
-      <c r="H339" s="3" t="n"/>
-      <c r="I339" s="3" t="n"/>
-    </row>
-    <row r="341">
-      <c r="A341" s="5" t="inlineStr">
+      <c r="C340" s="3" t="n"/>
+      <c r="D340" s="3" t="n"/>
+      <c r="E340" s="3" t="n"/>
+      <c r="F340" s="3" t="n"/>
+      <c r="G340" s="3" t="n"/>
+      <c r="H340" s="3" t="n"/>
+      <c r="I340" s="3" t="n"/>
+    </row>
+    <row r="342">
+      <c r="A342" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B341" s="5" t="n">
-        <v>311</v>
+      <c r="B342" s="5" t="n">
+        <v>312</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Prevent demo setup reconciliation from failing on redundant resets
Skip reapplying the setup account password during demo-mode setup reconciliation,
ignore no-op ECUBE group appends for users already in the target group, and treat
demo audit-write failures as logged diagnostics instead of setup-breaking errors.
Sync the operator and QA docs with the new demo setup and recovery behavior.
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I344"/>
+  <dimension ref="A1:I345"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7286,7 +7286,7 @@
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
         <is>
-          <t>TC-928</t>
+          <t>TC-929</t>
         </is>
       </c>
       <c r="B233" s="4" t="inlineStr">
@@ -7296,17 +7296,17 @@
       </c>
       <c r="C233" s="4" t="inlineStr">
         <is>
-          <t>Audit trail exists</t>
+          <t>Demo setup succeeds when the setup account is already the demo admin</t>
         </is>
       </c>
       <c r="D233" s="4" t="inlineStr">
         <is>
-          <t>Query audit logs for demo bootstrap and denied password actions</t>
+          <t>Enable demo mode, complete setup through the wizard using the configured demo admin account, then inspect /etc/passwd, /etc/group, and the login page</t>
         </is>
       </c>
       <c r="E233" s="4" t="inlineStr">
         <is>
-          <t>Audit entries exist for seed, reset, and authorization denial events</t>
+          <t>Setup completes without the generic demo-seeding failure banner, the remaining configured demo users are created, and the login page shows the shared demo credentials without requiring a restart or retry</t>
         </is>
       </c>
       <c r="F233" s="4" t="n"/>
@@ -7317,7 +7317,7 @@
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
         <is>
-          <t>TC-929</t>
+          <t>TC-930</t>
         </is>
       </c>
       <c r="B234" s="4" t="inlineStr">
@@ -7327,17 +7327,17 @@
       </c>
       <c r="C234" s="4" t="inlineStr">
         <is>
-          <t>No sample content is staged automatically</t>
+          <t>Audit trail exists</t>
         </is>
       </c>
       <c r="D234" s="4" t="inlineStr">
         <is>
-          <t>Review the install root and demo metadata after install.sh --demo</t>
+          <t>Query audit logs for demo bootstrap and denied password actions</t>
         </is>
       </c>
       <c r="E234" s="4" t="inlineStr">
         <is>
-          <t>Demo bootstrap affects demo accounts, login guidance, and role state only; it does not stage sample projects, files, USB state, or network mounts</t>
+          <t>Audit entries exist for seed, reset, and authorization denial events</t>
         </is>
       </c>
       <c r="F234" s="4" t="n"/>
@@ -7346,59 +7346,59 @@
       <c r="I234" s="4" t="n"/>
     </row>
     <row r="235">
-      <c r="A235" s="2" t="inlineStr">
+      <c r="A235" s="4" t="inlineStr">
+        <is>
+          <t>TC-931</t>
+        </is>
+      </c>
+      <c r="B235" s="4" t="inlineStr">
+        <is>
+          <t>12.9.2 Demo Mode Rollout Validation Checklist</t>
+        </is>
+      </c>
+      <c r="C235" s="4" t="inlineStr">
+        <is>
+          <t>No sample content is staged automatically</t>
+        </is>
+      </c>
+      <c r="D235" s="4" t="inlineStr">
+        <is>
+          <t>Review the install root and demo metadata after install.sh --demo</t>
+        </is>
+      </c>
+      <c r="E235" s="4" t="inlineStr">
+        <is>
+          <t>Demo bootstrap affects demo accounts, login guidance, and role state only; it does not stage sample projects, files, USB state, or network mounts</t>
+        </is>
+      </c>
+      <c r="F235" s="4" t="n"/>
+      <c r="G235" s="4" t="n"/>
+      <c r="H235" s="4" t="n"/>
+      <c r="I235" s="4" t="n"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="inlineStr">
         <is>
           <t>§12.10 Admin Log Viewing API</t>
         </is>
       </c>
-      <c r="B235" s="2" t="inlineStr">
+      <c r="B236" s="2" t="inlineStr">
         <is>
           <t>12.10 Admin Log Viewing API</t>
         </is>
       </c>
-      <c r="C235" s="3" t="n"/>
-      <c r="D235" s="3" t="n"/>
-      <c r="E235" s="3" t="n"/>
-      <c r="F235" s="3" t="n"/>
-      <c r="G235" s="3" t="n"/>
-      <c r="H235" s="3" t="n"/>
-      <c r="I235" s="3" t="n"/>
-    </row>
-    <row r="236">
-      <c r="A236" s="4" t="inlineStr">
-        <is>
-          <t>TC-1001</t>
-        </is>
-      </c>
-      <c r="B236" s="4" t="inlineStr">
-        <is>
-          <t>12.10 Admin Log Viewing API</t>
-        </is>
-      </c>
-      <c r="C236" s="4" t="inlineStr">
-        <is>
-          <t>View logs — unauthenticated</t>
-        </is>
-      </c>
-      <c r="D236" s="4" t="inlineStr">
-        <is>
-          <t>GET /admin/logs/view without token</t>
-        </is>
-      </c>
-      <c r="E236" s="4" t="inlineStr">
-        <is>
-          <t>401, UNAUTHORIZED</t>
-        </is>
-      </c>
-      <c r="F236" s="4" t="n"/>
-      <c r="G236" s="4" t="n"/>
-      <c r="H236" s="4" t="n"/>
-      <c r="I236" s="4" t="n"/>
+      <c r="C236" s="3" t="n"/>
+      <c r="D236" s="3" t="n"/>
+      <c r="E236" s="3" t="n"/>
+      <c r="F236" s="3" t="n"/>
+      <c r="G236" s="3" t="n"/>
+      <c r="H236" s="3" t="n"/>
+      <c r="I236" s="3" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="4" t="inlineStr">
         <is>
-          <t>TC-1002</t>
+          <t>TC-1001</t>
         </is>
       </c>
       <c r="B237" s="4" t="inlineStr">
@@ -7408,17 +7408,17 @@
       </c>
       <c r="C237" s="4" t="inlineStr">
         <is>
-          <t>View logs — non-admin denied</t>
+          <t>View logs — unauthenticated</t>
         </is>
       </c>
       <c r="D237" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/view with manager/processor/auditor token</t>
+          <t>GET /admin/logs/view without token</t>
         </is>
       </c>
       <c r="E237" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN; denied audit event recorded</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F237" s="4" t="n"/>
@@ -7429,7 +7429,7 @@
     <row r="238">
       <c r="A238" s="4" t="inlineStr">
         <is>
-          <t>TC-1003</t>
+          <t>TC-1002</t>
         </is>
       </c>
       <c r="B238" s="4" t="inlineStr">
@@ -7439,17 +7439,17 @@
       </c>
       <c r="C238" s="4" t="inlineStr">
         <is>
-          <t>View logs — unknown source</t>
+          <t>View logs — non-admin denied</t>
         </is>
       </c>
       <c r="D238" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/view?source=unknown with admin token</t>
+          <t>GET /admin/logs/view with manager/processor/auditor token</t>
         </is>
       </c>
       <c r="E238" s="4" t="inlineStr">
         <is>
-          <t>404, unknown log source</t>
+          <t>403, FORBIDDEN; denied audit event recorded</t>
         </is>
       </c>
       <c r="F238" s="4" t="n"/>
@@ -7460,7 +7460,7 @@
     <row r="239">
       <c r="A239" s="4" t="inlineStr">
         <is>
-          <t>TC-1004</t>
+          <t>TC-1003</t>
         </is>
       </c>
       <c r="B239" s="4" t="inlineStr">
@@ -7470,17 +7470,17 @@
       </c>
       <c r="C239" s="4" t="inlineStr">
         <is>
-          <t>View logs — baseline response shape</t>
+          <t>View logs — unknown source</t>
         </is>
       </c>
       <c r="D239" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/view?source=app&amp;limit=5&amp;offset=0</t>
+          <t>GET /admin/logs/view?source=unknown with admin token</t>
         </is>
       </c>
       <c r="E239" s="4" t="inlineStr">
         <is>
-          <t>200 with object fields: source, fetched_at, file_modified_at, offset, limit, returned, has_more, lines</t>
+          <t>404, unknown log source</t>
         </is>
       </c>
       <c r="F239" s="4" t="n"/>
@@ -7491,7 +7491,7 @@
     <row r="240">
       <c r="A240" s="4" t="inlineStr">
         <is>
-          <t>TC-1005</t>
+          <t>TC-1004</t>
         </is>
       </c>
       <c r="B240" s="4" t="inlineStr">
@@ -7501,17 +7501,17 @@
       </c>
       <c r="C240" s="4" t="inlineStr">
         <is>
-          <t>View logs — source path redaction</t>
+          <t>View logs — baseline response shape</t>
         </is>
       </c>
       <c r="D240" s="4" t="inlineStr">
         <is>
-          <t>Inspect source.path in successful response</t>
+          <t>GET /admin/logs/view?source=app&amp;limit=5&amp;offset=0</t>
         </is>
       </c>
       <c r="E240" s="4" t="inlineStr">
         <is>
-          <t>Basename only (for example app.log), no absolute filesystem path</t>
+          <t>200 with object fields: source, fetched_at, file_modified_at, offset, limit, returned, has_more, lines</t>
         </is>
       </c>
       <c r="F240" s="4" t="n"/>
@@ -7522,7 +7522,7 @@
     <row r="241">
       <c r="A241" s="4" t="inlineStr">
         <is>
-          <t>TC-1006</t>
+          <t>TC-1005</t>
         </is>
       </c>
       <c r="B241" s="4" t="inlineStr">
@@ -7532,17 +7532,17 @@
       </c>
       <c r="C241" s="4" t="inlineStr">
         <is>
-          <t>View logs — offset pagination</t>
+          <t>View logs — source path redaction</t>
         </is>
       </c>
       <c r="D241" s="4" t="inlineStr">
         <is>
-          <t>Create known numbered lines, call GET /admin/logs/view?limit=5&amp;offset=2</t>
+          <t>Inspect source.path in successful response</t>
         </is>
       </c>
       <c r="E241" s="4" t="inlineStr">
         <is>
-          <t>Returns correct window from tail semantics, returned &lt;= limit</t>
+          <t>Basename only (for example app.log), no absolute filesystem path</t>
         </is>
       </c>
       <c r="F241" s="4" t="n"/>
@@ -7553,7 +7553,7 @@
     <row r="242">
       <c r="A242" s="4" t="inlineStr">
         <is>
-          <t>TC-1007</t>
+          <t>TC-1006</t>
         </is>
       </c>
       <c r="B242" s="4" t="inlineStr">
@@ -7563,17 +7563,17 @@
       </c>
       <c r="C242" s="4" t="inlineStr">
         <is>
-          <t>View logs — reverse ordering</t>
+          <t>View logs — offset pagination</t>
         </is>
       </c>
       <c r="D242" s="4" t="inlineStr">
         <is>
-          <t>Compare reverse=false vs reverse=true on same query</t>
+          <t>Create known numbered lines, call GET /admin/logs/view?limit=5&amp;offset=2</t>
         </is>
       </c>
       <c r="E242" s="4" t="inlineStr">
         <is>
-          <t>Same selected window; line order is inverted when reverse=true</t>
+          <t>Returns correct window from tail semantics, returned &lt;= limit</t>
         </is>
       </c>
       <c r="F242" s="4" t="n"/>
@@ -7584,7 +7584,7 @@
     <row r="243">
       <c r="A243" s="4" t="inlineStr">
         <is>
-          <t>TC-1008</t>
+          <t>TC-1007</t>
         </is>
       </c>
       <c r="B243" s="4" t="inlineStr">
@@ -7594,17 +7594,17 @@
       </c>
       <c r="C243" s="4" t="inlineStr">
         <is>
-          <t>View logs — search filtering</t>
+          <t>View logs — reverse ordering</t>
         </is>
       </c>
       <c r="D243" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/view?search=error</t>
+          <t>Compare reverse=false vs reverse=true on same query</t>
         </is>
       </c>
       <c r="E243" s="4" t="inlineStr">
         <is>
-          <t>Only matching lines are returned (case-insensitive contains)</t>
+          <t>Same selected window; line order is inverted when reverse=true</t>
         </is>
       </c>
       <c r="F243" s="4" t="n"/>
@@ -7615,7 +7615,7 @@
     <row r="244">
       <c r="A244" s="4" t="inlineStr">
         <is>
-          <t>TC-1009</t>
+          <t>TC-1008</t>
         </is>
       </c>
       <c r="B244" s="4" t="inlineStr">
@@ -7625,17 +7625,17 @@
       </c>
       <c r="C244" s="4" t="inlineStr">
         <is>
-          <t>View logs — sensitive value redaction</t>
+          <t>View logs — search filtering</t>
         </is>
       </c>
       <c r="D244" s="4" t="inlineStr">
         <is>
-          <t>Include tokens/passwords in source log lines, call view endpoint</t>
+          <t>GET /admin/logs/view?search=error</t>
         </is>
       </c>
       <c r="E244" s="4" t="inlineStr">
         <is>
-          <t>Sensitive values replaced with redacted markers in lines[].content</t>
+          <t>Only matching lines are returned (case-insensitive contains)</t>
         </is>
       </c>
       <c r="F244" s="4" t="n"/>
@@ -7646,7 +7646,7 @@
     <row r="245">
       <c r="A245" s="4" t="inlineStr">
         <is>
-          <t>TC-1010</t>
+          <t>TC-1009</t>
         </is>
       </c>
       <c r="B245" s="4" t="inlineStr">
@@ -7656,17 +7656,17 @@
       </c>
       <c r="C245" s="4" t="inlineStr">
         <is>
-          <t>View logs — success audit</t>
+          <t>View logs — sensitive value redaction</t>
         </is>
       </c>
       <c r="D245" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=LOG_LINES_VIEWED after successful view</t>
+          <t>Include tokens/passwords in source log lines, call view endpoint</t>
         </is>
       </c>
       <c r="E245" s="4" t="inlineStr">
         <is>
-          <t>Audit entry includes source, limit, offset, returned, has_more, and basename log_file</t>
+          <t>Sensitive values replaced with redacted markers in lines[].content</t>
         </is>
       </c>
       <c r="F245" s="4" t="n"/>
@@ -7677,7 +7677,7 @@
     <row r="246">
       <c r="A246" s="4" t="inlineStr">
         <is>
-          <t>TC-1011</t>
+          <t>TC-1010</t>
         </is>
       </c>
       <c r="B246" s="4" t="inlineStr">
@@ -7687,17 +7687,17 @@
       </c>
       <c r="C246" s="4" t="inlineStr">
         <is>
-          <t>List logs — unauthenticated</t>
+          <t>View logs — success audit</t>
         </is>
       </c>
       <c r="D246" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs without token</t>
+          <t>GET /audit?action=LOG_LINES_VIEWED after successful view</t>
         </is>
       </c>
       <c r="E246" s="4" t="inlineStr">
         <is>
-          <t>401, UNAUTHORIZED</t>
+          <t>Audit entry includes source, limit, offset, returned, has_more, and basename log_file</t>
         </is>
       </c>
       <c r="F246" s="4" t="n"/>
@@ -7708,7 +7708,7 @@
     <row r="247">
       <c r="A247" s="4" t="inlineStr">
         <is>
-          <t>TC-1012</t>
+          <t>TC-1011</t>
         </is>
       </c>
       <c r="B247" s="4" t="inlineStr">
@@ -7718,17 +7718,17 @@
       </c>
       <c r="C247" s="4" t="inlineStr">
         <is>
-          <t>List logs — non-admin denied</t>
+          <t>List logs — unauthenticated</t>
         </is>
       </c>
       <c r="D247" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs with non-admin token</t>
+          <t>GET /admin/logs without token</t>
         </is>
       </c>
       <c r="E247" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN; denied audit event recorded</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F247" s="4" t="n"/>
@@ -7739,7 +7739,7 @@
     <row r="248">
       <c r="A248" s="4" t="inlineStr">
         <is>
-          <t>TC-1013</t>
+          <t>TC-1012</t>
         </is>
       </c>
       <c r="B248" s="4" t="inlineStr">
@@ -7749,17 +7749,17 @@
       </c>
       <c r="C248" s="4" t="inlineStr">
         <is>
-          <t>List logs — response envelope</t>
+          <t>List logs — non-admin denied</t>
         </is>
       </c>
       <c r="D248" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs with admin token and file logging configured</t>
+          <t>GET /admin/logs with non-admin token</t>
         </is>
       </c>
       <c r="E248" s="4" t="inlineStr">
         <is>
-          <t>200 object with log_files array and total_size; no log_directory field in response</t>
+          <t>403, FORBIDDEN; denied audit event recorded</t>
         </is>
       </c>
       <c r="F248" s="4" t="n"/>
@@ -7770,7 +7770,7 @@
     <row r="249">
       <c r="A249" s="4" t="inlineStr">
         <is>
-          <t>TC-1014</t>
+          <t>TC-1013</t>
         </is>
       </c>
       <c r="B249" s="4" t="inlineStr">
@@ -7780,17 +7780,17 @@
       </c>
       <c r="C249" s="4" t="inlineStr">
         <is>
-          <t>Download log — non-admin denied</t>
+          <t>List logs — response envelope</t>
         </is>
       </c>
       <c r="D249" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/app.log with non-admin token</t>
+          <t>GET /admin/logs with admin token and file logging configured</t>
         </is>
       </c>
       <c r="E249" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN; denied audit event recorded</t>
+          <t>200 object with log_files array and total_size; no log_directory field in response</t>
         </is>
       </c>
       <c r="F249" s="4" t="n"/>
@@ -7801,7 +7801,7 @@
     <row r="250">
       <c r="A250" s="4" t="inlineStr">
         <is>
-          <t>TC-1015</t>
+          <t>TC-1014</t>
         </is>
       </c>
       <c r="B250" s="4" t="inlineStr">
@@ -7811,17 +7811,17 @@
       </c>
       <c r="C250" s="4" t="inlineStr">
         <is>
-          <t>Download log — path traversal blocked</t>
+          <t>Download log — non-admin denied</t>
         </is>
       </c>
       <c r="D250" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/../../../etc/passwd</t>
+          <t>GET /admin/logs/app.log with non-admin token</t>
         </is>
       </c>
       <c r="E250" s="4" t="inlineStr">
         <is>
-          <t>Rejected (400/404/422), no file disclosure</t>
+          <t>403, FORBIDDEN; denied audit event recorded</t>
         </is>
       </c>
       <c r="F250" s="4" t="n"/>
@@ -7832,7 +7832,7 @@
     <row r="251">
       <c r="A251" s="4" t="inlineStr">
         <is>
-          <t>TC-1016</t>
+          <t>TC-1015</t>
         </is>
       </c>
       <c r="B251" s="4" t="inlineStr">
@@ -7842,17 +7842,17 @@
       </c>
       <c r="C251" s="4" t="inlineStr">
         <is>
-          <t>Download log — success audit</t>
+          <t>Download log — path traversal blocked</t>
         </is>
       </c>
       <c r="D251" s="4" t="inlineStr">
         <is>
-          <t>Download valid file as admin, then query audit</t>
+          <t>GET /admin/logs/../../../etc/passwd</t>
         </is>
       </c>
       <c r="E251" s="4" t="inlineStr">
         <is>
-          <t>LOG_FILE_DOWNLOADED entry includes requested filename</t>
+          <t>Rejected (400/404/422), no file disclosure</t>
         </is>
       </c>
       <c r="F251" s="4" t="n"/>
@@ -7861,59 +7861,59 @@
       <c r="I251" s="4" t="n"/>
     </row>
     <row r="252">
-      <c r="A252" s="2" t="inlineStr">
+      <c r="A252" s="4" t="inlineStr">
+        <is>
+          <t>TC-1016</t>
+        </is>
+      </c>
+      <c r="B252" s="4" t="inlineStr">
+        <is>
+          <t>12.10 Admin Log Viewing API</t>
+        </is>
+      </c>
+      <c r="C252" s="4" t="inlineStr">
+        <is>
+          <t>Download log — success audit</t>
+        </is>
+      </c>
+      <c r="D252" s="4" t="inlineStr">
+        <is>
+          <t>Download valid file as admin, then query audit</t>
+        </is>
+      </c>
+      <c r="E252" s="4" t="inlineStr">
+        <is>
+          <t>LOG_FILE_DOWNLOADED entry includes requested filename</t>
+        </is>
+      </c>
+      <c r="F252" s="4" t="n"/>
+      <c r="G252" s="4" t="n"/>
+      <c r="H252" s="4" t="n"/>
+      <c r="I252" s="4" t="n"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="inlineStr">
         <is>
           <t>§12.10.1 Runtime Configuration</t>
         </is>
       </c>
-      <c r="B252" s="2" t="inlineStr">
+      <c r="B253" s="2" t="inlineStr">
         <is>
           <t>12.10.1 Runtime Configuration</t>
         </is>
       </c>
-      <c r="C252" s="3" t="n"/>
-      <c r="D252" s="3" t="n"/>
-      <c r="E252" s="3" t="n"/>
-      <c r="F252" s="3" t="n"/>
-      <c r="G252" s="3" t="n"/>
-      <c r="H252" s="3" t="n"/>
-      <c r="I252" s="3" t="n"/>
-    </row>
-    <row r="253">
-      <c r="A253" s="4" t="inlineStr">
-        <is>
-          <t>TC-1011</t>
-        </is>
-      </c>
-      <c r="B253" s="4" t="inlineStr">
-        <is>
-          <t>12.10.1 Runtime Configuration</t>
-        </is>
-      </c>
-      <c r="C253" s="4" t="inlineStr">
-        <is>
-          <t>Get configuration — admin</t>
-        </is>
-      </c>
-      <c r="D253" s="4" t="inlineStr">
-        <is>
-          <t>GET /admin/configuration with admin token</t>
-        </is>
-      </c>
-      <c r="E253" s="4" t="inlineStr">
-        <is>
-          <t>200, response includes editable settings such as log_level and DB pool fields</t>
-        </is>
-      </c>
-      <c r="F253" s="4" t="n"/>
-      <c r="G253" s="4" t="n"/>
-      <c r="H253" s="4" t="n"/>
-      <c r="I253" s="4" t="n"/>
+      <c r="C253" s="3" t="n"/>
+      <c r="D253" s="3" t="n"/>
+      <c r="E253" s="3" t="n"/>
+      <c r="F253" s="3" t="n"/>
+      <c r="G253" s="3" t="n"/>
+      <c r="H253" s="3" t="n"/>
+      <c r="I253" s="3" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="4" t="inlineStr">
         <is>
-          <t>TC-1012</t>
+          <t>TC-1011</t>
         </is>
       </c>
       <c r="B254" s="4" t="inlineStr">
@@ -7923,17 +7923,17 @@
       </c>
       <c r="C254" s="4" t="inlineStr">
         <is>
-          <t>Get configuration — non-admin denied</t>
+          <t>Get configuration — admin</t>
         </is>
       </c>
       <c r="D254" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/configuration with manager/processor/auditor token</t>
+          <t>GET /admin/configuration with admin token</t>
         </is>
       </c>
       <c r="E254" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>200, response includes editable settings such as log_level and DB pool fields</t>
         </is>
       </c>
       <c r="F254" s="4" t="n"/>
@@ -7944,7 +7944,7 @@
     <row r="255">
       <c r="A255" s="4" t="inlineStr">
         <is>
-          <t>TC-1013</t>
+          <t>TC-1012</t>
         </is>
       </c>
       <c r="B255" s="4" t="inlineStr">
@@ -7954,17 +7954,17 @@
       </c>
       <c r="C255" s="4" t="inlineStr">
         <is>
-          <t>Update runtime-only setting</t>
+          <t>Get configuration — non-admin denied</t>
         </is>
       </c>
       <c r="D255" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/configuration with {"log_level": "DEBUG"}</t>
+          <t>GET /admin/configuration with manager/processor/auditor token</t>
         </is>
       </c>
       <c r="E255" s="4" t="inlineStr">
         <is>
-          <t>200, status: "updated", changed_settings includes log_level, restart_required is false</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F255" s="4" t="n"/>
@@ -7975,7 +7975,7 @@
     <row r="256">
       <c r="A256" s="4" t="inlineStr">
         <is>
-          <t>TC-1014</t>
+          <t>TC-1013</t>
         </is>
       </c>
       <c r="B256" s="4" t="inlineStr">
@@ -7985,17 +7985,17 @@
       </c>
       <c r="C256" s="4" t="inlineStr">
         <is>
-          <t>Update restart-required setting</t>
+          <t>Update runtime-only setting</t>
         </is>
       </c>
       <c r="D256" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/configuration with {"db_pool_recycle_seconds": 120}</t>
+          <t>PUT /admin/configuration with {"log_level": "DEBUG"}</t>
         </is>
       </c>
       <c r="E256" s="4" t="inlineStr">
         <is>
-          <t>200, restart_required is true and the response lists the restart-required setting</t>
+          <t>200, status: "updated", changed_settings includes log_level, restart_required is false</t>
         </is>
       </c>
       <c r="F256" s="4" t="n"/>
@@ -8006,7 +8006,7 @@
     <row r="257">
       <c r="A257" s="4" t="inlineStr">
         <is>
-          <t>TC-1015</t>
+          <t>TC-1014</t>
         </is>
       </c>
       <c r="B257" s="4" t="inlineStr">
@@ -8016,17 +8016,17 @@
       </c>
       <c r="C257" s="4" t="inlineStr">
         <is>
-          <t>Reject empty update payload</t>
+          <t>Update restart-required setting</t>
         </is>
       </c>
       <c r="D257" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/configuration with {}</t>
+          <t>PUT /admin/configuration with {"db_pool_recycle_seconds": 120}</t>
         </is>
       </c>
       <c r="E257" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>200, restart_required is true and the response lists the restart-required setting</t>
         </is>
       </c>
       <c r="F257" s="4" t="n"/>
@@ -8037,7 +8037,7 @@
     <row r="258">
       <c r="A258" s="4" t="inlineStr">
         <is>
-          <t>TC-1016</t>
+          <t>TC-1015</t>
         </is>
       </c>
       <c r="B258" s="4" t="inlineStr">
@@ -8047,17 +8047,17 @@
       </c>
       <c r="C258" s="4" t="inlineStr">
         <is>
-          <t>Reject unwritable log file path</t>
+          <t>Reject empty update payload</t>
         </is>
       </c>
       <c r="D258" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/configuration with {"log_file": "/var/log/ecube/denied.log"} when path is not writable</t>
+          <t>PUT /admin/configuration with {}</t>
         </is>
       </c>
       <c r="E258" s="4" t="inlineStr">
         <is>
-          <t>422, message indicates the log file cannot be written</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F258" s="4" t="n"/>
@@ -8068,7 +8068,7 @@
     <row r="259">
       <c r="A259" s="4" t="inlineStr">
         <is>
-          <t>TC-1017</t>
+          <t>TC-1016</t>
         </is>
       </c>
       <c r="B259" s="4" t="inlineStr">
@@ -8078,17 +8078,17 @@
       </c>
       <c r="C259" s="4" t="inlineStr">
         <is>
-          <t>Configuration update audit trail</t>
+          <t>Reject unwritable log file path</t>
         </is>
       </c>
       <c r="D259" s="4" t="inlineStr">
         <is>
-          <t>Update configuration, then query GET /audit?action=CONFIGURATION_UPDATED</t>
+          <t>PUT /admin/configuration with {"log_file": "/var/log/ecube/denied.log"} when path is not writable</t>
         </is>
       </c>
       <c r="E259" s="4" t="inlineStr">
         <is>
-          <t>Audit entry lists changed settings without leaking sensitive paths or secrets</t>
+          <t>422, message indicates the log file cannot be written</t>
         </is>
       </c>
       <c r="F259" s="4" t="n"/>
@@ -8099,7 +8099,7 @@
     <row r="260">
       <c r="A260" s="4" t="inlineStr">
         <is>
-          <t>TC-1018</t>
+          <t>TC-1017</t>
         </is>
       </c>
       <c r="B260" s="4" t="inlineStr">
@@ -8109,17 +8109,17 @@
       </c>
       <c r="C260" s="4" t="inlineStr">
         <is>
-          <t>Restart requires confirmation</t>
+          <t>Configuration update audit trail</t>
         </is>
       </c>
       <c r="D260" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/configuration/restart with {"confirm": false}</t>
+          <t>Update configuration, then query GET /audit?action=CONFIGURATION_UPDATED</t>
         </is>
       </c>
       <c r="E260" s="4" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>Audit entry lists changed settings without leaking sensitive paths or secrets</t>
         </is>
       </c>
       <c r="F260" s="4" t="n"/>
@@ -8130,7 +8130,7 @@
     <row r="261">
       <c r="A261" s="4" t="inlineStr">
         <is>
-          <t>TC-1019</t>
+          <t>TC-1018</t>
         </is>
       </c>
       <c r="B261" s="4" t="inlineStr">
@@ -8140,17 +8140,17 @@
       </c>
       <c r="C261" s="4" t="inlineStr">
         <is>
-          <t>Restart request accepted when confirmed</t>
+          <t>Restart requires confirmation</t>
         </is>
       </c>
       <c r="D261" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/configuration/restart with {"confirm": true}</t>
+          <t>POST /admin/configuration/restart with {"confirm": false}</t>
         </is>
       </c>
       <c r="E261" s="4" t="inlineStr">
         <is>
-          <t>200, status: "restart_requested", service: "ecube"</t>
+          <t>400</t>
         </is>
       </c>
       <c r="F261" s="4" t="n"/>
@@ -8161,7 +8161,7 @@
     <row r="262">
       <c r="A262" s="4" t="inlineStr">
         <is>
-          <t>TC-1020</t>
+          <t>TC-1019</t>
         </is>
       </c>
       <c r="B262" s="4" t="inlineStr">
@@ -8171,17 +8171,17 @@
       </c>
       <c r="C262" s="4" t="inlineStr">
         <is>
-          <t>Accept callback payload allowlist and mapping</t>
+          <t>Restart request accepted when confirmed</t>
         </is>
       </c>
       <c r="D262" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/configuration with {"callback_payload_fields": ["event", "project_id"], "callback_payload_field_map": {"type": "event", "project": "project_id"}}</t>
+          <t>POST /admin/configuration/restart with {"confirm": true}</t>
         </is>
       </c>
       <c r="E262" s="4" t="inlineStr">
         <is>
-          <t>200, changed settings include both callback payload fields</t>
+          <t>200, status: "restart_requested", service: "ecube"</t>
         </is>
       </c>
       <c r="F262" s="4" t="n"/>
@@ -8192,7 +8192,7 @@
     <row r="263">
       <c r="A263" s="4" t="inlineStr">
         <is>
-          <t>TC-1021</t>
+          <t>TC-1020</t>
         </is>
       </c>
       <c r="B263" s="4" t="inlineStr">
@@ -8202,17 +8202,17 @@
       </c>
       <c r="C263" s="4" t="inlineStr">
         <is>
-          <t>Reject invalid callback payload mapping</t>
+          <t>Accept callback payload allowlist and mapping</t>
         </is>
       </c>
       <c r="D263" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/configuration with {"callback_payload_field_map": {"summary": "${unknown_field}"}}</t>
+          <t>PUT /admin/configuration with {"callback_payload_fields": ["event", "project_id"], "callback_payload_field_map": {"type": "event", "project": "project_id"}}</t>
         </is>
       </c>
       <c r="E263" s="4" t="inlineStr">
         <is>
-          <t>422, validation error identifies the invalid mapping source field</t>
+          <t>200, changed settings include both callback payload fields</t>
         </is>
       </c>
       <c r="F263" s="4" t="n"/>
@@ -8221,59 +8221,59 @@
       <c r="I263" s="4" t="n"/>
     </row>
     <row r="264">
-      <c r="A264" s="2" t="inlineStr">
+      <c r="A264" s="4" t="inlineStr">
+        <is>
+          <t>TC-1021</t>
+        </is>
+      </c>
+      <c r="B264" s="4" t="inlineStr">
+        <is>
+          <t>12.10.1 Runtime Configuration</t>
+        </is>
+      </c>
+      <c r="C264" s="4" t="inlineStr">
+        <is>
+          <t>Reject invalid callback payload mapping</t>
+        </is>
+      </c>
+      <c r="D264" s="4" t="inlineStr">
+        <is>
+          <t>PUT /admin/configuration with {"callback_payload_field_map": {"summary": "${unknown_field}"}}</t>
+        </is>
+      </c>
+      <c r="E264" s="4" t="inlineStr">
+        <is>
+          <t>422, validation error identifies the invalid mapping source field</t>
+        </is>
+      </c>
+      <c r="F264" s="4" t="n"/>
+      <c r="G264" s="4" t="n"/>
+      <c r="H264" s="4" t="n"/>
+      <c r="I264" s="4" t="n"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="inlineStr">
         <is>
           <t>§12.10.2 Help System</t>
         </is>
       </c>
-      <c r="B264" s="2" t="inlineStr">
+      <c r="B265" s="2" t="inlineStr">
         <is>
           <t>12.10.2 Help System</t>
         </is>
       </c>
-      <c r="C264" s="3" t="n"/>
-      <c r="D264" s="3" t="n"/>
-      <c r="E264" s="3" t="n"/>
-      <c r="F264" s="3" t="n"/>
-      <c r="G264" s="3" t="n"/>
-      <c r="H264" s="3" t="n"/>
-      <c r="I264" s="3" t="n"/>
-    </row>
-    <row r="265">
-      <c r="A265" s="4" t="inlineStr">
-        <is>
-          <t>TC-1021</t>
-        </is>
-      </c>
-      <c r="B265" s="4" t="inlineStr">
-        <is>
-          <t>12.10.2 Help System</t>
-        </is>
-      </c>
-      <c r="C265" s="4" t="inlineStr">
-        <is>
-          <t>Help trigger is visible in authenticated shell</t>
-        </is>
-      </c>
-      <c r="D265" s="4" t="inlineStr">
-        <is>
-          <t>Sign in to the application and inspect the shell/header</t>
-        </is>
-      </c>
-      <c r="E265" s="4" t="inlineStr">
-        <is>
-          <t>A Help trigger is visible without navigating away from the current page</t>
-        </is>
-      </c>
-      <c r="F265" s="4" t="n"/>
-      <c r="G265" s="4" t="n"/>
-      <c r="H265" s="4" t="n"/>
-      <c r="I265" s="4" t="n"/>
+      <c r="C265" s="3" t="n"/>
+      <c r="D265" s="3" t="n"/>
+      <c r="E265" s="3" t="n"/>
+      <c r="F265" s="3" t="n"/>
+      <c r="G265" s="3" t="n"/>
+      <c r="H265" s="3" t="n"/>
+      <c r="I265" s="3" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="4" t="inlineStr">
         <is>
-          <t>TC-1022</t>
+          <t>TC-1021</t>
         </is>
       </c>
       <c r="B266" s="4" t="inlineStr">
@@ -8283,17 +8283,17 @@
       </c>
       <c r="C266" s="4" t="inlineStr">
         <is>
-          <t>Help opens in-app</t>
+          <t>Help trigger is visible in authenticated shell</t>
         </is>
       </c>
       <c r="D266" s="4" t="inlineStr">
         <is>
-          <t>Activate the Help trigger from any primary page</t>
+          <t>Sign in to the application and inspect the shell/header</t>
         </is>
       </c>
       <c r="E266" s="4" t="inlineStr">
         <is>
-          <t>Help opens in a modal or equivalent in-app panel</t>
+          <t>A Help trigger is visible without navigating away from the current page</t>
         </is>
       </c>
       <c r="F266" s="4" t="n"/>
@@ -8304,7 +8304,7 @@
     <row r="267">
       <c r="A267" s="4" t="inlineStr">
         <is>
-          <t>TC-1023</t>
+          <t>TC-1022</t>
         </is>
       </c>
       <c r="B267" s="4" t="inlineStr">
@@ -8314,17 +8314,17 @@
       </c>
       <c r="C267" s="4" t="inlineStr">
         <is>
-          <t>Help does not break current workflow context</t>
+          <t>Help opens in-app</t>
         </is>
       </c>
       <c r="D267" s="4" t="inlineStr">
         <is>
-          <t>Open Help while on Drives, Mounts, Jobs, or Audit, then close it</t>
+          <t>Activate the Help trigger from any primary page</t>
         </is>
       </c>
       <c r="E267" s="4" t="inlineStr">
         <is>
-          <t>Closing Help returns to the same page and preserved workflow context</t>
+          <t>Help opens in a modal or equivalent in-app panel</t>
         </is>
       </c>
       <c r="F267" s="4" t="n"/>
@@ -8335,7 +8335,7 @@
     <row r="268">
       <c r="A268" s="4" t="inlineStr">
         <is>
-          <t>TC-1024</t>
+          <t>TC-1023</t>
         </is>
       </c>
       <c r="B268" s="4" t="inlineStr">
@@ -8345,17 +8345,17 @@
       </c>
       <c r="C268" s="4" t="inlineStr">
         <is>
-          <t>Help content is curated and user-facing</t>
+          <t>Help does not break current workflow context</t>
         </is>
       </c>
       <c r="D268" s="4" t="inlineStr">
         <is>
-          <t>Review Help content in the modal</t>
+          <t>Open Help while on Drives, Mounts, Jobs, or Audit, then close it</t>
         </is>
       </c>
       <c r="E268" s="4" t="inlineStr">
         <is>
-          <t>Content is derived from the user manual and excludes installer-only or operator-only internals</t>
+          <t>Closing Help returns to the same page and preserved workflow context</t>
         </is>
       </c>
       <c r="F268" s="4" t="n"/>
@@ -8366,7 +8366,7 @@
     <row r="269">
       <c r="A269" s="4" t="inlineStr">
         <is>
-          <t>TC-1025</t>
+          <t>TC-1024</t>
         </is>
       </c>
       <c r="B269" s="4" t="inlineStr">
@@ -8376,17 +8376,17 @@
       </c>
       <c r="C269" s="4" t="inlineStr">
         <is>
-          <t>Open full help document works</t>
+          <t>Help content is curated and user-facing</t>
         </is>
       </c>
       <c r="D269" s="4" t="inlineStr">
         <is>
-          <t>Use the Help modal action to open the full document if present</t>
+          <t>Review Help content in the modal</t>
         </is>
       </c>
       <c r="E269" s="4" t="inlineStr">
         <is>
-          <t>Full help content opens successfully and remains consistent with the in-app content</t>
+          <t>Content is derived from the user manual and excludes installer-only or operator-only internals</t>
         </is>
       </c>
       <c r="F269" s="4" t="n"/>
@@ -8397,7 +8397,7 @@
     <row r="270">
       <c r="A270" s="4" t="inlineStr">
         <is>
-          <t>TC-1026</t>
+          <t>TC-1025</t>
         </is>
       </c>
       <c r="B270" s="4" t="inlineStr">
@@ -8407,17 +8407,17 @@
       </c>
       <c r="C270" s="4" t="inlineStr">
         <is>
-          <t>Missing help asset fails gracefully</t>
+          <t>Open full help document works</t>
         </is>
       </c>
       <c r="D270" s="4" t="inlineStr">
         <is>
-          <t>Test a build with the Help asset intentionally missing or inaccessible</t>
+          <t>Use the Help modal action to open the full document if present</t>
         </is>
       </c>
       <c r="E270" s="4" t="inlineStr">
         <is>
-          <t>UI shows a non-fatal fallback state with retry or operator guidance instead of breaking the app shell</t>
+          <t>Full help content opens successfully and remains consistent with the in-app content</t>
         </is>
       </c>
       <c r="F270" s="4" t="n"/>
@@ -8426,59 +8426,59 @@
       <c r="I270" s="4" t="n"/>
     </row>
     <row r="271">
-      <c r="A271" s="2" t="inlineStr">
+      <c r="A271" s="4" t="inlineStr">
+        <is>
+          <t>TC-1026</t>
+        </is>
+      </c>
+      <c r="B271" s="4" t="inlineStr">
+        <is>
+          <t>12.10.2 Help System</t>
+        </is>
+      </c>
+      <c r="C271" s="4" t="inlineStr">
+        <is>
+          <t>Missing help asset fails gracefully</t>
+        </is>
+      </c>
+      <c r="D271" s="4" t="inlineStr">
+        <is>
+          <t>Test a build with the Help asset intentionally missing or inaccessible</t>
+        </is>
+      </c>
+      <c r="E271" s="4" t="inlineStr">
+        <is>
+          <t>UI shows a non-fatal fallback state with retry or operator guidance instead of breaking the app shell</t>
+        </is>
+      </c>
+      <c r="F271" s="4" t="n"/>
+      <c r="G271" s="4" t="n"/>
+      <c r="H271" s="4" t="n"/>
+      <c r="I271" s="4" t="n"/>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="inlineStr">
         <is>
           <t>§12.11 First-Run Setup</t>
         </is>
       </c>
-      <c r="B271" s="2" t="inlineStr">
+      <c r="B272" s="2" t="inlineStr">
         <is>
           <t>12.11 First-Run Setup</t>
         </is>
       </c>
-      <c r="C271" s="3" t="n"/>
-      <c r="D271" s="3" t="n"/>
-      <c r="E271" s="3" t="n"/>
-      <c r="F271" s="3" t="n"/>
-      <c r="G271" s="3" t="n"/>
-      <c r="H271" s="3" t="n"/>
-      <c r="I271" s="3" t="n"/>
-    </row>
-    <row r="272">
-      <c r="A272" s="4" t="inlineStr">
-        <is>
-          <t>TC-1101</t>
-        </is>
-      </c>
-      <c r="B272" s="4" t="inlineStr">
-        <is>
-          <t>12.11 First-Run Setup</t>
-        </is>
-      </c>
-      <c r="C272" s="4" t="inlineStr">
-        <is>
-          <t>Status — not initialized</t>
-        </is>
-      </c>
-      <c r="D272" s="4" t="inlineStr">
-        <is>
-          <t>GET /setup/status on fresh database</t>
-        </is>
-      </c>
-      <c r="E272" s="4" t="inlineStr">
-        <is>
-          <t>200, {"initialized": false}</t>
-        </is>
-      </c>
-      <c r="F272" s="4" t="n"/>
-      <c r="G272" s="4" t="n"/>
-      <c r="H272" s="4" t="n"/>
-      <c r="I272" s="4" t="n"/>
+      <c r="C272" s="3" t="n"/>
+      <c r="D272" s="3" t="n"/>
+      <c r="E272" s="3" t="n"/>
+      <c r="F272" s="3" t="n"/>
+      <c r="G272" s="3" t="n"/>
+      <c r="H272" s="3" t="n"/>
+      <c r="I272" s="3" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="4" t="inlineStr">
         <is>
-          <t>TC-1102</t>
+          <t>TC-1101</t>
         </is>
       </c>
       <c r="B273" s="4" t="inlineStr">
@@ -8488,17 +8488,17 @@
       </c>
       <c r="C273" s="4" t="inlineStr">
         <is>
-          <t>Initialize</t>
+          <t>Status — not initialized</t>
         </is>
       </c>
       <c r="D273" s="4" t="inlineStr">
         <is>
-          <t>Complete the setup wizard with matching admin password and confirmation values</t>
+          <t>GET /setup/status on fresh database</t>
         </is>
       </c>
       <c r="E273" s="4" t="inlineStr">
         <is>
-          <t>200, returns message, username, groups_created</t>
+          <t>200, {"initialized": false}</t>
         </is>
       </c>
       <c r="F273" s="4" t="n"/>
@@ -8509,7 +8509,7 @@
     <row r="274">
       <c r="A274" s="4" t="inlineStr">
         <is>
-          <t>TC-1103</t>
+          <t>TC-1102</t>
         </is>
       </c>
       <c r="B274" s="4" t="inlineStr">
@@ -8519,17 +8519,17 @@
       </c>
       <c r="C274" s="4" t="inlineStr">
         <is>
-          <t>Status — initialized</t>
+          <t>Initialize</t>
         </is>
       </c>
       <c r="D274" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/status after initialization</t>
+          <t>Complete the setup wizard with matching admin password and confirmation values</t>
         </is>
       </c>
       <c r="E274" s="4" t="inlineStr">
         <is>
-          <t>200, {"initialized": true}</t>
+          <t>200, returns message, username, groups_created</t>
         </is>
       </c>
       <c r="F274" s="4" t="n"/>
@@ -8540,7 +8540,7 @@
     <row r="275">
       <c r="A275" s="4" t="inlineStr">
         <is>
-          <t>TC-1104</t>
+          <t>TC-1103</t>
         </is>
       </c>
       <c r="B275" s="4" t="inlineStr">
@@ -8550,17 +8550,17 @@
       </c>
       <c r="C275" s="4" t="inlineStr">
         <is>
-          <t>Re-initialize informational</t>
+          <t>Status — initialized</t>
         </is>
       </c>
       <c r="D275" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize again</t>
+          <t>GET /setup/status after initialization</t>
         </is>
       </c>
       <c r="E275" s="4" t="inlineStr">
         <is>
-          <t>200, status=already_initialized</t>
+          <t>200, {"initialized": true}</t>
         </is>
       </c>
       <c r="F275" s="4" t="n"/>
@@ -8571,7 +8571,7 @@
     <row r="276">
       <c r="A276" s="4" t="inlineStr">
         <is>
-          <t>TC-1105</t>
+          <t>TC-1104</t>
         </is>
       </c>
       <c r="B276" s="4" t="inlineStr">
@@ -8581,17 +8581,17 @@
       </c>
       <c r="C276" s="4" t="inlineStr">
         <is>
-          <t>Invalid username</t>
+          <t>Re-initialize informational</t>
         </is>
       </c>
       <c r="D276" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with uppercase or special chars</t>
+          <t>POST /setup/initialize again</t>
         </is>
       </c>
       <c r="E276" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>200, status=already_initialized</t>
         </is>
       </c>
       <c r="F276" s="4" t="n"/>
@@ -8602,7 +8602,7 @@
     <row r="277">
       <c r="A277" s="4" t="inlineStr">
         <is>
-          <t>TC-1106</t>
+          <t>TC-1105</t>
         </is>
       </c>
       <c r="B277" s="4" t="inlineStr">
@@ -8612,12 +8612,12 @@
       </c>
       <c r="C277" s="4" t="inlineStr">
         <is>
-          <t>Empty password</t>
+          <t>Invalid username</t>
         </is>
       </c>
       <c r="D277" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with {"password": ""}</t>
+          <t>POST /setup/initialize with uppercase or special chars</t>
         </is>
       </c>
       <c r="E277" s="4" t="inlineStr">
@@ -8633,7 +8633,7 @@
     <row r="278">
       <c r="A278" s="4" t="inlineStr">
         <is>
-          <t>TC-1107</t>
+          <t>TC-1106</t>
         </is>
       </c>
       <c r="B278" s="4" t="inlineStr">
@@ -8643,17 +8643,17 @@
       </c>
       <c r="C278" s="4" t="inlineStr">
         <is>
-          <t>Unsafe password chars</t>
+          <t>Empty password</t>
         </is>
       </c>
       <c r="D278" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with password containing newline or colon</t>
+          <t>POST /setup/initialize with {"password": ""}</t>
         </is>
       </c>
       <c r="E278" s="4" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F278" s="4" t="n"/>
@@ -8664,7 +8664,7 @@
     <row r="279">
       <c r="A279" s="4" t="inlineStr">
         <is>
-          <t>TC-1108</t>
+          <t>TC-1107</t>
         </is>
       </c>
       <c r="B279" s="4" t="inlineStr">
@@ -8674,17 +8674,17 @@
       </c>
       <c r="C279" s="4" t="inlineStr">
         <is>
-          <t>Login as initialized admin</t>
+          <t>Unsafe password chars</t>
         </is>
       </c>
       <c r="D279" s="4" t="inlineStr">
         <is>
-          <t>POST /auth/token with the admin credentials from step 2</t>
+          <t>POST /setup/initialize with password containing newline or colon</t>
         </is>
       </c>
       <c r="E279" s="4" t="inlineStr">
         <is>
-          <t>200, JWT contains admin role</t>
+          <t>422, unsafe characters</t>
         </is>
       </c>
       <c r="F279" s="4" t="n"/>
@@ -8695,7 +8695,7 @@
     <row r="280">
       <c r="A280" s="4" t="inlineStr">
         <is>
-          <t>TC-1109</t>
+          <t>TC-1108</t>
         </is>
       </c>
       <c r="B280" s="4" t="inlineStr">
@@ -8705,17 +8705,17 @@
       </c>
       <c r="C280" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM_INITIALIZED audit log</t>
+          <t>Login as initialized admin</t>
         </is>
       </c>
       <c r="D280" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
+          <t>POST /auth/token with the admin credentials from step 2</t>
         </is>
       </c>
       <c r="E280" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor</t>
+          <t>200, JWT contains admin role</t>
         </is>
       </c>
       <c r="F280" s="4" t="n"/>
@@ -8726,7 +8726,7 @@
     <row r="281">
       <c r="A281" s="4" t="inlineStr">
         <is>
-          <t>TC-1110</t>
+          <t>TC-1109</t>
         </is>
       </c>
       <c r="B281" s="4" t="inlineStr">
@@ -8736,17 +8736,17 @@
       </c>
       <c r="C281" s="4" t="inlineStr">
         <is>
-          <t>Initialize default proxy trust</t>
+          <t>SYSTEM_INITIALIZED audit log</t>
         </is>
       </c>
       <c r="D281" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize without trust_proxy_headers</t>
+          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
         </is>
       </c>
       <c r="E281" s="4" t="inlineStr">
         <is>
-          <t>200, runtime TRUST_PROXY_HEADERS=false persisted</t>
+          <t>Audit entry with actor</t>
         </is>
       </c>
       <c r="F281" s="4" t="n"/>
@@ -8757,7 +8757,7 @@
     <row r="282">
       <c r="A282" s="4" t="inlineStr">
         <is>
-          <t>TC-1111</t>
+          <t>TC-1110</t>
         </is>
       </c>
       <c r="B282" s="4" t="inlineStr">
@@ -8767,17 +8767,17 @@
       </c>
       <c r="C282" s="4" t="inlineStr">
         <is>
-          <t>Initialize explicit proxy trust</t>
+          <t>Initialize default proxy trust</t>
         </is>
       </c>
       <c r="D282" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with "trust_proxy_headers": true</t>
+          <t>POST /setup/initialize without trust_proxy_headers</t>
         </is>
       </c>
       <c r="E282" s="4" t="inlineStr">
         <is>
-          <t>200, runtime TRUST_PROXY_HEADERS=true persisted</t>
+          <t>200, runtime TRUST_PROXY_HEADERS=false persisted</t>
         </is>
       </c>
       <c r="F282" s="4" t="n"/>
@@ -8788,7 +8788,7 @@
     <row r="283">
       <c r="A283" s="4" t="inlineStr">
         <is>
-          <t>TC-1112</t>
+          <t>TC-1111</t>
         </is>
       </c>
       <c r="B283" s="4" t="inlineStr">
@@ -8798,17 +8798,17 @@
       </c>
       <c r="C283" s="4" t="inlineStr">
         <is>
-          <t>Re-initialize does not mutate runtime flags</t>
+          <t>Initialize explicit proxy trust</t>
         </is>
       </c>
       <c r="D283" s="4" t="inlineStr">
         <is>
-          <t>Call POST /setup/initialize after setup with a different trust_proxy_headers value</t>
+          <t>POST /setup/initialize with "trust_proxy_headers": true</t>
         </is>
       </c>
       <c r="E283" s="4" t="inlineStr">
         <is>
-          <t>200, status=already_initialized, runtime TRUST_PROXY_HEADERS remains unchanged</t>
+          <t>200, runtime TRUST_PROXY_HEADERS=true persisted</t>
         </is>
       </c>
       <c r="F283" s="4" t="n"/>
@@ -8819,7 +8819,7 @@
     <row r="284">
       <c r="A284" s="4" t="inlineStr">
         <is>
-          <t>TC-1113</t>
+          <t>TC-1112</t>
         </is>
       </c>
       <c r="B284" s="4" t="inlineStr">
@@ -8829,17 +8829,17 @@
       </c>
       <c r="C284" s="4" t="inlineStr">
         <is>
-          <t>Runtime env target consistency</t>
+          <t>Re-initialize does not mutate runtime flags</t>
         </is>
       </c>
       <c r="D284" s="4" t="inlineStr">
         <is>
-          <t>Validate running service env file target and setup persistence target are the same (ECUBE_ENV_FILE)</t>
+          <t>Call POST /setup/initialize after setup with a different trust_proxy_headers value</t>
         </is>
       </c>
       <c r="E284" s="4" t="inlineStr">
         <is>
-          <t>Runtime env file is updated, not a workspace-relative .env</t>
+          <t>200, status=already_initialized, runtime TRUST_PROXY_HEADERS remains unchanged</t>
         </is>
       </c>
       <c r="F284" s="4" t="n"/>
@@ -8850,7 +8850,7 @@
     <row r="285">
       <c r="A285" s="4" t="inlineStr">
         <is>
-          <t>TC-1114</t>
+          <t>TC-1113</t>
         </is>
       </c>
       <c r="B285" s="4" t="inlineStr">
@@ -8860,17 +8860,17 @@
       </c>
       <c r="C285" s="4" t="inlineStr">
         <is>
-          <t>Uninstall drop fails closed on invalid target</t>
+          <t>Runtime env target consistency</t>
         </is>
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t>Run install.sh --uninstall --drop-database with missing/invalid/maintenance DATABASE_URL</t>
+          <t>Validate running service env file target and setup persistence target are the same (ECUBE_ENV_FILE)</t>
         </is>
       </c>
       <c r="E285" s="4" t="inlineStr">
         <is>
-          <t>Installer exits non-zero with explicit drop-target error; uninstall does not silently continue</t>
+          <t>Runtime env file is updated, not a workspace-relative .env</t>
         </is>
       </c>
       <c r="F285" s="4" t="n"/>
@@ -8881,7 +8881,7 @@
     <row r="286">
       <c r="A286" s="4" t="inlineStr">
         <is>
-          <t>TC-1115</t>
+          <t>TC-1114</t>
         </is>
       </c>
       <c r="B286" s="4" t="inlineStr">
@@ -8891,17 +8891,17 @@
       </c>
       <c r="C286" s="4" t="inlineStr">
         <is>
-          <t>Setup-required API redirect</t>
+          <t>Uninstall drop fails closed on invalid target</t>
         </is>
       </c>
       <c r="D286" s="4" t="inlineStr">
         <is>
-          <t>While using a normal UI screen, trigger a backend response with status 503, code HTTP_503, and message Database is not configured yet. Complete setup first.</t>
+          <t>Run install.sh --uninstall --drop-database with missing/invalid/maintenance DATABASE_URL</t>
         </is>
       </c>
       <c r="E286" s="4" t="inlineStr">
         <is>
-          <t>The browser redirects to /setup and the operator is not left only with the generic server-error toast</t>
+          <t>Installer exits non-zero with explicit drop-target error; uninstall does not silently continue</t>
         </is>
       </c>
       <c r="F286" s="4" t="n"/>
@@ -8912,7 +8912,7 @@
     <row r="287">
       <c r="A287" s="4" t="inlineStr">
         <is>
-          <t>TC-1116</t>
+          <t>TC-1115</t>
         </is>
       </c>
       <c r="B287" s="4" t="inlineStr">
@@ -8922,17 +8922,17 @@
       </c>
       <c r="C287" s="4" t="inlineStr">
         <is>
-          <t>Setup password confirmation mismatch</t>
+          <t>Setup-required API redirect</t>
         </is>
       </c>
       <c r="D287" s="4" t="inlineStr">
         <is>
-          <t>In the final setup wizard step, enter different values in the admin password and confirmation fields</t>
+          <t>While using a normal UI screen, trigger a backend response with status 503, code HTTP_503, and message Database is not configured yet. Complete setup first.</t>
         </is>
       </c>
       <c r="E287" s="4" t="inlineStr">
         <is>
-          <t>The wizard shows a password-mismatch validation message and does not submit setup until the two values match</t>
+          <t>The browser redirects to /setup and the operator is not left only with the generic server-error toast</t>
         </is>
       </c>
       <c r="F287" s="4" t="n"/>
@@ -8941,59 +8941,59 @@
       <c r="I287" s="4" t="n"/>
     </row>
     <row r="288">
-      <c r="A288" s="2" t="inlineStr">
+      <c r="A288" s="4" t="inlineStr">
+        <is>
+          <t>TC-1116</t>
+        </is>
+      </c>
+      <c r="B288" s="4" t="inlineStr">
+        <is>
+          <t>12.11 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C288" s="4" t="inlineStr">
+        <is>
+          <t>Setup password confirmation mismatch</t>
+        </is>
+      </c>
+      <c r="D288" s="4" t="inlineStr">
+        <is>
+          <t>In the final setup wizard step, enter different values in the admin password and confirmation fields</t>
+        </is>
+      </c>
+      <c r="E288" s="4" t="inlineStr">
+        <is>
+          <t>The wizard shows a password-mismatch validation message and does not submit setup until the two values match</t>
+        </is>
+      </c>
+      <c r="F288" s="4" t="n"/>
+      <c r="G288" s="4" t="n"/>
+      <c r="H288" s="4" t="n"/>
+      <c r="I288" s="4" t="n"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="2" t="inlineStr">
         <is>
           <t>§12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
-      <c r="B288" s="2" t="inlineStr">
+      <c r="B289" s="2" t="inlineStr">
         <is>
           <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
-      <c r="C288" s="3" t="n"/>
-      <c r="D288" s="3" t="n"/>
-      <c r="E288" s="3" t="n"/>
-      <c r="F288" s="3" t="n"/>
-      <c r="G288" s="3" t="n"/>
-      <c r="H288" s="3" t="n"/>
-      <c r="I288" s="3" t="n"/>
-    </row>
-    <row r="289">
-      <c r="A289" s="4" t="inlineStr">
-        <is>
-          <t>TC-1201</t>
-        </is>
-      </c>
-      <c r="B289" s="4" t="inlineStr">
-        <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
-        </is>
-      </c>
-      <c r="C289" s="4" t="inlineStr">
-        <is>
-          <t>Retrieve stored CoC snapshot — archived job</t>
-        </is>
-      </c>
-      <c r="D289" s="4" t="inlineStr">
-        <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for an archived job that already has a stored snapshot</t>
-        </is>
-      </c>
-      <c r="E289" s="4" t="inlineStr">
-        <is>
-          <t>200, response contains the stored snapshot and snapshot metadata</t>
-        </is>
-      </c>
-      <c r="F289" s="4" t="n"/>
-      <c r="G289" s="4" t="n"/>
-      <c r="H289" s="4" t="n"/>
-      <c r="I289" s="4" t="n"/>
+      <c r="C289" s="3" t="n"/>
+      <c r="D289" s="3" t="n"/>
+      <c r="E289" s="3" t="n"/>
+      <c r="F289" s="3" t="n"/>
+      <c r="G289" s="3" t="n"/>
+      <c r="H289" s="3" t="n"/>
+      <c r="I289" s="3" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="4" t="inlineStr">
         <is>
-          <t>TC-1202</t>
+          <t>TC-1201</t>
         </is>
       </c>
       <c r="B290" s="4" t="inlineStr">
@@ -9003,17 +9003,17 @@
       </c>
       <c r="C290" s="4" t="inlineStr">
         <is>
-          <t>Retrieve stored CoC snapshot — active job</t>
+          <t>Retrieve stored CoC snapshot — archived job</t>
         </is>
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job that already has a stored snapshot</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for an archived job that already has a stored snapshot</t>
         </is>
       </c>
       <c r="E290" s="4" t="inlineStr">
         <is>
-          <t>200, response contains the stored snapshot and does not regenerate it</t>
+          <t>200, response contains the stored snapshot and snapshot metadata</t>
         </is>
       </c>
       <c r="F290" s="4" t="n"/>
@@ -9024,7 +9024,7 @@
     <row r="291">
       <c r="A291" s="4" t="inlineStr">
         <is>
-          <t>TC-1203</t>
+          <t>TC-1202</t>
         </is>
       </c>
       <c r="B291" s="4" t="inlineStr">
@@ -9034,17 +9034,17 @@
       </c>
       <c r="C291" s="4" t="inlineStr">
         <is>
-          <t>CoC read — missing stored snapshot</t>
+          <t>Retrieve stored CoC snapshot — active job</t>
         </is>
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job with no stored snapshot yet</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job that already has a stored snapshot</t>
         </is>
       </c>
       <c r="E291" s="4" t="inlineStr">
         <is>
-          <t>404, message explains that the report must be refreshed first</t>
+          <t>200, response contains the stored snapshot and does not regenerate it</t>
         </is>
       </c>
       <c r="F291" s="4" t="n"/>
@@ -9055,7 +9055,7 @@
     <row r="292">
       <c r="A292" s="4" t="inlineStr">
         <is>
-          <t>TC-1204</t>
+          <t>TC-1203</t>
         </is>
       </c>
       <c r="B292" s="4" t="inlineStr">
@@ -9065,17 +9065,17 @@
       </c>
       <c r="C292" s="4" t="inlineStr">
         <is>
-          <t>CoC read — processor denied</t>
+          <t>CoC read — missing stored snapshot</t>
         </is>
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody with processor token</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job with no stored snapshot yet</t>
         </is>
       </c>
       <c r="E292" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>404, message explains that the report must be refreshed first</t>
         </is>
       </c>
       <c r="F292" s="4" t="n"/>
@@ -9086,7 +9086,7 @@
     <row r="293">
       <c r="A293" s="4" t="inlineStr">
         <is>
-          <t>TC-1205</t>
+          <t>TC-1204</t>
         </is>
       </c>
       <c r="B293" s="4" t="inlineStr">
@@ -9096,17 +9096,17 @@
       </c>
       <c r="C293" s="4" t="inlineStr">
         <is>
-          <t>CoC read — unauthenticated denied</t>
+          <t>CoC read — processor denied</t>
         </is>
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody without token</t>
+          <t>GET /jobs/{job_id}/chain-of-custody with processor token</t>
         </is>
       </c>
       <c r="E293" s="4" t="inlineStr">
         <is>
-          <t>401, UNAUTHORIZED</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F293" s="4" t="n"/>
@@ -9117,7 +9117,7 @@
     <row r="294">
       <c r="A294" s="4" t="inlineStr">
         <is>
-          <t>TC-1206</t>
+          <t>TC-1205</t>
         </is>
       </c>
       <c r="B294" s="4" t="inlineStr">
@@ -9127,17 +9127,17 @@
       </c>
       <c r="C294" s="4" t="inlineStr">
         <is>
-          <t>CoC snapshot fields</t>
+          <t>CoC read — unauthenticated denied</t>
         </is>
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>Inspect any stored-snapshot response</t>
+          <t>GET /jobs/{job_id}/chain-of-custody without token</t>
         </is>
       </c>
       <c r="E294" s="4" t="inlineStr">
         <is>
-          <t>snapshot_stored_at, snapshot_updated_at, snapshot_stored_by, reports[], and manifest/custody fields are present</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F294" s="4" t="n"/>
@@ -9148,7 +9148,7 @@
     <row r="295">
       <c r="A295" s="4" t="inlineStr">
         <is>
-          <t>TC-1207</t>
+          <t>TC-1206</t>
         </is>
       </c>
       <c r="B295" s="4" t="inlineStr">
@@ -9158,17 +9158,17 @@
       </c>
       <c r="C295" s="4" t="inlineStr">
         <is>
-          <t>CoC events include lifecycle</t>
+          <t>CoC snapshot fields</t>
         </is>
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>Inspect chain_of_custody_events in a stored report for a completed job</t>
+          <t>Inspect any stored-snapshot response</t>
         </is>
       </c>
       <c r="E295" s="4" t="inlineStr">
         <is>
-          <t>Events include DRIVE_INITIALIZED, JOB_CREATED, JOB_STARTED, JOB_COMPLETED, DRIVE_EJECT_PREPARED, and COC_HANDOFF_CONFIRMED when applicable</t>
+          <t>snapshot_stored_at, snapshot_updated_at, snapshot_stored_by, reports[], and manifest/custody fields are present</t>
         </is>
       </c>
       <c r="F295" s="4" t="n"/>
@@ -9179,7 +9179,7 @@
     <row r="296">
       <c r="A296" s="4" t="inlineStr">
         <is>
-          <t>TC-1208</t>
+          <t>TC-1207</t>
         </is>
       </c>
       <c r="B296" s="4" t="inlineStr">
@@ -9189,17 +9189,17 @@
       </c>
       <c r="C296" s="4" t="inlineStr">
         <is>
-          <t>CoC manifest summary</t>
+          <t>CoC events include lifecycle</t>
         </is>
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t>Inspect manifest_summary in the stored report</t>
+          <t>Inspect chain_of_custody_events in a stored report for a completed job</t>
         </is>
       </c>
       <c r="E296" s="4" t="inlineStr">
         <is>
-          <t>Array of objects with job_id, evidence_number, processor_notes, total_files, total_bytes, and manifest_count</t>
+          <t>Events include DRIVE_INITIALIZED, JOB_CREATED, JOB_STARTED, JOB_COMPLETED, DRIVE_EJECT_PREPARED, and COC_HANDOFF_CONFIRMED when applicable</t>
         </is>
       </c>
       <c r="F296" s="4" t="n"/>
@@ -9210,7 +9210,7 @@
     <row r="297">
       <c r="A297" s="4" t="inlineStr">
         <is>
-          <t>TC-1209</t>
+          <t>TC-1208</t>
         </is>
       </c>
       <c r="B297" s="4" t="inlineStr">
@@ -9220,17 +9220,17 @@
       </c>
       <c r="C297" s="4" t="inlineStr">
         <is>
-          <t>CoC — delivery_time absence (no handoff)</t>
+          <t>CoC manifest summary</t>
         </is>
       </c>
       <c r="D297" s="4" t="inlineStr">
         <is>
-          <t>Complete a job and store a snapshot before handoff</t>
+          <t>Inspect manifest_summary in the stored report</t>
         </is>
       </c>
       <c r="E297" s="4" t="inlineStr">
         <is>
-          <t>chain_of_custody_events do not contain COC_HANDOFF_CONFIRMED; custody_complete is false</t>
+          <t>Array of objects with job_id, evidence_number, processor_notes, total_files, total_bytes, and manifest_count</t>
         </is>
       </c>
       <c r="F297" s="4" t="n"/>
@@ -9241,7 +9241,7 @@
     <row r="298">
       <c r="A298" s="4" t="inlineStr">
         <is>
-          <t>TC-1210</t>
+          <t>TC-1209</t>
         </is>
       </c>
       <c r="B298" s="4" t="inlineStr">
@@ -9251,17 +9251,17 @@
       </c>
       <c r="C298" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — valid</t>
+          <t>CoC — delivery_time absence (no handoff)</t>
         </is>
       </c>
       <c r="D298" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh with admin or manager token for a non-archived job with assignments</t>
+          <t>Complete a job and store a snapshot before handoff</t>
         </is>
       </c>
       <c r="E298" s="4" t="inlineStr">
         <is>
-          <t>200, response contains the refreshed stored snapshot and updated snapshot metadata</t>
+          <t>chain_of_custody_events do not contain COC_HANDOFF_CONFIRMED; custody_complete is false</t>
         </is>
       </c>
       <c r="F298" s="4" t="n"/>
@@ -9272,7 +9272,7 @@
     <row r="299">
       <c r="A299" s="4" t="inlineStr">
         <is>
-          <t>TC-1211</t>
+          <t>TC-1210</t>
         </is>
       </c>
       <c r="B299" s="4" t="inlineStr">
@@ -9282,17 +9282,17 @@
       </c>
       <c r="C299" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — auditor denied</t>
+          <t>CoC refresh — valid</t>
         </is>
       </c>
       <c r="D299" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh with auditor token</t>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh with admin or manager token for a non-archived job with assignments</t>
         </is>
       </c>
       <c r="E299" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>200, response contains the refreshed stored snapshot and updated snapshot metadata</t>
         </is>
       </c>
       <c r="F299" s="4" t="n"/>
@@ -9303,7 +9303,7 @@
     <row r="300">
       <c r="A300" s="4" t="inlineStr">
         <is>
-          <t>TC-1212</t>
+          <t>TC-1211</t>
         </is>
       </c>
       <c r="B300" s="4" t="inlineStr">
@@ -9313,17 +9313,17 @@
       </c>
       <c r="C300" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — archived job denied</t>
+          <t>CoC refresh — auditor denied</t>
         </is>
       </c>
       <c r="D300" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh for an archived job</t>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh with auditor token</t>
         </is>
       </c>
       <c r="E300" s="4" t="inlineStr">
         <is>
-          <t>409, archived jobs can only return the last stored snapshot</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F300" s="4" t="n"/>
@@ -9332,59 +9332,59 @@
       <c r="I300" s="4" t="n"/>
     </row>
     <row r="301">
-      <c r="A301" s="2" t="inlineStr">
+      <c r="A301" s="4" t="inlineStr">
+        <is>
+          <t>TC-1212</t>
+        </is>
+      </c>
+      <c r="B301" s="4" t="inlineStr">
+        <is>
+          <t>12.12 Chain-of-Custody Handoff</t>
+        </is>
+      </c>
+      <c r="C301" s="4" t="inlineStr">
+        <is>
+          <t>CoC refresh — archived job denied</t>
+        </is>
+      </c>
+      <c r="D301" s="4" t="inlineStr">
+        <is>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh for an archived job</t>
+        </is>
+      </c>
+      <c r="E301" s="4" t="inlineStr">
+        <is>
+          <t>409, archived jobs can only return the last stored snapshot</t>
+        </is>
+      </c>
+      <c r="F301" s="4" t="n"/>
+      <c r="G301" s="4" t="n"/>
+      <c r="H301" s="4" t="n"/>
+      <c r="I301" s="4" t="n"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="2" t="inlineStr">
         <is>
           <t>§12.14 Startup Reconciliation</t>
         </is>
       </c>
-      <c r="B301" s="2" t="inlineStr">
+      <c r="B302" s="2" t="inlineStr">
         <is>
           <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
-      <c r="C301" s="3" t="n"/>
-      <c r="D301" s="3" t="n"/>
-      <c r="E301" s="3" t="n"/>
-      <c r="F301" s="3" t="n"/>
-      <c r="G301" s="3" t="n"/>
-      <c r="H301" s="3" t="n"/>
-      <c r="I301" s="3" t="n"/>
-    </row>
-    <row r="302">
-      <c r="A302" s="4" t="inlineStr">
-        <is>
-          <t>TC-1401</t>
-        </is>
-      </c>
-      <c r="B302" s="4" t="inlineStr">
-        <is>
-          <t>12.14 Startup Reconciliation</t>
-        </is>
-      </c>
-      <c r="C302" s="4" t="inlineStr">
-        <is>
-          <t>Running job failed after restart</t>
-        </is>
-      </c>
-      <c r="D302" s="4" t="inlineStr">
-        <is>
-          <t>Create a job, start it, restart the service while RUNNING</t>
-        </is>
-      </c>
-      <c r="E302" s="4" t="inlineStr">
-        <is>
-          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
-        </is>
-      </c>
-      <c r="F302" s="4" t="n"/>
-      <c r="G302" s="4" t="n"/>
-      <c r="H302" s="4" t="n"/>
-      <c r="I302" s="4" t="n"/>
+      <c r="C302" s="3" t="n"/>
+      <c r="D302" s="3" t="n"/>
+      <c r="E302" s="3" t="n"/>
+      <c r="F302" s="3" t="n"/>
+      <c r="G302" s="3" t="n"/>
+      <c r="H302" s="3" t="n"/>
+      <c r="I302" s="3" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="4" t="inlineStr">
         <is>
-          <t>TC-1402</t>
+          <t>TC-1401</t>
         </is>
       </c>
       <c r="B303" s="4" t="inlineStr">
@@ -9394,17 +9394,17 @@
       </c>
       <c r="C303" s="4" t="inlineStr">
         <is>
-          <t>Verifying job failed after restart</t>
+          <t>Running job failed after restart</t>
         </is>
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>Start a job, let it reach VERIFYING, restart the service</t>
+          <t>Create a job, start it, restart the service while RUNNING</t>
         </is>
       </c>
       <c r="E303" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
+          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
         </is>
       </c>
       <c r="F303" s="4" t="n"/>
@@ -9415,7 +9415,7 @@
     <row r="304">
       <c r="A304" s="4" t="inlineStr">
         <is>
-          <t>TC-1403</t>
+          <t>TC-1402</t>
         </is>
       </c>
       <c r="B304" s="4" t="inlineStr">
@@ -9425,17 +9425,17 @@
       </c>
       <c r="C304" s="4" t="inlineStr">
         <is>
-          <t>Pending job not affected</t>
+          <t>Verifying job failed after restart</t>
         </is>
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>Create a job (PENDING), restart the service</t>
+          <t>Start a job, let it reach VERIFYING, restart the service</t>
         </is>
       </c>
       <c r="E304" s="4" t="inlineStr">
         <is>
-          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
+          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
         </is>
       </c>
       <c r="F304" s="4" t="n"/>
@@ -9446,7 +9446,7 @@
     <row r="305">
       <c r="A305" s="4" t="inlineStr">
         <is>
-          <t>TC-1404</t>
+          <t>TC-1403</t>
         </is>
       </c>
       <c r="B305" s="4" t="inlineStr">
@@ -9456,17 +9456,17 @@
       </c>
       <c r="C305" s="4" t="inlineStr">
         <is>
-          <t>Completed job not affected</t>
+          <t>Pending job not affected</t>
         </is>
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>Complete a job, restart the service</t>
+          <t>Create a job (PENDING), restart the service</t>
         </is>
       </c>
       <c r="E305" s="4" t="inlineStr">
         <is>
-          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
+          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
         </is>
       </c>
       <c r="F305" s="4" t="n"/>
@@ -9477,7 +9477,7 @@
     <row r="306">
       <c r="A306" s="4" t="inlineStr">
         <is>
-          <t>TC-1405</t>
+          <t>TC-1404</t>
         </is>
       </c>
       <c r="B306" s="4" t="inlineStr">
@@ -9487,17 +9487,17 @@
       </c>
       <c r="C306" s="4" t="inlineStr">
         <is>
-          <t>Stale mount corrected</t>
+          <t>Completed job not affected</t>
         </is>
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
+          <t>Complete a job, restart the service</t>
         </is>
       </c>
       <c r="E306" s="4" t="inlineStr">
         <is>
-          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
+          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F306" s="4" t="n"/>
@@ -9508,7 +9508,7 @@
     <row r="307">
       <c r="A307" s="4" t="inlineStr">
         <is>
-          <t>TC-1406</t>
+          <t>TC-1405</t>
         </is>
       </c>
       <c r="B307" s="4" t="inlineStr">
@@ -9518,17 +9518,17 @@
       </c>
       <c r="C307" s="4" t="inlineStr">
         <is>
-          <t>Active mount preserved</t>
+          <t>Stale mount corrected</t>
         </is>
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share (leave it mounted), restart the service</t>
+          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
         </is>
       </c>
       <c r="E307" s="4" t="inlineStr">
         <is>
-          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
+          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
         </is>
       </c>
       <c r="F307" s="4" t="n"/>
@@ -9539,7 +9539,7 @@
     <row r="308">
       <c r="A308" s="4" t="inlineStr">
         <is>
-          <t>TC-1407</t>
+          <t>TC-1406</t>
         </is>
       </c>
       <c r="B308" s="4" t="inlineStr">
@@ -9549,17 +9549,17 @@
       </c>
       <c r="C308" s="4" t="inlineStr">
         <is>
-          <t>USB drives re-discovered</t>
+          <t>Active mount preserved</t>
         </is>
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>Insert USB drives, restart the service</t>
+          <t>Add and mount a network share (leave it mounted), restart the service</t>
         </is>
       </c>
       <c r="E308" s="4" t="inlineStr">
         <is>
-          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
+          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F308" s="4" t="n"/>
@@ -9570,7 +9570,7 @@
     <row r="309">
       <c r="A309" s="4" t="inlineStr">
         <is>
-          <t>TC-1408</t>
+          <t>TC-1407</t>
         </is>
       </c>
       <c r="B309" s="4" t="inlineStr">
@@ -9580,17 +9580,17 @@
       </c>
       <c r="C309" s="4" t="inlineStr">
         <is>
-          <t>Idempotency</t>
+          <t>USB drives re-discovered</t>
         </is>
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>Restart the service twice without any state changes between restarts</t>
+          <t>Insert USB drives, restart the service</t>
         </is>
       </c>
       <c r="E309" s="4" t="inlineStr">
         <is>
-          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
+          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
         </is>
       </c>
       <c r="F309" s="4" t="n"/>
@@ -9601,7 +9601,7 @@
     <row r="310">
       <c r="A310" s="4" t="inlineStr">
         <is>
-          <t>TC-1409</t>
+          <t>TC-1408</t>
         </is>
       </c>
       <c r="B310" s="4" t="inlineStr">
@@ -9611,17 +9611,17 @@
       </c>
       <c r="C310" s="4" t="inlineStr">
         <is>
-          <t>Partial failure isolation</t>
+          <t>Idempotency</t>
         </is>
       </c>
       <c r="D310" s="4" t="inlineStr">
         <is>
-          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
+          <t>Restart the service twice without any state changes between restarts</t>
         </is>
       </c>
       <c r="E310" s="4" t="inlineStr">
         <is>
-          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
+          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
         </is>
       </c>
       <c r="F310" s="4" t="n"/>
@@ -9632,7 +9632,7 @@
     <row r="311">
       <c r="A311" s="4" t="inlineStr">
         <is>
-          <t>TC-1410</t>
+          <t>TC-1409</t>
         </is>
       </c>
       <c r="B311" s="4" t="inlineStr">
@@ -9642,17 +9642,17 @@
       </c>
       <c r="C311" s="4" t="inlineStr">
         <is>
-          <t>Cross-process lock — only one worker reconciles</t>
+          <t>Partial failure isolation</t>
         </is>
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
+          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
         </is>
       </c>
       <c r="E311" s="4" t="inlineStr">
         <is>
-          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
+          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
         </is>
       </c>
       <c r="F311" s="4" t="n"/>
@@ -9663,7 +9663,7 @@
     <row r="312">
       <c r="A312" s="4" t="inlineStr">
         <is>
-          <t>TC-1411</t>
+          <t>TC-1410</t>
         </is>
       </c>
       <c r="B312" s="4" t="inlineStr">
@@ -9673,17 +9673,17 @@
       </c>
       <c r="C312" s="4" t="inlineStr">
         <is>
-          <t>Stale lock reclaim</t>
+          <t>Cross-process lock — only one worker reconciles</t>
         </is>
       </c>
       <c r="D312" s="4" t="inlineStr">
         <is>
-          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
+          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
         </is>
       </c>
       <c r="E312" s="4" t="inlineStr">
         <is>
-          <t>Service reclaims the stale lock, reconciliation runs normally</t>
+          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
         </is>
       </c>
       <c r="F312" s="4" t="n"/>
@@ -9694,7 +9694,7 @@
     <row r="313">
       <c r="A313" s="4" t="inlineStr">
         <is>
-          <t>TC-1412</t>
+          <t>TC-1411</t>
         </is>
       </c>
       <c r="B313" s="4" t="inlineStr">
@@ -9704,17 +9704,17 @@
       </c>
       <c r="C313" s="4" t="inlineStr">
         <is>
-          <t>Lock released after failure</t>
+          <t>Stale lock reclaim</t>
         </is>
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
+          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
         </is>
       </c>
       <c r="E313" s="4" t="inlineStr">
         <is>
-          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
+          <t>Service reclaims the stale lock, reconciliation runs normally</t>
         </is>
       </c>
       <c r="F313" s="4" t="n"/>
@@ -9725,7 +9725,7 @@
     <row r="314">
       <c r="A314" s="4" t="inlineStr">
         <is>
-          <t>TC-1413</t>
+          <t>TC-1412</t>
         </is>
       </c>
       <c r="B314" s="4" t="inlineStr">
@@ -9735,17 +9735,17 @@
       </c>
       <c r="C314" s="4" t="inlineStr">
         <is>
-          <t>Jobs pass emits immediate startup result log</t>
+          <t>Lock released after failure</t>
         </is>
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>Create at least one RUNNING job, restart service, then inspect application logs around startup reconciliation</t>
+          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
         </is>
       </c>
       <c r="E314" s="4" t="inlineStr">
         <is>
-          <t>Logs include Startup reconciliation: checking jobs followed by an immediate Startup reconciliation: jobs result line with safe counts (jobs_checked, jobs_corrected) or safe failure classification</t>
+          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
         </is>
       </c>
       <c r="F314" s="4" t="n"/>
@@ -9756,7 +9756,7 @@
     <row r="315">
       <c r="A315" s="4" t="inlineStr">
         <is>
-          <t>TC-1414</t>
+          <t>TC-1413</t>
         </is>
       </c>
       <c r="B315" s="4" t="inlineStr">
@@ -9766,17 +9766,17 @@
       </c>
       <c r="C315" s="4" t="inlineStr">
         <is>
-          <t>Reconciled job persists restart-interruption failure reason</t>
+          <t>Jobs pass emits immediate startup result log</t>
         </is>
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>Create a RUNNING or VERIFYING job, restart service, then open Job Detail for that job</t>
+          <t>Create at least one RUNNING job, restart service, then inspect application logs around startup reconciliation</t>
         </is>
       </c>
       <c r="E315" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED and Job Detail shows a stable restart interruption reason (not the generic This job failed... fallback)</t>
+          <t>Logs include Startup reconciliation: checking jobs followed by an immediate Startup reconciliation: jobs result line with safe counts (jobs_checked, jobs_corrected) or safe failure classification</t>
         </is>
       </c>
       <c r="F315" s="4" t="n"/>
@@ -9787,7 +9787,7 @@
     <row r="316">
       <c r="A316" s="4" t="inlineStr">
         <is>
-          <t>TC-1415</t>
+          <t>TC-1414</t>
         </is>
       </c>
       <c r="B316" s="4" t="inlineStr">
@@ -9797,17 +9797,17 @@
       </c>
       <c r="C316" s="4" t="inlineStr">
         <is>
-          <t>Reconciled failed job shows correlated failure entry from audit fallback</t>
+          <t>Reconciled job persists restart-interruption failure reason</t>
         </is>
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>Restart with a RUNNING job, then inspect Job Detail when no matching file-log failure line is present</t>
+          <t>Create a RUNNING or VERIFYING job, restart service, then open Job Detail for that job</t>
         </is>
       </c>
       <c r="E316" s="4" t="inlineStr">
         <is>
-          <t>Job Detail still shows a related failure entry sourced from reconciliation evidence (JOB_RECONCILED) and the entry remains sanitized</t>
+          <t>Job status is FAILED and Job Detail shows a stable restart interruption reason (not the generic This job failed... fallback)</t>
         </is>
       </c>
       <c r="F316" s="4" t="n"/>
@@ -9818,7 +9818,7 @@
     <row r="317">
       <c r="A317" s="4" t="inlineStr">
         <is>
-          <t>TC-1416</t>
+          <t>TC-1415</t>
         </is>
       </c>
       <c r="B317" s="4" t="inlineStr">
@@ -9828,17 +9828,17 @@
       </c>
       <c r="C317" s="4" t="inlineStr">
         <is>
-          <t>Failed job API uses reconciliation audit fallback when file-log correlation is unavailable</t>
+          <t>Reconciled failed job shows correlated failure entry from audit fallback</t>
         </is>
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t>In a test environment, disable file-log correlation (log_file unset), then request GET /jobs/{job_id} for a restart-reconciled failed job</t>
+          <t>Restart with a RUNNING job, then inspect Job Detail when no matching file-log failure line is present</t>
         </is>
       </c>
       <c r="E317" s="4" t="inlineStr">
         <is>
-          <t>Response remains 200 and includes the stable restart failure reason plus a sanitized failure_log_entry derived from audit evidence (JOB_RECONCILED)</t>
+          <t>Job Detail still shows a related failure entry sourced from reconciliation evidence (JOB_RECONCILED) and the entry remains sanitized</t>
         </is>
       </c>
       <c r="F317" s="4" t="n"/>
@@ -9849,7 +9849,7 @@
     <row r="318">
       <c r="A318" s="4" t="inlineStr">
         <is>
-          <t>TC-1417</t>
+          <t>TC-1416</t>
         </is>
       </c>
       <c r="B318" s="4" t="inlineStr">
@@ -9859,17 +9859,17 @@
       </c>
       <c r="C318" s="4" t="inlineStr">
         <is>
-          <t>Jobs pass failure path emits safe startup result classification</t>
+          <t>Failed job API uses reconciliation audit fallback when file-log correlation is unavailable</t>
         </is>
       </c>
       <c r="D318" s="4" t="inlineStr">
         <is>
-          <t>In a controlled test environment, force a jobs-pass reconciliation exception, then restart service and inspect startup logs</t>
+          <t>In a test environment, disable file-log correlation (log_file unset), then request GET /jobs/{job_id} for a restart-reconciled failed job</t>
         </is>
       </c>
       <c r="E318" s="4" t="inlineStr">
         <is>
-          <t>Logs still include Startup reconciliation: jobs result with status=failed and reason=job_reconciliation_failed, without raw provider errors or host paths</t>
+          <t>Response remains 200 and includes the stable restart failure reason plus a sanitized failure_log_entry derived from audit evidence (JOB_RECONCILED)</t>
         </is>
       </c>
       <c r="F318" s="4" t="n"/>
@@ -9880,7 +9880,7 @@
     <row r="319">
       <c r="A319" s="4" t="inlineStr">
         <is>
-          <t>TC-1418</t>
+          <t>TC-1417</t>
         </is>
       </c>
       <c r="B319" s="4" t="inlineStr">
@@ -9890,17 +9890,17 @@
       </c>
       <c r="C319" s="4" t="inlineStr">
         <is>
-          <t>Restart clears stale in-progress startup analysis when no valid cache remains</t>
+          <t>Jobs pass failure path emits safe startup result classification</t>
         </is>
       </c>
       <c r="D319" s="4" t="inlineStr">
         <is>
-          <t>Trigger manual Analyze for a PENDING job, restart ECUBE before the scan completes, then reopen Job Detail</t>
+          <t>In a controlled test environment, force a jobs-pass reconciliation exception, then restart service and inspect startup logs</t>
         </is>
       </c>
       <c r="E319" s="4" t="inlineStr">
         <is>
-          <t>Job is no longer stuck in ANALYZING, startup-analysis state returns to NOT_ANALYZED, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "analysis_interrupted_by_restart", and Analyze or Start is available again</t>
+          <t>Logs still include Startup reconciliation: jobs result with status=failed and reason=job_reconciliation_failed, without raw provider errors or host paths</t>
         </is>
       </c>
       <c r="F319" s="4" t="n"/>
@@ -9911,7 +9911,7 @@
     <row r="320">
       <c r="A320" s="4" t="inlineStr">
         <is>
-          <t>TC-1419</t>
+          <t>TC-1418</t>
         </is>
       </c>
       <c r="B320" s="4" t="inlineStr">
@@ -9921,17 +9921,17 @@
       </c>
       <c r="C320" s="4" t="inlineStr">
         <is>
-          <t>Restart restores READY when the interrupted startup-analysis cache is still current</t>
+          <t>Restart clears stale in-progress startup analysis when no valid cache remains</t>
         </is>
       </c>
       <c r="D320" s="4" t="inlineStr">
         <is>
-          <t>Trigger manual Analyze for a job with a stable source tree, restart ECUBE after the reusable snapshot has been persisted but before the manual analyze workflow fully completes, then reopen Job Detail</t>
+          <t>Trigger manual Analyze for a PENDING job, restart ECUBE before the scan completes, then reopen Job Detail</t>
         </is>
       </c>
       <c r="E320" s="4" t="inlineStr">
         <is>
-          <t>Job shows startup_analysis_status: READY, the previous file and byte totals are still available, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "valid_cache_restored_after_restart", and Start can proceed without forcing a fresh scan</t>
+          <t>Job is no longer stuck in ANALYZING, startup-analysis state returns to NOT_ANALYZED, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "analysis_interrupted_by_restart", and Analyze or Start is available again</t>
         </is>
       </c>
       <c r="F320" s="4" t="n"/>
@@ -9940,59 +9940,59 @@
       <c r="I320" s="4" t="n"/>
     </row>
     <row r="321">
-      <c r="A321" s="2" t="inlineStr">
+      <c r="A321" s="4" t="inlineStr">
+        <is>
+          <t>TC-1419</t>
+        </is>
+      </c>
+      <c r="B321" s="4" t="inlineStr">
+        <is>
+          <t>12.14 Startup Reconciliation</t>
+        </is>
+      </c>
+      <c r="C321" s="4" t="inlineStr">
+        <is>
+          <t>Restart restores READY when the interrupted startup-analysis cache is still current</t>
+        </is>
+      </c>
+      <c r="D321" s="4" t="inlineStr">
+        <is>
+          <t>Trigger manual Analyze for a job with a stable source tree, restart ECUBE after the reusable snapshot has been persisted but before the manual analyze workflow fully completes, then reopen Job Detail</t>
+        </is>
+      </c>
+      <c r="E321" s="4" t="inlineStr">
+        <is>
+          <t>Job shows startup_analysis_status: READY, the previous file and byte totals are still available, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "valid_cache_restored_after_restart", and Start can proceed without forcing a fresh scan</t>
+        </is>
+      </c>
+      <c r="F321" s="4" t="n"/>
+      <c r="G321" s="4" t="n"/>
+      <c r="H321" s="4" t="n"/>
+      <c r="I321" s="4" t="n"/>
+    </row>
+    <row r="322">
+      <c r="A322" s="2" t="inlineStr">
         <is>
           <t>§12.15 System Health</t>
         </is>
       </c>
-      <c r="B321" s="2" t="inlineStr">
+      <c r="B322" s="2" t="inlineStr">
         <is>
           <t>12.15 System Health</t>
         </is>
       </c>
-      <c r="C321" s="3" t="n"/>
-      <c r="D321" s="3" t="n"/>
-      <c r="E321" s="3" t="n"/>
-      <c r="F321" s="3" t="n"/>
-      <c r="G321" s="3" t="n"/>
-      <c r="H321" s="3" t="n"/>
-      <c r="I321" s="3" t="n"/>
-    </row>
-    <row r="322">
-      <c r="A322" s="4" t="inlineStr">
-        <is>
-          <t>TC-1501</t>
-        </is>
-      </c>
-      <c r="B322" s="4" t="inlineStr">
-        <is>
-          <t>12.15 System Health</t>
-        </is>
-      </c>
-      <c r="C322" s="4" t="inlineStr">
-        <is>
-          <t>Healthy response</t>
-        </is>
-      </c>
-      <c r="D322" s="4" t="inlineStr">
-        <is>
-          <t>GET /introspection/system-health with valid token</t>
-        </is>
-      </c>
-      <c r="E322" s="4" t="inlineStr">
-        <is>
-          <t>200, status: "ok", database: "connected"</t>
-        </is>
-      </c>
-      <c r="F322" s="4" t="n"/>
-      <c r="G322" s="4" t="n"/>
-      <c r="H322" s="4" t="n"/>
-      <c r="I322" s="4" t="n"/>
+      <c r="C322" s="3" t="n"/>
+      <c r="D322" s="3" t="n"/>
+      <c r="E322" s="3" t="n"/>
+      <c r="F322" s="3" t="n"/>
+      <c r="G322" s="3" t="n"/>
+      <c r="H322" s="3" t="n"/>
+      <c r="I322" s="3" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="4" t="inlineStr">
         <is>
-          <t>TC-1502</t>
+          <t>TC-1501</t>
         </is>
       </c>
       <c r="B323" s="4" t="inlineStr">
@@ -10002,17 +10002,17 @@
       </c>
       <c r="C323" s="4" t="inlineStr">
         <is>
-          <t>CPU metric present</t>
+          <t>Healthy response</t>
         </is>
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>GET /introspection/system-health with valid token</t>
         </is>
       </c>
       <c r="E323" s="4" t="inlineStr">
         <is>
-          <t>cpu_percent is a number between 0 and 100</t>
+          <t>200, status: "ok", database: "connected"</t>
         </is>
       </c>
       <c r="F323" s="4" t="n"/>
@@ -10023,7 +10023,7 @@
     <row r="324">
       <c r="A324" s="4" t="inlineStr">
         <is>
-          <t>TC-1503</t>
+          <t>TC-1502</t>
         </is>
       </c>
       <c r="B324" s="4" t="inlineStr">
@@ -10033,7 +10033,7 @@
       </c>
       <c r="C324" s="4" t="inlineStr">
         <is>
-          <t>Memory metrics present</t>
+          <t>CPU metric present</t>
         </is>
       </c>
       <c r="D324" s="4" t="inlineStr">
@@ -10043,7 +10043,7 @@
       </c>
       <c r="E324" s="4" t="inlineStr">
         <is>
-          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
+          <t>cpu_percent is a number between 0 and 100</t>
         </is>
       </c>
       <c r="F324" s="4" t="n"/>
@@ -10054,7 +10054,7 @@
     <row r="325">
       <c r="A325" s="4" t="inlineStr">
         <is>
-          <t>TC-1504</t>
+          <t>TC-1503</t>
         </is>
       </c>
       <c r="B325" s="4" t="inlineStr">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C325" s="4" t="inlineStr">
         <is>
-          <t>Disk I/O metrics present</t>
+          <t>Memory metrics present</t>
         </is>
       </c>
       <c r="D325" s="4" t="inlineStr">
@@ -10074,7 +10074,7 @@
       </c>
       <c r="E325" s="4" t="inlineStr">
         <is>
-          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
+          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
         </is>
       </c>
       <c r="F325" s="4" t="n"/>
@@ -10085,7 +10085,7 @@
     <row r="326">
       <c r="A326" s="4" t="inlineStr">
         <is>
-          <t>TC-1505</t>
+          <t>TC-1504</t>
         </is>
       </c>
       <c r="B326" s="4" t="inlineStr">
@@ -10095,17 +10095,17 @@
       </c>
       <c r="C326" s="4" t="inlineStr">
         <is>
-          <t>Active jobs count</t>
+          <t>Disk I/O metrics present</t>
         </is>
       </c>
       <c r="D326" s="4" t="inlineStr">
         <is>
-          <t>Start an export job, call endpoint</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E326" s="4" t="inlineStr">
         <is>
-          <t>active_jobs ≥ 1</t>
+          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
         </is>
       </c>
       <c r="F326" s="4" t="n"/>
@@ -10116,7 +10116,7 @@
     <row r="327">
       <c r="A327" s="4" t="inlineStr">
         <is>
-          <t>TC-1506</t>
+          <t>TC-1505</t>
         </is>
       </c>
       <c r="B327" s="4" t="inlineStr">
@@ -10126,17 +10126,17 @@
       </c>
       <c r="C327" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size</t>
+          <t>Active jobs count</t>
         </is>
       </c>
       <c r="D327" s="4" t="inlineStr">
         <is>
-          <t>Create a PENDING job (created but not started), call endpoint</t>
+          <t>Start an export job, call endpoint</t>
         </is>
       </c>
       <c r="E327" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size ≥ 1</t>
+          <t>active_jobs ≥ 1</t>
         </is>
       </c>
       <c r="F327" s="4" t="n"/>
@@ -10147,7 +10147,7 @@
     <row r="328">
       <c r="A328" s="4" t="inlineStr">
         <is>
-          <t>TC-1507</t>
+          <t>TC-1506</t>
         </is>
       </c>
       <c r="B328" s="4" t="inlineStr">
@@ -10157,17 +10157,17 @@
       </c>
       <c r="C328" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size decrements</t>
+          <t>Worker queue size</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr">
         <is>
-          <t>Start the pending job, call endpoint again</t>
+          <t>Create a PENDING job (created but not started), call endpoint</t>
         </is>
       </c>
       <c r="E328" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
+          <t>worker_queue_size ≥ 1</t>
         </is>
       </c>
       <c r="F328" s="4" t="n"/>
@@ -10178,7 +10178,7 @@
     <row r="329">
       <c r="A329" s="4" t="inlineStr">
         <is>
-          <t>TC-1508</t>
+          <t>TC-1507</t>
         </is>
       </c>
       <c r="B329" s="4" t="inlineStr">
@@ -10188,17 +10188,17 @@
       </c>
       <c r="C329" s="4" t="inlineStr">
         <is>
-          <t>ECUBE process metrics present</t>
+          <t>Worker queue size decrements</t>
         </is>
       </c>
       <c r="D329" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Start the pending job, call endpoint again</t>
         </is>
       </c>
       <c r="E329" s="4" t="inlineStr">
         <is>
-          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
+          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
         </is>
       </c>
       <c r="F329" s="4" t="n"/>
@@ -10209,7 +10209,7 @@
     <row r="330">
       <c r="A330" s="4" t="inlineStr">
         <is>
-          <t>TC-1509</t>
+          <t>TC-1508</t>
         </is>
       </c>
       <c r="B330" s="4" t="inlineStr">
@@ -10219,17 +10219,17 @@
       </c>
       <c r="C330" s="4" t="inlineStr">
         <is>
-          <t>Active copy-thread correlation</t>
+          <t>ECUBE process metrics present</t>
         </is>
       </c>
       <c r="D330" s="4" t="inlineStr">
         <is>
-          <t>Run an export job with active copy workers, call endpoint during the run</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E330" s="4" t="inlineStr">
         <is>
-          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
+          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
         </is>
       </c>
       <c r="F330" s="4" t="n"/>
@@ -10240,7 +10240,7 @@
     <row r="331">
       <c r="A331" s="4" t="inlineStr">
         <is>
-          <t>TC-1510</t>
+          <t>TC-1509</t>
         </is>
       </c>
       <c r="B331" s="4" t="inlineStr">
@@ -10250,17 +10250,17 @@
       </c>
       <c r="C331" s="4" t="inlineStr">
         <is>
-          <t>ECUBE process metrics degrade safely</t>
+          <t>Active copy-thread correlation</t>
         </is>
       </c>
       <c r="D331" s="4" t="inlineStr">
         <is>
-          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
+          <t>Run an export job with active copy workers, call endpoint during the run</t>
         </is>
       </c>
       <c r="E331" s="4" t="inlineStr">
         <is>
-          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
+          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
         </is>
       </c>
       <c r="F331" s="4" t="n"/>
@@ -10271,7 +10271,7 @@
     <row r="332">
       <c r="A332" s="4" t="inlineStr">
         <is>
-          <t>TC-1511</t>
+          <t>TC-1510</t>
         </is>
       </c>
       <c r="B332" s="4" t="inlineStr">
@@ -10281,17 +10281,17 @@
       </c>
       <c r="C332" s="4" t="inlineStr">
         <is>
-          <t>Degraded when DB down</t>
+          <t>ECUBE process metrics degrade safely</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, call endpoint with valid token</t>
+          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
         </is>
       </c>
       <c r="E332" s="4" t="inlineStr">
         <is>
-          <t>200, status: "degraded", database: "error", database_error is non-null</t>
+          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
         </is>
       </c>
       <c r="F332" s="4" t="n"/>
@@ -10302,7 +10302,7 @@
     <row r="333">
       <c r="A333" s="4" t="inlineStr">
         <is>
-          <t>TC-1512</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B333" s="4" t="inlineStr">
@@ -10312,17 +10312,17 @@
       </c>
       <c r="C333" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated rejected</t>
+          <t>Degraded when DB down</t>
         </is>
       </c>
       <c r="D333" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health without token</t>
+          <t>Stop PostgreSQL, call endpoint with valid token</t>
         </is>
       </c>
       <c r="E333" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>200, status: "degraded", database: "error", database_error is non-null</t>
         </is>
       </c>
       <c r="F333" s="4" t="n"/>
@@ -10333,7 +10333,7 @@
     <row r="334">
       <c r="A334" s="4" t="inlineStr">
         <is>
-          <t>TC-1513</t>
+          <t>TC-1512</t>
         </is>
       </c>
       <c r="B334" s="4" t="inlineStr">
@@ -10343,17 +10343,17 @@
       </c>
       <c r="C334" s="4" t="inlineStr">
         <is>
-          <t>Processor role allowed</t>
+          <t>Unauthenticated rejected</t>
         </is>
       </c>
       <c r="D334" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with processor token</t>
+          <t>GET /introspection/system-health without token</t>
         </is>
       </c>
       <c r="E334" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F334" s="4" t="n"/>
@@ -10362,59 +10362,59 @@
       <c r="I334" s="4" t="n"/>
     </row>
     <row r="335">
-      <c r="A335" s="2" t="inlineStr">
+      <c r="A335" s="4" t="inlineStr">
+        <is>
+          <t>TC-1513</t>
+        </is>
+      </c>
+      <c r="B335" s="4" t="inlineStr">
+        <is>
+          <t>12.15 System Health</t>
+        </is>
+      </c>
+      <c r="C335" s="4" t="inlineStr">
+        <is>
+          <t>Processor role allowed</t>
+        </is>
+      </c>
+      <c r="D335" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/system-health with processor token</t>
+        </is>
+      </c>
+      <c r="E335" s="4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F335" s="4" t="n"/>
+      <c r="G335" s="4" t="n"/>
+      <c r="H335" s="4" t="n"/>
+      <c r="I335" s="4" t="n"/>
+    </row>
+    <row r="336">
+      <c r="A336" s="2" t="inlineStr">
         <is>
           <t>§12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
-      <c r="B335" s="2" t="inlineStr">
+      <c r="B336" s="2" t="inlineStr">
         <is>
           <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
-      <c r="C335" s="3" t="n"/>
-      <c r="D335" s="3" t="n"/>
-      <c r="E335" s="3" t="n"/>
-      <c r="F335" s="3" t="n"/>
-      <c r="G335" s="3" t="n"/>
-      <c r="H335" s="3" t="n"/>
-      <c r="I335" s="3" t="n"/>
-    </row>
-    <row r="336">
-      <c r="A336" s="4" t="inlineStr">
-        <is>
-          <t>TC-1511</t>
-        </is>
-      </c>
-      <c r="B336" s="4" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C336" s="4" t="inlineStr">
-        <is>
-          <t>Liveness endpoint is public</t>
-        </is>
-      </c>
-      <c r="D336" s="4" t="inlineStr">
-        <is>
-          <t>GET /health/live without token</t>
-        </is>
-      </c>
-      <c r="E336" s="4" t="inlineStr">
-        <is>
-          <t>200, service reports live</t>
-        </is>
-      </c>
-      <c r="F336" s="4" t="n"/>
-      <c r="G336" s="4" t="n"/>
-      <c r="H336" s="4" t="n"/>
-      <c r="I336" s="4" t="n"/>
+      <c r="C336" s="3" t="n"/>
+      <c r="D336" s="3" t="n"/>
+      <c r="E336" s="3" t="n"/>
+      <c r="F336" s="3" t="n"/>
+      <c r="G336" s="3" t="n"/>
+      <c r="H336" s="3" t="n"/>
+      <c r="I336" s="3" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="4" t="inlineStr">
         <is>
-          <t>TC-1512</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B337" s="4" t="inlineStr">
@@ -10424,17 +10424,17 @@
       </c>
       <c r="C337" s="4" t="inlineStr">
         <is>
-          <t>Readiness endpoint is public</t>
+          <t>Liveness endpoint is public</t>
         </is>
       </c>
       <c r="D337" s="4" t="inlineStr">
         <is>
-          <t>GET /health/ready without token on a healthy system</t>
+          <t>GET /health/live without token</t>
         </is>
       </c>
       <c r="E337" s="4" t="inlineStr">
         <is>
-          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
+          <t>200, service reports live</t>
         </is>
       </c>
       <c r="F337" s="4" t="n"/>
@@ -10445,7 +10445,7 @@
     <row r="338">
       <c r="A338" s="4" t="inlineStr">
         <is>
-          <t>TC-1513</t>
+          <t>TC-1512</t>
         </is>
       </c>
       <c r="B338" s="4" t="inlineStr">
@@ -10455,17 +10455,17 @@
       </c>
       <c r="C338" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports missing database configuration</t>
+          <t>Readiness endpoint is public</t>
         </is>
       </c>
       <c r="D338" s="4" t="inlineStr">
         <is>
-          <t>Clear DB config or test before configuration, then GET /health/ready</t>
+          <t>GET /health/ready without token on a healthy system</t>
         </is>
       </c>
       <c r="E338" s="4" t="inlineStr">
         <is>
-          <t>503, status: "not_ready", reason indicates database is not configured</t>
+          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
         </is>
       </c>
       <c r="F338" s="4" t="n"/>
@@ -10476,7 +10476,7 @@
     <row r="339">
       <c r="A339" s="4" t="inlineStr">
         <is>
-          <t>TC-1514</t>
+          <t>TC-1513</t>
         </is>
       </c>
       <c r="B339" s="4" t="inlineStr">
@@ -10486,17 +10486,17 @@
       </c>
       <c r="C339" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports mount or provider problems</t>
+          <t>Readiness reports missing database configuration</t>
         </is>
       </c>
       <c r="D339" s="4" t="inlineStr">
         <is>
-          <t>Break a configured mount or provider, then GET /health/ready</t>
+          <t>Clear DB config or test before configuration, then GET /health/ready</t>
         </is>
       </c>
       <c r="E339" s="4" t="inlineStr">
         <is>
-          <t>503, response identifies the failing check without using the generic error schema</t>
+          <t>503, status: "not_ready", reason indicates database is not configured</t>
         </is>
       </c>
       <c r="F339" s="4" t="n"/>
@@ -10507,7 +10507,7 @@
     <row r="340">
       <c r="A340" s="4" t="inlineStr">
         <is>
-          <t>TC-1515</t>
+          <t>TC-1514</t>
         </is>
       </c>
       <c r="B340" s="4" t="inlineStr">
@@ -10517,17 +10517,17 @@
       </c>
       <c r="C340" s="4" t="inlineStr">
         <is>
-          <t>Version endpoint is public</t>
+          <t>Readiness reports mount or provider problems</t>
         </is>
       </c>
       <c r="D340" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/version without token</t>
+          <t>Break a configured mount or provider, then GET /health/ready</t>
         </is>
       </c>
       <c r="E340" s="4" t="inlineStr">
         <is>
-          <t>200, returns version/application metadata</t>
+          <t>503, response identifies the failing check without using the generic error schema</t>
         </is>
       </c>
       <c r="F340" s="4" t="n"/>
@@ -10538,7 +10538,7 @@
     <row r="341">
       <c r="A341" s="4" t="inlineStr">
         <is>
-          <t>TC-1516</t>
+          <t>TC-1515</t>
         </is>
       </c>
       <c r="B341" s="4" t="inlineStr">
@@ -10548,17 +10548,17 @@
       </c>
       <c r="C341" s="4" t="inlineStr">
         <is>
-          <t>Readiness remains separate from authenticated system health</t>
+          <t>Version endpoint is public</t>
         </is>
       </c>
       <c r="D341" s="4" t="inlineStr">
         <is>
-          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+          <t>GET /introspection/version without token</t>
         </is>
       </c>
       <c r="E341" s="4" t="inlineStr">
         <is>
-          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+          <t>200, returns version/application metadata</t>
         </is>
       </c>
       <c r="F341" s="4" t="n"/>
@@ -10567,32 +10567,63 @@
       <c r="I341" s="4" t="n"/>
     </row>
     <row r="342">
-      <c r="A342" s="2" t="inlineStr">
+      <c r="A342" s="4" t="inlineStr">
+        <is>
+          <t>TC-1516</t>
+        </is>
+      </c>
+      <c r="B342" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C342" s="4" t="inlineStr">
+        <is>
+          <t>Readiness remains separate from authenticated system health</t>
+        </is>
+      </c>
+      <c r="D342" s="4" t="inlineStr">
+        <is>
+          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+        </is>
+      </c>
+      <c r="E342" s="4" t="inlineStr">
+        <is>
+          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+        </is>
+      </c>
+      <c r="F342" s="4" t="n"/>
+      <c r="G342" s="4" t="n"/>
+      <c r="H342" s="4" t="n"/>
+      <c r="I342" s="4" t="n"/>
+    </row>
+    <row r="343">
+      <c r="A343" s="2" t="inlineStr">
         <is>
           <t>§12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="B342" s="2" t="inlineStr">
+      <c r="B343" s="2" t="inlineStr">
         <is>
           <t>12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="C342" s="3" t="n"/>
-      <c r="D342" s="3" t="n"/>
-      <c r="E342" s="3" t="n"/>
-      <c r="F342" s="3" t="n"/>
-      <c r="G342" s="3" t="n"/>
-      <c r="H342" s="3" t="n"/>
-      <c r="I342" s="3" t="n"/>
-    </row>
-    <row r="344">
-      <c r="A344" s="5" t="inlineStr">
+      <c r="C343" s="3" t="n"/>
+      <c r="D343" s="3" t="n"/>
+      <c r="E343" s="3" t="n"/>
+      <c r="F343" s="3" t="n"/>
+      <c r="G343" s="3" t="n"/>
+      <c r="H343" s="3" t="n"/>
+      <c r="I343" s="3" t="n"/>
+    </row>
+    <row r="345">
+      <c r="A345" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B344" s="5" t="n">
-        <v>314</v>
+      <c r="B345" s="5" t="n">
+        <v>315</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restrict auditor UI to read-only operational views
Hide dashboard activity, drive browsing, mounted-share browsing, and
system topology tabs from auditors while keeping Mounts accessible as a
read-only surface.

Update frontend tests and operator/QA/help documentation to match the
new role-specific navigation, browse, and log-view behavior.
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I345"/>
+  <dimension ref="A1:I331"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4201,7 +4201,7 @@
       </c>
       <c r="D129" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/usb/topology and open the System USB Topology tab</t>
+          <t>Sign in as admin, manager, or processor, call GET /introspection/usb/topology, and open the System USB Topology tab</t>
         </is>
       </c>
       <c r="E129" s="4" t="inlineStr">
@@ -7439,17 +7439,17 @@
       </c>
       <c r="C238" s="4" t="inlineStr">
         <is>
-          <t>View logs — non-admin denied</t>
+          <t>View logs — manager allowed</t>
         </is>
       </c>
       <c r="D238" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/view with manager/processor/auditor token</t>
+          <t>GET /admin/logs/view with manager token</t>
         </is>
       </c>
       <c r="E238" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN; denied audit event recorded</t>
+          <t>200, redacted log payload returned</t>
         </is>
       </c>
       <c r="F238" s="4" t="n"/>
@@ -7458,60 +7458,48 @@
       <c r="I238" s="4" t="n"/>
     </row>
     <row r="239">
-      <c r="A239" s="4" t="inlineStr">
-        <is>
-          <t>TC-1003</t>
-        </is>
-      </c>
-      <c r="B239" s="4" t="inlineStr">
-        <is>
-          <t>12.10 Admin Log Viewing API</t>
-        </is>
-      </c>
-      <c r="C239" s="4" t="inlineStr">
-        <is>
-          <t>View logs — unknown source</t>
-        </is>
-      </c>
-      <c r="D239" s="4" t="inlineStr">
-        <is>
-          <t>GET /admin/logs/view?source=unknown with admin token</t>
-        </is>
-      </c>
-      <c r="E239" s="4" t="inlineStr">
-        <is>
-          <t>404, unknown log source</t>
-        </is>
-      </c>
-      <c r="F239" s="4" t="n"/>
-      <c r="G239" s="4" t="n"/>
-      <c r="H239" s="4" t="n"/>
-      <c r="I239" s="4" t="n"/>
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>§12.10.1 Runtime Configuration</t>
+        </is>
+      </c>
+      <c r="B239" s="2" t="inlineStr">
+        <is>
+          <t>12.10.1 Runtime Configuration</t>
+        </is>
+      </c>
+      <c r="C239" s="3" t="n"/>
+      <c r="D239" s="3" t="n"/>
+      <c r="E239" s="3" t="n"/>
+      <c r="F239" s="3" t="n"/>
+      <c r="G239" s="3" t="n"/>
+      <c r="H239" s="3" t="n"/>
+      <c r="I239" s="3" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="4" t="inlineStr">
         <is>
-          <t>TC-1004</t>
+          <t>TC-1011</t>
         </is>
       </c>
       <c r="B240" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.10.1 Runtime Configuration</t>
         </is>
       </c>
       <c r="C240" s="4" t="inlineStr">
         <is>
-          <t>View logs — baseline response shape</t>
+          <t>Get configuration — admin</t>
         </is>
       </c>
       <c r="D240" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/view?source=app&amp;limit=5&amp;offset=0</t>
+          <t>GET /admin/configuration with admin token</t>
         </is>
       </c>
       <c r="E240" s="4" t="inlineStr">
         <is>
-          <t>200 with object fields: source, fetched_at, file_modified_at, offset, limit, returned, has_more, lines</t>
+          <t>200, response includes editable settings such as log_level and DB pool fields</t>
         </is>
       </c>
       <c r="F240" s="4" t="n"/>
@@ -7522,27 +7510,27 @@
     <row r="241">
       <c r="A241" s="4" t="inlineStr">
         <is>
-          <t>TC-1005</t>
+          <t>TC-1012</t>
         </is>
       </c>
       <c r="B241" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.10.1 Runtime Configuration</t>
         </is>
       </c>
       <c r="C241" s="4" t="inlineStr">
         <is>
-          <t>View logs — source path redaction</t>
+          <t>Get configuration — non-admin denied</t>
         </is>
       </c>
       <c r="D241" s="4" t="inlineStr">
         <is>
-          <t>Inspect source.path in successful response</t>
+          <t>GET /admin/configuration with manager/processor/auditor token</t>
         </is>
       </c>
       <c r="E241" s="4" t="inlineStr">
         <is>
-          <t>Basename only (for example app.log), no absolute filesystem path</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F241" s="4" t="n"/>
@@ -7553,27 +7541,27 @@
     <row r="242">
       <c r="A242" s="4" t="inlineStr">
         <is>
-          <t>TC-1006</t>
+          <t>TC-1013</t>
         </is>
       </c>
       <c r="B242" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.10.1 Runtime Configuration</t>
         </is>
       </c>
       <c r="C242" s="4" t="inlineStr">
         <is>
-          <t>View logs — offset pagination</t>
+          <t>Update runtime-only setting</t>
         </is>
       </c>
       <c r="D242" s="4" t="inlineStr">
         <is>
-          <t>Create known numbered lines, call GET /admin/logs/view?limit=5&amp;offset=2</t>
+          <t>PUT /admin/configuration with {"log_level": "DEBUG"}</t>
         </is>
       </c>
       <c r="E242" s="4" t="inlineStr">
         <is>
-          <t>Returns correct window from tail semantics, returned &lt;= limit</t>
+          <t>200, status: "updated", changed_settings includes log_level, restart_required is false</t>
         </is>
       </c>
       <c r="F242" s="4" t="n"/>
@@ -7584,27 +7572,27 @@
     <row r="243">
       <c r="A243" s="4" t="inlineStr">
         <is>
-          <t>TC-1007</t>
+          <t>TC-1014</t>
         </is>
       </c>
       <c r="B243" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.10.1 Runtime Configuration</t>
         </is>
       </c>
       <c r="C243" s="4" t="inlineStr">
         <is>
-          <t>View logs — reverse ordering</t>
+          <t>Update restart-required setting</t>
         </is>
       </c>
       <c r="D243" s="4" t="inlineStr">
         <is>
-          <t>Compare reverse=false vs reverse=true on same query</t>
+          <t>PUT /admin/configuration with {"db_pool_recycle_seconds": 120}</t>
         </is>
       </c>
       <c r="E243" s="4" t="inlineStr">
         <is>
-          <t>Same selected window; line order is inverted when reverse=true</t>
+          <t>200, restart_required is true and the response lists the restart-required setting</t>
         </is>
       </c>
       <c r="F243" s="4" t="n"/>
@@ -7615,27 +7603,27 @@
     <row r="244">
       <c r="A244" s="4" t="inlineStr">
         <is>
-          <t>TC-1008</t>
+          <t>TC-1015</t>
         </is>
       </c>
       <c r="B244" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.10.1 Runtime Configuration</t>
         </is>
       </c>
       <c r="C244" s="4" t="inlineStr">
         <is>
-          <t>View logs — search filtering</t>
+          <t>Reject empty update payload</t>
         </is>
       </c>
       <c r="D244" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/view?search=error</t>
+          <t>PUT /admin/configuration with {}</t>
         </is>
       </c>
       <c r="E244" s="4" t="inlineStr">
         <is>
-          <t>Only matching lines are returned (case-insensitive contains)</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F244" s="4" t="n"/>
@@ -7646,27 +7634,27 @@
     <row r="245">
       <c r="A245" s="4" t="inlineStr">
         <is>
-          <t>TC-1009</t>
+          <t>TC-1016</t>
         </is>
       </c>
       <c r="B245" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.10.1 Runtime Configuration</t>
         </is>
       </c>
       <c r="C245" s="4" t="inlineStr">
         <is>
-          <t>View logs — sensitive value redaction</t>
+          <t>Reject unwritable log file path</t>
         </is>
       </c>
       <c r="D245" s="4" t="inlineStr">
         <is>
-          <t>Include tokens/passwords in source log lines, call view endpoint</t>
+          <t>PUT /admin/configuration with {"log_file": "/var/log/ecube/denied.log"} when path is not writable</t>
         </is>
       </c>
       <c r="E245" s="4" t="inlineStr">
         <is>
-          <t>Sensitive values replaced with redacted markers in lines[].content</t>
+          <t>422, message indicates the log file cannot be written</t>
         </is>
       </c>
       <c r="F245" s="4" t="n"/>
@@ -7677,27 +7665,27 @@
     <row r="246">
       <c r="A246" s="4" t="inlineStr">
         <is>
-          <t>TC-1010</t>
+          <t>TC-1017</t>
         </is>
       </c>
       <c r="B246" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.10.1 Runtime Configuration</t>
         </is>
       </c>
       <c r="C246" s="4" t="inlineStr">
         <is>
-          <t>View logs — success audit</t>
+          <t>Configuration update audit trail</t>
         </is>
       </c>
       <c r="D246" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=LOG_LINES_VIEWED after successful view</t>
+          <t>Update configuration, then query GET /audit?action=CONFIGURATION_UPDATED</t>
         </is>
       </c>
       <c r="E246" s="4" t="inlineStr">
         <is>
-          <t>Audit entry includes source, limit, offset, returned, has_more, and basename log_file</t>
+          <t>Audit entry lists changed settings without leaking sensitive paths or secrets</t>
         </is>
       </c>
       <c r="F246" s="4" t="n"/>
@@ -7708,27 +7696,27 @@
     <row r="247">
       <c r="A247" s="4" t="inlineStr">
         <is>
-          <t>TC-1011</t>
+          <t>TC-1018</t>
         </is>
       </c>
       <c r="B247" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.10.1 Runtime Configuration</t>
         </is>
       </c>
       <c r="C247" s="4" t="inlineStr">
         <is>
-          <t>List logs — unauthenticated</t>
+          <t>Restart requires confirmation</t>
         </is>
       </c>
       <c r="D247" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs without token</t>
+          <t>POST /admin/configuration/restart with {"confirm": false}</t>
         </is>
       </c>
       <c r="E247" s="4" t="inlineStr">
         <is>
-          <t>401, UNAUTHORIZED</t>
+          <t>400</t>
         </is>
       </c>
       <c r="F247" s="4" t="n"/>
@@ -7739,27 +7727,27 @@
     <row r="248">
       <c r="A248" s="4" t="inlineStr">
         <is>
-          <t>TC-1012</t>
+          <t>TC-1019</t>
         </is>
       </c>
       <c r="B248" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.10.1 Runtime Configuration</t>
         </is>
       </c>
       <c r="C248" s="4" t="inlineStr">
         <is>
-          <t>List logs — non-admin denied</t>
+          <t>Restart request accepted when confirmed</t>
         </is>
       </c>
       <c r="D248" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs with non-admin token</t>
+          <t>POST /admin/configuration/restart with {"confirm": true}</t>
         </is>
       </c>
       <c r="E248" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN; denied audit event recorded</t>
+          <t>200, status: "restart_requested", service: "ecube"</t>
         </is>
       </c>
       <c r="F248" s="4" t="n"/>
@@ -7770,27 +7758,27 @@
     <row r="249">
       <c r="A249" s="4" t="inlineStr">
         <is>
-          <t>TC-1013</t>
+          <t>TC-1020</t>
         </is>
       </c>
       <c r="B249" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.10.1 Runtime Configuration</t>
         </is>
       </c>
       <c r="C249" s="4" t="inlineStr">
         <is>
-          <t>List logs — response envelope</t>
+          <t>Accept callback payload allowlist and mapping</t>
         </is>
       </c>
       <c r="D249" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs with admin token and file logging configured</t>
+          <t>PUT /admin/configuration with {"callback_payload_fields": ["event", "project_id"], "callback_payload_field_map": {"type": "event", "project": "project_id"}}</t>
         </is>
       </c>
       <c r="E249" s="4" t="inlineStr">
         <is>
-          <t>200 object with log_files array and total_size; no log_directory field in response</t>
+          <t>200, changed settings include both callback payload fields</t>
         </is>
       </c>
       <c r="F249" s="4" t="n"/>
@@ -7801,27 +7789,27 @@
     <row r="250">
       <c r="A250" s="4" t="inlineStr">
         <is>
-          <t>TC-1014</t>
+          <t>TC-1021</t>
         </is>
       </c>
       <c r="B250" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.10.1 Runtime Configuration</t>
         </is>
       </c>
       <c r="C250" s="4" t="inlineStr">
         <is>
-          <t>Download log — non-admin denied</t>
+          <t>Reject invalid callback payload mapping</t>
         </is>
       </c>
       <c r="D250" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/logs/app.log with non-admin token</t>
+          <t>PUT /admin/configuration with {"callback_payload_field_map": {"summary": "${unknown_field}"}}</t>
         </is>
       </c>
       <c r="E250" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN; denied audit event recorded</t>
+          <t>422, validation error identifies the invalid mapping source field</t>
         </is>
       </c>
       <c r="F250" s="4" t="n"/>
@@ -7830,60 +7818,48 @@
       <c r="I250" s="4" t="n"/>
     </row>
     <row r="251">
-      <c r="A251" s="4" t="inlineStr">
-        <is>
-          <t>TC-1015</t>
-        </is>
-      </c>
-      <c r="B251" s="4" t="inlineStr">
-        <is>
-          <t>12.10 Admin Log Viewing API</t>
-        </is>
-      </c>
-      <c r="C251" s="4" t="inlineStr">
-        <is>
-          <t>Download log — path traversal blocked</t>
-        </is>
-      </c>
-      <c r="D251" s="4" t="inlineStr">
-        <is>
-          <t>GET /admin/logs/../../../etc/passwd</t>
-        </is>
-      </c>
-      <c r="E251" s="4" t="inlineStr">
-        <is>
-          <t>Rejected (400/404/422), no file disclosure</t>
-        </is>
-      </c>
-      <c r="F251" s="4" t="n"/>
-      <c r="G251" s="4" t="n"/>
-      <c r="H251" s="4" t="n"/>
-      <c r="I251" s="4" t="n"/>
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>§12.10.2 Help System</t>
+        </is>
+      </c>
+      <c r="B251" s="2" t="inlineStr">
+        <is>
+          <t>12.10.2 Help System</t>
+        </is>
+      </c>
+      <c r="C251" s="3" t="n"/>
+      <c r="D251" s="3" t="n"/>
+      <c r="E251" s="3" t="n"/>
+      <c r="F251" s="3" t="n"/>
+      <c r="G251" s="3" t="n"/>
+      <c r="H251" s="3" t="n"/>
+      <c r="I251" s="3" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="4" t="inlineStr">
         <is>
-          <t>TC-1016</t>
+          <t>TC-1021</t>
         </is>
       </c>
       <c r="B252" s="4" t="inlineStr">
         <is>
-          <t>12.10 Admin Log Viewing API</t>
+          <t>12.10.2 Help System</t>
         </is>
       </c>
       <c r="C252" s="4" t="inlineStr">
         <is>
-          <t>Download log — success audit</t>
+          <t>Help trigger is visible in authenticated shell</t>
         </is>
       </c>
       <c r="D252" s="4" t="inlineStr">
         <is>
-          <t>Download valid file as admin, then query audit</t>
+          <t>Sign in to the application and inspect the shell/header</t>
         </is>
       </c>
       <c r="E252" s="4" t="inlineStr">
         <is>
-          <t>LOG_FILE_DOWNLOADED entry includes requested filename</t>
+          <t>A Help trigger is visible without navigating away from the current page</t>
         </is>
       </c>
       <c r="F252" s="4" t="n"/>
@@ -7892,48 +7868,60 @@
       <c r="I252" s="4" t="n"/>
     </row>
     <row r="253">
-      <c r="A253" s="2" t="inlineStr">
-        <is>
-          <t>§12.10.1 Runtime Configuration</t>
-        </is>
-      </c>
-      <c r="B253" s="2" t="inlineStr">
-        <is>
-          <t>12.10.1 Runtime Configuration</t>
-        </is>
-      </c>
-      <c r="C253" s="3" t="n"/>
-      <c r="D253" s="3" t="n"/>
-      <c r="E253" s="3" t="n"/>
-      <c r="F253" s="3" t="n"/>
-      <c r="G253" s="3" t="n"/>
-      <c r="H253" s="3" t="n"/>
-      <c r="I253" s="3" t="n"/>
+      <c r="A253" s="4" t="inlineStr">
+        <is>
+          <t>TC-1022</t>
+        </is>
+      </c>
+      <c r="B253" s="4" t="inlineStr">
+        <is>
+          <t>12.10.2 Help System</t>
+        </is>
+      </c>
+      <c r="C253" s="4" t="inlineStr">
+        <is>
+          <t>Help opens in-app</t>
+        </is>
+      </c>
+      <c r="D253" s="4" t="inlineStr">
+        <is>
+          <t>Activate the Help trigger from any primary page</t>
+        </is>
+      </c>
+      <c r="E253" s="4" t="inlineStr">
+        <is>
+          <t>Help opens in a modal or equivalent in-app panel</t>
+        </is>
+      </c>
+      <c r="F253" s="4" t="n"/>
+      <c r="G253" s="4" t="n"/>
+      <c r="H253" s="4" t="n"/>
+      <c r="I253" s="4" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="4" t="inlineStr">
         <is>
-          <t>TC-1011</t>
+          <t>TC-1023</t>
         </is>
       </c>
       <c r="B254" s="4" t="inlineStr">
         <is>
-          <t>12.10.1 Runtime Configuration</t>
+          <t>12.10.2 Help System</t>
         </is>
       </c>
       <c r="C254" s="4" t="inlineStr">
         <is>
-          <t>Get configuration — admin</t>
+          <t>Help does not break current workflow context</t>
         </is>
       </c>
       <c r="D254" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/configuration with admin token</t>
+          <t>Open Help while on Drives, Mounts, Jobs, or Audit, then close it</t>
         </is>
       </c>
       <c r="E254" s="4" t="inlineStr">
         <is>
-          <t>200, response includes editable settings such as log_level and DB pool fields</t>
+          <t>Closing Help returns to the same page and preserved workflow context</t>
         </is>
       </c>
       <c r="F254" s="4" t="n"/>
@@ -7944,27 +7932,27 @@
     <row r="255">
       <c r="A255" s="4" t="inlineStr">
         <is>
-          <t>TC-1012</t>
+          <t>TC-1024</t>
         </is>
       </c>
       <c r="B255" s="4" t="inlineStr">
         <is>
-          <t>12.10.1 Runtime Configuration</t>
+          <t>12.10.2 Help System</t>
         </is>
       </c>
       <c r="C255" s="4" t="inlineStr">
         <is>
-          <t>Get configuration — non-admin denied</t>
+          <t>Help content is curated and user-facing</t>
         </is>
       </c>
       <c r="D255" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/configuration with manager/processor/auditor token</t>
+          <t>Review Help content in the modal</t>
         </is>
       </c>
       <c r="E255" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>Content is derived from the user manual and excludes installer-only or operator-only internals</t>
         </is>
       </c>
       <c r="F255" s="4" t="n"/>
@@ -7975,27 +7963,27 @@
     <row r="256">
       <c r="A256" s="4" t="inlineStr">
         <is>
-          <t>TC-1013</t>
+          <t>TC-1025</t>
         </is>
       </c>
       <c r="B256" s="4" t="inlineStr">
         <is>
-          <t>12.10.1 Runtime Configuration</t>
+          <t>12.10.2 Help System</t>
         </is>
       </c>
       <c r="C256" s="4" t="inlineStr">
         <is>
-          <t>Update runtime-only setting</t>
+          <t>Open full help document works</t>
         </is>
       </c>
       <c r="D256" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/configuration with {"log_level": "DEBUG"}</t>
+          <t>Use the Help modal action to open the full document if present</t>
         </is>
       </c>
       <c r="E256" s="4" t="inlineStr">
         <is>
-          <t>200, status: "updated", changed_settings includes log_level, restart_required is false</t>
+          <t>Full help content opens successfully and remains consistent with the in-app content</t>
         </is>
       </c>
       <c r="F256" s="4" t="n"/>
@@ -8006,27 +7994,27 @@
     <row r="257">
       <c r="A257" s="4" t="inlineStr">
         <is>
-          <t>TC-1014</t>
+          <t>TC-1026</t>
         </is>
       </c>
       <c r="B257" s="4" t="inlineStr">
         <is>
-          <t>12.10.1 Runtime Configuration</t>
+          <t>12.10.2 Help System</t>
         </is>
       </c>
       <c r="C257" s="4" t="inlineStr">
         <is>
-          <t>Update restart-required setting</t>
+          <t>Missing help asset fails gracefully</t>
         </is>
       </c>
       <c r="D257" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/configuration with {"db_pool_recycle_seconds": 120}</t>
+          <t>Test a build with the Help asset intentionally missing or inaccessible</t>
         </is>
       </c>
       <c r="E257" s="4" t="inlineStr">
         <is>
-          <t>200, restart_required is true and the response lists the restart-required setting</t>
+          <t>UI shows a non-fatal fallback state with retry or operator guidance instead of breaking the app shell</t>
         </is>
       </c>
       <c r="F257" s="4" t="n"/>
@@ -8035,60 +8023,48 @@
       <c r="I257" s="4" t="n"/>
     </row>
     <row r="258">
-      <c r="A258" s="4" t="inlineStr">
-        <is>
-          <t>TC-1015</t>
-        </is>
-      </c>
-      <c r="B258" s="4" t="inlineStr">
-        <is>
-          <t>12.10.1 Runtime Configuration</t>
-        </is>
-      </c>
-      <c r="C258" s="4" t="inlineStr">
-        <is>
-          <t>Reject empty update payload</t>
-        </is>
-      </c>
-      <c r="D258" s="4" t="inlineStr">
-        <is>
-          <t>PUT /admin/configuration with {}</t>
-        </is>
-      </c>
-      <c r="E258" s="4" t="inlineStr">
-        <is>
-          <t>422</t>
-        </is>
-      </c>
-      <c r="F258" s="4" t="n"/>
-      <c r="G258" s="4" t="n"/>
-      <c r="H258" s="4" t="n"/>
-      <c r="I258" s="4" t="n"/>
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>§12.11 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>12.11 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C258" s="3" t="n"/>
+      <c r="D258" s="3" t="n"/>
+      <c r="E258" s="3" t="n"/>
+      <c r="F258" s="3" t="n"/>
+      <c r="G258" s="3" t="n"/>
+      <c r="H258" s="3" t="n"/>
+      <c r="I258" s="3" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="4" t="inlineStr">
         <is>
-          <t>TC-1016</t>
+          <t>TC-1101</t>
         </is>
       </c>
       <c r="B259" s="4" t="inlineStr">
         <is>
-          <t>12.10.1 Runtime Configuration</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C259" s="4" t="inlineStr">
         <is>
-          <t>Reject unwritable log file path</t>
+          <t>Status — not initialized</t>
         </is>
       </c>
       <c r="D259" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/configuration with {"log_file": "/var/log/ecube/denied.log"} when path is not writable</t>
+          <t>GET /setup/status on fresh database</t>
         </is>
       </c>
       <c r="E259" s="4" t="inlineStr">
         <is>
-          <t>422, message indicates the log file cannot be written</t>
+          <t>200, {"initialized": false}</t>
         </is>
       </c>
       <c r="F259" s="4" t="n"/>
@@ -8099,27 +8075,27 @@
     <row r="260">
       <c r="A260" s="4" t="inlineStr">
         <is>
-          <t>TC-1017</t>
+          <t>TC-1102</t>
         </is>
       </c>
       <c r="B260" s="4" t="inlineStr">
         <is>
-          <t>12.10.1 Runtime Configuration</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C260" s="4" t="inlineStr">
         <is>
-          <t>Configuration update audit trail</t>
+          <t>Initialize</t>
         </is>
       </c>
       <c r="D260" s="4" t="inlineStr">
         <is>
-          <t>Update configuration, then query GET /audit?action=CONFIGURATION_UPDATED</t>
+          <t>Complete the setup wizard with matching admin password and confirmation values</t>
         </is>
       </c>
       <c r="E260" s="4" t="inlineStr">
         <is>
-          <t>Audit entry lists changed settings without leaking sensitive paths or secrets</t>
+          <t>200, returns message, username, groups_created</t>
         </is>
       </c>
       <c r="F260" s="4" t="n"/>
@@ -8130,27 +8106,27 @@
     <row r="261">
       <c r="A261" s="4" t="inlineStr">
         <is>
-          <t>TC-1018</t>
+          <t>TC-1103</t>
         </is>
       </c>
       <c r="B261" s="4" t="inlineStr">
         <is>
-          <t>12.10.1 Runtime Configuration</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C261" s="4" t="inlineStr">
         <is>
-          <t>Restart requires confirmation</t>
+          <t>Status — initialized</t>
         </is>
       </c>
       <c r="D261" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/configuration/restart with {"confirm": false}</t>
+          <t>GET /setup/status after initialization</t>
         </is>
       </c>
       <c r="E261" s="4" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>200, {"initialized": true}</t>
         </is>
       </c>
       <c r="F261" s="4" t="n"/>
@@ -8161,27 +8137,27 @@
     <row r="262">
       <c r="A262" s="4" t="inlineStr">
         <is>
-          <t>TC-1019</t>
+          <t>TC-1104</t>
         </is>
       </c>
       <c r="B262" s="4" t="inlineStr">
         <is>
-          <t>12.10.1 Runtime Configuration</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C262" s="4" t="inlineStr">
         <is>
-          <t>Restart request accepted when confirmed</t>
+          <t>Re-initialize informational</t>
         </is>
       </c>
       <c r="D262" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/configuration/restart with {"confirm": true}</t>
+          <t>POST /setup/initialize again</t>
         </is>
       </c>
       <c r="E262" s="4" t="inlineStr">
         <is>
-          <t>200, status: "restart_requested", service: "ecube"</t>
+          <t>200, status=already_initialized</t>
         </is>
       </c>
       <c r="F262" s="4" t="n"/>
@@ -8192,27 +8168,27 @@
     <row r="263">
       <c r="A263" s="4" t="inlineStr">
         <is>
-          <t>TC-1020</t>
+          <t>TC-1105</t>
         </is>
       </c>
       <c r="B263" s="4" t="inlineStr">
         <is>
-          <t>12.10.1 Runtime Configuration</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C263" s="4" t="inlineStr">
         <is>
-          <t>Accept callback payload allowlist and mapping</t>
+          <t>Invalid username</t>
         </is>
       </c>
       <c r="D263" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/configuration with {"callback_payload_fields": ["event", "project_id"], "callback_payload_field_map": {"type": "event", "project": "project_id"}}</t>
+          <t>POST /setup/initialize with uppercase or special chars</t>
         </is>
       </c>
       <c r="E263" s="4" t="inlineStr">
         <is>
-          <t>200, changed settings include both callback payload fields</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F263" s="4" t="n"/>
@@ -8223,27 +8199,27 @@
     <row r="264">
       <c r="A264" s="4" t="inlineStr">
         <is>
-          <t>TC-1021</t>
+          <t>TC-1106</t>
         </is>
       </c>
       <c r="B264" s="4" t="inlineStr">
         <is>
-          <t>12.10.1 Runtime Configuration</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C264" s="4" t="inlineStr">
         <is>
-          <t>Reject invalid callback payload mapping</t>
+          <t>Empty password</t>
         </is>
       </c>
       <c r="D264" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/configuration with {"callback_payload_field_map": {"summary": "${unknown_field}"}}</t>
+          <t>POST /setup/initialize with {"password": ""}</t>
         </is>
       </c>
       <c r="E264" s="4" t="inlineStr">
         <is>
-          <t>422, validation error identifies the invalid mapping source field</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F264" s="4" t="n"/>
@@ -8252,48 +8228,60 @@
       <c r="I264" s="4" t="n"/>
     </row>
     <row r="265">
-      <c r="A265" s="2" t="inlineStr">
-        <is>
-          <t>§12.10.2 Help System</t>
-        </is>
-      </c>
-      <c r="B265" s="2" t="inlineStr">
-        <is>
-          <t>12.10.2 Help System</t>
-        </is>
-      </c>
-      <c r="C265" s="3" t="n"/>
-      <c r="D265" s="3" t="n"/>
-      <c r="E265" s="3" t="n"/>
-      <c r="F265" s="3" t="n"/>
-      <c r="G265" s="3" t="n"/>
-      <c r="H265" s="3" t="n"/>
-      <c r="I265" s="3" t="n"/>
+      <c r="A265" s="4" t="inlineStr">
+        <is>
+          <t>TC-1107</t>
+        </is>
+      </c>
+      <c r="B265" s="4" t="inlineStr">
+        <is>
+          <t>12.11 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C265" s="4" t="inlineStr">
+        <is>
+          <t>Unsafe password chars</t>
+        </is>
+      </c>
+      <c r="D265" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/initialize with password containing newline or colon</t>
+        </is>
+      </c>
+      <c r="E265" s="4" t="inlineStr">
+        <is>
+          <t>422, unsafe characters</t>
+        </is>
+      </c>
+      <c r="F265" s="4" t="n"/>
+      <c r="G265" s="4" t="n"/>
+      <c r="H265" s="4" t="n"/>
+      <c r="I265" s="4" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="4" t="inlineStr">
         <is>
-          <t>TC-1021</t>
+          <t>TC-1108</t>
         </is>
       </c>
       <c r="B266" s="4" t="inlineStr">
         <is>
-          <t>12.10.2 Help System</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C266" s="4" t="inlineStr">
         <is>
-          <t>Help trigger is visible in authenticated shell</t>
+          <t>Login as initialized admin</t>
         </is>
       </c>
       <c r="D266" s="4" t="inlineStr">
         <is>
-          <t>Sign in to the application and inspect the shell/header</t>
+          <t>POST /auth/token with the admin credentials from step 2</t>
         </is>
       </c>
       <c r="E266" s="4" t="inlineStr">
         <is>
-          <t>A Help trigger is visible without navigating away from the current page</t>
+          <t>200, JWT contains admin role</t>
         </is>
       </c>
       <c r="F266" s="4" t="n"/>
@@ -8304,27 +8292,27 @@
     <row r="267">
       <c r="A267" s="4" t="inlineStr">
         <is>
-          <t>TC-1022</t>
+          <t>TC-1109</t>
         </is>
       </c>
       <c r="B267" s="4" t="inlineStr">
         <is>
-          <t>12.10.2 Help System</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C267" s="4" t="inlineStr">
         <is>
-          <t>Help opens in-app</t>
+          <t>SYSTEM_INITIALIZED audit log</t>
         </is>
       </c>
       <c r="D267" s="4" t="inlineStr">
         <is>
-          <t>Activate the Help trigger from any primary page</t>
+          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
         </is>
       </c>
       <c r="E267" s="4" t="inlineStr">
         <is>
-          <t>Help opens in a modal or equivalent in-app panel</t>
+          <t>Audit entry with actor</t>
         </is>
       </c>
       <c r="F267" s="4" t="n"/>
@@ -8335,27 +8323,27 @@
     <row r="268">
       <c r="A268" s="4" t="inlineStr">
         <is>
-          <t>TC-1023</t>
+          <t>TC-1110</t>
         </is>
       </c>
       <c r="B268" s="4" t="inlineStr">
         <is>
-          <t>12.10.2 Help System</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C268" s="4" t="inlineStr">
         <is>
-          <t>Help does not break current workflow context</t>
+          <t>Initialize default proxy trust</t>
         </is>
       </c>
       <c r="D268" s="4" t="inlineStr">
         <is>
-          <t>Open Help while on Drives, Mounts, Jobs, or Audit, then close it</t>
+          <t>POST /setup/initialize without trust_proxy_headers</t>
         </is>
       </c>
       <c r="E268" s="4" t="inlineStr">
         <is>
-          <t>Closing Help returns to the same page and preserved workflow context</t>
+          <t>200, runtime TRUST_PROXY_HEADERS=false persisted</t>
         </is>
       </c>
       <c r="F268" s="4" t="n"/>
@@ -8366,27 +8354,27 @@
     <row r="269">
       <c r="A269" s="4" t="inlineStr">
         <is>
-          <t>TC-1024</t>
+          <t>TC-1111</t>
         </is>
       </c>
       <c r="B269" s="4" t="inlineStr">
         <is>
-          <t>12.10.2 Help System</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C269" s="4" t="inlineStr">
         <is>
-          <t>Help content is curated and user-facing</t>
+          <t>Initialize explicit proxy trust</t>
         </is>
       </c>
       <c r="D269" s="4" t="inlineStr">
         <is>
-          <t>Review Help content in the modal</t>
+          <t>POST /setup/initialize with "trust_proxy_headers": true</t>
         </is>
       </c>
       <c r="E269" s="4" t="inlineStr">
         <is>
-          <t>Content is derived from the user manual and excludes installer-only or operator-only internals</t>
+          <t>200, runtime TRUST_PROXY_HEADERS=true persisted</t>
         </is>
       </c>
       <c r="F269" s="4" t="n"/>
@@ -8397,27 +8385,27 @@
     <row r="270">
       <c r="A270" s="4" t="inlineStr">
         <is>
-          <t>TC-1025</t>
+          <t>TC-1112</t>
         </is>
       </c>
       <c r="B270" s="4" t="inlineStr">
         <is>
-          <t>12.10.2 Help System</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C270" s="4" t="inlineStr">
         <is>
-          <t>Open full help document works</t>
+          <t>Re-initialize does not mutate runtime flags</t>
         </is>
       </c>
       <c r="D270" s="4" t="inlineStr">
         <is>
-          <t>Use the Help modal action to open the full document if present</t>
+          <t>Call POST /setup/initialize after setup with a different trust_proxy_headers value</t>
         </is>
       </c>
       <c r="E270" s="4" t="inlineStr">
         <is>
-          <t>Full help content opens successfully and remains consistent with the in-app content</t>
+          <t>200, status=already_initialized, runtime TRUST_PROXY_HEADERS remains unchanged</t>
         </is>
       </c>
       <c r="F270" s="4" t="n"/>
@@ -8428,27 +8416,27 @@
     <row r="271">
       <c r="A271" s="4" t="inlineStr">
         <is>
-          <t>TC-1026</t>
+          <t>TC-1113</t>
         </is>
       </c>
       <c r="B271" s="4" t="inlineStr">
         <is>
-          <t>12.10.2 Help System</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C271" s="4" t="inlineStr">
         <is>
-          <t>Missing help asset fails gracefully</t>
+          <t>Runtime env target consistency</t>
         </is>
       </c>
       <c r="D271" s="4" t="inlineStr">
         <is>
-          <t>Test a build with the Help asset intentionally missing or inaccessible</t>
+          <t>Validate running service env file target and setup persistence target are the same (ECUBE_ENV_FILE)</t>
         </is>
       </c>
       <c r="E271" s="4" t="inlineStr">
         <is>
-          <t>UI shows a non-fatal fallback state with retry or operator guidance instead of breaking the app shell</t>
+          <t>Runtime env file is updated, not a workspace-relative .env</t>
         </is>
       </c>
       <c r="F271" s="4" t="n"/>
@@ -8457,28 +8445,40 @@
       <c r="I271" s="4" t="n"/>
     </row>
     <row r="272">
-      <c r="A272" s="2" t="inlineStr">
-        <is>
-          <t>§12.11 First-Run Setup</t>
-        </is>
-      </c>
-      <c r="B272" s="2" t="inlineStr">
+      <c r="A272" s="4" t="inlineStr">
+        <is>
+          <t>TC-1114</t>
+        </is>
+      </c>
+      <c r="B272" s="4" t="inlineStr">
         <is>
           <t>12.11 First-Run Setup</t>
         </is>
       </c>
-      <c r="C272" s="3" t="n"/>
-      <c r="D272" s="3" t="n"/>
-      <c r="E272" s="3" t="n"/>
-      <c r="F272" s="3" t="n"/>
-      <c r="G272" s="3" t="n"/>
-      <c r="H272" s="3" t="n"/>
-      <c r="I272" s="3" t="n"/>
+      <c r="C272" s="4" t="inlineStr">
+        <is>
+          <t>Uninstall drop fails closed on invalid target</t>
+        </is>
+      </c>
+      <c r="D272" s="4" t="inlineStr">
+        <is>
+          <t>Run install.sh --uninstall --drop-database with missing/invalid/maintenance DATABASE_URL</t>
+        </is>
+      </c>
+      <c r="E272" s="4" t="inlineStr">
+        <is>
+          <t>Installer exits non-zero with explicit drop-target error; uninstall does not silently continue</t>
+        </is>
+      </c>
+      <c r="F272" s="4" t="n"/>
+      <c r="G272" s="4" t="n"/>
+      <c r="H272" s="4" t="n"/>
+      <c r="I272" s="4" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="4" t="inlineStr">
         <is>
-          <t>TC-1101</t>
+          <t>TC-1115</t>
         </is>
       </c>
       <c r="B273" s="4" t="inlineStr">
@@ -8488,17 +8488,17 @@
       </c>
       <c r="C273" s="4" t="inlineStr">
         <is>
-          <t>Status — not initialized</t>
+          <t>Setup-required API redirect</t>
         </is>
       </c>
       <c r="D273" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/status on fresh database</t>
+          <t>While using a normal UI screen, trigger a backend response with status 503, code HTTP_503, and message Database is not configured yet. Complete setup first.</t>
         </is>
       </c>
       <c r="E273" s="4" t="inlineStr">
         <is>
-          <t>200, {"initialized": false}</t>
+          <t>The browser redirects to /setup and the operator is not left only with the generic server-error toast</t>
         </is>
       </c>
       <c r="F273" s="4" t="n"/>
@@ -8509,7 +8509,7 @@
     <row r="274">
       <c r="A274" s="4" t="inlineStr">
         <is>
-          <t>TC-1102</t>
+          <t>TC-1116</t>
         </is>
       </c>
       <c r="B274" s="4" t="inlineStr">
@@ -8519,17 +8519,17 @@
       </c>
       <c r="C274" s="4" t="inlineStr">
         <is>
-          <t>Initialize</t>
+          <t>Setup password confirmation mismatch</t>
         </is>
       </c>
       <c r="D274" s="4" t="inlineStr">
         <is>
-          <t>Complete the setup wizard with matching admin password and confirmation values</t>
+          <t>In the final setup wizard step, enter different values in the admin password and confirmation fields</t>
         </is>
       </c>
       <c r="E274" s="4" t="inlineStr">
         <is>
-          <t>200, returns message, username, groups_created</t>
+          <t>The wizard shows a password-mismatch validation message and does not submit setup until the two values match</t>
         </is>
       </c>
       <c r="F274" s="4" t="n"/>
@@ -8538,60 +8538,48 @@
       <c r="I274" s="4" t="n"/>
     </row>
     <row r="275">
-      <c r="A275" s="4" t="inlineStr">
-        <is>
-          <t>TC-1103</t>
-        </is>
-      </c>
-      <c r="B275" s="4" t="inlineStr">
-        <is>
-          <t>12.11 First-Run Setup</t>
-        </is>
-      </c>
-      <c r="C275" s="4" t="inlineStr">
-        <is>
-          <t>Status — initialized</t>
-        </is>
-      </c>
-      <c r="D275" s="4" t="inlineStr">
-        <is>
-          <t>GET /setup/status after initialization</t>
-        </is>
-      </c>
-      <c r="E275" s="4" t="inlineStr">
-        <is>
-          <t>200, {"initialized": true}</t>
-        </is>
-      </c>
-      <c r="F275" s="4" t="n"/>
-      <c r="G275" s="4" t="n"/>
-      <c r="H275" s="4" t="n"/>
-      <c r="I275" s="4" t="n"/>
+      <c r="A275" s="2" t="inlineStr">
+        <is>
+          <t>§12.12 Chain-of-Custody Handoff</t>
+        </is>
+      </c>
+      <c r="B275" s="2" t="inlineStr">
+        <is>
+          <t>12.12 Chain-of-Custody Handoff</t>
+        </is>
+      </c>
+      <c r="C275" s="3" t="n"/>
+      <c r="D275" s="3" t="n"/>
+      <c r="E275" s="3" t="n"/>
+      <c r="F275" s="3" t="n"/>
+      <c r="G275" s="3" t="n"/>
+      <c r="H275" s="3" t="n"/>
+      <c r="I275" s="3" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="4" t="inlineStr">
         <is>
-          <t>TC-1104</t>
+          <t>TC-1201</t>
         </is>
       </c>
       <c r="B276" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
       <c r="C276" s="4" t="inlineStr">
         <is>
-          <t>Re-initialize informational</t>
+          <t>Retrieve stored CoC snapshot — archived job</t>
         </is>
       </c>
       <c r="D276" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize again</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for an archived job that already has a stored snapshot</t>
         </is>
       </c>
       <c r="E276" s="4" t="inlineStr">
         <is>
-          <t>200, status=already_initialized</t>
+          <t>200, response contains the stored snapshot and snapshot metadata</t>
         </is>
       </c>
       <c r="F276" s="4" t="n"/>
@@ -8602,27 +8590,27 @@
     <row r="277">
       <c r="A277" s="4" t="inlineStr">
         <is>
-          <t>TC-1105</t>
+          <t>TC-1202</t>
         </is>
       </c>
       <c r="B277" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
       <c r="C277" s="4" t="inlineStr">
         <is>
-          <t>Invalid username</t>
+          <t>Retrieve stored CoC snapshot — active job</t>
         </is>
       </c>
       <c r="D277" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with uppercase or special chars</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job that already has a stored snapshot</t>
         </is>
       </c>
       <c r="E277" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>200, response contains the stored snapshot and does not regenerate it</t>
         </is>
       </c>
       <c r="F277" s="4" t="n"/>
@@ -8633,27 +8621,27 @@
     <row r="278">
       <c r="A278" s="4" t="inlineStr">
         <is>
-          <t>TC-1106</t>
+          <t>TC-1203</t>
         </is>
       </c>
       <c r="B278" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
       <c r="C278" s="4" t="inlineStr">
         <is>
-          <t>Empty password</t>
+          <t>CoC read — missing stored snapshot</t>
         </is>
       </c>
       <c r="D278" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with {"password": ""}</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job with no stored snapshot yet</t>
         </is>
       </c>
       <c r="E278" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>404, message explains that the report must be refreshed first</t>
         </is>
       </c>
       <c r="F278" s="4" t="n"/>
@@ -8664,27 +8652,27 @@
     <row r="279">
       <c r="A279" s="4" t="inlineStr">
         <is>
-          <t>TC-1107</t>
+          <t>TC-1204</t>
         </is>
       </c>
       <c r="B279" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
       <c r="C279" s="4" t="inlineStr">
         <is>
-          <t>Unsafe password chars</t>
+          <t>CoC read — processor denied</t>
         </is>
       </c>
       <c r="D279" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with password containing newline or colon</t>
+          <t>GET /jobs/{job_id}/chain-of-custody with processor token</t>
         </is>
       </c>
       <c r="E279" s="4" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F279" s="4" t="n"/>
@@ -8695,27 +8683,27 @@
     <row r="280">
       <c r="A280" s="4" t="inlineStr">
         <is>
-          <t>TC-1108</t>
+          <t>TC-1205</t>
         </is>
       </c>
       <c r="B280" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
       <c r="C280" s="4" t="inlineStr">
         <is>
-          <t>Login as initialized admin</t>
+          <t>CoC read — unauthenticated denied</t>
         </is>
       </c>
       <c r="D280" s="4" t="inlineStr">
         <is>
-          <t>POST /auth/token with the admin credentials from step 2</t>
+          <t>GET /jobs/{job_id}/chain-of-custody without token</t>
         </is>
       </c>
       <c r="E280" s="4" t="inlineStr">
         <is>
-          <t>200, JWT contains admin role</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F280" s="4" t="n"/>
@@ -8726,27 +8714,27 @@
     <row r="281">
       <c r="A281" s="4" t="inlineStr">
         <is>
-          <t>TC-1109</t>
+          <t>TC-1206</t>
         </is>
       </c>
       <c r="B281" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
       <c r="C281" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM_INITIALIZED audit log</t>
+          <t>CoC snapshot fields</t>
         </is>
       </c>
       <c r="D281" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
+          <t>Inspect any stored-snapshot response</t>
         </is>
       </c>
       <c r="E281" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor</t>
+          <t>snapshot_stored_at, snapshot_updated_at, snapshot_stored_by, reports[], and manifest/custody fields are present</t>
         </is>
       </c>
       <c r="F281" s="4" t="n"/>
@@ -8757,27 +8745,27 @@
     <row r="282">
       <c r="A282" s="4" t="inlineStr">
         <is>
-          <t>TC-1110</t>
+          <t>TC-1207</t>
         </is>
       </c>
       <c r="B282" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
       <c r="C282" s="4" t="inlineStr">
         <is>
-          <t>Initialize default proxy trust</t>
+          <t>CoC events include lifecycle</t>
         </is>
       </c>
       <c r="D282" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize without trust_proxy_headers</t>
+          <t>Inspect chain_of_custody_events in a stored report for a completed job</t>
         </is>
       </c>
       <c r="E282" s="4" t="inlineStr">
         <is>
-          <t>200, runtime TRUST_PROXY_HEADERS=false persisted</t>
+          <t>Events include DRIVE_INITIALIZED, JOB_CREATED, JOB_STARTED, JOB_COMPLETED, DRIVE_EJECT_PREPARED, and COC_HANDOFF_CONFIRMED when applicable</t>
         </is>
       </c>
       <c r="F282" s="4" t="n"/>
@@ -8788,27 +8776,27 @@
     <row r="283">
       <c r="A283" s="4" t="inlineStr">
         <is>
-          <t>TC-1111</t>
+          <t>TC-1208</t>
         </is>
       </c>
       <c r="B283" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
       <c r="C283" s="4" t="inlineStr">
         <is>
-          <t>Initialize explicit proxy trust</t>
+          <t>CoC manifest summary</t>
         </is>
       </c>
       <c r="D283" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with "trust_proxy_headers": true</t>
+          <t>Inspect manifest_summary in the stored report</t>
         </is>
       </c>
       <c r="E283" s="4" t="inlineStr">
         <is>
-          <t>200, runtime TRUST_PROXY_HEADERS=true persisted</t>
+          <t>Array of objects with job_id, evidence_number, processor_notes, total_files, total_bytes, and manifest_count</t>
         </is>
       </c>
       <c r="F283" s="4" t="n"/>
@@ -8819,27 +8807,27 @@
     <row r="284">
       <c r="A284" s="4" t="inlineStr">
         <is>
-          <t>TC-1112</t>
+          <t>TC-1209</t>
         </is>
       </c>
       <c r="B284" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
       <c r="C284" s="4" t="inlineStr">
         <is>
-          <t>Re-initialize does not mutate runtime flags</t>
+          <t>CoC — delivery_time absence (no handoff)</t>
         </is>
       </c>
       <c r="D284" s="4" t="inlineStr">
         <is>
-          <t>Call POST /setup/initialize after setup with a different trust_proxy_headers value</t>
+          <t>Complete a job and store a snapshot before handoff</t>
         </is>
       </c>
       <c r="E284" s="4" t="inlineStr">
         <is>
-          <t>200, status=already_initialized, runtime TRUST_PROXY_HEADERS remains unchanged</t>
+          <t>chain_of_custody_events do not contain COC_HANDOFF_CONFIRMED; custody_complete is false</t>
         </is>
       </c>
       <c r="F284" s="4" t="n"/>
@@ -8850,27 +8838,27 @@
     <row r="285">
       <c r="A285" s="4" t="inlineStr">
         <is>
-          <t>TC-1113</t>
+          <t>TC-1210</t>
         </is>
       </c>
       <c r="B285" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
       <c r="C285" s="4" t="inlineStr">
         <is>
-          <t>Runtime env target consistency</t>
+          <t>CoC refresh — valid</t>
         </is>
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t>Validate running service env file target and setup persistence target are the same (ECUBE_ENV_FILE)</t>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh with admin or manager token for a non-archived job with assignments</t>
         </is>
       </c>
       <c r="E285" s="4" t="inlineStr">
         <is>
-          <t>Runtime env file is updated, not a workspace-relative .env</t>
+          <t>200, response contains the refreshed stored snapshot and updated snapshot metadata</t>
         </is>
       </c>
       <c r="F285" s="4" t="n"/>
@@ -8881,27 +8869,27 @@
     <row r="286">
       <c r="A286" s="4" t="inlineStr">
         <is>
-          <t>TC-1114</t>
+          <t>TC-1211</t>
         </is>
       </c>
       <c r="B286" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
       <c r="C286" s="4" t="inlineStr">
         <is>
-          <t>Uninstall drop fails closed on invalid target</t>
+          <t>CoC refresh — auditor denied</t>
         </is>
       </c>
       <c r="D286" s="4" t="inlineStr">
         <is>
-          <t>Run install.sh --uninstall --drop-database with missing/invalid/maintenance DATABASE_URL</t>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh with auditor token</t>
         </is>
       </c>
       <c r="E286" s="4" t="inlineStr">
         <is>
-          <t>Installer exits non-zero with explicit drop-target error; uninstall does not silently continue</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F286" s="4" t="n"/>
@@ -8912,27 +8900,27 @@
     <row r="287">
       <c r="A287" s="4" t="inlineStr">
         <is>
-          <t>TC-1115</t>
+          <t>TC-1212</t>
         </is>
       </c>
       <c r="B287" s="4" t="inlineStr">
         <is>
-          <t>12.11 First-Run Setup</t>
+          <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
       <c r="C287" s="4" t="inlineStr">
         <is>
-          <t>Setup-required API redirect</t>
+          <t>CoC refresh — archived job denied</t>
         </is>
       </c>
       <c r="D287" s="4" t="inlineStr">
         <is>
-          <t>While using a normal UI screen, trigger a backend response with status 503, code HTTP_503, and message Database is not configured yet. Complete setup first.</t>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh for an archived job</t>
         </is>
       </c>
       <c r="E287" s="4" t="inlineStr">
         <is>
-          <t>The browser redirects to /setup and the operator is not left only with the generic server-error toast</t>
+          <t>409, archived jobs can only return the last stored snapshot</t>
         </is>
       </c>
       <c r="F287" s="4" t="n"/>
@@ -8941,79 +8929,79 @@
       <c r="I287" s="4" t="n"/>
     </row>
     <row r="288">
-      <c r="A288" s="4" t="inlineStr">
-        <is>
-          <t>TC-1116</t>
-        </is>
-      </c>
-      <c r="B288" s="4" t="inlineStr">
-        <is>
-          <t>12.11 First-Run Setup</t>
-        </is>
-      </c>
-      <c r="C288" s="4" t="inlineStr">
-        <is>
-          <t>Setup password confirmation mismatch</t>
-        </is>
-      </c>
-      <c r="D288" s="4" t="inlineStr">
-        <is>
-          <t>In the final setup wizard step, enter different values in the admin password and confirmation fields</t>
-        </is>
-      </c>
-      <c r="E288" s="4" t="inlineStr">
-        <is>
-          <t>The wizard shows a password-mismatch validation message and does not submit setup until the two values match</t>
-        </is>
-      </c>
-      <c r="F288" s="4" t="n"/>
-      <c r="G288" s="4" t="n"/>
-      <c r="H288" s="4" t="n"/>
-      <c r="I288" s="4" t="n"/>
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>§12.14 Startup Reconciliation</t>
+        </is>
+      </c>
+      <c r="B288" s="2" t="inlineStr">
+        <is>
+          <t>12.14 Startup Reconciliation</t>
+        </is>
+      </c>
+      <c r="C288" s="3" t="n"/>
+      <c r="D288" s="3" t="n"/>
+      <c r="E288" s="3" t="n"/>
+      <c r="F288" s="3" t="n"/>
+      <c r="G288" s="3" t="n"/>
+      <c r="H288" s="3" t="n"/>
+      <c r="I288" s="3" t="n"/>
     </row>
     <row r="289">
-      <c r="A289" s="2" t="inlineStr">
-        <is>
-          <t>§12.12 Chain-of-Custody Handoff</t>
-        </is>
-      </c>
-      <c r="B289" s="2" t="inlineStr">
-        <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
-        </is>
-      </c>
-      <c r="C289" s="3" t="n"/>
-      <c r="D289" s="3" t="n"/>
-      <c r="E289" s="3" t="n"/>
-      <c r="F289" s="3" t="n"/>
-      <c r="G289" s="3" t="n"/>
-      <c r="H289" s="3" t="n"/>
-      <c r="I289" s="3" t="n"/>
+      <c r="A289" s="4" t="inlineStr">
+        <is>
+          <t>TC-1401</t>
+        </is>
+      </c>
+      <c r="B289" s="4" t="inlineStr">
+        <is>
+          <t>12.14 Startup Reconciliation</t>
+        </is>
+      </c>
+      <c r="C289" s="4" t="inlineStr">
+        <is>
+          <t>Running job failed after restart</t>
+        </is>
+      </c>
+      <c r="D289" s="4" t="inlineStr">
+        <is>
+          <t>Create a job, start it, restart the service while RUNNING</t>
+        </is>
+      </c>
+      <c r="E289" s="4" t="inlineStr">
+        <is>
+          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
+        </is>
+      </c>
+      <c r="F289" s="4" t="n"/>
+      <c r="G289" s="4" t="n"/>
+      <c r="H289" s="4" t="n"/>
+      <c r="I289" s="4" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="4" t="inlineStr">
         <is>
-          <t>TC-1201</t>
+          <t>TC-1402</t>
         </is>
       </c>
       <c r="B290" s="4" t="inlineStr">
         <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C290" s="4" t="inlineStr">
         <is>
-          <t>Retrieve stored CoC snapshot — archived job</t>
+          <t>Verifying job failed after restart</t>
         </is>
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for an archived job that already has a stored snapshot</t>
+          <t>Start a job, let it reach VERIFYING, restart the service</t>
         </is>
       </c>
       <c r="E290" s="4" t="inlineStr">
         <is>
-          <t>200, response contains the stored snapshot and snapshot metadata</t>
+          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
         </is>
       </c>
       <c r="F290" s="4" t="n"/>
@@ -9024,27 +9012,27 @@
     <row r="291">
       <c r="A291" s="4" t="inlineStr">
         <is>
-          <t>TC-1202</t>
+          <t>TC-1403</t>
         </is>
       </c>
       <c r="B291" s="4" t="inlineStr">
         <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C291" s="4" t="inlineStr">
         <is>
-          <t>Retrieve stored CoC snapshot — active job</t>
+          <t>Pending job not affected</t>
         </is>
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job that already has a stored snapshot</t>
+          <t>Create a job (PENDING), restart the service</t>
         </is>
       </c>
       <c r="E291" s="4" t="inlineStr">
         <is>
-          <t>200, response contains the stored snapshot and does not regenerate it</t>
+          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
         </is>
       </c>
       <c r="F291" s="4" t="n"/>
@@ -9055,27 +9043,27 @@
     <row r="292">
       <c r="A292" s="4" t="inlineStr">
         <is>
-          <t>TC-1203</t>
+          <t>TC-1404</t>
         </is>
       </c>
       <c r="B292" s="4" t="inlineStr">
         <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C292" s="4" t="inlineStr">
         <is>
-          <t>CoC read — missing stored snapshot</t>
+          <t>Completed job not affected</t>
         </is>
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job with no stored snapshot yet</t>
+          <t>Complete a job, restart the service</t>
         </is>
       </c>
       <c r="E292" s="4" t="inlineStr">
         <is>
-          <t>404, message explains that the report must be refreshed first</t>
+          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F292" s="4" t="n"/>
@@ -9086,27 +9074,27 @@
     <row r="293">
       <c r="A293" s="4" t="inlineStr">
         <is>
-          <t>TC-1204</t>
+          <t>TC-1405</t>
         </is>
       </c>
       <c r="B293" s="4" t="inlineStr">
         <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C293" s="4" t="inlineStr">
         <is>
-          <t>CoC read — processor denied</t>
+          <t>Stale mount corrected</t>
         </is>
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody with processor token</t>
+          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
         </is>
       </c>
       <c r="E293" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
         </is>
       </c>
       <c r="F293" s="4" t="n"/>
@@ -9117,27 +9105,27 @@
     <row r="294">
       <c r="A294" s="4" t="inlineStr">
         <is>
-          <t>TC-1205</t>
+          <t>TC-1406</t>
         </is>
       </c>
       <c r="B294" s="4" t="inlineStr">
         <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C294" s="4" t="inlineStr">
         <is>
-          <t>CoC read — unauthenticated denied</t>
+          <t>Active mount preserved</t>
         </is>
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody without token</t>
+          <t>Add and mount a network share (leave it mounted), restart the service</t>
         </is>
       </c>
       <c r="E294" s="4" t="inlineStr">
         <is>
-          <t>401, UNAUTHORIZED</t>
+          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F294" s="4" t="n"/>
@@ -9148,27 +9136,27 @@
     <row r="295">
       <c r="A295" s="4" t="inlineStr">
         <is>
-          <t>TC-1206</t>
+          <t>TC-1407</t>
         </is>
       </c>
       <c r="B295" s="4" t="inlineStr">
         <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C295" s="4" t="inlineStr">
         <is>
-          <t>CoC snapshot fields</t>
+          <t>USB drives re-discovered</t>
         </is>
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>Inspect any stored-snapshot response</t>
+          <t>Insert USB drives, restart the service</t>
         </is>
       </c>
       <c r="E295" s="4" t="inlineStr">
         <is>
-          <t>snapshot_stored_at, snapshot_updated_at, snapshot_stored_by, reports[], and manifest/custody fields are present</t>
+          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
         </is>
       </c>
       <c r="F295" s="4" t="n"/>
@@ -9179,27 +9167,27 @@
     <row r="296">
       <c r="A296" s="4" t="inlineStr">
         <is>
-          <t>TC-1207</t>
+          <t>TC-1408</t>
         </is>
       </c>
       <c r="B296" s="4" t="inlineStr">
         <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C296" s="4" t="inlineStr">
         <is>
-          <t>CoC events include lifecycle</t>
+          <t>Idempotency</t>
         </is>
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t>Inspect chain_of_custody_events in a stored report for a completed job</t>
+          <t>Restart the service twice without any state changes between restarts</t>
         </is>
       </c>
       <c r="E296" s="4" t="inlineStr">
         <is>
-          <t>Events include DRIVE_INITIALIZED, JOB_CREATED, JOB_STARTED, JOB_COMPLETED, DRIVE_EJECT_PREPARED, and COC_HANDOFF_CONFIRMED when applicable</t>
+          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
         </is>
       </c>
       <c r="F296" s="4" t="n"/>
@@ -9210,27 +9198,27 @@
     <row r="297">
       <c r="A297" s="4" t="inlineStr">
         <is>
-          <t>TC-1208</t>
+          <t>TC-1409</t>
         </is>
       </c>
       <c r="B297" s="4" t="inlineStr">
         <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C297" s="4" t="inlineStr">
         <is>
-          <t>CoC manifest summary</t>
+          <t>Partial failure isolation</t>
         </is>
       </c>
       <c r="D297" s="4" t="inlineStr">
         <is>
-          <t>Inspect manifest_summary in the stored report</t>
+          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
         </is>
       </c>
       <c r="E297" s="4" t="inlineStr">
         <is>
-          <t>Array of objects with job_id, evidence_number, processor_notes, total_files, total_bytes, and manifest_count</t>
+          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
         </is>
       </c>
       <c r="F297" s="4" t="n"/>
@@ -9241,27 +9229,27 @@
     <row r="298">
       <c r="A298" s="4" t="inlineStr">
         <is>
-          <t>TC-1209</t>
+          <t>TC-1410</t>
         </is>
       </c>
       <c r="B298" s="4" t="inlineStr">
         <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C298" s="4" t="inlineStr">
         <is>
-          <t>CoC — delivery_time absence (no handoff)</t>
+          <t>Cross-process lock — only one worker reconciles</t>
         </is>
       </c>
       <c r="D298" s="4" t="inlineStr">
         <is>
-          <t>Complete a job and store a snapshot before handoff</t>
+          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
         </is>
       </c>
       <c r="E298" s="4" t="inlineStr">
         <is>
-          <t>chain_of_custody_events do not contain COC_HANDOFF_CONFIRMED; custody_complete is false</t>
+          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
         </is>
       </c>
       <c r="F298" s="4" t="n"/>
@@ -9272,27 +9260,27 @@
     <row r="299">
       <c r="A299" s="4" t="inlineStr">
         <is>
-          <t>TC-1210</t>
+          <t>TC-1411</t>
         </is>
       </c>
       <c r="B299" s="4" t="inlineStr">
         <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C299" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — valid</t>
+          <t>Stale lock reclaim</t>
         </is>
       </c>
       <c r="D299" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh with admin or manager token for a non-archived job with assignments</t>
+          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
         </is>
       </c>
       <c r="E299" s="4" t="inlineStr">
         <is>
-          <t>200, response contains the refreshed stored snapshot and updated snapshot metadata</t>
+          <t>Service reclaims the stale lock, reconciliation runs normally</t>
         </is>
       </c>
       <c r="F299" s="4" t="n"/>
@@ -9303,27 +9291,27 @@
     <row r="300">
       <c r="A300" s="4" t="inlineStr">
         <is>
-          <t>TC-1211</t>
+          <t>TC-1412</t>
         </is>
       </c>
       <c r="B300" s="4" t="inlineStr">
         <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C300" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — auditor denied</t>
+          <t>Lock released after failure</t>
         </is>
       </c>
       <c r="D300" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh with auditor token</t>
+          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
         </is>
       </c>
       <c r="E300" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
         </is>
       </c>
       <c r="F300" s="4" t="n"/>
@@ -9334,27 +9322,27 @@
     <row r="301">
       <c r="A301" s="4" t="inlineStr">
         <is>
-          <t>TC-1212</t>
+          <t>TC-1413</t>
         </is>
       </c>
       <c r="B301" s="4" t="inlineStr">
         <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C301" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — archived job denied</t>
+          <t>Jobs pass emits immediate startup result log</t>
         </is>
       </c>
       <c r="D301" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh for an archived job</t>
+          <t>Create at least one RUNNING job, restart service, then inspect application logs around startup reconciliation</t>
         </is>
       </c>
       <c r="E301" s="4" t="inlineStr">
         <is>
-          <t>409, archived jobs can only return the last stored snapshot</t>
+          <t>Logs include Startup reconciliation: checking jobs followed by an immediate Startup reconciliation: jobs result line with safe counts (jobs_checked, jobs_corrected) or safe failure classification</t>
         </is>
       </c>
       <c r="F301" s="4" t="n"/>
@@ -9363,28 +9351,40 @@
       <c r="I301" s="4" t="n"/>
     </row>
     <row r="302">
-      <c r="A302" s="2" t="inlineStr">
-        <is>
-          <t>§12.14 Startup Reconciliation</t>
-        </is>
-      </c>
-      <c r="B302" s="2" t="inlineStr">
+      <c r="A302" s="4" t="inlineStr">
+        <is>
+          <t>TC-1414</t>
+        </is>
+      </c>
+      <c r="B302" s="4" t="inlineStr">
         <is>
           <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
-      <c r="C302" s="3" t="n"/>
-      <c r="D302" s="3" t="n"/>
-      <c r="E302" s="3" t="n"/>
-      <c r="F302" s="3" t="n"/>
-      <c r="G302" s="3" t="n"/>
-      <c r="H302" s="3" t="n"/>
-      <c r="I302" s="3" t="n"/>
+      <c r="C302" s="4" t="inlineStr">
+        <is>
+          <t>Reconciled job persists restart-interruption failure reason</t>
+        </is>
+      </c>
+      <c r="D302" s="4" t="inlineStr">
+        <is>
+          <t>Create a RUNNING or VERIFYING job, restart service, then open Job Detail for that job</t>
+        </is>
+      </c>
+      <c r="E302" s="4" t="inlineStr">
+        <is>
+          <t>Job status is FAILED and Job Detail shows a stable restart interruption reason (not the generic This job failed... fallback)</t>
+        </is>
+      </c>
+      <c r="F302" s="4" t="n"/>
+      <c r="G302" s="4" t="n"/>
+      <c r="H302" s="4" t="n"/>
+      <c r="I302" s="4" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="4" t="inlineStr">
         <is>
-          <t>TC-1401</t>
+          <t>TC-1415</t>
         </is>
       </c>
       <c r="B303" s="4" t="inlineStr">
@@ -9394,17 +9394,17 @@
       </c>
       <c r="C303" s="4" t="inlineStr">
         <is>
-          <t>Running job failed after restart</t>
+          <t>Reconciled failed job shows correlated failure entry from audit fallback</t>
         </is>
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>Create a job, start it, restart the service while RUNNING</t>
+          <t>Restart with a RUNNING job, then inspect Job Detail when no matching file-log failure line is present</t>
         </is>
       </c>
       <c r="E303" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
+          <t>Job Detail still shows a related failure entry sourced from reconciliation evidence (JOB_RECONCILED) and the entry remains sanitized</t>
         </is>
       </c>
       <c r="F303" s="4" t="n"/>
@@ -9415,7 +9415,7 @@
     <row r="304">
       <c r="A304" s="4" t="inlineStr">
         <is>
-          <t>TC-1402</t>
+          <t>TC-1416</t>
         </is>
       </c>
       <c r="B304" s="4" t="inlineStr">
@@ -9425,17 +9425,17 @@
       </c>
       <c r="C304" s="4" t="inlineStr">
         <is>
-          <t>Verifying job failed after restart</t>
+          <t>Failed job API uses reconciliation audit fallback when file-log correlation is unavailable</t>
         </is>
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>Start a job, let it reach VERIFYING, restart the service</t>
+          <t>In a test environment, disable file-log correlation (log_file unset), then request GET /jobs/{job_id} for a restart-reconciled failed job</t>
         </is>
       </c>
       <c r="E304" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
+          <t>Response remains 200 and includes the stable restart failure reason plus a sanitized failure_log_entry derived from audit evidence (JOB_RECONCILED)</t>
         </is>
       </c>
       <c r="F304" s="4" t="n"/>
@@ -9446,7 +9446,7 @@
     <row r="305">
       <c r="A305" s="4" t="inlineStr">
         <is>
-          <t>TC-1403</t>
+          <t>TC-1417</t>
         </is>
       </c>
       <c r="B305" s="4" t="inlineStr">
@@ -9456,17 +9456,17 @@
       </c>
       <c r="C305" s="4" t="inlineStr">
         <is>
-          <t>Pending job not affected</t>
+          <t>Jobs pass failure path emits safe startup result classification</t>
         </is>
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>Create a job (PENDING), restart the service</t>
+          <t>In a controlled test environment, force a jobs-pass reconciliation exception, then restart service and inspect startup logs</t>
         </is>
       </c>
       <c r="E305" s="4" t="inlineStr">
         <is>
-          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
+          <t>Logs still include Startup reconciliation: jobs result with status=failed and reason=job_reconciliation_failed, without raw provider errors or host paths</t>
         </is>
       </c>
       <c r="F305" s="4" t="n"/>
@@ -9477,7 +9477,7 @@
     <row r="306">
       <c r="A306" s="4" t="inlineStr">
         <is>
-          <t>TC-1404</t>
+          <t>TC-1418</t>
         </is>
       </c>
       <c r="B306" s="4" t="inlineStr">
@@ -9487,17 +9487,17 @@
       </c>
       <c r="C306" s="4" t="inlineStr">
         <is>
-          <t>Completed job not affected</t>
+          <t>Restart clears stale in-progress startup analysis when no valid cache remains</t>
         </is>
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>Complete a job, restart the service</t>
+          <t>Trigger manual Analyze for a PENDING job, restart ECUBE before the scan completes, then reopen Job Detail</t>
         </is>
       </c>
       <c r="E306" s="4" t="inlineStr">
         <is>
-          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
+          <t>Job is no longer stuck in ANALYZING, startup-analysis state returns to NOT_ANALYZED, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "analysis_interrupted_by_restart", and Analyze or Start is available again</t>
         </is>
       </c>
       <c r="F306" s="4" t="n"/>
@@ -9508,7 +9508,7 @@
     <row r="307">
       <c r="A307" s="4" t="inlineStr">
         <is>
-          <t>TC-1405</t>
+          <t>TC-1419</t>
         </is>
       </c>
       <c r="B307" s="4" t="inlineStr">
@@ -9518,17 +9518,17 @@
       </c>
       <c r="C307" s="4" t="inlineStr">
         <is>
-          <t>Stale mount corrected</t>
+          <t>Restart restores READY when the interrupted startup-analysis cache is still current</t>
         </is>
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
+          <t>Trigger manual Analyze for a job with a stable source tree, restart ECUBE after the reusable snapshot has been persisted but before the manual analyze workflow fully completes, then reopen Job Detail</t>
         </is>
       </c>
       <c r="E307" s="4" t="inlineStr">
         <is>
-          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
+          <t>Job shows startup_analysis_status: READY, the previous file and byte totals are still available, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "valid_cache_restored_after_restart", and Start can proceed without forcing a fresh scan</t>
         </is>
       </c>
       <c r="F307" s="4" t="n"/>
@@ -9537,60 +9537,48 @@
       <c r="I307" s="4" t="n"/>
     </row>
     <row r="308">
-      <c r="A308" s="4" t="inlineStr">
-        <is>
-          <t>TC-1406</t>
-        </is>
-      </c>
-      <c r="B308" s="4" t="inlineStr">
-        <is>
-          <t>12.14 Startup Reconciliation</t>
-        </is>
-      </c>
-      <c r="C308" s="4" t="inlineStr">
-        <is>
-          <t>Active mount preserved</t>
-        </is>
-      </c>
-      <c r="D308" s="4" t="inlineStr">
-        <is>
-          <t>Add and mount a network share (leave it mounted), restart the service</t>
-        </is>
-      </c>
-      <c r="E308" s="4" t="inlineStr">
-        <is>
-          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
-        </is>
-      </c>
-      <c r="F308" s="4" t="n"/>
-      <c r="G308" s="4" t="n"/>
-      <c r="H308" s="4" t="n"/>
-      <c r="I308" s="4" t="n"/>
+      <c r="A308" s="2" t="inlineStr">
+        <is>
+          <t>§12.15 System Health</t>
+        </is>
+      </c>
+      <c r="B308" s="2" t="inlineStr">
+        <is>
+          <t>12.15 System Health</t>
+        </is>
+      </c>
+      <c r="C308" s="3" t="n"/>
+      <c r="D308" s="3" t="n"/>
+      <c r="E308" s="3" t="n"/>
+      <c r="F308" s="3" t="n"/>
+      <c r="G308" s="3" t="n"/>
+      <c r="H308" s="3" t="n"/>
+      <c r="I308" s="3" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="4" t="inlineStr">
         <is>
-          <t>TC-1407</t>
+          <t>TC-1501</t>
         </is>
       </c>
       <c r="B309" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C309" s="4" t="inlineStr">
         <is>
-          <t>USB drives re-discovered</t>
+          <t>Healthy response</t>
         </is>
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>Insert USB drives, restart the service</t>
+          <t>GET /introspection/system-health with valid token</t>
         </is>
       </c>
       <c r="E309" s="4" t="inlineStr">
         <is>
-          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
+          <t>200, status: "ok", database: "connected"</t>
         </is>
       </c>
       <c r="F309" s="4" t="n"/>
@@ -9601,27 +9589,27 @@
     <row r="310">
       <c r="A310" s="4" t="inlineStr">
         <is>
-          <t>TC-1408</t>
+          <t>TC-1502</t>
         </is>
       </c>
       <c r="B310" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C310" s="4" t="inlineStr">
         <is>
-          <t>Idempotency</t>
+          <t>CPU metric present</t>
         </is>
       </c>
       <c r="D310" s="4" t="inlineStr">
         <is>
-          <t>Restart the service twice without any state changes between restarts</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E310" s="4" t="inlineStr">
         <is>
-          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
+          <t>cpu_percent is a number between 0 and 100</t>
         </is>
       </c>
       <c r="F310" s="4" t="n"/>
@@ -9632,27 +9620,27 @@
     <row r="311">
       <c r="A311" s="4" t="inlineStr">
         <is>
-          <t>TC-1409</t>
+          <t>TC-1503</t>
         </is>
       </c>
       <c r="B311" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C311" s="4" t="inlineStr">
         <is>
-          <t>Partial failure isolation</t>
+          <t>Memory metrics present</t>
         </is>
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E311" s="4" t="inlineStr">
         <is>
-          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
+          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
         </is>
       </c>
       <c r="F311" s="4" t="n"/>
@@ -9663,27 +9651,27 @@
     <row r="312">
       <c r="A312" s="4" t="inlineStr">
         <is>
-          <t>TC-1410</t>
+          <t>TC-1504</t>
         </is>
       </c>
       <c r="B312" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C312" s="4" t="inlineStr">
         <is>
-          <t>Cross-process lock — only one worker reconciles</t>
+          <t>Disk I/O metrics present</t>
         </is>
       </c>
       <c r="D312" s="4" t="inlineStr">
         <is>
-          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E312" s="4" t="inlineStr">
         <is>
-          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
+          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
         </is>
       </c>
       <c r="F312" s="4" t="n"/>
@@ -9694,27 +9682,27 @@
     <row r="313">
       <c r="A313" s="4" t="inlineStr">
         <is>
-          <t>TC-1411</t>
+          <t>TC-1505</t>
         </is>
       </c>
       <c r="B313" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C313" s="4" t="inlineStr">
         <is>
-          <t>Stale lock reclaim</t>
+          <t>Active jobs count</t>
         </is>
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
+          <t>Start an export job, call endpoint</t>
         </is>
       </c>
       <c r="E313" s="4" t="inlineStr">
         <is>
-          <t>Service reclaims the stale lock, reconciliation runs normally</t>
+          <t>active_jobs ≥ 1</t>
         </is>
       </c>
       <c r="F313" s="4" t="n"/>
@@ -9725,27 +9713,27 @@
     <row r="314">
       <c r="A314" s="4" t="inlineStr">
         <is>
-          <t>TC-1412</t>
+          <t>TC-1506</t>
         </is>
       </c>
       <c r="B314" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C314" s="4" t="inlineStr">
         <is>
-          <t>Lock released after failure</t>
+          <t>Worker queue size</t>
         </is>
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
+          <t>Create a PENDING job (created but not started), call endpoint</t>
         </is>
       </c>
       <c r="E314" s="4" t="inlineStr">
         <is>
-          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
+          <t>worker_queue_size ≥ 1</t>
         </is>
       </c>
       <c r="F314" s="4" t="n"/>
@@ -9756,27 +9744,27 @@
     <row r="315">
       <c r="A315" s="4" t="inlineStr">
         <is>
-          <t>TC-1413</t>
+          <t>TC-1507</t>
         </is>
       </c>
       <c r="B315" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C315" s="4" t="inlineStr">
         <is>
-          <t>Jobs pass emits immediate startup result log</t>
+          <t>Worker queue size decrements</t>
         </is>
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>Create at least one RUNNING job, restart service, then inspect application logs around startup reconciliation</t>
+          <t>Start the pending job, call endpoint again</t>
         </is>
       </c>
       <c r="E315" s="4" t="inlineStr">
         <is>
-          <t>Logs include Startup reconciliation: checking jobs followed by an immediate Startup reconciliation: jobs result line with safe counts (jobs_checked, jobs_corrected) or safe failure classification</t>
+          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
         </is>
       </c>
       <c r="F315" s="4" t="n"/>
@@ -9787,27 +9775,27 @@
     <row r="316">
       <c r="A316" s="4" t="inlineStr">
         <is>
-          <t>TC-1414</t>
+          <t>TC-1508</t>
         </is>
       </c>
       <c r="B316" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C316" s="4" t="inlineStr">
         <is>
-          <t>Reconciled job persists restart-interruption failure reason</t>
+          <t>ECUBE process metrics present</t>
         </is>
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>Create a RUNNING or VERIFYING job, restart service, then open Job Detail for that job</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E316" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED and Job Detail shows a stable restart interruption reason (not the generic This job failed... fallback)</t>
+          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
         </is>
       </c>
       <c r="F316" s="4" t="n"/>
@@ -9818,27 +9806,27 @@
     <row r="317">
       <c r="A317" s="4" t="inlineStr">
         <is>
-          <t>TC-1415</t>
+          <t>TC-1509</t>
         </is>
       </c>
       <c r="B317" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C317" s="4" t="inlineStr">
         <is>
-          <t>Reconciled failed job shows correlated failure entry from audit fallback</t>
+          <t>Active copy-thread correlation</t>
         </is>
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t>Restart with a RUNNING job, then inspect Job Detail when no matching file-log failure line is present</t>
+          <t>Run an export job with active copy workers, call endpoint during the run</t>
         </is>
       </c>
       <c r="E317" s="4" t="inlineStr">
         <is>
-          <t>Job Detail still shows a related failure entry sourced from reconciliation evidence (JOB_RECONCILED) and the entry remains sanitized</t>
+          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
         </is>
       </c>
       <c r="F317" s="4" t="n"/>
@@ -9849,27 +9837,27 @@
     <row r="318">
       <c r="A318" s="4" t="inlineStr">
         <is>
-          <t>TC-1416</t>
+          <t>TC-1510</t>
         </is>
       </c>
       <c r="B318" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C318" s="4" t="inlineStr">
         <is>
-          <t>Failed job API uses reconciliation audit fallback when file-log correlation is unavailable</t>
+          <t>ECUBE process metrics degrade safely</t>
         </is>
       </c>
       <c r="D318" s="4" t="inlineStr">
         <is>
-          <t>In a test environment, disable file-log correlation (log_file unset), then request GET /jobs/{job_id} for a restart-reconciled failed job</t>
+          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
         </is>
       </c>
       <c r="E318" s="4" t="inlineStr">
         <is>
-          <t>Response remains 200 and includes the stable restart failure reason plus a sanitized failure_log_entry derived from audit evidence (JOB_RECONCILED)</t>
+          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
         </is>
       </c>
       <c r="F318" s="4" t="n"/>
@@ -9880,27 +9868,27 @@
     <row r="319">
       <c r="A319" s="4" t="inlineStr">
         <is>
-          <t>TC-1417</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B319" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C319" s="4" t="inlineStr">
         <is>
-          <t>Jobs pass failure path emits safe startup result classification</t>
+          <t>Degraded when DB down</t>
         </is>
       </c>
       <c r="D319" s="4" t="inlineStr">
         <is>
-          <t>In a controlled test environment, force a jobs-pass reconciliation exception, then restart service and inspect startup logs</t>
+          <t>Stop PostgreSQL, call endpoint with valid token</t>
         </is>
       </c>
       <c r="E319" s="4" t="inlineStr">
         <is>
-          <t>Logs still include Startup reconciliation: jobs result with status=failed and reason=job_reconciliation_failed, without raw provider errors or host paths</t>
+          <t>200, status: "degraded", database: "error", database_error is non-null</t>
         </is>
       </c>
       <c r="F319" s="4" t="n"/>
@@ -9911,27 +9899,27 @@
     <row r="320">
       <c r="A320" s="4" t="inlineStr">
         <is>
-          <t>TC-1418</t>
+          <t>TC-1512</t>
         </is>
       </c>
       <c r="B320" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C320" s="4" t="inlineStr">
         <is>
-          <t>Restart clears stale in-progress startup analysis when no valid cache remains</t>
+          <t>Unauthenticated rejected</t>
         </is>
       </c>
       <c r="D320" s="4" t="inlineStr">
         <is>
-          <t>Trigger manual Analyze for a PENDING job, restart ECUBE before the scan completes, then reopen Job Detail</t>
+          <t>GET /introspection/system-health without token</t>
         </is>
       </c>
       <c r="E320" s="4" t="inlineStr">
         <is>
-          <t>Job is no longer stuck in ANALYZING, startup-analysis state returns to NOT_ANALYZED, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "analysis_interrupted_by_restart", and Analyze or Start is available again</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F320" s="4" t="n"/>
@@ -9942,27 +9930,27 @@
     <row r="321">
       <c r="A321" s="4" t="inlineStr">
         <is>
-          <t>TC-1419</t>
+          <t>TC-1513</t>
         </is>
       </c>
       <c r="B321" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C321" s="4" t="inlineStr">
         <is>
-          <t>Restart restores READY when the interrupted startup-analysis cache is still current</t>
+          <t>Processor role allowed</t>
         </is>
       </c>
       <c r="D321" s="4" t="inlineStr">
         <is>
-          <t>Trigger manual Analyze for a job with a stable source tree, restart ECUBE after the reusable snapshot has been persisted but before the manual analyze workflow fully completes, then reopen Job Detail</t>
+          <t>GET /introspection/system-health with processor token</t>
         </is>
       </c>
       <c r="E321" s="4" t="inlineStr">
         <is>
-          <t>Job shows startup_analysis_status: READY, the previous file and byte totals are still available, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "valid_cache_restored_after_restart", and Start can proceed without forcing a fresh scan</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F321" s="4" t="n"/>
@@ -9973,12 +9961,12 @@
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>§12.15 System Health</t>
+          <t>§12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
       <c r="B322" s="2" t="inlineStr">
         <is>
-          <t>12.15 System Health</t>
+          <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
       <c r="C322" s="3" t="n"/>
@@ -9992,27 +9980,27 @@
     <row r="323">
       <c r="A323" s="4" t="inlineStr">
         <is>
-          <t>TC-1501</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B323" s="4" t="inlineStr">
         <is>
-          <t>12.15 System Health</t>
+          <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
       <c r="C323" s="4" t="inlineStr">
         <is>
-          <t>Healthy response</t>
+          <t>Liveness endpoint is public</t>
         </is>
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with valid token</t>
+          <t>GET /health/live without token</t>
         </is>
       </c>
       <c r="E323" s="4" t="inlineStr">
         <is>
-          <t>200, status: "ok", database: "connected"</t>
+          <t>200, service reports live</t>
         </is>
       </c>
       <c r="F323" s="4" t="n"/>
@@ -10023,27 +10011,27 @@
     <row r="324">
       <c r="A324" s="4" t="inlineStr">
         <is>
-          <t>TC-1502</t>
+          <t>TC-1512</t>
         </is>
       </c>
       <c r="B324" s="4" t="inlineStr">
         <is>
-          <t>12.15 System Health</t>
+          <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
       <c r="C324" s="4" t="inlineStr">
         <is>
-          <t>CPU metric present</t>
+          <t>Readiness endpoint is public</t>
         </is>
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>GET /health/ready without token on a healthy system</t>
         </is>
       </c>
       <c r="E324" s="4" t="inlineStr">
         <is>
-          <t>cpu_percent is a number between 0 and 100</t>
+          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
         </is>
       </c>
       <c r="F324" s="4" t="n"/>
@@ -10054,27 +10042,27 @@
     <row r="325">
       <c r="A325" s="4" t="inlineStr">
         <is>
-          <t>TC-1503</t>
+          <t>TC-1513</t>
         </is>
       </c>
       <c r="B325" s="4" t="inlineStr">
         <is>
-          <t>12.15 System Health</t>
+          <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
       <c r="C325" s="4" t="inlineStr">
         <is>
-          <t>Memory metrics present</t>
+          <t>Readiness reports missing database configuration</t>
         </is>
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Clear DB config or test before configuration, then GET /health/ready</t>
         </is>
       </c>
       <c r="E325" s="4" t="inlineStr">
         <is>
-          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
+          <t>503, status: "not_ready", reason indicates database is not configured</t>
         </is>
       </c>
       <c r="F325" s="4" t="n"/>
@@ -10085,27 +10073,27 @@
     <row r="326">
       <c r="A326" s="4" t="inlineStr">
         <is>
-          <t>TC-1504</t>
+          <t>TC-1514</t>
         </is>
       </c>
       <c r="B326" s="4" t="inlineStr">
         <is>
-          <t>12.15 System Health</t>
+          <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
       <c r="C326" s="4" t="inlineStr">
         <is>
-          <t>Disk I/O metrics present</t>
+          <t>Readiness reports mount or provider problems</t>
         </is>
       </c>
       <c r="D326" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Break a configured mount or provider, then GET /health/ready</t>
         </is>
       </c>
       <c r="E326" s="4" t="inlineStr">
         <is>
-          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
+          <t>503, response identifies the failing check without using the generic error schema</t>
         </is>
       </c>
       <c r="F326" s="4" t="n"/>
@@ -10116,27 +10104,27 @@
     <row r="327">
       <c r="A327" s="4" t="inlineStr">
         <is>
-          <t>TC-1505</t>
+          <t>TC-1515</t>
         </is>
       </c>
       <c r="B327" s="4" t="inlineStr">
         <is>
-          <t>12.15 System Health</t>
+          <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
       <c r="C327" s="4" t="inlineStr">
         <is>
-          <t>Active jobs count</t>
+          <t>Version endpoint is public</t>
         </is>
       </c>
       <c r="D327" s="4" t="inlineStr">
         <is>
-          <t>Start an export job, call endpoint</t>
+          <t>GET /introspection/version without token</t>
         </is>
       </c>
       <c r="E327" s="4" t="inlineStr">
         <is>
-          <t>active_jobs ≥ 1</t>
+          <t>200, returns version/application metadata</t>
         </is>
       </c>
       <c r="F327" s="4" t="n"/>
@@ -10147,27 +10135,27 @@
     <row r="328">
       <c r="A328" s="4" t="inlineStr">
         <is>
-          <t>TC-1506</t>
+          <t>TC-1516</t>
         </is>
       </c>
       <c r="B328" s="4" t="inlineStr">
         <is>
-          <t>12.15 System Health</t>
+          <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
       <c r="C328" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size</t>
+          <t>Readiness remains separate from authenticated system health</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr">
         <is>
-          <t>Create a PENDING job (created but not started), call endpoint</t>
+          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
         </is>
       </c>
       <c r="E328" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size ≥ 1</t>
+          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
         </is>
       </c>
       <c r="F328" s="4" t="n"/>
@@ -10176,454 +10164,32 @@
       <c r="I328" s="4" t="n"/>
     </row>
     <row r="329">
-      <c r="A329" s="4" t="inlineStr">
-        <is>
-          <t>TC-1507</t>
-        </is>
-      </c>
-      <c r="B329" s="4" t="inlineStr">
-        <is>
-          <t>12.15 System Health</t>
-        </is>
-      </c>
-      <c r="C329" s="4" t="inlineStr">
-        <is>
-          <t>Worker queue size decrements</t>
-        </is>
-      </c>
-      <c r="D329" s="4" t="inlineStr">
-        <is>
-          <t>Start the pending job, call endpoint again</t>
-        </is>
-      </c>
-      <c r="E329" s="4" t="inlineStr">
-        <is>
-          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved to RUNNING)</t>
-        </is>
-      </c>
-      <c r="F329" s="4" t="n"/>
-      <c r="G329" s="4" t="n"/>
-      <c r="H329" s="4" t="n"/>
-      <c r="I329" s="4" t="n"/>
-    </row>
-    <row r="330">
-      <c r="A330" s="4" t="inlineStr">
-        <is>
-          <t>TC-1508</t>
-        </is>
-      </c>
-      <c r="B330" s="4" t="inlineStr">
-        <is>
-          <t>12.15 System Health</t>
-        </is>
-      </c>
-      <c r="C330" s="4" t="inlineStr">
-        <is>
-          <t>ECUBE process metrics present</t>
-        </is>
-      </c>
-      <c r="D330" s="4" t="inlineStr">
-        <is>
-          <t>Inspect response body</t>
-        </is>
-      </c>
-      <c r="E330" s="4" t="inlineStr">
-        <is>
-          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
-        </is>
-      </c>
-      <c r="F330" s="4" t="n"/>
-      <c r="G330" s="4" t="n"/>
-      <c r="H330" s="4" t="n"/>
-      <c r="I330" s="4" t="n"/>
+      <c r="A329" s="2" t="inlineStr">
+        <is>
+          <t>§12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
+        </is>
+      </c>
+      <c r="B329" s="2" t="inlineStr">
+        <is>
+          <t>12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
+        </is>
+      </c>
+      <c r="C329" s="3" t="n"/>
+      <c r="D329" s="3" t="n"/>
+      <c r="E329" s="3" t="n"/>
+      <c r="F329" s="3" t="n"/>
+      <c r="G329" s="3" t="n"/>
+      <c r="H329" s="3" t="n"/>
+      <c r="I329" s="3" t="n"/>
     </row>
     <row r="331">
-      <c r="A331" s="4" t="inlineStr">
-        <is>
-          <t>TC-1509</t>
-        </is>
-      </c>
-      <c r="B331" s="4" t="inlineStr">
-        <is>
-          <t>12.15 System Health</t>
-        </is>
-      </c>
-      <c r="C331" s="4" t="inlineStr">
-        <is>
-          <t>Active copy-thread correlation</t>
-        </is>
-      </c>
-      <c r="D331" s="4" t="inlineStr">
-        <is>
-          <t>Run an export job with active copy workers, call endpoint during the run</t>
-        </is>
-      </c>
-      <c r="E331" s="4" t="inlineStr">
-        <is>
-          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
-        </is>
-      </c>
-      <c r="F331" s="4" t="n"/>
-      <c r="G331" s="4" t="n"/>
-      <c r="H331" s="4" t="n"/>
-      <c r="I331" s="4" t="n"/>
-    </row>
-    <row r="332">
-      <c r="A332" s="4" t="inlineStr">
-        <is>
-          <t>TC-1510</t>
-        </is>
-      </c>
-      <c r="B332" s="4" t="inlineStr">
-        <is>
-          <t>12.15 System Health</t>
-        </is>
-      </c>
-      <c r="C332" s="4" t="inlineStr">
-        <is>
-          <t>ECUBE process metrics degrade safely</t>
-        </is>
-      </c>
-      <c r="D332" s="4" t="inlineStr">
-        <is>
-          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
-        </is>
-      </c>
-      <c r="E332" s="4" t="inlineStr">
-        <is>
-          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
-        </is>
-      </c>
-      <c r="F332" s="4" t="n"/>
-      <c r="G332" s="4" t="n"/>
-      <c r="H332" s="4" t="n"/>
-      <c r="I332" s="4" t="n"/>
-    </row>
-    <row r="333">
-      <c r="A333" s="4" t="inlineStr">
-        <is>
-          <t>TC-1511</t>
-        </is>
-      </c>
-      <c r="B333" s="4" t="inlineStr">
-        <is>
-          <t>12.15 System Health</t>
-        </is>
-      </c>
-      <c r="C333" s="4" t="inlineStr">
-        <is>
-          <t>Degraded when DB down</t>
-        </is>
-      </c>
-      <c r="D333" s="4" t="inlineStr">
-        <is>
-          <t>Stop PostgreSQL, call endpoint with valid token</t>
-        </is>
-      </c>
-      <c r="E333" s="4" t="inlineStr">
-        <is>
-          <t>200, status: "degraded", database: "error", database_error is non-null</t>
-        </is>
-      </c>
-      <c r="F333" s="4" t="n"/>
-      <c r="G333" s="4" t="n"/>
-      <c r="H333" s="4" t="n"/>
-      <c r="I333" s="4" t="n"/>
-    </row>
-    <row r="334">
-      <c r="A334" s="4" t="inlineStr">
-        <is>
-          <t>TC-1512</t>
-        </is>
-      </c>
-      <c r="B334" s="4" t="inlineStr">
-        <is>
-          <t>12.15 System Health</t>
-        </is>
-      </c>
-      <c r="C334" s="4" t="inlineStr">
-        <is>
-          <t>Unauthenticated rejected</t>
-        </is>
-      </c>
-      <c r="D334" s="4" t="inlineStr">
-        <is>
-          <t>GET /introspection/system-health without token</t>
-        </is>
-      </c>
-      <c r="E334" s="4" t="inlineStr">
-        <is>
-          <t>401</t>
-        </is>
-      </c>
-      <c r="F334" s="4" t="n"/>
-      <c r="G334" s="4" t="n"/>
-      <c r="H334" s="4" t="n"/>
-      <c r="I334" s="4" t="n"/>
-    </row>
-    <row r="335">
-      <c r="A335" s="4" t="inlineStr">
-        <is>
-          <t>TC-1513</t>
-        </is>
-      </c>
-      <c r="B335" s="4" t="inlineStr">
-        <is>
-          <t>12.15 System Health</t>
-        </is>
-      </c>
-      <c r="C335" s="4" t="inlineStr">
-        <is>
-          <t>Processor role allowed</t>
-        </is>
-      </c>
-      <c r="D335" s="4" t="inlineStr">
-        <is>
-          <t>GET /introspection/system-health with processor token</t>
-        </is>
-      </c>
-      <c r="E335" s="4" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="F335" s="4" t="n"/>
-      <c r="G335" s="4" t="n"/>
-      <c r="H335" s="4" t="n"/>
-      <c r="I335" s="4" t="n"/>
-    </row>
-    <row r="336">
-      <c r="A336" s="2" t="inlineStr">
-        <is>
-          <t>§12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="B336" s="2" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C336" s="3" t="n"/>
-      <c r="D336" s="3" t="n"/>
-      <c r="E336" s="3" t="n"/>
-      <c r="F336" s="3" t="n"/>
-      <c r="G336" s="3" t="n"/>
-      <c r="H336" s="3" t="n"/>
-      <c r="I336" s="3" t="n"/>
-    </row>
-    <row r="337">
-      <c r="A337" s="4" t="inlineStr">
-        <is>
-          <t>TC-1511</t>
-        </is>
-      </c>
-      <c r="B337" s="4" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C337" s="4" t="inlineStr">
-        <is>
-          <t>Liveness endpoint is public</t>
-        </is>
-      </c>
-      <c r="D337" s="4" t="inlineStr">
-        <is>
-          <t>GET /health/live without token</t>
-        </is>
-      </c>
-      <c r="E337" s="4" t="inlineStr">
-        <is>
-          <t>200, service reports live</t>
-        </is>
-      </c>
-      <c r="F337" s="4" t="n"/>
-      <c r="G337" s="4" t="n"/>
-      <c r="H337" s="4" t="n"/>
-      <c r="I337" s="4" t="n"/>
-    </row>
-    <row r="338">
-      <c r="A338" s="4" t="inlineStr">
-        <is>
-          <t>TC-1512</t>
-        </is>
-      </c>
-      <c r="B338" s="4" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C338" s="4" t="inlineStr">
-        <is>
-          <t>Readiness endpoint is public</t>
-        </is>
-      </c>
-      <c r="D338" s="4" t="inlineStr">
-        <is>
-          <t>GET /health/ready without token on a healthy system</t>
-        </is>
-      </c>
-      <c r="E338" s="4" t="inlineStr">
-        <is>
-          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
-        </is>
-      </c>
-      <c r="F338" s="4" t="n"/>
-      <c r="G338" s="4" t="n"/>
-      <c r="H338" s="4" t="n"/>
-      <c r="I338" s="4" t="n"/>
-    </row>
-    <row r="339">
-      <c r="A339" s="4" t="inlineStr">
-        <is>
-          <t>TC-1513</t>
-        </is>
-      </c>
-      <c r="B339" s="4" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C339" s="4" t="inlineStr">
-        <is>
-          <t>Readiness reports missing database configuration</t>
-        </is>
-      </c>
-      <c r="D339" s="4" t="inlineStr">
-        <is>
-          <t>Clear DB config or test before configuration, then GET /health/ready</t>
-        </is>
-      </c>
-      <c r="E339" s="4" t="inlineStr">
-        <is>
-          <t>503, status: "not_ready", reason indicates database is not configured</t>
-        </is>
-      </c>
-      <c r="F339" s="4" t="n"/>
-      <c r="G339" s="4" t="n"/>
-      <c r="H339" s="4" t="n"/>
-      <c r="I339" s="4" t="n"/>
-    </row>
-    <row r="340">
-      <c r="A340" s="4" t="inlineStr">
-        <is>
-          <t>TC-1514</t>
-        </is>
-      </c>
-      <c r="B340" s="4" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C340" s="4" t="inlineStr">
-        <is>
-          <t>Readiness reports mount or provider problems</t>
-        </is>
-      </c>
-      <c r="D340" s="4" t="inlineStr">
-        <is>
-          <t>Break a configured mount or provider, then GET /health/ready</t>
-        </is>
-      </c>
-      <c r="E340" s="4" t="inlineStr">
-        <is>
-          <t>503, response identifies the failing check without using the generic error schema</t>
-        </is>
-      </c>
-      <c r="F340" s="4" t="n"/>
-      <c r="G340" s="4" t="n"/>
-      <c r="H340" s="4" t="n"/>
-      <c r="I340" s="4" t="n"/>
-    </row>
-    <row r="341">
-      <c r="A341" s="4" t="inlineStr">
-        <is>
-          <t>TC-1515</t>
-        </is>
-      </c>
-      <c r="B341" s="4" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C341" s="4" t="inlineStr">
-        <is>
-          <t>Version endpoint is public</t>
-        </is>
-      </c>
-      <c r="D341" s="4" t="inlineStr">
-        <is>
-          <t>GET /introspection/version without token</t>
-        </is>
-      </c>
-      <c r="E341" s="4" t="inlineStr">
-        <is>
-          <t>200, returns version/application metadata</t>
-        </is>
-      </c>
-      <c r="F341" s="4" t="n"/>
-      <c r="G341" s="4" t="n"/>
-      <c r="H341" s="4" t="n"/>
-      <c r="I341" s="4" t="n"/>
-    </row>
-    <row r="342">
-      <c r="A342" s="4" t="inlineStr">
-        <is>
-          <t>TC-1516</t>
-        </is>
-      </c>
-      <c r="B342" s="4" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C342" s="4" t="inlineStr">
-        <is>
-          <t>Readiness remains separate from authenticated system health</t>
-        </is>
-      </c>
-      <c r="D342" s="4" t="inlineStr">
-        <is>
-          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
-        </is>
-      </c>
-      <c r="E342" s="4" t="inlineStr">
-        <is>
-          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
-        </is>
-      </c>
-      <c r="F342" s="4" t="n"/>
-      <c r="G342" s="4" t="n"/>
-      <c r="H342" s="4" t="n"/>
-      <c r="I342" s="4" t="n"/>
-    </row>
-    <row r="343">
-      <c r="A343" s="2" t="inlineStr">
-        <is>
-          <t>§12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
-        </is>
-      </c>
-      <c r="B343" s="2" t="inlineStr">
-        <is>
-          <t>12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
-        </is>
-      </c>
-      <c r="C343" s="3" t="n"/>
-      <c r="D343" s="3" t="n"/>
-      <c r="E343" s="3" t="n"/>
-      <c r="F343" s="3" t="n"/>
-      <c r="G343" s="3" t="n"/>
-      <c r="H343" s="3" t="n"/>
-      <c r="I343" s="3" t="n"/>
-    </row>
-    <row r="345">
-      <c r="A345" s="5" t="inlineStr">
+      <c r="A331" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B345" s="5" t="n">
-        <v>315</v>
+      <c r="B331" s="5" t="n">
+        <v>301</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ui test and qa documentation
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -4423,7 +4423,7 @@
       </c>
       <c r="E136" s="4" t="inlineStr">
         <is>
-          <t>Once formatting clears the project binding, Drive Detail shows Evidence and Job ID as -, the Drives row no longer shows the old job ID value, and stale job links are not shown for that drive</t>
+          <t>Once formatting clears the project binding, Drive Detail shows Evidence and Job ID as -, the Drives row does not show the prior job ID value, and stale job links are not shown for that drive</t>
         </is>
       </c>
       <c r="F136" s="4" t="n"/>
@@ -4547,7 +4547,7 @@
       </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
-          <t>The Drives list does not show a Size column, Drive Detail shows total capacity plus the last known available space value or - when no reading is available yet, and the mounted drive exposes a Browse button instead of a mount-path link</t>
+          <t>The Drives list does not show a Size column, Drive Detail shows total capacity plus the last known available space value or - when no reading is available yet, and the mounted drive exposes a Browse button without exposing a raw mount-path link</t>
         </is>
       </c>
       <c r="F140" s="4" t="n"/>
@@ -9497,7 +9497,7 @@
       </c>
       <c r="E306" s="4" t="inlineStr">
         <is>
-          <t>Job is no longer stuck in ANALYZING, startup-analysis state returns to NOT_ANALYZED, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "analysis_interrupted_by_restart", and Analyze or Start is available again</t>
+          <t>Job does not remain stuck in ANALYZING, startup-analysis state returns to NOT_ANALYZED, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "analysis_interrupted_by_restart", and Analyze or Start is available again</t>
         </is>
       </c>
       <c r="F306" s="4" t="n"/>

</xml_diff>

<commit_message>
Fix issue where correct serial number is not shown on CoC
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -8662,7 +8662,7 @@
       </c>
       <c r="C279" s="4" t="inlineStr">
         <is>
-          <t>CoC read — processor denied</t>
+          <t>CoC read — processor allowed</t>
         </is>
       </c>
       <c r="D279" s="4" t="inlineStr">
@@ -8672,7 +8672,7 @@
       </c>
       <c r="E279" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>200 when a stored snapshot exists; otherwise 404 with refresh guidance</t>
         </is>
       </c>
       <c r="F279" s="4" t="n"/>
@@ -8734,7 +8734,7 @@
       </c>
       <c r="E281" s="4" t="inlineStr">
         <is>
-          <t>snapshot_stored_at, snapshot_updated_at, snapshot_stored_by, reports[], and manifest/custody fields are present</t>
+          <t>snapshot_stored_at, snapshot_updated_at, snapshot_stored_by, reports[], and manifest/custody fields are present; drive_sn shows the parsed hardware serial when available and is blank when unavailable</t>
         </is>
       </c>
       <c r="F281" s="4" t="n"/>

</xml_diff>

<commit_message>
Show negotiated USB speed in USB topology and drive detail views
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -4206,7 +4206,7 @@
       </c>
       <c r="E129" s="4" t="inlineStr">
         <is>
-          <t>Shows real device values, serial numbers when available, sorted Device order, and no rows with entirely empty USB metadata</t>
+          <t>Shows real device values, serial numbers when available, negotiated USB speed when available, sorted Device order, and no rows with entirely empty USB metadata</t>
         </is>
       </c>
       <c r="F129" s="4" t="n"/>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>Mounted drive surfaces capacity, available space, and Browse entry</t>
+          <t>Mounted drive surfaces capacity, available space, speed, and Browse entry</t>
         </is>
       </c>
       <c r="D140" s="4" t="inlineStr">
@@ -4547,7 +4547,7 @@
       </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
-          <t>The Drives list does not show a Size column, Drive Detail shows total capacity plus the last known available space value or - when no reading is available yet, and the mounted drive exposes a Browse button without exposing a raw mount-path link</t>
+          <t>The Drives list does not show a Size column, Drive Detail shows total capacity, negotiated USB speed when available or - when it is unavailable, plus the last known available space value or - when no reading is available yet, and the mounted drive exposes a Browse button without exposing a raw mount-path link</t>
         </is>
       </c>
       <c r="F140" s="4" t="n"/>

</xml_diff>

<commit_message>
Add mounted drive/share throughput testing in detail views
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -4537,7 +4537,7 @@
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>Mounted drive surfaces capacity, available space, speed, and Browse entry</t>
+          <t>Mounted drive surfaces capacity, available space, speed, throughput, and Browse entry</t>
         </is>
       </c>
       <c r="D140" s="4" t="inlineStr">
@@ -4547,7 +4547,7 @@
       </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
-          <t>The Drives list does not show a Size column, Drive Detail shows total capacity, negotiated USB speed when available or - when it is unavailable, plus the last known available space value or - when no reading is available yet, and the mounted drive exposes a Browse button without exposing a raw mount-path link</t>
+          <t>The Drives list does not show a Size column, Drive Detail shows total capacity, negotiated USB speed when available or - when it is unavailable, the latest stored write-throughput values when a prior test exists, plus the last known available space value or - when no reading is available yet, and the mounted drive exposes Browse plus manager/admin Test Throughput without exposing a raw mount-path link</t>
         </is>
       </c>
       <c r="F140" s="4" t="n"/>

</xml_diff>

<commit_message>
Fixed more stale docs
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -3624,12 +3624,12 @@
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>Create an NFS mount, then POST /mounts/{mount_id}/validate</t>
+          <t>Create an NFS share, then POST /shares/{share_id}/validate</t>
         </is>
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
-          <t>200, mount remains MOUNTED, last_checked_at advances</t>
+          <t>200, share remains MOUNTED, last_checked_at advances</t>
         </is>
       </c>
       <c r="F110" s="4" t="n"/>
@@ -3655,12 +3655,12 @@
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>Create an SMB mount, then POST /mounts/{mount_id}/validate</t>
+          <t>Create an SMB share, then POST /shares/{share_id}/validate</t>
         </is>
       </c>
       <c r="E111" s="4" t="inlineStr">
         <is>
-          <t>200, mount remains MOUNTED</t>
+          <t>200, share remains MOUNTED</t>
         </is>
       </c>
       <c r="F111" s="4" t="n"/>
@@ -3681,17 +3681,17 @@
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>Validate disconnected mount</t>
+          <t>Validate disconnected share</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>Break connectivity or unmount externally, then POST /mounts/{mount_id}/validate</t>
+          <t>Break connectivity or unmount externally, then POST /shares/{share_id}/validate</t>
         </is>
       </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
-          <t>200, mount status becomes UNMOUNTED or ERROR with a descriptive error</t>
+          <t>200, share status becomes UNMOUNTED or ERROR with a descriptive error</t>
         </is>
       </c>
       <c r="F112" s="4" t="n"/>
@@ -3712,17 +3712,17 @@
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>Validate all mounts reports mixed states</t>
+          <t>Validate all shares reports mixed states</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>Register one reachable mount and one broken mount, then POST /mounts/validate</t>
+          <t>Register one reachable share and one broken share, then POST /shares/validate</t>
         </is>
       </c>
       <c r="E113" s="4" t="inlineStr">
         <is>
-          <t>200, response includes updated status for each mount</t>
+          <t>200, response includes updated status for each share</t>
         </is>
       </c>
       <c r="F113" s="4" t="n"/>
@@ -3743,12 +3743,12 @@
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>Validate missing mount</t>
+          <t>Validate missing share</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>POST /mounts/9999/validate</t>
+          <t>POST /shares/9999/validate</t>
         </is>
       </c>
       <c r="E114" s="4" t="inlineStr">
@@ -3774,12 +3774,12 @@
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>Processor cannot validate mounts</t>
+          <t>Processor cannot validate shares</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>POST /mounts/{mount_id}/validate with processor token</t>
+          <t>POST /shares/{share_id}/validate with processor token</t>
         </is>
       </c>
       <c r="E115" s="4" t="inlineStr">
@@ -3805,17 +3805,17 @@
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>Mount validation audit trail</t>
+          <t>Share validation audit trail</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>Validate a mount, then query GET /audit?action=MOUNT_VALIDATED</t>
+          <t>Validate a share, then query GET /audit?action=MOUNT_VALIDATED</t>
         </is>
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>Audit entry records actor, mount id, and resulting status</t>
+          <t>Audit entry records actor, share id, and resulting status</t>
         </is>
       </c>
       <c r="F116" s="4" t="n"/>
@@ -3841,7 +3841,7 @@
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>Create a mount, then submit the same remote_path again for the same project</t>
+          <t>Create a share, then submit the same remote_path again for the same project</t>
         </is>
       </c>
       <c r="E117" s="4" t="inlineStr">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="E119" s="4" t="inlineStr">
         <is>
-          <t>200, second mount is accepted</t>
+          <t>200, second share is accepted</t>
         </is>
       </c>
       <c r="F119" s="4" t="n"/>
@@ -3929,17 +3929,17 @@
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>Edit an active NFS mount with a new per-share client version</t>
+          <t>Edit an active NFS share with a new per-share client version</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>Update the mount through PATCH /mounts/{mount_id} or the Mount Detail Edit dialog while the share is MOUNTED</t>
+          <t>Update the share through PATCH /shares/{share_id} or the Share Detail Edit dialog while the share is MOUNTED</t>
         </is>
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>200, the mount remains MOUNTED, the returned nfs_client_version matches the edited override, and the live share is remounted with the new option</t>
+          <t>200, the share remains MOUNTED, the returned nfs_client_version matches the edited override, and the live share is remounted with the new option</t>
         </is>
       </c>
       <c r="F120" s="4" t="n"/>
@@ -3965,7 +3965,7 @@
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>Create an SMB mount with slash-separated path, then submit the same source with backslash separators</t>
+          <t>Create an SMB share with slash-separated path, then submit the same source with backslash separators</t>
         </is>
       </c>
       <c r="E121" s="4" t="inlineStr">
@@ -3996,12 +3996,12 @@
       </c>
       <c r="D122" s="4" t="inlineStr">
         <is>
-          <t>Submit two near-simultaneous add-mount requests for the same remote source from separate sessions</t>
+          <t>Submit two near-simultaneous add-share requests for the same remote source from separate sessions</t>
         </is>
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>Only one mount is created; the competing request returns a safe conflict instead of producing duplicates</t>
+          <t>Only one share is created; the competing request returns a safe conflict instead of producing duplicates</t>
         </is>
       </c>
       <c r="F122" s="4" t="n"/>
@@ -4027,7 +4027,7 @@
       </c>
       <c r="D123" s="4" t="inlineStr">
         <is>
-          <t>Edit an existing SMB mount in the UI, change only remote path or project ID, and save without entering credential values</t>
+          <t>Edit an existing SMB share in the UI, change only remote path or project ID, and save without entering credential values</t>
         </is>
       </c>
       <c r="E123" s="4" t="inlineStr">
@@ -4058,7 +4058,7 @@
       </c>
       <c r="D124" s="4" t="inlineStr">
         <is>
-          <t>Edit an existing SMB mount in the UI, click Clear saved credentials, and save</t>
+          <t>Edit an existing SMB share in the UI, click Clear saved credentials, and save</t>
         </is>
       </c>
       <c r="E124" s="4" t="inlineStr">
@@ -4084,12 +4084,12 @@
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>Returned mount error keeps edit dialog open</t>
+          <t>Returned share error keeps edit dialog open</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
         <is>
-          <t>Edit a mount so the backend returns an updated mount object with status: ERROR</t>
+          <t>Edit a share so the backend returns an updated share object with status: ERROR</t>
         </is>
       </c>
       <c r="E125" s="4" t="inlineStr">
@@ -4115,12 +4115,12 @@
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>Mounts list shows related Job ID for the mounted project</t>
+          <t>Shares list shows related Job ID for the mounted project</t>
         </is>
       </c>
       <c r="D126" s="4" t="inlineStr">
         <is>
-          <t>Seed or create a job for the same project as a listed mount, then open Mounts</t>
+          <t>Seed or create a job for the same project as a listed share, then open Shares</t>
         </is>
       </c>
       <c r="E126" s="4" t="inlineStr">
@@ -7761,7 +7761,7 @@
       </c>
       <c r="D249" s="4" t="inlineStr">
         <is>
-          <t>Open Help while on Drives, Mounts, Jobs, or Audit, then close it</t>
+          <t>Open Help while on Drives, Shares, Jobs, or Audit, then close it</t>
         </is>
       </c>
       <c r="E249" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Login page should never display demo shared password in plain text
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -6926,12 +6926,12 @@
       </c>
       <c r="D220" s="4" t="inlineStr">
         <is>
-          <t>Enable demo mode with DEMO_SHARED_PASSWORD unset, verify the login screen password, change Password Policy settings, restart ECUBE, then retry demo sign-in with the newly displayed password</t>
+          <t>Enable demo mode with DEMO_SHARED_PASSWORD unset, verify demo sign-in works, change Password Policy settings, restart ECUBE, then retry demo sign-in using the updated effective password from demo configuration</t>
         </is>
       </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
-          <t>The shared password shown on the login page changes to match the updated policy, and the restarted service accepts that password for the demo accounts</t>
+          <t>The restarted service accepts a password that matches the updated policy for the demo accounts, and the login page continues to prefill the password field without displaying the raw value</t>
         </is>
       </c>
       <c r="F220" s="4" t="n"/>

</xml_diff>

<commit_message>
Enumerate and displays both physical cores and logical CPUs in System Health Host Metrics
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I319"/>
+  <dimension ref="A1:I321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9286,17 +9286,17 @@
       </c>
       <c r="C299" s="4" t="inlineStr">
         <is>
-          <t>Memory metrics present</t>
+          <t>CPU topology metrics present</t>
         </is>
       </c>
       <c r="D299" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Inspect response body on a host where psutil reports CPU topology</t>
         </is>
       </c>
       <c r="E299" s="4" t="inlineStr">
         <is>
-          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
+          <t>physical_cores and logical_cpus are positive integers; logical_cpus ≥ physical_cores</t>
         </is>
       </c>
       <c r="F299" s="4" t="n"/>
@@ -9317,17 +9317,17 @@
       </c>
       <c r="C300" s="4" t="inlineStr">
         <is>
-          <t>Disk I/O metrics present</t>
+          <t>CPU topology metrics unavailable path</t>
         </is>
       </c>
       <c r="D300" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Exercise endpoint where psutil is unavailable</t>
         </is>
       </c>
       <c r="E300" s="4" t="inlineStr">
         <is>
-          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
+          <t>physical_cores and logical_cpus are null</t>
         </is>
       </c>
       <c r="F300" s="4" t="n"/>
@@ -9348,17 +9348,17 @@
       </c>
       <c r="C301" s="4" t="inlineStr">
         <is>
-          <t>Active jobs count</t>
+          <t>Memory metrics present</t>
         </is>
       </c>
       <c r="D301" s="4" t="inlineStr">
         <is>
-          <t>Start an export job, call endpoint</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E301" s="4" t="inlineStr">
         <is>
-          <t>active_jobs ≥ 1</t>
+          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
         </is>
       </c>
       <c r="F301" s="4" t="n"/>
@@ -9379,17 +9379,17 @@
       </c>
       <c r="C302" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size</t>
+          <t>Disk I/O metrics present</t>
         </is>
       </c>
       <c r="D302" s="4" t="inlineStr">
         <is>
-          <t>Create a PENDING job (created but not started), call endpoint</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E302" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size ≥ 1</t>
+          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
         </is>
       </c>
       <c r="F302" s="4" t="n"/>
@@ -9410,17 +9410,17 @@
       </c>
       <c r="C303" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size decrements</t>
+          <t>Active jobs count</t>
         </is>
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>Start the pending job, call endpoint again</t>
+          <t>Start an export job, call endpoint</t>
         </is>
       </c>
       <c r="E303" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved out of PENDING and can still be in PREPARING before it reaches RUNNING)</t>
+          <t>active_jobs ≥ 1</t>
         </is>
       </c>
       <c r="F303" s="4" t="n"/>
@@ -9441,17 +9441,17 @@
       </c>
       <c r="C304" s="4" t="inlineStr">
         <is>
-          <t>ECUBE process metrics present</t>
+          <t>Worker queue size</t>
         </is>
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Create a PENDING job (created but not started), call endpoint</t>
         </is>
       </c>
       <c r="E304" s="4" t="inlineStr">
         <is>
-          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
+          <t>worker_queue_size ≥ 1</t>
         </is>
       </c>
       <c r="F304" s="4" t="n"/>
@@ -9472,17 +9472,17 @@
       </c>
       <c r="C305" s="4" t="inlineStr">
         <is>
-          <t>Active copy-thread correlation</t>
+          <t>Worker queue size decrements</t>
         </is>
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>Run an export job with active copy workers, call endpoint during the run</t>
+          <t>Start the pending job, call endpoint again</t>
         </is>
       </c>
       <c r="E305" s="4" t="inlineStr">
         <is>
-          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
+          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved out of PENDING and can still be in PREPARING before it reaches RUNNING)</t>
         </is>
       </c>
       <c r="F305" s="4" t="n"/>
@@ -9503,17 +9503,17 @@
       </c>
       <c r="C306" s="4" t="inlineStr">
         <is>
-          <t>ECUBE process metrics degrade safely</t>
+          <t>ECUBE process metrics present</t>
         </is>
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E306" s="4" t="inlineStr">
         <is>
-          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
+          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
         </is>
       </c>
       <c r="F306" s="4" t="n"/>
@@ -9534,17 +9534,17 @@
       </c>
       <c r="C307" s="4" t="inlineStr">
         <is>
-          <t>Degraded when DB down</t>
+          <t>Active copy-thread correlation</t>
         </is>
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, call endpoint with valid token</t>
+          <t>Run an export job with active copy workers, call endpoint during the run</t>
         </is>
       </c>
       <c r="E307" s="4" t="inlineStr">
         <is>
-          <t>200, status: "degraded", database: "error", database_error is non-null</t>
+          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
         </is>
       </c>
       <c r="F307" s="4" t="n"/>
@@ -9565,17 +9565,17 @@
       </c>
       <c r="C308" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated rejected</t>
+          <t>ECUBE process metrics degrade safely</t>
         </is>
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health without token</t>
+          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
         </is>
       </c>
       <c r="E308" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
         </is>
       </c>
       <c r="F308" s="4" t="n"/>
@@ -9596,17 +9596,17 @@
       </c>
       <c r="C309" s="4" t="inlineStr">
         <is>
-          <t>Processor role allowed</t>
+          <t>Degraded when DB down</t>
         </is>
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with processor token</t>
+          <t>Stop PostgreSQL, call endpoint with valid token</t>
         </is>
       </c>
       <c r="E309" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, status: "degraded", database: "error", database_error is non-null</t>
         </is>
       </c>
       <c r="F309" s="4" t="n"/>
@@ -9615,48 +9615,60 @@
       <c r="I309" s="4" t="n"/>
     </row>
     <row r="310">
-      <c r="A310" s="2" t="inlineStr">
-        <is>
-          <t>§12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="B310" s="2" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C310" s="3" t="n"/>
-      <c r="D310" s="3" t="n"/>
-      <c r="E310" s="3" t="n"/>
-      <c r="F310" s="3" t="n"/>
-      <c r="G310" s="3" t="n"/>
-      <c r="H310" s="3" t="n"/>
-      <c r="I310" s="3" t="n"/>
+      <c r="A310" s="4" t="inlineStr">
+        <is>
+          <t>TC-1514</t>
+        </is>
+      </c>
+      <c r="B310" s="4" t="inlineStr">
+        <is>
+          <t>12.15 System Health</t>
+        </is>
+      </c>
+      <c r="C310" s="4" t="inlineStr">
+        <is>
+          <t>Unauthenticated rejected</t>
+        </is>
+      </c>
+      <c r="D310" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/system-health without token</t>
+        </is>
+      </c>
+      <c r="E310" s="4" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="F310" s="4" t="n"/>
+      <c r="G310" s="4" t="n"/>
+      <c r="H310" s="4" t="n"/>
+      <c r="I310" s="4" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="4" t="inlineStr">
         <is>
-          <t>TC-1511</t>
+          <t>TC-1515</t>
         </is>
       </c>
       <c r="B311" s="4" t="inlineStr">
         <is>
-          <t>12.15.1 Readiness &amp; Version</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C311" s="4" t="inlineStr">
         <is>
-          <t>Liveness endpoint is public</t>
+          <t>Processor role allowed</t>
         </is>
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>GET /health/live without token</t>
+          <t>GET /introspection/system-health with processor token</t>
         </is>
       </c>
       <c r="E311" s="4" t="inlineStr">
         <is>
-          <t>200, service reports live</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F311" s="4" t="n"/>
@@ -9665,40 +9677,28 @@
       <c r="I311" s="4" t="n"/>
     </row>
     <row r="312">
-      <c r="A312" s="4" t="inlineStr">
-        <is>
-          <t>TC-1512</t>
-        </is>
-      </c>
-      <c r="B312" s="4" t="inlineStr">
+      <c r="A312" s="2" t="inlineStr">
+        <is>
+          <t>§12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="B312" s="2" t="inlineStr">
         <is>
           <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
-      <c r="C312" s="4" t="inlineStr">
-        <is>
-          <t>Readiness endpoint is public</t>
-        </is>
-      </c>
-      <c r="D312" s="4" t="inlineStr">
-        <is>
-          <t>GET /health/ready without token on a healthy system</t>
-        </is>
-      </c>
-      <c r="E312" s="4" t="inlineStr">
-        <is>
-          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
-        </is>
-      </c>
-      <c r="F312" s="4" t="n"/>
-      <c r="G312" s="4" t="n"/>
-      <c r="H312" s="4" t="n"/>
-      <c r="I312" s="4" t="n"/>
+      <c r="C312" s="3" t="n"/>
+      <c r="D312" s="3" t="n"/>
+      <c r="E312" s="3" t="n"/>
+      <c r="F312" s="3" t="n"/>
+      <c r="G312" s="3" t="n"/>
+      <c r="H312" s="3" t="n"/>
+      <c r="I312" s="3" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="4" t="inlineStr">
         <is>
-          <t>TC-1513</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B313" s="4" t="inlineStr">
@@ -9708,17 +9708,17 @@
       </c>
       <c r="C313" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports missing database configuration</t>
+          <t>Liveness endpoint is public</t>
         </is>
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>Clear DB config or test before configuration, then GET /health/ready</t>
+          <t>GET /health/live without token</t>
         </is>
       </c>
       <c r="E313" s="4" t="inlineStr">
         <is>
-          <t>503, status: "not_ready", reason indicates database is not configured</t>
+          <t>200, service reports live</t>
         </is>
       </c>
       <c r="F313" s="4" t="n"/>
@@ -9729,7 +9729,7 @@
     <row r="314">
       <c r="A314" s="4" t="inlineStr">
         <is>
-          <t>TC-1514</t>
+          <t>TC-1512</t>
         </is>
       </c>
       <c r="B314" s="4" t="inlineStr">
@@ -9739,17 +9739,17 @@
       </c>
       <c r="C314" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports mount or provider problems</t>
+          <t>Readiness endpoint is public</t>
         </is>
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>Break a configured mount or provider, then GET /health/ready</t>
+          <t>GET /health/ready without token on a healthy system</t>
         </is>
       </c>
       <c r="E314" s="4" t="inlineStr">
         <is>
-          <t>503, response identifies the failing check without using the generic error schema</t>
+          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
         </is>
       </c>
       <c r="F314" s="4" t="n"/>
@@ -9760,7 +9760,7 @@
     <row r="315">
       <c r="A315" s="4" t="inlineStr">
         <is>
-          <t>TC-1515</t>
+          <t>TC-1513</t>
         </is>
       </c>
       <c r="B315" s="4" t="inlineStr">
@@ -9770,17 +9770,17 @@
       </c>
       <c r="C315" s="4" t="inlineStr">
         <is>
-          <t>Version endpoint is public</t>
+          <t>Readiness reports missing database configuration</t>
         </is>
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/version without token</t>
+          <t>Clear DB config or test before configuration, then GET /health/ready</t>
         </is>
       </c>
       <c r="E315" s="4" t="inlineStr">
         <is>
-          <t>200, returns version/application metadata</t>
+          <t>503, status: "not_ready", reason indicates database is not configured</t>
         </is>
       </c>
       <c r="F315" s="4" t="n"/>
@@ -9791,7 +9791,7 @@
     <row r="316">
       <c r="A316" s="4" t="inlineStr">
         <is>
-          <t>TC-1516</t>
+          <t>TC-1514</t>
         </is>
       </c>
       <c r="B316" s="4" t="inlineStr">
@@ -9801,17 +9801,17 @@
       </c>
       <c r="C316" s="4" t="inlineStr">
         <is>
-          <t>Readiness remains separate from authenticated system health</t>
+          <t>Readiness reports mount or provider problems</t>
         </is>
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+          <t>Break a configured mount or provider, then GET /health/ready</t>
         </is>
       </c>
       <c r="E316" s="4" t="inlineStr">
         <is>
-          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+          <t>503, response identifies the failing check without using the generic error schema</t>
         </is>
       </c>
       <c r="F316" s="4" t="n"/>
@@ -9820,32 +9820,94 @@
       <c r="I316" s="4" t="n"/>
     </row>
     <row r="317">
-      <c r="A317" s="2" t="inlineStr">
+      <c r="A317" s="4" t="inlineStr">
+        <is>
+          <t>TC-1515</t>
+        </is>
+      </c>
+      <c r="B317" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C317" s="4" t="inlineStr">
+        <is>
+          <t>Version endpoint is public</t>
+        </is>
+      </c>
+      <c r="D317" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/version without token</t>
+        </is>
+      </c>
+      <c r="E317" s="4" t="inlineStr">
+        <is>
+          <t>200, returns version/application metadata</t>
+        </is>
+      </c>
+      <c r="F317" s="4" t="n"/>
+      <c r="G317" s="4" t="n"/>
+      <c r="H317" s="4" t="n"/>
+      <c r="I317" s="4" t="n"/>
+    </row>
+    <row r="318">
+      <c r="A318" s="4" t="inlineStr">
+        <is>
+          <t>TC-1516</t>
+        </is>
+      </c>
+      <c r="B318" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C318" s="4" t="inlineStr">
+        <is>
+          <t>Readiness remains separate from authenticated system health</t>
+        </is>
+      </c>
+      <c r="D318" s="4" t="inlineStr">
+        <is>
+          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+        </is>
+      </c>
+      <c r="E318" s="4" t="inlineStr">
+        <is>
+          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+        </is>
+      </c>
+      <c r="F318" s="4" t="n"/>
+      <c r="G318" s="4" t="n"/>
+      <c r="H318" s="4" t="n"/>
+      <c r="I318" s="4" t="n"/>
+    </row>
+    <row r="319">
+      <c r="A319" s="2" t="inlineStr">
         <is>
           <t>§12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="B317" s="2" t="inlineStr">
+      <c r="B319" s="2" t="inlineStr">
         <is>
           <t>12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="C317" s="3" t="n"/>
-      <c r="D317" s="3" t="n"/>
-      <c r="E317" s="3" t="n"/>
-      <c r="F317" s="3" t="n"/>
-      <c r="G317" s="3" t="n"/>
-      <c r="H317" s="3" t="n"/>
-      <c r="I317" s="3" t="n"/>
-    </row>
-    <row r="319">
-      <c r="A319" s="5" t="inlineStr">
+      <c r="C319" s="3" t="n"/>
+      <c r="D319" s="3" t="n"/>
+      <c r="E319" s="3" t="n"/>
+      <c r="F319" s="3" t="n"/>
+      <c r="G319" s="3" t="n"/>
+      <c r="H319" s="3" t="n"/>
+      <c r="I319" s="3" t="n"/>
+    </row>
+    <row r="321">
+      <c r="A321" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B319" s="5" t="n">
-        <v>289</v>
+      <c r="B321" s="5" t="n">
+        <v>291</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added observability logs for CPU topology metric sampling failures Added QA guide scenario for UI fallback rendering
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I321"/>
+  <dimension ref="A1:I322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9348,17 +9348,17 @@
       </c>
       <c r="C301" s="4" t="inlineStr">
         <is>
-          <t>Memory metrics present</t>
+          <t>System page CPU topology fallback rendering</t>
         </is>
       </c>
       <c r="D301" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Open System -&gt; System Health when backend returns physical_cores: null and logical_cpus: null</t>
         </is>
       </c>
       <c r="E301" s="4" t="inlineStr">
         <is>
-          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
+          <t>Physical Cores and Logical CPUs display N/A; other host metrics continue rendering normally</t>
         </is>
       </c>
       <c r="F301" s="4" t="n"/>
@@ -9379,7 +9379,7 @@
       </c>
       <c r="C302" s="4" t="inlineStr">
         <is>
-          <t>Disk I/O metrics present</t>
+          <t>Memory metrics present</t>
         </is>
       </c>
       <c r="D302" s="4" t="inlineStr">
@@ -9389,7 +9389,7 @@
       </c>
       <c r="E302" s="4" t="inlineStr">
         <is>
-          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
+          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
         </is>
       </c>
       <c r="F302" s="4" t="n"/>
@@ -9410,17 +9410,17 @@
       </c>
       <c r="C303" s="4" t="inlineStr">
         <is>
-          <t>Active jobs count</t>
+          <t>Disk I/O metrics present</t>
         </is>
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>Start an export job, call endpoint</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E303" s="4" t="inlineStr">
         <is>
-          <t>active_jobs ≥ 1</t>
+          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
         </is>
       </c>
       <c r="F303" s="4" t="n"/>
@@ -9441,17 +9441,17 @@
       </c>
       <c r="C304" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size</t>
+          <t>Active jobs count</t>
         </is>
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>Create a PENDING job (created but not started), call endpoint</t>
+          <t>Start an export job, call endpoint</t>
         </is>
       </c>
       <c r="E304" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size ≥ 1</t>
+          <t>active_jobs ≥ 1</t>
         </is>
       </c>
       <c r="F304" s="4" t="n"/>
@@ -9472,17 +9472,17 @@
       </c>
       <c r="C305" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size decrements</t>
+          <t>Worker queue size</t>
         </is>
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>Start the pending job, call endpoint again</t>
+          <t>Create a PENDING job (created but not started), call endpoint</t>
         </is>
       </c>
       <c r="E305" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved out of PENDING and can still be in PREPARING before it reaches RUNNING)</t>
+          <t>worker_queue_size ≥ 1</t>
         </is>
       </c>
       <c r="F305" s="4" t="n"/>
@@ -9503,17 +9503,17 @@
       </c>
       <c r="C306" s="4" t="inlineStr">
         <is>
-          <t>ECUBE process metrics present</t>
+          <t>Worker queue size decrements</t>
         </is>
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Start the pending job, call endpoint again</t>
         </is>
       </c>
       <c r="E306" s="4" t="inlineStr">
         <is>
-          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
+          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved out of PENDING and can still be in PREPARING before it reaches RUNNING)</t>
         </is>
       </c>
       <c r="F306" s="4" t="n"/>
@@ -9534,17 +9534,17 @@
       </c>
       <c r="C307" s="4" t="inlineStr">
         <is>
-          <t>Active copy-thread correlation</t>
+          <t>ECUBE process metrics present</t>
         </is>
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>Run an export job with active copy workers, call endpoint during the run</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E307" s="4" t="inlineStr">
         <is>
-          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
+          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
         </is>
       </c>
       <c r="F307" s="4" t="n"/>
@@ -9565,17 +9565,17 @@
       </c>
       <c r="C308" s="4" t="inlineStr">
         <is>
-          <t>ECUBE process metrics degrade safely</t>
+          <t>Active copy-thread correlation</t>
         </is>
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
+          <t>Run an export job with active copy workers, call endpoint during the run</t>
         </is>
       </c>
       <c r="E308" s="4" t="inlineStr">
         <is>
-          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
+          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
         </is>
       </c>
       <c r="F308" s="4" t="n"/>
@@ -9596,17 +9596,17 @@
       </c>
       <c r="C309" s="4" t="inlineStr">
         <is>
-          <t>Degraded when DB down</t>
+          <t>ECUBE process metrics degrade safely</t>
         </is>
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, call endpoint with valid token</t>
+          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
         </is>
       </c>
       <c r="E309" s="4" t="inlineStr">
         <is>
-          <t>200, status: "degraded", database: "error", database_error is non-null</t>
+          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
         </is>
       </c>
       <c r="F309" s="4" t="n"/>
@@ -9627,17 +9627,17 @@
       </c>
       <c r="C310" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated rejected</t>
+          <t>Degraded when DB down</t>
         </is>
       </c>
       <c r="D310" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health without token</t>
+          <t>Stop PostgreSQL, call endpoint with valid token</t>
         </is>
       </c>
       <c r="E310" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>200, status: "degraded", database: "error", database_error is non-null</t>
         </is>
       </c>
       <c r="F310" s="4" t="n"/>
@@ -9658,17 +9658,17 @@
       </c>
       <c r="C311" s="4" t="inlineStr">
         <is>
-          <t>Processor role allowed</t>
+          <t>Unauthenticated rejected</t>
         </is>
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with processor token</t>
+          <t>GET /introspection/system-health without token</t>
         </is>
       </c>
       <c r="E311" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F311" s="4" t="n"/>
@@ -9677,59 +9677,59 @@
       <c r="I311" s="4" t="n"/>
     </row>
     <row r="312">
-      <c r="A312" s="2" t="inlineStr">
+      <c r="A312" s="4" t="inlineStr">
+        <is>
+          <t>TC-1516</t>
+        </is>
+      </c>
+      <c r="B312" s="4" t="inlineStr">
+        <is>
+          <t>12.15 System Health</t>
+        </is>
+      </c>
+      <c r="C312" s="4" t="inlineStr">
+        <is>
+          <t>Processor role allowed</t>
+        </is>
+      </c>
+      <c r="D312" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/system-health with processor token</t>
+        </is>
+      </c>
+      <c r="E312" s="4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F312" s="4" t="n"/>
+      <c r="G312" s="4" t="n"/>
+      <c r="H312" s="4" t="n"/>
+      <c r="I312" s="4" t="n"/>
+    </row>
+    <row r="313">
+      <c r="A313" s="2" t="inlineStr">
         <is>
           <t>§12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
-      <c r="B312" s="2" t="inlineStr">
+      <c r="B313" s="2" t="inlineStr">
         <is>
           <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
-      <c r="C312" s="3" t="n"/>
-      <c r="D312" s="3" t="n"/>
-      <c r="E312" s="3" t="n"/>
-      <c r="F312" s="3" t="n"/>
-      <c r="G312" s="3" t="n"/>
-      <c r="H312" s="3" t="n"/>
-      <c r="I312" s="3" t="n"/>
-    </row>
-    <row r="313">
-      <c r="A313" s="4" t="inlineStr">
-        <is>
-          <t>TC-1511</t>
-        </is>
-      </c>
-      <c r="B313" s="4" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C313" s="4" t="inlineStr">
-        <is>
-          <t>Liveness endpoint is public</t>
-        </is>
-      </c>
-      <c r="D313" s="4" t="inlineStr">
-        <is>
-          <t>GET /health/live without token</t>
-        </is>
-      </c>
-      <c r="E313" s="4" t="inlineStr">
-        <is>
-          <t>200, service reports live</t>
-        </is>
-      </c>
-      <c r="F313" s="4" t="n"/>
-      <c r="G313" s="4" t="n"/>
-      <c r="H313" s="4" t="n"/>
-      <c r="I313" s="4" t="n"/>
+      <c r="C313" s="3" t="n"/>
+      <c r="D313" s="3" t="n"/>
+      <c r="E313" s="3" t="n"/>
+      <c r="F313" s="3" t="n"/>
+      <c r="G313" s="3" t="n"/>
+      <c r="H313" s="3" t="n"/>
+      <c r="I313" s="3" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="4" t="inlineStr">
         <is>
-          <t>TC-1512</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B314" s="4" t="inlineStr">
@@ -9739,17 +9739,17 @@
       </c>
       <c r="C314" s="4" t="inlineStr">
         <is>
-          <t>Readiness endpoint is public</t>
+          <t>Liveness endpoint is public</t>
         </is>
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>GET /health/ready without token on a healthy system</t>
+          <t>GET /health/live without token</t>
         </is>
       </c>
       <c r="E314" s="4" t="inlineStr">
         <is>
-          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
+          <t>200, service reports live</t>
         </is>
       </c>
       <c r="F314" s="4" t="n"/>
@@ -9760,7 +9760,7 @@
     <row r="315">
       <c r="A315" s="4" t="inlineStr">
         <is>
-          <t>TC-1513</t>
+          <t>TC-1512</t>
         </is>
       </c>
       <c r="B315" s="4" t="inlineStr">
@@ -9770,17 +9770,17 @@
       </c>
       <c r="C315" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports missing database configuration</t>
+          <t>Readiness endpoint is public</t>
         </is>
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>Clear DB config or test before configuration, then GET /health/ready</t>
+          <t>GET /health/ready without token on a healthy system</t>
         </is>
       </c>
       <c r="E315" s="4" t="inlineStr">
         <is>
-          <t>503, status: "not_ready", reason indicates database is not configured</t>
+          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
         </is>
       </c>
       <c r="F315" s="4" t="n"/>
@@ -9791,7 +9791,7 @@
     <row r="316">
       <c r="A316" s="4" t="inlineStr">
         <is>
-          <t>TC-1514</t>
+          <t>TC-1513</t>
         </is>
       </c>
       <c r="B316" s="4" t="inlineStr">
@@ -9801,17 +9801,17 @@
       </c>
       <c r="C316" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports mount or provider problems</t>
+          <t>Readiness reports missing database configuration</t>
         </is>
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>Break a configured mount or provider, then GET /health/ready</t>
+          <t>Clear DB config or test before configuration, then GET /health/ready</t>
         </is>
       </c>
       <c r="E316" s="4" t="inlineStr">
         <is>
-          <t>503, response identifies the failing check without using the generic error schema</t>
+          <t>503, status: "not_ready", reason indicates database is not configured</t>
         </is>
       </c>
       <c r="F316" s="4" t="n"/>
@@ -9822,7 +9822,7 @@
     <row r="317">
       <c r="A317" s="4" t="inlineStr">
         <is>
-          <t>TC-1515</t>
+          <t>TC-1514</t>
         </is>
       </c>
       <c r="B317" s="4" t="inlineStr">
@@ -9832,17 +9832,17 @@
       </c>
       <c r="C317" s="4" t="inlineStr">
         <is>
-          <t>Version endpoint is public</t>
+          <t>Readiness reports mount or provider problems</t>
         </is>
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/version without token</t>
+          <t>Break a configured mount or provider, then GET /health/ready</t>
         </is>
       </c>
       <c r="E317" s="4" t="inlineStr">
         <is>
-          <t>200, returns version/application metadata</t>
+          <t>503, response identifies the failing check without using the generic error schema</t>
         </is>
       </c>
       <c r="F317" s="4" t="n"/>
@@ -9853,7 +9853,7 @@
     <row r="318">
       <c r="A318" s="4" t="inlineStr">
         <is>
-          <t>TC-1516</t>
+          <t>TC-1515</t>
         </is>
       </c>
       <c r="B318" s="4" t="inlineStr">
@@ -9863,17 +9863,17 @@
       </c>
       <c r="C318" s="4" t="inlineStr">
         <is>
-          <t>Readiness remains separate from authenticated system health</t>
+          <t>Version endpoint is public</t>
         </is>
       </c>
       <c r="D318" s="4" t="inlineStr">
         <is>
-          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+          <t>GET /introspection/version without token</t>
         </is>
       </c>
       <c r="E318" s="4" t="inlineStr">
         <is>
-          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+          <t>200, returns version/application metadata</t>
         </is>
       </c>
       <c r="F318" s="4" t="n"/>
@@ -9882,32 +9882,63 @@
       <c r="I318" s="4" t="n"/>
     </row>
     <row r="319">
-      <c r="A319" s="2" t="inlineStr">
+      <c r="A319" s="4" t="inlineStr">
+        <is>
+          <t>TC-1516</t>
+        </is>
+      </c>
+      <c r="B319" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C319" s="4" t="inlineStr">
+        <is>
+          <t>Readiness remains separate from authenticated system health</t>
+        </is>
+      </c>
+      <c r="D319" s="4" t="inlineStr">
+        <is>
+          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+        </is>
+      </c>
+      <c r="E319" s="4" t="inlineStr">
+        <is>
+          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+        </is>
+      </c>
+      <c r="F319" s="4" t="n"/>
+      <c r="G319" s="4" t="n"/>
+      <c r="H319" s="4" t="n"/>
+      <c r="I319" s="4" t="n"/>
+    </row>
+    <row r="320">
+      <c r="A320" s="2" t="inlineStr">
         <is>
           <t>§12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="B319" s="2" t="inlineStr">
+      <c r="B320" s="2" t="inlineStr">
         <is>
           <t>12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="C319" s="3" t="n"/>
-      <c r="D319" s="3" t="n"/>
-      <c r="E319" s="3" t="n"/>
-      <c r="F319" s="3" t="n"/>
-      <c r="G319" s="3" t="n"/>
-      <c r="H319" s="3" t="n"/>
-      <c r="I319" s="3" t="n"/>
-    </row>
-    <row r="321">
-      <c r="A321" s="5" t="inlineStr">
+      <c r="C320" s="3" t="n"/>
+      <c r="D320" s="3" t="n"/>
+      <c r="E320" s="3" t="n"/>
+      <c r="F320" s="3" t="n"/>
+      <c r="G320" s="3" t="n"/>
+      <c r="H320" s="3" t="n"/>
+      <c r="I320" s="3" t="n"/>
+    </row>
+    <row r="322">
+      <c r="A322" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B321" s="5" t="n">
-        <v>291</v>
+      <c r="B322" s="5" t="n">
+        <v>292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Make managed-account shell enforcement configurable and sync OS-user docs and regressions
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I323"/>
+  <dimension ref="A1:I324"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9944,32 +9944,63 @@
       <c r="I320" s="4" t="n"/>
     </row>
     <row r="321">
-      <c r="A321" s="2" t="inlineStr">
+      <c r="A321" s="4" t="inlineStr">
+        <is>
+          <t>TC-1517</t>
+        </is>
+      </c>
+      <c r="B321" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C321" s="4" t="inlineStr">
+        <is>
+          <t>Metrics endpoint enforces read-only observability roles</t>
+        </is>
+      </c>
+      <c r="D321" s="4" t="inlineStr">
+        <is>
+          <t>GET /metrics without a token, with a processor token, and with an auditor or admin token</t>
+        </is>
+      </c>
+      <c r="E321" s="4" t="inlineStr">
+        <is>
+          <t>Unauthenticated requests return 401, non-observability roles return 403, and admin/auditor receive Prometheus text exposition</t>
+        </is>
+      </c>
+      <c r="F321" s="4" t="n"/>
+      <c r="G321" s="4" t="n"/>
+      <c r="H321" s="4" t="n"/>
+      <c r="I321" s="4" t="n"/>
+    </row>
+    <row r="322">
+      <c r="A322" s="2" t="inlineStr">
         <is>
           <t>§12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="B321" s="2" t="inlineStr">
+      <c r="B322" s="2" t="inlineStr">
         <is>
           <t>12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="C321" s="3" t="n"/>
-      <c r="D321" s="3" t="n"/>
-      <c r="E321" s="3" t="n"/>
-      <c r="F321" s="3" t="n"/>
-      <c r="G321" s="3" t="n"/>
-      <c r="H321" s="3" t="n"/>
-      <c r="I321" s="3" t="n"/>
-    </row>
-    <row r="323">
-      <c r="A323" s="5" t="inlineStr">
+      <c r="C322" s="3" t="n"/>
+      <c r="D322" s="3" t="n"/>
+      <c r="E322" s="3" t="n"/>
+      <c r="F322" s="3" t="n"/>
+      <c r="G322" s="3" t="n"/>
+      <c r="H322" s="3" t="n"/>
+      <c r="I322" s="3" t="n"/>
+    </row>
+    <row r="324">
+      <c r="A324" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B323" s="5" t="n">
-        <v>293</v>
+      <c r="B324" s="5" t="n">
+        <v>294</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add real Docker auth-prep validation and document container PAM/password-policy behavior
</commit_message>
<xml_diff>
--- a/docs/testing/ecube-qa-test-cases.xlsx
+++ b/docs/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I324"/>
+  <dimension ref="A1:I326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8225,48 +8225,60 @@
       <c r="I263" s="4" t="n"/>
     </row>
     <row r="264">
-      <c r="A264" s="2" t="inlineStr">
-        <is>
-          <t>§12.12 Chain-of-Custody Handoff</t>
-        </is>
-      </c>
-      <c r="B264" s="2" t="inlineStr">
-        <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
-        </is>
-      </c>
-      <c r="C264" s="3" t="n"/>
-      <c r="D264" s="3" t="n"/>
-      <c r="E264" s="3" t="n"/>
-      <c r="F264" s="3" t="n"/>
-      <c r="G264" s="3" t="n"/>
-      <c r="H264" s="3" t="n"/>
-      <c r="I264" s="3" t="n"/>
+      <c r="A264" s="4" t="inlineStr">
+        <is>
+          <t>TC-1117</t>
+        </is>
+      </c>
+      <c r="B264" s="4" t="inlineStr">
+        <is>
+          <t>12.11 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C264" s="4" t="inlineStr">
+        <is>
+          <t>Docker Compose setup uses container PAM policy</t>
+        </is>
+      </c>
+      <c r="D264" s="4" t="inlineStr">
+        <is>
+          <t>Start docker compose -f docker-compose.ecube.yml up -d --build, open /setup, create a local admin password that satisfies the configured policy, and confirm the setup succeeds</t>
+        </is>
+      </c>
+      <c r="E264" s="4" t="inlineStr">
+        <is>
+          <t>Setup completes successfully, and docker compose exec ecube-app grep -F 'password	requisite	pam_pwquality.so local_users_only' /etc/pam.d/common-password shows the container-enforced password-quality stack</t>
+        </is>
+      </c>
+      <c r="F264" s="4" t="n"/>
+      <c r="G264" s="4" t="n"/>
+      <c r="H264" s="4" t="n"/>
+      <c r="I264" s="4" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="4" t="inlineStr">
         <is>
-          <t>TC-1201</t>
+          <t>TC-1118</t>
         </is>
       </c>
       <c r="B265" s="4" t="inlineStr">
         <is>
-          <t>12.12 Chain-of-Custody Handoff</t>
+          <t>12.11 First-Run Setup</t>
         </is>
       </c>
       <c r="C265" s="4" t="inlineStr">
         <is>
-          <t>Retrieve stored CoC snapshot — archived job</t>
+          <t>Docker Compose local password reset follows container policy</t>
         </is>
       </c>
       <c r="D265" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for an archived job that already has a stored snapshot</t>
+          <t>In a Compose deployment with demo mode or a local managed account enabled, trigger a password reset or demo-account reconciliation, then inspect docker compose logs ecube-app</t>
         </is>
       </c>
       <c r="E265" s="4" t="inlineStr">
         <is>
-          <t>200, response contains the stored snapshot and snapshot metadata</t>
+          <t>The password operation succeeds without Cracklib dictionary-load errors, and logs do not show repeated pam_chauthtok() password-policy failures for policy-compliant values</t>
         </is>
       </c>
       <c r="F265" s="4" t="n"/>
@@ -8275,40 +8287,28 @@
       <c r="I265" s="4" t="n"/>
     </row>
     <row r="266">
-      <c r="A266" s="4" t="inlineStr">
-        <is>
-          <t>TC-1202</t>
-        </is>
-      </c>
-      <c r="B266" s="4" t="inlineStr">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>§12.12 Chain-of-Custody Handoff</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
         <is>
           <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
-      <c r="C266" s="4" t="inlineStr">
-        <is>
-          <t>Retrieve stored CoC snapshot — active job</t>
-        </is>
-      </c>
-      <c r="D266" s="4" t="inlineStr">
-        <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job that already has a stored snapshot</t>
-        </is>
-      </c>
-      <c r="E266" s="4" t="inlineStr">
-        <is>
-          <t>200, response contains the stored snapshot and does not regenerate it</t>
-        </is>
-      </c>
-      <c r="F266" s="4" t="n"/>
-      <c r="G266" s="4" t="n"/>
-      <c r="H266" s="4" t="n"/>
-      <c r="I266" s="4" t="n"/>
+      <c r="C266" s="3" t="n"/>
+      <c r="D266" s="3" t="n"/>
+      <c r="E266" s="3" t="n"/>
+      <c r="F266" s="3" t="n"/>
+      <c r="G266" s="3" t="n"/>
+      <c r="H266" s="3" t="n"/>
+      <c r="I266" s="3" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="4" t="inlineStr">
         <is>
-          <t>TC-1203</t>
+          <t>TC-1201</t>
         </is>
       </c>
       <c r="B267" s="4" t="inlineStr">
@@ -8318,17 +8318,17 @@
       </c>
       <c r="C267" s="4" t="inlineStr">
         <is>
-          <t>CoC read — missing stored snapshot</t>
+          <t>Retrieve stored CoC snapshot — archived job</t>
         </is>
       </c>
       <c r="D267" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job with no stored snapshot yet</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for an archived job that already has a stored snapshot</t>
         </is>
       </c>
       <c r="E267" s="4" t="inlineStr">
         <is>
-          <t>404, message explains that the report must be refreshed first</t>
+          <t>200, response contains the stored snapshot and snapshot metadata</t>
         </is>
       </c>
       <c r="F267" s="4" t="n"/>
@@ -8339,7 +8339,7 @@
     <row r="268">
       <c r="A268" s="4" t="inlineStr">
         <is>
-          <t>TC-1204</t>
+          <t>TC-1202</t>
         </is>
       </c>
       <c r="B268" s="4" t="inlineStr">
@@ -8349,17 +8349,17 @@
       </c>
       <c r="C268" s="4" t="inlineStr">
         <is>
-          <t>CoC read — processor allowed</t>
+          <t>Retrieve stored CoC snapshot — active job</t>
         </is>
       </c>
       <c r="D268" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody with processor token</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job that already has a stored snapshot</t>
         </is>
       </c>
       <c r="E268" s="4" t="inlineStr">
         <is>
-          <t>200 when a stored snapshot exists; otherwise 404 with refresh guidance</t>
+          <t>200, response contains the stored snapshot and does not regenerate it</t>
         </is>
       </c>
       <c r="F268" s="4" t="n"/>
@@ -8370,7 +8370,7 @@
     <row r="269">
       <c r="A269" s="4" t="inlineStr">
         <is>
-          <t>TC-1205</t>
+          <t>TC-1203</t>
         </is>
       </c>
       <c r="B269" s="4" t="inlineStr">
@@ -8380,17 +8380,17 @@
       </c>
       <c r="C269" s="4" t="inlineStr">
         <is>
-          <t>CoC read — unauthenticated denied</t>
+          <t>CoC read — missing stored snapshot</t>
         </is>
       </c>
       <c r="D269" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/{job_id}/chain-of-custody without token</t>
+          <t>GET /jobs/{job_id}/chain-of-custody for a non-archived job with no stored snapshot yet</t>
         </is>
       </c>
       <c r="E269" s="4" t="inlineStr">
         <is>
-          <t>401, UNAUTHORIZED</t>
+          <t>404, message explains that the report must be refreshed first</t>
         </is>
       </c>
       <c r="F269" s="4" t="n"/>
@@ -8401,7 +8401,7 @@
     <row r="270">
       <c r="A270" s="4" t="inlineStr">
         <is>
-          <t>TC-1206</t>
+          <t>TC-1204</t>
         </is>
       </c>
       <c r="B270" s="4" t="inlineStr">
@@ -8411,17 +8411,17 @@
       </c>
       <c r="C270" s="4" t="inlineStr">
         <is>
-          <t>CoC snapshot fields</t>
+          <t>CoC read — processor allowed</t>
         </is>
       </c>
       <c r="D270" s="4" t="inlineStr">
         <is>
-          <t>Inspect any stored-snapshot response</t>
+          <t>GET /jobs/{job_id}/chain-of-custody with processor token</t>
         </is>
       </c>
       <c r="E270" s="4" t="inlineStr">
         <is>
-          <t>snapshot_stored_at, snapshot_updated_at, snapshot_stored_by, reports[], and manifest/custody fields are present; drive_sn shows the parsed hardware serial when available and is blank when unavailable</t>
+          <t>200 when a stored snapshot exists; otherwise 404 with refresh guidance</t>
         </is>
       </c>
       <c r="F270" s="4" t="n"/>
@@ -8432,7 +8432,7 @@
     <row r="271">
       <c r="A271" s="4" t="inlineStr">
         <is>
-          <t>TC-1207</t>
+          <t>TC-1205</t>
         </is>
       </c>
       <c r="B271" s="4" t="inlineStr">
@@ -8442,17 +8442,17 @@
       </c>
       <c r="C271" s="4" t="inlineStr">
         <is>
-          <t>CoC events include lifecycle</t>
+          <t>CoC read — unauthenticated denied</t>
         </is>
       </c>
       <c r="D271" s="4" t="inlineStr">
         <is>
-          <t>Inspect chain_of_custody_events in a stored report for a completed job</t>
+          <t>GET /jobs/{job_id}/chain-of-custody without token</t>
         </is>
       </c>
       <c r="E271" s="4" t="inlineStr">
         <is>
-          <t>Events include DRIVE_INITIALIZED, JOB_CREATED, JOB_STARTED, JOB_COMPLETED, DRIVE_EJECT_PREPARED, and COC_HANDOFF_CONFIRMED when applicable</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F271" s="4" t="n"/>
@@ -8463,7 +8463,7 @@
     <row r="272">
       <c r="A272" s="4" t="inlineStr">
         <is>
-          <t>TC-1208</t>
+          <t>TC-1206</t>
         </is>
       </c>
       <c r="B272" s="4" t="inlineStr">
@@ -8473,17 +8473,17 @@
       </c>
       <c r="C272" s="4" t="inlineStr">
         <is>
-          <t>CoC manifest summary</t>
+          <t>CoC snapshot fields</t>
         </is>
       </c>
       <c r="D272" s="4" t="inlineStr">
         <is>
-          <t>Inspect manifest_summary in the stored report</t>
+          <t>Inspect any stored-snapshot response</t>
         </is>
       </c>
       <c r="E272" s="4" t="inlineStr">
         <is>
-          <t>Array of objects with job_id, evidence_number, processor_notes, total_files, total_bytes, and manifest_count</t>
+          <t>snapshot_stored_at, snapshot_updated_at, snapshot_stored_by, reports[], and manifest/custody fields are present; drive_sn shows the parsed hardware serial when available and is blank when unavailable</t>
         </is>
       </c>
       <c r="F272" s="4" t="n"/>
@@ -8494,7 +8494,7 @@
     <row r="273">
       <c r="A273" s="4" t="inlineStr">
         <is>
-          <t>TC-1209</t>
+          <t>TC-1207</t>
         </is>
       </c>
       <c r="B273" s="4" t="inlineStr">
@@ -8504,17 +8504,17 @@
       </c>
       <c r="C273" s="4" t="inlineStr">
         <is>
-          <t>CoC — delivery_time absence (no handoff)</t>
+          <t>CoC events include lifecycle</t>
         </is>
       </c>
       <c r="D273" s="4" t="inlineStr">
         <is>
-          <t>Complete a job and store a snapshot before handoff</t>
+          <t>Inspect chain_of_custody_events in a stored report for a completed job</t>
         </is>
       </c>
       <c r="E273" s="4" t="inlineStr">
         <is>
-          <t>chain_of_custody_events do not contain COC_HANDOFF_CONFIRMED; custody_complete is false</t>
+          <t>Events include DRIVE_INITIALIZED, JOB_CREATED, JOB_STARTED, JOB_COMPLETED, DRIVE_EJECT_PREPARED, and COC_HANDOFF_CONFIRMED when applicable</t>
         </is>
       </c>
       <c r="F273" s="4" t="n"/>
@@ -8525,7 +8525,7 @@
     <row r="274">
       <c r="A274" s="4" t="inlineStr">
         <is>
-          <t>TC-1210</t>
+          <t>TC-1208</t>
         </is>
       </c>
       <c r="B274" s="4" t="inlineStr">
@@ -8535,17 +8535,17 @@
       </c>
       <c r="C274" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — valid</t>
+          <t>CoC manifest summary</t>
         </is>
       </c>
       <c r="D274" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh with admin or manager token for a non-archived job with assignments</t>
+          <t>Inspect manifest_summary in the stored report</t>
         </is>
       </c>
       <c r="E274" s="4" t="inlineStr">
         <is>
-          <t>200, response contains the refreshed stored snapshot and updated snapshot metadata</t>
+          <t>Array of objects with job_id, evidence_number, processor_notes, total_files, total_bytes, and manifest_count</t>
         </is>
       </c>
       <c r="F274" s="4" t="n"/>
@@ -8556,7 +8556,7 @@
     <row r="275">
       <c r="A275" s="4" t="inlineStr">
         <is>
-          <t>TC-1211</t>
+          <t>TC-1209</t>
         </is>
       </c>
       <c r="B275" s="4" t="inlineStr">
@@ -8566,17 +8566,17 @@
       </c>
       <c r="C275" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — auditor denied</t>
+          <t>CoC — delivery_time absence (no handoff)</t>
         </is>
       </c>
       <c r="D275" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh with auditor token</t>
+          <t>Complete a job and store a snapshot before handoff</t>
         </is>
       </c>
       <c r="E275" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>chain_of_custody_events do not contain COC_HANDOFF_CONFIRMED; custody_complete is false</t>
         </is>
       </c>
       <c r="F275" s="4" t="n"/>
@@ -8587,7 +8587,7 @@
     <row r="276">
       <c r="A276" s="4" t="inlineStr">
         <is>
-          <t>TC-1212</t>
+          <t>TC-1210</t>
         </is>
       </c>
       <c r="B276" s="4" t="inlineStr">
@@ -8597,17 +8597,17 @@
       </c>
       <c r="C276" s="4" t="inlineStr">
         <is>
-          <t>CoC refresh — archived job denied</t>
+          <t>CoC refresh — valid</t>
         </is>
       </c>
       <c r="D276" s="4" t="inlineStr">
         <is>
-          <t>POST /jobs/{job_id}/chain-of-custody/refresh for an archived job</t>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh with admin or manager token for a non-archived job with assignments</t>
         </is>
       </c>
       <c r="E276" s="4" t="inlineStr">
         <is>
-          <t>409, archived jobs can only return the last stored snapshot</t>
+          <t>200, response contains the refreshed stored snapshot and updated snapshot metadata</t>
         </is>
       </c>
       <c r="F276" s="4" t="n"/>
@@ -8616,48 +8616,60 @@
       <c r="I276" s="4" t="n"/>
     </row>
     <row r="277">
-      <c r="A277" s="2" t="inlineStr">
-        <is>
-          <t>§12.14 Startup Reconciliation</t>
-        </is>
-      </c>
-      <c r="B277" s="2" t="inlineStr">
-        <is>
-          <t>12.14 Startup Reconciliation</t>
-        </is>
-      </c>
-      <c r="C277" s="3" t="n"/>
-      <c r="D277" s="3" t="n"/>
-      <c r="E277" s="3" t="n"/>
-      <c r="F277" s="3" t="n"/>
-      <c r="G277" s="3" t="n"/>
-      <c r="H277" s="3" t="n"/>
-      <c r="I277" s="3" t="n"/>
+      <c r="A277" s="4" t="inlineStr">
+        <is>
+          <t>TC-1211</t>
+        </is>
+      </c>
+      <c r="B277" s="4" t="inlineStr">
+        <is>
+          <t>12.12 Chain-of-Custody Handoff</t>
+        </is>
+      </c>
+      <c r="C277" s="4" t="inlineStr">
+        <is>
+          <t>CoC refresh — auditor denied</t>
+        </is>
+      </c>
+      <c r="D277" s="4" t="inlineStr">
+        <is>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh with auditor token</t>
+        </is>
+      </c>
+      <c r="E277" s="4" t="inlineStr">
+        <is>
+          <t>403, FORBIDDEN</t>
+        </is>
+      </c>
+      <c r="F277" s="4" t="n"/>
+      <c r="G277" s="4" t="n"/>
+      <c r="H277" s="4" t="n"/>
+      <c r="I277" s="4" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="4" t="inlineStr">
         <is>
-          <t>TC-1401</t>
+          <t>TC-1212</t>
         </is>
       </c>
       <c r="B278" s="4" t="inlineStr">
         <is>
-          <t>12.14 Startup Reconciliation</t>
+          <t>12.12 Chain-of-Custody Handoff</t>
         </is>
       </c>
       <c r="C278" s="4" t="inlineStr">
         <is>
-          <t>Running job failed after restart</t>
+          <t>CoC refresh — archived job denied</t>
         </is>
       </c>
       <c r="D278" s="4" t="inlineStr">
         <is>
-          <t>Create a job, start it, restart the service while RUNNING</t>
+          <t>POST /jobs/{job_id}/chain-of-custody/refresh for an archived job</t>
         </is>
       </c>
       <c r="E278" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
+          <t>409, archived jobs can only return the last stored snapshot</t>
         </is>
       </c>
       <c r="F278" s="4" t="n"/>
@@ -8666,40 +8678,28 @@
       <c r="I278" s="4" t="n"/>
     </row>
     <row r="279">
-      <c r="A279" s="4" t="inlineStr">
-        <is>
-          <t>TC-1402</t>
-        </is>
-      </c>
-      <c r="B279" s="4" t="inlineStr">
+      <c r="A279" s="2" t="inlineStr">
+        <is>
+          <t>§12.14 Startup Reconciliation</t>
+        </is>
+      </c>
+      <c r="B279" s="2" t="inlineStr">
         <is>
           <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
-      <c r="C279" s="4" t="inlineStr">
-        <is>
-          <t>Verifying job failed after restart</t>
-        </is>
-      </c>
-      <c r="D279" s="4" t="inlineStr">
-        <is>
-          <t>Start a job, let it reach VERIFYING, restart the service</t>
-        </is>
-      </c>
-      <c r="E279" s="4" t="inlineStr">
-        <is>
-          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
-        </is>
-      </c>
-      <c r="F279" s="4" t="n"/>
-      <c r="G279" s="4" t="n"/>
-      <c r="H279" s="4" t="n"/>
-      <c r="I279" s="4" t="n"/>
+      <c r="C279" s="3" t="n"/>
+      <c r="D279" s="3" t="n"/>
+      <c r="E279" s="3" t="n"/>
+      <c r="F279" s="3" t="n"/>
+      <c r="G279" s="3" t="n"/>
+      <c r="H279" s="3" t="n"/>
+      <c r="I279" s="3" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="4" t="inlineStr">
         <is>
-          <t>TC-1403</t>
+          <t>TC-1401</t>
         </is>
       </c>
       <c r="B280" s="4" t="inlineStr">
@@ -8709,17 +8709,17 @@
       </c>
       <c r="C280" s="4" t="inlineStr">
         <is>
-          <t>Pending job not affected</t>
+          <t>Running job failed after restart</t>
         </is>
       </c>
       <c r="D280" s="4" t="inlineStr">
         <is>
-          <t>Create a job (PENDING), restart the service</t>
+          <t>Create a job, start it, restart the service while RUNNING</t>
         </is>
       </c>
       <c r="E280" s="4" t="inlineStr">
         <is>
-          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
+          <t>Job status is FAILED, completed_at is set, audit log contains JOB_RECONCILED with reason: "interrupted by restart"</t>
         </is>
       </c>
       <c r="F280" s="4" t="n"/>
@@ -8730,7 +8730,7 @@
     <row r="281">
       <c r="A281" s="4" t="inlineStr">
         <is>
-          <t>TC-1404</t>
+          <t>TC-1402</t>
         </is>
       </c>
       <c r="B281" s="4" t="inlineStr">
@@ -8740,17 +8740,17 @@
       </c>
       <c r="C281" s="4" t="inlineStr">
         <is>
-          <t>Completed job not affected</t>
+          <t>Verifying job failed after restart</t>
         </is>
       </c>
       <c r="D281" s="4" t="inlineStr">
         <is>
-          <t>Complete a job, restart the service</t>
+          <t>Start a job, let it reach VERIFYING, restart the service</t>
         </is>
       </c>
       <c r="E281" s="4" t="inlineStr">
         <is>
-          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
+          <t>Job status is FAILED, audit log contains JOB_RECONCILED with old_status: "VERIFYING"</t>
         </is>
       </c>
       <c r="F281" s="4" t="n"/>
@@ -8761,7 +8761,7 @@
     <row r="282">
       <c r="A282" s="4" t="inlineStr">
         <is>
-          <t>TC-1405</t>
+          <t>TC-1403</t>
         </is>
       </c>
       <c r="B282" s="4" t="inlineStr">
@@ -8771,17 +8771,17 @@
       </c>
       <c r="C282" s="4" t="inlineStr">
         <is>
-          <t>Stale mount corrected</t>
+          <t>Pending job not affected</t>
         </is>
       </c>
       <c r="D282" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
+          <t>Create a job (PENDING), restart the service</t>
         </is>
       </c>
       <c r="E282" s="4" t="inlineStr">
         <is>
-          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
+          <t>Job remains PENDING, no JOB_RECONCILED audit entry for this job</t>
         </is>
       </c>
       <c r="F282" s="4" t="n"/>
@@ -8792,7 +8792,7 @@
     <row r="283">
       <c r="A283" s="4" t="inlineStr">
         <is>
-          <t>TC-1406</t>
+          <t>TC-1404</t>
         </is>
       </c>
       <c r="B283" s="4" t="inlineStr">
@@ -8802,17 +8802,17 @@
       </c>
       <c r="C283" s="4" t="inlineStr">
         <is>
-          <t>Active mount preserved</t>
+          <t>Completed job not affected</t>
         </is>
       </c>
       <c r="D283" s="4" t="inlineStr">
         <is>
-          <t>Add and mount a network share (leave it mounted), restart the service</t>
+          <t>Complete a job, restart the service</t>
         </is>
       </c>
       <c r="E283" s="4" t="inlineStr">
         <is>
-          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
+          <t>Job remains COMPLETED, no JOB_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F283" s="4" t="n"/>
@@ -8823,7 +8823,7 @@
     <row r="284">
       <c r="A284" s="4" t="inlineStr">
         <is>
-          <t>TC-1407</t>
+          <t>TC-1405</t>
         </is>
       </c>
       <c r="B284" s="4" t="inlineStr">
@@ -8833,17 +8833,17 @@
       </c>
       <c r="C284" s="4" t="inlineStr">
         <is>
-          <t>USB drives re-discovered</t>
+          <t>Stale mount corrected</t>
         </is>
       </c>
       <c r="D284" s="4" t="inlineStr">
         <is>
-          <t>Insert USB drives, restart the service</t>
+          <t>Add and mount a network share, unmount it at OS level (sudo umount), restart the service</t>
         </is>
       </c>
       <c r="E284" s="4" t="inlineStr">
         <is>
-          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
+          <t>Mount status is UNMOUNTED, audit log contains MOUNT_RECONCILED</t>
         </is>
       </c>
       <c r="F284" s="4" t="n"/>
@@ -8854,7 +8854,7 @@
     <row r="285">
       <c r="A285" s="4" t="inlineStr">
         <is>
-          <t>TC-1408</t>
+          <t>TC-1406</t>
         </is>
       </c>
       <c r="B285" s="4" t="inlineStr">
@@ -8864,17 +8864,17 @@
       </c>
       <c r="C285" s="4" t="inlineStr">
         <is>
-          <t>Idempotency</t>
+          <t>Active mount preserved</t>
         </is>
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t>Restart the service twice without any state changes between restarts</t>
+          <t>Add and mount a network share (leave it mounted), restart the service</t>
         </is>
       </c>
       <c r="E285" s="4" t="inlineStr">
         <is>
-          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
+          <t>Mount status remains MOUNTED, no MOUNT_RECONCILED audit entry</t>
         </is>
       </c>
       <c r="F285" s="4" t="n"/>
@@ -8885,7 +8885,7 @@
     <row r="286">
       <c r="A286" s="4" t="inlineStr">
         <is>
-          <t>TC-1409</t>
+          <t>TC-1407</t>
         </is>
       </c>
       <c r="B286" s="4" t="inlineStr">
@@ -8895,17 +8895,17 @@
       </c>
       <c r="C286" s="4" t="inlineStr">
         <is>
-          <t>Partial failure isolation</t>
+          <t>USB drives re-discovered</t>
         </is>
       </c>
       <c r="D286" s="4" t="inlineStr">
         <is>
-          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
+          <t>Insert USB drives, restart the service</t>
         </is>
       </c>
       <c r="E286" s="4" t="inlineStr">
         <is>
-          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
+          <t>Drives re-appear with correct state (AVAILABLE on enabled ports), USB_DISCOVERY_SYNC audit entry present</t>
         </is>
       </c>
       <c r="F286" s="4" t="n"/>
@@ -8916,7 +8916,7 @@
     <row r="287">
       <c r="A287" s="4" t="inlineStr">
         <is>
-          <t>TC-1410</t>
+          <t>TC-1408</t>
         </is>
       </c>
       <c r="B287" s="4" t="inlineStr">
@@ -8926,17 +8926,17 @@
       </c>
       <c r="C287" s="4" t="inlineStr">
         <is>
-          <t>Cross-process lock — only one worker reconciles</t>
+          <t>Idempotency</t>
         </is>
       </c>
       <c r="D287" s="4" t="inlineStr">
         <is>
-          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
+          <t>Restart the service twice without any state changes between restarts</t>
         </is>
       </c>
       <c r="E287" s="4" t="inlineStr">
         <is>
-          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
+          <t>Second restart produces no additional MOUNT_RECONCILED or JOB_RECONCILED audit entries</t>
         </is>
       </c>
       <c r="F287" s="4" t="n"/>
@@ -8947,7 +8947,7 @@
     <row r="288">
       <c r="A288" s="4" t="inlineStr">
         <is>
-          <t>TC-1411</t>
+          <t>TC-1409</t>
         </is>
       </c>
       <c r="B288" s="4" t="inlineStr">
@@ -8957,17 +8957,17 @@
       </c>
       <c r="C288" s="4" t="inlineStr">
         <is>
-          <t>Stale lock reclaim</t>
+          <t>Partial failure isolation</t>
         </is>
       </c>
       <c r="D288" s="4" t="inlineStr">
         <is>
-          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
+          <t>Disconnect the NFS server (to cause mount check failure), have a RUNNING job, restart the service</t>
         </is>
       </c>
       <c r="E288" s="4" t="inlineStr">
         <is>
-          <t>Service reclaims the stale lock, reconciliation runs normally</t>
+          <t>Job is still reconciled to FAILED even though mount reconciliation may error; check logs for error message</t>
         </is>
       </c>
       <c r="F288" s="4" t="n"/>
@@ -8978,7 +8978,7 @@
     <row r="289">
       <c r="A289" s="4" t="inlineStr">
         <is>
-          <t>TC-1412</t>
+          <t>TC-1410</t>
         </is>
       </c>
       <c r="B289" s="4" t="inlineStr">
@@ -8988,17 +8988,17 @@
       </c>
       <c r="C289" s="4" t="inlineStr">
         <is>
-          <t>Lock released after failure</t>
+          <t>Cross-process lock — only one worker reconciles</t>
         </is>
       </c>
       <c r="D289" s="4" t="inlineStr">
         <is>
-          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
+          <t>Start Uvicorn with --workers 4, have a RUNNING job and a MOUNTED (but stale) mount</t>
         </is>
       </c>
       <c r="E289" s="4" t="inlineStr">
         <is>
-          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
+          <t>Exactly one JOB_RECONCILED and one MOUNT_RECONCILED audit entry; remaining workers log "skipping reconciliation" at INFO level</t>
         </is>
       </c>
       <c r="F289" s="4" t="n"/>
@@ -9009,7 +9009,7 @@
     <row r="290">
       <c r="A290" s="4" t="inlineStr">
         <is>
-          <t>TC-1413</t>
+          <t>TC-1411</t>
         </is>
       </c>
       <c r="B290" s="4" t="inlineStr">
@@ -9019,17 +9019,17 @@
       </c>
       <c r="C290" s="4" t="inlineStr">
         <is>
-          <t>Jobs pass emits immediate startup result log</t>
+          <t>Stale lock reclaim</t>
         </is>
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>Create at least one RUNNING job, restart service, then inspect application logs around startup reconciliation</t>
+          <t>Insert a stale lock row (locked_at &gt; 5 minutes ago) via SQL, restart the service</t>
         </is>
       </c>
       <c r="E290" s="4" t="inlineStr">
         <is>
-          <t>Logs include Startup reconciliation: checking jobs followed by an immediate Startup reconciliation: jobs result line with safe counts (jobs_checked, jobs_corrected) or safe failure classification</t>
+          <t>Service reclaims the stale lock, reconciliation runs normally</t>
         </is>
       </c>
       <c r="F290" s="4" t="n"/>
@@ -9040,7 +9040,7 @@
     <row r="291">
       <c r="A291" s="4" t="inlineStr">
         <is>
-          <t>TC-1414</t>
+          <t>TC-1412</t>
         </is>
       </c>
       <c r="B291" s="4" t="inlineStr">
@@ -9050,17 +9050,17 @@
       </c>
       <c r="C291" s="4" t="inlineStr">
         <is>
-          <t>Reconciled job persists restart-interruption failure reason</t>
+          <t>Lock released after failure</t>
         </is>
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>Create a RUNNING or VERIFYING job, restart service, then open Job Detail for that job</t>
+          <t>Disconnect NFS, restart the service, reconnect NFS, restart again</t>
         </is>
       </c>
       <c r="E291" s="4" t="inlineStr">
         <is>
-          <t>Job status is FAILED and Job Detail shows a stable restart interruption reason (not the generic This job failed... fallback)</t>
+          <t>Second restart acquires lock and runs reconciliation; lock table is empty after startup completes</t>
         </is>
       </c>
       <c r="F291" s="4" t="n"/>
@@ -9071,7 +9071,7 @@
     <row r="292">
       <c r="A292" s="4" t="inlineStr">
         <is>
-          <t>TC-1415</t>
+          <t>TC-1413</t>
         </is>
       </c>
       <c r="B292" s="4" t="inlineStr">
@@ -9081,17 +9081,17 @@
       </c>
       <c r="C292" s="4" t="inlineStr">
         <is>
-          <t>Reconciled failed job shows correlated failure entry from audit fallback</t>
+          <t>Jobs pass emits immediate startup result log</t>
         </is>
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>Restart with a RUNNING job, then inspect Job Detail when no matching file-log failure line is present</t>
+          <t>Create at least one RUNNING job, restart service, then inspect application logs around startup reconciliation</t>
         </is>
       </c>
       <c r="E292" s="4" t="inlineStr">
         <is>
-          <t>Job Detail still shows a related failure entry sourced from reconciliation evidence (JOB_RECONCILED) and the entry remains sanitized</t>
+          <t>Logs include Startup reconciliation: checking jobs followed by an immediate Startup reconciliation: jobs result line with safe counts (jobs_checked, jobs_corrected) or safe failure classification</t>
         </is>
       </c>
       <c r="F292" s="4" t="n"/>
@@ -9102,7 +9102,7 @@
     <row r="293">
       <c r="A293" s="4" t="inlineStr">
         <is>
-          <t>TC-1416</t>
+          <t>TC-1414</t>
         </is>
       </c>
       <c r="B293" s="4" t="inlineStr">
@@ -9112,17 +9112,17 @@
       </c>
       <c r="C293" s="4" t="inlineStr">
         <is>
-          <t>Failed job API uses reconciliation audit fallback when file-log correlation is unavailable</t>
+          <t>Reconciled job persists restart-interruption failure reason</t>
         </is>
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>In a test environment, disable file-log correlation (log_file unset), then request GET /jobs/{job_id} for a restart-reconciled failed job</t>
+          <t>Create a RUNNING or VERIFYING job, restart service, then open Job Detail for that job</t>
         </is>
       </c>
       <c r="E293" s="4" t="inlineStr">
         <is>
-          <t>Response remains 200 and includes the stable restart failure reason plus a sanitized failure_log_entry derived from audit evidence (JOB_RECONCILED)</t>
+          <t>Job status is FAILED and Job Detail shows a stable restart interruption reason (not the generic This job failed... fallback)</t>
         </is>
       </c>
       <c r="F293" s="4" t="n"/>
@@ -9133,7 +9133,7 @@
     <row r="294">
       <c r="A294" s="4" t="inlineStr">
         <is>
-          <t>TC-1417</t>
+          <t>TC-1415</t>
         </is>
       </c>
       <c r="B294" s="4" t="inlineStr">
@@ -9143,17 +9143,17 @@
       </c>
       <c r="C294" s="4" t="inlineStr">
         <is>
-          <t>Jobs pass failure path emits safe startup result classification</t>
+          <t>Reconciled failed job shows correlated failure entry from audit fallback</t>
         </is>
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>In a controlled test environment, force a jobs-pass reconciliation exception, then restart service and inspect startup logs</t>
+          <t>Restart with a RUNNING job, then inspect Job Detail when no matching file-log failure line is present</t>
         </is>
       </c>
       <c r="E294" s="4" t="inlineStr">
         <is>
-          <t>Logs still include Startup reconciliation: jobs result with status=failed and reason=job_reconciliation_failed, without raw provider errors or host paths</t>
+          <t>Job Detail still shows a related failure entry sourced from reconciliation evidence (JOB_RECONCILED) and the entry remains sanitized</t>
         </is>
       </c>
       <c r="F294" s="4" t="n"/>
@@ -9164,7 +9164,7 @@
     <row r="295">
       <c r="A295" s="4" t="inlineStr">
         <is>
-          <t>TC-1418</t>
+          <t>TC-1416</t>
         </is>
       </c>
       <c r="B295" s="4" t="inlineStr">
@@ -9174,17 +9174,17 @@
       </c>
       <c r="C295" s="4" t="inlineStr">
         <is>
-          <t>Restart clears stale in-progress startup analysis when no valid cache remains</t>
+          <t>Failed job API uses reconciliation audit fallback when file-log correlation is unavailable</t>
         </is>
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>Trigger manual Analyze for a PENDING job, restart ECUBE before the scan completes, then reopen Job Detail</t>
+          <t>In a test environment, disable file-log correlation (log_file unset), then request GET /jobs/{job_id} for a restart-reconciled failed job</t>
         </is>
       </c>
       <c r="E295" s="4" t="inlineStr">
         <is>
-          <t>Job does not remain stuck in ANALYZING, startup-analysis state returns to NOT_ANALYZED, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "analysis_interrupted_by_restart", and Analyze or Start is available again</t>
+          <t>Response remains 200 and includes the stable restart failure reason plus a sanitized failure_log_entry derived from audit evidence (JOB_RECONCILED)</t>
         </is>
       </c>
       <c r="F295" s="4" t="n"/>
@@ -9195,7 +9195,7 @@
     <row r="296">
       <c r="A296" s="4" t="inlineStr">
         <is>
-          <t>TC-1419</t>
+          <t>TC-1417</t>
         </is>
       </c>
       <c r="B296" s="4" t="inlineStr">
@@ -9205,17 +9205,17 @@
       </c>
       <c r="C296" s="4" t="inlineStr">
         <is>
-          <t>Restart restores READY when the interrupted startup-analysis cache is still current</t>
+          <t>Jobs pass failure path emits safe startup result classification</t>
         </is>
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t>Trigger manual Analyze for a job with a stable source tree, restart ECUBE after the reusable snapshot has been persisted but before the manual analyze workflow fully completes, then reopen Job Detail</t>
+          <t>In a controlled test environment, force a jobs-pass reconciliation exception, then restart service and inspect startup logs</t>
         </is>
       </c>
       <c r="E296" s="4" t="inlineStr">
         <is>
-          <t>Job shows startup_analysis_status: READY, the previous file and byte totals are still available, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "valid_cache_restored_after_restart", and Start can proceed without forcing a fresh scan</t>
+          <t>Logs still include Startup reconciliation: jobs result with status=failed and reason=job_reconciliation_failed, without raw provider errors or host paths</t>
         </is>
       </c>
       <c r="F296" s="4" t="n"/>
@@ -9224,48 +9224,60 @@
       <c r="I296" s="4" t="n"/>
     </row>
     <row r="297">
-      <c r="A297" s="2" t="inlineStr">
-        <is>
-          <t>§12.15 System Health</t>
-        </is>
-      </c>
-      <c r="B297" s="2" t="inlineStr">
-        <is>
-          <t>12.15 System Health</t>
-        </is>
-      </c>
-      <c r="C297" s="3" t="n"/>
-      <c r="D297" s="3" t="n"/>
-      <c r="E297" s="3" t="n"/>
-      <c r="F297" s="3" t="n"/>
-      <c r="G297" s="3" t="n"/>
-      <c r="H297" s="3" t="n"/>
-      <c r="I297" s="3" t="n"/>
+      <c r="A297" s="4" t="inlineStr">
+        <is>
+          <t>TC-1418</t>
+        </is>
+      </c>
+      <c r="B297" s="4" t="inlineStr">
+        <is>
+          <t>12.14 Startup Reconciliation</t>
+        </is>
+      </c>
+      <c r="C297" s="4" t="inlineStr">
+        <is>
+          <t>Restart clears stale in-progress startup analysis when no valid cache remains</t>
+        </is>
+      </c>
+      <c r="D297" s="4" t="inlineStr">
+        <is>
+          <t>Trigger manual Analyze for a PENDING job, restart ECUBE before the scan completes, then reopen Job Detail</t>
+        </is>
+      </c>
+      <c r="E297" s="4" t="inlineStr">
+        <is>
+          <t>Job does not remain stuck in ANALYZING, startup-analysis state returns to NOT_ANALYZED, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "analysis_interrupted_by_restart", and Analyze or Start is available again</t>
+        </is>
+      </c>
+      <c r="F297" s="4" t="n"/>
+      <c r="G297" s="4" t="n"/>
+      <c r="H297" s="4" t="n"/>
+      <c r="I297" s="4" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="4" t="inlineStr">
         <is>
-          <t>TC-1501</t>
+          <t>TC-1419</t>
         </is>
       </c>
       <c r="B298" s="4" t="inlineStr">
         <is>
-          <t>12.15 System Health</t>
+          <t>12.14 Startup Reconciliation</t>
         </is>
       </c>
       <c r="C298" s="4" t="inlineStr">
         <is>
-          <t>Healthy response</t>
+          <t>Restart restores READY when the interrupted startup-analysis cache is still current</t>
         </is>
       </c>
       <c r="D298" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with valid token</t>
+          <t>Trigger manual Analyze for a job with a stable source tree, restart ECUBE after the reusable snapshot has been persisted but before the manual analyze workflow fully completes, then reopen Job Detail</t>
         </is>
       </c>
       <c r="E298" s="4" t="inlineStr">
         <is>
-          <t>200, status: "ok", database: "connected"</t>
+          <t>Job shows startup_analysis_status: READY, the previous file and byte totals are still available, audit log contains JOB_STARTUP_ANALYSIS_RECONCILED with reason: "valid_cache_restored_after_restart", and Start can proceed without forcing a fresh scan</t>
         </is>
       </c>
       <c r="F298" s="4" t="n"/>
@@ -9274,40 +9286,28 @@
       <c r="I298" s="4" t="n"/>
     </row>
     <row r="299">
-      <c r="A299" s="4" t="inlineStr">
-        <is>
-          <t>TC-1502</t>
-        </is>
-      </c>
-      <c r="B299" s="4" t="inlineStr">
+      <c r="A299" s="2" t="inlineStr">
+        <is>
+          <t>§12.15 System Health</t>
+        </is>
+      </c>
+      <c r="B299" s="2" t="inlineStr">
         <is>
           <t>12.15 System Health</t>
         </is>
       </c>
-      <c r="C299" s="4" t="inlineStr">
-        <is>
-          <t>CPU metric present</t>
-        </is>
-      </c>
-      <c r="D299" s="4" t="inlineStr">
-        <is>
-          <t>Inspect response body</t>
-        </is>
-      </c>
-      <c r="E299" s="4" t="inlineStr">
-        <is>
-          <t>cpu_percent is a number between 0 and 100</t>
-        </is>
-      </c>
-      <c r="F299" s="4" t="n"/>
-      <c r="G299" s="4" t="n"/>
-      <c r="H299" s="4" t="n"/>
-      <c r="I299" s="4" t="n"/>
+      <c r="C299" s="3" t="n"/>
+      <c r="D299" s="3" t="n"/>
+      <c r="E299" s="3" t="n"/>
+      <c r="F299" s="3" t="n"/>
+      <c r="G299" s="3" t="n"/>
+      <c r="H299" s="3" t="n"/>
+      <c r="I299" s="3" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="4" t="inlineStr">
         <is>
-          <t>TC-1503</t>
+          <t>TC-1501</t>
         </is>
       </c>
       <c r="B300" s="4" t="inlineStr">
@@ -9317,17 +9317,17 @@
       </c>
       <c r="C300" s="4" t="inlineStr">
         <is>
-          <t>CPU topology metrics present</t>
+          <t>Healthy response</t>
         </is>
       </c>
       <c r="D300" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body on a host where psutil reports CPU topology</t>
+          <t>GET /introspection/system-health with valid token</t>
         </is>
       </c>
       <c r="E300" s="4" t="inlineStr">
         <is>
-          <t>physical_cores and logical_cpus are positive integers; logical_cpus ≥ physical_cores</t>
+          <t>200, status: "ok", database: "connected"</t>
         </is>
       </c>
       <c r="F300" s="4" t="n"/>
@@ -9338,7 +9338,7 @@
     <row r="301">
       <c r="A301" s="4" t="inlineStr">
         <is>
-          <t>TC-1504</t>
+          <t>TC-1502</t>
         </is>
       </c>
       <c r="B301" s="4" t="inlineStr">
@@ -9348,17 +9348,17 @@
       </c>
       <c r="C301" s="4" t="inlineStr">
         <is>
-          <t>CPU topology metrics unavailable path</t>
+          <t>CPU metric present</t>
         </is>
       </c>
       <c r="D301" s="4" t="inlineStr">
         <is>
-          <t>Exercise endpoint where psutil is unavailable</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E301" s="4" t="inlineStr">
         <is>
-          <t>physical_cores and logical_cpus are null</t>
+          <t>cpu_percent is a number between 0 and 100</t>
         </is>
       </c>
       <c r="F301" s="4" t="n"/>
@@ -9369,7 +9369,7 @@
     <row r="302">
       <c r="A302" s="4" t="inlineStr">
         <is>
-          <t>TC-1505</t>
+          <t>TC-1503</t>
         </is>
       </c>
       <c r="B302" s="4" t="inlineStr">
@@ -9379,17 +9379,17 @@
       </c>
       <c r="C302" s="4" t="inlineStr">
         <is>
-          <t>System page CPU topology fallback rendering</t>
+          <t>CPU topology metrics present</t>
         </is>
       </c>
       <c r="D302" s="4" t="inlineStr">
         <is>
-          <t>Open System -&gt; System Health when backend returns physical_cores: null and logical_cpus: null</t>
+          <t>Inspect response body on a host where psutil reports CPU topology</t>
         </is>
       </c>
       <c r="E302" s="4" t="inlineStr">
         <is>
-          <t>Physical Cores and Logical CPUs display N/A; other host metrics continue rendering normally</t>
+          <t>physical_cores and logical_cpus are positive integers; logical_cpus ≥ physical_cores</t>
         </is>
       </c>
       <c r="F302" s="4" t="n"/>
@@ -9400,7 +9400,7 @@
     <row r="303">
       <c r="A303" s="4" t="inlineStr">
         <is>
-          <t>TC-1506</t>
+          <t>TC-1504</t>
         </is>
       </c>
       <c r="B303" s="4" t="inlineStr">
@@ -9410,17 +9410,17 @@
       </c>
       <c r="C303" s="4" t="inlineStr">
         <is>
-          <t>Memory metrics present</t>
+          <t>CPU topology metrics unavailable path</t>
         </is>
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Exercise endpoint where psutil is unavailable</t>
         </is>
       </c>
       <c r="E303" s="4" t="inlineStr">
         <is>
-          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
+          <t>physical_cores and logical_cpus are null</t>
         </is>
       </c>
       <c r="F303" s="4" t="n"/>
@@ -9431,7 +9431,7 @@
     <row r="304">
       <c r="A304" s="4" t="inlineStr">
         <is>
-          <t>TC-1507</t>
+          <t>TC-1505</t>
         </is>
       </c>
       <c r="B304" s="4" t="inlineStr">
@@ -9441,17 +9441,17 @@
       </c>
       <c r="C304" s="4" t="inlineStr">
         <is>
-          <t>Disk I/O metrics present</t>
+          <t>System page CPU topology fallback rendering</t>
         </is>
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Open System -&gt; System Health when backend returns physical_cores: null and logical_cpus: null</t>
         </is>
       </c>
       <c r="E304" s="4" t="inlineStr">
         <is>
-          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
+          <t>Physical Cores and Logical CPUs display N/A; other host metrics continue rendering normally</t>
         </is>
       </c>
       <c r="F304" s="4" t="n"/>
@@ -9462,7 +9462,7 @@
     <row r="305">
       <c r="A305" s="4" t="inlineStr">
         <is>
-          <t>TC-1508</t>
+          <t>TC-1506</t>
         </is>
       </c>
       <c r="B305" s="4" t="inlineStr">
@@ -9472,17 +9472,17 @@
       </c>
       <c r="C305" s="4" t="inlineStr">
         <is>
-          <t>Active jobs count</t>
+          <t>Memory metrics present</t>
         </is>
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>Start an export job, call endpoint</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E305" s="4" t="inlineStr">
         <is>
-          <t>active_jobs ≥ 1</t>
+          <t>memory_percent is a number; memory_used_bytes and memory_total_bytes are positive integers; memory_used_bytes ≤ memory_total_bytes</t>
         </is>
       </c>
       <c r="F305" s="4" t="n"/>
@@ -9493,7 +9493,7 @@
     <row r="306">
       <c r="A306" s="4" t="inlineStr">
         <is>
-          <t>TC-1509</t>
+          <t>TC-1507</t>
         </is>
       </c>
       <c r="B306" s="4" t="inlineStr">
@@ -9503,17 +9503,17 @@
       </c>
       <c r="C306" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size</t>
+          <t>Disk I/O metrics present</t>
         </is>
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>Create a PENDING job (created but not started), call endpoint</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E306" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size ≥ 1</t>
+          <t>disk_read_bytes and disk_write_bytes are non-negative integers</t>
         </is>
       </c>
       <c r="F306" s="4" t="n"/>
@@ -9524,7 +9524,7 @@
     <row r="307">
       <c r="A307" s="4" t="inlineStr">
         <is>
-          <t>TC-1510</t>
+          <t>TC-1508</t>
         </is>
       </c>
       <c r="B307" s="4" t="inlineStr">
@@ -9534,17 +9534,17 @@
       </c>
       <c r="C307" s="4" t="inlineStr">
         <is>
-          <t>Worker queue size decrements</t>
+          <t>Active jobs count</t>
         </is>
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>Start the pending job, call endpoint again</t>
+          <t>Start an export job, call endpoint</t>
         </is>
       </c>
       <c r="E307" s="4" t="inlineStr">
         <is>
-          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved out of PENDING and can still be in PREPARING before it reaches RUNNING)</t>
+          <t>active_jobs ≥ 1</t>
         </is>
       </c>
       <c r="F307" s="4" t="n"/>
@@ -9555,7 +9555,7 @@
     <row r="308">
       <c r="A308" s="4" t="inlineStr">
         <is>
-          <t>TC-1511</t>
+          <t>TC-1509</t>
         </is>
       </c>
       <c r="B308" s="4" t="inlineStr">
@@ -9565,17 +9565,17 @@
       </c>
       <c r="C308" s="4" t="inlineStr">
         <is>
-          <t>ECUBE process metrics present</t>
+          <t>Worker queue size</t>
         </is>
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>Inspect response body</t>
+          <t>Create a PENDING job (created but not started), call endpoint</t>
         </is>
       </c>
       <c r="E308" s="4" t="inlineStr">
         <is>
-          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
+          <t>worker_queue_size ≥ 1</t>
         </is>
       </c>
       <c r="F308" s="4" t="n"/>
@@ -9586,7 +9586,7 @@
     <row r="309">
       <c r="A309" s="4" t="inlineStr">
         <is>
-          <t>TC-1512</t>
+          <t>TC-1510</t>
         </is>
       </c>
       <c r="B309" s="4" t="inlineStr">
@@ -9596,17 +9596,17 @@
       </c>
       <c r="C309" s="4" t="inlineStr">
         <is>
-          <t>Active copy-thread correlation</t>
+          <t>Worker queue size decrements</t>
         </is>
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>Run an export job with active copy workers, call endpoint during the run</t>
+          <t>Start the pending job, call endpoint again</t>
         </is>
       </c>
       <c r="E309" s="4" t="inlineStr">
         <is>
-          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
+          <t>worker_queue_size decreases by 1 (is 0 if no other PENDING jobs exist; job moved out of PENDING and can still be in PREPARING before it reaches RUNNING)</t>
         </is>
       </c>
       <c r="F309" s="4" t="n"/>
@@ -9617,7 +9617,7 @@
     <row r="310">
       <c r="A310" s="4" t="inlineStr">
         <is>
-          <t>TC-1513</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B310" s="4" t="inlineStr">
@@ -9627,17 +9627,17 @@
       </c>
       <c r="C310" s="4" t="inlineStr">
         <is>
-          <t>ECUBE process metrics degrade safely</t>
+          <t>ECUBE process metrics present</t>
         </is>
       </c>
       <c r="D310" s="4" t="inlineStr">
         <is>
-          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
+          <t>Inspect response body</t>
         </is>
       </c>
       <c r="E310" s="4" t="inlineStr">
         <is>
-          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
+          <t>ecube_process object exists with cpu_percent, cpu_time_seconds, memory_rss_bytes, memory_vms_bytes, thread_count, active_copy_thread_count, and active_copy_threads</t>
         </is>
       </c>
       <c r="F310" s="4" t="n"/>
@@ -9648,7 +9648,7 @@
     <row r="311">
       <c r="A311" s="4" t="inlineStr">
         <is>
-          <t>TC-1514</t>
+          <t>TC-1512</t>
         </is>
       </c>
       <c r="B311" s="4" t="inlineStr">
@@ -9658,17 +9658,17 @@
       </c>
       <c r="C311" s="4" t="inlineStr">
         <is>
-          <t>Degraded when DB down</t>
+          <t>Active copy-thread correlation</t>
         </is>
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, call endpoint with valid token</t>
+          <t>Run an export job with active copy workers, call endpoint during the run</t>
         </is>
       </c>
       <c r="E311" s="4" t="inlineStr">
         <is>
-          <t>200, status: "degraded", database: "error", database_error is non-null</t>
+          <t>Each returned active_copy_threads row includes job_id, project_id, job_status, configured_thread_count, worker_label, elapsed_seconds, and cpu_time_seconds</t>
         </is>
       </c>
       <c r="F311" s="4" t="n"/>
@@ -9679,7 +9679,7 @@
     <row r="312">
       <c r="A312" s="4" t="inlineStr">
         <is>
-          <t>TC-1515</t>
+          <t>TC-1513</t>
         </is>
       </c>
       <c r="B312" s="4" t="inlineStr">
@@ -9689,17 +9689,17 @@
       </c>
       <c r="C312" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated rejected</t>
+          <t>ECUBE process metrics degrade safely</t>
         </is>
       </c>
       <c r="D312" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health without token</t>
+          <t>Exercise the endpoint where process/thread metrics cannot be sampled reliably</t>
         </is>
       </c>
       <c r="E312" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>ecube_process still exists; unavailable per-thread values remain null or the list is empty rather than returning unsafe host details</t>
         </is>
       </c>
       <c r="F312" s="4" t="n"/>
@@ -9710,7 +9710,7 @@
     <row r="313">
       <c r="A313" s="4" t="inlineStr">
         <is>
-          <t>TC-1516</t>
+          <t>TC-1514</t>
         </is>
       </c>
       <c r="B313" s="4" t="inlineStr">
@@ -9720,17 +9720,17 @@
       </c>
       <c r="C313" s="4" t="inlineStr">
         <is>
-          <t>Processor role allowed</t>
+          <t>Degraded when DB down</t>
         </is>
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/system-health with processor token</t>
+          <t>Stop PostgreSQL, call endpoint with valid token</t>
         </is>
       </c>
       <c r="E313" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, status: "degraded", database: "error", database_error is non-null</t>
         </is>
       </c>
       <c r="F313" s="4" t="n"/>
@@ -9739,48 +9739,60 @@
       <c r="I313" s="4" t="n"/>
     </row>
     <row r="314">
-      <c r="A314" s="2" t="inlineStr">
-        <is>
-          <t>§12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="B314" s="2" t="inlineStr">
-        <is>
-          <t>12.15.1 Readiness &amp; Version</t>
-        </is>
-      </c>
-      <c r="C314" s="3" t="n"/>
-      <c r="D314" s="3" t="n"/>
-      <c r="E314" s="3" t="n"/>
-      <c r="F314" s="3" t="n"/>
-      <c r="G314" s="3" t="n"/>
-      <c r="H314" s="3" t="n"/>
-      <c r="I314" s="3" t="n"/>
+      <c r="A314" s="4" t="inlineStr">
+        <is>
+          <t>TC-1515</t>
+        </is>
+      </c>
+      <c r="B314" s="4" t="inlineStr">
+        <is>
+          <t>12.15 System Health</t>
+        </is>
+      </c>
+      <c r="C314" s="4" t="inlineStr">
+        <is>
+          <t>Unauthenticated rejected</t>
+        </is>
+      </c>
+      <c r="D314" s="4" t="inlineStr">
+        <is>
+          <t>GET /introspection/system-health without token</t>
+        </is>
+      </c>
+      <c r="E314" s="4" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="F314" s="4" t="n"/>
+      <c r="G314" s="4" t="n"/>
+      <c r="H314" s="4" t="n"/>
+      <c r="I314" s="4" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="4" t="inlineStr">
         <is>
-          <t>TC-1511</t>
+          <t>TC-1516</t>
         </is>
       </c>
       <c r="B315" s="4" t="inlineStr">
         <is>
-          <t>12.15.1 Readiness &amp; Version</t>
+          <t>12.15 System Health</t>
         </is>
       </c>
       <c r="C315" s="4" t="inlineStr">
         <is>
-          <t>Liveness endpoint is public</t>
+          <t>Processor role allowed</t>
         </is>
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>GET /health/live without token</t>
+          <t>GET /introspection/system-health with processor token</t>
         </is>
       </c>
       <c r="E315" s="4" t="inlineStr">
         <is>
-          <t>200, service reports live</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F315" s="4" t="n"/>
@@ -9789,40 +9801,28 @@
       <c r="I315" s="4" t="n"/>
     </row>
     <row r="316">
-      <c r="A316" s="4" t="inlineStr">
-        <is>
-          <t>TC-1512</t>
-        </is>
-      </c>
-      <c r="B316" s="4" t="inlineStr">
+      <c r="A316" s="2" t="inlineStr">
+        <is>
+          <t>§12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="B316" s="2" t="inlineStr">
         <is>
           <t>12.15.1 Readiness &amp; Version</t>
         </is>
       </c>
-      <c r="C316" s="4" t="inlineStr">
-        <is>
-          <t>Readiness endpoint is public</t>
-        </is>
-      </c>
-      <c r="D316" s="4" t="inlineStr">
-        <is>
-          <t>GET /health/ready without token on a healthy system</t>
-        </is>
-      </c>
-      <c r="E316" s="4" t="inlineStr">
-        <is>
-          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
-        </is>
-      </c>
-      <c r="F316" s="4" t="n"/>
-      <c r="G316" s="4" t="n"/>
-      <c r="H316" s="4" t="n"/>
-      <c r="I316" s="4" t="n"/>
+      <c r="C316" s="3" t="n"/>
+      <c r="D316" s="3" t="n"/>
+      <c r="E316" s="3" t="n"/>
+      <c r="F316" s="3" t="n"/>
+      <c r="G316" s="3" t="n"/>
+      <c r="H316" s="3" t="n"/>
+      <c r="I316" s="3" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="4" t="inlineStr">
         <is>
-          <t>TC-1513</t>
+          <t>TC-1511</t>
         </is>
       </c>
       <c r="B317" s="4" t="inlineStr">
@@ -9832,17 +9832,17 @@
       </c>
       <c r="C317" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports missing database configuration</t>
+          <t>Liveness endpoint is public</t>
         </is>
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t>Clear DB config or test before configuration, then GET /health/ready</t>
+          <t>GET /health/live without token</t>
         </is>
       </c>
       <c r="E317" s="4" t="inlineStr">
         <is>
-          <t>503, status: "not_ready", reason indicates database is not configured</t>
+          <t>200, service reports live</t>
         </is>
       </c>
       <c r="F317" s="4" t="n"/>
@@ -9853,7 +9853,7 @@
     <row r="318">
       <c r="A318" s="4" t="inlineStr">
         <is>
-          <t>TC-1514</t>
+          <t>TC-1512</t>
         </is>
       </c>
       <c r="B318" s="4" t="inlineStr">
@@ -9863,17 +9863,17 @@
       </c>
       <c r="C318" s="4" t="inlineStr">
         <is>
-          <t>Readiness reports mount or provider problems</t>
+          <t>Readiness endpoint is public</t>
         </is>
       </c>
       <c r="D318" s="4" t="inlineStr">
         <is>
-          <t>Break a configured mount or provider, then GET /health/ready</t>
+          <t>GET /health/ready without token on a healthy system</t>
         </is>
       </c>
       <c r="E318" s="4" t="inlineStr">
         <is>
-          <t>503, response identifies the failing check without using the generic error schema</t>
+          <t>200, status: "ready", checks show healthy or initialized dependencies</t>
         </is>
       </c>
       <c r="F318" s="4" t="n"/>
@@ -9884,7 +9884,7 @@
     <row r="319">
       <c r="A319" s="4" t="inlineStr">
         <is>
-          <t>TC-1515</t>
+          <t>TC-1513</t>
         </is>
       </c>
       <c r="B319" s="4" t="inlineStr">
@@ -9894,17 +9894,17 @@
       </c>
       <c r="C319" s="4" t="inlineStr">
         <is>
-          <t>Version endpoint is public</t>
+          <t>Readiness reports missing database configuration</t>
         </is>
       </c>
       <c r="D319" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/version without token</t>
+          <t>Clear DB config or test before configuration, then GET /health/ready</t>
         </is>
       </c>
       <c r="E319" s="4" t="inlineStr">
         <is>
-          <t>200, returns version/application metadata</t>
+          <t>503, status: "not_ready", reason indicates database is not configured</t>
         </is>
       </c>
       <c r="F319" s="4" t="n"/>
@@ -9915,7 +9915,7 @@
     <row r="320">
       <c r="A320" s="4" t="inlineStr">
         <is>
-          <t>TC-1516</t>
+          <t>TC-1514</t>
         </is>
       </c>
       <c r="B320" s="4" t="inlineStr">
@@ -9925,17 +9925,17 @@
       </c>
       <c r="C320" s="4" t="inlineStr">
         <is>
-          <t>Readiness remains separate from authenticated system health</t>
+          <t>Readiness reports mount or provider problems</t>
         </is>
       </c>
       <c r="D320" s="4" t="inlineStr">
         <is>
-          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+          <t>Break a configured mount or provider, then GET /health/ready</t>
         </is>
       </c>
       <c r="E320" s="4" t="inlineStr">
         <is>
-          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+          <t>503, response identifies the failing check without using the generic error schema</t>
         </is>
       </c>
       <c r="F320" s="4" t="n"/>
@@ -9946,7 +9946,7 @@
     <row r="321">
       <c r="A321" s="4" t="inlineStr">
         <is>
-          <t>TC-1517</t>
+          <t>TC-1515</t>
         </is>
       </c>
       <c r="B321" s="4" t="inlineStr">
@@ -9956,17 +9956,17 @@
       </c>
       <c r="C321" s="4" t="inlineStr">
         <is>
-          <t>Metrics endpoint enforces read-only observability roles</t>
+          <t>Version endpoint is public</t>
         </is>
       </c>
       <c r="D321" s="4" t="inlineStr">
         <is>
-          <t>GET /metrics without a token, with a processor token, and with an auditor or admin token</t>
+          <t>GET /introspection/version without token</t>
         </is>
       </c>
       <c r="E321" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated requests return 401, non-observability roles return 403, and admin/auditor receive Prometheus text exposition</t>
+          <t>200, returns version/application metadata</t>
         </is>
       </c>
       <c r="F321" s="4" t="n"/>
@@ -9975,32 +9975,94 @@
       <c r="I321" s="4" t="n"/>
     </row>
     <row r="322">
-      <c r="A322" s="2" t="inlineStr">
+      <c r="A322" s="4" t="inlineStr">
+        <is>
+          <t>TC-1516</t>
+        </is>
+      </c>
+      <c r="B322" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C322" s="4" t="inlineStr">
+        <is>
+          <t>Readiness remains separate from authenticated system health</t>
+        </is>
+      </c>
+      <c r="D322" s="4" t="inlineStr">
+        <is>
+          <t>Compare GET /health/ready and authenticated GET /introspection/system-health</t>
+        </is>
+      </c>
+      <c r="E322" s="4" t="inlineStr">
+        <is>
+          <t>Readiness stays public and fail-fast; system health returns richer operational metrics</t>
+        </is>
+      </c>
+      <c r="F322" s="4" t="n"/>
+      <c r="G322" s="4" t="n"/>
+      <c r="H322" s="4" t="n"/>
+      <c r="I322" s="4" t="n"/>
+    </row>
+    <row r="323">
+      <c r="A323" s="4" t="inlineStr">
+        <is>
+          <t>TC-1517</t>
+        </is>
+      </c>
+      <c r="B323" s="4" t="inlineStr">
+        <is>
+          <t>12.15.1 Readiness &amp; Version</t>
+        </is>
+      </c>
+      <c r="C323" s="4" t="inlineStr">
+        <is>
+          <t>Metrics endpoint enforces read-only observability roles</t>
+        </is>
+      </c>
+      <c r="D323" s="4" t="inlineStr">
+        <is>
+          <t>GET /metrics without a token, with a processor token, and with an auditor or admin token</t>
+        </is>
+      </c>
+      <c r="E323" s="4" t="inlineStr">
+        <is>
+          <t>Unauthenticated requests return 401, non-observability roles return 403, and admin/auditor receive Prometheus text exposition</t>
+        </is>
+      </c>
+      <c r="F323" s="4" t="n"/>
+      <c r="G323" s="4" t="n"/>
+      <c r="H323" s="4" t="n"/>
+      <c r="I323" s="4" t="n"/>
+    </row>
+    <row r="324">
+      <c r="A324" s="2" t="inlineStr">
         <is>
           <t>§12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="B322" s="2" t="inlineStr">
+      <c r="B324" s="2" t="inlineStr">
         <is>
           <t>12.16 Real-World Copy Performance &amp; Hashing Addendum</t>
         </is>
       </c>
-      <c r="C322" s="3" t="n"/>
-      <c r="D322" s="3" t="n"/>
-      <c r="E322" s="3" t="n"/>
-      <c r="F322" s="3" t="n"/>
-      <c r="G322" s="3" t="n"/>
-      <c r="H322" s="3" t="n"/>
-      <c r="I322" s="3" t="n"/>
-    </row>
-    <row r="324">
-      <c r="A324" s="5" t="inlineStr">
+      <c r="C324" s="3" t="n"/>
+      <c r="D324" s="3" t="n"/>
+      <c r="E324" s="3" t="n"/>
+      <c r="F324" s="3" t="n"/>
+      <c r="G324" s="3" t="n"/>
+      <c r="H324" s="3" t="n"/>
+      <c r="I324" s="3" t="n"/>
+    </row>
+    <row r="326">
+      <c r="A326" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B324" s="5" t="n">
-        <v>294</v>
+      <c r="B326" s="5" t="n">
+        <v>296</v>
       </c>
     </row>
   </sheetData>

</xml_diff>